<commit_message>
Update election results snapshot (45.8% counted)
TVK leads 110 seats, AIADMK 59, DMK 48. 9 lead changes this round;
9 seats still in play. TVK + allies projected past 118 majority mark.

https://claude.ai/code/session_01MizbUy44JG5sXyvaf3Wekb
</commit_message>
<xml_diff>
--- a/tn_election_results_may2026.xlsx
+++ b/tn_election_results_may2026.xlsx
@@ -91,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -127,18 +127,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -616,11 +604,11 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>11108</v>
+        <v>11948</v>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>8/31</t>
+          <t>9/31</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -629,10 +617,10 @@
         </is>
       </c>
       <c r="J2" s="4" t="n">
-        <v>43044</v>
+        <v>41154</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>1388.5</v>
+        <v>1327.555555555556</v>
       </c>
     </row>
     <row r="3">
@@ -695,30 +683,30 @@
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
+          <t>K R P PRABAKARAN</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>All India Anna Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
           <t>PAUL MANOJ PANDIAN</t>
         </is>
       </c>
-      <c r="D4" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E4" s="10" t="inlineStr">
-        <is>
-          <t>K R P PRABAKARAN</t>
-        </is>
-      </c>
       <c r="F4" s="10" t="inlineStr">
         <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
+          <t>Dravida Munnetra Kazhagam</t>
         </is>
       </c>
       <c r="G4" s="11" t="n">
-        <v>335</v>
+        <v>196</v>
       </c>
       <c r="H4" s="10" t="inlineStr">
         <is>
-          <t>12/24</t>
+          <t>13/24</t>
         </is>
       </c>
       <c r="I4" s="10" t="inlineStr">
@@ -727,10 +715,10 @@
         </is>
       </c>
       <c r="J4" s="11" t="n">
-        <v>670</v>
+        <v>362</v>
       </c>
       <c r="K4" s="12" t="n">
-        <v>27.91666666666667</v>
+        <v>15.07692307692308</v>
       </c>
     </row>
     <row r="5">
@@ -763,11 +751,11 @@
         </is>
       </c>
       <c r="G5" s="7" t="n">
-        <v>5818</v>
+        <v>5984</v>
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>13/23</t>
+          <t>14/23</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr">
@@ -776,10 +764,10 @@
         </is>
       </c>
       <c r="J5" s="7" t="n">
-        <v>10293</v>
+        <v>9831</v>
       </c>
       <c r="K5" s="8" t="n">
-        <v>447.5384615384616</v>
+        <v>427.4285714285714</v>
       </c>
     </row>
     <row r="6">
@@ -861,11 +849,11 @@
         </is>
       </c>
       <c r="G7" s="7" t="n">
-        <v>4614</v>
+        <v>6703</v>
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>7/22</t>
+          <t>8/22</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
@@ -874,10 +862,10 @@
         </is>
       </c>
       <c r="J7" s="7" t="n">
-        <v>14501</v>
+        <v>18433</v>
       </c>
       <c r="K7" s="8" t="n">
-        <v>659.1428571428571</v>
+        <v>837.875</v>
       </c>
     </row>
     <row r="8">
@@ -959,11 +947,11 @@
         </is>
       </c>
       <c r="G9" s="7" t="n">
-        <v>704</v>
+        <v>722</v>
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>11/25</t>
+          <t>12/25</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
@@ -972,10 +960,10 @@
         </is>
       </c>
       <c r="J9" s="7" t="n">
-        <v>1600</v>
+        <v>1504</v>
       </c>
       <c r="K9" s="8" t="n">
-        <v>64</v>
+        <v>60.16666666666666</v>
       </c>
     </row>
     <row r="10">
@@ -1057,11 +1045,11 @@
         </is>
       </c>
       <c r="G11" s="7" t="n">
-        <v>2221</v>
+        <v>2166</v>
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>14/20</t>
+          <t>15/20</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
@@ -1070,10 +1058,10 @@
         </is>
       </c>
       <c r="J11" s="7" t="n">
-        <v>3173</v>
+        <v>2888</v>
       </c>
       <c r="K11" s="8" t="n">
-        <v>158.6428571428571</v>
+        <v>144.4</v>
       </c>
     </row>
     <row r="12">
@@ -1106,11 +1094,11 @@
         </is>
       </c>
       <c r="G12" s="4" t="n">
-        <v>13523</v>
+        <v>14059</v>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>11/21</t>
+          <t>12/21</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
@@ -1119,10 +1107,10 @@
         </is>
       </c>
       <c r="J12" s="4" t="n">
-        <v>25817</v>
+        <v>24603</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1229.363636363636</v>
+        <v>1171.583333333333</v>
       </c>
     </row>
     <row r="13">
@@ -1204,11 +1192,11 @@
         </is>
       </c>
       <c r="G14" s="4" t="n">
-        <v>10296</v>
+        <v>11720</v>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>9/22</t>
+          <t>10/22</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
@@ -1217,10 +1205,10 @@
         </is>
       </c>
       <c r="J14" s="4" t="n">
-        <v>25168</v>
+        <v>25784</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>1144</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="15">
@@ -1302,11 +1290,11 @@
         </is>
       </c>
       <c r="G16" s="4" t="n">
-        <v>9899</v>
+        <v>11964</v>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>6/23</t>
+          <t>7/23</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
@@ -1315,10 +1303,10 @@
         </is>
       </c>
       <c r="J16" s="4" t="n">
-        <v>37946</v>
+        <v>39310</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>1649.833333333333</v>
+        <v>1709.142857142857</v>
       </c>
     </row>
     <row r="17">
@@ -1351,11 +1339,11 @@
         </is>
       </c>
       <c r="G17" s="7" t="n">
-        <v>9814</v>
+        <v>9960</v>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>13/24</t>
+          <t>14/24</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
@@ -1364,10 +1352,10 @@
         </is>
       </c>
       <c r="J17" s="7" t="n">
-        <v>18118</v>
+        <v>17074</v>
       </c>
       <c r="K17" s="8" t="n">
-        <v>754.9230769230769</v>
+        <v>711.4285714285714</v>
       </c>
     </row>
     <row r="18">
@@ -1400,11 +1388,11 @@
         </is>
       </c>
       <c r="G18" s="7" t="n">
-        <v>2147</v>
+        <v>2937</v>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>9/20</t>
+          <t>10/20</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr">
@@ -1413,10 +1401,10 @@
         </is>
       </c>
       <c r="J18" s="7" t="n">
-        <v>4771</v>
+        <v>5874</v>
       </c>
       <c r="K18" s="8" t="n">
-        <v>238.5555555555555</v>
+        <v>293.7</v>
       </c>
     </row>
     <row r="19">
@@ -1498,11 +1486,11 @@
         </is>
       </c>
       <c r="G20" s="7" t="n">
-        <v>11736</v>
+        <v>11672</v>
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>14/22</t>
+          <t>15/22</t>
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr">
@@ -1511,10 +1499,10 @@
         </is>
       </c>
       <c r="J20" s="7" t="n">
-        <v>18442</v>
+        <v>17119</v>
       </c>
       <c r="K20" s="8" t="n">
-        <v>838.2857142857143</v>
+        <v>778.1333333333334</v>
       </c>
     </row>
     <row r="21">
@@ -1694,11 +1682,11 @@
         </is>
       </c>
       <c r="G24" s="7" t="n">
-        <v>6904</v>
+        <v>8044</v>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>9/22</t>
+          <t>10/22</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr">
@@ -1707,10 +1695,10 @@
         </is>
       </c>
       <c r="J24" s="7" t="n">
-        <v>16876</v>
+        <v>17697</v>
       </c>
       <c r="K24" s="8" t="n">
-        <v>767.1111111111111</v>
+        <v>804.4</v>
       </c>
     </row>
     <row r="25">
@@ -1812,52 +1800,52 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="9" t="inlineStr">
+      <c r="A27" s="6" t="inlineStr">
         <is>
           <t>BODINAYAKANUR</t>
         </is>
       </c>
-      <c r="B27" s="10" t="n">
+      <c r="B27" s="6" t="n">
         <v>200</v>
       </c>
-      <c r="C27" s="10" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>PRAKASH.S</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>PANNEERSELVAM.O</t>
         </is>
       </c>
-      <c r="D27" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E27" s="10" t="inlineStr">
-        <is>
-          <t>PRAKASH.S</t>
-        </is>
-      </c>
-      <c r="F27" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G27" s="11" t="n">
-        <v>173</v>
-      </c>
-      <c r="H27" s="10" t="inlineStr">
-        <is>
-          <t>9/25</t>
-        </is>
-      </c>
-      <c r="I27" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J27" s="11" t="n">
-        <v>481</v>
-      </c>
-      <c r="K27" s="12" t="n">
-        <v>19.22222222222222</v>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="n">
+        <v>487</v>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>10/25</t>
+        </is>
+      </c>
+      <c r="I27" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J27" s="7" t="n">
+        <v>1218</v>
+      </c>
+      <c r="K27" s="8" t="n">
+        <v>48.7</v>
       </c>
     </row>
     <row r="28">
@@ -2037,11 +2025,11 @@
         </is>
       </c>
       <c r="G31" s="4" t="n">
-        <v>14219</v>
+        <v>14793</v>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>17/24</t>
+          <t>18/24</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -2050,10 +2038,10 @@
         </is>
       </c>
       <c r="J31" s="4" t="n">
-        <v>20074</v>
+        <v>19724</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>836.4117647058823</v>
+        <v>821.8333333333334</v>
       </c>
     </row>
     <row r="32">
@@ -2086,11 +2074,11 @@
         </is>
       </c>
       <c r="G32" s="7" t="n">
-        <v>2484</v>
+        <v>2771</v>
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>13/21</t>
+          <t>14/21</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
@@ -2099,10 +2087,10 @@
         </is>
       </c>
       <c r="J32" s="7" t="n">
-        <v>4013</v>
+        <v>4156</v>
       </c>
       <c r="K32" s="8" t="n">
-        <v>191.0769230769231</v>
+        <v>197.9285714285714</v>
       </c>
     </row>
     <row r="33">
@@ -2155,52 +2143,52 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="6" t="inlineStr">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>COIMBATORE (NORTH)</t>
         </is>
       </c>
-      <c r="B34" s="6" t="n">
+      <c r="B34" s="3" t="n">
         <v>118</v>
       </c>
-      <c r="C34" s="6" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>V. SAMPATHKUMAR</t>
         </is>
       </c>
-      <c r="D34" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E34" s="6" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
         <is>
           <t>DURAI. SENTHAMIL SELVAN B.E</t>
         </is>
       </c>
-      <c r="F34" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G34" s="7" t="n">
-        <v>4009</v>
-      </c>
-      <c r="H34" s="6" t="inlineStr">
-        <is>
-          <t>6/25</t>
-        </is>
-      </c>
-      <c r="I34" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J34" s="7" t="n">
-        <v>16704</v>
-      </c>
-      <c r="K34" s="8" t="n">
-        <v>668.1666666666666</v>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="n">
+        <v>5933</v>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>7/25</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J34" s="4" t="n">
+        <v>21189</v>
+      </c>
+      <c r="K34" s="5" t="n">
+        <v>847.5714285714284</v>
       </c>
     </row>
     <row r="35">
@@ -2282,11 +2270,11 @@
         </is>
       </c>
       <c r="G36" s="7" t="n">
-        <v>3585</v>
+        <v>3373</v>
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>6/23</t>
+          <t>7/23</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
@@ -2295,10 +2283,10 @@
         </is>
       </c>
       <c r="J36" s="7" t="n">
-        <v>13742</v>
+        <v>11083</v>
       </c>
       <c r="K36" s="8" t="n">
-        <v>597.5</v>
+        <v>481.8571428571428</v>
       </c>
     </row>
     <row r="37">
@@ -2576,11 +2564,11 @@
         </is>
       </c>
       <c r="G42" s="7" t="n">
-        <v>1649</v>
+        <v>1638</v>
       </c>
       <c r="H42" s="6" t="inlineStr">
         <is>
-          <t>12/24</t>
+          <t>13/24</t>
         </is>
       </c>
       <c r="I42" s="6" t="inlineStr">
@@ -2589,10 +2577,10 @@
         </is>
       </c>
       <c r="J42" s="7" t="n">
-        <v>3298</v>
+        <v>3024</v>
       </c>
       <c r="K42" s="8" t="n">
-        <v>137.4166666666667</v>
+        <v>126</v>
       </c>
     </row>
     <row r="43">
@@ -2674,11 +2662,11 @@
         </is>
       </c>
       <c r="G44" s="4" t="n">
-        <v>46079</v>
+        <v>50379</v>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>12/25</t>
+          <t>13/25</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
@@ -2687,10 +2675,10 @@
         </is>
       </c>
       <c r="J44" s="4" t="n">
-        <v>95998</v>
+        <v>96883</v>
       </c>
       <c r="K44" s="5" t="n">
-        <v>3839.916666666667</v>
+        <v>3875.307692307692</v>
       </c>
     </row>
     <row r="45">
@@ -2723,11 +2711,11 @@
         </is>
       </c>
       <c r="G45" s="7" t="n">
-        <v>9028</v>
+        <v>10722</v>
       </c>
       <c r="H45" s="6" t="inlineStr">
         <is>
-          <t>9/15</t>
+          <t>10/15</t>
         </is>
       </c>
       <c r="I45" s="6" t="inlineStr">
@@ -2736,10 +2724,10 @@
         </is>
       </c>
       <c r="J45" s="7" t="n">
-        <v>15047</v>
+        <v>16083</v>
       </c>
       <c r="K45" s="8" t="n">
-        <v>1003.111111111111</v>
+        <v>1072.2</v>
       </c>
     </row>
     <row r="46">
@@ -2861,20 +2849,20 @@
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>M. CHINNADURAI</t>
+          <t>C. UTHAYAKUMAR</t>
         </is>
       </c>
       <c r="F48" s="6" t="inlineStr">
         <is>
-          <t>Communist Party of India (Marxist)</t>
+          <t>Bharatiya Janata Party</t>
         </is>
       </c>
       <c r="G48" s="7" t="n">
-        <v>5081</v>
+        <v>5083</v>
       </c>
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>6/18</t>
+          <t>7/18</t>
         </is>
       </c>
       <c r="I48" s="6" t="inlineStr">
@@ -2883,10 +2871,10 @@
         </is>
       </c>
       <c r="J48" s="7" t="n">
-        <v>15243</v>
+        <v>13071</v>
       </c>
       <c r="K48" s="8" t="n">
-        <v>846.8333333333334</v>
+        <v>726.1428571428571</v>
       </c>
     </row>
     <row r="49">
@@ -3213,11 +3201,11 @@
         </is>
       </c>
       <c r="G55" s="7" t="n">
-        <v>3755</v>
+        <v>4706</v>
       </c>
       <c r="H55" s="6" t="inlineStr">
         <is>
-          <t>6/14</t>
+          <t>7/14</t>
         </is>
       </c>
       <c r="I55" s="6" t="inlineStr">
@@ -3226,10 +3214,10 @@
         </is>
       </c>
       <c r="J55" s="7" t="n">
-        <v>8762</v>
+        <v>9412</v>
       </c>
       <c r="K55" s="8" t="n">
-        <v>625.8333333333334</v>
+        <v>672.2857142857143</v>
       </c>
     </row>
     <row r="56">
@@ -3311,11 +3299,11 @@
         </is>
       </c>
       <c r="G57" s="4" t="n">
-        <v>22817</v>
+        <v>24107</v>
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>11/34</t>
+          <t>12/34</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr">
@@ -3324,10 +3312,10 @@
         </is>
       </c>
       <c r="J57" s="4" t="n">
-        <v>70525</v>
+        <v>68303</v>
       </c>
       <c r="K57" s="5" t="n">
-        <v>2074.272727272727</v>
+        <v>2008.916666666667</v>
       </c>
     </row>
     <row r="58">
@@ -3360,11 +3348,11 @@
         </is>
       </c>
       <c r="G58" s="4" t="n">
-        <v>9255</v>
+        <v>9693</v>
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>10/23</t>
+          <t>11/23</t>
         </is>
       </c>
       <c r="I58" s="3" t="inlineStr">
@@ -3373,10 +3361,10 @@
         </is>
       </c>
       <c r="J58" s="4" t="n">
-        <v>21286</v>
+        <v>20267</v>
       </c>
       <c r="K58" s="5" t="n">
-        <v>925.5</v>
+        <v>881.1818181818181</v>
       </c>
     </row>
     <row r="59">
@@ -3409,11 +3397,11 @@
         </is>
       </c>
       <c r="G59" s="7" t="n">
-        <v>6775</v>
+        <v>6986</v>
       </c>
       <c r="H59" s="6" t="inlineStr">
         <is>
-          <t>8/21</t>
+          <t>9/21</t>
         </is>
       </c>
       <c r="I59" s="6" t="inlineStr">
@@ -3422,10 +3410,10 @@
         </is>
       </c>
       <c r="J59" s="7" t="n">
-        <v>17784</v>
+        <v>16301</v>
       </c>
       <c r="K59" s="8" t="n">
-        <v>846.875</v>
+        <v>776.2222222222222</v>
       </c>
     </row>
     <row r="60">
@@ -3458,11 +3446,11 @@
         </is>
       </c>
       <c r="G60" s="7" t="n">
-        <v>2558</v>
+        <v>1912</v>
       </c>
       <c r="H60" s="6" t="inlineStr">
         <is>
-          <t>9/26</t>
+          <t>10/26</t>
         </is>
       </c>
       <c r="I60" s="6" t="inlineStr">
@@ -3471,10 +3459,10 @@
         </is>
       </c>
       <c r="J60" s="7" t="n">
-        <v>7390</v>
+        <v>4971</v>
       </c>
       <c r="K60" s="8" t="n">
-        <v>284.2222222222222</v>
+        <v>191.2</v>
       </c>
     </row>
     <row r="61">
@@ -3605,11 +3593,11 @@
         </is>
       </c>
       <c r="G63" s="7" t="n">
-        <v>1498</v>
+        <v>2044</v>
       </c>
       <c r="H63" s="6" t="inlineStr">
         <is>
-          <t>8/26</t>
+          <t>9/26</t>
         </is>
       </c>
       <c r="I63" s="6" t="inlineStr">
@@ -3618,10 +3606,10 @@
         </is>
       </c>
       <c r="J63" s="7" t="n">
-        <v>4868</v>
+        <v>5905</v>
       </c>
       <c r="K63" s="8" t="n">
-        <v>187.25</v>
+        <v>227.1111111111111</v>
       </c>
     </row>
     <row r="64">
@@ -3654,11 +3642,11 @@
         </is>
       </c>
       <c r="G64" s="7" t="n">
-        <v>3950</v>
+        <v>3853</v>
       </c>
       <c r="H64" s="6" t="inlineStr">
         <is>
-          <t>10/23</t>
+          <t>11/23</t>
         </is>
       </c>
       <c r="I64" s="6" t="inlineStr">
@@ -3667,10 +3655,10 @@
         </is>
       </c>
       <c r="J64" s="7" t="n">
-        <v>9085</v>
+        <v>8056</v>
       </c>
       <c r="K64" s="8" t="n">
-        <v>395</v>
+        <v>350.2727272727273</v>
       </c>
     </row>
     <row r="65">
@@ -3948,11 +3936,11 @@
         </is>
       </c>
       <c r="G70" s="4" t="n">
-        <v>28394</v>
+        <v>29048</v>
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>18/28</t>
+          <t>19/28</t>
         </is>
       </c>
       <c r="I70" s="3" t="inlineStr">
@@ -3961,10 +3949,10 @@
         </is>
       </c>
       <c r="J70" s="4" t="n">
-        <v>44168</v>
+        <v>42808</v>
       </c>
       <c r="K70" s="5" t="n">
-        <v>1577.444444444444</v>
+        <v>1528.842105263158</v>
       </c>
     </row>
     <row r="71">
@@ -4046,11 +4034,11 @@
         </is>
       </c>
       <c r="G72" s="4" t="n">
-        <v>24843</v>
+        <v>26000</v>
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>13/22</t>
+          <t>14/22</t>
         </is>
       </c>
       <c r="I72" s="3" t="inlineStr">
@@ -4059,10 +4047,10 @@
         </is>
       </c>
       <c r="J72" s="4" t="n">
-        <v>42042</v>
+        <v>40857</v>
       </c>
       <c r="K72" s="5" t="n">
-        <v>1911</v>
+        <v>1857.142857142857</v>
       </c>
     </row>
     <row r="73">
@@ -4144,11 +4132,11 @@
         </is>
       </c>
       <c r="G74" s="7" t="n">
-        <v>659</v>
+        <v>1667</v>
       </c>
       <c r="H74" s="6" t="inlineStr">
         <is>
-          <t>8/16</t>
+          <t>9/16</t>
         </is>
       </c>
       <c r="I74" s="6" t="inlineStr">
@@ -4157,10 +4145,10 @@
         </is>
       </c>
       <c r="J74" s="7" t="n">
-        <v>1318</v>
+        <v>2964</v>
       </c>
       <c r="K74" s="8" t="n">
-        <v>82.375</v>
+        <v>185.2222222222222</v>
       </c>
     </row>
     <row r="75">
@@ -4193,11 +4181,11 @@
         </is>
       </c>
       <c r="G75" s="7" t="n">
-        <v>10151</v>
+        <v>11230</v>
       </c>
       <c r="H75" s="6" t="inlineStr">
         <is>
-          <t>19/28</t>
+          <t>20/28</t>
         </is>
       </c>
       <c r="I75" s="6" t="inlineStr">
@@ -4206,10 +4194,10 @@
         </is>
       </c>
       <c r="J75" s="7" t="n">
-        <v>14959</v>
+        <v>15722</v>
       </c>
       <c r="K75" s="8" t="n">
-        <v>534.2631578947369</v>
+        <v>561.5</v>
       </c>
     </row>
     <row r="76">
@@ -4242,11 +4230,11 @@
         </is>
       </c>
       <c r="G76" s="7" t="n">
-        <v>8406</v>
+        <v>8019</v>
       </c>
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>10/22</t>
+          <t>11/22</t>
         </is>
       </c>
       <c r="I76" s="6" t="inlineStr">
@@ -4255,10 +4243,10 @@
         </is>
       </c>
       <c r="J76" s="7" t="n">
-        <v>18493</v>
+        <v>16038</v>
       </c>
       <c r="K76" s="8" t="n">
-        <v>840.6</v>
+        <v>729</v>
       </c>
     </row>
     <row r="77">
@@ -4340,11 +4328,11 @@
         </is>
       </c>
       <c r="G78" s="4" t="n">
-        <v>15921</v>
+        <v>17430</v>
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
-          <t>14/25</t>
+          <t>15/25</t>
         </is>
       </c>
       <c r="I78" s="3" t="inlineStr">
@@ -4353,10 +4341,10 @@
         </is>
       </c>
       <c r="J78" s="4" t="n">
-        <v>28430</v>
+        <v>29050</v>
       </c>
       <c r="K78" s="5" t="n">
-        <v>1137.214285714286</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="79">
@@ -4389,11 +4377,11 @@
         </is>
       </c>
       <c r="G79" s="7" t="n">
-        <v>808</v>
+        <v>1099</v>
       </c>
       <c r="H79" s="6" t="inlineStr">
         <is>
-          <t>7/20</t>
+          <t>8/20</t>
         </is>
       </c>
       <c r="I79" s="6" t="inlineStr">
@@ -4402,10 +4390,10 @@
         </is>
       </c>
       <c r="J79" s="7" t="n">
-        <v>2309</v>
+        <v>2748</v>
       </c>
       <c r="K79" s="8" t="n">
-        <v>115.4285714285714</v>
+        <v>137.375</v>
       </c>
     </row>
     <row r="80">
@@ -4487,11 +4475,11 @@
         </is>
       </c>
       <c r="G81" s="7" t="n">
-        <v>2681</v>
+        <v>2613</v>
       </c>
       <c r="H81" s="6" t="inlineStr">
         <is>
-          <t>7/24</t>
+          <t>8/24</t>
         </is>
       </c>
       <c r="I81" s="6" t="inlineStr">
@@ -4500,10 +4488,10 @@
         </is>
       </c>
       <c r="J81" s="7" t="n">
-        <v>9192</v>
+        <v>7839</v>
       </c>
       <c r="K81" s="8" t="n">
-        <v>383</v>
+        <v>326.625</v>
       </c>
     </row>
     <row r="82">
@@ -4536,11 +4524,11 @@
         </is>
       </c>
       <c r="G82" s="7" t="n">
-        <v>2037</v>
+        <v>2323</v>
       </c>
       <c r="H82" s="6" t="inlineStr">
         <is>
-          <t>13/22</t>
+          <t>14/22</t>
         </is>
       </c>
       <c r="I82" s="6" t="inlineStr">
@@ -4549,10 +4537,10 @@
         </is>
       </c>
       <c r="J82" s="7" t="n">
-        <v>3447</v>
+        <v>3650</v>
       </c>
       <c r="K82" s="8" t="n">
-        <v>156.6923076923077</v>
+        <v>165.9285714285714</v>
       </c>
     </row>
     <row r="83">
@@ -4585,11 +4573,11 @@
         </is>
       </c>
       <c r="G83" s="4" t="n">
-        <v>12879</v>
+        <v>13474</v>
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
-          <t>12/25</t>
+          <t>13/25</t>
         </is>
       </c>
       <c r="I83" s="3" t="inlineStr">
@@ -4598,59 +4586,59 @@
         </is>
       </c>
       <c r="J83" s="4" t="n">
-        <v>26831</v>
+        <v>25912</v>
       </c>
       <c r="K83" s="5" t="n">
-        <v>1073.25</v>
+        <v>1036.461538461539</v>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="9" t="inlineStr">
+      <c r="A84" s="6" t="inlineStr">
         <is>
           <t>KURINJIPADI</t>
         </is>
       </c>
-      <c r="B84" s="10" t="n">
+      <c r="B84" s="6" t="n">
         <v>156</v>
       </c>
-      <c r="C84" s="10" t="inlineStr">
+      <c r="C84" s="6" t="inlineStr">
+        <is>
+          <t>M.R.K.PANNEERSELVAM</t>
+        </is>
+      </c>
+      <c r="D84" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E84" s="6" t="inlineStr">
         <is>
           <t>A BHUVANENTHIRAN</t>
         </is>
       </c>
-      <c r="D84" s="10" t="inlineStr">
+      <c r="F84" s="6" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E84" s="10" t="inlineStr">
-        <is>
-          <t>M.R.K.PANNEERSELVAM</t>
-        </is>
-      </c>
-      <c r="F84" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G84" s="11" t="n">
-        <v>126</v>
-      </c>
-      <c r="H84" s="10" t="inlineStr">
-        <is>
-          <t>11/20</t>
-        </is>
-      </c>
-      <c r="I84" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J84" s="11" t="n">
-        <v>229</v>
-      </c>
-      <c r="K84" s="12" t="n">
-        <v>11.45454545454546</v>
+      <c r="G84" s="7" t="n">
+        <v>522</v>
+      </c>
+      <c r="H84" s="6" t="inlineStr">
+        <is>
+          <t>12/20</t>
+        </is>
+      </c>
+      <c r="I84" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J84" s="7" t="n">
+        <v>870</v>
+      </c>
+      <c r="K84" s="8" t="n">
+        <v>43.5</v>
       </c>
     </row>
     <row r="85">
@@ -4781,11 +4769,11 @@
         </is>
       </c>
       <c r="G87" s="4" t="n">
-        <v>52347</v>
+        <v>55635</v>
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
-          <t>11/19</t>
+          <t>12/19</t>
         </is>
       </c>
       <c r="I87" s="3" t="inlineStr">
@@ -4794,10 +4782,10 @@
         </is>
       </c>
       <c r="J87" s="4" t="n">
-        <v>90418</v>
+        <v>88089</v>
       </c>
       <c r="K87" s="5" t="n">
-        <v>4758.818181818182</v>
+        <v>4636.25</v>
       </c>
     </row>
     <row r="88">
@@ -4977,11 +4965,11 @@
         </is>
       </c>
       <c r="G91" s="7" t="n">
-        <v>11842</v>
+        <v>12848</v>
       </c>
       <c r="H91" s="6" t="inlineStr">
         <is>
-          <t>11/17</t>
+          <t>12/17</t>
         </is>
       </c>
       <c r="I91" s="6" t="inlineStr">
@@ -4990,10 +4978,10 @@
         </is>
       </c>
       <c r="J91" s="7" t="n">
-        <v>18301</v>
+        <v>18201</v>
       </c>
       <c r="K91" s="8" t="n">
-        <v>1076.545454545455</v>
+        <v>1070.666666666667</v>
       </c>
     </row>
     <row r="92">
@@ -5222,11 +5210,11 @@
         </is>
       </c>
       <c r="G96" s="7" t="n">
-        <v>8735</v>
+        <v>8837</v>
       </c>
       <c r="H96" s="6" t="inlineStr">
         <is>
-          <t>14/22</t>
+          <t>15/22</t>
         </is>
       </c>
       <c r="I96" s="6" t="inlineStr">
@@ -5235,10 +5223,10 @@
         </is>
       </c>
       <c r="J96" s="7" t="n">
-        <v>13726</v>
+        <v>12961</v>
       </c>
       <c r="K96" s="8" t="n">
-        <v>623.9285714285714</v>
+        <v>589.1333333333334</v>
       </c>
     </row>
     <row r="97">
@@ -5320,11 +5308,11 @@
         </is>
       </c>
       <c r="G98" s="7" t="n">
-        <v>5857</v>
+        <v>4341</v>
       </c>
       <c r="H98" s="6" t="inlineStr">
         <is>
-          <t>13/25</t>
+          <t>14/25</t>
         </is>
       </c>
       <c r="I98" s="6" t="inlineStr">
@@ -5333,10 +5321,10 @@
         </is>
       </c>
       <c r="J98" s="7" t="n">
-        <v>11263</v>
+        <v>7752</v>
       </c>
       <c r="K98" s="8" t="n">
-        <v>450.5384615384615</v>
+        <v>310.0714285714286</v>
       </c>
     </row>
     <row r="99">
@@ -5369,11 +5357,11 @@
         </is>
       </c>
       <c r="G99" s="7" t="n">
-        <v>2760</v>
+        <v>3165</v>
       </c>
       <c r="H99" s="6" t="inlineStr">
         <is>
-          <t>11/22</t>
+          <t>12/22</t>
         </is>
       </c>
       <c r="I99" s="6" t="inlineStr">
@@ -5382,10 +5370,10 @@
         </is>
       </c>
       <c r="J99" s="7" t="n">
-        <v>5520</v>
+        <v>5802</v>
       </c>
       <c r="K99" s="8" t="n">
-        <v>250.9090909090909</v>
+        <v>263.75</v>
       </c>
     </row>
     <row r="100">
@@ -5467,11 +5455,11 @@
         </is>
       </c>
       <c r="G101" s="7" t="n">
-        <v>2014</v>
+        <v>2697</v>
       </c>
       <c r="H101" s="6" t="inlineStr">
         <is>
-          <t>15/21</t>
+          <t>16/21</t>
         </is>
       </c>
       <c r="I101" s="6" t="inlineStr">
@@ -5480,10 +5468,10 @@
         </is>
       </c>
       <c r="J101" s="7" t="n">
-        <v>2820</v>
+        <v>3540</v>
       </c>
       <c r="K101" s="8" t="n">
-        <v>134.2666666666667</v>
+        <v>168.5625</v>
       </c>
     </row>
     <row r="102">
@@ -5654,20 +5642,20 @@
       </c>
       <c r="E105" s="6" t="inlineStr">
         <is>
-          <t>S.PANDI</t>
+          <t>MALARVIZHI. B</t>
         </is>
       </c>
       <c r="F105" s="6" t="inlineStr">
         <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
+          <t>Tamilaga Vettri Kazhagam</t>
         </is>
       </c>
       <c r="G105" s="7" t="n">
-        <v>5468</v>
+        <v>6999</v>
       </c>
       <c r="H105" s="6" t="inlineStr">
         <is>
-          <t>13/30</t>
+          <t>14/30</t>
         </is>
       </c>
       <c r="I105" s="6" t="inlineStr">
@@ -5676,10 +5664,10 @@
         </is>
       </c>
       <c r="J105" s="7" t="n">
-        <v>12618</v>
+        <v>14998</v>
       </c>
       <c r="K105" s="8" t="n">
-        <v>420.6153846153846</v>
+        <v>499.9285714285714</v>
       </c>
     </row>
     <row r="106">
@@ -6006,11 +5994,11 @@
         </is>
       </c>
       <c r="G112" s="4" t="n">
-        <v>22162</v>
+        <v>23555</v>
       </c>
       <c r="H112" s="3" t="inlineStr">
         <is>
-          <t>12/25</t>
+          <t>13/25</t>
         </is>
       </c>
       <c r="I112" s="3" t="inlineStr">
@@ -6019,10 +6007,10 @@
         </is>
       </c>
       <c r="J112" s="4" t="n">
-        <v>46171</v>
+        <v>45298</v>
       </c>
       <c r="K112" s="5" t="n">
-        <v>1846.833333333333</v>
+        <v>1811.923076923077</v>
       </c>
     </row>
     <row r="113">
@@ -6075,52 +6063,52 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="2" t="inlineStr">
+      <c r="A114" s="6" t="inlineStr">
         <is>
           <t>NEYVELI</t>
         </is>
       </c>
-      <c r="B114" s="3" t="n">
+      <c r="B114" s="6" t="n">
         <v>153</v>
       </c>
-      <c r="C114" s="3" t="inlineStr">
+      <c r="C114" s="6" t="inlineStr">
         <is>
           <t>RAJENDRAN.R</t>
         </is>
       </c>
-      <c r="D114" s="3" t="inlineStr">
+      <c r="D114" s="6" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E114" s="3" t="inlineStr">
+      <c r="E114" s="6" t="inlineStr">
         <is>
           <t>SABA.RAJENDRAN</t>
         </is>
       </c>
-      <c r="F114" s="3" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G114" s="4" t="n">
-        <v>14714</v>
-      </c>
-      <c r="H114" s="3" t="inlineStr">
-        <is>
-          <t>12/19</t>
-        </is>
-      </c>
-      <c r="I114" s="3" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J114" s="4" t="n">
-        <v>23297</v>
-      </c>
-      <c r="K114" s="5" t="n">
-        <v>1226.166666666667</v>
+      <c r="F114" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G114" s="7" t="n">
+        <v>13103</v>
+      </c>
+      <c r="H114" s="6" t="inlineStr">
+        <is>
+          <t>13/19</t>
+        </is>
+      </c>
+      <c r="I114" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J114" s="7" t="n">
+        <v>19151</v>
+      </c>
+      <c r="K114" s="8" t="n">
+        <v>1007.923076923077</v>
       </c>
     </row>
     <row r="115">
@@ -6153,11 +6141,11 @@
         </is>
       </c>
       <c r="G115" s="7" t="n">
-        <v>3093</v>
+        <v>2747</v>
       </c>
       <c r="H115" s="6" t="inlineStr">
         <is>
-          <t>7/23</t>
+          <t>8/23</t>
         </is>
       </c>
       <c r="I115" s="6" t="inlineStr">
@@ -6166,10 +6154,10 @@
         </is>
       </c>
       <c r="J115" s="7" t="n">
-        <v>10163</v>
+        <v>7898</v>
       </c>
       <c r="K115" s="8" t="n">
-        <v>441.8571428571428</v>
+        <v>343.375</v>
       </c>
     </row>
     <row r="116">
@@ -6251,11 +6239,11 @@
         </is>
       </c>
       <c r="G117" s="7" t="n">
-        <v>3791</v>
+        <v>4491</v>
       </c>
       <c r="H117" s="6" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>11/26</t>
         </is>
       </c>
       <c r="I117" s="6" t="inlineStr">
@@ -6264,10 +6252,10 @@
         </is>
       </c>
       <c r="J117" s="7" t="n">
-        <v>9857</v>
+        <v>10615</v>
       </c>
       <c r="K117" s="8" t="n">
-        <v>379.1</v>
+        <v>408.2727272727273</v>
       </c>
     </row>
     <row r="118">
@@ -6477,30 +6465,30 @@
       </c>
       <c r="C122" s="10" t="inlineStr">
         <is>
-          <t>PANDI. N</t>
+          <t>RAVIMANOHARAN. K</t>
         </is>
       </c>
       <c r="D122" s="10" t="inlineStr">
         <is>
-          <t>Communist Party of India (Marxist)</t>
+          <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
       <c r="E122" s="10" t="inlineStr">
         <is>
-          <t>RAVIMANOHARAN. K</t>
+          <t>DR. PRAVEEN KUMAR. M</t>
         </is>
       </c>
       <c r="F122" s="10" t="inlineStr">
         <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
+          <t>Tamilaga Vettri Kazhagam</t>
         </is>
       </c>
       <c r="G122" s="11" t="n">
-        <v>168</v>
+        <v>342</v>
       </c>
       <c r="H122" s="10" t="inlineStr">
         <is>
-          <t>10/25</t>
+          <t>11/25</t>
         </is>
       </c>
       <c r="I122" s="10" t="inlineStr">
@@ -6509,10 +6497,10 @@
         </is>
       </c>
       <c r="J122" s="11" t="n">
-        <v>420</v>
+        <v>777</v>
       </c>
       <c r="K122" s="12" t="n">
-        <v>16.8</v>
+        <v>31.09090909090909</v>
       </c>
     </row>
     <row r="123">
@@ -6594,11 +6582,11 @@
         </is>
       </c>
       <c r="G124" s="4" t="n">
-        <v>12177</v>
+        <v>13002</v>
       </c>
       <c r="H124" s="3" t="inlineStr">
         <is>
-          <t>11/35</t>
+          <t>12/35</t>
         </is>
       </c>
       <c r="I124" s="3" t="inlineStr">
@@ -6607,10 +6595,10 @@
         </is>
       </c>
       <c r="J124" s="4" t="n">
-        <v>38745</v>
+        <v>37922</v>
       </c>
       <c r="K124" s="5" t="n">
-        <v>1107</v>
+        <v>1083.5</v>
       </c>
     </row>
     <row r="125">
@@ -6643,11 +6631,11 @@
         </is>
       </c>
       <c r="G125" s="4" t="n">
-        <v>17640</v>
+        <v>18500</v>
       </c>
       <c r="H125" s="3" t="inlineStr">
         <is>
-          <t>10/34</t>
+          <t>11/34</t>
         </is>
       </c>
       <c r="I125" s="3" t="inlineStr">
@@ -6656,59 +6644,59 @@
         </is>
       </c>
       <c r="J125" s="4" t="n">
-        <v>59976</v>
+        <v>57182</v>
       </c>
       <c r="K125" s="5" t="n">
-        <v>1764</v>
+        <v>1681.818181818182</v>
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="13" t="inlineStr">
+      <c r="A126" s="6" t="inlineStr">
         <is>
           <t>PANRUTI</t>
         </is>
       </c>
-      <c r="B126" s="14" t="n">
+      <c r="B126" s="6" t="n">
         <v>154</v>
       </c>
-      <c r="C126" s="14" t="inlineStr">
+      <c r="C126" s="6" t="inlineStr">
+        <is>
+          <t>MOHAN. K</t>
+        </is>
+      </c>
+      <c r="D126" s="6" t="inlineStr">
+        <is>
+          <t>All India Anna Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E126" s="6" t="inlineStr">
         <is>
           <t>ABDUR RAHMAN. A.R</t>
         </is>
       </c>
-      <c r="D126" s="14" t="inlineStr">
+      <c r="F126" s="6" t="inlineStr">
         <is>
           <t>Viduthalai Chiruthaigal Katchi</t>
         </is>
       </c>
-      <c r="E126" s="14" t="inlineStr">
-        <is>
-          <t>MOHAN. K</t>
-        </is>
-      </c>
-      <c r="F126" s="14" t="inlineStr">
-        <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G126" s="15" t="n">
-        <v>71</v>
-      </c>
-      <c r="H126" s="14" t="inlineStr">
-        <is>
-          <t>11/23</t>
-        </is>
-      </c>
-      <c r="I126" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J126" s="15" t="n">
-        <v>148</v>
-      </c>
-      <c r="K126" s="16" t="n">
-        <v>6.454545454545454</v>
+      <c r="G126" s="7" t="n">
+        <v>2203</v>
+      </c>
+      <c r="H126" s="6" t="inlineStr">
+        <is>
+          <t>12/23</t>
+        </is>
+      </c>
+      <c r="I126" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J126" s="7" t="n">
+        <v>4222</v>
+      </c>
+      <c r="K126" s="8" t="n">
+        <v>183.5833333333333</v>
       </c>
     </row>
     <row r="127">
@@ -6732,20 +6720,20 @@
       </c>
       <c r="E127" s="6" t="inlineStr">
         <is>
-          <t>AZARUDEEN UDUMAN ALI</t>
+          <t>A.M. SHAHJAHAN</t>
         </is>
       </c>
       <c r="F127" s="6" t="inlineStr">
         <is>
-          <t>Tamilaga Vettri Kazhagam</t>
+          <t>Indian Union Muslim League</t>
         </is>
       </c>
       <c r="G127" s="7" t="n">
-        <v>2723</v>
+        <v>1487</v>
       </c>
       <c r="H127" s="6" t="inlineStr">
         <is>
-          <t>6/23</t>
+          <t>7/23</t>
         </is>
       </c>
       <c r="I127" s="6" t="inlineStr">
@@ -6754,10 +6742,10 @@
         </is>
       </c>
       <c r="J127" s="7" t="n">
-        <v>10438</v>
+        <v>4886</v>
       </c>
       <c r="K127" s="8" t="n">
-        <v>453.8333333333333</v>
+        <v>212.4285714285714</v>
       </c>
     </row>
     <row r="128">
@@ -6781,20 +6769,20 @@
       </c>
       <c r="E128" s="3" t="inlineStr">
         <is>
-          <t>THILAGAVATHI. S</t>
+          <t>PALANIAPPAN. P</t>
         </is>
       </c>
       <c r="F128" s="3" t="inlineStr">
         <is>
-          <t>Tamilaga Vettri Kazhagam</t>
+          <t>Dravida Munnetra Kazhagam</t>
         </is>
       </c>
       <c r="G128" s="4" t="n">
-        <v>31690</v>
+        <v>30604</v>
       </c>
       <c r="H128" s="3" t="inlineStr">
         <is>
-          <t>12/23</t>
+          <t>13/23</t>
         </is>
       </c>
       <c r="I128" s="3" t="inlineStr">
@@ -6803,10 +6791,10 @@
         </is>
       </c>
       <c r="J128" s="4" t="n">
-        <v>60739</v>
+        <v>54146</v>
       </c>
       <c r="K128" s="5" t="n">
-        <v>2640.833333333333</v>
+        <v>2354.153846153847</v>
       </c>
     </row>
     <row r="129">
@@ -6888,11 +6876,11 @@
         </is>
       </c>
       <c r="G130" s="7" t="n">
-        <v>787</v>
+        <v>1323</v>
       </c>
       <c r="H130" s="6" t="inlineStr">
         <is>
-          <t>7/20</t>
+          <t>8/20</t>
         </is>
       </c>
       <c r="I130" s="6" t="inlineStr">
@@ -6901,10 +6889,10 @@
         </is>
       </c>
       <c r="J130" s="7" t="n">
-        <v>2249</v>
+        <v>3308</v>
       </c>
       <c r="K130" s="8" t="n">
-        <v>112.4285714285714</v>
+        <v>165.375</v>
       </c>
     </row>
     <row r="131">
@@ -6937,11 +6925,11 @@
         </is>
       </c>
       <c r="G131" s="7" t="n">
-        <v>2729</v>
+        <v>2919</v>
       </c>
       <c r="H131" s="6" t="inlineStr">
         <is>
-          <t>7/23</t>
+          <t>8/23</t>
         </is>
       </c>
       <c r="I131" s="6" t="inlineStr">
@@ -6950,10 +6938,10 @@
         </is>
       </c>
       <c r="J131" s="7" t="n">
-        <v>8967</v>
+        <v>8392</v>
       </c>
       <c r="K131" s="8" t="n">
-        <v>389.8571428571428</v>
+        <v>364.875</v>
       </c>
     </row>
     <row r="132">
@@ -6986,11 +6974,11 @@
         </is>
       </c>
       <c r="G132" s="7" t="n">
-        <v>2953</v>
+        <v>3612</v>
       </c>
       <c r="H132" s="6" t="inlineStr">
         <is>
-          <t>4/23</t>
+          <t>5/23</t>
         </is>
       </c>
       <c r="I132" s="6" t="inlineStr">
@@ -6999,10 +6987,10 @@
         </is>
       </c>
       <c r="J132" s="7" t="n">
-        <v>16980</v>
+        <v>16615</v>
       </c>
       <c r="K132" s="8" t="n">
-        <v>738.25</v>
+        <v>722.4</v>
       </c>
     </row>
     <row r="133">
@@ -7035,11 +7023,11 @@
         </is>
       </c>
       <c r="G133" s="7" t="n">
-        <v>3323</v>
+        <v>4432</v>
       </c>
       <c r="H133" s="6" t="inlineStr">
         <is>
-          <t>13/28</t>
+          <t>14/28</t>
         </is>
       </c>
       <c r="I133" s="6" t="inlineStr">
@@ -7048,10 +7036,10 @@
         </is>
       </c>
       <c r="J133" s="7" t="n">
-        <v>7157</v>
+        <v>8864</v>
       </c>
       <c r="K133" s="8" t="n">
-        <v>255.6153846153846</v>
+        <v>316.5714285714286</v>
       </c>
     </row>
     <row r="134">
@@ -7084,11 +7072,11 @@
         </is>
       </c>
       <c r="G134" s="4" t="n">
-        <v>16452</v>
+        <v>19100</v>
       </c>
       <c r="H134" s="3" t="inlineStr">
         <is>
-          <t>7/22</t>
+          <t>8/22</t>
         </is>
       </c>
       <c r="I134" s="3" t="inlineStr">
@@ -7097,10 +7085,10 @@
         </is>
       </c>
       <c r="J134" s="4" t="n">
-        <v>51706</v>
+        <v>52525</v>
       </c>
       <c r="K134" s="5" t="n">
-        <v>2350.285714285714</v>
+        <v>2387.5</v>
       </c>
     </row>
     <row r="135">
@@ -7182,11 +7170,11 @@
         </is>
       </c>
       <c r="G136" s="7" t="n">
-        <v>2323</v>
+        <v>2241</v>
       </c>
       <c r="H136" s="6" t="inlineStr">
         <is>
-          <t>7/26</t>
+          <t>8/26</t>
         </is>
       </c>
       <c r="I136" s="6" t="inlineStr">
@@ -7195,10 +7183,10 @@
         </is>
       </c>
       <c r="J136" s="7" t="n">
-        <v>8628</v>
+        <v>7283</v>
       </c>
       <c r="K136" s="8" t="n">
-        <v>331.8571428571428</v>
+        <v>280.125</v>
       </c>
     </row>
     <row r="137">
@@ -7476,11 +7464,11 @@
         </is>
       </c>
       <c r="G142" s="4" t="n">
-        <v>33975</v>
+        <v>37823</v>
       </c>
       <c r="H142" s="3" t="inlineStr">
         <is>
-          <t>10/23</t>
+          <t>11/23</t>
         </is>
       </c>
       <c r="I142" s="3" t="inlineStr">
@@ -7489,10 +7477,10 @@
         </is>
       </c>
       <c r="J142" s="4" t="n">
-        <v>78142</v>
+        <v>79084</v>
       </c>
       <c r="K142" s="5" t="n">
-        <v>3397.5</v>
+        <v>3438.454545454545</v>
       </c>
     </row>
     <row r="143">
@@ -7574,11 +7562,11 @@
         </is>
       </c>
       <c r="G144" s="7" t="n">
-        <v>5451</v>
+        <v>6824</v>
       </c>
       <c r="H144" s="6" t="inlineStr">
         <is>
-          <t>16/24</t>
+          <t>17/24</t>
         </is>
       </c>
       <c r="I144" s="6" t="inlineStr">
@@ -7587,10 +7575,10 @@
         </is>
       </c>
       <c r="J144" s="7" t="n">
-        <v>8176</v>
+        <v>9634</v>
       </c>
       <c r="K144" s="8" t="n">
-        <v>340.6875</v>
+        <v>401.4117647058824</v>
       </c>
     </row>
     <row r="145">
@@ -7770,11 +7758,11 @@
         </is>
       </c>
       <c r="G148" s="7" t="n">
-        <v>8168</v>
+        <v>8970</v>
       </c>
       <c r="H148" s="6" t="inlineStr">
         <is>
-          <t>10/21</t>
+          <t>11/21</t>
         </is>
       </c>
       <c r="I148" s="6" t="inlineStr">
@@ -7783,10 +7771,10 @@
         </is>
       </c>
       <c r="J148" s="7" t="n">
-        <v>17153</v>
+        <v>17125</v>
       </c>
       <c r="K148" s="8" t="n">
-        <v>816.8</v>
+        <v>815.4545454545455</v>
       </c>
     </row>
     <row r="149">
@@ -7917,11 +7905,11 @@
         </is>
       </c>
       <c r="G151" s="4" t="n">
-        <v>13349</v>
+        <v>15009</v>
       </c>
       <c r="H151" s="3" t="inlineStr">
         <is>
-          <t>8/21</t>
+          <t>9/21</t>
         </is>
       </c>
       <c r="I151" s="3" t="inlineStr">
@@ -7930,10 +7918,10 @@
         </is>
       </c>
       <c r="J151" s="4" t="n">
-        <v>35041</v>
+        <v>35021</v>
       </c>
       <c r="K151" s="5" t="n">
-        <v>1668.625</v>
+        <v>1667.666666666667</v>
       </c>
     </row>
     <row r="152">
@@ -8113,11 +8101,11 @@
         </is>
       </c>
       <c r="G155" s="7" t="n">
-        <v>2886</v>
+        <v>3035</v>
       </c>
       <c r="H155" s="6" t="inlineStr">
         <is>
-          <t>11/23</t>
+          <t>12/23</t>
         </is>
       </c>
       <c r="I155" s="6" t="inlineStr">
@@ -8126,10 +8114,10 @@
         </is>
       </c>
       <c r="J155" s="7" t="n">
-        <v>6034</v>
+        <v>5817</v>
       </c>
       <c r="K155" s="8" t="n">
-        <v>262.3636363636364</v>
+        <v>252.9166666666667</v>
       </c>
     </row>
     <row r="156">
@@ -8182,52 +8170,52 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="9" t="inlineStr">
+      <c r="A157" s="6" t="inlineStr">
         <is>
           <t>SANKARI</t>
         </is>
       </c>
-      <c r="B157" s="10" t="n">
+      <c r="B157" s="6" t="n">
         <v>87</v>
       </c>
-      <c r="C157" s="10" t="inlineStr">
+      <c r="C157" s="6" t="inlineStr">
+        <is>
+          <t>VETRIVEL. S</t>
+        </is>
+      </c>
+      <c r="D157" s="6" t="inlineStr">
+        <is>
+          <t>All India Anna Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E157" s="6" t="inlineStr">
         <is>
           <t>SENTHILKUMAR. K</t>
         </is>
       </c>
-      <c r="D157" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E157" s="10" t="inlineStr">
-        <is>
-          <t>VETRIVEL. S</t>
-        </is>
-      </c>
-      <c r="F157" s="10" t="inlineStr">
-        <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G157" s="11" t="n">
-        <v>350</v>
-      </c>
-      <c r="H157" s="10" t="inlineStr">
-        <is>
-          <t>11/25</t>
-        </is>
-      </c>
-      <c r="I157" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J157" s="11" t="n">
-        <v>795</v>
-      </c>
-      <c r="K157" s="12" t="n">
-        <v>31.81818181818182</v>
+      <c r="F157" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G157" s="7" t="n">
+        <v>812</v>
+      </c>
+      <c r="H157" s="6" t="inlineStr">
+        <is>
+          <t>12/25</t>
+        </is>
+      </c>
+      <c r="I157" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J157" s="7" t="n">
+        <v>1692</v>
+      </c>
+      <c r="K157" s="8" t="n">
+        <v>67.66666666666667</v>
       </c>
     </row>
     <row r="158">
@@ -8309,11 +8297,11 @@
         </is>
       </c>
       <c r="G159" s="7" t="n">
-        <v>2801</v>
+        <v>2779</v>
       </c>
       <c r="H159" s="6" t="inlineStr">
         <is>
-          <t>10/22</t>
+          <t>11/22</t>
         </is>
       </c>
       <c r="I159" s="6" t="inlineStr">
@@ -8322,10 +8310,10 @@
         </is>
       </c>
       <c r="J159" s="7" t="n">
-        <v>6162</v>
+        <v>5558</v>
       </c>
       <c r="K159" s="8" t="n">
-        <v>280.1</v>
+        <v>252.6363636363636</v>
       </c>
     </row>
     <row r="160">
@@ -8407,11 +8395,11 @@
         </is>
       </c>
       <c r="G161" s="7" t="n">
-        <v>2351</v>
+        <v>3838</v>
       </c>
       <c r="H161" s="6" t="inlineStr">
         <is>
-          <t>6/25</t>
+          <t>7/25</t>
         </is>
       </c>
       <c r="I161" s="6" t="inlineStr">
@@ -8420,10 +8408,10 @@
         </is>
       </c>
       <c r="J161" s="7" t="n">
-        <v>9796</v>
+        <v>13707</v>
       </c>
       <c r="K161" s="8" t="n">
-        <v>391.8333333333333</v>
+        <v>548.2857142857142</v>
       </c>
     </row>
     <row r="162">
@@ -8456,11 +8444,11 @@
         </is>
       </c>
       <c r="G162" s="4" t="n">
-        <v>16600</v>
+        <v>20229</v>
       </c>
       <c r="H162" s="3" t="inlineStr">
         <is>
-          <t>6/30</t>
+          <t>7/30</t>
         </is>
       </c>
       <c r="I162" s="3" t="inlineStr">
@@ -8469,10 +8457,10 @@
         </is>
       </c>
       <c r="J162" s="4" t="n">
-        <v>83000</v>
+        <v>86696</v>
       </c>
       <c r="K162" s="5" t="n">
-        <v>2766.666666666667</v>
+        <v>2889.857142857143</v>
       </c>
     </row>
     <row r="163">
@@ -8505,11 +8493,11 @@
         </is>
       </c>
       <c r="G163" s="4" t="n">
-        <v>10152</v>
+        <v>11164</v>
       </c>
       <c r="H163" s="3" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>11/26</t>
         </is>
       </c>
       <c r="I163" s="3" t="inlineStr">
@@ -8518,10 +8506,10 @@
         </is>
       </c>
       <c r="J163" s="4" t="n">
-        <v>26395</v>
+        <v>26388</v>
       </c>
       <c r="K163" s="5" t="n">
-        <v>1015.2</v>
+        <v>1014.909090909091</v>
       </c>
     </row>
     <row r="164">
@@ -8545,20 +8533,20 @@
       </c>
       <c r="E164" s="6" t="inlineStr">
         <is>
-          <t>SAKTHI.M</t>
+          <t>GOPINATH.S</t>
         </is>
       </c>
       <c r="F164" s="6" t="inlineStr">
         <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
+          <t>Tamilaga Vettri Kazhagam</t>
         </is>
       </c>
       <c r="G164" s="7" t="n">
-        <v>6120</v>
+        <v>6941</v>
       </c>
       <c r="H164" s="6" t="inlineStr">
         <is>
-          <t>12/22</t>
+          <t>13/22</t>
         </is>
       </c>
       <c r="I164" s="6" t="inlineStr">
@@ -8567,10 +8555,10 @@
         </is>
       </c>
       <c r="J164" s="7" t="n">
-        <v>11220</v>
+        <v>11746</v>
       </c>
       <c r="K164" s="8" t="n">
-        <v>510</v>
+        <v>533.9230769230769</v>
       </c>
     </row>
     <row r="165">
@@ -8603,11 +8591,11 @@
         </is>
       </c>
       <c r="G165" s="7" t="n">
-        <v>4674</v>
+        <v>5936</v>
       </c>
       <c r="H165" s="6" t="inlineStr">
         <is>
-          <t>9/29</t>
+          <t>10/29</t>
         </is>
       </c>
       <c r="I165" s="6" t="inlineStr">
@@ -8616,10 +8604,10 @@
         </is>
       </c>
       <c r="J165" s="7" t="n">
-        <v>15061</v>
+        <v>17214</v>
       </c>
       <c r="K165" s="8" t="n">
-        <v>519.3333333333334</v>
+        <v>593.6</v>
       </c>
     </row>
     <row r="166">
@@ -8701,11 +8689,11 @@
         </is>
       </c>
       <c r="G167" s="4" t="n">
-        <v>19015</v>
+        <v>20017</v>
       </c>
       <c r="H167" s="3" t="inlineStr">
         <is>
-          <t>11/32</t>
+          <t>12/32</t>
         </is>
       </c>
       <c r="I167" s="3" t="inlineStr">
@@ -8714,10 +8702,10 @@
         </is>
       </c>
       <c r="J167" s="4" t="n">
-        <v>55316</v>
+        <v>53379</v>
       </c>
       <c r="K167" s="5" t="n">
-        <v>1728.636363636364</v>
+        <v>1668.083333333333</v>
       </c>
     </row>
     <row r="168">
@@ -8741,20 +8729,20 @@
       </c>
       <c r="E168" s="3" t="inlineStr">
         <is>
-          <t>S. DURAIRAJ</t>
+          <t>R.MANOHARAN</t>
         </is>
       </c>
       <c r="F168" s="3" t="inlineStr">
         <is>
-          <t>Dravida Munnetra Kazhagam</t>
+          <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
       <c r="G168" s="4" t="n">
-        <v>7231</v>
+        <v>7341</v>
       </c>
       <c r="H168" s="3" t="inlineStr">
         <is>
-          <t>6/27</t>
+          <t>7/27</t>
         </is>
       </c>
       <c r="I168" s="3" t="inlineStr">
@@ -8763,10 +8751,10 @@
         </is>
       </c>
       <c r="J168" s="4" t="n">
-        <v>32540</v>
+        <v>28315</v>
       </c>
       <c r="K168" s="5" t="n">
-        <v>1205.166666666667</v>
+        <v>1048.714285714286</v>
       </c>
     </row>
     <row r="169">
@@ -8897,11 +8885,11 @@
         </is>
       </c>
       <c r="G171" s="7" t="n">
-        <v>3107</v>
+        <v>3603</v>
       </c>
       <c r="H171" s="6" t="inlineStr">
         <is>
-          <t>8/28</t>
+          <t>9/28</t>
         </is>
       </c>
       <c r="I171" s="6" t="inlineStr">
@@ -8910,10 +8898,10 @@
         </is>
       </c>
       <c r="J171" s="7" t="n">
-        <v>10874</v>
+        <v>11209</v>
       </c>
       <c r="K171" s="8" t="n">
-        <v>388.375</v>
+        <v>400.3333333333333</v>
       </c>
     </row>
     <row r="172">
@@ -8946,11 +8934,11 @@
         </is>
       </c>
       <c r="G172" s="4" t="n">
-        <v>15074</v>
+        <v>15769</v>
       </c>
       <c r="H172" s="3" t="inlineStr">
         <is>
-          <t>17/34</t>
+          <t>18/34</t>
         </is>
       </c>
       <c r="I172" s="3" t="inlineStr">
@@ -8959,10 +8947,10 @@
         </is>
       </c>
       <c r="J172" s="4" t="n">
-        <v>30148</v>
+        <v>29786</v>
       </c>
       <c r="K172" s="5" t="n">
-        <v>886.7058823529412</v>
+        <v>876.0555555555555</v>
       </c>
     </row>
     <row r="173">
@@ -9093,11 +9081,11 @@
         </is>
       </c>
       <c r="G175" s="4" t="n">
-        <v>16286</v>
+        <v>17155</v>
       </c>
       <c r="H175" s="3" t="inlineStr">
         <is>
-          <t>18/23</t>
+          <t>19/23</t>
         </is>
       </c>
       <c r="I175" s="3" t="inlineStr">
@@ -9106,10 +9094,10 @@
         </is>
       </c>
       <c r="J175" s="4" t="n">
-        <v>20810</v>
+        <v>20767</v>
       </c>
       <c r="K175" s="5" t="n">
-        <v>904.7777777777778</v>
+        <v>902.8947368421053</v>
       </c>
     </row>
     <row r="176">
@@ -9191,11 +9179,11 @@
         </is>
       </c>
       <c r="G177" s="7" t="n">
-        <v>7083</v>
+        <v>7965</v>
       </c>
       <c r="H177" s="6" t="inlineStr">
         <is>
-          <t>13/26</t>
+          <t>14/26</t>
         </is>
       </c>
       <c r="I177" s="6" t="inlineStr">
@@ -9204,10 +9192,10 @@
         </is>
       </c>
       <c r="J177" s="7" t="n">
-        <v>14166</v>
+        <v>14792</v>
       </c>
       <c r="K177" s="8" t="n">
-        <v>544.8461538461538</v>
+        <v>568.9285714285714</v>
       </c>
     </row>
     <row r="178">
@@ -9240,11 +9228,11 @@
         </is>
       </c>
       <c r="G178" s="7" t="n">
-        <v>1478</v>
+        <v>1774</v>
       </c>
       <c r="H178" s="6" t="inlineStr">
         <is>
-          <t>5/22</t>
+          <t>6/22</t>
         </is>
       </c>
       <c r="I178" s="6" t="inlineStr">
@@ -9253,10 +9241,10 @@
         </is>
       </c>
       <c r="J178" s="7" t="n">
-        <v>6503</v>
+        <v>6505</v>
       </c>
       <c r="K178" s="8" t="n">
-        <v>295.6</v>
+        <v>295.6666666666667</v>
       </c>
     </row>
     <row r="179">
@@ -9289,11 +9277,11 @@
         </is>
       </c>
       <c r="G179" s="4" t="n">
-        <v>9253</v>
+        <v>10722</v>
       </c>
       <c r="H179" s="3" t="inlineStr">
         <is>
-          <t>9/26</t>
+          <t>10/26</t>
         </is>
       </c>
       <c r="I179" s="3" t="inlineStr">
@@ -9302,10 +9290,10 @@
         </is>
       </c>
       <c r="J179" s="4" t="n">
-        <v>26731</v>
+        <v>27877</v>
       </c>
       <c r="K179" s="5" t="n">
-        <v>1028.111111111111</v>
+        <v>1072.2</v>
       </c>
     </row>
     <row r="180">
@@ -9338,11 +9326,11 @@
         </is>
       </c>
       <c r="G180" s="4" t="n">
-        <v>16053</v>
+        <v>18071</v>
       </c>
       <c r="H180" s="3" t="inlineStr">
         <is>
-          <t>8/29</t>
+          <t>9/29</t>
         </is>
       </c>
       <c r="I180" s="3" t="inlineStr">
@@ -9351,10 +9339,10 @@
         </is>
       </c>
       <c r="J180" s="4" t="n">
-        <v>58192</v>
+        <v>58229</v>
       </c>
       <c r="K180" s="5" t="n">
-        <v>2006.625</v>
+        <v>2007.888888888889</v>
       </c>
     </row>
     <row r="181">
@@ -9730,11 +9718,11 @@
         </is>
       </c>
       <c r="G188" s="7" t="n">
-        <v>8553</v>
+        <v>9148</v>
       </c>
       <c r="H188" s="6" t="inlineStr">
         <is>
-          <t>9/18</t>
+          <t>10/18</t>
         </is>
       </c>
       <c r="I188" s="6" t="inlineStr">
@@ -9743,10 +9731,10 @@
         </is>
       </c>
       <c r="J188" s="7" t="n">
-        <v>17106</v>
+        <v>16466</v>
       </c>
       <c r="K188" s="8" t="n">
-        <v>950.3333333333334</v>
+        <v>914.8</v>
       </c>
     </row>
     <row r="189">
@@ -9779,11 +9767,11 @@
         </is>
       </c>
       <c r="G189" s="4" t="n">
-        <v>14976</v>
+        <v>14946</v>
       </c>
       <c r="H189" s="3" t="inlineStr">
         <is>
-          <t>9/27</t>
+          <t>10/27</t>
         </is>
       </c>
       <c r="I189" s="3" t="inlineStr">
@@ -9792,10 +9780,10 @@
         </is>
       </c>
       <c r="J189" s="4" t="n">
-        <v>44928</v>
+        <v>40354</v>
       </c>
       <c r="K189" s="5" t="n">
-        <v>1664</v>
+        <v>1494.6</v>
       </c>
     </row>
     <row r="190">
@@ -9877,11 +9865,11 @@
         </is>
       </c>
       <c r="G191" s="7" t="n">
-        <v>3524</v>
+        <v>4146</v>
       </c>
       <c r="H191" s="6" t="inlineStr">
         <is>
-          <t>5/18</t>
+          <t>6/18</t>
         </is>
       </c>
       <c r="I191" s="6" t="inlineStr">
@@ -9890,10 +9878,10 @@
         </is>
       </c>
       <c r="J191" s="7" t="n">
-        <v>12686</v>
+        <v>12438</v>
       </c>
       <c r="K191" s="8" t="n">
-        <v>704.8</v>
+        <v>691</v>
       </c>
     </row>
     <row r="192">
@@ -9926,11 +9914,11 @@
         </is>
       </c>
       <c r="G192" s="7" t="n">
-        <v>3474</v>
+        <v>3801</v>
       </c>
       <c r="H192" s="6" t="inlineStr">
         <is>
-          <t>12/22</t>
+          <t>13/22</t>
         </is>
       </c>
       <c r="I192" s="6" t="inlineStr">
@@ -9939,10 +9927,10 @@
         </is>
       </c>
       <c r="J192" s="7" t="n">
-        <v>6369</v>
+        <v>6432</v>
       </c>
       <c r="K192" s="8" t="n">
-        <v>289.5</v>
+        <v>292.3846153846154</v>
       </c>
     </row>
     <row r="193">
@@ -10024,11 +10012,11 @@
         </is>
       </c>
       <c r="G194" s="7" t="n">
-        <v>8277</v>
+        <v>7578</v>
       </c>
       <c r="H194" s="6" t="inlineStr">
         <is>
-          <t>12/22</t>
+          <t>13/22</t>
         </is>
       </c>
       <c r="I194" s="6" t="inlineStr">
@@ -10037,10 +10025,10 @@
         </is>
       </c>
       <c r="J194" s="7" t="n">
-        <v>15174</v>
+        <v>12824</v>
       </c>
       <c r="K194" s="8" t="n">
-        <v>689.75</v>
+        <v>582.9230769230769</v>
       </c>
     </row>
     <row r="195">
@@ -10073,11 +10061,11 @@
         </is>
       </c>
       <c r="G195" s="7" t="n">
-        <v>2177</v>
+        <v>3839</v>
       </c>
       <c r="H195" s="6" t="inlineStr">
         <is>
-          <t>6/21</t>
+          <t>7/21</t>
         </is>
       </c>
       <c r="I195" s="6" t="inlineStr">
@@ -10086,10 +10074,10 @@
         </is>
       </c>
       <c r="J195" s="7" t="n">
-        <v>7620</v>
+        <v>11517</v>
       </c>
       <c r="K195" s="8" t="n">
-        <v>362.8333333333333</v>
+        <v>548.4285714285714</v>
       </c>
     </row>
     <row r="196">
@@ -10122,11 +10110,11 @@
         </is>
       </c>
       <c r="G196" s="4" t="n">
-        <v>12173</v>
+        <v>12015</v>
       </c>
       <c r="H196" s="3" t="inlineStr">
         <is>
-          <t>7/22</t>
+          <t>8/22</t>
         </is>
       </c>
       <c r="I196" s="3" t="inlineStr">
@@ -10135,10 +10123,10 @@
         </is>
       </c>
       <c r="J196" s="4" t="n">
-        <v>38258</v>
+        <v>33041</v>
       </c>
       <c r="K196" s="5" t="n">
-        <v>1739</v>
+        <v>1501.875</v>
       </c>
     </row>
     <row r="197">
@@ -10171,11 +10159,11 @@
         </is>
       </c>
       <c r="G197" s="4" t="n">
-        <v>5689</v>
+        <v>5286</v>
       </c>
       <c r="H197" s="3" t="inlineStr">
         <is>
-          <t>19/24</t>
+          <t>20/24</t>
         </is>
       </c>
       <c r="I197" s="3" t="inlineStr">
@@ -10184,10 +10172,10 @@
         </is>
       </c>
       <c r="J197" s="4" t="n">
-        <v>7186</v>
+        <v>6343</v>
       </c>
       <c r="K197" s="5" t="n">
-        <v>299.421052631579</v>
+        <v>264.3</v>
       </c>
     </row>
     <row r="198">
@@ -10220,11 +10208,11 @@
         </is>
       </c>
       <c r="G198" s="7" t="n">
-        <v>466</v>
+        <v>1019</v>
       </c>
       <c r="H198" s="6" t="inlineStr">
         <is>
-          <t>5/21</t>
+          <t>6/21</t>
         </is>
       </c>
       <c r="I198" s="6" t="inlineStr">
@@ -10233,10 +10221,10 @@
         </is>
       </c>
       <c r="J198" s="7" t="n">
-        <v>1957</v>
+        <v>3566</v>
       </c>
       <c r="K198" s="8" t="n">
-        <v>93.2</v>
+        <v>169.8333333333333</v>
       </c>
     </row>
     <row r="199">
@@ -10269,11 +10257,11 @@
         </is>
       </c>
       <c r="G199" s="7" t="n">
-        <v>1438</v>
+        <v>799</v>
       </c>
       <c r="H199" s="6" t="inlineStr">
         <is>
-          <t>8/24</t>
+          <t>9/24</t>
         </is>
       </c>
       <c r="I199" s="6" t="inlineStr">
@@ -10282,10 +10270,10 @@
         </is>
       </c>
       <c r="J199" s="7" t="n">
-        <v>4314</v>
+        <v>2131</v>
       </c>
       <c r="K199" s="8" t="n">
-        <v>179.75</v>
+        <v>88.77777777777777</v>
       </c>
     </row>
     <row r="200">
@@ -10318,11 +10306,11 @@
         </is>
       </c>
       <c r="G200" s="7" t="n">
-        <v>4035</v>
+        <v>4782</v>
       </c>
       <c r="H200" s="6" t="inlineStr">
         <is>
-          <t>17/28</t>
+          <t>18/28</t>
         </is>
       </c>
       <c r="I200" s="6" t="inlineStr">
@@ -10331,10 +10319,10 @@
         </is>
       </c>
       <c r="J200" s="7" t="n">
-        <v>6646</v>
+        <v>7439</v>
       </c>
       <c r="K200" s="8" t="n">
-        <v>237.3529411764706</v>
+        <v>265.6666666666667</v>
       </c>
     </row>
     <row r="201">
@@ -10416,11 +10404,11 @@
         </is>
       </c>
       <c r="G202" s="7" t="n">
-        <v>3459</v>
+        <v>4531</v>
       </c>
       <c r="H202" s="6" t="inlineStr">
         <is>
-          <t>7/27</t>
+          <t>8/27</t>
         </is>
       </c>
       <c r="I202" s="6" t="inlineStr">
@@ -10429,10 +10417,10 @@
         </is>
       </c>
       <c r="J202" s="7" t="n">
-        <v>13342</v>
+        <v>15292</v>
       </c>
       <c r="K202" s="8" t="n">
-        <v>494.1428571428572</v>
+        <v>566.375</v>
       </c>
     </row>
     <row r="203">
@@ -10465,11 +10453,11 @@
         </is>
       </c>
       <c r="G203" s="4" t="n">
-        <v>24414</v>
+        <v>28543</v>
       </c>
       <c r="H203" s="3" t="inlineStr">
         <is>
-          <t>11/32</t>
+          <t>12/32</t>
         </is>
       </c>
       <c r="I203" s="3" t="inlineStr">
@@ -10478,10 +10466,10 @@
         </is>
       </c>
       <c r="J203" s="4" t="n">
-        <v>71023</v>
+        <v>76115</v>
       </c>
       <c r="K203" s="5" t="n">
-        <v>2219.454545454545</v>
+        <v>2378.583333333333</v>
       </c>
     </row>
     <row r="204">
@@ -10563,11 +10551,11 @@
         </is>
       </c>
       <c r="G205" s="7" t="n">
-        <v>1575</v>
+        <v>3116</v>
       </c>
       <c r="H205" s="6" t="inlineStr">
         <is>
-          <t>7/25</t>
+          <t>8/25</t>
         </is>
       </c>
       <c r="I205" s="6" t="inlineStr">
@@ -10576,10 +10564,10 @@
         </is>
       </c>
       <c r="J205" s="7" t="n">
-        <v>5625</v>
+        <v>9738</v>
       </c>
       <c r="K205" s="8" t="n">
-        <v>225</v>
+        <v>389.5</v>
       </c>
     </row>
     <row r="206">
@@ -10593,30 +10581,30 @@
       </c>
       <c r="C206" s="10" t="inlineStr">
         <is>
+          <t>RAJEEV</t>
+        </is>
+      </c>
+      <c r="D206" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E206" s="10" t="inlineStr">
+        <is>
           <t>M.KEERTHIKA</t>
         </is>
       </c>
-      <c r="D206" s="10" t="inlineStr">
+      <c r="F206" s="10" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E206" s="10" t="inlineStr">
-        <is>
-          <t>RAJEEV</t>
-        </is>
-      </c>
-      <c r="F206" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
       <c r="G206" s="11" t="n">
-        <v>480</v>
+        <v>439</v>
       </c>
       <c r="H206" s="10" t="inlineStr">
         <is>
-          <t>13/27</t>
+          <t>15/27</t>
         </is>
       </c>
       <c r="I206" s="10" t="inlineStr">
@@ -10625,10 +10613,10 @@
         </is>
       </c>
       <c r="J206" s="11" t="n">
-        <v>997</v>
+        <v>790</v>
       </c>
       <c r="K206" s="12" t="n">
-        <v>36.92307692307692</v>
+        <v>29.26666666666667</v>
       </c>
     </row>
     <row r="207">
@@ -10759,11 +10747,11 @@
         </is>
       </c>
       <c r="G209" s="7" t="n">
-        <v>2835</v>
+        <v>2903</v>
       </c>
       <c r="H209" s="6" t="inlineStr">
         <is>
-          <t>13/19</t>
+          <t>14/19</t>
         </is>
       </c>
       <c r="I209" s="6" t="inlineStr">
@@ -10772,10 +10760,10 @@
         </is>
       </c>
       <c r="J209" s="7" t="n">
-        <v>4143</v>
+        <v>3940</v>
       </c>
       <c r="K209" s="8" t="n">
-        <v>218.0769230769231</v>
+        <v>207.3571428571429</v>
       </c>
     </row>
     <row r="210">
@@ -10906,11 +10894,11 @@
         </is>
       </c>
       <c r="G212" s="7" t="n">
-        <v>2718</v>
+        <v>2491</v>
       </c>
       <c r="H212" s="6" t="inlineStr">
         <is>
-          <t>7/25</t>
+          <t>8/25</t>
         </is>
       </c>
       <c r="I212" s="6" t="inlineStr">
@@ -10919,10 +10907,10 @@
         </is>
       </c>
       <c r="J212" s="7" t="n">
-        <v>9707</v>
+        <v>7784</v>
       </c>
       <c r="K212" s="8" t="n">
-        <v>388.2857142857142</v>
+        <v>311.375</v>
       </c>
     </row>
     <row r="213">
@@ -10955,11 +10943,11 @@
         </is>
       </c>
       <c r="G213" s="7" t="n">
-        <v>3912</v>
+        <v>4632</v>
       </c>
       <c r="H213" s="6" t="inlineStr">
         <is>
-          <t>13/23</t>
+          <t>14/23</t>
         </is>
       </c>
       <c r="I213" s="6" t="inlineStr">
@@ -10968,10 +10956,10 @@
         </is>
       </c>
       <c r="J213" s="7" t="n">
-        <v>6921</v>
+        <v>7610</v>
       </c>
       <c r="K213" s="8" t="n">
-        <v>300.923076923077</v>
+        <v>330.8571428571428</v>
       </c>
     </row>
     <row r="214">
@@ -11151,11 +11139,11 @@
         </is>
       </c>
       <c r="G217" s="7" t="n">
-        <v>10193</v>
+        <v>9614</v>
       </c>
       <c r="H217" s="6" t="inlineStr">
         <is>
-          <t>16/23</t>
+          <t>17/23</t>
         </is>
       </c>
       <c r="I217" s="6" t="inlineStr">
@@ -11164,10 +11152,10 @@
         </is>
       </c>
       <c r="J217" s="7" t="n">
-        <v>14652</v>
+        <v>13007</v>
       </c>
       <c r="K217" s="8" t="n">
-        <v>637.0625</v>
+        <v>565.5294117647059</v>
       </c>
     </row>
     <row r="218">
@@ -11200,11 +11188,11 @@
         </is>
       </c>
       <c r="G218" s="7" t="n">
-        <v>2149</v>
+        <v>2445</v>
       </c>
       <c r="H218" s="6" t="inlineStr">
         <is>
-          <t>8/22</t>
+          <t>9/22</t>
         </is>
       </c>
       <c r="I218" s="6" t="inlineStr">
@@ -11213,10 +11201,10 @@
         </is>
       </c>
       <c r="J218" s="7" t="n">
-        <v>5910</v>
+        <v>5977</v>
       </c>
       <c r="K218" s="8" t="n">
-        <v>268.625</v>
+        <v>271.6666666666667</v>
       </c>
     </row>
     <row r="219">
@@ -11249,11 +11237,11 @@
         </is>
       </c>
       <c r="G219" s="7" t="n">
-        <v>1749</v>
+        <v>5475</v>
       </c>
       <c r="H219" s="6" t="inlineStr">
         <is>
-          <t>10/23</t>
+          <t>11/23</t>
         </is>
       </c>
       <c r="I219" s="6" t="inlineStr">
@@ -11262,10 +11250,10 @@
         </is>
       </c>
       <c r="J219" s="7" t="n">
-        <v>4023</v>
+        <v>11448</v>
       </c>
       <c r="K219" s="8" t="n">
-        <v>174.9</v>
+        <v>497.7272727272727</v>
       </c>
     </row>
     <row r="220">
@@ -11298,11 +11286,11 @@
         </is>
       </c>
       <c r="G220" s="7" t="n">
-        <v>5916</v>
+        <v>6411</v>
       </c>
       <c r="H220" s="6" t="inlineStr">
         <is>
-          <t>8/18</t>
+          <t>9/18</t>
         </is>
       </c>
       <c r="I220" s="6" t="inlineStr">
@@ -11311,10 +11299,10 @@
         </is>
       </c>
       <c r="J220" s="7" t="n">
-        <v>13311</v>
+        <v>12822</v>
       </c>
       <c r="K220" s="8" t="n">
-        <v>739.5</v>
+        <v>712.3333333333334</v>
       </c>
     </row>
     <row r="221">
@@ -11396,11 +11384,11 @@
         </is>
       </c>
       <c r="G222" s="7" t="n">
-        <v>3588</v>
+        <v>2716</v>
       </c>
       <c r="H222" s="6" t="inlineStr">
         <is>
-          <t>10/23</t>
+          <t>11/23</t>
         </is>
       </c>
       <c r="I222" s="6" t="inlineStr">
@@ -11409,10 +11397,10 @@
         </is>
       </c>
       <c r="J222" s="7" t="n">
-        <v>8252</v>
+        <v>5679</v>
       </c>
       <c r="K222" s="8" t="n">
-        <v>358.8</v>
+        <v>246.9090909090909</v>
       </c>
     </row>
     <row r="223">
@@ -11436,20 +11424,20 @@
       </c>
       <c r="E223" s="3" t="inlineStr">
         <is>
-          <t>ASHOK. M.K</t>
+          <t>AASSAN MAULAANA J.M.H</t>
         </is>
       </c>
       <c r="F223" s="3" t="inlineStr">
         <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
+          <t>Indian National Congress</t>
         </is>
       </c>
       <c r="G223" s="4" t="n">
-        <v>14048</v>
+        <v>16428</v>
       </c>
       <c r="H223" s="3" t="inlineStr">
         <is>
-          <t>9/23</t>
+          <t>10/23</t>
         </is>
       </c>
       <c r="I223" s="3" t="inlineStr">
@@ -11458,10 +11446,10 @@
         </is>
       </c>
       <c r="J223" s="4" t="n">
-        <v>35900</v>
+        <v>37784</v>
       </c>
       <c r="K223" s="5" t="n">
-        <v>1560.888888888889</v>
+        <v>1642.8</v>
       </c>
     </row>
     <row r="224">
@@ -11690,11 +11678,11 @@
         </is>
       </c>
       <c r="G228" s="4" t="n">
-        <v>11249</v>
+        <v>12286</v>
       </c>
       <c r="H228" s="3" t="inlineStr">
         <is>
-          <t>8/22</t>
+          <t>9/22</t>
         </is>
       </c>
       <c r="I228" s="3" t="inlineStr">
@@ -11703,10 +11691,10 @@
         </is>
       </c>
       <c r="J228" s="4" t="n">
-        <v>30935</v>
+        <v>30032</v>
       </c>
       <c r="K228" s="5" t="n">
-        <v>1406.125</v>
+        <v>1365.111111111111</v>
       </c>
     </row>
     <row r="229">
@@ -11788,11 +11776,11 @@
         </is>
       </c>
       <c r="G230" s="7" t="n">
-        <v>1431</v>
+        <v>1015</v>
       </c>
       <c r="H230" s="6" t="inlineStr">
         <is>
-          <t>10/24</t>
+          <t>11/24</t>
         </is>
       </c>
       <c r="I230" s="6" t="inlineStr">
@@ -11801,10 +11789,10 @@
         </is>
       </c>
       <c r="J230" s="7" t="n">
-        <v>3434</v>
+        <v>2215</v>
       </c>
       <c r="K230" s="8" t="n">
-        <v>143.1</v>
+        <v>92.27272727272727</v>
       </c>
     </row>
     <row r="231">
@@ -11837,11 +11825,11 @@
         </is>
       </c>
       <c r="G231" s="4" t="n">
-        <v>14892</v>
+        <v>19764</v>
       </c>
       <c r="H231" s="3" t="inlineStr">
         <is>
-          <t>6/20</t>
+          <t>7/20</t>
         </is>
       </c>
       <c r="I231" s="3" t="inlineStr">
@@ -11850,10 +11838,10 @@
         </is>
       </c>
       <c r="J231" s="4" t="n">
-        <v>49640</v>
+        <v>56469</v>
       </c>
       <c r="K231" s="5" t="n">
-        <v>2482</v>
+        <v>2823.428571428572</v>
       </c>
     </row>
     <row r="232">
@@ -11984,11 +11972,11 @@
         </is>
       </c>
       <c r="G234" s="7" t="n">
-        <v>1414</v>
+        <v>1961</v>
       </c>
       <c r="H234" s="6" t="inlineStr">
         <is>
-          <t>11/23</t>
+          <t>12/23</t>
         </is>
       </c>
       <c r="I234" s="6" t="inlineStr">
@@ -11997,10 +11985,10 @@
         </is>
       </c>
       <c r="J234" s="7" t="n">
-        <v>2957</v>
+        <v>3759</v>
       </c>
       <c r="K234" s="8" t="n">
-        <v>128.5454545454545</v>
+        <v>163.4166666666667</v>
       </c>
     </row>
     <row r="235">
@@ -12072,29 +12060,29 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B1" s="17" t="inlineStr">
+      <c r="B1" s="13" t="inlineStr">
         <is>
           <t>Colour</t>
         </is>
       </c>
-      <c r="C1" s="17" t="inlineStr">
+      <c r="C1" s="13" t="inlineStr">
         <is>
           <t>Meaning</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="18" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>knife-edge</t>
         </is>
       </c>
-      <c r="B2" s="19" t="n"/>
+      <c r="B2" s="15" t="n"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>Contest index ≤ 10  — margin tiny relative to rounds left</t>
@@ -12102,12 +12090,12 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="18" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>competitive</t>
         </is>
       </c>
-      <c r="B3" s="20" t="n"/>
+      <c r="B3" s="16" t="n"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>Contest index 10–40 — still very much in play</t>
@@ -12115,12 +12103,12 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>decided</t>
         </is>
       </c>
-      <c r="B4" s="21" t="n"/>
+      <c r="B4" s="17" t="n"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>Projected margin ≥ 20k or counting 75%+ done with big lead</t>

</xml_diff>

<commit_message>
Update election results snapshot (46.9% counted)
TVK 111, AIADMK 58, DMK 48. 5 lead changes; NAMAKKAL (49 votes) and
NAGERCOIL (66 votes) are new knife-edge seats. 11 seats still in play.

https://claude.ai/code/session_01MizbUy44JG5sXyvaf3Wekb
</commit_message>
<xml_diff>
--- a/tn_election_results_may2026.xlsx
+++ b/tn_election_results_may2026.xlsx
@@ -91,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -127,6 +127,18 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -702,11 +714,11 @@
         </is>
       </c>
       <c r="G4" s="11" t="n">
-        <v>196</v>
+        <v>291</v>
       </c>
       <c r="H4" s="10" t="inlineStr">
         <is>
-          <t>13/24</t>
+          <t>14/24</t>
         </is>
       </c>
       <c r="I4" s="10" t="inlineStr">
@@ -715,10 +727,10 @@
         </is>
       </c>
       <c r="J4" s="11" t="n">
-        <v>362</v>
+        <v>499</v>
       </c>
       <c r="K4" s="12" t="n">
-        <v>15.07692307692308</v>
+        <v>20.78571428571428</v>
       </c>
     </row>
     <row r="5">
@@ -800,11 +812,11 @@
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>29124</v>
+        <v>32123</v>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>11/27</t>
+          <t>12/27</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -813,10 +825,10 @@
         </is>
       </c>
       <c r="J6" s="4" t="n">
-        <v>71486</v>
+        <v>72277</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>2647.636363636364</v>
+        <v>2676.916666666667</v>
       </c>
     </row>
     <row r="7">
@@ -1094,11 +1106,11 @@
         </is>
       </c>
       <c r="G12" s="4" t="n">
-        <v>14059</v>
+        <v>14666</v>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>12/21</t>
+          <t>13/21</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
@@ -1107,10 +1119,10 @@
         </is>
       </c>
       <c r="J12" s="4" t="n">
-        <v>24603</v>
+        <v>23691</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1171.583333333333</v>
+        <v>1128.153846153846</v>
       </c>
     </row>
     <row r="13">
@@ -1437,11 +1449,11 @@
         </is>
       </c>
       <c r="G19" s="4" t="n">
-        <v>10347</v>
+        <v>10746</v>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>9/25</t>
+          <t>10/25</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -1450,10 +1462,10 @@
         </is>
       </c>
       <c r="J19" s="4" t="n">
-        <v>28742</v>
+        <v>26865</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>1149.666666666667</v>
+        <v>1074.6</v>
       </c>
     </row>
     <row r="20">
@@ -1535,11 +1547,11 @@
         </is>
       </c>
       <c r="G21" s="4" t="n">
-        <v>24790</v>
+        <v>28067</v>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>9/26</t>
+          <t>10/26</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -1548,10 +1560,10 @@
         </is>
       </c>
       <c r="J21" s="4" t="n">
-        <v>71616</v>
+        <v>72974</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>2754.444444444444</v>
+        <v>2806.7</v>
       </c>
     </row>
     <row r="22">
@@ -1810,30 +1822,30 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
+          <t>PANNEERSELVAM.O</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
           <t>PRAKASH.S</t>
         </is>
       </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="inlineStr">
-        <is>
-          <t>PANNEERSELVAM.O</t>
-        </is>
-      </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>Dravida Munnetra Kazhagam</t>
+          <t>Tamilaga Vettri Kazhagam</t>
         </is>
       </c>
       <c r="G27" s="7" t="n">
-        <v>487</v>
+        <v>919</v>
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>10/25</t>
+          <t>11/25</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
@@ -1842,10 +1854,10 @@
         </is>
       </c>
       <c r="J27" s="7" t="n">
-        <v>1218</v>
+        <v>2089</v>
       </c>
       <c r="K27" s="8" t="n">
-        <v>48.7</v>
+        <v>83.54545454545455</v>
       </c>
     </row>
     <row r="28">
@@ -2074,11 +2086,11 @@
         </is>
       </c>
       <c r="G32" s="7" t="n">
-        <v>2771</v>
+        <v>2543</v>
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>14/21</t>
+          <t>15/21</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
@@ -2087,10 +2099,10 @@
         </is>
       </c>
       <c r="J32" s="7" t="n">
-        <v>4156</v>
+        <v>3560</v>
       </c>
       <c r="K32" s="8" t="n">
-        <v>197.9285714285714</v>
+        <v>169.5333333333333</v>
       </c>
     </row>
     <row r="33">
@@ -2613,11 +2625,11 @@
         </is>
       </c>
       <c r="G43" s="4" t="n">
-        <v>10364</v>
+        <v>13161</v>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>5/18</t>
+          <t>6/18</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
@@ -2626,10 +2638,10 @@
         </is>
       </c>
       <c r="J43" s="4" t="n">
-        <v>37310</v>
+        <v>39483</v>
       </c>
       <c r="K43" s="5" t="n">
-        <v>2072.8</v>
+        <v>2193.5</v>
       </c>
     </row>
     <row r="44">
@@ -2809,11 +2821,11 @@
         </is>
       </c>
       <c r="G47" s="4" t="n">
-        <v>9181</v>
+        <v>11184</v>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>8/24</t>
+          <t>9/24</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
@@ -2822,10 +2834,10 @@
         </is>
       </c>
       <c r="J47" s="4" t="n">
-        <v>27543</v>
+        <v>29824</v>
       </c>
       <c r="K47" s="5" t="n">
-        <v>1147.625</v>
+        <v>1242.666666666667</v>
       </c>
     </row>
     <row r="48">
@@ -3005,11 +3017,11 @@
         </is>
       </c>
       <c r="G51" s="7" t="n">
-        <v>10072</v>
+        <v>11074</v>
       </c>
       <c r="H51" s="6" t="inlineStr">
         <is>
-          <t>13/23</t>
+          <t>14/23</t>
         </is>
       </c>
       <c r="I51" s="6" t="inlineStr">
@@ -3018,10 +3030,10 @@
         </is>
       </c>
       <c r="J51" s="7" t="n">
-        <v>17820</v>
+        <v>18193</v>
       </c>
       <c r="K51" s="8" t="n">
-        <v>774.7692307692308</v>
+        <v>791</v>
       </c>
     </row>
     <row r="52">
@@ -3152,11 +3164,11 @@
         </is>
       </c>
       <c r="G54" s="4" t="n">
-        <v>10560</v>
+        <v>11906</v>
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>9/25</t>
+          <t>10/25</t>
         </is>
       </c>
       <c r="I54" s="3" t="inlineStr">
@@ -3165,10 +3177,10 @@
         </is>
       </c>
       <c r="J54" s="4" t="n">
-        <v>29333</v>
+        <v>29765</v>
       </c>
       <c r="K54" s="5" t="n">
-        <v>1173.333333333333</v>
+        <v>1190.6</v>
       </c>
     </row>
     <row r="55">
@@ -3250,11 +3262,11 @@
         </is>
       </c>
       <c r="G56" s="7" t="n">
-        <v>6518</v>
+        <v>5988</v>
       </c>
       <c r="H56" s="6" t="inlineStr">
         <is>
-          <t>15/23</t>
+          <t>16/23</t>
         </is>
       </c>
       <c r="I56" s="6" t="inlineStr">
@@ -3263,10 +3275,10 @@
         </is>
       </c>
       <c r="J56" s="7" t="n">
-        <v>9994</v>
+        <v>8608</v>
       </c>
       <c r="K56" s="8" t="n">
-        <v>434.5333333333334</v>
+        <v>374.25</v>
       </c>
     </row>
     <row r="57">
@@ -3299,11 +3311,11 @@
         </is>
       </c>
       <c r="G57" s="4" t="n">
-        <v>24107</v>
+        <v>25159</v>
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>12/34</t>
+          <t>13/34</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr">
@@ -3312,10 +3324,10 @@
         </is>
       </c>
       <c r="J57" s="4" t="n">
-        <v>68303</v>
+        <v>65800</v>
       </c>
       <c r="K57" s="5" t="n">
-        <v>2008.916666666667</v>
+        <v>1935.307692307692</v>
       </c>
     </row>
     <row r="58">
@@ -3348,11 +3360,11 @@
         </is>
       </c>
       <c r="G58" s="4" t="n">
-        <v>9693</v>
+        <v>10583</v>
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>11/23</t>
+          <t>12/23</t>
         </is>
       </c>
       <c r="I58" s="3" t="inlineStr">
@@ -3361,10 +3373,10 @@
         </is>
       </c>
       <c r="J58" s="4" t="n">
-        <v>20267</v>
+        <v>20284</v>
       </c>
       <c r="K58" s="5" t="n">
-        <v>881.1818181818181</v>
+        <v>881.9166666666666</v>
       </c>
     </row>
     <row r="59">
@@ -3936,11 +3948,11 @@
         </is>
       </c>
       <c r="G70" s="4" t="n">
-        <v>29048</v>
+        <v>30820</v>
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>19/28</t>
+          <t>20/28</t>
         </is>
       </c>
       <c r="I70" s="3" t="inlineStr">
@@ -3949,10 +3961,10 @@
         </is>
       </c>
       <c r="J70" s="4" t="n">
-        <v>42808</v>
+        <v>43148</v>
       </c>
       <c r="K70" s="5" t="n">
-        <v>1528.842105263158</v>
+        <v>1541</v>
       </c>
     </row>
     <row r="71">
@@ -4230,11 +4242,11 @@
         </is>
       </c>
       <c r="G76" s="7" t="n">
-        <v>8019</v>
+        <v>8048</v>
       </c>
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>11/22</t>
+          <t>12/22</t>
         </is>
       </c>
       <c r="I76" s="6" t="inlineStr">
@@ -4243,10 +4255,10 @@
         </is>
       </c>
       <c r="J76" s="7" t="n">
-        <v>16038</v>
+        <v>14755</v>
       </c>
       <c r="K76" s="8" t="n">
-        <v>729</v>
+        <v>670.6666666666666</v>
       </c>
     </row>
     <row r="77">
@@ -4397,52 +4409,52 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="9" t="inlineStr">
+      <c r="A80" s="6" t="inlineStr">
         <is>
           <t>KULITHALAI</t>
         </is>
       </c>
-      <c r="B80" s="10" t="n">
+      <c r="B80" s="6" t="n">
         <v>137</v>
       </c>
-      <c r="C80" s="10" t="inlineStr">
+      <c r="C80" s="6" t="inlineStr">
         <is>
           <t>G.BALASUBRAMANI</t>
         </is>
       </c>
-      <c r="D80" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E80" s="10" t="inlineStr">
+      <c r="D80" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E80" s="6" t="inlineStr">
         <is>
           <t>SURIYANUR. A. CHANDRAN</t>
         </is>
       </c>
-      <c r="F80" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G80" s="11" t="n">
-        <v>131</v>
-      </c>
-      <c r="H80" s="10" t="inlineStr">
-        <is>
-          <t>9/21</t>
-        </is>
-      </c>
-      <c r="I80" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J80" s="11" t="n">
-        <v>306</v>
-      </c>
-      <c r="K80" s="12" t="n">
-        <v>14.55555555555556</v>
+      <c r="F80" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G80" s="7" t="n">
+        <v>530</v>
+      </c>
+      <c r="H80" s="6" t="inlineStr">
+        <is>
+          <t>10/21</t>
+        </is>
+      </c>
+      <c r="I80" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J80" s="7" t="n">
+        <v>1113</v>
+      </c>
+      <c r="K80" s="8" t="n">
+        <v>53</v>
       </c>
     </row>
     <row r="81">
@@ -4524,11 +4536,11 @@
         </is>
       </c>
       <c r="G82" s="7" t="n">
-        <v>2323</v>
+        <v>2170</v>
       </c>
       <c r="H82" s="6" t="inlineStr">
         <is>
-          <t>14/22</t>
+          <t>15/22</t>
         </is>
       </c>
       <c r="I82" s="6" t="inlineStr">
@@ -4537,10 +4549,10 @@
         </is>
       </c>
       <c r="J82" s="7" t="n">
-        <v>3650</v>
+        <v>3183</v>
       </c>
       <c r="K82" s="8" t="n">
-        <v>165.9285714285714</v>
+        <v>144.6666666666667</v>
       </c>
     </row>
     <row r="83">
@@ -4769,11 +4781,11 @@
         </is>
       </c>
       <c r="G87" s="4" t="n">
-        <v>55635</v>
+        <v>61467</v>
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
-          <t>12/19</t>
+          <t>13/19</t>
         </is>
       </c>
       <c r="I87" s="3" t="inlineStr">
@@ -4782,10 +4794,10 @@
         </is>
       </c>
       <c r="J87" s="4" t="n">
-        <v>88089</v>
+        <v>89836</v>
       </c>
       <c r="K87" s="5" t="n">
-        <v>4636.25</v>
+        <v>4728.23076923077</v>
       </c>
     </row>
     <row r="88">
@@ -4818,11 +4830,11 @@
         </is>
       </c>
       <c r="G88" s="4" t="n">
-        <v>11051</v>
+        <v>12896</v>
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>6/19</t>
+          <t>7/19</t>
         </is>
       </c>
       <c r="I88" s="3" t="inlineStr">
@@ -4831,10 +4843,10 @@
         </is>
       </c>
       <c r="J88" s="4" t="n">
-        <v>34995</v>
+        <v>35003</v>
       </c>
       <c r="K88" s="5" t="n">
-        <v>1841.833333333333</v>
+        <v>1842.285714285714</v>
       </c>
     </row>
     <row r="89">
@@ -4916,11 +4928,11 @@
         </is>
       </c>
       <c r="G90" s="4" t="n">
-        <v>11927</v>
+        <v>13514</v>
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>9/19</t>
+          <t>10/19</t>
         </is>
       </c>
       <c r="I90" s="3" t="inlineStr">
@@ -4929,10 +4941,10 @@
         </is>
       </c>
       <c r="J90" s="4" t="n">
-        <v>25179</v>
+        <v>25677</v>
       </c>
       <c r="K90" s="5" t="n">
-        <v>1325.222222222222</v>
+        <v>1351.4</v>
       </c>
     </row>
     <row r="91">
@@ -5161,11 +5173,11 @@
         </is>
       </c>
       <c r="G95" s="4" t="n">
-        <v>18886</v>
+        <v>20405</v>
       </c>
       <c r="H95" s="3" t="inlineStr">
         <is>
-          <t>11/20</t>
+          <t>12/20</t>
         </is>
       </c>
       <c r="I95" s="3" t="inlineStr">
@@ -5174,10 +5186,10 @@
         </is>
       </c>
       <c r="J95" s="4" t="n">
-        <v>34338</v>
+        <v>34008</v>
       </c>
       <c r="K95" s="5" t="n">
-        <v>1716.909090909091</v>
+        <v>1700.416666666667</v>
       </c>
     </row>
     <row r="96">
@@ -5446,20 +5458,20 @@
       </c>
       <c r="E101" s="6" t="inlineStr">
         <is>
-          <t>P.PERIYAPULLAN (A) SELVAM</t>
+          <t>A.MADURAIVEERAN</t>
         </is>
       </c>
       <c r="F101" s="6" t="inlineStr">
         <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
+          <t>Tamilaga Vettri Kazhagam</t>
         </is>
       </c>
       <c r="G101" s="7" t="n">
-        <v>2697</v>
+        <v>3770</v>
       </c>
       <c r="H101" s="6" t="inlineStr">
         <is>
-          <t>16/21</t>
+          <t>17/21</t>
         </is>
       </c>
       <c r="I101" s="6" t="inlineStr">
@@ -5468,10 +5480,10 @@
         </is>
       </c>
       <c r="J101" s="7" t="n">
-        <v>3540</v>
+        <v>4657</v>
       </c>
       <c r="K101" s="8" t="n">
-        <v>168.5625</v>
+        <v>221.7647058823529</v>
       </c>
     </row>
     <row r="102">
@@ -5602,11 +5614,11 @@
         </is>
       </c>
       <c r="G104" s="7" t="n">
-        <v>3414</v>
+        <v>3092</v>
       </c>
       <c r="H104" s="6" t="inlineStr">
         <is>
-          <t>10/21</t>
+          <t>11/21</t>
         </is>
       </c>
       <c r="I104" s="6" t="inlineStr">
@@ -5615,10 +5627,10 @@
         </is>
       </c>
       <c r="J104" s="7" t="n">
-        <v>7169</v>
+        <v>5903</v>
       </c>
       <c r="K104" s="8" t="n">
-        <v>341.4</v>
+        <v>281.0909090909091</v>
       </c>
     </row>
     <row r="105">
@@ -5700,11 +5712,11 @@
         </is>
       </c>
       <c r="G106" s="7" t="n">
-        <v>12122</v>
+        <v>12453</v>
       </c>
       <c r="H106" s="6" t="inlineStr">
         <is>
-          <t>13/21</t>
+          <t>14/21</t>
         </is>
       </c>
       <c r="I106" s="6" t="inlineStr">
@@ -5713,10 +5725,10 @@
         </is>
       </c>
       <c r="J106" s="7" t="n">
-        <v>19582</v>
+        <v>18680</v>
       </c>
       <c r="K106" s="8" t="n">
-        <v>932.4615384615385</v>
+        <v>889.5</v>
       </c>
     </row>
     <row r="107">
@@ -5749,11 +5761,11 @@
         </is>
       </c>
       <c r="G107" s="4" t="n">
-        <v>18182</v>
+        <v>18652</v>
       </c>
       <c r="H107" s="3" t="inlineStr">
         <is>
-          <t>11/20</t>
+          <t>12/20</t>
         </is>
       </c>
       <c r="I107" s="3" t="inlineStr">
@@ -5762,10 +5774,10 @@
         </is>
       </c>
       <c r="J107" s="4" t="n">
-        <v>33058</v>
+        <v>31087</v>
       </c>
       <c r="K107" s="5" t="n">
-        <v>1652.909090909091</v>
+        <v>1554.333333333333</v>
       </c>
     </row>
     <row r="108">
@@ -5798,11 +5810,11 @@
         </is>
       </c>
       <c r="G108" s="4" t="n">
-        <v>5829</v>
+        <v>6096</v>
       </c>
       <c r="H108" s="3" t="inlineStr">
         <is>
-          <t>4/18</t>
+          <t>5/18</t>
         </is>
       </c>
       <c r="I108" s="3" t="inlineStr">
@@ -5811,108 +5823,108 @@
         </is>
       </c>
       <c r="J108" s="4" t="n">
-        <v>26230</v>
+        <v>21946</v>
       </c>
       <c r="K108" s="5" t="n">
-        <v>1457.25</v>
+        <v>1219.2</v>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="6" t="inlineStr">
+      <c r="A109" s="13" t="inlineStr">
         <is>
           <t>NAGERCOIL</t>
         </is>
       </c>
-      <c r="B109" s="6" t="n">
+      <c r="B109" s="14" t="n">
         <v>230</v>
       </c>
-      <c r="C109" s="6" t="inlineStr">
+      <c r="C109" s="14" t="inlineStr">
+        <is>
+          <t>BERVIN KINGS G</t>
+        </is>
+      </c>
+      <c r="D109" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E109" s="14" t="inlineStr">
         <is>
           <t>AUSTIN</t>
         </is>
       </c>
-      <c r="D109" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E109" s="6" t="inlineStr">
-        <is>
-          <t>BERVIN KINGS G</t>
-        </is>
-      </c>
-      <c r="F109" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G109" s="7" t="n">
-        <v>774</v>
-      </c>
-      <c r="H109" s="6" t="inlineStr">
-        <is>
-          <t>9/23</t>
-        </is>
-      </c>
-      <c r="I109" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J109" s="7" t="n">
-        <v>1978</v>
-      </c>
-      <c r="K109" s="8" t="n">
-        <v>86</v>
+      <c r="F109" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G109" s="15" t="n">
+        <v>66</v>
+      </c>
+      <c r="H109" s="14" t="inlineStr">
+        <is>
+          <t>10/23</t>
+        </is>
+      </c>
+      <c r="I109" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J109" s="15" t="n">
+        <v>152</v>
+      </c>
+      <c r="K109" s="16" t="n">
+        <v>6.6</v>
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="6" t="inlineStr">
+      <c r="A110" s="13" t="inlineStr">
         <is>
           <t>NAMAKKAL</t>
         </is>
       </c>
-      <c r="B110" s="6" t="n">
+      <c r="B110" s="14" t="n">
         <v>94</v>
       </c>
-      <c r="C110" s="6" t="inlineStr">
+      <c r="C110" s="14" t="inlineStr">
+        <is>
+          <t>DILIP C S</t>
+        </is>
+      </c>
+      <c r="D110" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E110" s="14" t="inlineStr">
         <is>
           <t>SRIDEVI MOHAN P S</t>
         </is>
       </c>
-      <c r="D110" s="6" t="inlineStr">
+      <c r="F110" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E110" s="6" t="inlineStr">
-        <is>
-          <t>DILIP C S</t>
-        </is>
-      </c>
-      <c r="F110" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G110" s="7" t="n">
-        <v>460</v>
-      </c>
-      <c r="H110" s="6" t="inlineStr">
-        <is>
-          <t>7/23</t>
-        </is>
-      </c>
-      <c r="I110" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J110" s="7" t="n">
-        <v>1511</v>
-      </c>
-      <c r="K110" s="8" t="n">
-        <v>65.71428571428571</v>
+      <c r="G110" s="15" t="n">
+        <v>49</v>
+      </c>
+      <c r="H110" s="14" t="inlineStr">
+        <is>
+          <t>8/23</t>
+        </is>
+      </c>
+      <c r="I110" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J110" s="15" t="n">
+        <v>141</v>
+      </c>
+      <c r="K110" s="16" t="n">
+        <v>6.125</v>
       </c>
     </row>
     <row r="111">
@@ -6386,11 +6398,11 @@
         </is>
       </c>
       <c r="G120" s="7" t="n">
-        <v>6507</v>
+        <v>7993</v>
       </c>
       <c r="H120" s="6" t="inlineStr">
         <is>
-          <t>11/23</t>
+          <t>12/23</t>
         </is>
       </c>
       <c r="I120" s="6" t="inlineStr">
@@ -6399,10 +6411,10 @@
         </is>
       </c>
       <c r="J120" s="7" t="n">
-        <v>13606</v>
+        <v>15320</v>
       </c>
       <c r="K120" s="8" t="n">
-        <v>591.5454545454545</v>
+        <v>666.0833333333334</v>
       </c>
     </row>
     <row r="121">
@@ -6582,11 +6594,11 @@
         </is>
       </c>
       <c r="G124" s="4" t="n">
-        <v>13002</v>
+        <v>12313</v>
       </c>
       <c r="H124" s="3" t="inlineStr">
         <is>
-          <t>12/35</t>
+          <t>13/35</t>
         </is>
       </c>
       <c r="I124" s="3" t="inlineStr">
@@ -6595,10 +6607,10 @@
         </is>
       </c>
       <c r="J124" s="4" t="n">
-        <v>37922</v>
+        <v>33150</v>
       </c>
       <c r="K124" s="5" t="n">
-        <v>1083.5</v>
+        <v>947.1538461538462</v>
       </c>
     </row>
     <row r="125">
@@ -6680,11 +6692,11 @@
         </is>
       </c>
       <c r="G126" s="7" t="n">
-        <v>2203</v>
+        <v>3264</v>
       </c>
       <c r="H126" s="6" t="inlineStr">
         <is>
-          <t>12/23</t>
+          <t>13/23</t>
         </is>
       </c>
       <c r="I126" s="6" t="inlineStr">
@@ -6693,10 +6705,10 @@
         </is>
       </c>
       <c r="J126" s="7" t="n">
-        <v>4222</v>
+        <v>5775</v>
       </c>
       <c r="K126" s="8" t="n">
-        <v>183.5833333333333</v>
+        <v>251.0769230769231</v>
       </c>
     </row>
     <row r="127">
@@ -6778,11 +6790,11 @@
         </is>
       </c>
       <c r="G128" s="4" t="n">
-        <v>30604</v>
+        <v>33492</v>
       </c>
       <c r="H128" s="3" t="inlineStr">
         <is>
-          <t>13/23</t>
+          <t>14/23</t>
         </is>
       </c>
       <c r="I128" s="3" t="inlineStr">
@@ -6791,10 +6803,10 @@
         </is>
       </c>
       <c r="J128" s="4" t="n">
-        <v>54146</v>
+        <v>55023</v>
       </c>
       <c r="K128" s="5" t="n">
-        <v>2354.153846153847</v>
+        <v>2392.285714285714</v>
       </c>
     </row>
     <row r="129">
@@ -6974,11 +6986,11 @@
         </is>
       </c>
       <c r="G132" s="7" t="n">
-        <v>3612</v>
+        <v>4459</v>
       </c>
       <c r="H132" s="6" t="inlineStr">
         <is>
-          <t>5/23</t>
+          <t>6/23</t>
         </is>
       </c>
       <c r="I132" s="6" t="inlineStr">
@@ -6987,10 +6999,10 @@
         </is>
       </c>
       <c r="J132" s="7" t="n">
-        <v>16615</v>
+        <v>17093</v>
       </c>
       <c r="K132" s="8" t="n">
-        <v>722.4</v>
+        <v>743.1666666666666</v>
       </c>
     </row>
     <row r="133">
@@ -7415,11 +7427,11 @@
         </is>
       </c>
       <c r="G141" s="7" t="n">
-        <v>2947</v>
+        <v>1388</v>
       </c>
       <c r="H141" s="6" t="inlineStr">
         <is>
-          <t>9/25</t>
+          <t>10/25</t>
         </is>
       </c>
       <c r="I141" s="6" t="inlineStr">
@@ -7428,10 +7440,10 @@
         </is>
       </c>
       <c r="J141" s="7" t="n">
-        <v>8186</v>
+        <v>3470</v>
       </c>
       <c r="K141" s="8" t="n">
-        <v>327.4444444444445</v>
+        <v>138.8</v>
       </c>
     </row>
     <row r="142">
@@ -7660,11 +7672,11 @@
         </is>
       </c>
       <c r="G146" s="4" t="n">
-        <v>12113</v>
+        <v>11898</v>
       </c>
       <c r="H146" s="3" t="inlineStr">
         <is>
-          <t>16/29</t>
+          <t>17/29</t>
         </is>
       </c>
       <c r="I146" s="3" t="inlineStr">
@@ -7673,10 +7685,10 @@
         </is>
       </c>
       <c r="J146" s="4" t="n">
-        <v>21955</v>
+        <v>20297</v>
       </c>
       <c r="K146" s="5" t="n">
-        <v>757.0625</v>
+        <v>699.8823529411765</v>
       </c>
     </row>
     <row r="147">
@@ -8542,11 +8554,11 @@
         </is>
       </c>
       <c r="G164" s="7" t="n">
-        <v>6941</v>
+        <v>7337</v>
       </c>
       <c r="H164" s="6" t="inlineStr">
         <is>
-          <t>13/22</t>
+          <t>14/22</t>
         </is>
       </c>
       <c r="I164" s="6" t="inlineStr">
@@ -8555,10 +8567,10 @@
         </is>
       </c>
       <c r="J164" s="7" t="n">
-        <v>11746</v>
+        <v>11530</v>
       </c>
       <c r="K164" s="8" t="n">
-        <v>533.9230769230769</v>
+        <v>524.0714285714286</v>
       </c>
     </row>
     <row r="165">
@@ -8836,11 +8848,11 @@
         </is>
       </c>
       <c r="G170" s="7" t="n">
-        <v>4725</v>
+        <v>4697</v>
       </c>
       <c r="H170" s="6" t="inlineStr">
         <is>
-          <t>6/22</t>
+          <t>7/22</t>
         </is>
       </c>
       <c r="I170" s="6" t="inlineStr">
@@ -8849,10 +8861,10 @@
         </is>
       </c>
       <c r="J170" s="7" t="n">
-        <v>17325</v>
+        <v>14762</v>
       </c>
       <c r="K170" s="8" t="n">
-        <v>787.5</v>
+        <v>671</v>
       </c>
     </row>
     <row r="171">
@@ -8885,11 +8897,11 @@
         </is>
       </c>
       <c r="G171" s="7" t="n">
-        <v>3603</v>
+        <v>4540</v>
       </c>
       <c r="H171" s="6" t="inlineStr">
         <is>
-          <t>9/28</t>
+          <t>10/28</t>
         </is>
       </c>
       <c r="I171" s="6" t="inlineStr">
@@ -8898,10 +8910,10 @@
         </is>
       </c>
       <c r="J171" s="7" t="n">
-        <v>11209</v>
+        <v>12712</v>
       </c>
       <c r="K171" s="8" t="n">
-        <v>400.3333333333333</v>
+        <v>454</v>
       </c>
     </row>
     <row r="172">
@@ -8954,52 +8966,52 @@
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="2" t="inlineStr">
+      <c r="A173" s="6" t="inlineStr">
         <is>
           <t>TENKASI</t>
         </is>
       </c>
-      <c r="B173" s="3" t="n">
+      <c r="B173" s="6" t="n">
         <v>222</v>
       </c>
-      <c r="C173" s="3" t="inlineStr">
+      <c r="C173" s="6" t="inlineStr">
         <is>
           <t>DR.KALAI KATHIRAVAN</t>
         </is>
       </c>
-      <c r="D173" s="3" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E173" s="3" t="inlineStr">
+      <c r="D173" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E173" s="6" t="inlineStr">
         <is>
           <t>S.SELVA MOHANDAS PANDIAN</t>
         </is>
       </c>
-      <c r="F173" s="3" t="inlineStr">
+      <c r="F173" s="6" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G173" s="4" t="n">
-        <v>8498</v>
-      </c>
-      <c r="H173" s="3" t="inlineStr">
-        <is>
-          <t>10/26</t>
-        </is>
-      </c>
-      <c r="I173" s="3" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J173" s="4" t="n">
-        <v>22095</v>
-      </c>
-      <c r="K173" s="5" t="n">
-        <v>849.8</v>
+      <c r="G173" s="7" t="n">
+        <v>7799</v>
+      </c>
+      <c r="H173" s="6" t="inlineStr">
+        <is>
+          <t>11/26</t>
+        </is>
+      </c>
+      <c r="I173" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J173" s="7" t="n">
+        <v>18434</v>
+      </c>
+      <c r="K173" s="8" t="n">
+        <v>709</v>
       </c>
     </row>
     <row r="174">
@@ -9081,11 +9093,11 @@
         </is>
       </c>
       <c r="G175" s="4" t="n">
-        <v>17155</v>
+        <v>16999</v>
       </c>
       <c r="H175" s="3" t="inlineStr">
         <is>
-          <t>19/23</t>
+          <t>20/23</t>
         </is>
       </c>
       <c r="I175" s="3" t="inlineStr">
@@ -9094,10 +9106,10 @@
         </is>
       </c>
       <c r="J175" s="4" t="n">
-        <v>20767</v>
+        <v>19549</v>
       </c>
       <c r="K175" s="5" t="n">
-        <v>902.8947368421053</v>
+        <v>849.95</v>
       </c>
     </row>
     <row r="176">
@@ -9179,11 +9191,11 @@
         </is>
       </c>
       <c r="G177" s="7" t="n">
-        <v>7965</v>
+        <v>8849</v>
       </c>
       <c r="H177" s="6" t="inlineStr">
         <is>
-          <t>14/26</t>
+          <t>15/26</t>
         </is>
       </c>
       <c r="I177" s="6" t="inlineStr">
@@ -9192,10 +9204,10 @@
         </is>
       </c>
       <c r="J177" s="7" t="n">
-        <v>14792</v>
+        <v>15338</v>
       </c>
       <c r="K177" s="8" t="n">
-        <v>568.9285714285714</v>
+        <v>589.9333333333334</v>
       </c>
     </row>
     <row r="178">
@@ -9277,11 +9289,11 @@
         </is>
       </c>
       <c r="G179" s="4" t="n">
-        <v>10722</v>
+        <v>14007</v>
       </c>
       <c r="H179" s="3" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>11/26</t>
         </is>
       </c>
       <c r="I179" s="3" t="inlineStr">
@@ -9290,10 +9302,10 @@
         </is>
       </c>
       <c r="J179" s="4" t="n">
-        <v>27877</v>
+        <v>33107</v>
       </c>
       <c r="K179" s="5" t="n">
-        <v>1072.2</v>
+        <v>1273.363636363636</v>
       </c>
     </row>
     <row r="180">
@@ -9669,11 +9681,11 @@
         </is>
       </c>
       <c r="G187" s="4" t="n">
-        <v>22458</v>
+        <v>24680</v>
       </c>
       <c r="H187" s="3" t="inlineStr">
         <is>
-          <t>10/25</t>
+          <t>11/25</t>
         </is>
       </c>
       <c r="I187" s="3" t="inlineStr">
@@ -9682,10 +9694,10 @@
         </is>
       </c>
       <c r="J187" s="4" t="n">
-        <v>56145</v>
+        <v>56091</v>
       </c>
       <c r="K187" s="5" t="n">
-        <v>2245.8</v>
+        <v>2243.636363636364</v>
       </c>
     </row>
     <row r="188">
@@ -9718,11 +9730,11 @@
         </is>
       </c>
       <c r="G188" s="7" t="n">
-        <v>9148</v>
+        <v>9788</v>
       </c>
       <c r="H188" s="6" t="inlineStr">
         <is>
-          <t>10/18</t>
+          <t>11/18</t>
         </is>
       </c>
       <c r="I188" s="6" t="inlineStr">
@@ -9731,10 +9743,10 @@
         </is>
       </c>
       <c r="J188" s="7" t="n">
-        <v>16466</v>
+        <v>16017</v>
       </c>
       <c r="K188" s="8" t="n">
-        <v>914.8</v>
+        <v>889.8181818181819</v>
       </c>
     </row>
     <row r="189">
@@ -9816,11 +9828,11 @@
         </is>
       </c>
       <c r="G190" s="4" t="n">
-        <v>21872</v>
+        <v>23166</v>
       </c>
       <c r="H190" s="3" t="inlineStr">
         <is>
-          <t>13/26</t>
+          <t>14/26</t>
         </is>
       </c>
       <c r="I190" s="3" t="inlineStr">
@@ -9829,10 +9841,10 @@
         </is>
       </c>
       <c r="J190" s="4" t="n">
-        <v>43744</v>
+        <v>43023</v>
       </c>
       <c r="K190" s="5" t="n">
-        <v>1682.461538461539</v>
+        <v>1654.714285714286</v>
       </c>
     </row>
     <row r="191">
@@ -9963,11 +9975,11 @@
         </is>
       </c>
       <c r="G193" s="7" t="n">
-        <v>2882</v>
+        <v>2122</v>
       </c>
       <c r="H193" s="6" t="inlineStr">
         <is>
-          <t>7/21</t>
+          <t>8/21</t>
         </is>
       </c>
       <c r="I193" s="6" t="inlineStr">
@@ -9976,10 +9988,10 @@
         </is>
       </c>
       <c r="J193" s="7" t="n">
-        <v>8646</v>
+        <v>5570</v>
       </c>
       <c r="K193" s="8" t="n">
-        <v>411.7142857142857</v>
+        <v>265.25</v>
       </c>
     </row>
     <row r="194">
@@ -10012,11 +10024,11 @@
         </is>
       </c>
       <c r="G194" s="7" t="n">
-        <v>7578</v>
+        <v>8355</v>
       </c>
       <c r="H194" s="6" t="inlineStr">
         <is>
-          <t>13/22</t>
+          <t>14/22</t>
         </is>
       </c>
       <c r="I194" s="6" t="inlineStr">
@@ -10025,10 +10037,10 @@
         </is>
       </c>
       <c r="J194" s="7" t="n">
-        <v>12824</v>
+        <v>13129</v>
       </c>
       <c r="K194" s="8" t="n">
-        <v>582.9230769230769</v>
+        <v>596.7857142857143</v>
       </c>
     </row>
     <row r="195">
@@ -10355,11 +10367,11 @@
         </is>
       </c>
       <c r="G201" s="4" t="n">
-        <v>15965</v>
+        <v>12445</v>
       </c>
       <c r="H201" s="3" t="inlineStr">
         <is>
-          <t>6/22</t>
+          <t>7/22</t>
         </is>
       </c>
       <c r="I201" s="3" t="inlineStr">
@@ -10368,10 +10380,10 @@
         </is>
       </c>
       <c r="J201" s="4" t="n">
-        <v>58538</v>
+        <v>39113</v>
       </c>
       <c r="K201" s="5" t="n">
-        <v>2660.833333333333</v>
+        <v>1777.857142857143</v>
       </c>
     </row>
     <row r="202">
@@ -10502,11 +10514,11 @@
         </is>
       </c>
       <c r="G204" s="4" t="n">
-        <v>9408</v>
+        <v>11503</v>
       </c>
       <c r="H204" s="3" t="inlineStr">
         <is>
-          <t>8/21</t>
+          <t>9/21</t>
         </is>
       </c>
       <c r="I204" s="3" t="inlineStr">
@@ -10515,10 +10527,10 @@
         </is>
       </c>
       <c r="J204" s="4" t="n">
-        <v>24696</v>
+        <v>26840</v>
       </c>
       <c r="K204" s="5" t="n">
-        <v>1176</v>
+        <v>1278.111111111111</v>
       </c>
     </row>
     <row r="205">
@@ -10649,11 +10661,11 @@
         </is>
       </c>
       <c r="G207" s="7" t="n">
-        <v>1094</v>
+        <v>1079</v>
       </c>
       <c r="H207" s="6" t="inlineStr">
         <is>
-          <t>7/23</t>
+          <t>8/23</t>
         </is>
       </c>
       <c r="I207" s="6" t="inlineStr">
@@ -10662,10 +10674,10 @@
         </is>
       </c>
       <c r="J207" s="7" t="n">
-        <v>3595</v>
+        <v>3102</v>
       </c>
       <c r="K207" s="8" t="n">
-        <v>156.2857142857143</v>
+        <v>134.875</v>
       </c>
     </row>
     <row r="208">
@@ -10738,20 +10750,20 @@
       </c>
       <c r="E209" s="6" t="inlineStr">
         <is>
-          <t>RAMACHANDRAN.B</t>
+          <t>BHOJARAJAN.M</t>
         </is>
       </c>
       <c r="F209" s="6" t="inlineStr">
         <is>
-          <t>Indian National Congress</t>
+          <t>Bharatiya Janata Party</t>
         </is>
       </c>
       <c r="G209" s="7" t="n">
-        <v>2903</v>
+        <v>1130</v>
       </c>
       <c r="H209" s="6" t="inlineStr">
         <is>
-          <t>14/19</t>
+          <t>15/19</t>
         </is>
       </c>
       <c r="I209" s="6" t="inlineStr">
@@ -10760,10 +10772,10 @@
         </is>
       </c>
       <c r="J209" s="7" t="n">
-        <v>3940</v>
+        <v>1431</v>
       </c>
       <c r="K209" s="8" t="n">
-        <v>207.3571428571429</v>
+        <v>75.33333333333333</v>
       </c>
     </row>
     <row r="210">
@@ -10796,11 +10808,11 @@
         </is>
       </c>
       <c r="G210" s="7" t="n">
-        <v>2469</v>
+        <v>3400</v>
       </c>
       <c r="H210" s="6" t="inlineStr">
         <is>
-          <t>12/22</t>
+          <t>13/22</t>
         </is>
       </c>
       <c r="I210" s="6" t="inlineStr">
@@ -10809,10 +10821,10 @@
         </is>
       </c>
       <c r="J210" s="7" t="n">
-        <v>4526</v>
+        <v>5754</v>
       </c>
       <c r="K210" s="8" t="n">
-        <v>205.75</v>
+        <v>261.5384615384615</v>
       </c>
     </row>
     <row r="211">
@@ -11041,7 +11053,7 @@
         </is>
       </c>
       <c r="G215" s="7" t="n">
-        <v>3790</v>
+        <v>4164</v>
       </c>
       <c r="H215" s="6" t="inlineStr">
         <is>
@@ -11054,10 +11066,10 @@
         </is>
       </c>
       <c r="J215" s="7" t="n">
-        <v>4548</v>
+        <v>4997</v>
       </c>
       <c r="K215" s="8" t="n">
-        <v>252.6666666666667</v>
+        <v>277.6</v>
       </c>
     </row>
     <row r="216">
@@ -11237,11 +11249,11 @@
         </is>
       </c>
       <c r="G219" s="7" t="n">
-        <v>5475</v>
+        <v>6793</v>
       </c>
       <c r="H219" s="6" t="inlineStr">
         <is>
-          <t>11/23</t>
+          <t>12/23</t>
         </is>
       </c>
       <c r="I219" s="6" t="inlineStr">
@@ -11250,10 +11262,10 @@
         </is>
       </c>
       <c r="J219" s="7" t="n">
-        <v>11448</v>
+        <v>13020</v>
       </c>
       <c r="K219" s="8" t="n">
-        <v>497.7272727272727</v>
+        <v>566.0833333333334</v>
       </c>
     </row>
     <row r="220">
@@ -11551,52 +11563,52 @@
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="6" t="inlineStr">
+      <c r="A226" s="9" t="inlineStr">
         <is>
           <t>VIKRAVANDI</t>
         </is>
       </c>
-      <c r="B226" s="6" t="n">
+      <c r="B226" s="10" t="n">
         <v>75</v>
       </c>
-      <c r="C226" s="6" t="inlineStr">
+      <c r="C226" s="10" t="inlineStr">
         <is>
           <t>SIVAKUMAR C</t>
         </is>
       </c>
-      <c r="D226" s="6" t="inlineStr">
+      <c r="D226" s="10" t="inlineStr">
         <is>
           <t>Pattali Makkal Katchi</t>
         </is>
       </c>
-      <c r="E226" s="6" t="inlineStr">
+      <c r="E226" s="10" t="inlineStr">
         <is>
           <t>VIJAI VADIVEL A</t>
         </is>
       </c>
-      <c r="F226" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G226" s="7" t="n">
-        <v>547</v>
-      </c>
-      <c r="H226" s="6" t="inlineStr">
-        <is>
-          <t>5/23</t>
-        </is>
-      </c>
-      <c r="I226" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J226" s="7" t="n">
-        <v>2516</v>
-      </c>
-      <c r="K226" s="8" t="n">
-        <v>109.4</v>
+      <c r="F226" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G226" s="11" t="n">
+        <v>102</v>
+      </c>
+      <c r="H226" s="10" t="inlineStr">
+        <is>
+          <t>6/23</t>
+        </is>
+      </c>
+      <c r="I226" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J226" s="11" t="n">
+        <v>391</v>
+      </c>
+      <c r="K226" s="12" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="227">
@@ -11776,11 +11788,11 @@
         </is>
       </c>
       <c r="G230" s="7" t="n">
-        <v>1015</v>
+        <v>1272</v>
       </c>
       <c r="H230" s="6" t="inlineStr">
         <is>
-          <t>11/24</t>
+          <t>12/24</t>
         </is>
       </c>
       <c r="I230" s="6" t="inlineStr">
@@ -11789,10 +11801,10 @@
         </is>
       </c>
       <c r="J230" s="7" t="n">
-        <v>2215</v>
+        <v>2544</v>
       </c>
       <c r="K230" s="8" t="n">
-        <v>92.27272727272727</v>
+        <v>106</v>
       </c>
     </row>
     <row r="231">
@@ -11972,11 +11984,11 @@
         </is>
       </c>
       <c r="G234" s="7" t="n">
-        <v>1961</v>
+        <v>2466</v>
       </c>
       <c r="H234" s="6" t="inlineStr">
         <is>
-          <t>12/23</t>
+          <t>13/23</t>
         </is>
       </c>
       <c r="I234" s="6" t="inlineStr">
@@ -11985,10 +11997,10 @@
         </is>
       </c>
       <c r="J234" s="7" t="n">
-        <v>3759</v>
+        <v>4363</v>
       </c>
       <c r="K234" s="8" t="n">
-        <v>163.4166666666667</v>
+        <v>189.6923076923077</v>
       </c>
     </row>
     <row r="235">
@@ -12021,11 +12033,11 @@
         </is>
       </c>
       <c r="G235" s="7" t="n">
-        <v>1604</v>
+        <v>2680</v>
       </c>
       <c r="H235" s="6" t="inlineStr">
         <is>
-          <t>7/24</t>
+          <t>8/24</t>
         </is>
       </c>
       <c r="I235" s="6" t="inlineStr">
@@ -12034,10 +12046,10 @@
         </is>
       </c>
       <c r="J235" s="7" t="n">
-        <v>5499</v>
+        <v>8040</v>
       </c>
       <c r="K235" s="8" t="n">
-        <v>229.1428571428571</v>
+        <v>335</v>
       </c>
     </row>
   </sheetData>
@@ -12060,29 +12072,29 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B1" s="13" t="inlineStr">
+      <c r="B1" s="17" t="inlineStr">
         <is>
           <t>Colour</t>
         </is>
       </c>
-      <c r="C1" s="13" t="inlineStr">
+      <c r="C1" s="17" t="inlineStr">
         <is>
           <t>Meaning</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="14" t="inlineStr">
+      <c r="A2" s="18" t="inlineStr">
         <is>
           <t>knife-edge</t>
         </is>
       </c>
-      <c r="B2" s="15" t="n"/>
+      <c r="B2" s="19" t="n"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>Contest index ≤ 10  — margin tiny relative to rounds left</t>
@@ -12090,12 +12102,12 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="18" t="inlineStr">
         <is>
           <t>competitive</t>
         </is>
       </c>
-      <c r="B3" s="16" t="n"/>
+      <c r="B3" s="20" t="n"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>Contest index 10–40 — still very much in play</t>
@@ -12103,12 +12115,12 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="14" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>decided</t>
         </is>
       </c>
-      <c r="B4" s="17" t="n"/>
+      <c r="B4" s="21" t="n"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>Projected margin ≥ 20k or counting 75%+ done with big lead</t>

</xml_diff>

<commit_message>
Update election results snapshot (48.2% counted)
TVK 110, AIADMK 58, DMK 49. 6 lead changes; THALLI (30 votes) is new
tightest seat. BJP lost lead to CPI. 14 seats still in play.

https://claude.ai/code/session_01MizbUy44JG5sXyvaf3Wekb
</commit_message>
<xml_diff>
--- a/tn_election_results_may2026.xlsx
+++ b/tn_election_results_may2026.xlsx
@@ -665,11 +665,11 @@
         </is>
       </c>
       <c r="G3" s="7" t="n">
-        <v>3523</v>
+        <v>4388</v>
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
-          <t>7/20</t>
+          <t>8/20</t>
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr">
@@ -678,10 +678,10 @@
         </is>
       </c>
       <c r="J3" s="7" t="n">
-        <v>10066</v>
+        <v>10970</v>
       </c>
       <c r="K3" s="8" t="n">
-        <v>503.2857142857143</v>
+        <v>548.5</v>
       </c>
     </row>
     <row r="4">
@@ -763,11 +763,11 @@
         </is>
       </c>
       <c r="G5" s="7" t="n">
-        <v>5984</v>
+        <v>7002</v>
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>14/23</t>
+          <t>15/23</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr">
@@ -776,10 +776,10 @@
         </is>
       </c>
       <c r="J5" s="7" t="n">
-        <v>9831</v>
+        <v>10736</v>
       </c>
       <c r="K5" s="8" t="n">
-        <v>427.4285714285714</v>
+        <v>466.8</v>
       </c>
     </row>
     <row r="6">
@@ -861,11 +861,11 @@
         </is>
       </c>
       <c r="G7" s="7" t="n">
-        <v>6703</v>
+        <v>8055</v>
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>8/22</t>
+          <t>9/22</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
@@ -874,10 +874,10 @@
         </is>
       </c>
       <c r="J7" s="7" t="n">
-        <v>18433</v>
+        <v>19690</v>
       </c>
       <c r="K7" s="8" t="n">
-        <v>837.875</v>
+        <v>895</v>
       </c>
     </row>
     <row r="8">
@@ -1008,11 +1008,11 @@
         </is>
       </c>
       <c r="G10" s="4" t="n">
-        <v>15704</v>
+        <v>16817</v>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>14/20</t>
+          <t>15/20</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
@@ -1021,10 +1021,10 @@
         </is>
       </c>
       <c r="J10" s="4" t="n">
-        <v>22434</v>
+        <v>22423</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>1121.714285714286</v>
+        <v>1121.133333333333</v>
       </c>
     </row>
     <row r="11">
@@ -1106,11 +1106,11 @@
         </is>
       </c>
       <c r="G12" s="4" t="n">
-        <v>14666</v>
+        <v>15833</v>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>13/21</t>
+          <t>14/21</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
@@ -1119,10 +1119,10 @@
         </is>
       </c>
       <c r="J12" s="4" t="n">
-        <v>23691</v>
+        <v>23749</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1128.153846153846</v>
+        <v>1130.928571428571</v>
       </c>
     </row>
     <row r="13">
@@ -1155,11 +1155,11 @@
         </is>
       </c>
       <c r="G13" s="7" t="n">
-        <v>4524</v>
+        <v>3800</v>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>14/24</t>
+          <t>15/24</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
@@ -1168,10 +1168,10 @@
         </is>
       </c>
       <c r="J13" s="7" t="n">
-        <v>7755</v>
+        <v>6080</v>
       </c>
       <c r="K13" s="8" t="n">
-        <v>323.1428571428572</v>
+        <v>253.3333333333333</v>
       </c>
     </row>
     <row r="14">
@@ -1645,11 +1645,11 @@
         </is>
       </c>
       <c r="G23" s="7" t="n">
-        <v>1259</v>
+        <v>2208</v>
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>9/24</t>
+          <t>10/24</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr">
@@ -1658,10 +1658,10 @@
         </is>
       </c>
       <c r="J23" s="7" t="n">
-        <v>3357</v>
+        <v>5299</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>139.8888888888889</v>
+        <v>220.8</v>
       </c>
     </row>
     <row r="24">
@@ -1890,11 +1890,11 @@
         </is>
       </c>
       <c r="G28" s="4" t="n">
-        <v>12738</v>
+        <v>14207</v>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>8/36</t>
+          <t>9/36</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
@@ -1903,10 +1903,10 @@
         </is>
       </c>
       <c r="J28" s="4" t="n">
-        <v>57321</v>
+        <v>56828</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>1592.25</v>
+        <v>1578.555555555556</v>
       </c>
     </row>
     <row r="29">
@@ -2037,11 +2037,11 @@
         </is>
       </c>
       <c r="G31" s="4" t="n">
-        <v>14793</v>
+        <v>16511</v>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>18/24</t>
+          <t>19/24</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -2050,10 +2050,10 @@
         </is>
       </c>
       <c r="J31" s="4" t="n">
-        <v>19724</v>
+        <v>20856</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>821.8333333333334</v>
+        <v>869</v>
       </c>
     </row>
     <row r="32">
@@ -2429,11 +2429,11 @@
         </is>
       </c>
       <c r="G39" s="7" t="n">
-        <v>3002</v>
+        <v>3918</v>
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>8/25</t>
+          <t>9/25</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr">
@@ -2442,10 +2442,10 @@
         </is>
       </c>
       <c r="J39" s="7" t="n">
-        <v>9381</v>
+        <v>10883</v>
       </c>
       <c r="K39" s="8" t="n">
-        <v>375.25</v>
+        <v>435.3333333333333</v>
       </c>
     </row>
     <row r="40">
@@ -2527,11 +2527,11 @@
         </is>
       </c>
       <c r="G41" s="7" t="n">
-        <v>6817</v>
+        <v>6228</v>
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>12/23</t>
+          <t>13/23</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr">
@@ -2540,10 +2540,10 @@
         </is>
       </c>
       <c r="J41" s="7" t="n">
-        <v>13066</v>
+        <v>11019</v>
       </c>
       <c r="K41" s="8" t="n">
-        <v>568.0833333333334</v>
+        <v>479.0769230769232</v>
       </c>
     </row>
     <row r="42">
@@ -2674,11 +2674,11 @@
         </is>
       </c>
       <c r="G44" s="4" t="n">
-        <v>50379</v>
+        <v>54458</v>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>13/25</t>
+          <t>14/25</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
@@ -2687,10 +2687,10 @@
         </is>
       </c>
       <c r="J44" s="4" t="n">
-        <v>96883</v>
+        <v>97246</v>
       </c>
       <c r="K44" s="5" t="n">
-        <v>3875.307692307692</v>
+        <v>3889.857142857142</v>
       </c>
     </row>
     <row r="45">
@@ -2968,11 +2968,11 @@
         </is>
       </c>
       <c r="G50" s="7" t="n">
-        <v>4334</v>
+        <v>4912</v>
       </c>
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>5/23</t>
+          <t>6/23</t>
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr">
@@ -2981,10 +2981,10 @@
         </is>
       </c>
       <c r="J50" s="7" t="n">
-        <v>19936</v>
+        <v>18829</v>
       </c>
       <c r="K50" s="8" t="n">
-        <v>866.8</v>
+        <v>818.6666666666666</v>
       </c>
     </row>
     <row r="51">
@@ -3066,11 +3066,11 @@
         </is>
       </c>
       <c r="G52" s="4" t="n">
-        <v>22520</v>
+        <v>22833</v>
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>17/18</t>
+          <t>18/18</t>
         </is>
       </c>
       <c r="I52" s="3" t="inlineStr">
@@ -3079,10 +3079,10 @@
         </is>
       </c>
       <c r="J52" s="4" t="n">
-        <v>23845</v>
+        <v>22833</v>
       </c>
       <c r="K52" s="5" t="n">
-        <v>1324.705882352941</v>
+        <v>1268.5</v>
       </c>
     </row>
     <row r="53">
@@ -3262,11 +3262,11 @@
         </is>
       </c>
       <c r="G56" s="7" t="n">
-        <v>5988</v>
+        <v>5663</v>
       </c>
       <c r="H56" s="6" t="inlineStr">
         <is>
-          <t>16/23</t>
+          <t>17/23</t>
         </is>
       </c>
       <c r="I56" s="6" t="inlineStr">
@@ -3275,10 +3275,10 @@
         </is>
       </c>
       <c r="J56" s="7" t="n">
-        <v>8608</v>
+        <v>7662</v>
       </c>
       <c r="K56" s="8" t="n">
-        <v>374.25</v>
+        <v>333.1176470588235</v>
       </c>
     </row>
     <row r="57">
@@ -3556,11 +3556,11 @@
         </is>
       </c>
       <c r="G62" s="7" t="n">
-        <v>1898</v>
+        <v>1259</v>
       </c>
       <c r="H62" s="6" t="inlineStr">
         <is>
-          <t>5/27</t>
+          <t>6/27</t>
         </is>
       </c>
       <c r="I62" s="6" t="inlineStr">
@@ -3569,10 +3569,10 @@
         </is>
       </c>
       <c r="J62" s="7" t="n">
-        <v>10249</v>
+        <v>5666</v>
       </c>
       <c r="K62" s="8" t="n">
-        <v>379.6</v>
+        <v>209.8333333333333</v>
       </c>
     </row>
     <row r="63">
@@ -3752,11 +3752,11 @@
         </is>
       </c>
       <c r="G66" s="4" t="n">
-        <v>15168</v>
+        <v>17895</v>
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>9/28</t>
+          <t>10/28</t>
         </is>
       </c>
       <c r="I66" s="3" t="inlineStr">
@@ -3765,10 +3765,10 @@
         </is>
       </c>
       <c r="J66" s="4" t="n">
-        <v>47189</v>
+        <v>50106</v>
       </c>
       <c r="K66" s="5" t="n">
-        <v>1685.333333333333</v>
+        <v>1789.5</v>
       </c>
     </row>
     <row r="67">
@@ -4095,11 +4095,11 @@
         </is>
       </c>
       <c r="G73" s="7" t="n">
-        <v>5213</v>
+        <v>5556</v>
       </c>
       <c r="H73" s="6" t="inlineStr">
         <is>
-          <t>5/19</t>
+          <t>6/19</t>
         </is>
       </c>
       <c r="I73" s="6" t="inlineStr">
@@ -4108,10 +4108,10 @@
         </is>
       </c>
       <c r="J73" s="7" t="n">
-        <v>19809</v>
+        <v>17594</v>
       </c>
       <c r="K73" s="8" t="n">
-        <v>1042.6</v>
+        <v>926</v>
       </c>
     </row>
     <row r="74">
@@ -4340,11 +4340,11 @@
         </is>
       </c>
       <c r="G78" s="4" t="n">
-        <v>17430</v>
+        <v>17967</v>
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
-          <t>15/25</t>
+          <t>16/25</t>
         </is>
       </c>
       <c r="I78" s="3" t="inlineStr">
@@ -4353,10 +4353,10 @@
         </is>
       </c>
       <c r="J78" s="4" t="n">
-        <v>29050</v>
+        <v>28073</v>
       </c>
       <c r="K78" s="5" t="n">
-        <v>1162</v>
+        <v>1122.9375</v>
       </c>
     </row>
     <row r="79">
@@ -4389,11 +4389,11 @@
         </is>
       </c>
       <c r="G79" s="7" t="n">
-        <v>1099</v>
+        <v>2216</v>
       </c>
       <c r="H79" s="6" t="inlineStr">
         <is>
-          <t>8/20</t>
+          <t>9/20</t>
         </is>
       </c>
       <c r="I79" s="6" t="inlineStr">
@@ -4402,10 +4402,10 @@
         </is>
       </c>
       <c r="J79" s="7" t="n">
-        <v>2748</v>
+        <v>4924</v>
       </c>
       <c r="K79" s="8" t="n">
-        <v>137.375</v>
+        <v>246.2222222222222</v>
       </c>
     </row>
     <row r="80">
@@ -4487,11 +4487,11 @@
         </is>
       </c>
       <c r="G81" s="7" t="n">
-        <v>2613</v>
+        <v>3205</v>
       </c>
       <c r="H81" s="6" t="inlineStr">
         <is>
-          <t>8/24</t>
+          <t>9/24</t>
         </is>
       </c>
       <c r="I81" s="6" t="inlineStr">
@@ -4500,10 +4500,10 @@
         </is>
       </c>
       <c r="J81" s="7" t="n">
-        <v>7839</v>
+        <v>8547</v>
       </c>
       <c r="K81" s="8" t="n">
-        <v>326.625</v>
+        <v>356.1111111111111</v>
       </c>
     </row>
     <row r="82">
@@ -4536,11 +4536,11 @@
         </is>
       </c>
       <c r="G82" s="7" t="n">
-        <v>2170</v>
+        <v>1314</v>
       </c>
       <c r="H82" s="6" t="inlineStr">
         <is>
-          <t>15/22</t>
+          <t>16/22</t>
         </is>
       </c>
       <c r="I82" s="6" t="inlineStr">
@@ -4549,10 +4549,10 @@
         </is>
       </c>
       <c r="J82" s="7" t="n">
-        <v>3183</v>
+        <v>1807</v>
       </c>
       <c r="K82" s="8" t="n">
-        <v>144.6666666666667</v>
+        <v>82.125</v>
       </c>
     </row>
     <row r="83">
@@ -4948,52 +4948,52 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="6" t="inlineStr">
+      <c r="A91" s="2" t="inlineStr">
         <is>
           <t>MADURAI SOUTH</t>
         </is>
       </c>
-      <c r="B91" s="6" t="n">
+      <c r="B91" s="3" t="n">
         <v>192</v>
       </c>
-      <c r="C91" s="6" t="inlineStr">
+      <c r="C91" s="3" t="inlineStr">
         <is>
           <t>M.M.GOPISON</t>
         </is>
       </c>
-      <c r="D91" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E91" s="6" t="inlineStr">
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E91" s="3" t="inlineStr">
         <is>
           <t>M.BOOMINATHAN</t>
         </is>
       </c>
-      <c r="F91" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G91" s="7" t="n">
-        <v>12848</v>
-      </c>
-      <c r="H91" s="6" t="inlineStr">
-        <is>
-          <t>12/17</t>
-        </is>
-      </c>
-      <c r="I91" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J91" s="7" t="n">
-        <v>18201</v>
-      </c>
-      <c r="K91" s="8" t="n">
-        <v>1070.666666666667</v>
+      <c r="F91" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G91" s="4" t="n">
+        <v>14180</v>
+      </c>
+      <c r="H91" s="3" t="inlineStr">
+        <is>
+          <t>13/17</t>
+        </is>
+      </c>
+      <c r="I91" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J91" s="4" t="n">
+        <v>18543</v>
+      </c>
+      <c r="K91" s="5" t="n">
+        <v>1090.769230769231</v>
       </c>
     </row>
     <row r="92">
@@ -5222,11 +5222,11 @@
         </is>
       </c>
       <c r="G96" s="7" t="n">
-        <v>8837</v>
+        <v>9581</v>
       </c>
       <c r="H96" s="6" t="inlineStr">
         <is>
-          <t>15/22</t>
+          <t>16/22</t>
         </is>
       </c>
       <c r="I96" s="6" t="inlineStr">
@@ -5235,10 +5235,10 @@
         </is>
       </c>
       <c r="J96" s="7" t="n">
-        <v>12961</v>
+        <v>13174</v>
       </c>
       <c r="K96" s="8" t="n">
-        <v>589.1333333333334</v>
+        <v>598.8125</v>
       </c>
     </row>
     <row r="97">
@@ -5320,11 +5320,11 @@
         </is>
       </c>
       <c r="G98" s="7" t="n">
-        <v>4341</v>
+        <v>3087</v>
       </c>
       <c r="H98" s="6" t="inlineStr">
         <is>
-          <t>14/25</t>
+          <t>15/25</t>
         </is>
       </c>
       <c r="I98" s="6" t="inlineStr">
@@ -5333,10 +5333,10 @@
         </is>
       </c>
       <c r="J98" s="7" t="n">
-        <v>7752</v>
+        <v>5145</v>
       </c>
       <c r="K98" s="8" t="n">
-        <v>310.0714285714286</v>
+        <v>205.8</v>
       </c>
     </row>
     <row r="99">
@@ -5467,11 +5467,11 @@
         </is>
       </c>
       <c r="G101" s="7" t="n">
-        <v>3770</v>
+        <v>3093</v>
       </c>
       <c r="H101" s="6" t="inlineStr">
         <is>
-          <t>17/21</t>
+          <t>18/21</t>
         </is>
       </c>
       <c r="I101" s="6" t="inlineStr">
@@ -5480,10 +5480,10 @@
         </is>
       </c>
       <c r="J101" s="7" t="n">
-        <v>4657</v>
+        <v>3608</v>
       </c>
       <c r="K101" s="8" t="n">
-        <v>221.7647058823529</v>
+        <v>171.8333333333333</v>
       </c>
     </row>
     <row r="102">
@@ -5516,11 +5516,11 @@
         </is>
       </c>
       <c r="G102" s="7" t="n">
-        <v>2380</v>
+        <v>2712</v>
       </c>
       <c r="H102" s="6" t="inlineStr">
         <is>
-          <t>9/26</t>
+          <t>10/26</t>
         </is>
       </c>
       <c r="I102" s="6" t="inlineStr">
@@ -5529,10 +5529,10 @@
         </is>
       </c>
       <c r="J102" s="7" t="n">
-        <v>6876</v>
+        <v>7051</v>
       </c>
       <c r="K102" s="8" t="n">
-        <v>264.4444444444445</v>
+        <v>271.2</v>
       </c>
     </row>
     <row r="103">
@@ -5614,11 +5614,11 @@
         </is>
       </c>
       <c r="G104" s="7" t="n">
-        <v>3092</v>
+        <v>3820</v>
       </c>
       <c r="H104" s="6" t="inlineStr">
         <is>
-          <t>11/21</t>
+          <t>12/21</t>
         </is>
       </c>
       <c r="I104" s="6" t="inlineStr">
@@ -5627,10 +5627,10 @@
         </is>
       </c>
       <c r="J104" s="7" t="n">
-        <v>5903</v>
+        <v>6685</v>
       </c>
       <c r="K104" s="8" t="n">
-        <v>281.0909090909091</v>
+        <v>318.3333333333333</v>
       </c>
     </row>
     <row r="105">
@@ -5663,11 +5663,11 @@
         </is>
       </c>
       <c r="G105" s="7" t="n">
-        <v>6999</v>
+        <v>7815</v>
       </c>
       <c r="H105" s="6" t="inlineStr">
         <is>
-          <t>14/30</t>
+          <t>15/30</t>
         </is>
       </c>
       <c r="I105" s="6" t="inlineStr">
@@ -5676,10 +5676,10 @@
         </is>
       </c>
       <c r="J105" s="7" t="n">
-        <v>14998</v>
+        <v>15630</v>
       </c>
       <c r="K105" s="8" t="n">
-        <v>499.9285714285714</v>
+        <v>521</v>
       </c>
     </row>
     <row r="106">
@@ -5761,11 +5761,11 @@
         </is>
       </c>
       <c r="G107" s="4" t="n">
-        <v>18652</v>
+        <v>19501</v>
       </c>
       <c r="H107" s="3" t="inlineStr">
         <is>
-          <t>12/20</t>
+          <t>13/20</t>
         </is>
       </c>
       <c r="I107" s="3" t="inlineStr">
@@ -5774,10 +5774,10 @@
         </is>
       </c>
       <c r="J107" s="4" t="n">
-        <v>31087</v>
+        <v>30002</v>
       </c>
       <c r="K107" s="5" t="n">
-        <v>1554.333333333333</v>
+        <v>1500.076923076923</v>
       </c>
     </row>
     <row r="108">
@@ -6006,11 +6006,11 @@
         </is>
       </c>
       <c r="G112" s="4" t="n">
-        <v>23555</v>
+        <v>24173</v>
       </c>
       <c r="H112" s="3" t="inlineStr">
         <is>
-          <t>13/25</t>
+          <t>14/25</t>
         </is>
       </c>
       <c r="I112" s="3" t="inlineStr">
@@ -6019,10 +6019,10 @@
         </is>
       </c>
       <c r="J112" s="4" t="n">
-        <v>45298</v>
+        <v>43166</v>
       </c>
       <c r="K112" s="5" t="n">
-        <v>1811.923076923077</v>
+        <v>1726.642857142857</v>
       </c>
     </row>
     <row r="113">
@@ -6104,11 +6104,11 @@
         </is>
       </c>
       <c r="G114" s="7" t="n">
-        <v>13103</v>
+        <v>11972</v>
       </c>
       <c r="H114" s="6" t="inlineStr">
         <is>
-          <t>13/19</t>
+          <t>14/19</t>
         </is>
       </c>
       <c r="I114" s="6" t="inlineStr">
@@ -6117,10 +6117,10 @@
         </is>
       </c>
       <c r="J114" s="7" t="n">
-        <v>19151</v>
+        <v>16248</v>
       </c>
       <c r="K114" s="8" t="n">
-        <v>1007.923076923077</v>
+        <v>855.1428571428571</v>
       </c>
     </row>
     <row r="115">
@@ -6153,11 +6153,11 @@
         </is>
       </c>
       <c r="G115" s="7" t="n">
-        <v>2747</v>
+        <v>3366</v>
       </c>
       <c r="H115" s="6" t="inlineStr">
         <is>
-          <t>8/23</t>
+          <t>9/23</t>
         </is>
       </c>
       <c r="I115" s="6" t="inlineStr">
@@ -6166,10 +6166,10 @@
         </is>
       </c>
       <c r="J115" s="7" t="n">
-        <v>7898</v>
+        <v>8602</v>
       </c>
       <c r="K115" s="8" t="n">
-        <v>343.375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="116">
@@ -6202,11 +6202,11 @@
         </is>
       </c>
       <c r="G116" s="4" t="n">
-        <v>20612</v>
+        <v>22813</v>
       </c>
       <c r="H116" s="3" t="inlineStr">
         <is>
-          <t>11/24</t>
+          <t>12/24</t>
         </is>
       </c>
       <c r="I116" s="3" t="inlineStr">
@@ -6215,10 +6215,10 @@
         </is>
       </c>
       <c r="J116" s="4" t="n">
-        <v>44972</v>
+        <v>45626</v>
       </c>
       <c r="K116" s="5" t="n">
-        <v>1873.818181818182</v>
+        <v>1901.083333333333</v>
       </c>
     </row>
     <row r="117">
@@ -6251,11 +6251,11 @@
         </is>
       </c>
       <c r="G117" s="7" t="n">
-        <v>4491</v>
+        <v>3727</v>
       </c>
       <c r="H117" s="6" t="inlineStr">
         <is>
-          <t>11/26</t>
+          <t>12/26</t>
         </is>
       </c>
       <c r="I117" s="6" t="inlineStr">
@@ -6264,10 +6264,10 @@
         </is>
       </c>
       <c r="J117" s="7" t="n">
-        <v>10615</v>
+        <v>8075</v>
       </c>
       <c r="K117" s="8" t="n">
-        <v>408.2727272727273</v>
+        <v>310.5833333333333</v>
       </c>
     </row>
     <row r="118">
@@ -6300,11 +6300,11 @@
         </is>
       </c>
       <c r="G118" s="4" t="n">
-        <v>18247</v>
+        <v>19449</v>
       </c>
       <c r="H118" s="3" t="inlineStr">
         <is>
-          <t>13/23</t>
+          <t>14/23</t>
         </is>
       </c>
       <c r="I118" s="3" t="inlineStr">
@@ -6313,10 +6313,10 @@
         </is>
       </c>
       <c r="J118" s="4" t="n">
-        <v>32283</v>
+        <v>31952</v>
       </c>
       <c r="K118" s="5" t="n">
-        <v>1403.615384615385</v>
+        <v>1389.214285714286</v>
       </c>
     </row>
     <row r="119">
@@ -6349,11 +6349,11 @@
         </is>
       </c>
       <c r="G119" s="4" t="n">
-        <v>15087</v>
+        <v>17875</v>
       </c>
       <c r="H119" s="3" t="inlineStr">
         <is>
-          <t>10/23</t>
+          <t>11/23</t>
         </is>
       </c>
       <c r="I119" s="3" t="inlineStr">
@@ -6362,10 +6362,10 @@
         </is>
       </c>
       <c r="J119" s="4" t="n">
-        <v>34700</v>
+        <v>37375</v>
       </c>
       <c r="K119" s="5" t="n">
-        <v>1508.7</v>
+        <v>1625</v>
       </c>
     </row>
     <row r="120">
@@ -6447,11 +6447,11 @@
         </is>
       </c>
       <c r="G121" s="4" t="n">
-        <v>19335</v>
+        <v>21627</v>
       </c>
       <c r="H121" s="3" t="inlineStr">
         <is>
-          <t>12/23</t>
+          <t>13/23</t>
         </is>
       </c>
       <c r="I121" s="3" t="inlineStr">
@@ -6460,10 +6460,10 @@
         </is>
       </c>
       <c r="J121" s="4" t="n">
-        <v>37059</v>
+        <v>38263</v>
       </c>
       <c r="K121" s="5" t="n">
-        <v>1611.25</v>
+        <v>1663.615384615385</v>
       </c>
     </row>
     <row r="122">
@@ -6545,11 +6545,11 @@
         </is>
       </c>
       <c r="G123" s="7" t="n">
-        <v>9570</v>
+        <v>8811</v>
       </c>
       <c r="H123" s="6" t="inlineStr">
         <is>
-          <t>15/22</t>
+          <t>16/22</t>
         </is>
       </c>
       <c r="I123" s="6" t="inlineStr">
@@ -6558,10 +6558,10 @@
         </is>
       </c>
       <c r="J123" s="7" t="n">
-        <v>14036</v>
+        <v>12115</v>
       </c>
       <c r="K123" s="8" t="n">
-        <v>638.0000000000001</v>
+        <v>550.6875</v>
       </c>
     </row>
     <row r="124">
@@ -6594,11 +6594,11 @@
         </is>
       </c>
       <c r="G124" s="4" t="n">
-        <v>12313</v>
+        <v>12266</v>
       </c>
       <c r="H124" s="3" t="inlineStr">
         <is>
-          <t>13/35</t>
+          <t>14/35</t>
         </is>
       </c>
       <c r="I124" s="3" t="inlineStr">
@@ -6607,10 +6607,10 @@
         </is>
       </c>
       <c r="J124" s="4" t="n">
-        <v>33150</v>
+        <v>30665</v>
       </c>
       <c r="K124" s="5" t="n">
-        <v>947.1538461538462</v>
+        <v>876.1428571428571</v>
       </c>
     </row>
     <row r="125">
@@ -6643,11 +6643,11 @@
         </is>
       </c>
       <c r="G125" s="4" t="n">
-        <v>18500</v>
+        <v>19916</v>
       </c>
       <c r="H125" s="3" t="inlineStr">
         <is>
-          <t>11/34</t>
+          <t>12/34</t>
         </is>
       </c>
       <c r="I125" s="3" t="inlineStr">
@@ -6656,10 +6656,10 @@
         </is>
       </c>
       <c r="J125" s="4" t="n">
-        <v>57182</v>
+        <v>56429</v>
       </c>
       <c r="K125" s="5" t="n">
-        <v>1681.818181818182</v>
+        <v>1659.666666666667</v>
       </c>
     </row>
     <row r="126">
@@ -6692,11 +6692,11 @@
         </is>
       </c>
       <c r="G126" s="7" t="n">
-        <v>3264</v>
+        <v>4658</v>
       </c>
       <c r="H126" s="6" t="inlineStr">
         <is>
-          <t>13/23</t>
+          <t>14/23</t>
         </is>
       </c>
       <c r="I126" s="6" t="inlineStr">
@@ -6705,10 +6705,10 @@
         </is>
       </c>
       <c r="J126" s="7" t="n">
-        <v>5775</v>
+        <v>7652</v>
       </c>
       <c r="K126" s="8" t="n">
-        <v>251.0769230769231</v>
+        <v>332.7142857142857</v>
       </c>
     </row>
     <row r="127">
@@ -6986,11 +6986,11 @@
         </is>
       </c>
       <c r="G132" s="7" t="n">
-        <v>4459</v>
+        <v>5684</v>
       </c>
       <c r="H132" s="6" t="inlineStr">
         <is>
-          <t>6/23</t>
+          <t>7/23</t>
         </is>
       </c>
       <c r="I132" s="6" t="inlineStr">
@@ -6999,10 +6999,10 @@
         </is>
       </c>
       <c r="J132" s="7" t="n">
-        <v>17093</v>
+        <v>18676</v>
       </c>
       <c r="K132" s="8" t="n">
-        <v>743.1666666666666</v>
+        <v>812</v>
       </c>
     </row>
     <row r="133">
@@ -7026,20 +7026,20 @@
       </c>
       <c r="E133" s="6" t="inlineStr">
         <is>
-          <t>THAMIZHSELVAN. R</t>
+          <t>DR. JAYALAKSHMI. S.T</t>
         </is>
       </c>
       <c r="F133" s="6" t="inlineStr">
         <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
+          <t>Dravida Munnetra Kazhagam</t>
         </is>
       </c>
       <c r="G133" s="7" t="n">
-        <v>4432</v>
+        <v>5750</v>
       </c>
       <c r="H133" s="6" t="inlineStr">
         <is>
-          <t>14/28</t>
+          <t>15/28</t>
         </is>
       </c>
       <c r="I133" s="6" t="inlineStr">
@@ -7048,10 +7048,10 @@
         </is>
       </c>
       <c r="J133" s="7" t="n">
-        <v>8864</v>
+        <v>10733</v>
       </c>
       <c r="K133" s="8" t="n">
-        <v>316.5714285714286</v>
+        <v>383.3333333333333</v>
       </c>
     </row>
     <row r="134">
@@ -7182,11 +7182,11 @@
         </is>
       </c>
       <c r="G136" s="7" t="n">
-        <v>2241</v>
+        <v>1884</v>
       </c>
       <c r="H136" s="6" t="inlineStr">
         <is>
-          <t>8/26</t>
+          <t>9/26</t>
         </is>
       </c>
       <c r="I136" s="6" t="inlineStr">
@@ -7195,10 +7195,10 @@
         </is>
       </c>
       <c r="J136" s="7" t="n">
-        <v>7283</v>
+        <v>5443</v>
       </c>
       <c r="K136" s="8" t="n">
-        <v>280.125</v>
+        <v>209.3333333333333</v>
       </c>
     </row>
     <row r="137">
@@ -7506,30 +7506,30 @@
       </c>
       <c r="C143" s="6" t="inlineStr">
         <is>
+          <t>V. MUTHURAJA</t>
+        </is>
+      </c>
+      <c r="D143" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E143" s="6" t="inlineStr">
+        <is>
           <t>K.M. SHARIFF</t>
         </is>
       </c>
-      <c r="D143" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E143" s="6" t="inlineStr">
-        <is>
-          <t>V. MUTHURAJA</t>
-        </is>
-      </c>
       <c r="F143" s="6" t="inlineStr">
         <is>
-          <t>Dravida Munnetra Kazhagam</t>
+          <t>Tamilaga Vettri Kazhagam</t>
         </is>
       </c>
       <c r="G143" s="7" t="n">
-        <v>410</v>
+        <v>675</v>
       </c>
       <c r="H143" s="6" t="inlineStr">
         <is>
-          <t>9/22</t>
+          <t>10/22</t>
         </is>
       </c>
       <c r="I143" s="6" t="inlineStr">
@@ -7538,59 +7538,59 @@
         </is>
       </c>
       <c r="J143" s="7" t="n">
-        <v>1002</v>
+        <v>1485</v>
       </c>
       <c r="K143" s="8" t="n">
-        <v>45.55555555555556</v>
+        <v>67.5</v>
       </c>
     </row>
     <row r="144">
-      <c r="A144" s="6" t="inlineStr">
+      <c r="A144" s="2" t="inlineStr">
         <is>
           <t>RADHAPURAM</t>
         </is>
       </c>
-      <c r="B144" s="6" t="n">
+      <c r="B144" s="3" t="n">
         <v>228</v>
       </c>
-      <c r="C144" s="6" t="inlineStr">
+      <c r="C144" s="3" t="inlineStr">
         <is>
           <t>DR.SATHISH CHRISTOPHER</t>
         </is>
       </c>
-      <c r="D144" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E144" s="6" t="inlineStr">
+      <c r="D144" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E144" s="3" t="inlineStr">
         <is>
           <t>APPAVU.M</t>
         </is>
       </c>
-      <c r="F144" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G144" s="7" t="n">
-        <v>6824</v>
-      </c>
-      <c r="H144" s="6" t="inlineStr">
-        <is>
-          <t>17/24</t>
-        </is>
-      </c>
-      <c r="I144" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J144" s="7" t="n">
-        <v>9634</v>
-      </c>
-      <c r="K144" s="8" t="n">
-        <v>401.4117647058824</v>
+      <c r="F144" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G144" s="4" t="n">
+        <v>6870</v>
+      </c>
+      <c r="H144" s="3" t="inlineStr">
+        <is>
+          <t>18/24</t>
+        </is>
+      </c>
+      <c r="I144" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J144" s="4" t="n">
+        <v>9160</v>
+      </c>
+      <c r="K144" s="5" t="n">
+        <v>381.6666666666667</v>
       </c>
     </row>
     <row r="145">
@@ -7643,52 +7643,52 @@
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="2" t="inlineStr">
+      <c r="A146" s="6" t="inlineStr">
         <is>
           <t>RAMANATHAPURAM</t>
         </is>
       </c>
-      <c r="B146" s="3" t="n">
+      <c r="B146" s="6" t="n">
         <v>211</v>
       </c>
-      <c r="C146" s="3" t="inlineStr">
+      <c r="C146" s="6" t="inlineStr">
         <is>
           <t>KATHARBATCHA MUTHURAMALINGAM</t>
         </is>
       </c>
-      <c r="D146" s="3" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E146" s="3" t="inlineStr">
+      <c r="D146" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E146" s="6" t="inlineStr">
         <is>
           <t>SHAHUL HAMEED</t>
         </is>
       </c>
-      <c r="F146" s="3" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G146" s="4" t="n">
-        <v>11898</v>
-      </c>
-      <c r="H146" s="3" t="inlineStr">
-        <is>
-          <t>17/29</t>
-        </is>
-      </c>
-      <c r="I146" s="3" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J146" s="4" t="n">
-        <v>20297</v>
-      </c>
-      <c r="K146" s="5" t="n">
-        <v>699.8823529411765</v>
+      <c r="F146" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G146" s="7" t="n">
+        <v>11440</v>
+      </c>
+      <c r="H146" s="6" t="inlineStr">
+        <is>
+          <t>18/29</t>
+        </is>
+      </c>
+      <c r="I146" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J146" s="7" t="n">
+        <v>18431</v>
+      </c>
+      <c r="K146" s="8" t="n">
+        <v>635.5555555555555</v>
       </c>
     </row>
     <row r="147">
@@ -7721,11 +7721,11 @@
         </is>
       </c>
       <c r="G147" s="7" t="n">
-        <v>6605</v>
+        <v>6308</v>
       </c>
       <c r="H147" s="6" t="inlineStr">
         <is>
-          <t>9/22</t>
+          <t>10/22</t>
         </is>
       </c>
       <c r="I147" s="6" t="inlineStr">
@@ -7734,10 +7734,10 @@
         </is>
       </c>
       <c r="J147" s="7" t="n">
-        <v>16146</v>
+        <v>13878</v>
       </c>
       <c r="K147" s="8" t="n">
-        <v>733.8888888888889</v>
+        <v>630.8</v>
       </c>
     </row>
     <row r="148">
@@ -7819,11 +7819,11 @@
         </is>
       </c>
       <c r="G149" s="7" t="n">
-        <v>503</v>
+        <v>1211</v>
       </c>
       <c r="H149" s="6" t="inlineStr">
         <is>
-          <t>7/25</t>
+          <t>8/25</t>
         </is>
       </c>
       <c r="I149" s="6" t="inlineStr">
@@ -7832,10 +7832,10 @@
         </is>
       </c>
       <c r="J149" s="7" t="n">
-        <v>1796</v>
+        <v>3784</v>
       </c>
       <c r="K149" s="8" t="n">
-        <v>71.85714285714285</v>
+        <v>151.375</v>
       </c>
     </row>
     <row r="150">
@@ -7868,11 +7868,11 @@
         </is>
       </c>
       <c r="G150" s="7" t="n">
-        <v>11340</v>
+        <v>12633</v>
       </c>
       <c r="H150" s="6" t="inlineStr">
         <is>
-          <t>8/14</t>
+          <t>9/14</t>
         </is>
       </c>
       <c r="I150" s="6" t="inlineStr">
@@ -7881,10 +7881,10 @@
         </is>
       </c>
       <c r="J150" s="7" t="n">
-        <v>19845</v>
+        <v>19651</v>
       </c>
       <c r="K150" s="8" t="n">
-        <v>1417.5</v>
+        <v>1403.666666666667</v>
       </c>
     </row>
     <row r="151">
@@ -7917,11 +7917,11 @@
         </is>
       </c>
       <c r="G151" s="4" t="n">
-        <v>15009</v>
+        <v>16067</v>
       </c>
       <c r="H151" s="3" t="inlineStr">
         <is>
-          <t>9/21</t>
+          <t>10/21</t>
         </is>
       </c>
       <c r="I151" s="3" t="inlineStr">
@@ -7930,10 +7930,10 @@
         </is>
       </c>
       <c r="J151" s="4" t="n">
-        <v>35021</v>
+        <v>33741</v>
       </c>
       <c r="K151" s="5" t="n">
-        <v>1667.666666666667</v>
+        <v>1606.7</v>
       </c>
     </row>
     <row r="152">
@@ -8113,11 +8113,11 @@
         </is>
       </c>
       <c r="G155" s="7" t="n">
-        <v>3035</v>
+        <v>1530</v>
       </c>
       <c r="H155" s="6" t="inlineStr">
         <is>
-          <t>12/23</t>
+          <t>13/23</t>
         </is>
       </c>
       <c r="I155" s="6" t="inlineStr">
@@ -8126,10 +8126,10 @@
         </is>
       </c>
       <c r="J155" s="7" t="n">
-        <v>5817</v>
+        <v>2707</v>
       </c>
       <c r="K155" s="8" t="n">
-        <v>252.9166666666667</v>
+        <v>117.6923076923077</v>
       </c>
     </row>
     <row r="156">
@@ -8211,11 +8211,11 @@
         </is>
       </c>
       <c r="G157" s="7" t="n">
-        <v>812</v>
+        <v>3516</v>
       </c>
       <c r="H157" s="6" t="inlineStr">
         <is>
-          <t>12/25</t>
+          <t>13/25</t>
         </is>
       </c>
       <c r="I157" s="6" t="inlineStr">
@@ -8224,10 +8224,10 @@
         </is>
       </c>
       <c r="J157" s="7" t="n">
-        <v>1692</v>
+        <v>6762</v>
       </c>
       <c r="K157" s="8" t="n">
-        <v>67.66666666666667</v>
+        <v>270.4615384615385</v>
       </c>
     </row>
     <row r="158">
@@ -8358,11 +8358,11 @@
         </is>
       </c>
       <c r="G160" s="7" t="n">
-        <v>311</v>
+        <v>385</v>
       </c>
       <c r="H160" s="6" t="inlineStr">
         <is>
-          <t>5/19</t>
+          <t>6/19</t>
         </is>
       </c>
       <c r="I160" s="6" t="inlineStr">
@@ -8371,10 +8371,10 @@
         </is>
       </c>
       <c r="J160" s="7" t="n">
-        <v>1182</v>
+        <v>1219</v>
       </c>
       <c r="K160" s="8" t="n">
-        <v>62.2</v>
+        <v>64.16666666666667</v>
       </c>
     </row>
     <row r="161">
@@ -8799,11 +8799,11 @@
         </is>
       </c>
       <c r="G169" s="7" t="n">
-        <v>955</v>
+        <v>652</v>
       </c>
       <c r="H169" s="6" t="inlineStr">
         <is>
-          <t>15/21</t>
+          <t>16/21</t>
         </is>
       </c>
       <c r="I169" s="6" t="inlineStr">
@@ -8812,10 +8812,10 @@
         </is>
       </c>
       <c r="J169" s="7" t="n">
-        <v>1337</v>
+        <v>856</v>
       </c>
       <c r="K169" s="8" t="n">
-        <v>63.66666666666666</v>
+        <v>40.75</v>
       </c>
     </row>
     <row r="170">
@@ -8946,11 +8946,11 @@
         </is>
       </c>
       <c r="G172" s="4" t="n">
-        <v>15769</v>
+        <v>16215</v>
       </c>
       <c r="H172" s="3" t="inlineStr">
         <is>
-          <t>18/34</t>
+          <t>19/34</t>
         </is>
       </c>
       <c r="I172" s="3" t="inlineStr">
@@ -8959,10 +8959,10 @@
         </is>
       </c>
       <c r="J172" s="4" t="n">
-        <v>29786</v>
+        <v>29016</v>
       </c>
       <c r="K172" s="5" t="n">
-        <v>876.0555555555555</v>
+        <v>853.421052631579</v>
       </c>
     </row>
     <row r="173">
@@ -9015,52 +9015,52 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="6" t="inlineStr">
+      <c r="A174" s="13" t="inlineStr">
         <is>
           <t>THALLI</t>
         </is>
       </c>
-      <c r="B174" s="6" t="n">
+      <c r="B174" s="14" t="n">
         <v>56</v>
       </c>
-      <c r="C174" s="6" t="inlineStr">
+      <c r="C174" s="14" t="inlineStr">
+        <is>
+          <t>RAMACHANDRAN. T</t>
+        </is>
+      </c>
+      <c r="D174" s="14" t="inlineStr">
+        <is>
+          <t>Communist Party of India</t>
+        </is>
+      </c>
+      <c r="E174" s="14" t="inlineStr">
         <is>
           <t>DR.NAGESH KUMAR. C</t>
         </is>
       </c>
-      <c r="D174" s="6" t="inlineStr">
+      <c r="F174" s="14" t="inlineStr">
         <is>
           <t>Bharatiya Janata Party</t>
         </is>
       </c>
-      <c r="E174" s="6" t="inlineStr">
-        <is>
-          <t>RAMACHANDRAN. T</t>
-        </is>
-      </c>
-      <c r="F174" s="6" t="inlineStr">
-        <is>
-          <t>Communist Party of India</t>
-        </is>
-      </c>
-      <c r="G174" s="7" t="n">
-        <v>1235</v>
-      </c>
-      <c r="H174" s="6" t="inlineStr">
-        <is>
-          <t>7/24</t>
-        </is>
-      </c>
-      <c r="I174" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J174" s="7" t="n">
-        <v>4234</v>
-      </c>
-      <c r="K174" s="8" t="n">
-        <v>176.4285714285714</v>
+      <c r="G174" s="15" t="n">
+        <v>30</v>
+      </c>
+      <c r="H174" s="14" t="inlineStr">
+        <is>
+          <t>8/24</t>
+        </is>
+      </c>
+      <c r="I174" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J174" s="15" t="n">
+        <v>90</v>
+      </c>
+      <c r="K174" s="16" t="n">
+        <v>3.75</v>
       </c>
     </row>
     <row r="175">
@@ -9093,11 +9093,11 @@
         </is>
       </c>
       <c r="G175" s="4" t="n">
-        <v>16999</v>
+        <v>17272</v>
       </c>
       <c r="H175" s="3" t="inlineStr">
         <is>
-          <t>20/23</t>
+          <t>21/23</t>
         </is>
       </c>
       <c r="I175" s="3" t="inlineStr">
@@ -9106,10 +9106,10 @@
         </is>
       </c>
       <c r="J175" s="4" t="n">
-        <v>19549</v>
+        <v>18917</v>
       </c>
       <c r="K175" s="5" t="n">
-        <v>849.95</v>
+        <v>822.4761904761905</v>
       </c>
     </row>
     <row r="176">
@@ -9142,11 +9142,11 @@
         </is>
       </c>
       <c r="G176" s="4" t="n">
-        <v>15408</v>
+        <v>14112</v>
       </c>
       <c r="H176" s="3" t="inlineStr">
         <is>
-          <t>9/17</t>
+          <t>10/17</t>
         </is>
       </c>
       <c r="I176" s="3" t="inlineStr">
@@ -9155,10 +9155,10 @@
         </is>
       </c>
       <c r="J176" s="4" t="n">
-        <v>29104</v>
+        <v>23990</v>
       </c>
       <c r="K176" s="5" t="n">
-        <v>1712</v>
+        <v>1411.2</v>
       </c>
     </row>
     <row r="177">
@@ -9583,11 +9583,11 @@
         </is>
       </c>
       <c r="G185" s="7" t="n">
-        <v>423</v>
+        <v>601</v>
       </c>
       <c r="H185" s="6" t="inlineStr">
         <is>
-          <t>6/23</t>
+          <t>7/23</t>
         </is>
       </c>
       <c r="I185" s="6" t="inlineStr">
@@ -9596,10 +9596,10 @@
         </is>
       </c>
       <c r="J185" s="7" t="n">
-        <v>1622</v>
+        <v>1975</v>
       </c>
       <c r="K185" s="8" t="n">
-        <v>70.5</v>
+        <v>85.85714285714286</v>
       </c>
     </row>
     <row r="186">
@@ -9632,11 +9632,11 @@
         </is>
       </c>
       <c r="G186" s="7" t="n">
-        <v>6761</v>
+        <v>7966</v>
       </c>
       <c r="H186" s="6" t="inlineStr">
         <is>
-          <t>9/24</t>
+          <t>10/24</t>
         </is>
       </c>
       <c r="I186" s="6" t="inlineStr">
@@ -9645,10 +9645,10 @@
         </is>
       </c>
       <c r="J186" s="7" t="n">
-        <v>18029</v>
+        <v>19118</v>
       </c>
       <c r="K186" s="8" t="n">
-        <v>751.2222222222222</v>
+        <v>796.6</v>
       </c>
     </row>
     <row r="187">
@@ -10220,11 +10220,11 @@
         </is>
       </c>
       <c r="G198" s="7" t="n">
-        <v>1019</v>
+        <v>1914</v>
       </c>
       <c r="H198" s="6" t="inlineStr">
         <is>
-          <t>6/21</t>
+          <t>7/21</t>
         </is>
       </c>
       <c r="I198" s="6" t="inlineStr">
@@ -10233,59 +10233,59 @@
         </is>
       </c>
       <c r="J198" s="7" t="n">
-        <v>3566</v>
+        <v>5742</v>
       </c>
       <c r="K198" s="8" t="n">
-        <v>169.8333333333333</v>
+        <v>273.4285714285714</v>
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="6" t="inlineStr">
+      <c r="A199" s="13" t="inlineStr">
         <is>
           <t>TIRUKKOYILUR</t>
         </is>
       </c>
-      <c r="B199" s="6" t="n">
+      <c r="B199" s="14" t="n">
         <v>76</v>
       </c>
-      <c r="C199" s="6" t="inlineStr">
+      <c r="C199" s="14" t="inlineStr">
+        <is>
+          <t>VIJAY R BARANIBALAAJI</t>
+        </is>
+      </c>
+      <c r="D199" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E199" s="14" t="inlineStr">
         <is>
           <t>PALANISAMY S</t>
         </is>
       </c>
-      <c r="D199" s="6" t="inlineStr">
+      <c r="F199" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E199" s="6" t="inlineStr">
-        <is>
-          <t>VIJAY R BARANIBALAAJI</t>
-        </is>
-      </c>
-      <c r="F199" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G199" s="7" t="n">
-        <v>799</v>
-      </c>
-      <c r="H199" s="6" t="inlineStr">
-        <is>
-          <t>9/24</t>
-        </is>
-      </c>
-      <c r="I199" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J199" s="7" t="n">
-        <v>2131</v>
-      </c>
-      <c r="K199" s="8" t="n">
-        <v>88.77777777777777</v>
+      <c r="G199" s="15" t="n">
+        <v>54</v>
+      </c>
+      <c r="H199" s="14" t="inlineStr">
+        <is>
+          <t>10/24</t>
+        </is>
+      </c>
+      <c r="I199" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J199" s="15" t="n">
+        <v>130</v>
+      </c>
+      <c r="K199" s="16" t="n">
+        <v>5.4</v>
       </c>
     </row>
     <row r="200">
@@ -10416,11 +10416,11 @@
         </is>
       </c>
       <c r="G202" s="7" t="n">
-        <v>4531</v>
+        <v>4603</v>
       </c>
       <c r="H202" s="6" t="inlineStr">
         <is>
-          <t>8/27</t>
+          <t>9/27</t>
         </is>
       </c>
       <c r="I202" s="6" t="inlineStr">
@@ -10429,10 +10429,10 @@
         </is>
       </c>
       <c r="J202" s="7" t="n">
-        <v>15292</v>
+        <v>13809</v>
       </c>
       <c r="K202" s="8" t="n">
-        <v>566.375</v>
+        <v>511.4444444444445</v>
       </c>
     </row>
     <row r="203">
@@ -10593,30 +10593,30 @@
       </c>
       <c r="C206" s="10" t="inlineStr">
         <is>
+          <t>M.KEERTHIKA</t>
+        </is>
+      </c>
+      <c r="D206" s="10" t="inlineStr">
+        <is>
+          <t>All India Anna Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E206" s="10" t="inlineStr">
+        <is>
           <t>RAJEEV</t>
         </is>
       </c>
-      <c r="D206" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E206" s="10" t="inlineStr">
-        <is>
-          <t>M.KEERTHIKA</t>
-        </is>
-      </c>
       <c r="F206" s="10" t="inlineStr">
         <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
+          <t>Tamilaga Vettri Kazhagam</t>
         </is>
       </c>
       <c r="G206" s="11" t="n">
-        <v>439</v>
+        <v>482</v>
       </c>
       <c r="H206" s="10" t="inlineStr">
         <is>
-          <t>15/27</t>
+          <t>16/27</t>
         </is>
       </c>
       <c r="I206" s="10" t="inlineStr">
@@ -10625,10 +10625,10 @@
         </is>
       </c>
       <c r="J206" s="11" t="n">
-        <v>790</v>
+        <v>813</v>
       </c>
       <c r="K206" s="12" t="n">
-        <v>29.26666666666667</v>
+        <v>30.125</v>
       </c>
     </row>
     <row r="207">
@@ -10710,11 +10710,11 @@
         </is>
       </c>
       <c r="G208" s="7" t="n">
-        <v>2157</v>
+        <v>2253</v>
       </c>
       <c r="H208" s="6" t="inlineStr">
         <is>
-          <t>7/20</t>
+          <t>8/20</t>
         </is>
       </c>
       <c r="I208" s="6" t="inlineStr">
@@ -10723,59 +10723,59 @@
         </is>
       </c>
       <c r="J208" s="7" t="n">
-        <v>6163</v>
+        <v>5632</v>
       </c>
       <c r="K208" s="8" t="n">
-        <v>308.1428571428572</v>
+        <v>281.625</v>
       </c>
     </row>
     <row r="209">
-      <c r="A209" s="6" t="inlineStr">
+      <c r="A209" s="9" t="inlineStr">
         <is>
           <t>UDHAGAMANDALAM</t>
         </is>
       </c>
-      <c r="B209" s="6" t="n">
+      <c r="B209" s="10" t="n">
         <v>108</v>
       </c>
-      <c r="C209" s="6" t="inlineStr">
+      <c r="C209" s="10" t="inlineStr">
         <is>
           <t>IBRAHIM.R</t>
         </is>
       </c>
-      <c r="D209" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E209" s="6" t="inlineStr">
+      <c r="D209" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E209" s="10" t="inlineStr">
         <is>
           <t>BHOJARAJAN.M</t>
         </is>
       </c>
-      <c r="F209" s="6" t="inlineStr">
+      <c r="F209" s="10" t="inlineStr">
         <is>
           <t>Bharatiya Janata Party</t>
         </is>
       </c>
-      <c r="G209" s="7" t="n">
-        <v>1130</v>
-      </c>
-      <c r="H209" s="6" t="inlineStr">
-        <is>
-          <t>15/19</t>
-        </is>
-      </c>
-      <c r="I209" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J209" s="7" t="n">
-        <v>1431</v>
-      </c>
-      <c r="K209" s="8" t="n">
-        <v>75.33333333333333</v>
+      <c r="G209" s="11" t="n">
+        <v>495</v>
+      </c>
+      <c r="H209" s="10" t="inlineStr">
+        <is>
+          <t>16/19</t>
+        </is>
+      </c>
+      <c r="I209" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J209" s="11" t="n">
+        <v>588</v>
+      </c>
+      <c r="K209" s="12" t="n">
+        <v>30.9375</v>
       </c>
     </row>
     <row r="210">
@@ -11200,11 +11200,11 @@
         </is>
       </c>
       <c r="G218" s="7" t="n">
-        <v>2445</v>
+        <v>1943</v>
       </c>
       <c r="H218" s="6" t="inlineStr">
         <is>
-          <t>9/22</t>
+          <t>10/22</t>
         </is>
       </c>
       <c r="I218" s="6" t="inlineStr">
@@ -11213,10 +11213,10 @@
         </is>
       </c>
       <c r="J218" s="7" t="n">
-        <v>5977</v>
+        <v>4275</v>
       </c>
       <c r="K218" s="8" t="n">
-        <v>271.6666666666667</v>
+        <v>194.3</v>
       </c>
     </row>
     <row r="219">
@@ -11347,11 +11347,11 @@
         </is>
       </c>
       <c r="G221" s="7" t="n">
-        <v>5406</v>
+        <v>5824</v>
       </c>
       <c r="H221" s="6" t="inlineStr">
         <is>
-          <t>9/24</t>
+          <t>10/24</t>
         </is>
       </c>
       <c r="I221" s="6" t="inlineStr">
@@ -11360,10 +11360,10 @@
         </is>
       </c>
       <c r="J221" s="7" t="n">
-        <v>14416</v>
+        <v>13978</v>
       </c>
       <c r="K221" s="8" t="n">
-        <v>600.6666666666666</v>
+        <v>582.4</v>
       </c>
     </row>
     <row r="222">
@@ -11445,11 +11445,11 @@
         </is>
       </c>
       <c r="G223" s="4" t="n">
-        <v>16428</v>
+        <v>19004</v>
       </c>
       <c r="H223" s="3" t="inlineStr">
         <is>
-          <t>10/23</t>
+          <t>11/23</t>
         </is>
       </c>
       <c r="I223" s="3" t="inlineStr">
@@ -11458,10 +11458,10 @@
         </is>
       </c>
       <c r="J223" s="4" t="n">
-        <v>37784</v>
+        <v>39736</v>
       </c>
       <c r="K223" s="5" t="n">
-        <v>1642.8</v>
+        <v>1727.636363636364</v>
       </c>
     </row>
     <row r="224">
@@ -11494,11 +11494,11 @@
         </is>
       </c>
       <c r="G224" s="7" t="n">
-        <v>5610</v>
+        <v>4058</v>
       </c>
       <c r="H224" s="6" t="inlineStr">
         <is>
-          <t>9/20</t>
+          <t>10/21</t>
         </is>
       </c>
       <c r="I224" s="6" t="inlineStr">
@@ -11507,10 +11507,10 @@
         </is>
       </c>
       <c r="J224" s="7" t="n">
-        <v>12467</v>
+        <v>8522</v>
       </c>
       <c r="K224" s="8" t="n">
-        <v>623.3333333333334</v>
+        <v>405.8</v>
       </c>
     </row>
     <row r="225">
@@ -11690,11 +11690,11 @@
         </is>
       </c>
       <c r="G228" s="4" t="n">
-        <v>12286</v>
+        <v>12456</v>
       </c>
       <c r="H228" s="3" t="inlineStr">
         <is>
-          <t>9/22</t>
+          <t>10/22</t>
         </is>
       </c>
       <c r="I228" s="3" t="inlineStr">
@@ -11703,10 +11703,10 @@
         </is>
       </c>
       <c r="J228" s="4" t="n">
-        <v>30032</v>
+        <v>27403</v>
       </c>
       <c r="K228" s="5" t="n">
-        <v>1365.111111111111</v>
+        <v>1245.6</v>
       </c>
     </row>
     <row r="229">
@@ -11837,11 +11837,11 @@
         </is>
       </c>
       <c r="G231" s="4" t="n">
-        <v>19764</v>
+        <v>23773</v>
       </c>
       <c r="H231" s="3" t="inlineStr">
         <is>
-          <t>7/20</t>
+          <t>8/20</t>
         </is>
       </c>
       <c r="I231" s="3" t="inlineStr">
@@ -11850,10 +11850,10 @@
         </is>
       </c>
       <c r="J231" s="4" t="n">
-        <v>56469</v>
+        <v>59432</v>
       </c>
       <c r="K231" s="5" t="n">
-        <v>2823.428571428572</v>
+        <v>2971.625</v>
       </c>
     </row>
     <row r="232">

</xml_diff>

<commit_message>
Update election results snapshot (49.6% counted)
TVK 108, AIADMK 55, DMK 52. DMK gained 3 seats this round. 7 lead
changes; BJP took UDHAGAMANDALAM, DMK took NAGERCOIL. 12 seats in play.

https://claude.ai/code/session_01MizbUy44JG5sXyvaf3Wekb
</commit_message>
<xml_diff>
--- a/tn_election_results_may2026.xlsx
+++ b/tn_election_results_may2026.xlsx
@@ -685,52 +685,52 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>ALANGULAM</t>
         </is>
       </c>
-      <c r="B4" s="10" t="n">
+      <c r="B4" s="6" t="n">
         <v>223</v>
       </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>K R P PRABAKARAN</t>
         </is>
       </c>
-      <c r="D4" s="10" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>PAUL MANOJ PANDIAN</t>
         </is>
       </c>
-      <c r="F4" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G4" s="11" t="n">
-        <v>291</v>
-      </c>
-      <c r="H4" s="10" t="inlineStr">
-        <is>
-          <t>14/24</t>
-        </is>
-      </c>
-      <c r="I4" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J4" s="11" t="n">
-        <v>499</v>
-      </c>
-      <c r="K4" s="12" t="n">
-        <v>20.78571428571428</v>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>719</v>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>15/24</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J4" s="7" t="n">
+        <v>1150</v>
+      </c>
+      <c r="K4" s="8" t="n">
+        <v>47.93333333333333</v>
       </c>
     </row>
     <row r="5">
@@ -763,11 +763,11 @@
         </is>
       </c>
       <c r="G5" s="7" t="n">
-        <v>7002</v>
+        <v>7892</v>
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>15/23</t>
+          <t>16/23</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr">
@@ -776,10 +776,10 @@
         </is>
       </c>
       <c r="J5" s="7" t="n">
-        <v>10736</v>
+        <v>11345</v>
       </c>
       <c r="K5" s="8" t="n">
-        <v>466.8</v>
+        <v>493.25</v>
       </c>
     </row>
     <row r="6">
@@ -1008,11 +1008,11 @@
         </is>
       </c>
       <c r="G10" s="4" t="n">
-        <v>16817</v>
+        <v>18473</v>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>15/20</t>
+          <t>16/20</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
@@ -1021,10 +1021,10 @@
         </is>
       </c>
       <c r="J10" s="4" t="n">
-        <v>22423</v>
+        <v>23091</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>1121.133333333333</v>
+        <v>1154.5625</v>
       </c>
     </row>
     <row r="11">
@@ -1106,11 +1106,11 @@
         </is>
       </c>
       <c r="G12" s="4" t="n">
-        <v>15833</v>
+        <v>17178</v>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>14/21</t>
+          <t>15/21</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
@@ -1119,10 +1119,10 @@
         </is>
       </c>
       <c r="J12" s="4" t="n">
-        <v>23749</v>
+        <v>24049</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1130.928571428571</v>
+        <v>1145.2</v>
       </c>
     </row>
     <row r="13">
@@ -1204,11 +1204,11 @@
         </is>
       </c>
       <c r="G14" s="4" t="n">
-        <v>11720</v>
+        <v>12442</v>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>10/22</t>
+          <t>11/22</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
@@ -1217,10 +1217,10 @@
         </is>
       </c>
       <c r="J14" s="4" t="n">
-        <v>25784</v>
+        <v>24884</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>1172</v>
+        <v>1131.090909090909</v>
       </c>
     </row>
     <row r="15">
@@ -1400,11 +1400,11 @@
         </is>
       </c>
       <c r="G18" s="7" t="n">
-        <v>2937</v>
+        <v>3996</v>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>10/20</t>
+          <t>11/20</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr">
@@ -1413,10 +1413,10 @@
         </is>
       </c>
       <c r="J18" s="7" t="n">
-        <v>5874</v>
+        <v>7265</v>
       </c>
       <c r="K18" s="8" t="n">
-        <v>293.7</v>
+        <v>363.2727272727273</v>
       </c>
     </row>
     <row r="19">
@@ -1449,11 +1449,11 @@
         </is>
       </c>
       <c r="G19" s="4" t="n">
-        <v>10746</v>
+        <v>11601</v>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>10/25</t>
+          <t>11/25</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -1462,10 +1462,10 @@
         </is>
       </c>
       <c r="J19" s="4" t="n">
-        <v>26865</v>
+        <v>26366</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>1074.6</v>
+        <v>1054.636363636364</v>
       </c>
     </row>
     <row r="20">
@@ -1743,11 +1743,11 @@
         </is>
       </c>
       <c r="G25" s="7" t="n">
-        <v>1552</v>
+        <v>2156</v>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>12/24</t>
+          <t>13/24</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
@@ -1756,10 +1756,10 @@
         </is>
       </c>
       <c r="J25" s="7" t="n">
-        <v>3104</v>
+        <v>3980</v>
       </c>
       <c r="K25" s="8" t="n">
-        <v>129.3333333333333</v>
+        <v>165.8461538461538</v>
       </c>
     </row>
     <row r="26">
@@ -1939,11 +1939,11 @@
         </is>
       </c>
       <c r="G29" s="7" t="n">
-        <v>2408</v>
+        <v>3126</v>
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>7/25</t>
+          <t>8/25</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
@@ -1952,10 +1952,10 @@
         </is>
       </c>
       <c r="J29" s="7" t="n">
-        <v>8600</v>
+        <v>9769</v>
       </c>
       <c r="K29" s="8" t="n">
-        <v>343.9999999999999</v>
+        <v>390.75</v>
       </c>
     </row>
     <row r="30">
@@ -1988,11 +1988,11 @@
         </is>
       </c>
       <c r="G30" s="7" t="n">
-        <v>1048</v>
+        <v>839</v>
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>8/17</t>
+          <t>9/17</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
@@ -2001,10 +2001,10 @@
         </is>
       </c>
       <c r="J30" s="7" t="n">
-        <v>2227</v>
+        <v>1585</v>
       </c>
       <c r="K30" s="8" t="n">
-        <v>131</v>
+        <v>93.22222222222223</v>
       </c>
     </row>
     <row r="31">
@@ -2037,11 +2037,11 @@
         </is>
       </c>
       <c r="G31" s="4" t="n">
-        <v>16511</v>
+        <v>18046</v>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>19/24</t>
+          <t>20/24</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -2050,10 +2050,10 @@
         </is>
       </c>
       <c r="J31" s="4" t="n">
-        <v>20856</v>
+        <v>21655</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>869</v>
+        <v>902.3</v>
       </c>
     </row>
     <row r="32">
@@ -2116,30 +2116,30 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
+          <t>THAMIMUN ANSARI. M</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
           <t>PANDIAN. K.A</t>
         </is>
       </c>
-      <c r="D33" s="6" t="inlineStr">
+      <c r="F33" s="6" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E33" s="6" t="inlineStr">
-        <is>
-          <t>THAMIMUN ANSARI. M</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
       <c r="G33" s="7" t="n">
-        <v>436</v>
+        <v>915</v>
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>9/22</t>
+          <t>10/22</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
@@ -2148,10 +2148,10 @@
         </is>
       </c>
       <c r="J33" s="7" t="n">
-        <v>1066</v>
+        <v>2013</v>
       </c>
       <c r="K33" s="8" t="n">
-        <v>48.44444444444444</v>
+        <v>91.5</v>
       </c>
     </row>
     <row r="34">
@@ -2282,11 +2282,11 @@
         </is>
       </c>
       <c r="G36" s="7" t="n">
-        <v>3373</v>
+        <v>4613</v>
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>7/23</t>
+          <t>8/23</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
@@ -2295,10 +2295,10 @@
         </is>
       </c>
       <c r="J36" s="7" t="n">
-        <v>11083</v>
+        <v>13262</v>
       </c>
       <c r="K36" s="8" t="n">
-        <v>481.8571428571428</v>
+        <v>576.625</v>
       </c>
     </row>
     <row r="37">
@@ -2478,11 +2478,11 @@
         </is>
       </c>
       <c r="G40" s="7" t="n">
-        <v>9057</v>
+        <v>9605</v>
       </c>
       <c r="H40" s="6" t="inlineStr">
         <is>
-          <t>14/23</t>
+          <t>15/23</t>
         </is>
       </c>
       <c r="I40" s="6" t="inlineStr">
@@ -2491,10 +2491,10 @@
         </is>
       </c>
       <c r="J40" s="7" t="n">
-        <v>14879</v>
+        <v>14728</v>
       </c>
       <c r="K40" s="8" t="n">
-        <v>646.9285714285714</v>
+        <v>640.3333333333334</v>
       </c>
     </row>
     <row r="41">
@@ -2527,11 +2527,11 @@
         </is>
       </c>
       <c r="G41" s="7" t="n">
-        <v>6228</v>
+        <v>6186</v>
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>13/23</t>
+          <t>14/23</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr">
@@ -2540,10 +2540,10 @@
         </is>
       </c>
       <c r="J41" s="7" t="n">
-        <v>11019</v>
+        <v>10163</v>
       </c>
       <c r="K41" s="8" t="n">
-        <v>479.0769230769232</v>
+        <v>441.8571428571428</v>
       </c>
     </row>
     <row r="42">
@@ -2576,11 +2576,11 @@
         </is>
       </c>
       <c r="G42" s="7" t="n">
-        <v>1638</v>
+        <v>1093</v>
       </c>
       <c r="H42" s="6" t="inlineStr">
         <is>
-          <t>13/24</t>
+          <t>14/24</t>
         </is>
       </c>
       <c r="I42" s="6" t="inlineStr">
@@ -2589,10 +2589,10 @@
         </is>
       </c>
       <c r="J42" s="7" t="n">
-        <v>3024</v>
+        <v>1874</v>
       </c>
       <c r="K42" s="8" t="n">
-        <v>126</v>
+        <v>78.07142857142857</v>
       </c>
     </row>
     <row r="43">
@@ -2772,11 +2772,11 @@
         </is>
       </c>
       <c r="G46" s="4" t="n">
-        <v>16626</v>
+        <v>17719</v>
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>11/19</t>
+          <t>12/19</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
@@ -2785,10 +2785,10 @@
         </is>
       </c>
       <c r="J46" s="4" t="n">
-        <v>28718</v>
+        <v>28055</v>
       </c>
       <c r="K46" s="5" t="n">
-        <v>1511.454545454545</v>
+        <v>1476.583333333333</v>
       </c>
     </row>
     <row r="47">
@@ -2870,11 +2870,11 @@
         </is>
       </c>
       <c r="G48" s="7" t="n">
-        <v>5083</v>
+        <v>5559</v>
       </c>
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>7/18</t>
+          <t>8/18</t>
         </is>
       </c>
       <c r="I48" s="6" t="inlineStr">
@@ -2883,10 +2883,10 @@
         </is>
       </c>
       <c r="J48" s="7" t="n">
-        <v>13071</v>
+        <v>12508</v>
       </c>
       <c r="K48" s="8" t="n">
-        <v>726.1428571428571</v>
+        <v>694.875</v>
       </c>
     </row>
     <row r="49">
@@ -3017,11 +3017,11 @@
         </is>
       </c>
       <c r="G51" s="7" t="n">
-        <v>11074</v>
+        <v>11964</v>
       </c>
       <c r="H51" s="6" t="inlineStr">
         <is>
-          <t>14/23</t>
+          <t>15/23</t>
         </is>
       </c>
       <c r="I51" s="6" t="inlineStr">
@@ -3030,10 +3030,10 @@
         </is>
       </c>
       <c r="J51" s="7" t="n">
-        <v>18193</v>
+        <v>18345</v>
       </c>
       <c r="K51" s="8" t="n">
-        <v>791</v>
+        <v>797.6</v>
       </c>
     </row>
     <row r="52">
@@ -3262,11 +3262,11 @@
         </is>
       </c>
       <c r="G56" s="7" t="n">
-        <v>5663</v>
+        <v>3691</v>
       </c>
       <c r="H56" s="6" t="inlineStr">
         <is>
-          <t>17/23</t>
+          <t>18/23</t>
         </is>
       </c>
       <c r="I56" s="6" t="inlineStr">
@@ -3275,10 +3275,10 @@
         </is>
       </c>
       <c r="J56" s="7" t="n">
-        <v>7662</v>
+        <v>4716</v>
       </c>
       <c r="K56" s="8" t="n">
-        <v>333.1176470588235</v>
+        <v>205.0555555555555</v>
       </c>
     </row>
     <row r="57">
@@ -3674,52 +3674,52 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="9" t="inlineStr">
+      <c r="A65" s="6" t="inlineStr">
         <is>
           <t>KANNIYAKUMARI</t>
         </is>
       </c>
-      <c r="B65" s="10" t="n">
+      <c r="B65" s="6" t="n">
         <v>229</v>
       </c>
-      <c r="C65" s="10" t="inlineStr">
+      <c r="C65" s="6" t="inlineStr">
         <is>
           <t>THALAVAI SUNDARAM. N</t>
         </is>
       </c>
-      <c r="D65" s="10" t="inlineStr">
+      <c r="D65" s="6" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E65" s="10" t="inlineStr">
+      <c r="E65" s="6" t="inlineStr">
         <is>
           <t>MAHESH.R</t>
         </is>
       </c>
-      <c r="F65" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G65" s="11" t="n">
-        <v>138</v>
-      </c>
-      <c r="H65" s="10" t="inlineStr">
-        <is>
-          <t>10/26</t>
-        </is>
-      </c>
-      <c r="I65" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J65" s="11" t="n">
-        <v>359</v>
-      </c>
-      <c r="K65" s="12" t="n">
-        <v>13.8</v>
+      <c r="F65" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G65" s="7" t="n">
+        <v>1078</v>
+      </c>
+      <c r="H65" s="6" t="inlineStr">
+        <is>
+          <t>11/26</t>
+        </is>
+      </c>
+      <c r="I65" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J65" s="7" t="n">
+        <v>2548</v>
+      </c>
+      <c r="K65" s="8" t="n">
+        <v>98</v>
       </c>
     </row>
     <row r="66">
@@ -3821,52 +3821,52 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="inlineStr">
+      <c r="A68" s="6" t="inlineStr">
         <is>
           <t>KATPADI</t>
         </is>
       </c>
-      <c r="B68" s="3" t="n">
+      <c r="B68" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="C68" s="3" t="inlineStr">
+      <c r="C68" s="6" t="inlineStr">
         <is>
           <t>V. RAMU</t>
         </is>
       </c>
-      <c r="D68" s="3" t="inlineStr">
+      <c r="D68" s="6" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E68" s="3" t="inlineStr">
-        <is>
-          <t>DURAIMURUGAN</t>
-        </is>
-      </c>
-      <c r="F68" s="3" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G68" s="4" t="n">
-        <v>7634</v>
-      </c>
-      <c r="H68" s="3" t="inlineStr">
-        <is>
-          <t>7/20</t>
-        </is>
-      </c>
-      <c r="I68" s="3" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J68" s="4" t="n">
-        <v>21811</v>
-      </c>
-      <c r="K68" s="5" t="n">
-        <v>1090.571428571429</v>
+      <c r="E68" s="6" t="inlineStr">
+        <is>
+          <t>DR M SUDHAKAR</t>
+        </is>
+      </c>
+      <c r="F68" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G68" s="7" t="n">
+        <v>4206</v>
+      </c>
+      <c r="H68" s="6" t="inlineStr">
+        <is>
+          <t>8/20</t>
+        </is>
+      </c>
+      <c r="I68" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J68" s="7" t="n">
+        <v>10515</v>
+      </c>
+      <c r="K68" s="8" t="n">
+        <v>525.75</v>
       </c>
     </row>
     <row r="69">
@@ -4242,11 +4242,11 @@
         </is>
       </c>
       <c r="G76" s="7" t="n">
-        <v>8048</v>
+        <v>8455</v>
       </c>
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>12/22</t>
+          <t>13/22</t>
         </is>
       </c>
       <c r="I76" s="6" t="inlineStr">
@@ -4255,10 +4255,10 @@
         </is>
       </c>
       <c r="J76" s="7" t="n">
-        <v>14755</v>
+        <v>14308</v>
       </c>
       <c r="K76" s="8" t="n">
-        <v>670.6666666666666</v>
+        <v>650.3846153846154</v>
       </c>
     </row>
     <row r="77">
@@ -4291,11 +4291,11 @@
         </is>
       </c>
       <c r="G77" s="7" t="n">
-        <v>2951</v>
+        <v>2514</v>
       </c>
       <c r="H77" s="6" t="inlineStr">
         <is>
-          <t>8/23</t>
+          <t>9/23</t>
         </is>
       </c>
       <c r="I77" s="6" t="inlineStr">
@@ -4304,10 +4304,10 @@
         </is>
       </c>
       <c r="J77" s="7" t="n">
-        <v>8484</v>
+        <v>6425</v>
       </c>
       <c r="K77" s="8" t="n">
-        <v>368.875</v>
+        <v>279.3333333333333</v>
       </c>
     </row>
     <row r="78">
@@ -4821,20 +4821,20 @@
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>SUNDAR C</t>
+          <t>PALANIVEL THIAGA RAJAN</t>
         </is>
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
+          <t>Dravida Munnetra Kazhagam</t>
         </is>
       </c>
       <c r="G88" s="4" t="n">
-        <v>12896</v>
+        <v>13976</v>
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>7/19</t>
+          <t>8/19</t>
         </is>
       </c>
       <c r="I88" s="3" t="inlineStr">
@@ -4843,10 +4843,10 @@
         </is>
       </c>
       <c r="J88" s="4" t="n">
-        <v>35003</v>
+        <v>33193</v>
       </c>
       <c r="K88" s="5" t="n">
-        <v>1842.285714285714</v>
+        <v>1747</v>
       </c>
     </row>
     <row r="89">
@@ -4879,11 +4879,11 @@
         </is>
       </c>
       <c r="G89" s="7" t="n">
-        <v>5742</v>
+        <v>6633</v>
       </c>
       <c r="H89" s="6" t="inlineStr">
         <is>
-          <t>14/29</t>
+          <t>15/29</t>
         </is>
       </c>
       <c r="I89" s="6" t="inlineStr">
@@ -4892,10 +4892,10 @@
         </is>
       </c>
       <c r="J89" s="7" t="n">
-        <v>11894</v>
+        <v>12824</v>
       </c>
       <c r="K89" s="8" t="n">
-        <v>410.1428571428572</v>
+        <v>442.1999999999999</v>
       </c>
     </row>
     <row r="90">
@@ -4928,11 +4928,11 @@
         </is>
       </c>
       <c r="G90" s="4" t="n">
-        <v>13514</v>
+        <v>14435</v>
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>10/19</t>
+          <t>11/19</t>
         </is>
       </c>
       <c r="I90" s="3" t="inlineStr">
@@ -4941,10 +4941,10 @@
         </is>
       </c>
       <c r="J90" s="4" t="n">
-        <v>25677</v>
+        <v>24933</v>
       </c>
       <c r="K90" s="5" t="n">
-        <v>1351.4</v>
+        <v>1312.272727272727</v>
       </c>
     </row>
     <row r="91">
@@ -5026,11 +5026,11 @@
         </is>
       </c>
       <c r="G92" s="7" t="n">
-        <v>2289</v>
+        <v>2645</v>
       </c>
       <c r="H92" s="6" t="inlineStr">
         <is>
-          <t>11/24</t>
+          <t>12/24</t>
         </is>
       </c>
       <c r="I92" s="6" t="inlineStr">
@@ -5039,10 +5039,10 @@
         </is>
       </c>
       <c r="J92" s="7" t="n">
-        <v>4994</v>
+        <v>5290</v>
       </c>
       <c r="K92" s="8" t="n">
-        <v>208.0909090909091</v>
+        <v>220.4166666666667</v>
       </c>
     </row>
     <row r="93">
@@ -5173,11 +5173,11 @@
         </is>
       </c>
       <c r="G95" s="4" t="n">
-        <v>20405</v>
+        <v>22002</v>
       </c>
       <c r="H95" s="3" t="inlineStr">
         <is>
-          <t>12/20</t>
+          <t>13/20</t>
         </is>
       </c>
       <c r="I95" s="3" t="inlineStr">
@@ -5186,10 +5186,10 @@
         </is>
       </c>
       <c r="J95" s="4" t="n">
-        <v>34008</v>
+        <v>33849</v>
       </c>
       <c r="K95" s="5" t="n">
-        <v>1700.416666666667</v>
+        <v>1692.461538461539</v>
       </c>
     </row>
     <row r="96">
@@ -5418,11 +5418,11 @@
         </is>
       </c>
       <c r="G100" s="7" t="n">
-        <v>6014</v>
+        <v>6104</v>
       </c>
       <c r="H100" s="6" t="inlineStr">
         <is>
-          <t>8/22</t>
+          <t>9/22</t>
         </is>
       </c>
       <c r="I100" s="6" t="inlineStr">
@@ -5431,10 +5431,10 @@
         </is>
       </c>
       <c r="J100" s="7" t="n">
-        <v>16538</v>
+        <v>14921</v>
       </c>
       <c r="K100" s="8" t="n">
-        <v>751.75</v>
+        <v>678.2222222222222</v>
       </c>
     </row>
     <row r="101">
@@ -5467,11 +5467,11 @@
         </is>
       </c>
       <c r="G101" s="7" t="n">
-        <v>3093</v>
+        <v>2706</v>
       </c>
       <c r="H101" s="6" t="inlineStr">
         <is>
-          <t>18/21</t>
+          <t>19/21</t>
         </is>
       </c>
       <c r="I101" s="6" t="inlineStr">
@@ -5480,10 +5480,10 @@
         </is>
       </c>
       <c r="J101" s="7" t="n">
-        <v>3608</v>
+        <v>2991</v>
       </c>
       <c r="K101" s="8" t="n">
-        <v>171.8333333333333</v>
+        <v>142.421052631579</v>
       </c>
     </row>
     <row r="102">
@@ -5565,11 +5565,11 @@
         </is>
       </c>
       <c r="G103" s="7" t="n">
-        <v>597</v>
+        <v>1391</v>
       </c>
       <c r="H103" s="6" t="inlineStr">
         <is>
-          <t>9/24</t>
+          <t>10/24</t>
         </is>
       </c>
       <c r="I103" s="6" t="inlineStr">
@@ -5578,10 +5578,10 @@
         </is>
       </c>
       <c r="J103" s="7" t="n">
-        <v>1592</v>
+        <v>3338</v>
       </c>
       <c r="K103" s="8" t="n">
-        <v>66.33333333333333</v>
+        <v>139.1</v>
       </c>
     </row>
     <row r="104">
@@ -5712,11 +5712,11 @@
         </is>
       </c>
       <c r="G106" s="7" t="n">
-        <v>12453</v>
+        <v>13342</v>
       </c>
       <c r="H106" s="6" t="inlineStr">
         <is>
-          <t>14/21</t>
+          <t>15/21</t>
         </is>
       </c>
       <c r="I106" s="6" t="inlineStr">
@@ -5725,10 +5725,10 @@
         </is>
       </c>
       <c r="J106" s="7" t="n">
-        <v>18680</v>
+        <v>18679</v>
       </c>
       <c r="K106" s="8" t="n">
-        <v>889.5</v>
+        <v>889.4666666666667</v>
       </c>
     </row>
     <row r="107">
@@ -5830,52 +5830,52 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="13" t="inlineStr">
+      <c r="A109" s="9" t="inlineStr">
         <is>
           <t>NAGERCOIL</t>
         </is>
       </c>
-      <c r="B109" s="14" t="n">
+      <c r="B109" s="10" t="n">
         <v>230</v>
       </c>
-      <c r="C109" s="14" t="inlineStr">
+      <c r="C109" s="10" t="inlineStr">
+        <is>
+          <t>AUSTIN</t>
+        </is>
+      </c>
+      <c r="D109" s="10" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E109" s="10" t="inlineStr">
         <is>
           <t>BERVIN KINGS G</t>
         </is>
       </c>
-      <c r="D109" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E109" s="14" t="inlineStr">
-        <is>
-          <t>AUSTIN</t>
-        </is>
-      </c>
-      <c r="F109" s="14" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G109" s="15" t="n">
-        <v>66</v>
-      </c>
-      <c r="H109" s="14" t="inlineStr">
-        <is>
-          <t>10/23</t>
-        </is>
-      </c>
-      <c r="I109" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J109" s="15" t="n">
-        <v>152</v>
-      </c>
-      <c r="K109" s="16" t="n">
-        <v>6.6</v>
+      <c r="F109" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G109" s="11" t="n">
+        <v>211</v>
+      </c>
+      <c r="H109" s="10" t="inlineStr">
+        <is>
+          <t>11/23</t>
+        </is>
+      </c>
+      <c r="I109" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J109" s="11" t="n">
+        <v>441</v>
+      </c>
+      <c r="K109" s="12" t="n">
+        <v>19.18181818181818</v>
       </c>
     </row>
     <row r="110">
@@ -5957,11 +5957,11 @@
         </is>
       </c>
       <c r="G111" s="7" t="n">
-        <v>7533</v>
+        <v>8783</v>
       </c>
       <c r="H111" s="6" t="inlineStr">
         <is>
-          <t>17/25</t>
+          <t>18/25</t>
         </is>
       </c>
       <c r="I111" s="6" t="inlineStr">
@@ -5970,10 +5970,10 @@
         </is>
       </c>
       <c r="J111" s="7" t="n">
-        <v>11078</v>
+        <v>12199</v>
       </c>
       <c r="K111" s="8" t="n">
-        <v>443.1176470588235</v>
+        <v>487.9444444444445</v>
       </c>
     </row>
     <row r="112">
@@ -6055,11 +6055,11 @@
         </is>
       </c>
       <c r="G113" s="7" t="n">
-        <v>4323</v>
+        <v>5232</v>
       </c>
       <c r="H113" s="6" t="inlineStr">
         <is>
-          <t>12/26</t>
+          <t>13/26</t>
         </is>
       </c>
       <c r="I113" s="6" t="inlineStr">
@@ -6068,10 +6068,10 @@
         </is>
       </c>
       <c r="J113" s="7" t="n">
-        <v>9366</v>
+        <v>10464</v>
       </c>
       <c r="K113" s="8" t="n">
-        <v>360.25</v>
+        <v>402.4615384615385</v>
       </c>
     </row>
     <row r="114">
@@ -6300,11 +6300,11 @@
         </is>
       </c>
       <c r="G118" s="4" t="n">
-        <v>19449</v>
+        <v>21040</v>
       </c>
       <c r="H118" s="3" t="inlineStr">
         <is>
-          <t>14/23</t>
+          <t>15/23</t>
         </is>
       </c>
       <c r="I118" s="3" t="inlineStr">
@@ -6313,10 +6313,10 @@
         </is>
       </c>
       <c r="J118" s="4" t="n">
-        <v>31952</v>
+        <v>32261</v>
       </c>
       <c r="K118" s="5" t="n">
-        <v>1389.214285714286</v>
+        <v>1402.666666666667</v>
       </c>
     </row>
     <row r="119">
@@ -6447,11 +6447,11 @@
         </is>
       </c>
       <c r="G121" s="4" t="n">
-        <v>21627</v>
+        <v>22255</v>
       </c>
       <c r="H121" s="3" t="inlineStr">
         <is>
-          <t>13/23</t>
+          <t>14/23</t>
         </is>
       </c>
       <c r="I121" s="3" t="inlineStr">
@@ -6460,59 +6460,59 @@
         </is>
       </c>
       <c r="J121" s="4" t="n">
-        <v>38263</v>
+        <v>36562</v>
       </c>
       <c r="K121" s="5" t="n">
-        <v>1663.615384615385</v>
+        <v>1589.642857142857</v>
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="9" t="inlineStr">
+      <c r="A122" s="6" t="inlineStr">
         <is>
           <t>PALANI</t>
         </is>
       </c>
-      <c r="B122" s="10" t="n">
+      <c r="B122" s="6" t="n">
         <v>127</v>
       </c>
-      <c r="C122" s="10" t="inlineStr">
+      <c r="C122" s="6" t="inlineStr">
         <is>
           <t>RAVIMANOHARAN. K</t>
         </is>
       </c>
-      <c r="D122" s="10" t="inlineStr">
+      <c r="D122" s="6" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E122" s="10" t="inlineStr">
+      <c r="E122" s="6" t="inlineStr">
         <is>
           <t>DR. PRAVEEN KUMAR. M</t>
         </is>
       </c>
-      <c r="F122" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G122" s="11" t="n">
-        <v>342</v>
-      </c>
-      <c r="H122" s="10" t="inlineStr">
-        <is>
-          <t>11/25</t>
-        </is>
-      </c>
-      <c r="I122" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J122" s="11" t="n">
-        <v>777</v>
-      </c>
-      <c r="K122" s="12" t="n">
-        <v>31.09090909090909</v>
+      <c r="F122" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G122" s="7" t="n">
+        <v>1188</v>
+      </c>
+      <c r="H122" s="6" t="inlineStr">
+        <is>
+          <t>12/25</t>
+        </is>
+      </c>
+      <c r="I122" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J122" s="7" t="n">
+        <v>2475</v>
+      </c>
+      <c r="K122" s="8" t="n">
+        <v>99</v>
       </c>
     </row>
     <row r="123">
@@ -6643,11 +6643,11 @@
         </is>
       </c>
       <c r="G125" s="4" t="n">
-        <v>19916</v>
+        <v>21154</v>
       </c>
       <c r="H125" s="3" t="inlineStr">
         <is>
-          <t>12/34</t>
+          <t>13/34</t>
         </is>
       </c>
       <c r="I125" s="3" t="inlineStr">
@@ -6656,10 +6656,10 @@
         </is>
       </c>
       <c r="J125" s="4" t="n">
-        <v>56429</v>
+        <v>55326</v>
       </c>
       <c r="K125" s="5" t="n">
-        <v>1659.666666666667</v>
+        <v>1627.230769230769</v>
       </c>
     </row>
     <row r="126">
@@ -6692,11 +6692,11 @@
         </is>
       </c>
       <c r="G126" s="7" t="n">
-        <v>4658</v>
+        <v>5219</v>
       </c>
       <c r="H126" s="6" t="inlineStr">
         <is>
-          <t>14/23</t>
+          <t>15/23</t>
         </is>
       </c>
       <c r="I126" s="6" t="inlineStr">
@@ -6705,10 +6705,10 @@
         </is>
       </c>
       <c r="J126" s="7" t="n">
-        <v>7652</v>
+        <v>8002</v>
       </c>
       <c r="K126" s="8" t="n">
-        <v>332.7142857142857</v>
+        <v>347.9333333333333</v>
       </c>
     </row>
     <row r="127">
@@ -6722,30 +6722,30 @@
       </c>
       <c r="C127" s="6" t="inlineStr">
         <is>
+          <t>A.M. SHAHJAHAN</t>
+        </is>
+      </c>
+      <c r="D127" s="6" t="inlineStr">
+        <is>
+          <t>Indian Union Muslim League</t>
+        </is>
+      </c>
+      <c r="E127" s="6" t="inlineStr">
+        <is>
           <t>DORAI. SHANMUGA PRABU</t>
         </is>
       </c>
-      <c r="D127" s="6" t="inlineStr">
+      <c r="F127" s="6" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E127" s="6" t="inlineStr">
-        <is>
-          <t>A.M. SHAHJAHAN</t>
-        </is>
-      </c>
-      <c r="F127" s="6" t="inlineStr">
-        <is>
-          <t>Indian Union Muslim League</t>
-        </is>
-      </c>
       <c r="G127" s="7" t="n">
-        <v>1487</v>
+        <v>1875</v>
       </c>
       <c r="H127" s="6" t="inlineStr">
         <is>
-          <t>7/23</t>
+          <t>8/23</t>
         </is>
       </c>
       <c r="I127" s="6" t="inlineStr">
@@ -6754,10 +6754,10 @@
         </is>
       </c>
       <c r="J127" s="7" t="n">
-        <v>4886</v>
+        <v>5391</v>
       </c>
       <c r="K127" s="8" t="n">
-        <v>212.4285714285714</v>
+        <v>234.375</v>
       </c>
     </row>
     <row r="128">
@@ -6790,11 +6790,11 @@
         </is>
       </c>
       <c r="G128" s="4" t="n">
-        <v>33492</v>
+        <v>36152</v>
       </c>
       <c r="H128" s="3" t="inlineStr">
         <is>
-          <t>14/23</t>
+          <t>15/23</t>
         </is>
       </c>
       <c r="I128" s="3" t="inlineStr">
@@ -6803,10 +6803,10 @@
         </is>
       </c>
       <c r="J128" s="4" t="n">
-        <v>55023</v>
+        <v>55433</v>
       </c>
       <c r="K128" s="5" t="n">
-        <v>2392.285714285714</v>
+        <v>2410.133333333333</v>
       </c>
     </row>
     <row r="129">
@@ -6937,11 +6937,11 @@
         </is>
       </c>
       <c r="G131" s="7" t="n">
-        <v>2919</v>
+        <v>3061</v>
       </c>
       <c r="H131" s="6" t="inlineStr">
         <is>
-          <t>8/23</t>
+          <t>9/23</t>
         </is>
       </c>
       <c r="I131" s="6" t="inlineStr">
@@ -6950,10 +6950,10 @@
         </is>
       </c>
       <c r="J131" s="7" t="n">
-        <v>8392</v>
+        <v>7823</v>
       </c>
       <c r="K131" s="8" t="n">
-        <v>364.875</v>
+        <v>340.1111111111111</v>
       </c>
     </row>
     <row r="132">
@@ -7378,11 +7378,11 @@
         </is>
       </c>
       <c r="G140" s="4" t="n">
-        <v>25979</v>
+        <v>29155</v>
       </c>
       <c r="H140" s="3" t="inlineStr">
         <is>
-          <t>12/24</t>
+          <t>13/24</t>
         </is>
       </c>
       <c r="I140" s="3" t="inlineStr">
@@ -7391,10 +7391,10 @@
         </is>
       </c>
       <c r="J140" s="4" t="n">
-        <v>51958</v>
+        <v>53825</v>
       </c>
       <c r="K140" s="5" t="n">
-        <v>2164.916666666667</v>
+        <v>2242.692307692308</v>
       </c>
     </row>
     <row r="141">
@@ -7408,30 +7408,30 @@
       </c>
       <c r="C141" s="6" t="inlineStr">
         <is>
+          <t>NIVEDHA M MURUGAN</t>
+        </is>
+      </c>
+      <c r="D141" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E141" s="6" t="inlineStr">
+        <is>
           <t>PAVUNRAJ. S</t>
         </is>
       </c>
-      <c r="D141" s="6" t="inlineStr">
+      <c r="F141" s="6" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E141" s="6" t="inlineStr">
-        <is>
-          <t>NIVEDHA M MURUGAN</t>
-        </is>
-      </c>
-      <c r="F141" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
       <c r="G141" s="7" t="n">
-        <v>1388</v>
+        <v>985</v>
       </c>
       <c r="H141" s="6" t="inlineStr">
         <is>
-          <t>10/25</t>
+          <t>11/25</t>
         </is>
       </c>
       <c r="I141" s="6" t="inlineStr">
@@ -7440,10 +7440,10 @@
         </is>
       </c>
       <c r="J141" s="7" t="n">
-        <v>3470</v>
+        <v>2239</v>
       </c>
       <c r="K141" s="8" t="n">
-        <v>138.8</v>
+        <v>89.54545454545455</v>
       </c>
     </row>
     <row r="142">
@@ -7476,11 +7476,11 @@
         </is>
       </c>
       <c r="G142" s="4" t="n">
-        <v>37823</v>
+        <v>41556</v>
       </c>
       <c r="H142" s="3" t="inlineStr">
         <is>
-          <t>11/23</t>
+          <t>12/23</t>
         </is>
       </c>
       <c r="I142" s="3" t="inlineStr">
@@ -7489,10 +7489,10 @@
         </is>
       </c>
       <c r="J142" s="4" t="n">
-        <v>79084</v>
+        <v>79649</v>
       </c>
       <c r="K142" s="5" t="n">
-        <v>3438.454545454545</v>
+        <v>3463</v>
       </c>
     </row>
     <row r="143">
@@ -7672,11 +7672,11 @@
         </is>
       </c>
       <c r="G146" s="7" t="n">
-        <v>11440</v>
+        <v>12407</v>
       </c>
       <c r="H146" s="6" t="inlineStr">
         <is>
-          <t>18/29</t>
+          <t>19/29</t>
         </is>
       </c>
       <c r="I146" s="6" t="inlineStr">
@@ -7685,10 +7685,10 @@
         </is>
       </c>
       <c r="J146" s="7" t="n">
-        <v>18431</v>
+        <v>18937</v>
       </c>
       <c r="K146" s="8" t="n">
-        <v>635.5555555555555</v>
+        <v>653</v>
       </c>
     </row>
     <row r="147">
@@ -7868,11 +7868,11 @@
         </is>
       </c>
       <c r="G150" s="7" t="n">
-        <v>12633</v>
+        <v>13304</v>
       </c>
       <c r="H150" s="6" t="inlineStr">
         <is>
-          <t>9/14</t>
+          <t>10/14</t>
         </is>
       </c>
       <c r="I150" s="6" t="inlineStr">
@@ -7881,10 +7881,10 @@
         </is>
       </c>
       <c r="J150" s="7" t="n">
-        <v>19651</v>
+        <v>18626</v>
       </c>
       <c r="K150" s="8" t="n">
-        <v>1403.666666666667</v>
+        <v>1330.4</v>
       </c>
     </row>
     <row r="151">
@@ -7966,11 +7966,11 @@
         </is>
       </c>
       <c r="G152" s="7" t="n">
-        <v>4451</v>
+        <v>5508</v>
       </c>
       <c r="H152" s="6" t="inlineStr">
         <is>
-          <t>9/21</t>
+          <t>10/21</t>
         </is>
       </c>
       <c r="I152" s="6" t="inlineStr">
@@ -7979,10 +7979,10 @@
         </is>
       </c>
       <c r="J152" s="7" t="n">
-        <v>10386</v>
+        <v>11567</v>
       </c>
       <c r="K152" s="8" t="n">
-        <v>494.5555555555555</v>
+        <v>550.8</v>
       </c>
     </row>
     <row r="153">
@@ -8309,11 +8309,11 @@
         </is>
       </c>
       <c r="G159" s="7" t="n">
-        <v>2779</v>
+        <v>2976</v>
       </c>
       <c r="H159" s="6" t="inlineStr">
         <is>
-          <t>11/22</t>
+          <t>12/22</t>
         </is>
       </c>
       <c r="I159" s="6" t="inlineStr">
@@ -8322,10 +8322,10 @@
         </is>
       </c>
       <c r="J159" s="7" t="n">
-        <v>5558</v>
+        <v>5456</v>
       </c>
       <c r="K159" s="8" t="n">
-        <v>252.6363636363636</v>
+        <v>248</v>
       </c>
     </row>
     <row r="160">
@@ -8505,11 +8505,11 @@
         </is>
       </c>
       <c r="G163" s="4" t="n">
-        <v>11164</v>
+        <v>11675</v>
       </c>
       <c r="H163" s="3" t="inlineStr">
         <is>
-          <t>11/26</t>
+          <t>12/26</t>
         </is>
       </c>
       <c r="I163" s="3" t="inlineStr">
@@ -8518,10 +8518,10 @@
         </is>
       </c>
       <c r="J163" s="4" t="n">
-        <v>26388</v>
+        <v>25296</v>
       </c>
       <c r="K163" s="5" t="n">
-        <v>1014.909090909091</v>
+        <v>972.9166666666666</v>
       </c>
     </row>
     <row r="164">
@@ -8623,52 +8623,52 @@
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="6" t="inlineStr">
+      <c r="A166" s="9" t="inlineStr">
         <is>
           <t>SIVAKASI</t>
         </is>
       </c>
-      <c r="B166" s="6" t="n">
+      <c r="B166" s="10" t="n">
         <v>205</v>
       </c>
-      <c r="C166" s="6" t="inlineStr">
+      <c r="C166" s="10" t="inlineStr">
         <is>
           <t>RAJENTHRABHALAJI K T</t>
         </is>
       </c>
-      <c r="D166" s="6" t="inlineStr">
+      <c r="D166" s="10" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E166" s="6" t="inlineStr">
+      <c r="E166" s="10" t="inlineStr">
         <is>
           <t>KEERTHANA S</t>
         </is>
       </c>
-      <c r="F166" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G166" s="7" t="n">
-        <v>1261</v>
-      </c>
-      <c r="H166" s="6" t="inlineStr">
-        <is>
-          <t>5/21</t>
-        </is>
-      </c>
-      <c r="I166" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J166" s="7" t="n">
-        <v>5296</v>
-      </c>
-      <c r="K166" s="8" t="n">
-        <v>252.2</v>
+      <c r="F166" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G166" s="11" t="n">
+        <v>63</v>
+      </c>
+      <c r="H166" s="10" t="inlineStr">
+        <is>
+          <t>6/21</t>
+        </is>
+      </c>
+      <c r="I166" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J166" s="11" t="n">
+        <v>220</v>
+      </c>
+      <c r="K166" s="12" t="n">
+        <v>10.5</v>
       </c>
     </row>
     <row r="167">
@@ -9093,7 +9093,7 @@
         </is>
       </c>
       <c r="G175" s="4" t="n">
-        <v>17272</v>
+        <v>16692</v>
       </c>
       <c r="H175" s="3" t="inlineStr">
         <is>
@@ -9106,10 +9106,10 @@
         </is>
       </c>
       <c r="J175" s="4" t="n">
-        <v>18917</v>
+        <v>18282</v>
       </c>
       <c r="K175" s="5" t="n">
-        <v>822.4761904761905</v>
+        <v>794.8571428571429</v>
       </c>
     </row>
     <row r="176">
@@ -9191,11 +9191,11 @@
         </is>
       </c>
       <c r="G177" s="7" t="n">
-        <v>8849</v>
+        <v>10764</v>
       </c>
       <c r="H177" s="6" t="inlineStr">
         <is>
-          <t>15/26</t>
+          <t>16/26</t>
         </is>
       </c>
       <c r="I177" s="6" t="inlineStr">
@@ -9204,10 +9204,10 @@
         </is>
       </c>
       <c r="J177" s="7" t="n">
-        <v>15338</v>
+        <v>17492</v>
       </c>
       <c r="K177" s="8" t="n">
-        <v>589.9333333333334</v>
+        <v>672.75</v>
       </c>
     </row>
     <row r="178">
@@ -9338,11 +9338,11 @@
         </is>
       </c>
       <c r="G180" s="4" t="n">
-        <v>18071</v>
+        <v>19539</v>
       </c>
       <c r="H180" s="3" t="inlineStr">
         <is>
-          <t>9/29</t>
+          <t>10/29</t>
         </is>
       </c>
       <c r="I180" s="3" t="inlineStr">
@@ -9351,10 +9351,10 @@
         </is>
       </c>
       <c r="J180" s="4" t="n">
-        <v>58229</v>
+        <v>56663</v>
       </c>
       <c r="K180" s="5" t="n">
-        <v>2007.888888888889</v>
+        <v>1953.9</v>
       </c>
     </row>
     <row r="181">
@@ -9681,11 +9681,11 @@
         </is>
       </c>
       <c r="G187" s="4" t="n">
-        <v>24680</v>
+        <v>27799</v>
       </c>
       <c r="H187" s="3" t="inlineStr">
         <is>
-          <t>11/25</t>
+          <t>12/25</t>
         </is>
       </c>
       <c r="I187" s="3" t="inlineStr">
@@ -9694,10 +9694,10 @@
         </is>
       </c>
       <c r="J187" s="4" t="n">
-        <v>56091</v>
+        <v>57915</v>
       </c>
       <c r="K187" s="5" t="n">
-        <v>2243.636363636364</v>
+        <v>2316.583333333333</v>
       </c>
     </row>
     <row r="188">
@@ -9877,11 +9877,11 @@
         </is>
       </c>
       <c r="G191" s="7" t="n">
-        <v>4146</v>
+        <v>3887</v>
       </c>
       <c r="H191" s="6" t="inlineStr">
         <is>
-          <t>6/18</t>
+          <t>7/18</t>
         </is>
       </c>
       <c r="I191" s="6" t="inlineStr">
@@ -9890,10 +9890,10 @@
         </is>
       </c>
       <c r="J191" s="7" t="n">
-        <v>12438</v>
+        <v>9995</v>
       </c>
       <c r="K191" s="8" t="n">
-        <v>691</v>
+        <v>555.2857142857143</v>
       </c>
     </row>
     <row r="192">
@@ -9975,11 +9975,11 @@
         </is>
       </c>
       <c r="G193" s="7" t="n">
-        <v>2122</v>
+        <v>2048</v>
       </c>
       <c r="H193" s="6" t="inlineStr">
         <is>
-          <t>8/21</t>
+          <t>9/21</t>
         </is>
       </c>
       <c r="I193" s="6" t="inlineStr">
@@ -9988,10 +9988,10 @@
         </is>
       </c>
       <c r="J193" s="7" t="n">
-        <v>5570</v>
+        <v>4779</v>
       </c>
       <c r="K193" s="8" t="n">
-        <v>265.25</v>
+        <v>227.5555555555555</v>
       </c>
     </row>
     <row r="194">
@@ -10024,11 +10024,11 @@
         </is>
       </c>
       <c r="G194" s="7" t="n">
-        <v>8355</v>
+        <v>7580</v>
       </c>
       <c r="H194" s="6" t="inlineStr">
         <is>
-          <t>14/22</t>
+          <t>15/22</t>
         </is>
       </c>
       <c r="I194" s="6" t="inlineStr">
@@ -10037,10 +10037,10 @@
         </is>
       </c>
       <c r="J194" s="7" t="n">
-        <v>13129</v>
+        <v>11117</v>
       </c>
       <c r="K194" s="8" t="n">
-        <v>596.7857142857143</v>
+        <v>505.3333333333334</v>
       </c>
     </row>
     <row r="195">
@@ -10122,11 +10122,11 @@
         </is>
       </c>
       <c r="G196" s="4" t="n">
-        <v>12015</v>
+        <v>13500</v>
       </c>
       <c r="H196" s="3" t="inlineStr">
         <is>
-          <t>8/22</t>
+          <t>9/22</t>
         </is>
       </c>
       <c r="I196" s="3" t="inlineStr">
@@ -10135,10 +10135,10 @@
         </is>
       </c>
       <c r="J196" s="4" t="n">
-        <v>33041</v>
+        <v>33000</v>
       </c>
       <c r="K196" s="5" t="n">
-        <v>1501.875</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="197">
@@ -10416,11 +10416,11 @@
         </is>
       </c>
       <c r="G202" s="7" t="n">
-        <v>4603</v>
+        <v>4902</v>
       </c>
       <c r="H202" s="6" t="inlineStr">
         <is>
-          <t>9/27</t>
+          <t>10/27</t>
         </is>
       </c>
       <c r="I202" s="6" t="inlineStr">
@@ -10429,10 +10429,10 @@
         </is>
       </c>
       <c r="J202" s="7" t="n">
-        <v>13809</v>
+        <v>13235</v>
       </c>
       <c r="K202" s="8" t="n">
-        <v>511.4444444444445</v>
+        <v>490.2</v>
       </c>
     </row>
     <row r="203">
@@ -10563,11 +10563,11 @@
         </is>
       </c>
       <c r="G205" s="7" t="n">
-        <v>3116</v>
+        <v>3881</v>
       </c>
       <c r="H205" s="6" t="inlineStr">
         <is>
-          <t>8/25</t>
+          <t>9/25</t>
         </is>
       </c>
       <c r="I205" s="6" t="inlineStr">
@@ -10576,10 +10576,10 @@
         </is>
       </c>
       <c r="J205" s="7" t="n">
-        <v>9738</v>
+        <v>10781</v>
       </c>
       <c r="K205" s="8" t="n">
-        <v>389.5</v>
+        <v>431.2222222222222</v>
       </c>
     </row>
     <row r="206">
@@ -10740,30 +10740,30 @@
       </c>
       <c r="C209" s="10" t="inlineStr">
         <is>
+          <t>BHOJARAJAN.M</t>
+        </is>
+      </c>
+      <c r="D209" s="10" t="inlineStr">
+        <is>
+          <t>Bharatiya Janata Party</t>
+        </is>
+      </c>
+      <c r="E209" s="10" t="inlineStr">
+        <is>
           <t>IBRAHIM.R</t>
         </is>
       </c>
-      <c r="D209" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E209" s="10" t="inlineStr">
-        <is>
-          <t>BHOJARAJAN.M</t>
-        </is>
-      </c>
       <c r="F209" s="10" t="inlineStr">
         <is>
-          <t>Bharatiya Janata Party</t>
+          <t>Tamilaga Vettri Kazhagam</t>
         </is>
       </c>
       <c r="G209" s="11" t="n">
-        <v>495</v>
+        <v>189</v>
       </c>
       <c r="H209" s="10" t="inlineStr">
         <is>
-          <t>16/19</t>
+          <t>17/19</t>
         </is>
       </c>
       <c r="I209" s="10" t="inlineStr">
@@ -10772,10 +10772,10 @@
         </is>
       </c>
       <c r="J209" s="11" t="n">
-        <v>588</v>
+        <v>211</v>
       </c>
       <c r="K209" s="12" t="n">
-        <v>30.9375</v>
+        <v>11.11764705882353</v>
       </c>
     </row>
     <row r="210">
@@ -11024,52 +11024,52 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="6" t="inlineStr">
+      <c r="A215" s="2" t="inlineStr">
         <is>
           <t>VALPARAI</t>
         </is>
       </c>
-      <c r="B215" s="6" t="n">
+      <c r="B215" s="3" t="n">
         <v>124</v>
       </c>
-      <c r="C215" s="6" t="inlineStr">
+      <c r="C215" s="3" t="inlineStr">
         <is>
           <t>KUTTY (ALIAS) SUDHAKAR. A</t>
         </is>
       </c>
-      <c r="D215" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E215" s="6" t="inlineStr">
+      <c r="D215" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E215" s="3" t="inlineStr">
         <is>
           <t>DR. SRIDHARAN. A</t>
         </is>
       </c>
-      <c r="F215" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G215" s="7" t="n">
-        <v>4164</v>
-      </c>
-      <c r="H215" s="6" t="inlineStr">
-        <is>
-          <t>15/18</t>
-        </is>
-      </c>
-      <c r="I215" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J215" s="7" t="n">
-        <v>4997</v>
-      </c>
-      <c r="K215" s="8" t="n">
-        <v>277.6</v>
+      <c r="F215" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G215" s="4" t="n">
+        <v>5788</v>
+      </c>
+      <c r="H215" s="3" t="inlineStr">
+        <is>
+          <t>16/18</t>
+        </is>
+      </c>
+      <c r="I215" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J215" s="4" t="n">
+        <v>6512</v>
+      </c>
+      <c r="K215" s="5" t="n">
+        <v>361.75</v>
       </c>
     </row>
     <row r="216">
@@ -11249,11 +11249,11 @@
         </is>
       </c>
       <c r="G219" s="7" t="n">
-        <v>6793</v>
+        <v>6277</v>
       </c>
       <c r="H219" s="6" t="inlineStr">
         <is>
-          <t>12/23</t>
+          <t>13/23</t>
         </is>
       </c>
       <c r="I219" s="6" t="inlineStr">
@@ -11262,10 +11262,10 @@
         </is>
       </c>
       <c r="J219" s="7" t="n">
-        <v>13020</v>
+        <v>11105</v>
       </c>
       <c r="K219" s="8" t="n">
-        <v>566.0833333333334</v>
+        <v>482.8461538461539</v>
       </c>
     </row>
     <row r="220">
@@ -11298,11 +11298,11 @@
         </is>
       </c>
       <c r="G220" s="7" t="n">
-        <v>6411</v>
+        <v>6619</v>
       </c>
       <c r="H220" s="6" t="inlineStr">
         <is>
-          <t>9/18</t>
+          <t>10/18</t>
         </is>
       </c>
       <c r="I220" s="6" t="inlineStr">
@@ -11311,10 +11311,10 @@
         </is>
       </c>
       <c r="J220" s="7" t="n">
-        <v>12822</v>
+        <v>11914</v>
       </c>
       <c r="K220" s="8" t="n">
-        <v>712.3333333333334</v>
+        <v>661.9</v>
       </c>
     </row>
     <row r="221">
@@ -11498,7 +11498,7 @@
       </c>
       <c r="H224" s="6" t="inlineStr">
         <is>
-          <t>10/21</t>
+          <t>10/20</t>
         </is>
       </c>
       <c r="I224" s="6" t="inlineStr">
@@ -11507,7 +11507,7 @@
         </is>
       </c>
       <c r="J224" s="7" t="n">
-        <v>8522</v>
+        <v>8116</v>
       </c>
       <c r="K224" s="8" t="n">
         <v>405.8</v>
@@ -11543,11 +11543,11 @@
         </is>
       </c>
       <c r="G225" s="7" t="n">
-        <v>2031</v>
+        <v>2533</v>
       </c>
       <c r="H225" s="6" t="inlineStr">
         <is>
-          <t>12/25</t>
+          <t>13/25</t>
         </is>
       </c>
       <c r="I225" s="6" t="inlineStr">
@@ -11556,10 +11556,10 @@
         </is>
       </c>
       <c r="J225" s="7" t="n">
-        <v>4231</v>
+        <v>4871</v>
       </c>
       <c r="K225" s="8" t="n">
-        <v>169.25</v>
+        <v>194.8461538461538</v>
       </c>
     </row>
     <row r="226">
@@ -11641,11 +11641,11 @@
         </is>
       </c>
       <c r="G227" s="7" t="n">
-        <v>5418</v>
+        <v>4570</v>
       </c>
       <c r="H227" s="6" t="inlineStr">
         <is>
-          <t>11/20</t>
+          <t>12/20</t>
         </is>
       </c>
       <c r="I227" s="6" t="inlineStr">
@@ -11654,10 +11654,10 @@
         </is>
       </c>
       <c r="J227" s="7" t="n">
-        <v>9851</v>
+        <v>7617</v>
       </c>
       <c r="K227" s="8" t="n">
-        <v>492.5454545454546</v>
+        <v>380.8333333333333</v>
       </c>
     </row>
     <row r="228">
@@ -11739,11 +11739,11 @@
         </is>
       </c>
       <c r="G229" s="7" t="n">
-        <v>8502</v>
+        <v>9247</v>
       </c>
       <c r="H229" s="6" t="inlineStr">
         <is>
-          <t>9/19</t>
+          <t>10/19</t>
         </is>
       </c>
       <c r="I229" s="6" t="inlineStr">
@@ -11752,10 +11752,10 @@
         </is>
       </c>
       <c r="J229" s="7" t="n">
-        <v>17949</v>
+        <v>17569</v>
       </c>
       <c r="K229" s="8" t="n">
-        <v>944.6666666666666</v>
+        <v>924.7</v>
       </c>
     </row>
     <row r="230">

</xml_diff>

<commit_message>
Update election results snapshot (52.2% counted)
TVK 106, AIADMK 55, DMK 54. First result declared (GUDALUR, DMK).
ALANGULAM down to 16-vote AIADMK lead — tightest seat so far.

https://claude.ai/code/session_01MizbUy44JG5sXyvaf3Wekb
</commit_message>
<xml_diff>
--- a/tn_election_results_may2026.xlsx
+++ b/tn_election_results_may2026.xlsx
@@ -56,12 +56,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFB347"/>
+        <fgColor rgb="00FF6B6B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FF6B6B"/>
+        <fgColor rgb="00FFB347"/>
       </patternFill>
     </fill>
   </fills>
@@ -145,8 +145,8 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -616,11 +616,11 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>11948</v>
+        <v>13488</v>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>9/31</t>
+          <t>10/31</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -629,10 +629,10 @@
         </is>
       </c>
       <c r="J2" s="4" t="n">
-        <v>41154</v>
+        <v>41813</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>1327.555555555556</v>
+        <v>1348.8</v>
       </c>
     </row>
     <row r="3">
@@ -685,52 +685,52 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>ALANGULAM</t>
         </is>
       </c>
-      <c r="B4" s="6" t="n">
+      <c r="B4" s="10" t="n">
         <v>223</v>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
         <is>
           <t>K R P PRABAKARAN</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="10" t="inlineStr">
         <is>
           <t>PAUL MANOJ PANDIAN</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G4" s="7" t="n">
-        <v>719</v>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>15/24</t>
-        </is>
-      </c>
-      <c r="I4" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J4" s="7" t="n">
-        <v>1150</v>
-      </c>
-      <c r="K4" s="8" t="n">
-        <v>47.93333333333333</v>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>16/24</t>
+        </is>
+      </c>
+      <c r="I4" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J4" s="11" t="n">
+        <v>24</v>
+      </c>
+      <c r="K4" s="12" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -812,11 +812,11 @@
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>32123</v>
+        <v>34254</v>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>12/27</t>
+          <t>13/27</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -825,10 +825,10 @@
         </is>
       </c>
       <c r="J6" s="4" t="n">
-        <v>72277</v>
+        <v>71143</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>2676.916666666667</v>
+        <v>2634.923076923077</v>
       </c>
     </row>
     <row r="7">
@@ -910,11 +910,11 @@
         </is>
       </c>
       <c r="G8" s="7" t="n">
-        <v>2980</v>
+        <v>3955</v>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>9/22</t>
+          <t>10/22</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
@@ -923,10 +923,10 @@
         </is>
       </c>
       <c r="J8" s="7" t="n">
-        <v>7284</v>
+        <v>8701</v>
       </c>
       <c r="K8" s="8" t="n">
-        <v>331.1111111111111</v>
+        <v>395.5</v>
       </c>
     </row>
     <row r="9">
@@ -959,11 +959,11 @@
         </is>
       </c>
       <c r="G9" s="7" t="n">
-        <v>722</v>
+        <v>614</v>
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>12/25</t>
+          <t>13/25</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
@@ -972,10 +972,10 @@
         </is>
       </c>
       <c r="J9" s="7" t="n">
-        <v>1504</v>
+        <v>1181</v>
       </c>
       <c r="K9" s="8" t="n">
-        <v>60.16666666666666</v>
+        <v>47.23076923076923</v>
       </c>
     </row>
     <row r="10">
@@ -1008,11 +1008,11 @@
         </is>
       </c>
       <c r="G10" s="4" t="n">
-        <v>18473</v>
+        <v>19916</v>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>16/20</t>
+          <t>17/20</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
@@ -1021,10 +1021,10 @@
         </is>
       </c>
       <c r="J10" s="4" t="n">
-        <v>23091</v>
+        <v>23431</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>1154.5625</v>
+        <v>1171.529411764706</v>
       </c>
     </row>
     <row r="11">
@@ -1048,20 +1048,20 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>VIJAY VENKATESH.M</t>
+          <t>SIVABALAN.M</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>Tamilaga Vettri Kazhagam</t>
+          <t>Dravida Munnetra Kazhagam</t>
         </is>
       </c>
       <c r="G11" s="7" t="n">
-        <v>2166</v>
+        <v>2647</v>
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>15/20</t>
+          <t>16/20</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
@@ -1070,10 +1070,10 @@
         </is>
       </c>
       <c r="J11" s="7" t="n">
-        <v>2888</v>
+        <v>3309</v>
       </c>
       <c r="K11" s="8" t="n">
-        <v>144.4</v>
+        <v>165.4375</v>
       </c>
     </row>
     <row r="12">
@@ -1106,11 +1106,11 @@
         </is>
       </c>
       <c r="G12" s="4" t="n">
-        <v>17178</v>
+        <v>19983</v>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>15/21</t>
+          <t>17/21</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
@@ -1119,10 +1119,10 @@
         </is>
       </c>
       <c r="J12" s="4" t="n">
-        <v>24049</v>
+        <v>24685</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1145.2</v>
+        <v>1175.470588235294</v>
       </c>
     </row>
     <row r="13">
@@ -1155,11 +1155,11 @@
         </is>
       </c>
       <c r="G13" s="7" t="n">
-        <v>3800</v>
+        <v>2887</v>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>15/24</t>
+          <t>16/24</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
@@ -1168,10 +1168,10 @@
         </is>
       </c>
       <c r="J13" s="7" t="n">
-        <v>6080</v>
+        <v>4330</v>
       </c>
       <c r="K13" s="8" t="n">
-        <v>253.3333333333333</v>
+        <v>180.4375</v>
       </c>
     </row>
     <row r="14">
@@ -1224,52 +1224,52 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>ARAVAKURICHI</t>
         </is>
       </c>
-      <c r="B15" s="10" t="n">
+      <c r="B15" s="6" t="n">
         <v>134</v>
       </c>
-      <c r="C15" s="10" t="inlineStr">
-        <is>
-          <t>KARTHIKEYAN. P</t>
-        </is>
-      </c>
-      <c r="D15" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E15" s="10" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>SELVAKUMAR. K</t>
         </is>
       </c>
-      <c r="F15" s="10" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G15" s="11" t="n">
-        <v>310</v>
-      </c>
-      <c r="H15" s="10" t="inlineStr">
-        <is>
-          <t>13/20</t>
-        </is>
-      </c>
-      <c r="I15" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J15" s="11" t="n">
-        <v>477</v>
-      </c>
-      <c r="K15" s="12" t="n">
-        <v>23.84615384615385</v>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>ELANGO. R</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="n">
+        <v>661</v>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>14/20</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>944</v>
+      </c>
+      <c r="K15" s="8" t="n">
+        <v>47.21428571428572</v>
       </c>
     </row>
     <row r="16">
@@ -1449,11 +1449,11 @@
         </is>
       </c>
       <c r="G19" s="4" t="n">
-        <v>11601</v>
+        <v>12414</v>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>11/25</t>
+          <t>12/25</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -1462,10 +1462,10 @@
         </is>
       </c>
       <c r="J19" s="4" t="n">
-        <v>26366</v>
+        <v>25862</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>1054.636363636364</v>
+        <v>1034.5</v>
       </c>
     </row>
     <row r="20">
@@ -1547,11 +1547,11 @@
         </is>
       </c>
       <c r="G21" s="4" t="n">
-        <v>28067</v>
+        <v>30512</v>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>11/26</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -1560,10 +1560,10 @@
         </is>
       </c>
       <c r="J21" s="4" t="n">
-        <v>72974</v>
+        <v>72119</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>2806.7</v>
+        <v>2773.818181818182</v>
       </c>
     </row>
     <row r="22">
@@ -1596,11 +1596,11 @@
         </is>
       </c>
       <c r="G22" s="7" t="n">
-        <v>2066</v>
+        <v>1653</v>
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>13/27</t>
+          <t>14/27</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr">
@@ -1609,10 +1609,10 @@
         </is>
       </c>
       <c r="J22" s="7" t="n">
-        <v>4291</v>
+        <v>3188</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>158.9230769230769</v>
+        <v>118.0714285714286</v>
       </c>
     </row>
     <row r="23">
@@ -1645,11 +1645,11 @@
         </is>
       </c>
       <c r="G23" s="7" t="n">
-        <v>2208</v>
+        <v>2365</v>
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>10/24</t>
+          <t>11/24</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr">
@@ -1658,10 +1658,10 @@
         </is>
       </c>
       <c r="J23" s="7" t="n">
-        <v>5299</v>
+        <v>5160</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>220.8</v>
+        <v>215</v>
       </c>
     </row>
     <row r="24">
@@ -1694,11 +1694,11 @@
         </is>
       </c>
       <c r="G24" s="7" t="n">
-        <v>8044</v>
+        <v>8354</v>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>10/22</t>
+          <t>11/22</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr">
@@ -1707,10 +1707,10 @@
         </is>
       </c>
       <c r="J24" s="7" t="n">
-        <v>17697</v>
+        <v>16708</v>
       </c>
       <c r="K24" s="8" t="n">
-        <v>804.4</v>
+        <v>759.4545454545455</v>
       </c>
     </row>
     <row r="25">
@@ -1792,11 +1792,11 @@
         </is>
       </c>
       <c r="G26" s="7" t="n">
-        <v>7519</v>
+        <v>6082</v>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>9/22</t>
+          <t>10/22</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
@@ -1805,10 +1805,10 @@
         </is>
       </c>
       <c r="J26" s="7" t="n">
-        <v>18380</v>
+        <v>13380</v>
       </c>
       <c r="K26" s="8" t="n">
-        <v>835.4444444444445</v>
+        <v>608.2</v>
       </c>
     </row>
     <row r="27">
@@ -1939,11 +1939,11 @@
         </is>
       </c>
       <c r="G29" s="7" t="n">
-        <v>3126</v>
+        <v>3778</v>
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>8/25</t>
+          <t>9/25</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
@@ -1952,10 +1952,10 @@
         </is>
       </c>
       <c r="J29" s="7" t="n">
-        <v>9769</v>
+        <v>10494</v>
       </c>
       <c r="K29" s="8" t="n">
-        <v>390.75</v>
+        <v>419.7777777777778</v>
       </c>
     </row>
     <row r="30">
@@ -1988,11 +1988,11 @@
         </is>
       </c>
       <c r="G30" s="7" t="n">
-        <v>839</v>
+        <v>1365</v>
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>9/17</t>
+          <t>10/17</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
@@ -2001,10 +2001,10 @@
         </is>
       </c>
       <c r="J30" s="7" t="n">
-        <v>1585</v>
+        <v>2320</v>
       </c>
       <c r="K30" s="8" t="n">
-        <v>93.22222222222223</v>
+        <v>136.5</v>
       </c>
     </row>
     <row r="31">
@@ -2037,11 +2037,11 @@
         </is>
       </c>
       <c r="G31" s="4" t="n">
-        <v>18046</v>
+        <v>18962</v>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>20/24</t>
+          <t>21/24</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -2050,10 +2050,10 @@
         </is>
       </c>
       <c r="J31" s="4" t="n">
-        <v>21655</v>
+        <v>21671</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>902.3</v>
+        <v>902.952380952381</v>
       </c>
     </row>
     <row r="32">
@@ -2155,52 +2155,52 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="A34" s="6" t="inlineStr">
         <is>
           <t>COIMBATORE (NORTH)</t>
         </is>
       </c>
-      <c r="B34" s="3" t="n">
+      <c r="B34" s="6" t="n">
         <v>118</v>
       </c>
-      <c r="C34" s="3" t="inlineStr">
+      <c r="C34" s="6" t="inlineStr">
         <is>
           <t>V. SAMPATHKUMAR</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="inlineStr">
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
         <is>
           <t>DURAI. SENTHAMIL SELVAN B.E</t>
         </is>
       </c>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G34" s="4" t="n">
-        <v>5933</v>
-      </c>
-      <c r="H34" s="3" t="inlineStr">
-        <is>
-          <t>7/25</t>
-        </is>
-      </c>
-      <c r="I34" s="3" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J34" s="4" t="n">
-        <v>21189</v>
-      </c>
-      <c r="K34" s="5" t="n">
-        <v>847.5714285714284</v>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G34" s="7" t="n">
+        <v>6367</v>
+      </c>
+      <c r="H34" s="6" t="inlineStr">
+        <is>
+          <t>8/25</t>
+        </is>
+      </c>
+      <c r="I34" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J34" s="7" t="n">
+        <v>19897</v>
+      </c>
+      <c r="K34" s="8" t="n">
+        <v>795.875</v>
       </c>
     </row>
     <row r="35">
@@ -2233,11 +2233,11 @@
         </is>
       </c>
       <c r="G35" s="7" t="n">
-        <v>821</v>
+        <v>1124</v>
       </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>8/20</t>
+          <t>9/20</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
@@ -2246,10 +2246,10 @@
         </is>
       </c>
       <c r="J35" s="7" t="n">
-        <v>2052</v>
+        <v>2498</v>
       </c>
       <c r="K35" s="8" t="n">
-        <v>102.625</v>
+        <v>124.8888888888889</v>
       </c>
     </row>
     <row r="36">
@@ -2380,11 +2380,11 @@
         </is>
       </c>
       <c r="G38" s="7" t="n">
-        <v>1980</v>
+        <v>3182</v>
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>9/19</t>
+          <t>10/19</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr">
@@ -2393,10 +2393,10 @@
         </is>
       </c>
       <c r="J38" s="7" t="n">
-        <v>4180</v>
+        <v>6046</v>
       </c>
       <c r="K38" s="8" t="n">
-        <v>220</v>
+        <v>318.2</v>
       </c>
     </row>
     <row r="39">
@@ -2478,11 +2478,11 @@
         </is>
       </c>
       <c r="G40" s="7" t="n">
-        <v>9605</v>
+        <v>9771</v>
       </c>
       <c r="H40" s="6" t="inlineStr">
         <is>
-          <t>15/23</t>
+          <t>16/23</t>
         </is>
       </c>
       <c r="I40" s="6" t="inlineStr">
@@ -2491,10 +2491,10 @@
         </is>
       </c>
       <c r="J40" s="7" t="n">
-        <v>14728</v>
+        <v>14046</v>
       </c>
       <c r="K40" s="8" t="n">
-        <v>640.3333333333334</v>
+        <v>610.6875</v>
       </c>
     </row>
     <row r="41">
@@ -2527,11 +2527,11 @@
         </is>
       </c>
       <c r="G41" s="7" t="n">
-        <v>6186</v>
+        <v>7609</v>
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>14/23</t>
+          <t>15/23</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr">
@@ -2540,10 +2540,10 @@
         </is>
       </c>
       <c r="J41" s="7" t="n">
-        <v>10163</v>
+        <v>11667</v>
       </c>
       <c r="K41" s="8" t="n">
-        <v>441.8571428571428</v>
+        <v>507.2666666666667</v>
       </c>
     </row>
     <row r="42">
@@ -2557,30 +2557,30 @@
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
+          <t>SENTHILKUMAR. I.P</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
           <t>NAZEER RAJA. G</t>
         </is>
       </c>
-      <c r="D42" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E42" s="6" t="inlineStr">
-        <is>
-          <t>SENTHILKUMAR. I.P</t>
-        </is>
-      </c>
       <c r="F42" s="6" t="inlineStr">
         <is>
-          <t>Dravida Munnetra Kazhagam</t>
+          <t>Tamilaga Vettri Kazhagam</t>
         </is>
       </c>
       <c r="G42" s="7" t="n">
-        <v>1093</v>
+        <v>1005</v>
       </c>
       <c r="H42" s="6" t="inlineStr">
         <is>
-          <t>14/24</t>
+          <t>15/24</t>
         </is>
       </c>
       <c r="I42" s="6" t="inlineStr">
@@ -2589,10 +2589,10 @@
         </is>
       </c>
       <c r="J42" s="7" t="n">
-        <v>1874</v>
+        <v>1608</v>
       </c>
       <c r="K42" s="8" t="n">
-        <v>78.07142857142857</v>
+        <v>67</v>
       </c>
     </row>
     <row r="43">
@@ -2674,11 +2674,11 @@
         </is>
       </c>
       <c r="G44" s="4" t="n">
-        <v>54458</v>
+        <v>57809</v>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>14/25</t>
+          <t>15/25</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
@@ -2687,10 +2687,10 @@
         </is>
       </c>
       <c r="J44" s="4" t="n">
-        <v>97246</v>
+        <v>96348</v>
       </c>
       <c r="K44" s="5" t="n">
-        <v>3889.857142857142</v>
+        <v>3853.933333333333</v>
       </c>
     </row>
     <row r="45">
@@ -2772,11 +2772,11 @@
         </is>
       </c>
       <c r="G46" s="4" t="n">
-        <v>17719</v>
+        <v>17484</v>
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>12/19</t>
+          <t>13/19</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
@@ -2785,10 +2785,10 @@
         </is>
       </c>
       <c r="J46" s="4" t="n">
-        <v>28055</v>
+        <v>25554</v>
       </c>
       <c r="K46" s="5" t="n">
-        <v>1476.583333333333</v>
+        <v>1344.923076923077</v>
       </c>
     </row>
     <row r="47">
@@ -2821,11 +2821,11 @@
         </is>
       </c>
       <c r="G47" s="4" t="n">
-        <v>11184</v>
+        <v>13279</v>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>9/24</t>
+          <t>10/24</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
@@ -2834,10 +2834,10 @@
         </is>
       </c>
       <c r="J47" s="4" t="n">
-        <v>29824</v>
+        <v>31870</v>
       </c>
       <c r="K47" s="5" t="n">
-        <v>1242.666666666667</v>
+        <v>1327.9</v>
       </c>
     </row>
     <row r="48">
@@ -3017,11 +3017,11 @@
         </is>
       </c>
       <c r="G51" s="7" t="n">
-        <v>11964</v>
+        <v>13046</v>
       </c>
       <c r="H51" s="6" t="inlineStr">
         <is>
-          <t>15/23</t>
+          <t>16/23</t>
         </is>
       </c>
       <c r="I51" s="6" t="inlineStr">
@@ -3030,10 +3030,10 @@
         </is>
       </c>
       <c r="J51" s="7" t="n">
-        <v>18345</v>
+        <v>18754</v>
       </c>
       <c r="K51" s="8" t="n">
-        <v>797.6</v>
+        <v>815.375</v>
       </c>
     </row>
     <row r="52">
@@ -3075,7 +3075,7 @@
       </c>
       <c r="I52" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J52" s="4" t="n">
@@ -3164,11 +3164,11 @@
         </is>
       </c>
       <c r="G54" s="4" t="n">
-        <v>11906</v>
+        <v>13646</v>
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>10/25</t>
+          <t>11/25</t>
         </is>
       </c>
       <c r="I54" s="3" t="inlineStr">
@@ -3177,10 +3177,10 @@
         </is>
       </c>
       <c r="J54" s="4" t="n">
-        <v>29765</v>
+        <v>31014</v>
       </c>
       <c r="K54" s="5" t="n">
-        <v>1190.6</v>
+        <v>1240.545454545455</v>
       </c>
     </row>
     <row r="55">
@@ -3213,11 +3213,11 @@
         </is>
       </c>
       <c r="G55" s="7" t="n">
-        <v>4706</v>
+        <v>6443</v>
       </c>
       <c r="H55" s="6" t="inlineStr">
         <is>
-          <t>7/14</t>
+          <t>8/14</t>
         </is>
       </c>
       <c r="I55" s="6" t="inlineStr">
@@ -3226,10 +3226,10 @@
         </is>
       </c>
       <c r="J55" s="7" t="n">
-        <v>9412</v>
+        <v>11275</v>
       </c>
       <c r="K55" s="8" t="n">
-        <v>672.2857142857143</v>
+        <v>805.375</v>
       </c>
     </row>
     <row r="56">
@@ -3262,11 +3262,11 @@
         </is>
       </c>
       <c r="G56" s="7" t="n">
-        <v>3691</v>
+        <v>4248</v>
       </c>
       <c r="H56" s="6" t="inlineStr">
         <is>
-          <t>18/23</t>
+          <t>19/23</t>
         </is>
       </c>
       <c r="I56" s="6" t="inlineStr">
@@ -3275,10 +3275,10 @@
         </is>
       </c>
       <c r="J56" s="7" t="n">
-        <v>4716</v>
+        <v>5142</v>
       </c>
       <c r="K56" s="8" t="n">
-        <v>205.0555555555555</v>
+        <v>223.578947368421</v>
       </c>
     </row>
     <row r="57">
@@ -3331,52 +3331,52 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="inlineStr">
+      <c r="A58" s="6" t="inlineStr">
         <is>
           <t>JAYANKONDAM</t>
         </is>
       </c>
-      <c r="B58" s="3" t="n">
+      <c r="B58" s="6" t="n">
         <v>150</v>
       </c>
-      <c r="C58" s="3" t="inlineStr">
+      <c r="C58" s="6" t="inlineStr">
         <is>
           <t>VAITHILINGAM G.</t>
         </is>
       </c>
-      <c r="D58" s="3" t="inlineStr">
+      <c r="D58" s="6" t="inlineStr">
         <is>
           <t>Pattali Makkal Katchi</t>
         </is>
       </c>
-      <c r="E58" s="3" t="inlineStr">
+      <c r="E58" s="6" t="inlineStr">
         <is>
           <t>KANNAN KA.SO.KA.</t>
         </is>
       </c>
-      <c r="F58" s="3" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G58" s="4" t="n">
-        <v>10583</v>
-      </c>
-      <c r="H58" s="3" t="inlineStr">
-        <is>
-          <t>12/23</t>
-        </is>
-      </c>
-      <c r="I58" s="3" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J58" s="4" t="n">
-        <v>20284</v>
-      </c>
-      <c r="K58" s="5" t="n">
-        <v>881.9166666666666</v>
+      <c r="F58" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G58" s="7" t="n">
+        <v>10348</v>
+      </c>
+      <c r="H58" s="6" t="inlineStr">
+        <is>
+          <t>13/23</t>
+        </is>
+      </c>
+      <c r="I58" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J58" s="7" t="n">
+        <v>18308</v>
+      </c>
+      <c r="K58" s="8" t="n">
+        <v>796.0000000000001</v>
       </c>
     </row>
     <row r="59">
@@ -3409,11 +3409,11 @@
         </is>
       </c>
       <c r="G59" s="7" t="n">
-        <v>6986</v>
+        <v>8485</v>
       </c>
       <c r="H59" s="6" t="inlineStr">
         <is>
-          <t>9/21</t>
+          <t>11/21</t>
         </is>
       </c>
       <c r="I59" s="6" t="inlineStr">
@@ -3422,10 +3422,10 @@
         </is>
       </c>
       <c r="J59" s="7" t="n">
-        <v>16301</v>
+        <v>16199</v>
       </c>
       <c r="K59" s="8" t="n">
-        <v>776.2222222222222</v>
+        <v>771.3636363636364</v>
       </c>
     </row>
     <row r="60">
@@ -3458,11 +3458,11 @@
         </is>
       </c>
       <c r="G60" s="7" t="n">
-        <v>1912</v>
+        <v>2959</v>
       </c>
       <c r="H60" s="6" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>11/26</t>
         </is>
       </c>
       <c r="I60" s="6" t="inlineStr">
@@ -3471,10 +3471,10 @@
         </is>
       </c>
       <c r="J60" s="7" t="n">
-        <v>4971</v>
+        <v>6994</v>
       </c>
       <c r="K60" s="8" t="n">
-        <v>191.2</v>
+        <v>269</v>
       </c>
     </row>
     <row r="61">
@@ -3556,11 +3556,11 @@
         </is>
       </c>
       <c r="G62" s="7" t="n">
-        <v>1259</v>
+        <v>1472</v>
       </c>
       <c r="H62" s="6" t="inlineStr">
         <is>
-          <t>6/27</t>
+          <t>7/27</t>
         </is>
       </c>
       <c r="I62" s="6" t="inlineStr">
@@ -3569,10 +3569,10 @@
         </is>
       </c>
       <c r="J62" s="7" t="n">
-        <v>5666</v>
+        <v>5678</v>
       </c>
       <c r="K62" s="8" t="n">
-        <v>209.8333333333333</v>
+        <v>210.2857142857143</v>
       </c>
     </row>
     <row r="63">
@@ -3605,11 +3605,11 @@
         </is>
       </c>
       <c r="G63" s="7" t="n">
-        <v>2044</v>
+        <v>2446</v>
       </c>
       <c r="H63" s="6" t="inlineStr">
         <is>
-          <t>9/26</t>
+          <t>10/26</t>
         </is>
       </c>
       <c r="I63" s="6" t="inlineStr">
@@ -3618,10 +3618,10 @@
         </is>
       </c>
       <c r="J63" s="7" t="n">
-        <v>5905</v>
+        <v>6360</v>
       </c>
       <c r="K63" s="8" t="n">
-        <v>227.1111111111111</v>
+        <v>244.6</v>
       </c>
     </row>
     <row r="64">
@@ -3654,11 +3654,11 @@
         </is>
       </c>
       <c r="G64" s="7" t="n">
-        <v>3853</v>
+        <v>3346</v>
       </c>
       <c r="H64" s="6" t="inlineStr">
         <is>
-          <t>11/23</t>
+          <t>12/23</t>
         </is>
       </c>
       <c r="I64" s="6" t="inlineStr">
@@ -3667,10 +3667,10 @@
         </is>
       </c>
       <c r="J64" s="7" t="n">
-        <v>8056</v>
+        <v>6413</v>
       </c>
       <c r="K64" s="8" t="n">
-        <v>350.2727272727273</v>
+        <v>278.8333333333333</v>
       </c>
     </row>
     <row r="65">
@@ -3703,11 +3703,11 @@
         </is>
       </c>
       <c r="G65" s="7" t="n">
-        <v>1078</v>
+        <v>2153</v>
       </c>
       <c r="H65" s="6" t="inlineStr">
         <is>
-          <t>11/26</t>
+          <t>12/26</t>
         </is>
       </c>
       <c r="I65" s="6" t="inlineStr">
@@ -3716,10 +3716,10 @@
         </is>
       </c>
       <c r="J65" s="7" t="n">
-        <v>2548</v>
+        <v>4665</v>
       </c>
       <c r="K65" s="8" t="n">
-        <v>98</v>
+        <v>179.4166666666667</v>
       </c>
     </row>
     <row r="66">
@@ -3801,11 +3801,11 @@
         </is>
       </c>
       <c r="G67" s="7" t="n">
-        <v>3121</v>
+        <v>3742</v>
       </c>
       <c r="H67" s="6" t="inlineStr">
         <is>
-          <t>8/21</t>
+          <t>9/21</t>
         </is>
       </c>
       <c r="I67" s="6" t="inlineStr">
@@ -3814,10 +3814,10 @@
         </is>
       </c>
       <c r="J67" s="7" t="n">
-        <v>8193</v>
+        <v>8731</v>
       </c>
       <c r="K67" s="8" t="n">
-        <v>390.125</v>
+        <v>415.7777777777778</v>
       </c>
     </row>
     <row r="68">
@@ -3997,11 +3997,11 @@
         </is>
       </c>
       <c r="G71" s="7" t="n">
-        <v>774</v>
+        <v>1115</v>
       </c>
       <c r="H71" s="6" t="inlineStr">
         <is>
-          <t>10/22</t>
+          <t>11/22</t>
         </is>
       </c>
       <c r="I71" s="6" t="inlineStr">
@@ -4010,10 +4010,10 @@
         </is>
       </c>
       <c r="J71" s="7" t="n">
-        <v>1703</v>
+        <v>2230</v>
       </c>
       <c r="K71" s="8" t="n">
-        <v>77.40000000000001</v>
+        <v>101.3636363636364</v>
       </c>
     </row>
     <row r="72">
@@ -4095,11 +4095,11 @@
         </is>
       </c>
       <c r="G73" s="7" t="n">
-        <v>5556</v>
+        <v>6692</v>
       </c>
       <c r="H73" s="6" t="inlineStr">
         <is>
-          <t>6/19</t>
+          <t>7/19</t>
         </is>
       </c>
       <c r="I73" s="6" t="inlineStr">
@@ -4108,10 +4108,10 @@
         </is>
       </c>
       <c r="J73" s="7" t="n">
-        <v>17594</v>
+        <v>18164</v>
       </c>
       <c r="K73" s="8" t="n">
-        <v>926</v>
+        <v>956</v>
       </c>
     </row>
     <row r="74">
@@ -4340,11 +4340,11 @@
         </is>
       </c>
       <c r="G78" s="4" t="n">
-        <v>17967</v>
+        <v>17386</v>
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
-          <t>16/25</t>
+          <t>17/25</t>
         </is>
       </c>
       <c r="I78" s="3" t="inlineStr">
@@ -4353,10 +4353,10 @@
         </is>
       </c>
       <c r="J78" s="4" t="n">
-        <v>28073</v>
+        <v>25568</v>
       </c>
       <c r="K78" s="5" t="n">
-        <v>1122.9375</v>
+        <v>1022.705882352941</v>
       </c>
     </row>
     <row r="79">
@@ -4438,11 +4438,11 @@
         </is>
       </c>
       <c r="G80" s="7" t="n">
-        <v>530</v>
+        <v>928</v>
       </c>
       <c r="H80" s="6" t="inlineStr">
         <is>
-          <t>10/21</t>
+          <t>11/21</t>
         </is>
       </c>
       <c r="I80" s="6" t="inlineStr">
@@ -4451,10 +4451,10 @@
         </is>
       </c>
       <c r="J80" s="7" t="n">
-        <v>1113</v>
+        <v>1772</v>
       </c>
       <c r="K80" s="8" t="n">
-        <v>53</v>
+        <v>84.36363636363636</v>
       </c>
     </row>
     <row r="81">
@@ -4487,11 +4487,11 @@
         </is>
       </c>
       <c r="G81" s="7" t="n">
-        <v>3205</v>
+        <v>2455</v>
       </c>
       <c r="H81" s="6" t="inlineStr">
         <is>
-          <t>9/24</t>
+          <t>10/24</t>
         </is>
       </c>
       <c r="I81" s="6" t="inlineStr">
@@ -4500,59 +4500,59 @@
         </is>
       </c>
       <c r="J81" s="7" t="n">
-        <v>8547</v>
+        <v>5892</v>
       </c>
       <c r="K81" s="8" t="n">
-        <v>356.1111111111111</v>
+        <v>245.5</v>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="6" t="inlineStr">
+      <c r="A82" s="13" t="inlineStr">
         <is>
           <t>KUMBAKONAM</t>
         </is>
       </c>
-      <c r="B82" s="6" t="n">
+      <c r="B82" s="14" t="n">
         <v>171</v>
       </c>
-      <c r="C82" s="6" t="inlineStr">
+      <c r="C82" s="14" t="inlineStr">
         <is>
           <t>ANBALAGAN G</t>
         </is>
       </c>
-      <c r="D82" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E82" s="6" t="inlineStr">
+      <c r="D82" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E82" s="14" t="inlineStr">
         <is>
           <t>VINOTH</t>
         </is>
       </c>
-      <c r="F82" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G82" s="7" t="n">
-        <v>1314</v>
-      </c>
-      <c r="H82" s="6" t="inlineStr">
-        <is>
-          <t>16/22</t>
-        </is>
-      </c>
-      <c r="I82" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J82" s="7" t="n">
-        <v>1807</v>
-      </c>
-      <c r="K82" s="8" t="n">
-        <v>82.125</v>
+      <c r="F82" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G82" s="15" t="n">
+        <v>632</v>
+      </c>
+      <c r="H82" s="14" t="inlineStr">
+        <is>
+          <t>18/22</t>
+        </is>
+      </c>
+      <c r="I82" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J82" s="15" t="n">
+        <v>772</v>
+      </c>
+      <c r="K82" s="16" t="n">
+        <v>35.11111111111111</v>
       </c>
     </row>
     <row r="83">
@@ -4634,11 +4634,11 @@
         </is>
       </c>
       <c r="G84" s="7" t="n">
-        <v>522</v>
+        <v>776</v>
       </c>
       <c r="H84" s="6" t="inlineStr">
         <is>
-          <t>12/20</t>
+          <t>13/20</t>
         </is>
       </c>
       <c r="I84" s="6" t="inlineStr">
@@ -4647,10 +4647,10 @@
         </is>
       </c>
       <c r="J84" s="7" t="n">
-        <v>870</v>
+        <v>1194</v>
       </c>
       <c r="K84" s="8" t="n">
-        <v>43.5</v>
+        <v>59.69230769230769</v>
       </c>
     </row>
     <row r="85">
@@ -4683,11 +4683,11 @@
         </is>
       </c>
       <c r="G85" s="7" t="n">
-        <v>2806</v>
+        <v>2502</v>
       </c>
       <c r="H85" s="6" t="inlineStr">
         <is>
-          <t>10/20</t>
+          <t>11/20</t>
         </is>
       </c>
       <c r="I85" s="6" t="inlineStr">
@@ -4696,10 +4696,10 @@
         </is>
       </c>
       <c r="J85" s="7" t="n">
-        <v>5612</v>
+        <v>4549</v>
       </c>
       <c r="K85" s="8" t="n">
-        <v>280.6</v>
+        <v>227.4545454545455</v>
       </c>
     </row>
     <row r="86">
@@ -4732,11 +4732,11 @@
         </is>
       </c>
       <c r="G86" s="7" t="n">
-        <v>691</v>
+        <v>1725</v>
       </c>
       <c r="H86" s="6" t="inlineStr">
         <is>
-          <t>8/21</t>
+          <t>9/21</t>
         </is>
       </c>
       <c r="I86" s="6" t="inlineStr">
@@ -4745,10 +4745,10 @@
         </is>
       </c>
       <c r="J86" s="7" t="n">
-        <v>1814</v>
+        <v>4025</v>
       </c>
       <c r="K86" s="8" t="n">
-        <v>86.375</v>
+        <v>191.6666666666667</v>
       </c>
     </row>
     <row r="87">
@@ -4781,11 +4781,11 @@
         </is>
       </c>
       <c r="G87" s="4" t="n">
-        <v>61467</v>
+        <v>67983</v>
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
-          <t>13/19</t>
+          <t>14/19</t>
         </is>
       </c>
       <c r="I87" s="3" t="inlineStr">
@@ -4794,10 +4794,10 @@
         </is>
       </c>
       <c r="J87" s="4" t="n">
-        <v>89836</v>
+        <v>92263</v>
       </c>
       <c r="K87" s="5" t="n">
-        <v>4728.23076923077</v>
+        <v>4855.928571428572</v>
       </c>
     </row>
     <row r="88">
@@ -4879,11 +4879,11 @@
         </is>
       </c>
       <c r="G89" s="7" t="n">
-        <v>6633</v>
+        <v>5853</v>
       </c>
       <c r="H89" s="6" t="inlineStr">
         <is>
-          <t>15/29</t>
+          <t>16/29</t>
         </is>
       </c>
       <c r="I89" s="6" t="inlineStr">
@@ -4892,10 +4892,10 @@
         </is>
       </c>
       <c r="J89" s="7" t="n">
-        <v>12824</v>
+        <v>10609</v>
       </c>
       <c r="K89" s="8" t="n">
-        <v>442.1999999999999</v>
+        <v>365.8125</v>
       </c>
     </row>
     <row r="90">
@@ -4977,11 +4977,11 @@
         </is>
       </c>
       <c r="G91" s="4" t="n">
-        <v>14180</v>
+        <v>16384</v>
       </c>
       <c r="H91" s="3" t="inlineStr">
         <is>
-          <t>13/17</t>
+          <t>14/17</t>
         </is>
       </c>
       <c r="I91" s="3" t="inlineStr">
@@ -4990,10 +4990,10 @@
         </is>
       </c>
       <c r="J91" s="4" t="n">
-        <v>18543</v>
+        <v>19895</v>
       </c>
       <c r="K91" s="5" t="n">
-        <v>1090.769230769231</v>
+        <v>1170.285714285714</v>
       </c>
     </row>
     <row r="92">
@@ -5026,11 +5026,11 @@
         </is>
       </c>
       <c r="G92" s="7" t="n">
-        <v>2645</v>
+        <v>2887</v>
       </c>
       <c r="H92" s="6" t="inlineStr">
         <is>
-          <t>12/24</t>
+          <t>13/24</t>
         </is>
       </c>
       <c r="I92" s="6" t="inlineStr">
@@ -5039,10 +5039,10 @@
         </is>
       </c>
       <c r="J92" s="7" t="n">
-        <v>5290</v>
+        <v>5330</v>
       </c>
       <c r="K92" s="8" t="n">
-        <v>220.4166666666667</v>
+        <v>222.0769230769231</v>
       </c>
     </row>
     <row r="93">
@@ -5124,11 +5124,11 @@
         </is>
       </c>
       <c r="G94" s="4" t="n">
-        <v>19158</v>
+        <v>23376</v>
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
-          <t>7/25</t>
+          <t>8/25</t>
         </is>
       </c>
       <c r="I94" s="3" t="inlineStr">
@@ -5137,10 +5137,10 @@
         </is>
       </c>
       <c r="J94" s="4" t="n">
-        <v>68421</v>
+        <v>73050</v>
       </c>
       <c r="K94" s="5" t="n">
-        <v>2736.857142857143</v>
+        <v>2922</v>
       </c>
     </row>
     <row r="95">
@@ -5271,11 +5271,11 @@
         </is>
       </c>
       <c r="G97" s="7" t="n">
-        <v>4087</v>
+        <v>4031</v>
       </c>
       <c r="H97" s="6" t="inlineStr">
         <is>
-          <t>7/27</t>
+          <t>8/27</t>
         </is>
       </c>
       <c r="I97" s="6" t="inlineStr">
@@ -5284,10 +5284,10 @@
         </is>
       </c>
       <c r="J97" s="7" t="n">
-        <v>15764</v>
+        <v>13605</v>
       </c>
       <c r="K97" s="8" t="n">
-        <v>583.8571428571429</v>
+        <v>503.875</v>
       </c>
     </row>
     <row r="98">
@@ -5320,11 +5320,11 @@
         </is>
       </c>
       <c r="G98" s="7" t="n">
-        <v>3087</v>
+        <v>1851</v>
       </c>
       <c r="H98" s="6" t="inlineStr">
         <is>
-          <t>15/25</t>
+          <t>16/25</t>
         </is>
       </c>
       <c r="I98" s="6" t="inlineStr">
@@ -5333,10 +5333,10 @@
         </is>
       </c>
       <c r="J98" s="7" t="n">
-        <v>5145</v>
+        <v>2892</v>
       </c>
       <c r="K98" s="8" t="n">
-        <v>205.8</v>
+        <v>115.6875</v>
       </c>
     </row>
     <row r="99">
@@ -5369,11 +5369,11 @@
         </is>
       </c>
       <c r="G99" s="7" t="n">
-        <v>3165</v>
+        <v>2778</v>
       </c>
       <c r="H99" s="6" t="inlineStr">
         <is>
-          <t>12/22</t>
+          <t>13/22</t>
         </is>
       </c>
       <c r="I99" s="6" t="inlineStr">
@@ -5382,10 +5382,10 @@
         </is>
       </c>
       <c r="J99" s="7" t="n">
-        <v>5802</v>
+        <v>4701</v>
       </c>
       <c r="K99" s="8" t="n">
-        <v>263.75</v>
+        <v>213.6923076923077</v>
       </c>
     </row>
     <row r="100">
@@ -5418,11 +5418,11 @@
         </is>
       </c>
       <c r="G100" s="7" t="n">
-        <v>6104</v>
+        <v>5837</v>
       </c>
       <c r="H100" s="6" t="inlineStr">
         <is>
-          <t>9/22</t>
+          <t>10/22</t>
         </is>
       </c>
       <c r="I100" s="6" t="inlineStr">
@@ -5431,10 +5431,10 @@
         </is>
       </c>
       <c r="J100" s="7" t="n">
-        <v>14921</v>
+        <v>12841</v>
       </c>
       <c r="K100" s="8" t="n">
-        <v>678.2222222222222</v>
+        <v>583.7</v>
       </c>
     </row>
     <row r="101">
@@ -5467,11 +5467,11 @@
         </is>
       </c>
       <c r="G101" s="7" t="n">
-        <v>2706</v>
+        <v>2509</v>
       </c>
       <c r="H101" s="6" t="inlineStr">
         <is>
-          <t>19/21</t>
+          <t>20/21</t>
         </is>
       </c>
       <c r="I101" s="6" t="inlineStr">
@@ -5480,10 +5480,10 @@
         </is>
       </c>
       <c r="J101" s="7" t="n">
-        <v>2991</v>
+        <v>2634</v>
       </c>
       <c r="K101" s="8" t="n">
-        <v>142.421052631579</v>
+        <v>125.45</v>
       </c>
     </row>
     <row r="102">
@@ -5516,11 +5516,11 @@
         </is>
       </c>
       <c r="G102" s="7" t="n">
-        <v>2712</v>
+        <v>2296</v>
       </c>
       <c r="H102" s="6" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>11/26</t>
         </is>
       </c>
       <c r="I102" s="6" t="inlineStr">
@@ -5529,10 +5529,10 @@
         </is>
       </c>
       <c r="J102" s="7" t="n">
-        <v>7051</v>
+        <v>5427</v>
       </c>
       <c r="K102" s="8" t="n">
-        <v>271.2</v>
+        <v>208.7272727272727</v>
       </c>
     </row>
     <row r="103">
@@ -5614,11 +5614,11 @@
         </is>
       </c>
       <c r="G104" s="7" t="n">
-        <v>3820</v>
+        <v>4145</v>
       </c>
       <c r="H104" s="6" t="inlineStr">
         <is>
-          <t>12/21</t>
+          <t>13/21</t>
         </is>
       </c>
       <c r="I104" s="6" t="inlineStr">
@@ -5627,10 +5627,10 @@
         </is>
       </c>
       <c r="J104" s="7" t="n">
-        <v>6685</v>
+        <v>6696</v>
       </c>
       <c r="K104" s="8" t="n">
-        <v>318.3333333333333</v>
+        <v>318.8461538461539</v>
       </c>
     </row>
     <row r="105">
@@ -5654,20 +5654,20 @@
       </c>
       <c r="E105" s="6" t="inlineStr">
         <is>
-          <t>MALARVIZHI. B</t>
+          <t>S.PANDI</t>
         </is>
       </c>
       <c r="F105" s="6" t="inlineStr">
         <is>
-          <t>Tamilaga Vettri Kazhagam</t>
+          <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
       <c r="G105" s="7" t="n">
-        <v>7815</v>
+        <v>8171</v>
       </c>
       <c r="H105" s="6" t="inlineStr">
         <is>
-          <t>15/30</t>
+          <t>16/30</t>
         </is>
       </c>
       <c r="I105" s="6" t="inlineStr">
@@ -5676,10 +5676,10 @@
         </is>
       </c>
       <c r="J105" s="7" t="n">
-        <v>15630</v>
+        <v>15321</v>
       </c>
       <c r="K105" s="8" t="n">
-        <v>521</v>
+        <v>510.6875</v>
       </c>
     </row>
     <row r="106">
@@ -5761,11 +5761,11 @@
         </is>
       </c>
       <c r="G107" s="4" t="n">
-        <v>19501</v>
+        <v>20914</v>
       </c>
       <c r="H107" s="3" t="inlineStr">
         <is>
-          <t>13/20</t>
+          <t>14/20</t>
         </is>
       </c>
       <c r="I107" s="3" t="inlineStr">
@@ -5774,10 +5774,10 @@
         </is>
       </c>
       <c r="J107" s="4" t="n">
-        <v>30002</v>
+        <v>29877</v>
       </c>
       <c r="K107" s="5" t="n">
-        <v>1500.076923076923</v>
+        <v>1493.857142857143</v>
       </c>
     </row>
     <row r="108">
@@ -5830,150 +5830,150 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="9" t="inlineStr">
+      <c r="A109" s="6" t="inlineStr">
         <is>
           <t>NAGERCOIL</t>
         </is>
       </c>
-      <c r="B109" s="10" t="n">
+      <c r="B109" s="6" t="n">
         <v>230</v>
       </c>
-      <c r="C109" s="10" t="inlineStr">
+      <c r="C109" s="6" t="inlineStr">
         <is>
           <t>AUSTIN</t>
         </is>
       </c>
-      <c r="D109" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E109" s="10" t="inlineStr">
+      <c r="D109" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E109" s="6" t="inlineStr">
         <is>
           <t>BERVIN KINGS G</t>
         </is>
       </c>
-      <c r="F109" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G109" s="11" t="n">
-        <v>211</v>
-      </c>
-      <c r="H109" s="10" t="inlineStr">
-        <is>
-          <t>11/23</t>
-        </is>
-      </c>
-      <c r="I109" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J109" s="11" t="n">
-        <v>441</v>
-      </c>
-      <c r="K109" s="12" t="n">
-        <v>19.18181818181818</v>
+      <c r="F109" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G109" s="7" t="n">
+        <v>2232</v>
+      </c>
+      <c r="H109" s="6" t="inlineStr">
+        <is>
+          <t>12/23</t>
+        </is>
+      </c>
+      <c r="I109" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J109" s="7" t="n">
+        <v>4278</v>
+      </c>
+      <c r="K109" s="8" t="n">
+        <v>186</v>
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="13" t="inlineStr">
+      <c r="A110" s="9" t="inlineStr">
         <is>
           <t>NAMAKKAL</t>
         </is>
       </c>
-      <c r="B110" s="14" t="n">
+      <c r="B110" s="10" t="n">
         <v>94</v>
       </c>
-      <c r="C110" s="14" t="inlineStr">
+      <c r="C110" s="10" t="inlineStr">
         <is>
           <t>DILIP C S</t>
         </is>
       </c>
-      <c r="D110" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E110" s="14" t="inlineStr">
+      <c r="D110" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E110" s="10" t="inlineStr">
         <is>
           <t>SRIDEVI MOHAN P S</t>
         </is>
       </c>
-      <c r="F110" s="14" t="inlineStr">
+      <c r="F110" s="10" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G110" s="15" t="n">
+      <c r="G110" s="11" t="n">
         <v>49</v>
       </c>
-      <c r="H110" s="14" t="inlineStr">
+      <c r="H110" s="10" t="inlineStr">
         <is>
           <t>8/23</t>
         </is>
       </c>
-      <c r="I110" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J110" s="15" t="n">
+      <c r="I110" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J110" s="11" t="n">
         <v>141</v>
       </c>
-      <c r="K110" s="16" t="n">
+      <c r="K110" s="12" t="n">
         <v>6.125</v>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="6" t="inlineStr">
+      <c r="A111" s="2" t="inlineStr">
         <is>
           <t>NANGUNERI</t>
         </is>
       </c>
-      <c r="B111" s="6" t="n">
+      <c r="B111" s="3" t="n">
         <v>227</v>
       </c>
-      <c r="C111" s="6" t="inlineStr">
+      <c r="C111" s="3" t="inlineStr">
         <is>
           <t>REDDIARPATTI V. NARAYANAN</t>
         </is>
       </c>
-      <c r="D111" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E111" s="6" t="inlineStr">
+      <c r="D111" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E111" s="3" t="inlineStr">
         <is>
           <t>RUBY.R.MANOHARAN</t>
         </is>
       </c>
-      <c r="F111" s="6" t="inlineStr">
+      <c r="F111" s="3" t="inlineStr">
         <is>
           <t>Indian National Congress</t>
         </is>
       </c>
-      <c r="G111" s="7" t="n">
-        <v>8783</v>
-      </c>
-      <c r="H111" s="6" t="inlineStr">
-        <is>
-          <t>18/25</t>
-        </is>
-      </c>
-      <c r="I111" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J111" s="7" t="n">
-        <v>12199</v>
-      </c>
-      <c r="K111" s="8" t="n">
-        <v>487.9444444444445</v>
+      <c r="G111" s="4" t="n">
+        <v>9599</v>
+      </c>
+      <c r="H111" s="3" t="inlineStr">
+        <is>
+          <t>19/25</t>
+        </is>
+      </c>
+      <c r="I111" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J111" s="4" t="n">
+        <v>12630</v>
+      </c>
+      <c r="K111" s="5" t="n">
+        <v>505.2105263157895</v>
       </c>
     </row>
     <row r="112">
@@ -6006,11 +6006,11 @@
         </is>
       </c>
       <c r="G112" s="4" t="n">
-        <v>24173</v>
+        <v>26020</v>
       </c>
       <c r="H112" s="3" t="inlineStr">
         <is>
-          <t>14/25</t>
+          <t>15/25</t>
         </is>
       </c>
       <c r="I112" s="3" t="inlineStr">
@@ -6019,10 +6019,10 @@
         </is>
       </c>
       <c r="J112" s="4" t="n">
-        <v>43166</v>
+        <v>43367</v>
       </c>
       <c r="K112" s="5" t="n">
-        <v>1726.642857142857</v>
+        <v>1734.666666666667</v>
       </c>
     </row>
     <row r="113">
@@ -6055,11 +6055,11 @@
         </is>
       </c>
       <c r="G113" s="7" t="n">
-        <v>5232</v>
+        <v>5567</v>
       </c>
       <c r="H113" s="6" t="inlineStr">
         <is>
-          <t>13/26</t>
+          <t>14/26</t>
         </is>
       </c>
       <c r="I113" s="6" t="inlineStr">
@@ -6068,10 +6068,10 @@
         </is>
       </c>
       <c r="J113" s="7" t="n">
-        <v>10464</v>
+        <v>10339</v>
       </c>
       <c r="K113" s="8" t="n">
-        <v>402.4615384615385</v>
+        <v>397.6428571428572</v>
       </c>
     </row>
     <row r="114">
@@ -6202,11 +6202,11 @@
         </is>
       </c>
       <c r="G116" s="4" t="n">
-        <v>22813</v>
+        <v>23696</v>
       </c>
       <c r="H116" s="3" t="inlineStr">
         <is>
-          <t>12/24</t>
+          <t>13/24</t>
         </is>
       </c>
       <c r="I116" s="3" t="inlineStr">
@@ -6215,10 +6215,10 @@
         </is>
       </c>
       <c r="J116" s="4" t="n">
-        <v>45626</v>
+        <v>43746</v>
       </c>
       <c r="K116" s="5" t="n">
-        <v>1901.083333333333</v>
+        <v>1822.769230769231</v>
       </c>
     </row>
     <row r="117">
@@ -6251,11 +6251,11 @@
         </is>
       </c>
       <c r="G117" s="7" t="n">
-        <v>3727</v>
+        <v>3449</v>
       </c>
       <c r="H117" s="6" t="inlineStr">
         <is>
-          <t>12/26</t>
+          <t>13/26</t>
         </is>
       </c>
       <c r="I117" s="6" t="inlineStr">
@@ -6264,10 +6264,10 @@
         </is>
       </c>
       <c r="J117" s="7" t="n">
-        <v>8075</v>
+        <v>6898</v>
       </c>
       <c r="K117" s="8" t="n">
-        <v>310.5833333333333</v>
+        <v>265.3076923076923</v>
       </c>
     </row>
     <row r="118">
@@ -6300,11 +6300,11 @@
         </is>
       </c>
       <c r="G118" s="4" t="n">
-        <v>21040</v>
+        <v>23237</v>
       </c>
       <c r="H118" s="3" t="inlineStr">
         <is>
-          <t>15/23</t>
+          <t>16/23</t>
         </is>
       </c>
       <c r="I118" s="3" t="inlineStr">
@@ -6313,10 +6313,10 @@
         </is>
       </c>
       <c r="J118" s="4" t="n">
-        <v>32261</v>
+        <v>33403</v>
       </c>
       <c r="K118" s="5" t="n">
-        <v>1402.666666666667</v>
+        <v>1452.3125</v>
       </c>
     </row>
     <row r="119">
@@ -6349,11 +6349,11 @@
         </is>
       </c>
       <c r="G119" s="4" t="n">
-        <v>17875</v>
+        <v>19273</v>
       </c>
       <c r="H119" s="3" t="inlineStr">
         <is>
-          <t>11/23</t>
+          <t>12/23</t>
         </is>
       </c>
       <c r="I119" s="3" t="inlineStr">
@@ -6362,10 +6362,10 @@
         </is>
       </c>
       <c r="J119" s="4" t="n">
-        <v>37375</v>
+        <v>36940</v>
       </c>
       <c r="K119" s="5" t="n">
-        <v>1625</v>
+        <v>1606.083333333333</v>
       </c>
     </row>
     <row r="120">
@@ -6447,11 +6447,11 @@
         </is>
       </c>
       <c r="G121" s="4" t="n">
-        <v>22255</v>
+        <v>24005</v>
       </c>
       <c r="H121" s="3" t="inlineStr">
         <is>
-          <t>14/23</t>
+          <t>15/23</t>
         </is>
       </c>
       <c r="I121" s="3" t="inlineStr">
@@ -6460,10 +6460,10 @@
         </is>
       </c>
       <c r="J121" s="4" t="n">
-        <v>36562</v>
+        <v>36808</v>
       </c>
       <c r="K121" s="5" t="n">
-        <v>1589.642857142857</v>
+        <v>1600.333333333333</v>
       </c>
     </row>
     <row r="122">
@@ -6496,11 +6496,11 @@
         </is>
       </c>
       <c r="G122" s="7" t="n">
-        <v>1188</v>
+        <v>2061</v>
       </c>
       <c r="H122" s="6" t="inlineStr">
         <is>
-          <t>12/25</t>
+          <t>13/25</t>
         </is>
       </c>
       <c r="I122" s="6" t="inlineStr">
@@ -6509,59 +6509,59 @@
         </is>
       </c>
       <c r="J122" s="7" t="n">
-        <v>2475</v>
+        <v>3963</v>
       </c>
       <c r="K122" s="8" t="n">
-        <v>99</v>
+        <v>158.5384615384615</v>
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="6" t="inlineStr">
+      <c r="A123" s="2" t="inlineStr">
         <is>
           <t>PALAYAMKOTTAI</t>
         </is>
       </c>
-      <c r="B123" s="6" t="n">
+      <c r="B123" s="3" t="n">
         <v>226</v>
       </c>
-      <c r="C123" s="6" t="inlineStr">
+      <c r="C123" s="3" t="inlineStr">
         <is>
           <t>MARIA JOHN</t>
         </is>
       </c>
-      <c r="D123" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E123" s="6" t="inlineStr">
+      <c r="D123" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E123" s="3" t="inlineStr">
         <is>
           <t>M.ABDUL WAHAB</t>
         </is>
       </c>
-      <c r="F123" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G123" s="7" t="n">
-        <v>8811</v>
-      </c>
-      <c r="H123" s="6" t="inlineStr">
-        <is>
-          <t>16/22</t>
-        </is>
-      </c>
-      <c r="I123" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J123" s="7" t="n">
-        <v>12115</v>
-      </c>
-      <c r="K123" s="8" t="n">
-        <v>550.6875</v>
+      <c r="F123" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G123" s="4" t="n">
+        <v>5606</v>
+      </c>
+      <c r="H123" s="3" t="inlineStr">
+        <is>
+          <t>17/22</t>
+        </is>
+      </c>
+      <c r="I123" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J123" s="4" t="n">
+        <v>7255</v>
+      </c>
+      <c r="K123" s="5" t="n">
+        <v>329.7647058823529</v>
       </c>
     </row>
     <row r="124">
@@ -6594,11 +6594,11 @@
         </is>
       </c>
       <c r="G124" s="4" t="n">
-        <v>12266</v>
+        <v>13893</v>
       </c>
       <c r="H124" s="3" t="inlineStr">
         <is>
-          <t>14/35</t>
+          <t>15/35</t>
         </is>
       </c>
       <c r="I124" s="3" t="inlineStr">
@@ -6607,10 +6607,10 @@
         </is>
       </c>
       <c r="J124" s="4" t="n">
-        <v>30665</v>
+        <v>32417</v>
       </c>
       <c r="K124" s="5" t="n">
-        <v>876.1428571428571</v>
+        <v>926.2</v>
       </c>
     </row>
     <row r="125">
@@ -6692,11 +6692,11 @@
         </is>
       </c>
       <c r="G126" s="7" t="n">
-        <v>5219</v>
+        <v>6559</v>
       </c>
       <c r="H126" s="6" t="inlineStr">
         <is>
-          <t>15/23</t>
+          <t>16/23</t>
         </is>
       </c>
       <c r="I126" s="6" t="inlineStr">
@@ -6705,10 +6705,10 @@
         </is>
       </c>
       <c r="J126" s="7" t="n">
-        <v>8002</v>
+        <v>9429</v>
       </c>
       <c r="K126" s="8" t="n">
-        <v>347.9333333333333</v>
+        <v>409.9375</v>
       </c>
     </row>
     <row r="127">
@@ -6741,11 +6741,11 @@
         </is>
       </c>
       <c r="G127" s="7" t="n">
-        <v>1875</v>
+        <v>4981</v>
       </c>
       <c r="H127" s="6" t="inlineStr">
         <is>
-          <t>8/23</t>
+          <t>9/23</t>
         </is>
       </c>
       <c r="I127" s="6" t="inlineStr">
@@ -6754,10 +6754,10 @@
         </is>
       </c>
       <c r="J127" s="7" t="n">
-        <v>5391</v>
+        <v>12729</v>
       </c>
       <c r="K127" s="8" t="n">
-        <v>234.375</v>
+        <v>553.4444444444445</v>
       </c>
     </row>
     <row r="128">
@@ -6790,11 +6790,11 @@
         </is>
       </c>
       <c r="G128" s="4" t="n">
-        <v>36152</v>
+        <v>36425</v>
       </c>
       <c r="H128" s="3" t="inlineStr">
         <is>
-          <t>15/23</t>
+          <t>16/23</t>
         </is>
       </c>
       <c r="I128" s="3" t="inlineStr">
@@ -6803,10 +6803,10 @@
         </is>
       </c>
       <c r="J128" s="4" t="n">
-        <v>55433</v>
+        <v>52361</v>
       </c>
       <c r="K128" s="5" t="n">
-        <v>2410.133333333333</v>
+        <v>2276.5625</v>
       </c>
     </row>
     <row r="129">
@@ -6839,11 +6839,11 @@
         </is>
       </c>
       <c r="G129" s="7" t="n">
-        <v>1730</v>
+        <v>1946</v>
       </c>
       <c r="H129" s="6" t="inlineStr">
         <is>
-          <t>13/24</t>
+          <t>14/24</t>
         </is>
       </c>
       <c r="I129" s="6" t="inlineStr">
@@ -6852,10 +6852,10 @@
         </is>
       </c>
       <c r="J129" s="7" t="n">
-        <v>3194</v>
+        <v>3336</v>
       </c>
       <c r="K129" s="8" t="n">
-        <v>133.0769230769231</v>
+        <v>139</v>
       </c>
     </row>
     <row r="130">
@@ -6986,11 +6986,11 @@
         </is>
       </c>
       <c r="G132" s="7" t="n">
-        <v>5684</v>
+        <v>5300</v>
       </c>
       <c r="H132" s="6" t="inlineStr">
         <is>
-          <t>7/23</t>
+          <t>8/23</t>
         </is>
       </c>
       <c r="I132" s="6" t="inlineStr">
@@ -6999,10 +6999,10 @@
         </is>
       </c>
       <c r="J132" s="7" t="n">
-        <v>18676</v>
+        <v>15238</v>
       </c>
       <c r="K132" s="8" t="n">
-        <v>812</v>
+        <v>662.5</v>
       </c>
     </row>
     <row r="133">
@@ -7084,11 +7084,11 @@
         </is>
       </c>
       <c r="G134" s="4" t="n">
-        <v>19100</v>
+        <v>21275</v>
       </c>
       <c r="H134" s="3" t="inlineStr">
         <is>
-          <t>8/22</t>
+          <t>9/22</t>
         </is>
       </c>
       <c r="I134" s="3" t="inlineStr">
@@ -7097,10 +7097,10 @@
         </is>
       </c>
       <c r="J134" s="4" t="n">
-        <v>52525</v>
+        <v>52006</v>
       </c>
       <c r="K134" s="5" t="n">
-        <v>2387.5</v>
+        <v>2363.888888888889</v>
       </c>
     </row>
     <row r="135">
@@ -7182,11 +7182,11 @@
         </is>
       </c>
       <c r="G136" s="7" t="n">
-        <v>1884</v>
+        <v>2209</v>
       </c>
       <c r="H136" s="6" t="inlineStr">
         <is>
-          <t>9/26</t>
+          <t>10/26</t>
         </is>
       </c>
       <c r="I136" s="6" t="inlineStr">
@@ -7195,10 +7195,10 @@
         </is>
       </c>
       <c r="J136" s="7" t="n">
-        <v>5443</v>
+        <v>5743</v>
       </c>
       <c r="K136" s="8" t="n">
-        <v>209.3333333333333</v>
+        <v>220.9</v>
       </c>
     </row>
     <row r="137">
@@ -7251,52 +7251,52 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="9" t="inlineStr">
+      <c r="A138" s="13" t="inlineStr">
         <is>
           <t>POLLACHI</t>
         </is>
       </c>
-      <c r="B138" s="10" t="n">
+      <c r="B138" s="14" t="n">
         <v>123</v>
       </c>
-      <c r="C138" s="10" t="inlineStr">
+      <c r="C138" s="14" t="inlineStr">
+        <is>
+          <t>K. NITHYANANDHAN</t>
+        </is>
+      </c>
+      <c r="D138" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E138" s="14" t="inlineStr">
         <is>
           <t>POLLACHI V. JAYARAMAN</t>
         </is>
       </c>
-      <c r="D138" s="10" t="inlineStr">
+      <c r="F138" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E138" s="10" t="inlineStr">
-        <is>
-          <t>K. NITHYANANDHAN</t>
-        </is>
-      </c>
-      <c r="F138" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G138" s="11" t="n">
-        <v>535</v>
-      </c>
-      <c r="H138" s="10" t="inlineStr">
-        <is>
-          <t>14/20</t>
-        </is>
-      </c>
-      <c r="I138" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J138" s="11" t="n">
-        <v>764</v>
-      </c>
-      <c r="K138" s="12" t="n">
-        <v>38.21428571428572</v>
+      <c r="G138" s="15" t="n">
+        <v>232</v>
+      </c>
+      <c r="H138" s="14" t="inlineStr">
+        <is>
+          <t>15/20</t>
+        </is>
+      </c>
+      <c r="I138" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J138" s="15" t="n">
+        <v>309</v>
+      </c>
+      <c r="K138" s="16" t="n">
+        <v>15.46666666666667</v>
       </c>
     </row>
     <row r="139">
@@ -7329,11 +7329,11 @@
         </is>
       </c>
       <c r="G139" s="7" t="n">
-        <v>1854</v>
+        <v>1431</v>
       </c>
       <c r="H139" s="6" t="inlineStr">
         <is>
-          <t>7/22</t>
+          <t>8/22</t>
         </is>
       </c>
       <c r="I139" s="6" t="inlineStr">
@@ -7342,10 +7342,10 @@
         </is>
       </c>
       <c r="J139" s="7" t="n">
-        <v>5827</v>
+        <v>3935</v>
       </c>
       <c r="K139" s="8" t="n">
-        <v>264.8571428571428</v>
+        <v>178.875</v>
       </c>
     </row>
     <row r="140">
@@ -7378,7 +7378,7 @@
         </is>
       </c>
       <c r="G140" s="4" t="n">
-        <v>29155</v>
+        <v>29235</v>
       </c>
       <c r="H140" s="3" t="inlineStr">
         <is>
@@ -7391,10 +7391,10 @@
         </is>
       </c>
       <c r="J140" s="4" t="n">
-        <v>53825</v>
+        <v>53972</v>
       </c>
       <c r="K140" s="5" t="n">
-        <v>2242.692307692308</v>
+        <v>2248.846153846154</v>
       </c>
     </row>
     <row r="141">
@@ -7476,11 +7476,11 @@
         </is>
       </c>
       <c r="G142" s="4" t="n">
-        <v>41556</v>
+        <v>45877</v>
       </c>
       <c r="H142" s="3" t="inlineStr">
         <is>
-          <t>12/23</t>
+          <t>13/23</t>
         </is>
       </c>
       <c r="I142" s="3" t="inlineStr">
@@ -7489,10 +7489,10 @@
         </is>
       </c>
       <c r="J142" s="4" t="n">
-        <v>79649</v>
+        <v>81167</v>
       </c>
       <c r="K142" s="5" t="n">
-        <v>3463</v>
+        <v>3529</v>
       </c>
     </row>
     <row r="143">
@@ -7574,11 +7574,11 @@
         </is>
       </c>
       <c r="G144" s="4" t="n">
-        <v>6870</v>
+        <v>7768</v>
       </c>
       <c r="H144" s="3" t="inlineStr">
         <is>
-          <t>18/24</t>
+          <t>19/24</t>
         </is>
       </c>
       <c r="I144" s="3" t="inlineStr">
@@ -7587,10 +7587,10 @@
         </is>
       </c>
       <c r="J144" s="4" t="n">
-        <v>9160</v>
+        <v>9812</v>
       </c>
       <c r="K144" s="5" t="n">
-        <v>381.6666666666667</v>
+        <v>408.8421052631579</v>
       </c>
     </row>
     <row r="145">
@@ -7623,11 +7623,11 @@
         </is>
       </c>
       <c r="G145" s="7" t="n">
-        <v>9331</v>
+        <v>8662</v>
       </c>
       <c r="H145" s="6" t="inlineStr">
         <is>
-          <t>11/20</t>
+          <t>12/20</t>
         </is>
       </c>
       <c r="I145" s="6" t="inlineStr">
@@ -7636,10 +7636,10 @@
         </is>
       </c>
       <c r="J145" s="7" t="n">
-        <v>16965</v>
+        <v>14437</v>
       </c>
       <c r="K145" s="8" t="n">
-        <v>848.2727272727273</v>
+        <v>721.8333333333334</v>
       </c>
     </row>
     <row r="146">
@@ -7672,11 +7672,11 @@
         </is>
       </c>
       <c r="G146" s="7" t="n">
-        <v>12407</v>
+        <v>13400</v>
       </c>
       <c r="H146" s="6" t="inlineStr">
         <is>
-          <t>19/29</t>
+          <t>20/29</t>
         </is>
       </c>
       <c r="I146" s="6" t="inlineStr">
@@ -7685,10 +7685,10 @@
         </is>
       </c>
       <c r="J146" s="7" t="n">
-        <v>18937</v>
+        <v>19430</v>
       </c>
       <c r="K146" s="8" t="n">
-        <v>653</v>
+        <v>670</v>
       </c>
     </row>
     <row r="147">
@@ -7721,11 +7721,11 @@
         </is>
       </c>
       <c r="G147" s="7" t="n">
-        <v>6308</v>
+        <v>4673</v>
       </c>
       <c r="H147" s="6" t="inlineStr">
         <is>
-          <t>10/22</t>
+          <t>11/22</t>
         </is>
       </c>
       <c r="I147" s="6" t="inlineStr">
@@ -7734,10 +7734,10 @@
         </is>
       </c>
       <c r="J147" s="7" t="n">
-        <v>13878</v>
+        <v>9346</v>
       </c>
       <c r="K147" s="8" t="n">
-        <v>630.8</v>
+        <v>424.8181818181818</v>
       </c>
     </row>
     <row r="148">
@@ -7966,11 +7966,11 @@
         </is>
       </c>
       <c r="G152" s="7" t="n">
-        <v>5508</v>
+        <v>6479</v>
       </c>
       <c r="H152" s="6" t="inlineStr">
         <is>
-          <t>10/21</t>
+          <t>11/21</t>
         </is>
       </c>
       <c r="I152" s="6" t="inlineStr">
@@ -7979,10 +7979,10 @@
         </is>
       </c>
       <c r="J152" s="7" t="n">
-        <v>11567</v>
+        <v>12369</v>
       </c>
       <c r="K152" s="8" t="n">
-        <v>550.8</v>
+        <v>589</v>
       </c>
     </row>
     <row r="153">
@@ -8015,11 +8015,11 @@
         </is>
       </c>
       <c r="G153" s="4" t="n">
-        <v>22547</v>
+        <v>25110</v>
       </c>
       <c r="H153" s="3" t="inlineStr">
         <is>
-          <t>11/20</t>
+          <t>12/20</t>
         </is>
       </c>
       <c r="I153" s="3" t="inlineStr">
@@ -8028,10 +8028,10 @@
         </is>
       </c>
       <c r="J153" s="4" t="n">
-        <v>40995</v>
+        <v>41850</v>
       </c>
       <c r="K153" s="5" t="n">
-        <v>2049.727272727273</v>
+        <v>2092.5</v>
       </c>
     </row>
     <row r="154">
@@ -8064,11 +8064,11 @@
         </is>
       </c>
       <c r="G154" s="4" t="n">
-        <v>22570</v>
+        <v>26034</v>
       </c>
       <c r="H154" s="3" t="inlineStr">
         <is>
-          <t>7/23</t>
+          <t>8/23</t>
         </is>
       </c>
       <c r="I154" s="3" t="inlineStr">
@@ -8077,10 +8077,10 @@
         </is>
       </c>
       <c r="J154" s="4" t="n">
-        <v>74159</v>
+        <v>74848</v>
       </c>
       <c r="K154" s="5" t="n">
-        <v>3224.285714285714</v>
+        <v>3254.25</v>
       </c>
     </row>
     <row r="155">
@@ -8113,11 +8113,11 @@
         </is>
       </c>
       <c r="G155" s="7" t="n">
-        <v>1530</v>
+        <v>1836</v>
       </c>
       <c r="H155" s="6" t="inlineStr">
         <is>
-          <t>13/23</t>
+          <t>14/23</t>
         </is>
       </c>
       <c r="I155" s="6" t="inlineStr">
@@ -8126,58 +8126,58 @@
         </is>
       </c>
       <c r="J155" s="7" t="n">
-        <v>2707</v>
+        <v>3016</v>
       </c>
       <c r="K155" s="8" t="n">
-        <v>117.6923076923077</v>
+        <v>131.1428571428571</v>
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="9" t="inlineStr">
+      <c r="A156" s="13" t="inlineStr">
         <is>
           <t>SANKARAPURAM</t>
         </is>
       </c>
-      <c r="B156" s="10" t="n">
+      <c r="B156" s="14" t="n">
         <v>79</v>
       </c>
-      <c r="C156" s="10" t="inlineStr">
+      <c r="C156" s="14" t="inlineStr">
         <is>
           <t>UDHAYASURIYAN T</t>
         </is>
       </c>
-      <c r="D156" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E156" s="10" t="inlineStr">
+      <c r="D156" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E156" s="14" t="inlineStr">
         <is>
           <t>RAKESH R</t>
         </is>
       </c>
-      <c r="F156" s="10" t="inlineStr">
+      <c r="F156" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G156" s="11" t="n">
+      <c r="G156" s="15" t="n">
         <v>254</v>
       </c>
-      <c r="H156" s="10" t="inlineStr">
+      <c r="H156" s="14" t="inlineStr">
         <is>
           <t>7/25</t>
         </is>
       </c>
-      <c r="I156" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J156" s="11" t="n">
+      <c r="I156" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J156" s="15" t="n">
         <v>907</v>
       </c>
-      <c r="K156" s="12" t="n">
+      <c r="K156" s="16" t="n">
         <v>36.28571428571428</v>
       </c>
     </row>
@@ -8211,11 +8211,11 @@
         </is>
       </c>
       <c r="G157" s="7" t="n">
-        <v>3516</v>
+        <v>4777</v>
       </c>
       <c r="H157" s="6" t="inlineStr">
         <is>
-          <t>13/25</t>
+          <t>14/25</t>
         </is>
       </c>
       <c r="I157" s="6" t="inlineStr">
@@ -8224,10 +8224,10 @@
         </is>
       </c>
       <c r="J157" s="7" t="n">
-        <v>6762</v>
+        <v>8530</v>
       </c>
       <c r="K157" s="8" t="n">
-        <v>270.4615384615385</v>
+        <v>341.2142857142857</v>
       </c>
     </row>
     <row r="158">
@@ -8251,20 +8251,20 @@
       </c>
       <c r="E158" s="6" t="inlineStr">
         <is>
-          <t>KADARKARAIRAJ. A</t>
+          <t>NAINAR NAGENTHRAN</t>
         </is>
       </c>
       <c r="F158" s="6" t="inlineStr">
         <is>
-          <t>Dravida Munnetra Kazhagam</t>
+          <t>Bharatiya Janata Party</t>
         </is>
       </c>
       <c r="G158" s="7" t="n">
-        <v>654</v>
+        <v>648</v>
       </c>
       <c r="H158" s="6" t="inlineStr">
         <is>
-          <t>4/21</t>
+          <t>5/21</t>
         </is>
       </c>
       <c r="I158" s="6" t="inlineStr">
@@ -8273,10 +8273,10 @@
         </is>
       </c>
       <c r="J158" s="7" t="n">
-        <v>3434</v>
+        <v>2722</v>
       </c>
       <c r="K158" s="8" t="n">
-        <v>163.5</v>
+        <v>129.6</v>
       </c>
     </row>
     <row r="159">
@@ -8309,11 +8309,11 @@
         </is>
       </c>
       <c r="G159" s="7" t="n">
-        <v>2976</v>
+        <v>3404</v>
       </c>
       <c r="H159" s="6" t="inlineStr">
         <is>
-          <t>12/22</t>
+          <t>13/22</t>
         </is>
       </c>
       <c r="I159" s="6" t="inlineStr">
@@ -8322,10 +8322,10 @@
         </is>
       </c>
       <c r="J159" s="7" t="n">
-        <v>5456</v>
+        <v>5761</v>
       </c>
       <c r="K159" s="8" t="n">
-        <v>248</v>
+        <v>261.8461538461539</v>
       </c>
     </row>
     <row r="160">
@@ -8398,20 +8398,20 @@
       </c>
       <c r="E161" s="6" t="inlineStr">
         <is>
-          <t>A.M.MUNIRATHINAM</t>
+          <t>K.SARAVANAN</t>
         </is>
       </c>
       <c r="F161" s="6" t="inlineStr">
         <is>
-          <t>Indian National Congress</t>
+          <t>Pattali Makkal Katchi</t>
         </is>
       </c>
       <c r="G161" s="7" t="n">
-        <v>3838</v>
+        <v>2909</v>
       </c>
       <c r="H161" s="6" t="inlineStr">
         <is>
-          <t>7/25</t>
+          <t>8/25</t>
         </is>
       </c>
       <c r="I161" s="6" t="inlineStr">
@@ -8420,10 +8420,10 @@
         </is>
       </c>
       <c r="J161" s="7" t="n">
-        <v>13707</v>
+        <v>9091</v>
       </c>
       <c r="K161" s="8" t="n">
-        <v>548.2857142857142</v>
+        <v>363.625</v>
       </c>
     </row>
     <row r="162">
@@ -8603,11 +8603,11 @@
         </is>
       </c>
       <c r="G165" s="7" t="n">
-        <v>5936</v>
+        <v>6650</v>
       </c>
       <c r="H165" s="6" t="inlineStr">
         <is>
-          <t>10/29</t>
+          <t>11/29</t>
         </is>
       </c>
       <c r="I165" s="6" t="inlineStr">
@@ -8616,58 +8616,58 @@
         </is>
       </c>
       <c r="J165" s="7" t="n">
-        <v>17214</v>
+        <v>17532</v>
       </c>
       <c r="K165" s="8" t="n">
-        <v>593.6</v>
+        <v>604.5454545454545</v>
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="9" t="inlineStr">
+      <c r="A166" s="13" t="inlineStr">
         <is>
           <t>SIVAKASI</t>
         </is>
       </c>
-      <c r="B166" s="10" t="n">
+      <c r="B166" s="14" t="n">
         <v>205</v>
       </c>
-      <c r="C166" s="10" t="inlineStr">
+      <c r="C166" s="14" t="inlineStr">
         <is>
           <t>RAJENTHRABHALAJI K T</t>
         </is>
       </c>
-      <c r="D166" s="10" t="inlineStr">
+      <c r="D166" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E166" s="10" t="inlineStr">
+      <c r="E166" s="14" t="inlineStr">
         <is>
           <t>KEERTHANA S</t>
         </is>
       </c>
-      <c r="F166" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G166" s="11" t="n">
+      <c r="F166" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G166" s="15" t="n">
         <v>63</v>
       </c>
-      <c r="H166" s="10" t="inlineStr">
+      <c r="H166" s="14" t="inlineStr">
         <is>
           <t>6/21</t>
         </is>
       </c>
-      <c r="I166" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J166" s="11" t="n">
+      <c r="I166" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J166" s="15" t="n">
         <v>220</v>
       </c>
-      <c r="K166" s="12" t="n">
+      <c r="K166" s="16" t="n">
         <v>10.5</v>
       </c>
     </row>
@@ -8750,11 +8750,11 @@
         </is>
       </c>
       <c r="G168" s="4" t="n">
-        <v>7341</v>
+        <v>9213</v>
       </c>
       <c r="H168" s="3" t="inlineStr">
         <is>
-          <t>7/27</t>
+          <t>8/27</t>
         </is>
       </c>
       <c r="I168" s="3" t="inlineStr">
@@ -8763,10 +8763,10 @@
         </is>
       </c>
       <c r="J168" s="4" t="n">
-        <v>28315</v>
+        <v>31094</v>
       </c>
       <c r="K168" s="5" t="n">
-        <v>1048.714285714286</v>
+        <v>1151.625</v>
       </c>
     </row>
     <row r="169">
@@ -8868,52 +8868,52 @@
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="6" t="inlineStr">
+      <c r="A171" s="2" t="inlineStr">
         <is>
           <t>SULUR</t>
         </is>
       </c>
-      <c r="B171" s="6" t="n">
+      <c r="B171" s="3" t="n">
         <v>116</v>
       </c>
-      <c r="C171" s="6" t="inlineStr">
+      <c r="C171" s="3" t="inlineStr">
         <is>
           <t>NM.SUKUMAR</t>
         </is>
       </c>
-      <c r="D171" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E171" s="6" t="inlineStr">
-        <is>
-          <t>V.P.KANDASAMY</t>
-        </is>
-      </c>
-      <c r="F171" s="6" t="inlineStr">
-        <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G171" s="7" t="n">
-        <v>4540</v>
-      </c>
-      <c r="H171" s="6" t="inlineStr">
-        <is>
-          <t>10/28</t>
-        </is>
-      </c>
-      <c r="I171" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J171" s="7" t="n">
-        <v>12712</v>
-      </c>
-      <c r="K171" s="8" t="n">
-        <v>454</v>
+      <c r="D171" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E171" s="3" t="inlineStr">
+        <is>
+          <t>THALAPATHY MURUGESAN</t>
+        </is>
+      </c>
+      <c r="F171" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G171" s="4" t="n">
+        <v>8726</v>
+      </c>
+      <c r="H171" s="3" t="inlineStr">
+        <is>
+          <t>12/28</t>
+        </is>
+      </c>
+      <c r="I171" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J171" s="4" t="n">
+        <v>20361</v>
+      </c>
+      <c r="K171" s="5" t="n">
+        <v>727.1666666666666</v>
       </c>
     </row>
     <row r="172">
@@ -8946,11 +8946,11 @@
         </is>
       </c>
       <c r="G172" s="4" t="n">
-        <v>16215</v>
+        <v>17063</v>
       </c>
       <c r="H172" s="3" t="inlineStr">
         <is>
-          <t>19/34</t>
+          <t>20/34</t>
         </is>
       </c>
       <c r="I172" s="3" t="inlineStr">
@@ -8959,10 +8959,10 @@
         </is>
       </c>
       <c r="J172" s="4" t="n">
-        <v>29016</v>
+        <v>29007</v>
       </c>
       <c r="K172" s="5" t="n">
-        <v>853.421052631579</v>
+        <v>853.15</v>
       </c>
     </row>
     <row r="173">
@@ -8995,11 +8995,11 @@
         </is>
       </c>
       <c r="G173" s="7" t="n">
-        <v>7799</v>
+        <v>7451</v>
       </c>
       <c r="H173" s="6" t="inlineStr">
         <is>
-          <t>11/26</t>
+          <t>12/26</t>
         </is>
       </c>
       <c r="I173" s="6" t="inlineStr">
@@ -9008,59 +9008,59 @@
         </is>
       </c>
       <c r="J173" s="7" t="n">
-        <v>18434</v>
+        <v>16144</v>
       </c>
       <c r="K173" s="8" t="n">
-        <v>709</v>
+        <v>620.9166666666666</v>
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="13" t="inlineStr">
+      <c r="A174" s="6" t="inlineStr">
         <is>
           <t>THALLI</t>
         </is>
       </c>
-      <c r="B174" s="14" t="n">
+      <c r="B174" s="6" t="n">
         <v>56</v>
       </c>
-      <c r="C174" s="14" t="inlineStr">
+      <c r="C174" s="6" t="inlineStr">
         <is>
           <t>RAMACHANDRAN. T</t>
         </is>
       </c>
-      <c r="D174" s="14" t="inlineStr">
+      <c r="D174" s="6" t="inlineStr">
         <is>
           <t>Communist Party of India</t>
         </is>
       </c>
-      <c r="E174" s="14" t="inlineStr">
+      <c r="E174" s="6" t="inlineStr">
         <is>
           <t>DR.NAGESH KUMAR. C</t>
         </is>
       </c>
-      <c r="F174" s="14" t="inlineStr">
+      <c r="F174" s="6" t="inlineStr">
         <is>
           <t>Bharatiya Janata Party</t>
         </is>
       </c>
-      <c r="G174" s="15" t="n">
-        <v>30</v>
-      </c>
-      <c r="H174" s="14" t="inlineStr">
-        <is>
-          <t>8/24</t>
-        </is>
-      </c>
-      <c r="I174" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J174" s="15" t="n">
-        <v>90</v>
-      </c>
-      <c r="K174" s="16" t="n">
-        <v>3.75</v>
+      <c r="G174" s="7" t="n">
+        <v>608</v>
+      </c>
+      <c r="H174" s="6" t="inlineStr">
+        <is>
+          <t>9/24</t>
+        </is>
+      </c>
+      <c r="I174" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J174" s="7" t="n">
+        <v>1621</v>
+      </c>
+      <c r="K174" s="8" t="n">
+        <v>67.55555555555556</v>
       </c>
     </row>
     <row r="175">
@@ -9142,11 +9142,11 @@
         </is>
       </c>
       <c r="G176" s="4" t="n">
-        <v>14112</v>
+        <v>17033</v>
       </c>
       <c r="H176" s="3" t="inlineStr">
         <is>
-          <t>10/17</t>
+          <t>12/17</t>
         </is>
       </c>
       <c r="I176" s="3" t="inlineStr">
@@ -9155,10 +9155,10 @@
         </is>
       </c>
       <c r="J176" s="4" t="n">
-        <v>23990</v>
+        <v>24130</v>
       </c>
       <c r="K176" s="5" t="n">
-        <v>1411.2</v>
+        <v>1419.416666666667</v>
       </c>
     </row>
     <row r="177">
@@ -9289,11 +9289,11 @@
         </is>
       </c>
       <c r="G179" s="4" t="n">
-        <v>14007</v>
+        <v>15346</v>
       </c>
       <c r="H179" s="3" t="inlineStr">
         <is>
-          <t>11/26</t>
+          <t>12/26</t>
         </is>
       </c>
       <c r="I179" s="3" t="inlineStr">
@@ -9302,10 +9302,10 @@
         </is>
       </c>
       <c r="J179" s="4" t="n">
-        <v>33107</v>
+        <v>33250</v>
       </c>
       <c r="K179" s="5" t="n">
-        <v>1273.363636363636</v>
+        <v>1278.833333333333</v>
       </c>
     </row>
     <row r="180">
@@ -9338,11 +9338,11 @@
         </is>
       </c>
       <c r="G180" s="4" t="n">
-        <v>19539</v>
+        <v>20856</v>
       </c>
       <c r="H180" s="3" t="inlineStr">
         <is>
-          <t>10/29</t>
+          <t>11/29</t>
         </is>
       </c>
       <c r="I180" s="3" t="inlineStr">
@@ -9351,10 +9351,10 @@
         </is>
       </c>
       <c r="J180" s="4" t="n">
-        <v>56663</v>
+        <v>54984</v>
       </c>
       <c r="K180" s="5" t="n">
-        <v>1953.9</v>
+        <v>1896</v>
       </c>
     </row>
     <row r="181">
@@ -9387,11 +9387,11 @@
         </is>
       </c>
       <c r="G181" s="7" t="n">
-        <v>6950</v>
+        <v>7003</v>
       </c>
       <c r="H181" s="6" t="inlineStr">
         <is>
-          <t>12/21</t>
+          <t>13/21</t>
         </is>
       </c>
       <c r="I181" s="6" t="inlineStr">
@@ -9400,10 +9400,10 @@
         </is>
       </c>
       <c r="J181" s="7" t="n">
-        <v>12162</v>
+        <v>11313</v>
       </c>
       <c r="K181" s="8" t="n">
-        <v>579.1666666666666</v>
+        <v>538.6923076923077</v>
       </c>
     </row>
     <row r="182">
@@ -9436,11 +9436,11 @@
         </is>
       </c>
       <c r="G182" s="7" t="n">
-        <v>4885</v>
+        <v>5336</v>
       </c>
       <c r="H182" s="6" t="inlineStr">
         <is>
-          <t>7/25</t>
+          <t>8/25</t>
         </is>
       </c>
       <c r="I182" s="6" t="inlineStr">
@@ -9449,10 +9449,10 @@
         </is>
       </c>
       <c r="J182" s="7" t="n">
-        <v>17446</v>
+        <v>16675</v>
       </c>
       <c r="K182" s="8" t="n">
-        <v>697.8571428571428</v>
+        <v>667</v>
       </c>
     </row>
     <row r="183">
@@ -9485,11 +9485,11 @@
         </is>
       </c>
       <c r="G183" s="7" t="n">
-        <v>7537</v>
+        <v>9141</v>
       </c>
       <c r="H183" s="6" t="inlineStr">
         <is>
-          <t>12/24</t>
+          <t>13/24</t>
         </is>
       </c>
       <c r="I183" s="6" t="inlineStr">
@@ -9498,10 +9498,10 @@
         </is>
       </c>
       <c r="J183" s="7" t="n">
-        <v>15074</v>
+        <v>16876</v>
       </c>
       <c r="K183" s="8" t="n">
-        <v>628.0833333333334</v>
+        <v>703.1538461538462</v>
       </c>
     </row>
     <row r="184">
@@ -9583,11 +9583,11 @@
         </is>
       </c>
       <c r="G185" s="7" t="n">
-        <v>601</v>
+        <v>1077</v>
       </c>
       <c r="H185" s="6" t="inlineStr">
         <is>
-          <t>7/23</t>
+          <t>8/23</t>
         </is>
       </c>
       <c r="I185" s="6" t="inlineStr">
@@ -9596,10 +9596,10 @@
         </is>
       </c>
       <c r="J185" s="7" t="n">
-        <v>1975</v>
+        <v>3096</v>
       </c>
       <c r="K185" s="8" t="n">
-        <v>85.85714285714286</v>
+        <v>134.625</v>
       </c>
     </row>
     <row r="186">
@@ -9632,11 +9632,11 @@
         </is>
       </c>
       <c r="G186" s="7" t="n">
-        <v>7966</v>
+        <v>8162</v>
       </c>
       <c r="H186" s="6" t="inlineStr">
         <is>
-          <t>10/24</t>
+          <t>11/24</t>
         </is>
       </c>
       <c r="I186" s="6" t="inlineStr">
@@ -9645,10 +9645,10 @@
         </is>
       </c>
       <c r="J186" s="7" t="n">
-        <v>19118</v>
+        <v>17808</v>
       </c>
       <c r="K186" s="8" t="n">
-        <v>796.6</v>
+        <v>742</v>
       </c>
     </row>
     <row r="187">
@@ -9730,11 +9730,11 @@
         </is>
       </c>
       <c r="G188" s="7" t="n">
-        <v>9788</v>
+        <v>10721</v>
       </c>
       <c r="H188" s="6" t="inlineStr">
         <is>
-          <t>11/18</t>
+          <t>12/18</t>
         </is>
       </c>
       <c r="I188" s="6" t="inlineStr">
@@ -9743,10 +9743,10 @@
         </is>
       </c>
       <c r="J188" s="7" t="n">
-        <v>16017</v>
+        <v>16082</v>
       </c>
       <c r="K188" s="8" t="n">
-        <v>889.8181818181819</v>
+        <v>893.4166666666666</v>
       </c>
     </row>
     <row r="189">
@@ -10073,11 +10073,11 @@
         </is>
       </c>
       <c r="G195" s="7" t="n">
-        <v>3839</v>
+        <v>5443</v>
       </c>
       <c r="H195" s="6" t="inlineStr">
         <is>
-          <t>7/21</t>
+          <t>8/21</t>
         </is>
       </c>
       <c r="I195" s="6" t="inlineStr">
@@ -10086,10 +10086,10 @@
         </is>
       </c>
       <c r="J195" s="7" t="n">
-        <v>11517</v>
+        <v>14288</v>
       </c>
       <c r="K195" s="8" t="n">
-        <v>548.4285714285714</v>
+        <v>680.375</v>
       </c>
     </row>
     <row r="196">
@@ -10269,11 +10269,11 @@
         </is>
       </c>
       <c r="G199" s="15" t="n">
-        <v>54</v>
+        <v>335</v>
       </c>
       <c r="H199" s="14" t="inlineStr">
         <is>
-          <t>10/24</t>
+          <t>11/24</t>
         </is>
       </c>
       <c r="I199" s="14" t="inlineStr">
@@ -10282,10 +10282,10 @@
         </is>
       </c>
       <c r="J199" s="15" t="n">
-        <v>130</v>
+        <v>731</v>
       </c>
       <c r="K199" s="16" t="n">
-        <v>5.4</v>
+        <v>30.45454545454545</v>
       </c>
     </row>
     <row r="200">
@@ -10318,11 +10318,11 @@
         </is>
       </c>
       <c r="G200" s="7" t="n">
-        <v>4782</v>
+        <v>5718</v>
       </c>
       <c r="H200" s="6" t="inlineStr">
         <is>
-          <t>18/28</t>
+          <t>19/28</t>
         </is>
       </c>
       <c r="I200" s="6" t="inlineStr">
@@ -10331,10 +10331,10 @@
         </is>
       </c>
       <c r="J200" s="7" t="n">
-        <v>7439</v>
+        <v>8427</v>
       </c>
       <c r="K200" s="8" t="n">
-        <v>265.6666666666667</v>
+        <v>300.9473684210527</v>
       </c>
     </row>
     <row r="201">
@@ -10416,11 +10416,11 @@
         </is>
       </c>
       <c r="G202" s="7" t="n">
-        <v>4902</v>
+        <v>4157</v>
       </c>
       <c r="H202" s="6" t="inlineStr">
         <is>
-          <t>10/27</t>
+          <t>11/27</t>
         </is>
       </c>
       <c r="I202" s="6" t="inlineStr">
@@ -10429,10 +10429,10 @@
         </is>
       </c>
       <c r="J202" s="7" t="n">
-        <v>13235</v>
+        <v>10204</v>
       </c>
       <c r="K202" s="8" t="n">
-        <v>490.2</v>
+        <v>377.9090909090909</v>
       </c>
     </row>
     <row r="203">
@@ -10514,11 +10514,11 @@
         </is>
       </c>
       <c r="G204" s="4" t="n">
-        <v>11503</v>
+        <v>12273</v>
       </c>
       <c r="H204" s="3" t="inlineStr">
         <is>
-          <t>9/21</t>
+          <t>10/21</t>
         </is>
       </c>
       <c r="I204" s="3" t="inlineStr">
@@ -10527,10 +10527,10 @@
         </is>
       </c>
       <c r="J204" s="4" t="n">
-        <v>26840</v>
+        <v>25773</v>
       </c>
       <c r="K204" s="5" t="n">
-        <v>1278.111111111111</v>
+        <v>1227.3</v>
       </c>
     </row>
     <row r="205">
@@ -10563,11 +10563,11 @@
         </is>
       </c>
       <c r="G205" s="7" t="n">
-        <v>3881</v>
+        <v>4588</v>
       </c>
       <c r="H205" s="6" t="inlineStr">
         <is>
-          <t>9/25</t>
+          <t>10/25</t>
         </is>
       </c>
       <c r="I205" s="6" t="inlineStr">
@@ -10576,58 +10576,58 @@
         </is>
       </c>
       <c r="J205" s="7" t="n">
-        <v>10781</v>
+        <v>11470</v>
       </c>
       <c r="K205" s="8" t="n">
-        <v>431.2222222222222</v>
+        <v>458.8</v>
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="9" t="inlineStr">
+      <c r="A206" s="13" t="inlineStr">
         <is>
           <t>TIRUVADANAI</t>
         </is>
       </c>
-      <c r="B206" s="10" t="n">
+      <c r="B206" s="14" t="n">
         <v>210</v>
       </c>
-      <c r="C206" s="10" t="inlineStr">
+      <c r="C206" s="14" t="inlineStr">
         <is>
           <t>M.KEERTHIKA</t>
         </is>
       </c>
-      <c r="D206" s="10" t="inlineStr">
+      <c r="D206" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E206" s="10" t="inlineStr">
+      <c r="E206" s="14" t="inlineStr">
         <is>
           <t>RAJEEV</t>
         </is>
       </c>
-      <c r="F206" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G206" s="11" t="n">
+      <c r="F206" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G206" s="15" t="n">
         <v>482</v>
       </c>
-      <c r="H206" s="10" t="inlineStr">
+      <c r="H206" s="14" t="inlineStr">
         <is>
           <t>16/27</t>
         </is>
       </c>
-      <c r="I206" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J206" s="11" t="n">
+      <c r="I206" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J206" s="15" t="n">
         <v>813</v>
       </c>
-      <c r="K206" s="12" t="n">
+      <c r="K206" s="16" t="n">
         <v>30.125</v>
       </c>
     </row>
@@ -10661,11 +10661,11 @@
         </is>
       </c>
       <c r="G207" s="7" t="n">
-        <v>1079</v>
+        <v>1107</v>
       </c>
       <c r="H207" s="6" t="inlineStr">
         <is>
-          <t>8/23</t>
+          <t>9/23</t>
         </is>
       </c>
       <c r="I207" s="6" t="inlineStr">
@@ -10674,10 +10674,10 @@
         </is>
       </c>
       <c r="J207" s="7" t="n">
-        <v>3102</v>
+        <v>2829</v>
       </c>
       <c r="K207" s="8" t="n">
-        <v>134.875</v>
+        <v>123</v>
       </c>
     </row>
     <row r="208">
@@ -10730,51 +10730,51 @@
       </c>
     </row>
     <row r="209">
-      <c r="A209" s="9" t="inlineStr">
+      <c r="A209" s="13" t="inlineStr">
         <is>
           <t>UDHAGAMANDALAM</t>
         </is>
       </c>
-      <c r="B209" s="10" t="n">
+      <c r="B209" s="14" t="n">
         <v>108</v>
       </c>
-      <c r="C209" s="10" t="inlineStr">
+      <c r="C209" s="14" t="inlineStr">
         <is>
           <t>BHOJARAJAN.M</t>
         </is>
       </c>
-      <c r="D209" s="10" t="inlineStr">
+      <c r="D209" s="14" t="inlineStr">
         <is>
           <t>Bharatiya Janata Party</t>
         </is>
       </c>
-      <c r="E209" s="10" t="inlineStr">
+      <c r="E209" s="14" t="inlineStr">
         <is>
           <t>IBRAHIM.R</t>
         </is>
       </c>
-      <c r="F209" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G209" s="11" t="n">
+      <c r="F209" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G209" s="15" t="n">
         <v>189</v>
       </c>
-      <c r="H209" s="10" t="inlineStr">
+      <c r="H209" s="14" t="inlineStr">
         <is>
           <t>17/19</t>
         </is>
       </c>
-      <c r="I209" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J209" s="11" t="n">
+      <c r="I209" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J209" s="15" t="n">
         <v>211</v>
       </c>
-      <c r="K209" s="12" t="n">
+      <c r="K209" s="16" t="n">
         <v>11.11764705882353</v>
       </c>
     </row>
@@ -10857,11 +10857,11 @@
         </is>
       </c>
       <c r="G211" s="11" t="n">
-        <v>85</v>
+        <v>38</v>
       </c>
       <c r="H211" s="10" t="inlineStr">
         <is>
-          <t>8/27</t>
+          <t>9/27</t>
         </is>
       </c>
       <c r="I211" s="10" t="inlineStr">
@@ -10870,10 +10870,10 @@
         </is>
       </c>
       <c r="J211" s="11" t="n">
-        <v>287</v>
+        <v>114</v>
       </c>
       <c r="K211" s="12" t="n">
-        <v>10.625</v>
+        <v>4.222222222222222</v>
       </c>
     </row>
     <row r="212">
@@ -10955,11 +10955,11 @@
         </is>
       </c>
       <c r="G213" s="7" t="n">
-        <v>4632</v>
+        <v>3268</v>
       </c>
       <c r="H213" s="6" t="inlineStr">
         <is>
-          <t>14/23</t>
+          <t>15/23</t>
         </is>
       </c>
       <c r="I213" s="6" t="inlineStr">
@@ -10968,10 +10968,10 @@
         </is>
       </c>
       <c r="J213" s="7" t="n">
-        <v>7610</v>
+        <v>5011</v>
       </c>
       <c r="K213" s="8" t="n">
-        <v>330.8571428571428</v>
+        <v>217.8666666666667</v>
       </c>
     </row>
     <row r="214">
@@ -11004,11 +11004,11 @@
         </is>
       </c>
       <c r="G214" s="4" t="n">
-        <v>12899</v>
+        <v>13518</v>
       </c>
       <c r="H214" s="3" t="inlineStr">
         <is>
-          <t>13/23</t>
+          <t>14/23</t>
         </is>
       </c>
       <c r="I214" s="3" t="inlineStr">
@@ -11017,10 +11017,10 @@
         </is>
       </c>
       <c r="J214" s="4" t="n">
-        <v>22821</v>
+        <v>22208</v>
       </c>
       <c r="K214" s="5" t="n">
-        <v>992.2307692307694</v>
+        <v>965.5714285714286</v>
       </c>
     </row>
     <row r="215">
@@ -11053,11 +11053,11 @@
         </is>
       </c>
       <c r="G215" s="4" t="n">
-        <v>5788</v>
+        <v>7910</v>
       </c>
       <c r="H215" s="3" t="inlineStr">
         <is>
-          <t>16/18</t>
+          <t>17/18</t>
         </is>
       </c>
       <c r="I215" s="3" t="inlineStr">
@@ -11066,10 +11066,10 @@
         </is>
       </c>
       <c r="J215" s="4" t="n">
-        <v>6512</v>
+        <v>8375</v>
       </c>
       <c r="K215" s="5" t="n">
-        <v>361.75</v>
+        <v>465.2941176470588</v>
       </c>
     </row>
     <row r="216">
@@ -11102,11 +11102,11 @@
         </is>
       </c>
       <c r="G216" s="7" t="n">
-        <v>3750</v>
+        <v>3759</v>
       </c>
       <c r="H216" s="6" t="inlineStr">
         <is>
-          <t>10/21</t>
+          <t>11/21</t>
         </is>
       </c>
       <c r="I216" s="6" t="inlineStr">
@@ -11115,59 +11115,59 @@
         </is>
       </c>
       <c r="J216" s="7" t="n">
-        <v>7875</v>
+        <v>7176</v>
       </c>
       <c r="K216" s="8" t="n">
-        <v>375</v>
+        <v>341.7272727272727</v>
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="6" t="inlineStr">
+      <c r="A217" s="2" t="inlineStr">
         <is>
           <t>VANIYAMBADI</t>
         </is>
       </c>
-      <c r="B217" s="6" t="n">
+      <c r="B217" s="3" t="n">
         <v>47</v>
       </c>
-      <c r="C217" s="6" t="inlineStr">
+      <c r="C217" s="3" t="inlineStr">
         <is>
           <t>SYED FAROOQ BASHA SSB</t>
         </is>
       </c>
-      <c r="D217" s="6" t="inlineStr">
+      <c r="D217" s="3" t="inlineStr">
         <is>
           <t>Indian Union Muslim League</t>
         </is>
       </c>
-      <c r="E217" s="6" t="inlineStr">
+      <c r="E217" s="3" t="inlineStr">
         <is>
           <t>SYED BHURHANUDEEN</t>
         </is>
       </c>
-      <c r="F217" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G217" s="7" t="n">
-        <v>9614</v>
-      </c>
-      <c r="H217" s="6" t="inlineStr">
-        <is>
-          <t>17/23</t>
-        </is>
-      </c>
-      <c r="I217" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J217" s="7" t="n">
-        <v>13007</v>
-      </c>
-      <c r="K217" s="8" t="n">
-        <v>565.5294117647059</v>
+      <c r="F217" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G217" s="4" t="n">
+        <v>9343</v>
+      </c>
+      <c r="H217" s="3" t="inlineStr">
+        <is>
+          <t>18/23</t>
+        </is>
+      </c>
+      <c r="I217" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J217" s="4" t="n">
+        <v>11938</v>
+      </c>
+      <c r="K217" s="5" t="n">
+        <v>519.0555555555555</v>
       </c>
     </row>
     <row r="218">
@@ -11347,11 +11347,11 @@
         </is>
       </c>
       <c r="G221" s="7" t="n">
-        <v>5824</v>
+        <v>6272</v>
       </c>
       <c r="H221" s="6" t="inlineStr">
         <is>
-          <t>10/24</t>
+          <t>11/24</t>
         </is>
       </c>
       <c r="I221" s="6" t="inlineStr">
@@ -11360,10 +11360,10 @@
         </is>
       </c>
       <c r="J221" s="7" t="n">
-        <v>13978</v>
+        <v>13684</v>
       </c>
       <c r="K221" s="8" t="n">
-        <v>582.4</v>
+        <v>570.1818181818181</v>
       </c>
     </row>
     <row r="222">
@@ -11396,11 +11396,11 @@
         </is>
       </c>
       <c r="G222" s="7" t="n">
-        <v>2716</v>
+        <v>3120</v>
       </c>
       <c r="H222" s="6" t="inlineStr">
         <is>
-          <t>11/23</t>
+          <t>12/23</t>
         </is>
       </c>
       <c r="I222" s="6" t="inlineStr">
@@ -11409,10 +11409,10 @@
         </is>
       </c>
       <c r="J222" s="7" t="n">
-        <v>5679</v>
+        <v>5980</v>
       </c>
       <c r="K222" s="8" t="n">
-        <v>246.9090909090909</v>
+        <v>260</v>
       </c>
     </row>
     <row r="223">
@@ -11445,11 +11445,11 @@
         </is>
       </c>
       <c r="G223" s="4" t="n">
-        <v>19004</v>
+        <v>21068</v>
       </c>
       <c r="H223" s="3" t="inlineStr">
         <is>
-          <t>11/23</t>
+          <t>12/23</t>
         </is>
       </c>
       <c r="I223" s="3" t="inlineStr">
@@ -11458,10 +11458,10 @@
         </is>
       </c>
       <c r="J223" s="4" t="n">
-        <v>39736</v>
+        <v>40380</v>
       </c>
       <c r="K223" s="5" t="n">
-        <v>1727.636363636364</v>
+        <v>1755.666666666667</v>
       </c>
     </row>
     <row r="224">
@@ -11563,51 +11563,51 @@
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="9" t="inlineStr">
+      <c r="A226" s="13" t="inlineStr">
         <is>
           <t>VIKRAVANDI</t>
         </is>
       </c>
-      <c r="B226" s="10" t="n">
+      <c r="B226" s="14" t="n">
         <v>75</v>
       </c>
-      <c r="C226" s="10" t="inlineStr">
+      <c r="C226" s="14" t="inlineStr">
         <is>
           <t>SIVAKUMAR C</t>
         </is>
       </c>
-      <c r="D226" s="10" t="inlineStr">
+      <c r="D226" s="14" t="inlineStr">
         <is>
           <t>Pattali Makkal Katchi</t>
         </is>
       </c>
-      <c r="E226" s="10" t="inlineStr">
+      <c r="E226" s="14" t="inlineStr">
         <is>
           <t>VIJAI VADIVEL A</t>
         </is>
       </c>
-      <c r="F226" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G226" s="11" t="n">
+      <c r="F226" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G226" s="15" t="n">
         <v>102</v>
       </c>
-      <c r="H226" s="10" t="inlineStr">
+      <c r="H226" s="14" t="inlineStr">
         <is>
           <t>6/23</t>
         </is>
       </c>
-      <c r="I226" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J226" s="11" t="n">
+      <c r="I226" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J226" s="15" t="n">
         <v>391</v>
       </c>
-      <c r="K226" s="12" t="n">
+      <c r="K226" s="16" t="n">
         <v>17</v>
       </c>
     </row>
@@ -11690,11 +11690,11 @@
         </is>
       </c>
       <c r="G228" s="4" t="n">
-        <v>12456</v>
+        <v>13237</v>
       </c>
       <c r="H228" s="3" t="inlineStr">
         <is>
-          <t>10/22</t>
+          <t>11/22</t>
         </is>
       </c>
       <c r="I228" s="3" t="inlineStr">
@@ -11703,10 +11703,10 @@
         </is>
       </c>
       <c r="J228" s="4" t="n">
-        <v>27403</v>
+        <v>26474</v>
       </c>
       <c r="K228" s="5" t="n">
-        <v>1245.6</v>
+        <v>1203.363636363636</v>
       </c>
     </row>
     <row r="229">
@@ -11739,11 +11739,11 @@
         </is>
       </c>
       <c r="G229" s="7" t="n">
-        <v>9247</v>
+        <v>10330</v>
       </c>
       <c r="H229" s="6" t="inlineStr">
         <is>
-          <t>10/19</t>
+          <t>11/19</t>
         </is>
       </c>
       <c r="I229" s="6" t="inlineStr">
@@ -11752,10 +11752,10 @@
         </is>
       </c>
       <c r="J229" s="7" t="n">
-        <v>17569</v>
+        <v>17843</v>
       </c>
       <c r="K229" s="8" t="n">
-        <v>924.7</v>
+        <v>939.0909090909091</v>
       </c>
     </row>
     <row r="230">
@@ -11788,11 +11788,11 @@
         </is>
       </c>
       <c r="G230" s="7" t="n">
-        <v>1272</v>
+        <v>1478</v>
       </c>
       <c r="H230" s="6" t="inlineStr">
         <is>
-          <t>12/24</t>
+          <t>13/24</t>
         </is>
       </c>
       <c r="I230" s="6" t="inlineStr">
@@ -11801,10 +11801,10 @@
         </is>
       </c>
       <c r="J230" s="7" t="n">
-        <v>2544</v>
+        <v>2729</v>
       </c>
       <c r="K230" s="8" t="n">
-        <v>106</v>
+        <v>113.6923076923077</v>
       </c>
     </row>
     <row r="231">
@@ -11886,11 +11886,11 @@
         </is>
       </c>
       <c r="G232" s="7" t="n">
-        <v>2455</v>
+        <v>1970</v>
       </c>
       <c r="H232" s="6" t="inlineStr">
         <is>
-          <t>9/21</t>
+          <t>10/21</t>
         </is>
       </c>
       <c r="I232" s="6" t="inlineStr">
@@ -11899,10 +11899,10 @@
         </is>
       </c>
       <c r="J232" s="7" t="n">
-        <v>5728</v>
+        <v>4137</v>
       </c>
       <c r="K232" s="8" t="n">
-        <v>272.7777777777778</v>
+        <v>197</v>
       </c>
     </row>
     <row r="233">
@@ -11935,11 +11935,11 @@
         </is>
       </c>
       <c r="G233" s="4" t="n">
-        <v>8002</v>
+        <v>9056</v>
       </c>
       <c r="H233" s="3" t="inlineStr">
         <is>
-          <t>8/23</t>
+          <t>9/23</t>
         </is>
       </c>
       <c r="I233" s="3" t="inlineStr">
@@ -11948,10 +11948,10 @@
         </is>
       </c>
       <c r="J233" s="4" t="n">
-        <v>23006</v>
+        <v>23143</v>
       </c>
       <c r="K233" s="5" t="n">
-        <v>1000.25</v>
+        <v>1006.222222222222</v>
       </c>
     </row>
     <row r="234">
@@ -12033,11 +12033,11 @@
         </is>
       </c>
       <c r="G235" s="7" t="n">
-        <v>2680</v>
+        <v>2668</v>
       </c>
       <c r="H235" s="6" t="inlineStr">
         <is>
-          <t>8/24</t>
+          <t>9/24</t>
         </is>
       </c>
       <c r="I235" s="6" t="inlineStr">
@@ -12046,10 +12046,10 @@
         </is>
       </c>
       <c r="J235" s="7" t="n">
-        <v>8040</v>
+        <v>7115</v>
       </c>
       <c r="K235" s="8" t="n">
-        <v>335</v>
+        <v>296.4444444444445</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix classification to catch small projected-margin seats like Sholavandan
Old logic only used contest_index, missing seats with large CI but tiny
projected margins. New dual criteria: knife-edge if CI <= 10 OR projected
margin < 500; competitive if CI <= 40 OR projected margin < 3000.

https://claude.ai/code/session_01MizbUy44JG5sXyvaf3Wekb
</commit_message>
<xml_diff>
--- a/tn_election_results_may2026.xlsx
+++ b/tn_election_results_may2026.xlsx
@@ -930,52 +930,52 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>ANDIPATTI</t>
         </is>
       </c>
-      <c r="B9" s="6" t="n">
+      <c r="B9" s="14" t="n">
         <v>198</v>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>MAHARAJAN.A</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>LOGIRAJAN.A</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="F9" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>MAHARAJAN.A</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G9" s="7" t="n">
-        <v>614</v>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>13/25</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J9" s="7" t="n">
-        <v>1181</v>
-      </c>
-      <c r="K9" s="8" t="n">
-        <v>47.23076923076923</v>
+      <c r="G9" s="15" t="n">
+        <v>502</v>
+      </c>
+      <c r="H9" s="14" t="inlineStr">
+        <is>
+          <t>14/25</t>
+        </is>
+      </c>
+      <c r="I9" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J9" s="15" t="n">
+        <v>896</v>
+      </c>
+      <c r="K9" s="16" t="n">
+        <v>35.85714285714285</v>
       </c>
     </row>
     <row r="10">
@@ -1028,52 +1028,52 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>ANTHIYUR</t>
         </is>
       </c>
-      <c r="B11" s="6" t="n">
+      <c r="B11" s="14" t="n">
         <v>105</v>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C11" s="14" t="inlineStr">
         <is>
           <t>HARIBASKAR.P</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="D11" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E11" s="14" t="inlineStr">
         <is>
           <t>SIVABALAN.M</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G11" s="7" t="n">
-        <v>1995</v>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>17/20</t>
-        </is>
-      </c>
-      <c r="I11" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J11" s="7" t="n">
-        <v>2347</v>
-      </c>
-      <c r="K11" s="8" t="n">
-        <v>117.3529411764706</v>
+      <c r="F11" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G11" s="15" t="n">
+        <v>1310</v>
+      </c>
+      <c r="H11" s="14" t="inlineStr">
+        <is>
+          <t>18/20</t>
+        </is>
+      </c>
+      <c r="I11" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J11" s="15" t="n">
+        <v>1456</v>
+      </c>
+      <c r="K11" s="16" t="n">
+        <v>72.77777777777777</v>
       </c>
     </row>
     <row r="12">
@@ -1126,101 +1126,101 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>ARANI</t>
         </is>
       </c>
-      <c r="B13" s="6" t="n">
+      <c r="B13" s="14" t="n">
         <v>67</v>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="14" t="inlineStr">
         <is>
           <t>JAYASUDHA. L</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="D13" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E13" s="14" t="inlineStr">
         <is>
           <t>VENKATESH KUMAR. D</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G13" s="7" t="n">
-        <v>2467</v>
-      </c>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>17/24</t>
-        </is>
-      </c>
-      <c r="I13" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J13" s="7" t="n">
-        <v>3483</v>
-      </c>
-      <c r="K13" s="8" t="n">
-        <v>145.1176470588235</v>
+      <c r="F13" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G13" s="15" t="n">
+        <v>2135</v>
+      </c>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>18/24</t>
+        </is>
+      </c>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J13" s="15" t="n">
+        <v>2847</v>
+      </c>
+      <c r="K13" s="16" t="n">
+        <v>118.6111111111111</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>ARANTHANGI</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n">
+      <c r="B14" s="6" t="n">
         <v>183</v>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>MOHAMED FARVAS. J</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>RAMACHANDRAN . T</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>Indian National Congress</t>
         </is>
       </c>
-      <c r="G14" s="4" t="n">
-        <v>11149</v>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>12/22</t>
-        </is>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J14" s="4" t="n">
-        <v>20440</v>
-      </c>
-      <c r="K14" s="5" t="n">
-        <v>929.0833333333334</v>
+      <c r="G14" s="7" t="n">
+        <v>10804</v>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>13/22</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>18284</v>
+      </c>
+      <c r="K14" s="8" t="n">
+        <v>831.0769230769231</v>
       </c>
     </row>
     <row r="15">
@@ -1351,11 +1351,11 @@
         </is>
       </c>
       <c r="G17" s="7" t="n">
-        <v>12109</v>
+        <v>12123</v>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>16/24</t>
+          <t>17/24</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
@@ -1364,10 +1364,10 @@
         </is>
       </c>
       <c r="J17" s="7" t="n">
-        <v>18164</v>
+        <v>17115</v>
       </c>
       <c r="K17" s="8" t="n">
-        <v>756.8125</v>
+        <v>713.1176470588235</v>
       </c>
     </row>
     <row r="18">
@@ -1596,11 +1596,11 @@
         </is>
       </c>
       <c r="G22" s="7" t="n">
-        <v>2476</v>
+        <v>4357</v>
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>15/27</t>
+          <t>16/27</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr">
@@ -1609,10 +1609,10 @@
         </is>
       </c>
       <c r="J22" s="7" t="n">
-        <v>4457</v>
+        <v>7352</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>165.0666666666667</v>
+        <v>272.3125</v>
       </c>
     </row>
     <row r="23">
@@ -1714,52 +1714,52 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
+      <c r="A25" s="13" t="inlineStr">
         <is>
           <t>BHAVANISAGAR</t>
         </is>
       </c>
-      <c r="B25" s="6" t="n">
+      <c r="B25" s="14" t="n">
         <v>107</v>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C25" s="14" t="inlineStr">
         <is>
           <t>A.BANNARI</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
+      <c r="D25" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E25" s="6" t="inlineStr">
+      <c r="E25" s="14" t="inlineStr">
         <is>
           <t>V.P.TAMILSELVI</t>
         </is>
       </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G25" s="7" t="n">
-        <v>1898</v>
-      </c>
-      <c r="H25" s="6" t="inlineStr">
-        <is>
-          <t>14/24</t>
-        </is>
-      </c>
-      <c r="I25" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J25" s="7" t="n">
-        <v>3254</v>
-      </c>
-      <c r="K25" s="8" t="n">
-        <v>135.5714285714286</v>
+      <c r="F25" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G25" s="15" t="n">
+        <v>967</v>
+      </c>
+      <c r="H25" s="14" t="inlineStr">
+        <is>
+          <t>15/24</t>
+        </is>
+      </c>
+      <c r="I25" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J25" s="15" t="n">
+        <v>1547</v>
+      </c>
+      <c r="K25" s="16" t="n">
+        <v>64.46666666666667</v>
       </c>
     </row>
     <row r="26">
@@ -1812,51 +1812,51 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="inlineStr">
+      <c r="A27" s="13" t="inlineStr">
         <is>
           <t>BODINAYAKANUR</t>
         </is>
       </c>
-      <c r="B27" s="6" t="n">
+      <c r="B27" s="14" t="n">
         <v>200</v>
       </c>
-      <c r="C27" s="6" t="inlineStr">
+      <c r="C27" s="14" t="inlineStr">
         <is>
           <t>PANNEERSELVAM.O</t>
         </is>
       </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="inlineStr">
+      <c r="D27" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E27" s="14" t="inlineStr">
         <is>
           <t>PRAKASH.S</t>
         </is>
       </c>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G27" s="7" t="n">
+      <c r="F27" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G27" s="15" t="n">
         <v>919</v>
       </c>
-      <c r="H27" s="6" t="inlineStr">
+      <c r="H27" s="14" t="inlineStr">
         <is>
           <t>11/25</t>
         </is>
       </c>
-      <c r="I27" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J27" s="7" t="n">
+      <c r="I27" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J27" s="15" t="n">
         <v>2089</v>
       </c>
-      <c r="K27" s="8" t="n">
+      <c r="K27" s="16" t="n">
         <v>83.54545454545455</v>
       </c>
     </row>
@@ -1959,51 +1959,51 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="inlineStr">
+      <c r="A30" s="13" t="inlineStr">
         <is>
           <t>CHEPAUK-THIRUVALLIKENI</t>
         </is>
       </c>
-      <c r="B30" s="6" t="n">
+      <c r="B30" s="14" t="n">
         <v>19</v>
       </c>
-      <c r="C30" s="6" t="inlineStr">
+      <c r="C30" s="14" t="inlineStr">
         <is>
           <t>UDHAYANIDHI STALIN</t>
         </is>
       </c>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="inlineStr">
+      <c r="D30" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E30" s="14" t="inlineStr">
         <is>
           <t>SELVAM. D</t>
         </is>
       </c>
-      <c r="F30" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G30" s="7" t="n">
+      <c r="F30" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G30" s="15" t="n">
         <v>1365</v>
       </c>
-      <c r="H30" s="6" t="inlineStr">
+      <c r="H30" s="14" t="inlineStr">
         <is>
           <t>10/17</t>
         </is>
       </c>
-      <c r="I30" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J30" s="7" t="n">
+      <c r="I30" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J30" s="15" t="n">
         <v>2320</v>
       </c>
-      <c r="K30" s="8" t="n">
+      <c r="K30" s="16" t="n">
         <v>136.5</v>
       </c>
     </row>
@@ -2037,7 +2037,7 @@
         </is>
       </c>
       <c r="G31" s="4" t="n">
-        <v>19279</v>
+        <v>19638</v>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
@@ -2050,10 +2050,10 @@
         </is>
       </c>
       <c r="J31" s="4" t="n">
-        <v>21032</v>
+        <v>21423</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>876.3181818181819</v>
+        <v>892.6363636363636</v>
       </c>
     </row>
     <row r="32">
@@ -2086,11 +2086,11 @@
         </is>
       </c>
       <c r="G32" s="7" t="n">
-        <v>2248</v>
+        <v>2562</v>
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>16/21</t>
+          <t>17/21</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
@@ -2099,10 +2099,10 @@
         </is>
       </c>
       <c r="J32" s="7" t="n">
-        <v>2950</v>
+        <v>3165</v>
       </c>
       <c r="K32" s="8" t="n">
-        <v>140.5</v>
+        <v>150.7058823529412</v>
       </c>
     </row>
     <row r="33">
@@ -2135,11 +2135,11 @@
         </is>
       </c>
       <c r="G33" s="7" t="n">
-        <v>2669</v>
+        <v>3727</v>
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>11/22</t>
+          <t>12/22</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
@@ -2148,108 +2148,108 @@
         </is>
       </c>
       <c r="J33" s="7" t="n">
-        <v>5338</v>
+        <v>6833</v>
       </c>
       <c r="K33" s="8" t="n">
-        <v>242.6363636363636</v>
+        <v>310.5833333333333</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="6" t="inlineStr">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>COIMBATORE (NORTH)</t>
         </is>
       </c>
-      <c r="B34" s="6" t="n">
+      <c r="B34" s="3" t="n">
         <v>118</v>
       </c>
-      <c r="C34" s="6" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>V. SAMPATHKUMAR</t>
         </is>
       </c>
-      <c r="D34" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E34" s="6" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
         <is>
           <t>DURAI. SENTHAMIL SELVAN B.E</t>
         </is>
       </c>
-      <c r="F34" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G34" s="7" t="n">
-        <v>6367</v>
-      </c>
-      <c r="H34" s="6" t="inlineStr">
-        <is>
-          <t>8/25</t>
-        </is>
-      </c>
-      <c r="I34" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J34" s="7" t="n">
-        <v>19897</v>
-      </c>
-      <c r="K34" s="8" t="n">
-        <v>795.875</v>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="n">
+        <v>7846</v>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>9/25</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J34" s="4" t="n">
+        <v>21794</v>
+      </c>
+      <c r="K34" s="5" t="n">
+        <v>871.7777777777778</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="6" t="inlineStr">
+      <c r="A35" s="13" t="inlineStr">
         <is>
           <t>COIMBATORE (SOUTH)</t>
         </is>
       </c>
-      <c r="B35" s="6" t="n">
+      <c r="B35" s="14" t="n">
         <v>120</v>
       </c>
-      <c r="C35" s="6" t="inlineStr">
+      <c r="C35" s="14" t="inlineStr">
         <is>
           <t>V SENTHILBALAJI</t>
         </is>
       </c>
-      <c r="D35" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E35" s="6" t="inlineStr">
+      <c r="D35" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E35" s="14" t="inlineStr">
         <is>
           <t>V. SENTHILKUMAR</t>
         </is>
       </c>
-      <c r="F35" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G35" s="7" t="n">
-        <v>1124</v>
-      </c>
-      <c r="H35" s="6" t="inlineStr">
-        <is>
-          <t>9/20</t>
-        </is>
-      </c>
-      <c r="I35" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J35" s="7" t="n">
-        <v>2498</v>
-      </c>
-      <c r="K35" s="8" t="n">
-        <v>124.8888888888889</v>
+      <c r="F35" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G35" s="15" t="n">
+        <v>855</v>
+      </c>
+      <c r="H35" s="14" t="inlineStr">
+        <is>
+          <t>10/20</t>
+        </is>
+      </c>
+      <c r="I35" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J35" s="15" t="n">
+        <v>1710</v>
+      </c>
+      <c r="K35" s="16" t="n">
+        <v>85.5</v>
       </c>
     </row>
     <row r="36">
@@ -2282,11 +2282,11 @@
         </is>
       </c>
       <c r="G36" s="7" t="n">
-        <v>5513</v>
+        <v>6877</v>
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>9/23</t>
+          <t>10/23</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
@@ -2295,10 +2295,10 @@
         </is>
       </c>
       <c r="J36" s="7" t="n">
-        <v>14089</v>
+        <v>15817</v>
       </c>
       <c r="K36" s="8" t="n">
-        <v>612.5555555555555</v>
+        <v>687.7</v>
       </c>
     </row>
     <row r="37">
@@ -2322,20 +2322,20 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>C. THANGARAJU</t>
+          <t>A. RAMU</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>Tamilaga Vettri Kazhagam</t>
+          <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
       <c r="G37" s="4" t="n">
-        <v>7044</v>
+        <v>7322</v>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>16/18</t>
+          <t>17/18</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
@@ -2344,10 +2344,10 @@
         </is>
       </c>
       <c r="J37" s="4" t="n">
-        <v>7924</v>
+        <v>7753</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>440.25</v>
+        <v>430.7058823529412</v>
       </c>
     </row>
     <row r="38">
@@ -2449,52 +2449,52 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="inlineStr">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>DHARAPURAM</t>
         </is>
       </c>
-      <c r="B40" s="6" t="n">
+      <c r="B40" s="3" t="n">
         <v>101</v>
       </c>
-      <c r="C40" s="6" t="inlineStr">
+      <c r="C40" s="3" t="inlineStr">
         <is>
           <t>SATHYABAMA.P</t>
         </is>
       </c>
-      <c r="D40" s="6" t="inlineStr">
+      <c r="D40" s="3" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E40" s="6" t="inlineStr">
+      <c r="E40" s="3" t="inlineStr">
         <is>
           <t>INDIRANI.T</t>
         </is>
       </c>
-      <c r="F40" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G40" s="7" t="n">
-        <v>9806</v>
-      </c>
-      <c r="H40" s="6" t="inlineStr">
-        <is>
-          <t>17/23</t>
-        </is>
-      </c>
-      <c r="I40" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J40" s="7" t="n">
-        <v>13267</v>
-      </c>
-      <c r="K40" s="8" t="n">
-        <v>576.8235294117648</v>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="n">
+        <v>11447</v>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>18/23</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="n">
+        <v>14627</v>
+      </c>
+      <c r="K40" s="5" t="n">
+        <v>635.9444444444445</v>
       </c>
     </row>
     <row r="41">
@@ -2527,11 +2527,11 @@
         </is>
       </c>
       <c r="G41" s="7" t="n">
-        <v>9108</v>
+        <v>10961</v>
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>16/23</t>
+          <t>17/23</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr">
@@ -2540,10 +2540,10 @@
         </is>
       </c>
       <c r="J41" s="7" t="n">
-        <v>13093</v>
+        <v>14830</v>
       </c>
       <c r="K41" s="8" t="n">
-        <v>569.25</v>
+        <v>644.7647058823529</v>
       </c>
     </row>
     <row r="42">
@@ -2576,11 +2576,11 @@
         </is>
       </c>
       <c r="G42" s="7" t="n">
-        <v>1005</v>
+        <v>2199</v>
       </c>
       <c r="H42" s="6" t="inlineStr">
         <is>
-          <t>15/24</t>
+          <t>16/24</t>
         </is>
       </c>
       <c r="I42" s="6" t="inlineStr">
@@ -2589,10 +2589,10 @@
         </is>
       </c>
       <c r="J42" s="7" t="n">
-        <v>1608</v>
+        <v>3298</v>
       </c>
       <c r="K42" s="8" t="n">
-        <v>67</v>
+        <v>137.4375</v>
       </c>
     </row>
     <row r="43">
@@ -2625,11 +2625,11 @@
         </is>
       </c>
       <c r="G43" s="4" t="n">
-        <v>13161</v>
+        <v>16461</v>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>6/18</t>
+          <t>7/18</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
@@ -2638,10 +2638,10 @@
         </is>
       </c>
       <c r="J43" s="4" t="n">
-        <v>39483</v>
+        <v>42328</v>
       </c>
       <c r="K43" s="5" t="n">
-        <v>2193.5</v>
+        <v>2351.571428571428</v>
       </c>
     </row>
     <row r="44">
@@ -2674,11 +2674,11 @@
         </is>
       </c>
       <c r="G44" s="4" t="n">
-        <v>61643</v>
+        <v>65656</v>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>16/25</t>
+          <t>17/25</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
@@ -2687,10 +2687,10 @@
         </is>
       </c>
       <c r="J44" s="4" t="n">
-        <v>96317</v>
+        <v>96553</v>
       </c>
       <c r="K44" s="5" t="n">
-        <v>3852.6875</v>
+        <v>3862.117647058823</v>
       </c>
     </row>
     <row r="45">
@@ -2821,11 +2821,11 @@
         </is>
       </c>
       <c r="G47" s="4" t="n">
-        <v>14624</v>
+        <v>15343</v>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>11/24</t>
+          <t>12/24</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
@@ -2834,10 +2834,10 @@
         </is>
       </c>
       <c r="J47" s="4" t="n">
-        <v>31907</v>
+        <v>30686</v>
       </c>
       <c r="K47" s="5" t="n">
-        <v>1329.454545454545</v>
+        <v>1278.583333333333</v>
       </c>
     </row>
     <row r="48">
@@ -3106,20 +3106,20 @@
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>PARITHA PURUSHOTHAMAN.G</t>
+          <t>K.B.PRADAP</t>
         </is>
       </c>
       <c r="F53" s="6" t="inlineStr">
         <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
+          <t>Desiya Murpokku Dravida Kazhagam</t>
         </is>
       </c>
       <c r="G53" s="7" t="n">
-        <v>6154</v>
+        <v>2419</v>
       </c>
       <c r="H53" s="6" t="inlineStr">
         <is>
-          <t>11/23</t>
+          <t>12/23</t>
         </is>
       </c>
       <c r="I53" s="6" t="inlineStr">
@@ -3128,10 +3128,10 @@
         </is>
       </c>
       <c r="J53" s="7" t="n">
-        <v>12867</v>
+        <v>4636</v>
       </c>
       <c r="K53" s="8" t="n">
-        <v>559.4545454545455</v>
+        <v>201.5833333333333</v>
       </c>
     </row>
     <row r="54">
@@ -3360,11 +3360,11 @@
         </is>
       </c>
       <c r="G58" s="7" t="n">
-        <v>10348</v>
+        <v>9882</v>
       </c>
       <c r="H58" s="6" t="inlineStr">
         <is>
-          <t>13/23</t>
+          <t>14/23</t>
         </is>
       </c>
       <c r="I58" s="6" t="inlineStr">
@@ -3373,10 +3373,10 @@
         </is>
       </c>
       <c r="J58" s="7" t="n">
-        <v>18308</v>
+        <v>16235</v>
       </c>
       <c r="K58" s="8" t="n">
-        <v>796.0000000000001</v>
+        <v>705.8571428571429</v>
       </c>
     </row>
     <row r="59">
@@ -3409,11 +3409,11 @@
         </is>
       </c>
       <c r="G59" s="7" t="n">
-        <v>9190</v>
+        <v>9110</v>
       </c>
       <c r="H59" s="6" t="inlineStr">
         <is>
-          <t>12/21</t>
+          <t>13/21</t>
         </is>
       </c>
       <c r="I59" s="6" t="inlineStr">
@@ -3422,59 +3422,59 @@
         </is>
       </c>
       <c r="J59" s="7" t="n">
-        <v>16082</v>
+        <v>14716</v>
       </c>
       <c r="K59" s="8" t="n">
-        <v>765.8333333333334</v>
+        <v>700.7692307692307</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="6" t="inlineStr">
+      <c r="A60" s="13" t="inlineStr">
         <is>
           <t>KADAYANALLUR</t>
         </is>
       </c>
-      <c r="B60" s="6" t="n">
+      <c r="B60" s="14" t="n">
         <v>221</v>
       </c>
-      <c r="C60" s="6" t="inlineStr">
+      <c r="C60" s="14" t="inlineStr">
         <is>
           <t>RAJENDRAN. T. M</t>
         </is>
       </c>
-      <c r="D60" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E60" s="6" t="inlineStr">
+      <c r="D60" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E60" s="14" t="inlineStr">
         <is>
           <t>C. KRISHNAMURALI</t>
         </is>
       </c>
-      <c r="F60" s="6" t="inlineStr">
+      <c r="F60" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G60" s="7" t="n">
-        <v>2959</v>
-      </c>
-      <c r="H60" s="6" t="inlineStr">
-        <is>
-          <t>11/26</t>
-        </is>
-      </c>
-      <c r="I60" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J60" s="7" t="n">
-        <v>6994</v>
-      </c>
-      <c r="K60" s="8" t="n">
-        <v>269</v>
+      <c r="G60" s="15" t="n">
+        <v>1038</v>
+      </c>
+      <c r="H60" s="14" t="inlineStr">
+        <is>
+          <t>12/26</t>
+        </is>
+      </c>
+      <c r="I60" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J60" s="15" t="n">
+        <v>2249</v>
+      </c>
+      <c r="K60" s="16" t="n">
+        <v>86.5</v>
       </c>
     </row>
     <row r="61">
@@ -3507,11 +3507,11 @@
         </is>
       </c>
       <c r="G61" s="4" t="n">
-        <v>14412</v>
+        <v>14457</v>
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>11/22</t>
+          <t>12/22</t>
         </is>
       </c>
       <c r="I61" s="3" t="inlineStr">
@@ -3520,10 +3520,10 @@
         </is>
       </c>
       <c r="J61" s="4" t="n">
-        <v>28824</v>
+        <v>26504</v>
       </c>
       <c r="K61" s="5" t="n">
-        <v>1310.181818181818</v>
+        <v>1204.75</v>
       </c>
     </row>
     <row r="62">
@@ -3556,11 +3556,11 @@
         </is>
       </c>
       <c r="G62" s="7" t="n">
-        <v>2139</v>
+        <v>2873</v>
       </c>
       <c r="H62" s="6" t="inlineStr">
         <is>
-          <t>9/27</t>
+          <t>10/27</t>
         </is>
       </c>
       <c r="I62" s="6" t="inlineStr">
@@ -3569,10 +3569,10 @@
         </is>
       </c>
       <c r="J62" s="7" t="n">
-        <v>6417</v>
+        <v>7757</v>
       </c>
       <c r="K62" s="8" t="n">
-        <v>237.6666666666667</v>
+        <v>287.3</v>
       </c>
     </row>
     <row r="63">
@@ -4115,51 +4115,51 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="6" t="inlineStr">
+      <c r="A74" s="13" t="inlineStr">
         <is>
           <t>KILVELUR</t>
         </is>
       </c>
-      <c r="B74" s="6" t="n">
+      <c r="B74" s="14" t="n">
         <v>164</v>
       </c>
-      <c r="C74" s="6" t="inlineStr">
+      <c r="C74" s="14" t="inlineStr">
         <is>
           <t>SENTHIL PANDIAN. P</t>
         </is>
       </c>
-      <c r="D74" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E74" s="6" t="inlineStr">
+      <c r="D74" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E74" s="14" t="inlineStr">
         <is>
           <t>LATHA. T</t>
         </is>
       </c>
-      <c r="F74" s="6" t="inlineStr">
+      <c r="F74" s="14" t="inlineStr">
         <is>
           <t>Communist Party of India (Marxist)</t>
         </is>
       </c>
-      <c r="G74" s="7" t="n">
+      <c r="G74" s="15" t="n">
         <v>1667</v>
       </c>
-      <c r="H74" s="6" t="inlineStr">
+      <c r="H74" s="14" t="inlineStr">
         <is>
           <t>9/16</t>
         </is>
       </c>
-      <c r="I74" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J74" s="7" t="n">
+      <c r="I74" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J74" s="15" t="n">
         <v>2964</v>
       </c>
-      <c r="K74" s="8" t="n">
+      <c r="K74" s="16" t="n">
         <v>185.2222222222222</v>
       </c>
     </row>
@@ -4193,11 +4193,11 @@
         </is>
       </c>
       <c r="G75" s="4" t="n">
-        <v>11514</v>
+        <v>11498</v>
       </c>
       <c r="H75" s="3" t="inlineStr">
         <is>
-          <t>21/28</t>
+          <t>22/28</t>
         </is>
       </c>
       <c r="I75" s="3" t="inlineStr">
@@ -4206,10 +4206,10 @@
         </is>
       </c>
       <c r="J75" s="4" t="n">
-        <v>15352</v>
+        <v>14634</v>
       </c>
       <c r="K75" s="5" t="n">
-        <v>548.2857142857143</v>
+        <v>522.6363636363636</v>
       </c>
     </row>
     <row r="76">
@@ -4340,11 +4340,11 @@
         </is>
       </c>
       <c r="G78" s="4" t="n">
-        <v>18198</v>
+        <v>18131</v>
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
-          <t>18/25</t>
+          <t>19/25</t>
         </is>
       </c>
       <c r="I78" s="3" t="inlineStr">
@@ -4353,10 +4353,10 @@
         </is>
       </c>
       <c r="J78" s="4" t="n">
-        <v>25275</v>
+        <v>23857</v>
       </c>
       <c r="K78" s="5" t="n">
-        <v>1011</v>
+        <v>954.2631578947369</v>
       </c>
     </row>
     <row r="79">
@@ -4409,51 +4409,51 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="6" t="inlineStr">
+      <c r="A80" s="13" t="inlineStr">
         <is>
           <t>KULITHALAI</t>
         </is>
       </c>
-      <c r="B80" s="6" t="n">
+      <c r="B80" s="14" t="n">
         <v>137</v>
       </c>
-      <c r="C80" s="6" t="inlineStr">
+      <c r="C80" s="14" t="inlineStr">
         <is>
           <t>G.BALASUBRAMANI</t>
         </is>
       </c>
-      <c r="D80" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E80" s="6" t="inlineStr">
+      <c r="D80" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E80" s="14" t="inlineStr">
         <is>
           <t>SURIYANUR. A. CHANDRAN</t>
         </is>
       </c>
-      <c r="F80" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G80" s="7" t="n">
+      <c r="F80" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G80" s="15" t="n">
         <v>1446</v>
       </c>
-      <c r="H80" s="6" t="inlineStr">
+      <c r="H80" s="14" t="inlineStr">
         <is>
           <t>12/21</t>
         </is>
       </c>
-      <c r="I80" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J80" s="7" t="n">
+      <c r="I80" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J80" s="15" t="n">
         <v>2530</v>
       </c>
-      <c r="K80" s="8" t="n">
+      <c r="K80" s="16" t="n">
         <v>120.5</v>
       </c>
     </row>
@@ -4634,11 +4634,11 @@
         </is>
       </c>
       <c r="G84" s="7" t="n">
-        <v>776</v>
+        <v>2195</v>
       </c>
       <c r="H84" s="6" t="inlineStr">
         <is>
-          <t>13/20</t>
+          <t>14/20</t>
         </is>
       </c>
       <c r="I84" s="6" t="inlineStr">
@@ -4647,58 +4647,58 @@
         </is>
       </c>
       <c r="J84" s="7" t="n">
-        <v>1194</v>
+        <v>3136</v>
       </c>
       <c r="K84" s="8" t="n">
-        <v>59.69230769230769</v>
+        <v>156.7857142857143</v>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="6" t="inlineStr">
+      <c r="A85" s="13" t="inlineStr">
         <is>
           <t>LALGUDI</t>
         </is>
       </c>
-      <c r="B85" s="6" t="n">
+      <c r="B85" s="14" t="n">
         <v>143</v>
       </c>
-      <c r="C85" s="6" t="inlineStr">
+      <c r="C85" s="14" t="inlineStr">
         <is>
           <t>LEEMAROSE MARTIN</t>
         </is>
       </c>
-      <c r="D85" s="6" t="inlineStr">
+      <c r="D85" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E85" s="6" t="inlineStr">
+      <c r="E85" s="14" t="inlineStr">
         <is>
           <t>KU PA KRISHNAN</t>
         </is>
       </c>
-      <c r="F85" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G85" s="7" t="n">
+      <c r="F85" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G85" s="15" t="n">
         <v>1663</v>
       </c>
-      <c r="H85" s="6" t="inlineStr">
+      <c r="H85" s="14" t="inlineStr">
         <is>
           <t>12/20</t>
         </is>
       </c>
-      <c r="I85" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J85" s="7" t="n">
+      <c r="I85" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J85" s="15" t="n">
         <v>2772</v>
       </c>
-      <c r="K85" s="8" t="n">
+      <c r="K85" s="16" t="n">
         <v>138.5833333333333</v>
       </c>
     </row>
@@ -4732,11 +4732,11 @@
         </is>
       </c>
       <c r="G86" s="7" t="n">
-        <v>1725</v>
+        <v>2845</v>
       </c>
       <c r="H86" s="6" t="inlineStr">
         <is>
-          <t>9/21</t>
+          <t>10/21</t>
         </is>
       </c>
       <c r="I86" s="6" t="inlineStr">
@@ -4745,10 +4745,10 @@
         </is>
       </c>
       <c r="J86" s="7" t="n">
-        <v>4025</v>
+        <v>5974</v>
       </c>
       <c r="K86" s="8" t="n">
-        <v>191.6666666666667</v>
+        <v>284.5</v>
       </c>
     </row>
     <row r="87">
@@ -4781,11 +4781,11 @@
         </is>
       </c>
       <c r="G87" s="4" t="n">
-        <v>67983</v>
+        <v>74243</v>
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
-          <t>14/19</t>
+          <t>15/19</t>
         </is>
       </c>
       <c r="I87" s="3" t="inlineStr">
@@ -4794,10 +4794,10 @@
         </is>
       </c>
       <c r="J87" s="4" t="n">
-        <v>92263</v>
+        <v>94041</v>
       </c>
       <c r="K87" s="5" t="n">
-        <v>4855.928571428572</v>
+        <v>4949.533333333334</v>
       </c>
     </row>
     <row r="88">
@@ -4928,11 +4928,11 @@
         </is>
       </c>
       <c r="G90" s="4" t="n">
-        <v>14435</v>
+        <v>15151</v>
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>11/19</t>
+          <t>12/19</t>
         </is>
       </c>
       <c r="I90" s="3" t="inlineStr">
@@ -4941,10 +4941,10 @@
         </is>
       </c>
       <c r="J90" s="4" t="n">
-        <v>24933</v>
+        <v>23989</v>
       </c>
       <c r="K90" s="5" t="n">
-        <v>1312.272727272727</v>
+        <v>1262.583333333333</v>
       </c>
     </row>
     <row r="91">
@@ -4977,11 +4977,11 @@
         </is>
       </c>
       <c r="G91" s="4" t="n">
-        <v>16384</v>
+        <v>18354</v>
       </c>
       <c r="H91" s="3" t="inlineStr">
         <is>
-          <t>14/17</t>
+          <t>15/17</t>
         </is>
       </c>
       <c r="I91" s="3" t="inlineStr">
@@ -4990,10 +4990,10 @@
         </is>
       </c>
       <c r="J91" s="4" t="n">
-        <v>19895</v>
+        <v>20801</v>
       </c>
       <c r="K91" s="5" t="n">
-        <v>1170.285714285714</v>
+        <v>1223.6</v>
       </c>
     </row>
     <row r="92">
@@ -5173,11 +5173,11 @@
         </is>
       </c>
       <c r="G95" s="4" t="n">
-        <v>23108</v>
+        <v>25203</v>
       </c>
       <c r="H95" s="3" t="inlineStr">
         <is>
-          <t>14/20</t>
+          <t>15/20</t>
         </is>
       </c>
       <c r="I95" s="3" t="inlineStr">
@@ -5186,10 +5186,10 @@
         </is>
       </c>
       <c r="J95" s="4" t="n">
-        <v>33011</v>
+        <v>33604</v>
       </c>
       <c r="K95" s="5" t="n">
-        <v>1650.571428571429</v>
+        <v>1680.2</v>
       </c>
     </row>
     <row r="96">
@@ -5291,51 +5291,51 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="6" t="inlineStr">
+      <c r="A98" s="13" t="inlineStr">
         <is>
           <t>MANAPPARAI</t>
         </is>
       </c>
-      <c r="B98" s="6" t="n">
+      <c r="B98" s="14" t="n">
         <v>138</v>
       </c>
-      <c r="C98" s="6" t="inlineStr">
+      <c r="C98" s="14" t="inlineStr">
         <is>
           <t>R. KATHIRAVAN</t>
         </is>
       </c>
-      <c r="D98" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E98" s="6" t="inlineStr">
+      <c r="D98" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E98" s="14" t="inlineStr">
         <is>
           <t>DR. PL. VIJAYAKUMAR</t>
         </is>
       </c>
-      <c r="F98" s="6" t="inlineStr">
+      <c r="F98" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G98" s="7" t="n">
+      <c r="G98" s="15" t="n">
         <v>1625</v>
       </c>
-      <c r="H98" s="6" t="inlineStr">
+      <c r="H98" s="14" t="inlineStr">
         <is>
           <t>17/25</t>
         </is>
       </c>
-      <c r="I98" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J98" s="7" t="n">
+      <c r="I98" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J98" s="15" t="n">
         <v>2390</v>
       </c>
-      <c r="K98" s="8" t="n">
+      <c r="K98" s="16" t="n">
         <v>95.58823529411765</v>
       </c>
     </row>
@@ -5438,150 +5438,150 @@
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="6" t="inlineStr">
+      <c r="A101" s="13" t="inlineStr">
         <is>
           <t>MELUR</t>
         </is>
       </c>
-      <c r="B101" s="6" t="n">
+      <c r="B101" s="14" t="n">
         <v>188</v>
       </c>
-      <c r="C101" s="6" t="inlineStr">
+      <c r="C101" s="14" t="inlineStr">
         <is>
           <t>P.VISWANATHAN</t>
         </is>
       </c>
-      <c r="D101" s="6" t="inlineStr">
+      <c r="D101" s="14" t="inlineStr">
         <is>
           <t>Indian National Congress</t>
         </is>
       </c>
-      <c r="E101" s="6" t="inlineStr">
+      <c r="E101" s="14" t="inlineStr">
         <is>
           <t>A.MADURAIVEERAN</t>
         </is>
       </c>
-      <c r="F101" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G101" s="7" t="n">
+      <c r="F101" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G101" s="15" t="n">
         <v>2724</v>
       </c>
-      <c r="H101" s="6" t="inlineStr">
+      <c r="H101" s="14" t="inlineStr">
         <is>
           <t>21/21</t>
         </is>
       </c>
-      <c r="I101" s="6" t="inlineStr">
+      <c r="I101" s="14" t="inlineStr">
         <is>
           <t>Result Declared</t>
         </is>
       </c>
-      <c r="J101" s="7" t="n">
+      <c r="J101" s="15" t="n">
         <v>2724</v>
       </c>
-      <c r="K101" s="8" t="n">
+      <c r="K101" s="16" t="n">
         <v>129.7142857142857</v>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="6" t="inlineStr">
+      <c r="A102" s="13" t="inlineStr">
         <is>
           <t>METTUPPALAYAM</t>
         </is>
       </c>
-      <c r="B102" s="6" t="n">
+      <c r="B102" s="14" t="n">
         <v>111</v>
       </c>
-      <c r="C102" s="6" t="inlineStr">
+      <c r="C102" s="14" t="inlineStr">
         <is>
           <t>SMT.KAVITHA KALYANASUNDARAM</t>
         </is>
       </c>
-      <c r="D102" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E102" s="6" t="inlineStr">
+      <c r="D102" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E102" s="14" t="inlineStr">
         <is>
           <t>SUNILANAND</t>
         </is>
       </c>
-      <c r="F102" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G102" s="7" t="n">
-        <v>1436</v>
-      </c>
-      <c r="H102" s="6" t="inlineStr">
-        <is>
-          <t>12/26</t>
-        </is>
-      </c>
-      <c r="I102" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J102" s="7" t="n">
-        <v>3111</v>
-      </c>
-      <c r="K102" s="8" t="n">
-        <v>119.6666666666667</v>
+      <c r="F102" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G102" s="15" t="n">
+        <v>691</v>
+      </c>
+      <c r="H102" s="14" t="inlineStr">
+        <is>
+          <t>13/26</t>
+        </is>
+      </c>
+      <c r="I102" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J102" s="15" t="n">
+        <v>1382</v>
+      </c>
+      <c r="K102" s="16" t="n">
+        <v>53.15384615384615</v>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="6" t="inlineStr">
+      <c r="A103" s="13" t="inlineStr">
         <is>
           <t>METTUR</t>
         </is>
       </c>
-      <c r="B103" s="6" t="n">
+      <c r="B103" s="14" t="n">
         <v>85</v>
       </c>
-      <c r="C103" s="6" t="inlineStr">
+      <c r="C103" s="14" t="inlineStr">
         <is>
           <t>MIDHUN CHAKRAVARTHY. M</t>
         </is>
       </c>
-      <c r="D103" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E103" s="6" t="inlineStr">
+      <c r="D103" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E103" s="14" t="inlineStr">
         <is>
           <t>VENKATACHALAM. G</t>
         </is>
       </c>
-      <c r="F103" s="6" t="inlineStr">
+      <c r="F103" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G103" s="7" t="n">
-        <v>1391</v>
-      </c>
-      <c r="H103" s="6" t="inlineStr">
-        <is>
-          <t>10/24</t>
-        </is>
-      </c>
-      <c r="I103" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J103" s="7" t="n">
-        <v>3338</v>
-      </c>
-      <c r="K103" s="8" t="n">
-        <v>139.1</v>
+      <c r="G103" s="15" t="n">
+        <v>869</v>
+      </c>
+      <c r="H103" s="14" t="inlineStr">
+        <is>
+          <t>11/24</t>
+        </is>
+      </c>
+      <c r="I103" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J103" s="15" t="n">
+        <v>1896</v>
+      </c>
+      <c r="K103" s="16" t="n">
+        <v>79</v>
       </c>
     </row>
     <row r="104">
@@ -5614,11 +5614,11 @@
         </is>
       </c>
       <c r="G104" s="7" t="n">
-        <v>3695</v>
+        <v>3383</v>
       </c>
       <c r="H104" s="6" t="inlineStr">
         <is>
-          <t>14/21</t>
+          <t>15/21</t>
         </is>
       </c>
       <c r="I104" s="6" t="inlineStr">
@@ -5627,10 +5627,10 @@
         </is>
       </c>
       <c r="J104" s="7" t="n">
-        <v>5542</v>
+        <v>4736</v>
       </c>
       <c r="K104" s="8" t="n">
-        <v>263.9285714285714</v>
+        <v>225.5333333333333</v>
       </c>
     </row>
     <row r="105">
@@ -5663,11 +5663,11 @@
         </is>
       </c>
       <c r="G105" s="7" t="n">
-        <v>8171</v>
+        <v>8843</v>
       </c>
       <c r="H105" s="6" t="inlineStr">
         <is>
-          <t>16/30</t>
+          <t>17/30</t>
         </is>
       </c>
       <c r="I105" s="6" t="inlineStr">
@@ -5676,10 +5676,10 @@
         </is>
       </c>
       <c r="J105" s="7" t="n">
-        <v>15321</v>
+        <v>15605</v>
       </c>
       <c r="K105" s="8" t="n">
-        <v>510.6875</v>
+        <v>520.1764705882352</v>
       </c>
     </row>
     <row r="106">
@@ -5761,11 +5761,11 @@
         </is>
       </c>
       <c r="G107" s="4" t="n">
-        <v>20914</v>
+        <v>22514</v>
       </c>
       <c r="H107" s="3" t="inlineStr">
         <is>
-          <t>14/20</t>
+          <t>15/20</t>
         </is>
       </c>
       <c r="I107" s="3" t="inlineStr">
@@ -5774,10 +5774,10 @@
         </is>
       </c>
       <c r="J107" s="4" t="n">
-        <v>29877</v>
+        <v>30019</v>
       </c>
       <c r="K107" s="5" t="n">
-        <v>1493.857142857143</v>
+        <v>1500.933333333333</v>
       </c>
     </row>
     <row r="108">
@@ -5879,52 +5879,52 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="9" t="inlineStr">
+      <c r="A110" s="13" t="inlineStr">
         <is>
           <t>NAMAKKAL</t>
         </is>
       </c>
-      <c r="B110" s="10" t="n">
+      <c r="B110" s="14" t="n">
         <v>94</v>
       </c>
-      <c r="C110" s="10" t="inlineStr">
+      <c r="C110" s="14" t="inlineStr">
+        <is>
+          <t>SRIDEVI MOHAN P S</t>
+        </is>
+      </c>
+      <c r="D110" s="14" t="inlineStr">
+        <is>
+          <t>All India Anna Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E110" s="14" t="inlineStr">
         <is>
           <t>DILIP C S</t>
         </is>
       </c>
-      <c r="D110" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E110" s="10" t="inlineStr">
-        <is>
-          <t>SRIDEVI MOHAN P S</t>
-        </is>
-      </c>
-      <c r="F110" s="10" t="inlineStr">
-        <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G110" s="11" t="n">
-        <v>49</v>
-      </c>
-      <c r="H110" s="10" t="inlineStr">
-        <is>
-          <t>8/23</t>
-        </is>
-      </c>
-      <c r="I110" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J110" s="11" t="n">
-        <v>141</v>
-      </c>
-      <c r="K110" s="12" t="n">
-        <v>6.125</v>
+      <c r="F110" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G110" s="15" t="n">
+        <v>502</v>
+      </c>
+      <c r="H110" s="14" t="inlineStr">
+        <is>
+          <t>9/23</t>
+        </is>
+      </c>
+      <c r="I110" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J110" s="15" t="n">
+        <v>1283</v>
+      </c>
+      <c r="K110" s="16" t="n">
+        <v>55.77777777777778</v>
       </c>
     </row>
     <row r="111">
@@ -6300,11 +6300,11 @@
         </is>
       </c>
       <c r="G118" s="4" t="n">
-        <v>25411</v>
+        <v>27558</v>
       </c>
       <c r="H118" s="3" t="inlineStr">
         <is>
-          <t>17/23</t>
+          <t>18/23</t>
         </is>
       </c>
       <c r="I118" s="3" t="inlineStr">
@@ -6313,10 +6313,10 @@
         </is>
       </c>
       <c r="J118" s="4" t="n">
-        <v>34380</v>
+        <v>35213</v>
       </c>
       <c r="K118" s="5" t="n">
-        <v>1494.764705882353</v>
+        <v>1531</v>
       </c>
     </row>
     <row r="119">
@@ -6447,11 +6447,11 @@
         </is>
       </c>
       <c r="G121" s="4" t="n">
-        <v>24005</v>
+        <v>24982</v>
       </c>
       <c r="H121" s="3" t="inlineStr">
         <is>
-          <t>15/23</t>
+          <t>16/23</t>
         </is>
       </c>
       <c r="I121" s="3" t="inlineStr">
@@ -6460,10 +6460,10 @@
         </is>
       </c>
       <c r="J121" s="4" t="n">
-        <v>36808</v>
+        <v>35912</v>
       </c>
       <c r="K121" s="5" t="n">
-        <v>1600.333333333333</v>
+        <v>1561.375</v>
       </c>
     </row>
     <row r="122">
@@ -6487,20 +6487,20 @@
       </c>
       <c r="E122" s="6" t="inlineStr">
         <is>
-          <t>DR. PRAVEEN KUMAR. M</t>
+          <t>PANDI. N</t>
         </is>
       </c>
       <c r="F122" s="6" t="inlineStr">
         <is>
-          <t>Tamilaga Vettri Kazhagam</t>
+          <t>Communist Party of India (Marxist)</t>
         </is>
       </c>
       <c r="G122" s="7" t="n">
-        <v>2004</v>
+        <v>2390</v>
       </c>
       <c r="H122" s="6" t="inlineStr">
         <is>
-          <t>14/25</t>
+          <t>15/25</t>
         </is>
       </c>
       <c r="I122" s="6" t="inlineStr">
@@ -6509,58 +6509,58 @@
         </is>
       </c>
       <c r="J122" s="7" t="n">
-        <v>3579</v>
+        <v>3983</v>
       </c>
       <c r="K122" s="8" t="n">
-        <v>143.1428571428571</v>
+        <v>159.3333333333333</v>
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="6" t="inlineStr">
+      <c r="A123" s="13" t="inlineStr">
         <is>
           <t>PALAYAMKOTTAI</t>
         </is>
       </c>
-      <c r="B123" s="6" t="n">
+      <c r="B123" s="14" t="n">
         <v>226</v>
       </c>
-      <c r="C123" s="6" t="inlineStr">
+      <c r="C123" s="14" t="inlineStr">
         <is>
           <t>MARIA JOHN</t>
         </is>
       </c>
-      <c r="D123" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E123" s="6" t="inlineStr">
+      <c r="D123" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E123" s="14" t="inlineStr">
         <is>
           <t>M.ABDUL WAHAB</t>
         </is>
       </c>
-      <c r="F123" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G123" s="7" t="n">
+      <c r="F123" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G123" s="15" t="n">
         <v>792</v>
       </c>
-      <c r="H123" s="6" t="inlineStr">
+      <c r="H123" s="14" t="inlineStr">
         <is>
           <t>18/22</t>
         </is>
       </c>
-      <c r="I123" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J123" s="7" t="n">
+      <c r="I123" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J123" s="15" t="n">
         <v>968</v>
       </c>
-      <c r="K123" s="8" t="n">
+      <c r="K123" s="16" t="n">
         <v>44</v>
       </c>
     </row>
@@ -6594,11 +6594,11 @@
         </is>
       </c>
       <c r="G124" s="4" t="n">
-        <v>16763</v>
+        <v>19049</v>
       </c>
       <c r="H124" s="3" t="inlineStr">
         <is>
-          <t>17/35</t>
+          <t>18/35</t>
         </is>
       </c>
       <c r="I124" s="3" t="inlineStr">
@@ -6607,10 +6607,10 @@
         </is>
       </c>
       <c r="J124" s="4" t="n">
-        <v>34512</v>
+        <v>37040</v>
       </c>
       <c r="K124" s="5" t="n">
-        <v>986.0588235294117</v>
+        <v>1058.277777777778</v>
       </c>
     </row>
     <row r="125">
@@ -6643,11 +6643,11 @@
         </is>
       </c>
       <c r="G125" s="4" t="n">
-        <v>21154</v>
+        <v>22492</v>
       </c>
       <c r="H125" s="3" t="inlineStr">
         <is>
-          <t>13/34</t>
+          <t>14/34</t>
         </is>
       </c>
       <c r="I125" s="3" t="inlineStr">
@@ -6656,10 +6656,10 @@
         </is>
       </c>
       <c r="J125" s="4" t="n">
-        <v>55326</v>
+        <v>54623</v>
       </c>
       <c r="K125" s="5" t="n">
-        <v>1627.230769230769</v>
+        <v>1606.571428571429</v>
       </c>
     </row>
     <row r="126">
@@ -6692,11 +6692,11 @@
         </is>
       </c>
       <c r="G126" s="4" t="n">
-        <v>7813</v>
+        <v>8447</v>
       </c>
       <c r="H126" s="3" t="inlineStr">
         <is>
-          <t>18/23</t>
+          <t>19/23</t>
         </is>
       </c>
       <c r="I126" s="3" t="inlineStr">
@@ -6705,10 +6705,10 @@
         </is>
       </c>
       <c r="J126" s="4" t="n">
-        <v>9983</v>
+        <v>10225</v>
       </c>
       <c r="K126" s="5" t="n">
-        <v>434.0555555555555</v>
+        <v>444.578947368421</v>
       </c>
     </row>
     <row r="127">
@@ -6810,100 +6810,100 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="6" t="inlineStr">
+      <c r="A129" s="13" t="inlineStr">
         <is>
           <t>PARAMAKUDI</t>
         </is>
       </c>
-      <c r="B129" s="6" t="n">
+      <c r="B129" s="14" t="n">
         <v>209</v>
       </c>
-      <c r="C129" s="6" t="inlineStr">
+      <c r="C129" s="14" t="inlineStr">
         <is>
           <t>GOPIRAJAN. G</t>
         </is>
       </c>
-      <c r="D129" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E129" s="6" t="inlineStr">
+      <c r="D129" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E129" s="14" t="inlineStr">
         <is>
           <t>ADVOCATE. KATHIRAVAN. K.K</t>
         </is>
       </c>
-      <c r="F129" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G129" s="7" t="n">
-        <v>2046</v>
-      </c>
-      <c r="H129" s="6" t="inlineStr">
-        <is>
-          <t>15/24</t>
-        </is>
-      </c>
-      <c r="I129" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J129" s="7" t="n">
-        <v>3274</v>
-      </c>
-      <c r="K129" s="8" t="n">
-        <v>136.4</v>
+      <c r="F129" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G129" s="15" t="n">
+        <v>1155</v>
+      </c>
+      <c r="H129" s="14" t="inlineStr">
+        <is>
+          <t>16/24</t>
+        </is>
+      </c>
+      <c r="I129" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J129" s="15" t="n">
+        <v>1732</v>
+      </c>
+      <c r="K129" s="16" t="n">
+        <v>72.1875</v>
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="6" t="inlineStr">
+      <c r="A130" s="13" t="inlineStr">
         <is>
           <t>PARAMATHI-VELUR</t>
         </is>
       </c>
-      <c r="B130" s="6" t="n">
+      <c r="B130" s="14" t="n">
         <v>95</v>
       </c>
-      <c r="C130" s="6" t="inlineStr">
+      <c r="C130" s="14" t="inlineStr">
         <is>
           <t>MOORTHIY K S</t>
         </is>
       </c>
-      <c r="D130" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E130" s="6" t="inlineStr">
+      <c r="D130" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E130" s="14" t="inlineStr">
         <is>
           <t>SEKAR S</t>
         </is>
       </c>
-      <c r="F130" s="6" t="inlineStr">
+      <c r="F130" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G130" s="7" t="n">
+      <c r="G130" s="15" t="n">
         <v>1146</v>
       </c>
-      <c r="H130" s="6" t="inlineStr">
+      <c r="H130" s="14" t="inlineStr">
         <is>
           <t>9/20</t>
         </is>
       </c>
-      <c r="I130" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J130" s="7" t="n">
+      <c r="I130" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J130" s="15" t="n">
         <v>2547</v>
       </c>
-      <c r="K130" s="8" t="n">
+      <c r="K130" s="16" t="n">
         <v>127.3333333333333</v>
       </c>
     </row>
@@ -6937,11 +6937,11 @@
         </is>
       </c>
       <c r="G131" s="7" t="n">
-        <v>3061</v>
+        <v>3919</v>
       </c>
       <c r="H131" s="6" t="inlineStr">
         <is>
-          <t>9/23</t>
+          <t>10/23</t>
         </is>
       </c>
       <c r="I131" s="6" t="inlineStr">
@@ -6950,10 +6950,10 @@
         </is>
       </c>
       <c r="J131" s="7" t="n">
-        <v>7823</v>
+        <v>9014</v>
       </c>
       <c r="K131" s="8" t="n">
-        <v>340.1111111111111</v>
+        <v>391.9</v>
       </c>
     </row>
     <row r="132">
@@ -6986,11 +6986,11 @@
         </is>
       </c>
       <c r="G132" s="7" t="n">
-        <v>5430</v>
+        <v>5801</v>
       </c>
       <c r="H132" s="6" t="inlineStr">
         <is>
-          <t>9/23</t>
+          <t>10/23</t>
         </is>
       </c>
       <c r="I132" s="6" t="inlineStr">
@@ -6999,10 +6999,10 @@
         </is>
       </c>
       <c r="J132" s="7" t="n">
-        <v>13877</v>
+        <v>13342</v>
       </c>
       <c r="K132" s="8" t="n">
-        <v>603.3333333333334</v>
+        <v>580.1</v>
       </c>
     </row>
     <row r="133">
@@ -7035,11 +7035,11 @@
         </is>
       </c>
       <c r="G133" s="7" t="n">
-        <v>6902</v>
+        <v>6931</v>
       </c>
       <c r="H133" s="6" t="inlineStr">
         <is>
-          <t>16/28</t>
+          <t>17/28</t>
         </is>
       </c>
       <c r="I133" s="6" t="inlineStr">
@@ -7048,10 +7048,10 @@
         </is>
       </c>
       <c r="J133" s="7" t="n">
-        <v>12078</v>
+        <v>11416</v>
       </c>
       <c r="K133" s="8" t="n">
-        <v>431.375</v>
+        <v>407.7058823529412</v>
       </c>
     </row>
     <row r="134">
@@ -7084,11 +7084,11 @@
         </is>
       </c>
       <c r="G134" s="4" t="n">
-        <v>21275</v>
+        <v>23207</v>
       </c>
       <c r="H134" s="3" t="inlineStr">
         <is>
-          <t>9/22</t>
+          <t>10/22</t>
         </is>
       </c>
       <c r="I134" s="3" t="inlineStr">
@@ -7097,10 +7097,10 @@
         </is>
       </c>
       <c r="J134" s="4" t="n">
-        <v>52006</v>
+        <v>51055</v>
       </c>
       <c r="K134" s="5" t="n">
-        <v>2363.888888888889</v>
+        <v>2320.7</v>
       </c>
     </row>
     <row r="135">
@@ -7182,11 +7182,11 @@
         </is>
       </c>
       <c r="G136" s="7" t="n">
-        <v>1008</v>
+        <v>1961</v>
       </c>
       <c r="H136" s="6" t="inlineStr">
         <is>
-          <t>11/26</t>
+          <t>12/26</t>
         </is>
       </c>
       <c r="I136" s="6" t="inlineStr">
@@ -7195,10 +7195,10 @@
         </is>
       </c>
       <c r="J136" s="7" t="n">
-        <v>2383</v>
+        <v>4249</v>
       </c>
       <c r="K136" s="8" t="n">
-        <v>91.63636363636364</v>
+        <v>163.4166666666667</v>
       </c>
     </row>
     <row r="137">
@@ -7231,11 +7231,11 @@
         </is>
       </c>
       <c r="G137" s="7" t="n">
-        <v>5288</v>
+        <v>5498</v>
       </c>
       <c r="H137" s="6" t="inlineStr">
         <is>
-          <t>12/21</t>
+          <t>13/21</t>
         </is>
       </c>
       <c r="I137" s="6" t="inlineStr">
@@ -7244,58 +7244,58 @@
         </is>
       </c>
       <c r="J137" s="7" t="n">
-        <v>9254</v>
+        <v>8881</v>
       </c>
       <c r="K137" s="8" t="n">
-        <v>440.6666666666667</v>
+        <v>422.9230769230769</v>
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="13" t="inlineStr">
+      <c r="A138" s="9" t="inlineStr">
         <is>
           <t>POLLACHI</t>
         </is>
       </c>
-      <c r="B138" s="14" t="n">
+      <c r="B138" s="10" t="n">
         <v>123</v>
       </c>
-      <c r="C138" s="14" t="inlineStr">
+      <c r="C138" s="10" t="inlineStr">
         <is>
           <t>K. NITHYANANDHAN</t>
         </is>
       </c>
-      <c r="D138" s="14" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E138" s="14" t="inlineStr">
+      <c r="D138" s="10" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E138" s="10" t="inlineStr">
         <is>
           <t>POLLACHI V. JAYARAMAN</t>
         </is>
       </c>
-      <c r="F138" s="14" t="inlineStr">
+      <c r="F138" s="10" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G138" s="15" t="n">
+      <c r="G138" s="11" t="n">
         <v>232</v>
       </c>
-      <c r="H138" s="14" t="inlineStr">
+      <c r="H138" s="10" t="inlineStr">
         <is>
           <t>15/20</t>
         </is>
       </c>
-      <c r="I138" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J138" s="15" t="n">
+      <c r="I138" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J138" s="11" t="n">
         <v>309</v>
       </c>
-      <c r="K138" s="16" t="n">
+      <c r="K138" s="12" t="n">
         <v>15.46666666666667</v>
       </c>
     </row>
@@ -7427,11 +7427,11 @@
         </is>
       </c>
       <c r="G141" s="7" t="n">
-        <v>985</v>
+        <v>2208</v>
       </c>
       <c r="H141" s="6" t="inlineStr">
         <is>
-          <t>11/25</t>
+          <t>12/25</t>
         </is>
       </c>
       <c r="I141" s="6" t="inlineStr">
@@ -7440,10 +7440,10 @@
         </is>
       </c>
       <c r="J141" s="7" t="n">
-        <v>2239</v>
+        <v>4600</v>
       </c>
       <c r="K141" s="8" t="n">
-        <v>89.54545454545455</v>
+        <v>184</v>
       </c>
     </row>
     <row r="142">
@@ -7476,11 +7476,11 @@
         </is>
       </c>
       <c r="G142" s="4" t="n">
-        <v>45877</v>
+        <v>49527</v>
       </c>
       <c r="H142" s="3" t="inlineStr">
         <is>
-          <t>13/23</t>
+          <t>14/23</t>
         </is>
       </c>
       <c r="I142" s="3" t="inlineStr">
@@ -7489,10 +7489,10 @@
         </is>
       </c>
       <c r="J142" s="4" t="n">
-        <v>81167</v>
+        <v>81366</v>
       </c>
       <c r="K142" s="5" t="n">
-        <v>3529</v>
+        <v>3537.642857142857</v>
       </c>
     </row>
     <row r="143">
@@ -7574,11 +7574,11 @@
         </is>
       </c>
       <c r="G144" s="4" t="n">
-        <v>7836</v>
+        <v>9113</v>
       </c>
       <c r="H144" s="3" t="inlineStr">
         <is>
-          <t>20/24</t>
+          <t>21/24</t>
         </is>
       </c>
       <c r="I144" s="3" t="inlineStr">
@@ -7587,10 +7587,10 @@
         </is>
       </c>
       <c r="J144" s="4" t="n">
-        <v>9403</v>
+        <v>10415</v>
       </c>
       <c r="K144" s="5" t="n">
-        <v>391.8</v>
+        <v>433.952380952381</v>
       </c>
     </row>
     <row r="145">
@@ -7623,11 +7623,11 @@
         </is>
       </c>
       <c r="G145" s="7" t="n">
-        <v>8662</v>
+        <v>8738</v>
       </c>
       <c r="H145" s="6" t="inlineStr">
         <is>
-          <t>12/20</t>
+          <t>13/20</t>
         </is>
       </c>
       <c r="I145" s="6" t="inlineStr">
@@ -7636,10 +7636,10 @@
         </is>
       </c>
       <c r="J145" s="7" t="n">
-        <v>14437</v>
+        <v>13443</v>
       </c>
       <c r="K145" s="8" t="n">
-        <v>721.8333333333334</v>
+        <v>672.1538461538462</v>
       </c>
     </row>
     <row r="146">
@@ -7966,11 +7966,11 @@
         </is>
       </c>
       <c r="G152" s="7" t="n">
-        <v>6479</v>
+        <v>8002</v>
       </c>
       <c r="H152" s="6" t="inlineStr">
         <is>
-          <t>11/21</t>
+          <t>12/21</t>
         </is>
       </c>
       <c r="I152" s="6" t="inlineStr">
@@ -7979,10 +7979,10 @@
         </is>
       </c>
       <c r="J152" s="7" t="n">
-        <v>12369</v>
+        <v>14004</v>
       </c>
       <c r="K152" s="8" t="n">
-        <v>589</v>
+        <v>666.8333333333334</v>
       </c>
     </row>
     <row r="153">
@@ -8064,11 +8064,11 @@
         </is>
       </c>
       <c r="G154" s="4" t="n">
-        <v>29780</v>
+        <v>32150</v>
       </c>
       <c r="H154" s="3" t="inlineStr">
         <is>
-          <t>9/23</t>
+          <t>10/23</t>
         </is>
       </c>
       <c r="I154" s="3" t="inlineStr">
@@ -8077,10 +8077,10 @@
         </is>
       </c>
       <c r="J154" s="4" t="n">
-        <v>76104</v>
+        <v>73945</v>
       </c>
       <c r="K154" s="5" t="n">
-        <v>3308.888888888889</v>
+        <v>3215</v>
       </c>
     </row>
     <row r="155">
@@ -8162,11 +8162,11 @@
         </is>
       </c>
       <c r="G156" s="15" t="n">
-        <v>254</v>
+        <v>632</v>
       </c>
       <c r="H156" s="14" t="inlineStr">
         <is>
-          <t>7/25</t>
+          <t>8/25</t>
         </is>
       </c>
       <c r="I156" s="14" t="inlineStr">
@@ -8175,10 +8175,10 @@
         </is>
       </c>
       <c r="J156" s="15" t="n">
-        <v>907</v>
+        <v>1975</v>
       </c>
       <c r="K156" s="16" t="n">
-        <v>36.28571428571428</v>
+        <v>79</v>
       </c>
     </row>
     <row r="157">
@@ -8211,11 +8211,11 @@
         </is>
       </c>
       <c r="G157" s="7" t="n">
-        <v>4689</v>
+        <v>3976</v>
       </c>
       <c r="H157" s="6" t="inlineStr">
         <is>
-          <t>15/25</t>
+          <t>16/25</t>
         </is>
       </c>
       <c r="I157" s="6" t="inlineStr">
@@ -8224,59 +8224,59 @@
         </is>
       </c>
       <c r="J157" s="7" t="n">
-        <v>7815</v>
+        <v>6212</v>
       </c>
       <c r="K157" s="8" t="n">
-        <v>312.6</v>
+        <v>248.5</v>
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="6" t="inlineStr">
+      <c r="A158" s="9" t="inlineStr">
         <is>
           <t>SATTUR</t>
         </is>
       </c>
-      <c r="B158" s="6" t="n">
+      <c r="B158" s="10" t="n">
         <v>204</v>
       </c>
-      <c r="C158" s="6" t="inlineStr">
+      <c r="C158" s="10" t="inlineStr">
+        <is>
+          <t>KADARKARAIRAJ. A</t>
+        </is>
+      </c>
+      <c r="D158" s="10" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E158" s="10" t="inlineStr">
         <is>
           <t>AJITH. M</t>
         </is>
       </c>
-      <c r="D158" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E158" s="6" t="inlineStr">
-        <is>
-          <t>NAINAR NAGENTHRAN</t>
-        </is>
-      </c>
-      <c r="F158" s="6" t="inlineStr">
-        <is>
-          <t>Bharatiya Janata Party</t>
-        </is>
-      </c>
-      <c r="G158" s="7" t="n">
-        <v>648</v>
-      </c>
-      <c r="H158" s="6" t="inlineStr">
-        <is>
-          <t>5/21</t>
-        </is>
-      </c>
-      <c r="I158" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J158" s="7" t="n">
-        <v>2722</v>
-      </c>
-      <c r="K158" s="8" t="n">
-        <v>129.6</v>
+      <c r="F158" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G158" s="11" t="n">
+        <v>46</v>
+      </c>
+      <c r="H158" s="10" t="inlineStr">
+        <is>
+          <t>6/21</t>
+        </is>
+      </c>
+      <c r="I158" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J158" s="11" t="n">
+        <v>161</v>
+      </c>
+      <c r="K158" s="12" t="n">
+        <v>7.666666666666667</v>
       </c>
     </row>
     <row r="159">
@@ -8329,52 +8329,52 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="6" t="inlineStr">
+      <c r="A160" s="9" t="inlineStr">
         <is>
           <t>SHOLAVANDAN</t>
         </is>
       </c>
-      <c r="B160" s="6" t="n">
+      <c r="B160" s="10" t="n">
         <v>190</v>
       </c>
-      <c r="C160" s="6" t="inlineStr">
+      <c r="C160" s="10" t="inlineStr">
+        <is>
+          <t>VENKATESAN.A</t>
+        </is>
+      </c>
+      <c r="D160" s="10" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E160" s="10" t="inlineStr">
         <is>
           <t>KARUPPAIAH.M.V</t>
         </is>
       </c>
-      <c r="D160" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E160" s="6" t="inlineStr">
-        <is>
-          <t>VENKATESAN.A</t>
-        </is>
-      </c>
-      <c r="F160" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G160" s="7" t="n">
-        <v>385</v>
-      </c>
-      <c r="H160" s="6" t="inlineStr">
-        <is>
-          <t>6/19</t>
-        </is>
-      </c>
-      <c r="I160" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J160" s="7" t="n">
-        <v>1219</v>
-      </c>
-      <c r="K160" s="8" t="n">
-        <v>64.16666666666667</v>
+      <c r="F160" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G160" s="11" t="n">
+        <v>100</v>
+      </c>
+      <c r="H160" s="10" t="inlineStr">
+        <is>
+          <t>7/19</t>
+        </is>
+      </c>
+      <c r="I160" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J160" s="11" t="n">
+        <v>271</v>
+      </c>
+      <c r="K160" s="12" t="n">
+        <v>14.28571428571429</v>
       </c>
     </row>
     <row r="161">
@@ -8701,11 +8701,11 @@
         </is>
       </c>
       <c r="G167" s="4" t="n">
-        <v>22056</v>
+        <v>22421</v>
       </c>
       <c r="H167" s="3" t="inlineStr">
         <is>
-          <t>13/32</t>
+          <t>14/32</t>
         </is>
       </c>
       <c r="I167" s="3" t="inlineStr">
@@ -8714,10 +8714,10 @@
         </is>
       </c>
       <c r="J167" s="4" t="n">
-        <v>54292</v>
+        <v>51248</v>
       </c>
       <c r="K167" s="5" t="n">
-        <v>1696.615384615385</v>
+        <v>1601.5</v>
       </c>
     </row>
     <row r="168">
@@ -8995,11 +8995,11 @@
         </is>
       </c>
       <c r="G173" s="7" t="n">
-        <v>7451</v>
+        <v>6597</v>
       </c>
       <c r="H173" s="6" t="inlineStr">
         <is>
-          <t>12/26</t>
+          <t>13/26</t>
         </is>
       </c>
       <c r="I173" s="6" t="inlineStr">
@@ -9008,10 +9008,10 @@
         </is>
       </c>
       <c r="J173" s="7" t="n">
-        <v>16144</v>
+        <v>13194</v>
       </c>
       <c r="K173" s="8" t="n">
-        <v>620.9166666666666</v>
+        <v>507.4615384615385</v>
       </c>
     </row>
     <row r="174">
@@ -9142,11 +9142,11 @@
         </is>
       </c>
       <c r="G176" s="4" t="n">
-        <v>17033</v>
+        <v>18505</v>
       </c>
       <c r="H176" s="3" t="inlineStr">
         <is>
-          <t>12/17</t>
+          <t>13/17</t>
         </is>
       </c>
       <c r="I176" s="3" t="inlineStr">
@@ -9155,10 +9155,10 @@
         </is>
       </c>
       <c r="J176" s="4" t="n">
-        <v>24130</v>
+        <v>24199</v>
       </c>
       <c r="K176" s="5" t="n">
-        <v>1419.416666666667</v>
+        <v>1423.461538461539</v>
       </c>
     </row>
     <row r="177">
@@ -9191,11 +9191,11 @@
         </is>
       </c>
       <c r="G177" s="7" t="n">
-        <v>10764</v>
+        <v>12637</v>
       </c>
       <c r="H177" s="6" t="inlineStr">
         <is>
-          <t>16/26</t>
+          <t>17/26</t>
         </is>
       </c>
       <c r="I177" s="6" t="inlineStr">
@@ -9204,10 +9204,10 @@
         </is>
       </c>
       <c r="J177" s="7" t="n">
-        <v>17492</v>
+        <v>19327</v>
       </c>
       <c r="K177" s="8" t="n">
-        <v>672.75</v>
+        <v>743.3529411764706</v>
       </c>
     </row>
     <row r="178">
@@ -9387,11 +9387,11 @@
         </is>
       </c>
       <c r="G181" s="7" t="n">
-        <v>7276</v>
+        <v>7552</v>
       </c>
       <c r="H181" s="6" t="inlineStr">
         <is>
-          <t>14/21</t>
+          <t>15/21</t>
         </is>
       </c>
       <c r="I181" s="6" t="inlineStr">
@@ -9400,10 +9400,10 @@
         </is>
       </c>
       <c r="J181" s="7" t="n">
-        <v>10914</v>
+        <v>10573</v>
       </c>
       <c r="K181" s="8" t="n">
-        <v>519.7142857142857</v>
+        <v>503.4666666666666</v>
       </c>
     </row>
     <row r="182">
@@ -9436,11 +9436,11 @@
         </is>
       </c>
       <c r="G182" s="7" t="n">
-        <v>5715</v>
+        <v>6214</v>
       </c>
       <c r="H182" s="6" t="inlineStr">
         <is>
-          <t>9/25</t>
+          <t>10/25</t>
         </is>
       </c>
       <c r="I182" s="6" t="inlineStr">
@@ -9449,10 +9449,10 @@
         </is>
       </c>
       <c r="J182" s="7" t="n">
-        <v>15875</v>
+        <v>15535</v>
       </c>
       <c r="K182" s="8" t="n">
-        <v>635</v>
+        <v>621.4</v>
       </c>
     </row>
     <row r="183">
@@ -9534,11 +9534,11 @@
         </is>
       </c>
       <c r="G184" s="4" t="n">
-        <v>14874</v>
+        <v>15935</v>
       </c>
       <c r="H184" s="3" t="inlineStr">
         <is>
-          <t>21/24</t>
+          <t>22/24</t>
         </is>
       </c>
       <c r="I184" s="3" t="inlineStr">
@@ -9547,10 +9547,10 @@
         </is>
       </c>
       <c r="J184" s="4" t="n">
-        <v>16999</v>
+        <v>17384</v>
       </c>
       <c r="K184" s="5" t="n">
-        <v>708.2857142857143</v>
+        <v>724.3181818181819</v>
       </c>
     </row>
     <row r="185">
@@ -9632,11 +9632,11 @@
         </is>
       </c>
       <c r="G186" s="7" t="n">
-        <v>8162</v>
+        <v>7720</v>
       </c>
       <c r="H186" s="6" t="inlineStr">
         <is>
-          <t>11/24</t>
+          <t>12/24</t>
         </is>
       </c>
       <c r="I186" s="6" t="inlineStr">
@@ -9645,10 +9645,10 @@
         </is>
       </c>
       <c r="J186" s="7" t="n">
-        <v>17808</v>
+        <v>15440</v>
       </c>
       <c r="K186" s="8" t="n">
-        <v>742</v>
+        <v>643.3333333333334</v>
       </c>
     </row>
     <row r="187">
@@ -9681,11 +9681,11 @@
         </is>
       </c>
       <c r="G187" s="4" t="n">
-        <v>31253</v>
+        <v>33635</v>
       </c>
       <c r="H187" s="3" t="inlineStr">
         <is>
-          <t>13/25</t>
+          <t>14/25</t>
         </is>
       </c>
       <c r="I187" s="3" t="inlineStr">
@@ -9694,10 +9694,10 @@
         </is>
       </c>
       <c r="J187" s="4" t="n">
-        <v>60102</v>
+        <v>60062</v>
       </c>
       <c r="K187" s="5" t="n">
-        <v>2404.076923076923</v>
+        <v>2402.5</v>
       </c>
     </row>
     <row r="188">
@@ -9730,11 +9730,11 @@
         </is>
       </c>
       <c r="G188" s="7" t="n">
-        <v>10721</v>
+        <v>11423</v>
       </c>
       <c r="H188" s="6" t="inlineStr">
         <is>
-          <t>12/18</t>
+          <t>13/18</t>
         </is>
       </c>
       <c r="I188" s="6" t="inlineStr">
@@ -9743,10 +9743,10 @@
         </is>
       </c>
       <c r="J188" s="7" t="n">
-        <v>16082</v>
+        <v>15816</v>
       </c>
       <c r="K188" s="8" t="n">
-        <v>893.4166666666666</v>
+        <v>878.6923076923077</v>
       </c>
     </row>
     <row r="189">
@@ -9779,11 +9779,11 @@
         </is>
       </c>
       <c r="G189" s="4" t="n">
-        <v>14946</v>
+        <v>14769</v>
       </c>
       <c r="H189" s="3" t="inlineStr">
         <is>
-          <t>10/27</t>
+          <t>11/27</t>
         </is>
       </c>
       <c r="I189" s="3" t="inlineStr">
@@ -9792,10 +9792,10 @@
         </is>
       </c>
       <c r="J189" s="4" t="n">
-        <v>40354</v>
+        <v>36251</v>
       </c>
       <c r="K189" s="5" t="n">
-        <v>1494.6</v>
+        <v>1342.636363636364</v>
       </c>
     </row>
     <row r="190">
@@ -9877,11 +9877,11 @@
         </is>
       </c>
       <c r="G191" s="7" t="n">
-        <v>4534</v>
+        <v>5258</v>
       </c>
       <c r="H191" s="6" t="inlineStr">
         <is>
-          <t>8/18</t>
+          <t>9/18</t>
         </is>
       </c>
       <c r="I191" s="6" t="inlineStr">
@@ -9890,10 +9890,10 @@
         </is>
       </c>
       <c r="J191" s="7" t="n">
-        <v>10202</v>
+        <v>10516</v>
       </c>
       <c r="K191" s="8" t="n">
-        <v>566.75</v>
+        <v>584.2222222222222</v>
       </c>
     </row>
     <row r="192">
@@ -9946,51 +9946,51 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="13" t="inlineStr">
+      <c r="A193" s="9" t="inlineStr">
         <is>
           <t>TINDIVANAM</t>
         </is>
       </c>
-      <c r="B193" s="14" t="n">
+      <c r="B193" s="10" t="n">
         <v>72</v>
       </c>
-      <c r="C193" s="14" t="inlineStr">
+      <c r="C193" s="10" t="inlineStr">
         <is>
           <t>ARJUNAN. P</t>
         </is>
       </c>
-      <c r="D193" s="14" t="inlineStr">
+      <c r="D193" s="10" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E193" s="14" t="inlineStr">
+      <c r="E193" s="10" t="inlineStr">
         <is>
           <t>VANNI ARASU</t>
         </is>
       </c>
-      <c r="F193" s="14" t="inlineStr">
+      <c r="F193" s="10" t="inlineStr">
         <is>
           <t>Viduthalai Chiruthaigal Katchi</t>
         </is>
       </c>
-      <c r="G193" s="15" t="n">
+      <c r="G193" s="11" t="n">
         <v>144</v>
       </c>
-      <c r="H193" s="14" t="inlineStr">
+      <c r="H193" s="10" t="inlineStr">
         <is>
           <t>10/21</t>
         </is>
       </c>
-      <c r="I193" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J193" s="15" t="n">
+      <c r="I193" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J193" s="11" t="n">
         <v>302</v>
       </c>
-      <c r="K193" s="16" t="n">
+      <c r="K193" s="12" t="n">
         <v>14.4</v>
       </c>
     </row>
@@ -10122,11 +10122,11 @@
         </is>
       </c>
       <c r="G196" s="4" t="n">
-        <v>12657</v>
+        <v>13879</v>
       </c>
       <c r="H196" s="3" t="inlineStr">
         <is>
-          <t>10/22</t>
+          <t>11/22</t>
         </is>
       </c>
       <c r="I196" s="3" t="inlineStr">
@@ -10135,10 +10135,10 @@
         </is>
       </c>
       <c r="J196" s="4" t="n">
-        <v>27845</v>
+        <v>27758</v>
       </c>
       <c r="K196" s="5" t="n">
-        <v>1265.7</v>
+        <v>1261.727272727273</v>
       </c>
     </row>
     <row r="197">
@@ -10250,30 +10250,30 @@
       </c>
       <c r="C199" s="14" t="inlineStr">
         <is>
+          <t>PALANISAMY S</t>
+        </is>
+      </c>
+      <c r="D199" s="14" t="inlineStr">
+        <is>
+          <t>All India Anna Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E199" s="14" t="inlineStr">
+        <is>
           <t>VIJAY R BARANIBALAAJI</t>
         </is>
       </c>
-      <c r="D199" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E199" s="14" t="inlineStr">
-        <is>
-          <t>PALANISAMY S</t>
-        </is>
-      </c>
       <c r="F199" s="14" t="inlineStr">
         <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
+          <t>Tamilaga Vettri Kazhagam</t>
         </is>
       </c>
       <c r="G199" s="15" t="n">
-        <v>335</v>
+        <v>279</v>
       </c>
       <c r="H199" s="14" t="inlineStr">
         <is>
-          <t>11/24</t>
+          <t>12/24</t>
         </is>
       </c>
       <c r="I199" s="14" t="inlineStr">
@@ -10282,10 +10282,10 @@
         </is>
       </c>
       <c r="J199" s="15" t="n">
-        <v>731</v>
+        <v>558</v>
       </c>
       <c r="K199" s="16" t="n">
-        <v>30.45454545454545</v>
+        <v>23.25</v>
       </c>
     </row>
     <row r="200">
@@ -10318,11 +10318,11 @@
         </is>
       </c>
       <c r="G200" s="4" t="n">
-        <v>5735</v>
+        <v>6363</v>
       </c>
       <c r="H200" s="3" t="inlineStr">
         <is>
-          <t>21/28</t>
+          <t>22/28</t>
         </is>
       </c>
       <c r="I200" s="3" t="inlineStr">
@@ -10331,10 +10331,10 @@
         </is>
       </c>
       <c r="J200" s="4" t="n">
-        <v>7647</v>
+        <v>8098</v>
       </c>
       <c r="K200" s="5" t="n">
-        <v>273.0952380952381</v>
+        <v>289.2272727272727</v>
       </c>
     </row>
     <row r="201">
@@ -10514,11 +10514,11 @@
         </is>
       </c>
       <c r="G204" s="4" t="n">
-        <v>12273</v>
+        <v>13479</v>
       </c>
       <c r="H204" s="3" t="inlineStr">
         <is>
-          <t>10/21</t>
+          <t>11/21</t>
         </is>
       </c>
       <c r="I204" s="3" t="inlineStr">
@@ -10527,10 +10527,10 @@
         </is>
       </c>
       <c r="J204" s="4" t="n">
-        <v>25773</v>
+        <v>25733</v>
       </c>
       <c r="K204" s="5" t="n">
-        <v>1227.3</v>
+        <v>1225.363636363636</v>
       </c>
     </row>
     <row r="205">
@@ -10563,11 +10563,11 @@
         </is>
       </c>
       <c r="G205" s="7" t="n">
-        <v>4588</v>
+        <v>6509</v>
       </c>
       <c r="H205" s="6" t="inlineStr">
         <is>
-          <t>10/25</t>
+          <t>11/25</t>
         </is>
       </c>
       <c r="I205" s="6" t="inlineStr">
@@ -10576,10 +10576,10 @@
         </is>
       </c>
       <c r="J205" s="7" t="n">
-        <v>11470</v>
+        <v>14793</v>
       </c>
       <c r="K205" s="8" t="n">
-        <v>458.8</v>
+        <v>591.7272727272727</v>
       </c>
     </row>
     <row r="206">
@@ -10710,11 +10710,11 @@
         </is>
       </c>
       <c r="G208" s="7" t="n">
-        <v>2253</v>
+        <v>2021</v>
       </c>
       <c r="H208" s="6" t="inlineStr">
         <is>
-          <t>8/20</t>
+          <t>9/20</t>
         </is>
       </c>
       <c r="I208" s="6" t="inlineStr">
@@ -10723,58 +10723,58 @@
         </is>
       </c>
       <c r="J208" s="7" t="n">
-        <v>5632</v>
+        <v>4491</v>
       </c>
       <c r="K208" s="8" t="n">
-        <v>281.625</v>
+        <v>224.5555555555555</v>
       </c>
     </row>
     <row r="209">
-      <c r="A209" s="13" t="inlineStr">
+      <c r="A209" s="9" t="inlineStr">
         <is>
           <t>UDHAGAMANDALAM</t>
         </is>
       </c>
-      <c r="B209" s="14" t="n">
+      <c r="B209" s="10" t="n">
         <v>108</v>
       </c>
-      <c r="C209" s="14" t="inlineStr">
+      <c r="C209" s="10" t="inlineStr">
         <is>
           <t>BHOJARAJAN.M</t>
         </is>
       </c>
-      <c r="D209" s="14" t="inlineStr">
+      <c r="D209" s="10" t="inlineStr">
         <is>
           <t>Bharatiya Janata Party</t>
         </is>
       </c>
-      <c r="E209" s="14" t="inlineStr">
+      <c r="E209" s="10" t="inlineStr">
         <is>
           <t>IBRAHIM.R</t>
         </is>
       </c>
-      <c r="F209" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G209" s="15" t="n">
+      <c r="F209" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G209" s="11" t="n">
         <v>189</v>
       </c>
-      <c r="H209" s="14" t="inlineStr">
+      <c r="H209" s="10" t="inlineStr">
         <is>
           <t>17/19</t>
         </is>
       </c>
-      <c r="I209" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J209" s="15" t="n">
+      <c r="I209" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J209" s="11" t="n">
         <v>211</v>
       </c>
-      <c r="K209" s="16" t="n">
+      <c r="K209" s="12" t="n">
         <v>11.11764705882353</v>
       </c>
     </row>
@@ -10828,52 +10828,52 @@
       </c>
     </row>
     <row r="211">
-      <c r="A211" s="6" t="inlineStr">
+      <c r="A211" s="13" t="inlineStr">
         <is>
           <t>ULUNDURPETTAI</t>
         </is>
       </c>
-      <c r="B211" s="6" t="n">
+      <c r="B211" s="14" t="n">
         <v>77</v>
       </c>
-      <c r="C211" s="6" t="inlineStr">
+      <c r="C211" s="14" t="inlineStr">
         <is>
           <t>VASANTHAVEL G R</t>
         </is>
       </c>
-      <c r="D211" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E211" s="6" t="inlineStr">
+      <c r="D211" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E211" s="14" t="inlineStr">
         <is>
           <t>KUMARAGURU R</t>
         </is>
       </c>
-      <c r="F211" s="6" t="inlineStr">
+      <c r="F211" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G211" s="7" t="n">
-        <v>590</v>
-      </c>
-      <c r="H211" s="6" t="inlineStr">
-        <is>
-          <t>10/27</t>
-        </is>
-      </c>
-      <c r="I211" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J211" s="7" t="n">
-        <v>1593</v>
-      </c>
-      <c r="K211" s="8" t="n">
-        <v>59</v>
+      <c r="G211" s="15" t="n">
+        <v>913</v>
+      </c>
+      <c r="H211" s="14" t="inlineStr">
+        <is>
+          <t>11/27</t>
+        </is>
+      </c>
+      <c r="I211" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J211" s="15" t="n">
+        <v>2241</v>
+      </c>
+      <c r="K211" s="16" t="n">
+        <v>83</v>
       </c>
     </row>
     <row r="212">
@@ -10955,11 +10955,11 @@
         </is>
       </c>
       <c r="G213" s="7" t="n">
-        <v>3312</v>
+        <v>4544</v>
       </c>
       <c r="H213" s="6" t="inlineStr">
         <is>
-          <t>16/23</t>
+          <t>17/23</t>
         </is>
       </c>
       <c r="I213" s="6" t="inlineStr">
@@ -10968,10 +10968,10 @@
         </is>
       </c>
       <c r="J213" s="7" t="n">
-        <v>4761</v>
+        <v>6148</v>
       </c>
       <c r="K213" s="8" t="n">
-        <v>207</v>
+        <v>267.2941176470588</v>
       </c>
     </row>
     <row r="214">
@@ -11004,11 +11004,11 @@
         </is>
       </c>
       <c r="G214" s="4" t="n">
-        <v>13518</v>
+        <v>13510</v>
       </c>
       <c r="H214" s="3" t="inlineStr">
         <is>
-          <t>14/23</t>
+          <t>15/23</t>
         </is>
       </c>
       <c r="I214" s="3" t="inlineStr">
@@ -11017,10 +11017,10 @@
         </is>
       </c>
       <c r="J214" s="4" t="n">
-        <v>22208</v>
+        <v>20715</v>
       </c>
       <c r="K214" s="5" t="n">
-        <v>965.5714285714286</v>
+        <v>900.6666666666666</v>
       </c>
     </row>
     <row r="215">
@@ -11249,11 +11249,11 @@
         </is>
       </c>
       <c r="G219" s="7" t="n">
-        <v>6277</v>
+        <v>6212</v>
       </c>
       <c r="H219" s="6" t="inlineStr">
         <is>
-          <t>13/23</t>
+          <t>14/23</t>
         </is>
       </c>
       <c r="I219" s="6" t="inlineStr">
@@ -11262,10 +11262,10 @@
         </is>
       </c>
       <c r="J219" s="7" t="n">
-        <v>11105</v>
+        <v>10205</v>
       </c>
       <c r="K219" s="8" t="n">
-        <v>482.8461538461539</v>
+        <v>443.7142857142857</v>
       </c>
     </row>
     <row r="220">
@@ -11445,11 +11445,11 @@
         </is>
       </c>
       <c r="G223" s="4" t="n">
-        <v>22174</v>
+        <v>23400</v>
       </c>
       <c r="H223" s="3" t="inlineStr">
         <is>
-          <t>13/23</t>
+          <t>14/23</t>
         </is>
       </c>
       <c r="I223" s="3" t="inlineStr">
@@ -11458,59 +11458,59 @@
         </is>
       </c>
       <c r="J223" s="4" t="n">
-        <v>39231</v>
+        <v>38443</v>
       </c>
       <c r="K223" s="5" t="n">
-        <v>1705.692307692308</v>
+        <v>1671.428571428571</v>
       </c>
     </row>
     <row r="224">
-      <c r="A224" s="6" t="inlineStr">
+      <c r="A224" s="13" t="inlineStr">
         <is>
           <t>VELLORE</t>
         </is>
       </c>
-      <c r="B224" s="6" t="n">
+      <c r="B224" s="14" t="n">
         <v>43</v>
       </c>
-      <c r="C224" s="6" t="inlineStr">
+      <c r="C224" s="14" t="inlineStr">
         <is>
           <t>P.KARTHIKEYAN</t>
         </is>
       </c>
-      <c r="D224" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E224" s="6" t="inlineStr">
+      <c r="D224" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E224" s="14" t="inlineStr">
         <is>
           <t>M.M.VINOTH KANNAN</t>
         </is>
       </c>
-      <c r="F224" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G224" s="7" t="n">
-        <v>1822</v>
-      </c>
-      <c r="H224" s="6" t="inlineStr">
-        <is>
-          <t>11/20</t>
-        </is>
-      </c>
-      <c r="I224" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J224" s="7" t="n">
-        <v>3313</v>
-      </c>
-      <c r="K224" s="8" t="n">
-        <v>165.6363636363636</v>
+      <c r="F224" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G224" s="15" t="n">
+        <v>1240</v>
+      </c>
+      <c r="H224" s="14" t="inlineStr">
+        <is>
+          <t>12/20</t>
+        </is>
+      </c>
+      <c r="I224" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J224" s="15" t="n">
+        <v>2067</v>
+      </c>
+      <c r="K224" s="16" t="n">
+        <v>103.3333333333333</v>
       </c>
     </row>
     <row r="225">
@@ -11563,51 +11563,51 @@
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="6" t="inlineStr">
+      <c r="A226" s="13" t="inlineStr">
         <is>
           <t>VIKRAVANDI</t>
         </is>
       </c>
-      <c r="B226" s="6" t="n">
+      <c r="B226" s="14" t="n">
         <v>75</v>
       </c>
-      <c r="C226" s="6" t="inlineStr">
+      <c r="C226" s="14" t="inlineStr">
         <is>
           <t>VIJAI VADIVEL A</t>
         </is>
       </c>
-      <c r="D226" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E226" s="6" t="inlineStr">
+      <c r="D226" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E226" s="14" t="inlineStr">
         <is>
           <t>SIVAKUMAR C</t>
         </is>
       </c>
-      <c r="F226" s="6" t="inlineStr">
+      <c r="F226" s="14" t="inlineStr">
         <is>
           <t>Pattali Makkal Katchi</t>
         </is>
       </c>
-      <c r="G226" s="7" t="n">
+      <c r="G226" s="15" t="n">
         <v>542</v>
       </c>
-      <c r="H226" s="6" t="inlineStr">
+      <c r="H226" s="14" t="inlineStr">
         <is>
           <t>7/23</t>
         </is>
       </c>
-      <c r="I226" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J226" s="7" t="n">
+      <c r="I226" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J226" s="15" t="n">
         <v>1781</v>
       </c>
-      <c r="K226" s="8" t="n">
+      <c r="K226" s="16" t="n">
         <v>77.42857142857143</v>
       </c>
     </row>
@@ -11641,11 +11641,11 @@
         </is>
       </c>
       <c r="G227" s="7" t="n">
-        <v>4521</v>
+        <v>4883</v>
       </c>
       <c r="H227" s="6" t="inlineStr">
         <is>
-          <t>14/20</t>
+          <t>15/20</t>
         </is>
       </c>
       <c r="I227" s="6" t="inlineStr">
@@ -11654,10 +11654,10 @@
         </is>
       </c>
       <c r="J227" s="7" t="n">
-        <v>6459</v>
+        <v>6511</v>
       </c>
       <c r="K227" s="8" t="n">
-        <v>322.9285714285714</v>
+        <v>325.5333333333334</v>
       </c>
     </row>
     <row r="228">
@@ -11690,11 +11690,11 @@
         </is>
       </c>
       <c r="G228" s="4" t="n">
-        <v>13237</v>
+        <v>14202</v>
       </c>
       <c r="H228" s="3" t="inlineStr">
         <is>
-          <t>11/22</t>
+          <t>12/22</t>
         </is>
       </c>
       <c r="I228" s="3" t="inlineStr">
@@ -11703,10 +11703,10 @@
         </is>
       </c>
       <c r="J228" s="4" t="n">
-        <v>26474</v>
+        <v>26037</v>
       </c>
       <c r="K228" s="5" t="n">
-        <v>1203.363636363636</v>
+        <v>1183.5</v>
       </c>
     </row>
     <row r="229">
@@ -11759,51 +11759,51 @@
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="6" t="inlineStr">
+      <c r="A230" s="13" t="inlineStr">
         <is>
           <t>VILUPPURAM</t>
         </is>
       </c>
-      <c r="B230" s="6" t="n">
+      <c r="B230" s="14" t="n">
         <v>74</v>
       </c>
-      <c r="C230" s="6" t="inlineStr">
+      <c r="C230" s="14" t="inlineStr">
         <is>
           <t>LAKSHMANAN R</t>
         </is>
       </c>
-      <c r="D230" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E230" s="6" t="inlineStr">
+      <c r="D230" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E230" s="14" t="inlineStr">
         <is>
           <t>MOHANRAJ N</t>
         </is>
       </c>
-      <c r="F230" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G230" s="7" t="n">
+      <c r="F230" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G230" s="15" t="n">
         <v>1148</v>
       </c>
-      <c r="H230" s="6" t="inlineStr">
+      <c r="H230" s="14" t="inlineStr">
         <is>
           <t>14/24</t>
         </is>
       </c>
-      <c r="I230" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J230" s="7" t="n">
+      <c r="I230" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J230" s="15" t="n">
         <v>1968</v>
       </c>
-      <c r="K230" s="8" t="n">
+      <c r="K230" s="16" t="n">
         <v>82</v>
       </c>
     </row>
@@ -11837,11 +11837,11 @@
         </is>
       </c>
       <c r="G231" s="4" t="n">
-        <v>27640</v>
+        <v>30932</v>
       </c>
       <c r="H231" s="3" t="inlineStr">
         <is>
-          <t>9/20</t>
+          <t>10/20</t>
         </is>
       </c>
       <c r="I231" s="3" t="inlineStr">
@@ -11850,10 +11850,10 @@
         </is>
       </c>
       <c r="J231" s="4" t="n">
-        <v>61422</v>
+        <v>61864</v>
       </c>
       <c r="K231" s="5" t="n">
-        <v>3071.111111111111</v>
+        <v>3093.2</v>
       </c>
     </row>
     <row r="232">
@@ -11886,11 +11886,11 @@
         </is>
       </c>
       <c r="G232" s="7" t="n">
-        <v>1970</v>
+        <v>2769</v>
       </c>
       <c r="H232" s="6" t="inlineStr">
         <is>
-          <t>10/21</t>
+          <t>11/21</t>
         </is>
       </c>
       <c r="I232" s="6" t="inlineStr">
@@ -11899,10 +11899,10 @@
         </is>
       </c>
       <c r="J232" s="7" t="n">
-        <v>4137</v>
+        <v>5286</v>
       </c>
       <c r="K232" s="8" t="n">
-        <v>197</v>
+        <v>251.7272727272727</v>
       </c>
     </row>
     <row r="233">
@@ -12097,7 +12097,7 @@
       <c r="B2" s="19" t="n"/>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Contest index ≤ 10  — margin tiny relative to rounds left</t>
+          <t>Contest index ≤ 10 OR projected margin &lt; 500 — could flip any round</t>
         </is>
       </c>
     </row>
@@ -12110,7 +12110,7 @@
       <c r="B3" s="20" t="n"/>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Contest index 10–40 — still very much in play</t>
+          <t>Contest index 10–40 OR projected margin &lt; 3000 — still very much in play</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update election results snapshot (59.2% counted)
TVK 106, DMK 59, AIADMK 50. TIRUVADANAI down to 17-vote TVK lead,
tied with ALANGULAM as tightest seats. 9 knife-edge seats, 39 in play.

https://claude.ai/code/session_01MizbUy44JG5sXyvaf3Wekb
</commit_message>
<xml_diff>
--- a/tn_election_results_may2026.xlsx
+++ b/tn_election_results_may2026.xlsx
@@ -665,11 +665,11 @@
         </is>
       </c>
       <c r="G3" s="7" t="n">
-        <v>4388</v>
+        <v>4654</v>
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
-          <t>8/20</t>
+          <t>9/20</t>
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr">
@@ -678,10 +678,10 @@
         </is>
       </c>
       <c r="J3" s="7" t="n">
-        <v>10970</v>
+        <v>10342</v>
       </c>
       <c r="K3" s="8" t="n">
-        <v>548.5</v>
+        <v>517.1111111111111</v>
       </c>
     </row>
     <row r="4">
@@ -763,11 +763,11 @@
         </is>
       </c>
       <c r="G5" s="4" t="n">
-        <v>8422</v>
+        <v>9100</v>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>18/23</t>
+          <t>19/23</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -776,10 +776,10 @@
         </is>
       </c>
       <c r="J5" s="4" t="n">
-        <v>10761</v>
+        <v>11016</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>467.8888888888889</v>
+        <v>478.9473684210527</v>
       </c>
     </row>
     <row r="6">
@@ -812,11 +812,11 @@
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>35744</v>
+        <v>38162</v>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>14/27</t>
+          <t>15/27</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -825,10 +825,10 @@
         </is>
       </c>
       <c r="J6" s="4" t="n">
-        <v>68935</v>
+        <v>68692</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>2553.142857142857</v>
+        <v>2544.133333333333</v>
       </c>
     </row>
     <row r="7">
@@ -852,20 +852,20 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>VENKATESAN. R</t>
+          <t>VILWANATHAN. A.C.</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
+          <t>Dravida Munnetra Kazhagam</t>
         </is>
       </c>
       <c r="G7" s="7" t="n">
-        <v>8055</v>
+        <v>6012</v>
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>9/22</t>
+          <t>10/22</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
@@ -874,10 +874,10 @@
         </is>
       </c>
       <c r="J7" s="7" t="n">
-        <v>19690</v>
+        <v>13226</v>
       </c>
       <c r="K7" s="8" t="n">
-        <v>895</v>
+        <v>601.2</v>
       </c>
     </row>
     <row r="8">
@@ -910,11 +910,11 @@
         </is>
       </c>
       <c r="G8" s="7" t="n">
-        <v>5844</v>
+        <v>5762</v>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>11/22</t>
+          <t>12/22</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
@@ -923,10 +923,10 @@
         </is>
       </c>
       <c r="J8" s="7" t="n">
-        <v>11688</v>
+        <v>10564</v>
       </c>
       <c r="K8" s="8" t="n">
-        <v>531.2727272727273</v>
+        <v>480.1666666666667</v>
       </c>
     </row>
     <row r="9">
@@ -1008,11 +1008,11 @@
         </is>
       </c>
       <c r="G10" s="4" t="n">
-        <v>19774</v>
+        <v>21194</v>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>18/20</t>
+          <t>19/20</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
@@ -1021,10 +1021,10 @@
         </is>
       </c>
       <c r="J10" s="4" t="n">
-        <v>21971</v>
+        <v>22309</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>1098.555555555556</v>
+        <v>1115.473684210526</v>
       </c>
     </row>
     <row r="11">
@@ -1106,11 +1106,11 @@
         </is>
       </c>
       <c r="G12" s="4" t="n">
-        <v>20738</v>
+        <v>22198</v>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>18/21</t>
+          <t>19/22</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
@@ -1119,10 +1119,10 @@
         </is>
       </c>
       <c r="J12" s="4" t="n">
-        <v>24194</v>
+        <v>25703</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>1152.111111111111</v>
+        <v>1168.315789473684</v>
       </c>
     </row>
     <row r="13">
@@ -1302,11 +1302,11 @@
         </is>
       </c>
       <c r="G16" s="4" t="n">
-        <v>13905</v>
+        <v>14036</v>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>8/23</t>
+          <t>9/23</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
@@ -1315,59 +1315,59 @@
         </is>
       </c>
       <c r="J16" s="4" t="n">
-        <v>39977</v>
+        <v>35870</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>1738.125</v>
+        <v>1559.555555555556</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>ARIYALUR</t>
         </is>
       </c>
-      <c r="B17" s="6" t="n">
+      <c r="B17" s="3" t="n">
         <v>149</v>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>RAJENDRAN S</t>
         </is>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>LATHA BALU</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G17" s="7" t="n">
-        <v>12123</v>
-      </c>
-      <c r="H17" s="6" t="inlineStr">
-        <is>
-          <t>17/24</t>
-        </is>
-      </c>
-      <c r="I17" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J17" s="7" t="n">
-        <v>17115</v>
-      </c>
-      <c r="K17" s="8" t="n">
-        <v>713.1176470588235</v>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>13447</v>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>18/24</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="n">
+        <v>17929</v>
+      </c>
+      <c r="K17" s="5" t="n">
+        <v>747.0555555555555</v>
       </c>
     </row>
     <row r="18">
@@ -1596,11 +1596,11 @@
         </is>
       </c>
       <c r="G22" s="7" t="n">
-        <v>4357</v>
+        <v>6474</v>
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>16/27</t>
+          <t>17/27</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr">
@@ -1609,10 +1609,10 @@
         </is>
       </c>
       <c r="J22" s="7" t="n">
-        <v>7352</v>
+        <v>10282</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>272.3125</v>
+        <v>380.8235294117647</v>
       </c>
     </row>
     <row r="23">
@@ -1645,11 +1645,11 @@
         </is>
       </c>
       <c r="G23" s="7" t="n">
-        <v>2690</v>
+        <v>1877</v>
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>12/24</t>
+          <t>13/24</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr">
@@ -1658,10 +1658,10 @@
         </is>
       </c>
       <c r="J23" s="7" t="n">
-        <v>5380</v>
+        <v>3465</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>224.1666666666667</v>
+        <v>144.3846153846154</v>
       </c>
     </row>
     <row r="24">
@@ -1743,7 +1743,7 @@
         </is>
       </c>
       <c r="G25" s="15" t="n">
-        <v>967</v>
+        <v>1161</v>
       </c>
       <c r="H25" s="14" t="inlineStr">
         <is>
@@ -1756,10 +1756,10 @@
         </is>
       </c>
       <c r="J25" s="15" t="n">
-        <v>1547</v>
+        <v>1858</v>
       </c>
       <c r="K25" s="16" t="n">
-        <v>64.46666666666667</v>
+        <v>77.40000000000001</v>
       </c>
     </row>
     <row r="26">
@@ -1792,11 +1792,11 @@
         </is>
       </c>
       <c r="G26" s="7" t="n">
-        <v>5635</v>
+        <v>6810</v>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>11/22</t>
+          <t>12/22</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
@@ -1805,59 +1805,59 @@
         </is>
       </c>
       <c r="J26" s="7" t="n">
-        <v>11270</v>
+        <v>12485</v>
       </c>
       <c r="K26" s="8" t="n">
-        <v>512.2727272727273</v>
+        <v>567.5</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="13" t="inlineStr">
+      <c r="A27" s="6" t="inlineStr">
         <is>
           <t>BODINAYAKANUR</t>
         </is>
       </c>
-      <c r="B27" s="14" t="n">
+      <c r="B27" s="6" t="n">
         <v>200</v>
       </c>
-      <c r="C27" s="14" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>PANNEERSELVAM.O</t>
         </is>
       </c>
-      <c r="D27" s="14" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E27" s="14" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>PRAKASH.S</t>
         </is>
       </c>
-      <c r="F27" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G27" s="15" t="n">
-        <v>919</v>
-      </c>
-      <c r="H27" s="14" t="inlineStr">
-        <is>
-          <t>11/25</t>
-        </is>
-      </c>
-      <c r="I27" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J27" s="15" t="n">
-        <v>2089</v>
-      </c>
-      <c r="K27" s="16" t="n">
-        <v>83.54545454545455</v>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="n">
+        <v>2284</v>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>12/25</t>
+        </is>
+      </c>
+      <c r="I27" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J27" s="7" t="n">
+        <v>4758</v>
+      </c>
+      <c r="K27" s="8" t="n">
+        <v>190.3333333333333</v>
       </c>
     </row>
     <row r="28">
@@ -1890,11 +1890,11 @@
         </is>
       </c>
       <c r="G28" s="4" t="n">
-        <v>15060</v>
+        <v>15424</v>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>10/36</t>
+          <t>11/36</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
@@ -1903,10 +1903,10 @@
         </is>
       </c>
       <c r="J28" s="4" t="n">
-        <v>54216</v>
+        <v>50479</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>1506</v>
+        <v>1402.181818181818</v>
       </c>
     </row>
     <row r="29">
@@ -1959,52 +1959,52 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="13" t="inlineStr">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>CHEPAUK-THIRUVALLIKENI</t>
         </is>
       </c>
-      <c r="B30" s="14" t="n">
+      <c r="B30" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="C30" s="14" t="inlineStr">
+      <c r="C30" s="6" t="inlineStr">
         <is>
           <t>UDHAYANIDHI STALIN</t>
         </is>
       </c>
-      <c r="D30" s="14" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E30" s="14" t="inlineStr">
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
         <is>
           <t>SELVAM. D</t>
         </is>
       </c>
-      <c r="F30" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G30" s="15" t="n">
-        <v>1365</v>
-      </c>
-      <c r="H30" s="14" t="inlineStr">
-        <is>
-          <t>10/17</t>
-        </is>
-      </c>
-      <c r="I30" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J30" s="15" t="n">
-        <v>2320</v>
-      </c>
-      <c r="K30" s="16" t="n">
-        <v>136.5</v>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G30" s="7" t="n">
+        <v>4103</v>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>11/17</t>
+        </is>
+      </c>
+      <c r="I30" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J30" s="7" t="n">
+        <v>6341</v>
+      </c>
+      <c r="K30" s="8" t="n">
+        <v>373</v>
       </c>
     </row>
     <row r="31">
@@ -2037,11 +2037,11 @@
         </is>
       </c>
       <c r="G31" s="4" t="n">
-        <v>19638</v>
+        <v>19848</v>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>22/24</t>
+          <t>23/24</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -2050,10 +2050,10 @@
         </is>
       </c>
       <c r="J31" s="4" t="n">
-        <v>21423</v>
+        <v>20711</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>892.6363636363636</v>
+        <v>862.9565217391304</v>
       </c>
     </row>
     <row r="32">
@@ -2086,11 +2086,11 @@
         </is>
       </c>
       <c r="G32" s="7" t="n">
-        <v>2562</v>
+        <v>3193</v>
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>17/21</t>
+          <t>18/21</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
@@ -2099,10 +2099,10 @@
         </is>
       </c>
       <c r="J32" s="7" t="n">
-        <v>3165</v>
+        <v>3725</v>
       </c>
       <c r="K32" s="8" t="n">
-        <v>150.7058823529412</v>
+        <v>177.3888888888889</v>
       </c>
     </row>
     <row r="33">
@@ -2135,11 +2135,11 @@
         </is>
       </c>
       <c r="G33" s="7" t="n">
-        <v>3727</v>
+        <v>4154</v>
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>12/22</t>
+          <t>13/22</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
@@ -2148,10 +2148,10 @@
         </is>
       </c>
       <c r="J33" s="7" t="n">
-        <v>6833</v>
+        <v>7030</v>
       </c>
       <c r="K33" s="8" t="n">
-        <v>310.5833333333333</v>
+        <v>319.5384615384615</v>
       </c>
     </row>
     <row r="34">
@@ -2331,11 +2331,11 @@
         </is>
       </c>
       <c r="G37" s="4" t="n">
-        <v>7322</v>
+        <v>8099</v>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>17/18</t>
+          <t>18/18</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
@@ -2344,10 +2344,10 @@
         </is>
       </c>
       <c r="J37" s="4" t="n">
-        <v>7753</v>
+        <v>8099</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>430.7058823529412</v>
+        <v>449.9444444444445</v>
       </c>
     </row>
     <row r="38">
@@ -2380,11 +2380,11 @@
         </is>
       </c>
       <c r="G38" s="7" t="n">
-        <v>3182</v>
+        <v>5903</v>
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>10/19</t>
+          <t>11/19</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr">
@@ -2393,10 +2393,10 @@
         </is>
       </c>
       <c r="J38" s="7" t="n">
-        <v>6046</v>
+        <v>10196</v>
       </c>
       <c r="K38" s="8" t="n">
-        <v>318.2</v>
+        <v>536.6363636363636</v>
       </c>
     </row>
     <row r="39">
@@ -2429,11 +2429,11 @@
         </is>
       </c>
       <c r="G39" s="7" t="n">
-        <v>3918</v>
+        <v>3369</v>
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>9/25</t>
+          <t>10/25</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr">
@@ -2442,10 +2442,10 @@
         </is>
       </c>
       <c r="J39" s="7" t="n">
-        <v>10883</v>
+        <v>8422</v>
       </c>
       <c r="K39" s="8" t="n">
-        <v>435.3333333333333</v>
+        <v>336.9</v>
       </c>
     </row>
     <row r="40">
@@ -2498,101 +2498,101 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="6" t="inlineStr">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>DHARMAPURI</t>
         </is>
       </c>
-      <c r="B41" s="6" t="n">
+      <c r="B41" s="3" t="n">
         <v>59</v>
       </c>
-      <c r="C41" s="6" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr">
         <is>
           <t>SOWMIYA ANBUMANI</t>
         </is>
       </c>
-      <c r="D41" s="6" t="inlineStr">
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>Pattali Makkal Katchi</t>
         </is>
       </c>
-      <c r="E41" s="6" t="inlineStr">
+      <c r="E41" s="3" t="inlineStr">
         <is>
           <t>SIVAN. M.</t>
         </is>
       </c>
-      <c r="F41" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G41" s="7" t="n">
-        <v>10961</v>
-      </c>
-      <c r="H41" s="6" t="inlineStr">
-        <is>
-          <t>17/23</t>
-        </is>
-      </c>
-      <c r="I41" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J41" s="7" t="n">
-        <v>14830</v>
-      </c>
-      <c r="K41" s="8" t="n">
-        <v>644.7647058823529</v>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="n">
+        <v>12893</v>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>18/23</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J41" s="4" t="n">
+        <v>16474</v>
+      </c>
+      <c r="K41" s="5" t="n">
+        <v>716.2777777777778</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="6" t="inlineStr">
+      <c r="A42" s="13" t="inlineStr">
         <is>
           <t>DINDIGUL</t>
         </is>
       </c>
-      <c r="B42" s="6" t="n">
+      <c r="B42" s="14" t="n">
         <v>132</v>
       </c>
-      <c r="C42" s="6" t="inlineStr">
+      <c r="C42" s="14" t="inlineStr">
         <is>
           <t>SENTHILKUMAR. I.P</t>
         </is>
       </c>
-      <c r="D42" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E42" s="6" t="inlineStr">
+      <c r="D42" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E42" s="14" t="inlineStr">
         <is>
           <t>NAZEER RAJA. G</t>
         </is>
       </c>
-      <c r="F42" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G42" s="7" t="n">
-        <v>2199</v>
-      </c>
-      <c r="H42" s="6" t="inlineStr">
-        <is>
-          <t>16/24</t>
-        </is>
-      </c>
-      <c r="I42" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J42" s="7" t="n">
-        <v>3298</v>
-      </c>
-      <c r="K42" s="8" t="n">
-        <v>137.4375</v>
+      <c r="F42" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G42" s="15" t="n">
+        <v>1079</v>
+      </c>
+      <c r="H42" s="14" t="inlineStr">
+        <is>
+          <t>17/24</t>
+        </is>
+      </c>
+      <c r="I42" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J42" s="15" t="n">
+        <v>1523</v>
+      </c>
+      <c r="K42" s="16" t="n">
+        <v>63.47058823529412</v>
       </c>
     </row>
     <row r="43">
@@ -2674,11 +2674,11 @@
         </is>
       </c>
       <c r="G44" s="4" t="n">
-        <v>65656</v>
+        <v>69697</v>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>17/25</t>
+          <t>18/25</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
@@ -2687,59 +2687,59 @@
         </is>
       </c>
       <c r="J44" s="4" t="n">
-        <v>96553</v>
+        <v>96801</v>
       </c>
       <c r="K44" s="5" t="n">
-        <v>3862.117647058823</v>
+        <v>3872.055555555556</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="6" t="inlineStr">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>EGMORE</t>
         </is>
       </c>
-      <c r="B45" s="6" t="n">
+      <c r="B45" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="C45" s="6" t="inlineStr">
+      <c r="C45" s="3" t="inlineStr">
         <is>
           <t>RAJMOHAN</t>
         </is>
       </c>
-      <c r="D45" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E45" s="6" t="inlineStr">
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
         <is>
           <t>TAMILAN PRASANNA</t>
         </is>
       </c>
-      <c r="F45" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G45" s="7" t="n">
-        <v>11400</v>
-      </c>
-      <c r="H45" s="6" t="inlineStr">
-        <is>
-          <t>11/15</t>
-        </is>
-      </c>
-      <c r="I45" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J45" s="7" t="n">
-        <v>15545</v>
-      </c>
-      <c r="K45" s="8" t="n">
-        <v>1036.363636363636</v>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="n">
+        <v>12407</v>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>12/15</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J45" s="4" t="n">
+        <v>15509</v>
+      </c>
+      <c r="K45" s="5" t="n">
+        <v>1033.916666666667</v>
       </c>
     </row>
     <row r="46">
@@ -2772,11 +2772,11 @@
         </is>
       </c>
       <c r="G46" s="4" t="n">
-        <v>19455</v>
+        <v>20100</v>
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>14/19</t>
+          <t>15/19</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
@@ -2785,10 +2785,10 @@
         </is>
       </c>
       <c r="J46" s="4" t="n">
-        <v>26403</v>
+        <v>25460</v>
       </c>
       <c r="K46" s="5" t="n">
-        <v>1389.642857142857</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="47">
@@ -2919,11 +2919,11 @@
         </is>
       </c>
       <c r="G49" s="4" t="n">
-        <v>10693</v>
+        <v>11363</v>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>10/20</t>
+          <t>11/20</t>
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr">
@@ -2932,10 +2932,10 @@
         </is>
       </c>
       <c r="J49" s="4" t="n">
-        <v>21386</v>
+        <v>20660</v>
       </c>
       <c r="K49" s="5" t="n">
-        <v>1069.3</v>
+        <v>1033</v>
       </c>
     </row>
     <row r="50">
@@ -3115,11 +3115,11 @@
         </is>
       </c>
       <c r="G53" s="7" t="n">
-        <v>2419</v>
+        <v>3341</v>
       </c>
       <c r="H53" s="6" t="inlineStr">
         <is>
-          <t>12/23</t>
+          <t>13/23</t>
         </is>
       </c>
       <c r="I53" s="6" t="inlineStr">
@@ -3128,10 +3128,10 @@
         </is>
       </c>
       <c r="J53" s="7" t="n">
-        <v>4636</v>
+        <v>5911</v>
       </c>
       <c r="K53" s="8" t="n">
-        <v>201.5833333333333</v>
+        <v>257.0000000000001</v>
       </c>
     </row>
     <row r="54">
@@ -3164,11 +3164,11 @@
         </is>
       </c>
       <c r="G54" s="4" t="n">
-        <v>14322</v>
+        <v>15549</v>
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>12/25</t>
+          <t>13/25</t>
         </is>
       </c>
       <c r="I54" s="3" t="inlineStr">
@@ -3177,10 +3177,10 @@
         </is>
       </c>
       <c r="J54" s="4" t="n">
-        <v>29838</v>
+        <v>29902</v>
       </c>
       <c r="K54" s="5" t="n">
-        <v>1193.5</v>
+        <v>1196.076923076923</v>
       </c>
     </row>
     <row r="55">
@@ -3311,11 +3311,11 @@
         </is>
       </c>
       <c r="G57" s="4" t="n">
-        <v>25090</v>
+        <v>24891</v>
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>14/34</t>
+          <t>15/34</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr">
@@ -3324,10 +3324,10 @@
         </is>
       </c>
       <c r="J57" s="4" t="n">
-        <v>60933</v>
+        <v>56420</v>
       </c>
       <c r="K57" s="5" t="n">
-        <v>1792.142857142857</v>
+        <v>1659.4</v>
       </c>
     </row>
     <row r="58">
@@ -3556,11 +3556,11 @@
         </is>
       </c>
       <c r="G62" s="7" t="n">
-        <v>2873</v>
+        <v>3278</v>
       </c>
       <c r="H62" s="6" t="inlineStr">
         <is>
-          <t>10/27</t>
+          <t>11/27</t>
         </is>
       </c>
       <c r="I62" s="6" t="inlineStr">
@@ -3569,10 +3569,10 @@
         </is>
       </c>
       <c r="J62" s="7" t="n">
-        <v>7757</v>
+        <v>8046</v>
       </c>
       <c r="K62" s="8" t="n">
-        <v>287.3</v>
+        <v>298</v>
       </c>
     </row>
     <row r="63">
@@ -3752,11 +3752,11 @@
         </is>
       </c>
       <c r="G66" s="4" t="n">
-        <v>19730</v>
+        <v>21854</v>
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>11/28</t>
+          <t>12/28</t>
         </is>
       </c>
       <c r="I66" s="3" t="inlineStr">
@@ -3765,10 +3765,10 @@
         </is>
       </c>
       <c r="J66" s="4" t="n">
-        <v>50222</v>
+        <v>50993</v>
       </c>
       <c r="K66" s="5" t="n">
-        <v>1793.636363636364</v>
+        <v>1821.166666666667</v>
       </c>
     </row>
     <row r="67">
@@ -3870,52 +3870,52 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="6" t="inlineStr">
+      <c r="A69" s="2" t="inlineStr">
         <is>
           <t>KATTUMANNARKOIL</t>
         </is>
       </c>
-      <c r="B69" s="6" t="n">
+      <c r="B69" s="3" t="n">
         <v>159</v>
       </c>
-      <c r="C69" s="6" t="inlineStr">
+      <c r="C69" s="3" t="inlineStr">
         <is>
           <t>L.E. JOTHIMANI</t>
         </is>
       </c>
-      <c r="D69" s="6" t="inlineStr">
+      <c r="D69" s="3" t="inlineStr">
         <is>
           <t>Viduthalai Chiruthaigal Katchi</t>
         </is>
       </c>
-      <c r="E69" s="6" t="inlineStr">
+      <c r="E69" s="3" t="inlineStr">
         <is>
           <t>A. SOZHAN</t>
         </is>
       </c>
-      <c r="F69" s="6" t="inlineStr">
+      <c r="F69" s="3" t="inlineStr">
         <is>
           <t>Pattali Makkal Katchi</t>
         </is>
       </c>
-      <c r="G69" s="7" t="n">
-        <v>9498</v>
-      </c>
-      <c r="H69" s="6" t="inlineStr">
-        <is>
-          <t>10/21</t>
-        </is>
-      </c>
-      <c r="I69" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J69" s="7" t="n">
-        <v>19946</v>
-      </c>
-      <c r="K69" s="8" t="n">
-        <v>949.8</v>
+      <c r="G69" s="4" t="n">
+        <v>14055</v>
+      </c>
+      <c r="H69" s="3" t="inlineStr">
+        <is>
+          <t>11/21</t>
+        </is>
+      </c>
+      <c r="I69" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J69" s="4" t="n">
+        <v>26832</v>
+      </c>
+      <c r="K69" s="5" t="n">
+        <v>1277.727272727273</v>
       </c>
     </row>
     <row r="70">
@@ -3948,11 +3948,11 @@
         </is>
       </c>
       <c r="G70" s="4" t="n">
-        <v>32853</v>
+        <v>35308</v>
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>21/28</t>
+          <t>22/28</t>
         </is>
       </c>
       <c r="I70" s="3" t="inlineStr">
@@ -3961,59 +3961,59 @@
         </is>
       </c>
       <c r="J70" s="4" t="n">
-        <v>43804</v>
+        <v>44937</v>
       </c>
       <c r="K70" s="5" t="n">
-        <v>1564.428571428571</v>
+        <v>1604.909090909091</v>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="6" t="inlineStr">
+      <c r="A71" s="9" t="inlineStr">
         <is>
           <t>KILLIYOOR</t>
         </is>
       </c>
-      <c r="B71" s="6" t="n">
+      <c r="B71" s="10" t="n">
         <v>234</v>
       </c>
-      <c r="C71" s="6" t="inlineStr">
+      <c r="C71" s="10" t="inlineStr">
         <is>
           <t>SABIN. S</t>
         </is>
       </c>
-      <c r="D71" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E71" s="6" t="inlineStr">
+      <c r="D71" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E71" s="10" t="inlineStr">
         <is>
           <t>RAJESH KUMAR. S</t>
         </is>
       </c>
-      <c r="F71" s="6" t="inlineStr">
+      <c r="F71" s="10" t="inlineStr">
         <is>
           <t>Indian National Congress</t>
         </is>
       </c>
-      <c r="G71" s="7" t="n">
-        <v>1794</v>
-      </c>
-      <c r="H71" s="6" t="inlineStr">
-        <is>
-          <t>12/22</t>
-        </is>
-      </c>
-      <c r="I71" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J71" s="7" t="n">
-        <v>3289</v>
-      </c>
-      <c r="K71" s="8" t="n">
-        <v>149.5</v>
+      <c r="G71" s="11" t="n">
+        <v>151</v>
+      </c>
+      <c r="H71" s="10" t="inlineStr">
+        <is>
+          <t>13/22</t>
+        </is>
+      </c>
+      <c r="I71" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J71" s="11" t="n">
+        <v>256</v>
+      </c>
+      <c r="K71" s="12" t="n">
+        <v>11.61538461538461</v>
       </c>
     </row>
     <row r="72">
@@ -4046,11 +4046,11 @@
         </is>
       </c>
       <c r="G72" s="4" t="n">
-        <v>26000</v>
+        <v>28935</v>
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>14/22</t>
+          <t>16/22</t>
         </is>
       </c>
       <c r="I72" s="3" t="inlineStr">
@@ -4059,10 +4059,10 @@
         </is>
       </c>
       <c r="J72" s="4" t="n">
-        <v>40857</v>
+        <v>39786</v>
       </c>
       <c r="K72" s="5" t="n">
-        <v>1857.142857142857</v>
+        <v>1808.4375</v>
       </c>
     </row>
     <row r="73">
@@ -4193,11 +4193,11 @@
         </is>
       </c>
       <c r="G75" s="4" t="n">
-        <v>11498</v>
+        <v>11677</v>
       </c>
       <c r="H75" s="3" t="inlineStr">
         <is>
-          <t>22/28</t>
+          <t>23/28</t>
         </is>
       </c>
       <c r="I75" s="3" t="inlineStr">
@@ -4206,10 +4206,10 @@
         </is>
       </c>
       <c r="J75" s="4" t="n">
-        <v>14634</v>
+        <v>14215</v>
       </c>
       <c r="K75" s="5" t="n">
-        <v>522.6363636363636</v>
+        <v>507.6956521739131</v>
       </c>
     </row>
     <row r="76">
@@ -4242,11 +4242,11 @@
         </is>
       </c>
       <c r="G76" s="7" t="n">
-        <v>7738</v>
+        <v>7074</v>
       </c>
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>14/22</t>
+          <t>15/22</t>
         </is>
       </c>
       <c r="I76" s="6" t="inlineStr">
@@ -4255,10 +4255,10 @@
         </is>
       </c>
       <c r="J76" s="7" t="n">
-        <v>12160</v>
+        <v>10375</v>
       </c>
       <c r="K76" s="8" t="n">
-        <v>552.7142857142857</v>
+        <v>471.6000000000001</v>
       </c>
     </row>
     <row r="77">
@@ -4291,11 +4291,11 @@
         </is>
       </c>
       <c r="G77" s="7" t="n">
-        <v>1728</v>
+        <v>3150</v>
       </c>
       <c r="H77" s="6" t="inlineStr">
         <is>
-          <t>11/23</t>
+          <t>12/23</t>
         </is>
       </c>
       <c r="I77" s="6" t="inlineStr">
@@ -4304,10 +4304,10 @@
         </is>
       </c>
       <c r="J77" s="7" t="n">
-        <v>3613</v>
+        <v>6038</v>
       </c>
       <c r="K77" s="8" t="n">
-        <v>157.0909090909091</v>
+        <v>262.5</v>
       </c>
     </row>
     <row r="78">
@@ -4389,11 +4389,11 @@
         </is>
       </c>
       <c r="G79" s="7" t="n">
-        <v>2980</v>
+        <v>2630</v>
       </c>
       <c r="H79" s="6" t="inlineStr">
         <is>
-          <t>10/20</t>
+          <t>11/20</t>
         </is>
       </c>
       <c r="I79" s="6" t="inlineStr">
@@ -4402,10 +4402,10 @@
         </is>
       </c>
       <c r="J79" s="7" t="n">
-        <v>5960</v>
+        <v>4782</v>
       </c>
       <c r="K79" s="8" t="n">
-        <v>298</v>
+        <v>239.0909090909091</v>
       </c>
     </row>
     <row r="80">
@@ -4438,11 +4438,11 @@
         </is>
       </c>
       <c r="G80" s="15" t="n">
-        <v>1446</v>
+        <v>1825</v>
       </c>
       <c r="H80" s="14" t="inlineStr">
         <is>
-          <t>12/21</t>
+          <t>13/21</t>
         </is>
       </c>
       <c r="I80" s="14" t="inlineStr">
@@ -4451,10 +4451,10 @@
         </is>
       </c>
       <c r="J80" s="15" t="n">
-        <v>2530</v>
+        <v>2948</v>
       </c>
       <c r="K80" s="16" t="n">
-        <v>120.5</v>
+        <v>140.3846153846154</v>
       </c>
     </row>
     <row r="81">
@@ -4585,11 +4585,11 @@
         </is>
       </c>
       <c r="G83" s="4" t="n">
-        <v>13820</v>
+        <v>14886</v>
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
-          <t>14/25</t>
+          <t>15/25</t>
         </is>
       </c>
       <c r="I83" s="3" t="inlineStr">
@@ -4598,10 +4598,10 @@
         </is>
       </c>
       <c r="J83" s="4" t="n">
-        <v>24679</v>
+        <v>24810</v>
       </c>
       <c r="K83" s="5" t="n">
-        <v>987.142857142857</v>
+        <v>992.4</v>
       </c>
     </row>
     <row r="84">
@@ -4683,11 +4683,11 @@
         </is>
       </c>
       <c r="G85" s="15" t="n">
-        <v>1663</v>
+        <v>974</v>
       </c>
       <c r="H85" s="14" t="inlineStr">
         <is>
-          <t>12/20</t>
+          <t>13/20</t>
         </is>
       </c>
       <c r="I85" s="14" t="inlineStr">
@@ -4696,10 +4696,10 @@
         </is>
       </c>
       <c r="J85" s="15" t="n">
-        <v>2772</v>
+        <v>1498</v>
       </c>
       <c r="K85" s="16" t="n">
-        <v>138.5833333333333</v>
+        <v>74.92307692307692</v>
       </c>
     </row>
     <row r="86">
@@ -4830,11 +4830,11 @@
         </is>
       </c>
       <c r="G88" s="4" t="n">
-        <v>15631</v>
+        <v>16020</v>
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>9/19</t>
+          <t>10/19</t>
         </is>
       </c>
       <c r="I88" s="3" t="inlineStr">
@@ -4843,10 +4843,10 @@
         </is>
       </c>
       <c r="J88" s="4" t="n">
-        <v>32999</v>
+        <v>30438</v>
       </c>
       <c r="K88" s="5" t="n">
-        <v>1736.777777777778</v>
+        <v>1602</v>
       </c>
     </row>
     <row r="89">
@@ -4879,11 +4879,11 @@
         </is>
       </c>
       <c r="G89" s="7" t="n">
-        <v>5981</v>
+        <v>6673</v>
       </c>
       <c r="H89" s="6" t="inlineStr">
         <is>
-          <t>17/29</t>
+          <t>18/29</t>
         </is>
       </c>
       <c r="I89" s="6" t="inlineStr">
@@ -4892,10 +4892,10 @@
         </is>
       </c>
       <c r="J89" s="7" t="n">
-        <v>10203</v>
+        <v>10751</v>
       </c>
       <c r="K89" s="8" t="n">
-        <v>351.8235294117647</v>
+        <v>370.7222222222222</v>
       </c>
     </row>
     <row r="90">
@@ -4977,7 +4977,7 @@
         </is>
       </c>
       <c r="G91" s="4" t="n">
-        <v>18354</v>
+        <v>18321</v>
       </c>
       <c r="H91" s="3" t="inlineStr">
         <is>
@@ -4990,10 +4990,10 @@
         </is>
       </c>
       <c r="J91" s="4" t="n">
-        <v>20801</v>
+        <v>20764</v>
       </c>
       <c r="K91" s="5" t="n">
-        <v>1223.6</v>
+        <v>1221.4</v>
       </c>
     </row>
     <row r="92">
@@ -5075,11 +5075,11 @@
         </is>
       </c>
       <c r="G93" s="7" t="n">
-        <v>2208</v>
+        <v>3574</v>
       </c>
       <c r="H93" s="6" t="inlineStr">
         <is>
-          <t>12/21</t>
+          <t>13/21</t>
         </is>
       </c>
       <c r="I93" s="6" t="inlineStr">
@@ -5088,10 +5088,10 @@
         </is>
       </c>
       <c r="J93" s="7" t="n">
-        <v>3864</v>
+        <v>5773</v>
       </c>
       <c r="K93" s="8" t="n">
-        <v>184</v>
+        <v>274.9230769230769</v>
       </c>
     </row>
     <row r="94">
@@ -5222,11 +5222,11 @@
         </is>
       </c>
       <c r="G96" s="4" t="n">
-        <v>9620</v>
+        <v>9716</v>
       </c>
       <c r="H96" s="3" t="inlineStr">
         <is>
-          <t>17/22</t>
+          <t>18/22</t>
         </is>
       </c>
       <c r="I96" s="3" t="inlineStr">
@@ -5235,10 +5235,10 @@
         </is>
       </c>
       <c r="J96" s="4" t="n">
-        <v>12449</v>
+        <v>11875</v>
       </c>
       <c r="K96" s="5" t="n">
-        <v>565.8823529411765</v>
+        <v>539.7777777777778</v>
       </c>
     </row>
     <row r="97">
@@ -5291,52 +5291,52 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="13" t="inlineStr">
+      <c r="A98" s="9" t="inlineStr">
         <is>
           <t>MANAPPARAI</t>
         </is>
       </c>
-      <c r="B98" s="14" t="n">
+      <c r="B98" s="10" t="n">
         <v>138</v>
       </c>
-      <c r="C98" s="14" t="inlineStr">
+      <c r="C98" s="10" t="inlineStr">
         <is>
           <t>R. KATHIRAVAN</t>
         </is>
       </c>
-      <c r="D98" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E98" s="14" t="inlineStr">
+      <c r="D98" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E98" s="10" t="inlineStr">
         <is>
           <t>DR. PL. VIJAYAKUMAR</t>
         </is>
       </c>
-      <c r="F98" s="14" t="inlineStr">
+      <c r="F98" s="10" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G98" s="15" t="n">
-        <v>1625</v>
-      </c>
-      <c r="H98" s="14" t="inlineStr">
-        <is>
-          <t>17/25</t>
-        </is>
-      </c>
-      <c r="I98" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J98" s="15" t="n">
-        <v>2390</v>
-      </c>
-      <c r="K98" s="16" t="n">
-        <v>95.58823529411765</v>
+      <c r="G98" s="11" t="n">
+        <v>157</v>
+      </c>
+      <c r="H98" s="10" t="inlineStr">
+        <is>
+          <t>18/25</t>
+        </is>
+      </c>
+      <c r="I98" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J98" s="11" t="n">
+        <v>218</v>
+      </c>
+      <c r="K98" s="12" t="n">
+        <v>8.722222222222221</v>
       </c>
     </row>
     <row r="99">
@@ -5369,11 +5369,11 @@
         </is>
       </c>
       <c r="G99" s="7" t="n">
-        <v>2252</v>
+        <v>2179</v>
       </c>
       <c r="H99" s="6" t="inlineStr">
         <is>
-          <t>14/22</t>
+          <t>15/22</t>
         </is>
       </c>
       <c r="I99" s="6" t="inlineStr">
@@ -5382,10 +5382,10 @@
         </is>
       </c>
       <c r="J99" s="7" t="n">
-        <v>3539</v>
+        <v>3196</v>
       </c>
       <c r="K99" s="8" t="n">
-        <v>160.8571428571429</v>
+        <v>145.2666666666667</v>
       </c>
     </row>
     <row r="100">
@@ -5418,11 +5418,11 @@
         </is>
       </c>
       <c r="G100" s="7" t="n">
-        <v>5802</v>
+        <v>6762</v>
       </c>
       <c r="H100" s="6" t="inlineStr">
         <is>
-          <t>11/22</t>
+          <t>12/22</t>
         </is>
       </c>
       <c r="I100" s="6" t="inlineStr">
@@ -5431,10 +5431,10 @@
         </is>
       </c>
       <c r="J100" s="7" t="n">
-        <v>11604</v>
+        <v>12397</v>
       </c>
       <c r="K100" s="8" t="n">
-        <v>527.4545454545455</v>
+        <v>563.5</v>
       </c>
     </row>
     <row r="101">
@@ -5712,11 +5712,11 @@
         </is>
       </c>
       <c r="G106" s="4" t="n">
-        <v>14115</v>
+        <v>14938</v>
       </c>
       <c r="H106" s="3" t="inlineStr">
         <is>
-          <t>16/21</t>
+          <t>17/21</t>
         </is>
       </c>
       <c r="I106" s="3" t="inlineStr">
@@ -5725,10 +5725,10 @@
         </is>
       </c>
       <c r="J106" s="4" t="n">
-        <v>18526</v>
+        <v>18453</v>
       </c>
       <c r="K106" s="5" t="n">
-        <v>882.1875</v>
+        <v>878.7058823529412</v>
       </c>
     </row>
     <row r="107">
@@ -5761,11 +5761,11 @@
         </is>
       </c>
       <c r="G107" s="4" t="n">
-        <v>22514</v>
+        <v>23844</v>
       </c>
       <c r="H107" s="3" t="inlineStr">
         <is>
-          <t>15/20</t>
+          <t>16/20</t>
         </is>
       </c>
       <c r="I107" s="3" t="inlineStr">
@@ -5774,10 +5774,10 @@
         </is>
       </c>
       <c r="J107" s="4" t="n">
-        <v>30019</v>
+        <v>29805</v>
       </c>
       <c r="K107" s="5" t="n">
-        <v>1500.933333333333</v>
+        <v>1490.25</v>
       </c>
     </row>
     <row r="108">
@@ -5810,11 +5810,11 @@
         </is>
       </c>
       <c r="G108" s="7" t="n">
-        <v>5945</v>
+        <v>5690</v>
       </c>
       <c r="H108" s="6" t="inlineStr">
         <is>
-          <t>6/18</t>
+          <t>7/18</t>
         </is>
       </c>
       <c r="I108" s="6" t="inlineStr">
@@ -5823,10 +5823,10 @@
         </is>
       </c>
       <c r="J108" s="7" t="n">
-        <v>17835</v>
+        <v>14631</v>
       </c>
       <c r="K108" s="8" t="n">
-        <v>990.8333333333334</v>
+        <v>812.8571428571429</v>
       </c>
     </row>
     <row r="109">
@@ -5859,11 +5859,11 @@
         </is>
       </c>
       <c r="G109" s="7" t="n">
-        <v>2285</v>
+        <v>2675</v>
       </c>
       <c r="H109" s="6" t="inlineStr">
         <is>
-          <t>13/23</t>
+          <t>15/23</t>
         </is>
       </c>
       <c r="I109" s="6" t="inlineStr">
@@ -5872,10 +5872,10 @@
         </is>
       </c>
       <c r="J109" s="7" t="n">
-        <v>4043</v>
+        <v>4102</v>
       </c>
       <c r="K109" s="8" t="n">
-        <v>175.7692307692308</v>
+        <v>178.3333333333333</v>
       </c>
     </row>
     <row r="110">
@@ -5957,11 +5957,11 @@
         </is>
       </c>
       <c r="G111" s="4" t="n">
-        <v>11502</v>
+        <v>13190</v>
       </c>
       <c r="H111" s="3" t="inlineStr">
         <is>
-          <t>21/25</t>
+          <t>22/25</t>
         </is>
       </c>
       <c r="I111" s="3" t="inlineStr">
@@ -5970,10 +5970,10 @@
         </is>
       </c>
       <c r="J111" s="4" t="n">
-        <v>13693</v>
+        <v>14989</v>
       </c>
       <c r="K111" s="5" t="n">
-        <v>547.7142857142857</v>
+        <v>599.5454545454545</v>
       </c>
     </row>
     <row r="112">
@@ -6006,11 +6006,11 @@
         </is>
       </c>
       <c r="G112" s="4" t="n">
-        <v>27455</v>
+        <v>28836</v>
       </c>
       <c r="H112" s="3" t="inlineStr">
         <is>
-          <t>16/25</t>
+          <t>17/25</t>
         </is>
       </c>
       <c r="I112" s="3" t="inlineStr">
@@ -6019,10 +6019,10 @@
         </is>
       </c>
       <c r="J112" s="4" t="n">
-        <v>42898</v>
+        <v>42406</v>
       </c>
       <c r="K112" s="5" t="n">
-        <v>1715.9375</v>
+        <v>1696.235294117647</v>
       </c>
     </row>
     <row r="113">
@@ -6075,52 +6075,52 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="6" t="inlineStr">
+      <c r="A114" s="2" t="inlineStr">
         <is>
           <t>NEYVELI</t>
         </is>
       </c>
-      <c r="B114" s="6" t="n">
+      <c r="B114" s="3" t="n">
         <v>153</v>
       </c>
-      <c r="C114" s="6" t="inlineStr">
+      <c r="C114" s="3" t="inlineStr">
         <is>
           <t>RAJENDRAN.R</t>
         </is>
       </c>
-      <c r="D114" s="6" t="inlineStr">
+      <c r="D114" s="3" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E114" s="6" t="inlineStr">
+      <c r="E114" s="3" t="inlineStr">
         <is>
           <t>SABA.RAJENDRAN</t>
         </is>
       </c>
-      <c r="F114" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G114" s="7" t="n">
-        <v>11972</v>
-      </c>
-      <c r="H114" s="6" t="inlineStr">
-        <is>
-          <t>14/19</t>
-        </is>
-      </c>
-      <c r="I114" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J114" s="7" t="n">
-        <v>16248</v>
-      </c>
-      <c r="K114" s="8" t="n">
-        <v>855.1428571428571</v>
+      <c r="F114" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G114" s="4" t="n">
+        <v>11169</v>
+      </c>
+      <c r="H114" s="3" t="inlineStr">
+        <is>
+          <t>15/19</t>
+        </is>
+      </c>
+      <c r="I114" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J114" s="4" t="n">
+        <v>14147</v>
+      </c>
+      <c r="K114" s="5" t="n">
+        <v>744.6</v>
       </c>
     </row>
     <row r="115">
@@ -6251,11 +6251,11 @@
         </is>
       </c>
       <c r="G117" s="7" t="n">
-        <v>4546</v>
+        <v>5074</v>
       </c>
       <c r="H117" s="6" t="inlineStr">
         <is>
-          <t>14/26</t>
+          <t>15/26</t>
         </is>
       </c>
       <c r="I117" s="6" t="inlineStr">
@@ -6264,10 +6264,10 @@
         </is>
       </c>
       <c r="J117" s="7" t="n">
-        <v>8443</v>
+        <v>8795</v>
       </c>
       <c r="K117" s="8" t="n">
-        <v>324.7142857142857</v>
+        <v>338.2666666666667</v>
       </c>
     </row>
     <row r="118">
@@ -6349,11 +6349,11 @@
         </is>
       </c>
       <c r="G119" s="4" t="n">
-        <v>20331</v>
+        <v>21980</v>
       </c>
       <c r="H119" s="3" t="inlineStr">
         <is>
-          <t>13/23</t>
+          <t>14/23</t>
         </is>
       </c>
       <c r="I119" s="3" t="inlineStr">
@@ -6362,10 +6362,10 @@
         </is>
       </c>
       <c r="J119" s="4" t="n">
-        <v>35970</v>
+        <v>36110</v>
       </c>
       <c r="K119" s="5" t="n">
-        <v>1563.923076923077</v>
+        <v>1570</v>
       </c>
     </row>
     <row r="120">
@@ -6447,11 +6447,11 @@
         </is>
       </c>
       <c r="G121" s="4" t="n">
-        <v>24982</v>
+        <v>27492</v>
       </c>
       <c r="H121" s="3" t="inlineStr">
         <is>
-          <t>16/23</t>
+          <t>17/23</t>
         </is>
       </c>
       <c r="I121" s="3" t="inlineStr">
@@ -6460,10 +6460,10 @@
         </is>
       </c>
       <c r="J121" s="4" t="n">
-        <v>35912</v>
+        <v>37195</v>
       </c>
       <c r="K121" s="5" t="n">
-        <v>1561.375</v>
+        <v>1617.176470588235</v>
       </c>
     </row>
     <row r="122">
@@ -6594,11 +6594,11 @@
         </is>
       </c>
       <c r="G124" s="4" t="n">
-        <v>19049</v>
+        <v>21640</v>
       </c>
       <c r="H124" s="3" t="inlineStr">
         <is>
-          <t>18/35</t>
+          <t>19/35</t>
         </is>
       </c>
       <c r="I124" s="3" t="inlineStr">
@@ -6607,10 +6607,10 @@
         </is>
       </c>
       <c r="J124" s="4" t="n">
-        <v>37040</v>
+        <v>39863</v>
       </c>
       <c r="K124" s="5" t="n">
-        <v>1058.277777777778</v>
+        <v>1138.947368421053</v>
       </c>
     </row>
     <row r="125">
@@ -6643,11 +6643,11 @@
         </is>
       </c>
       <c r="G125" s="4" t="n">
-        <v>22492</v>
+        <v>24691</v>
       </c>
       <c r="H125" s="3" t="inlineStr">
         <is>
-          <t>14/34</t>
+          <t>15/34</t>
         </is>
       </c>
       <c r="I125" s="3" t="inlineStr">
@@ -6656,10 +6656,10 @@
         </is>
       </c>
       <c r="J125" s="4" t="n">
-        <v>54623</v>
+        <v>55966</v>
       </c>
       <c r="K125" s="5" t="n">
-        <v>1606.571428571429</v>
+        <v>1646.066666666667</v>
       </c>
     </row>
     <row r="126">
@@ -6692,11 +6692,11 @@
         </is>
       </c>
       <c r="G126" s="4" t="n">
-        <v>8447</v>
+        <v>10318</v>
       </c>
       <c r="H126" s="3" t="inlineStr">
         <is>
-          <t>19/23</t>
+          <t>20/23</t>
         </is>
       </c>
       <c r="I126" s="3" t="inlineStr">
@@ -6705,10 +6705,10 @@
         </is>
       </c>
       <c r="J126" s="4" t="n">
-        <v>10225</v>
+        <v>11866</v>
       </c>
       <c r="K126" s="5" t="n">
-        <v>444.578947368421</v>
+        <v>515.9</v>
       </c>
     </row>
     <row r="127">
@@ -6790,11 +6790,11 @@
         </is>
       </c>
       <c r="G128" s="4" t="n">
-        <v>36425</v>
+        <v>35875</v>
       </c>
       <c r="H128" s="3" t="inlineStr">
         <is>
-          <t>16/23</t>
+          <t>17/23</t>
         </is>
       </c>
       <c r="I128" s="3" t="inlineStr">
@@ -6803,10 +6803,10 @@
         </is>
       </c>
       <c r="J128" s="4" t="n">
-        <v>52361</v>
+        <v>48537</v>
       </c>
       <c r="K128" s="5" t="n">
-        <v>2276.5625</v>
+        <v>2110.294117647059</v>
       </c>
     </row>
     <row r="129">
@@ -6839,11 +6839,11 @@
         </is>
       </c>
       <c r="G129" s="15" t="n">
-        <v>1155</v>
+        <v>908</v>
       </c>
       <c r="H129" s="14" t="inlineStr">
         <is>
-          <t>16/24</t>
+          <t>17/24</t>
         </is>
       </c>
       <c r="I129" s="14" t="inlineStr">
@@ -6852,10 +6852,10 @@
         </is>
       </c>
       <c r="J129" s="15" t="n">
-        <v>1732</v>
+        <v>1282</v>
       </c>
       <c r="K129" s="16" t="n">
-        <v>72.1875</v>
+        <v>53.41176470588236</v>
       </c>
     </row>
     <row r="130">
@@ -6986,11 +6986,11 @@
         </is>
       </c>
       <c r="G132" s="7" t="n">
-        <v>5801</v>
+        <v>3963</v>
       </c>
       <c r="H132" s="6" t="inlineStr">
         <is>
-          <t>10/23</t>
+          <t>11/23</t>
         </is>
       </c>
       <c r="I132" s="6" t="inlineStr">
@@ -6999,10 +6999,10 @@
         </is>
       </c>
       <c r="J132" s="7" t="n">
-        <v>13342</v>
+        <v>8286</v>
       </c>
       <c r="K132" s="8" t="n">
-        <v>580.1</v>
+        <v>360.2727272727273</v>
       </c>
     </row>
     <row r="133">
@@ -7104,52 +7104,52 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="6" t="inlineStr">
+      <c r="A135" s="13" t="inlineStr">
         <is>
           <t>PERAVURANI</t>
         </is>
       </c>
-      <c r="B135" s="6" t="n">
+      <c r="B135" s="14" t="n">
         <v>177</v>
       </c>
-      <c r="C135" s="6" t="inlineStr">
+      <c r="C135" s="14" t="inlineStr">
         <is>
           <t>GOVI.ELANGO</t>
         </is>
       </c>
-      <c r="D135" s="6" t="inlineStr">
+      <c r="D135" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E135" s="6" t="inlineStr">
+      <c r="E135" s="14" t="inlineStr">
         <is>
           <t>ASHOKKUMAR. N</t>
         </is>
       </c>
-      <c r="F135" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G135" s="7" t="n">
-        <v>1142</v>
-      </c>
-      <c r="H135" s="6" t="inlineStr">
-        <is>
-          <t>5/21</t>
-        </is>
-      </c>
-      <c r="I135" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J135" s="7" t="n">
-        <v>4796</v>
-      </c>
-      <c r="K135" s="8" t="n">
-        <v>228.4</v>
+      <c r="F135" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G135" s="15" t="n">
+        <v>546</v>
+      </c>
+      <c r="H135" s="14" t="inlineStr">
+        <is>
+          <t>6/21</t>
+        </is>
+      </c>
+      <c r="I135" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J135" s="15" t="n">
+        <v>1911</v>
+      </c>
+      <c r="K135" s="16" t="n">
+        <v>91</v>
       </c>
     </row>
     <row r="136">
@@ -7182,11 +7182,11 @@
         </is>
       </c>
       <c r="G136" s="7" t="n">
-        <v>1961</v>
+        <v>3910</v>
       </c>
       <c r="H136" s="6" t="inlineStr">
         <is>
-          <t>12/26</t>
+          <t>13/26</t>
         </is>
       </c>
       <c r="I136" s="6" t="inlineStr">
@@ -7195,10 +7195,10 @@
         </is>
       </c>
       <c r="J136" s="7" t="n">
-        <v>4249</v>
+        <v>7820</v>
       </c>
       <c r="K136" s="8" t="n">
-        <v>163.4166666666667</v>
+        <v>300.7692307692308</v>
       </c>
     </row>
     <row r="137">
@@ -7251,52 +7251,52 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="9" t="inlineStr">
+      <c r="A138" s="13" t="inlineStr">
         <is>
           <t>POLLACHI</t>
         </is>
       </c>
-      <c r="B138" s="10" t="n">
+      <c r="B138" s="14" t="n">
         <v>123</v>
       </c>
-      <c r="C138" s="10" t="inlineStr">
+      <c r="C138" s="14" t="inlineStr">
         <is>
           <t>K. NITHYANANDHAN</t>
         </is>
       </c>
-      <c r="D138" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E138" s="10" t="inlineStr">
+      <c r="D138" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E138" s="14" t="inlineStr">
         <is>
           <t>POLLACHI V. JAYARAMAN</t>
         </is>
       </c>
-      <c r="F138" s="10" t="inlineStr">
+      <c r="F138" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G138" s="11" t="n">
-        <v>232</v>
-      </c>
-      <c r="H138" s="10" t="inlineStr">
-        <is>
-          <t>15/20</t>
-        </is>
-      </c>
-      <c r="I138" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J138" s="11" t="n">
-        <v>309</v>
-      </c>
-      <c r="K138" s="12" t="n">
-        <v>15.46666666666667</v>
+      <c r="G138" s="15" t="n">
+        <v>1326</v>
+      </c>
+      <c r="H138" s="14" t="inlineStr">
+        <is>
+          <t>16/20</t>
+        </is>
+      </c>
+      <c r="I138" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J138" s="15" t="n">
+        <v>1658</v>
+      </c>
+      <c r="K138" s="16" t="n">
+        <v>82.875</v>
       </c>
     </row>
     <row r="139">
@@ -7378,11 +7378,11 @@
         </is>
       </c>
       <c r="G140" s="4" t="n">
-        <v>31617</v>
+        <v>34010</v>
       </c>
       <c r="H140" s="3" t="inlineStr">
         <is>
-          <t>14/24</t>
+          <t>15/24</t>
         </is>
       </c>
       <c r="I140" s="3" t="inlineStr">
@@ -7391,10 +7391,10 @@
         </is>
       </c>
       <c r="J140" s="4" t="n">
-        <v>54201</v>
+        <v>54416</v>
       </c>
       <c r="K140" s="5" t="n">
-        <v>2258.357142857143</v>
+        <v>2267.333333333333</v>
       </c>
     </row>
     <row r="141">
@@ -7476,11 +7476,11 @@
         </is>
       </c>
       <c r="G142" s="4" t="n">
-        <v>49527</v>
+        <v>52284</v>
       </c>
       <c r="H142" s="3" t="inlineStr">
         <is>
-          <t>14/23</t>
+          <t>15/23</t>
         </is>
       </c>
       <c r="I142" s="3" t="inlineStr">
@@ -7489,10 +7489,10 @@
         </is>
       </c>
       <c r="J142" s="4" t="n">
-        <v>81366</v>
+        <v>80169</v>
       </c>
       <c r="K142" s="5" t="n">
-        <v>3537.642857142857</v>
+        <v>3485.6</v>
       </c>
     </row>
     <row r="143">
@@ -7574,11 +7574,11 @@
         </is>
       </c>
       <c r="G144" s="4" t="n">
-        <v>9113</v>
+        <v>10268</v>
       </c>
       <c r="H144" s="3" t="inlineStr">
         <is>
-          <t>21/24</t>
+          <t>22/24</t>
         </is>
       </c>
       <c r="I144" s="3" t="inlineStr">
@@ -7587,10 +7587,10 @@
         </is>
       </c>
       <c r="J144" s="4" t="n">
-        <v>10415</v>
+        <v>11201</v>
       </c>
       <c r="K144" s="5" t="n">
-        <v>433.952380952381</v>
+        <v>466.7272727272727</v>
       </c>
     </row>
     <row r="145">
@@ -7623,11 +7623,11 @@
         </is>
       </c>
       <c r="G145" s="7" t="n">
-        <v>8738</v>
+        <v>9519</v>
       </c>
       <c r="H145" s="6" t="inlineStr">
         <is>
-          <t>13/20</t>
+          <t>14/20</t>
         </is>
       </c>
       <c r="I145" s="6" t="inlineStr">
@@ -7636,59 +7636,59 @@
         </is>
       </c>
       <c r="J145" s="7" t="n">
-        <v>13443</v>
+        <v>13599</v>
       </c>
       <c r="K145" s="8" t="n">
-        <v>672.1538461538462</v>
+        <v>679.9285714285714</v>
       </c>
     </row>
     <row r="146">
-      <c r="A146" s="6" t="inlineStr">
+      <c r="A146" s="2" t="inlineStr">
         <is>
           <t>RAMANATHAPURAM</t>
         </is>
       </c>
-      <c r="B146" s="6" t="n">
+      <c r="B146" s="3" t="n">
         <v>211</v>
       </c>
-      <c r="C146" s="6" t="inlineStr">
+      <c r="C146" s="3" t="inlineStr">
         <is>
           <t>KATHARBATCHA MUTHURAMALINGAM</t>
         </is>
       </c>
-      <c r="D146" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E146" s="6" t="inlineStr">
+      <c r="D146" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E146" s="3" t="inlineStr">
         <is>
           <t>SHAHUL HAMEED</t>
         </is>
       </c>
-      <c r="F146" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G146" s="7" t="n">
-        <v>14255</v>
-      </c>
-      <c r="H146" s="6" t="inlineStr">
-        <is>
-          <t>21/29</t>
-        </is>
-      </c>
-      <c r="I146" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J146" s="7" t="n">
-        <v>19685</v>
-      </c>
-      <c r="K146" s="8" t="n">
-        <v>678.8095238095239</v>
+      <c r="F146" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G146" s="4" t="n">
+        <v>15337</v>
+      </c>
+      <c r="H146" s="3" t="inlineStr">
+        <is>
+          <t>22/29</t>
+        </is>
+      </c>
+      <c r="I146" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J146" s="4" t="n">
+        <v>20217</v>
+      </c>
+      <c r="K146" s="5" t="n">
+        <v>697.1363636363636</v>
       </c>
     </row>
     <row r="147">
@@ -7721,11 +7721,11 @@
         </is>
       </c>
       <c r="G147" s="7" t="n">
-        <v>2983</v>
+        <v>2137</v>
       </c>
       <c r="H147" s="6" t="inlineStr">
         <is>
-          <t>12/22</t>
+          <t>13/22</t>
         </is>
       </c>
       <c r="I147" s="6" t="inlineStr">
@@ -7734,10 +7734,10 @@
         </is>
       </c>
       <c r="J147" s="7" t="n">
-        <v>5469</v>
+        <v>3616</v>
       </c>
       <c r="K147" s="8" t="n">
-        <v>248.5833333333333</v>
+        <v>164.3846153846154</v>
       </c>
     </row>
     <row r="148">
@@ -7770,11 +7770,11 @@
         </is>
       </c>
       <c r="G148" s="7" t="n">
-        <v>10136</v>
+        <v>11430</v>
       </c>
       <c r="H148" s="6" t="inlineStr">
         <is>
-          <t>12/21</t>
+          <t>13/21</t>
         </is>
       </c>
       <c r="I148" s="6" t="inlineStr">
@@ -7783,10 +7783,10 @@
         </is>
       </c>
       <c r="J148" s="7" t="n">
-        <v>17738</v>
+        <v>18464</v>
       </c>
       <c r="K148" s="8" t="n">
-        <v>844.6666666666666</v>
+        <v>879.2307692307693</v>
       </c>
     </row>
     <row r="149">
@@ -7819,11 +7819,11 @@
         </is>
       </c>
       <c r="G149" s="7" t="n">
-        <v>1722</v>
+        <v>2647</v>
       </c>
       <c r="H149" s="6" t="inlineStr">
         <is>
-          <t>9/25</t>
+          <t>10/25</t>
         </is>
       </c>
       <c r="I149" s="6" t="inlineStr">
@@ -7832,59 +7832,59 @@
         </is>
       </c>
       <c r="J149" s="7" t="n">
-        <v>4783</v>
+        <v>6618</v>
       </c>
       <c r="K149" s="8" t="n">
-        <v>191.3333333333333</v>
+        <v>264.7</v>
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="6" t="inlineStr">
+      <c r="A150" s="2" t="inlineStr">
         <is>
           <t>ROYAPURAM</t>
         </is>
       </c>
-      <c r="B150" s="6" t="n">
+      <c r="B150" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="C150" s="6" t="inlineStr">
+      <c r="C150" s="3" t="inlineStr">
         <is>
           <t>K.V. VIJAY DAMU</t>
         </is>
       </c>
-      <c r="D150" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E150" s="6" t="inlineStr">
+      <c r="D150" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E150" s="3" t="inlineStr">
         <is>
           <t>DR. A. SUBAIR KHAN</t>
         </is>
       </c>
-      <c r="F150" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G150" s="7" t="n">
-        <v>13304</v>
-      </c>
-      <c r="H150" s="6" t="inlineStr">
-        <is>
-          <t>10/14</t>
-        </is>
-      </c>
-      <c r="I150" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J150" s="7" t="n">
-        <v>18626</v>
-      </c>
-      <c r="K150" s="8" t="n">
-        <v>1330.4</v>
+      <c r="F150" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G150" s="4" t="n">
+        <v>13104</v>
+      </c>
+      <c r="H150" s="3" t="inlineStr">
+        <is>
+          <t>11/14</t>
+        </is>
+      </c>
+      <c r="I150" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J150" s="4" t="n">
+        <v>16678</v>
+      </c>
+      <c r="K150" s="5" t="n">
+        <v>1191.272727272727</v>
       </c>
     </row>
     <row r="151">
@@ -7917,11 +7917,11 @@
         </is>
       </c>
       <c r="G151" s="4" t="n">
-        <v>17751</v>
+        <v>18551</v>
       </c>
       <c r="H151" s="3" t="inlineStr">
         <is>
-          <t>11/21</t>
+          <t>12/21</t>
         </is>
       </c>
       <c r="I151" s="3" t="inlineStr">
@@ -7930,10 +7930,10 @@
         </is>
       </c>
       <c r="J151" s="4" t="n">
-        <v>33888</v>
+        <v>32464</v>
       </c>
       <c r="K151" s="5" t="n">
-        <v>1613.727272727273</v>
+        <v>1545.916666666667</v>
       </c>
     </row>
     <row r="152">
@@ -8015,11 +8015,11 @@
         </is>
       </c>
       <c r="G153" s="4" t="n">
-        <v>26383</v>
+        <v>27504</v>
       </c>
       <c r="H153" s="3" t="inlineStr">
         <is>
-          <t>13/20</t>
+          <t>14/20</t>
         </is>
       </c>
       <c r="I153" s="3" t="inlineStr">
@@ -8028,10 +8028,10 @@
         </is>
       </c>
       <c r="J153" s="4" t="n">
-        <v>40589</v>
+        <v>39291</v>
       </c>
       <c r="K153" s="5" t="n">
-        <v>2029.461538461539</v>
+        <v>1964.571428571429</v>
       </c>
     </row>
     <row r="154">
@@ -8309,11 +8309,11 @@
         </is>
       </c>
       <c r="G159" s="7" t="n">
-        <v>3240</v>
+        <v>2971</v>
       </c>
       <c r="H159" s="6" t="inlineStr">
         <is>
-          <t>14/22</t>
+          <t>15/22</t>
         </is>
       </c>
       <c r="I159" s="6" t="inlineStr">
@@ -8322,10 +8322,10 @@
         </is>
       </c>
       <c r="J159" s="7" t="n">
-        <v>5091</v>
+        <v>4357</v>
       </c>
       <c r="K159" s="8" t="n">
-        <v>231.4285714285714</v>
+        <v>198.0666666666667</v>
       </c>
     </row>
     <row r="160">
@@ -8378,52 +8378,52 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="6" t="inlineStr">
+      <c r="A161" s="13" t="inlineStr">
         <is>
           <t>SHOLINGUR</t>
         </is>
       </c>
-      <c r="B161" s="6" t="n">
+      <c r="B161" s="14" t="n">
         <v>39</v>
       </c>
-      <c r="C161" s="6" t="inlineStr">
+      <c r="C161" s="14" t="inlineStr">
         <is>
           <t>G.KAPIL</t>
         </is>
       </c>
-      <c r="D161" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E161" s="6" t="inlineStr">
+      <c r="D161" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E161" s="14" t="inlineStr">
         <is>
           <t>K.SARAVANAN</t>
         </is>
       </c>
-      <c r="F161" s="6" t="inlineStr">
+      <c r="F161" s="14" t="inlineStr">
         <is>
           <t>Pattali Makkal Katchi</t>
         </is>
       </c>
-      <c r="G161" s="7" t="n">
-        <v>2909</v>
-      </c>
-      <c r="H161" s="6" t="inlineStr">
-        <is>
-          <t>8/25</t>
-        </is>
-      </c>
-      <c r="I161" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J161" s="7" t="n">
-        <v>9091</v>
-      </c>
-      <c r="K161" s="8" t="n">
-        <v>363.625</v>
+      <c r="G161" s="15" t="n">
+        <v>841</v>
+      </c>
+      <c r="H161" s="14" t="inlineStr">
+        <is>
+          <t>9/25</t>
+        </is>
+      </c>
+      <c r="I161" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J161" s="15" t="n">
+        <v>2336</v>
+      </c>
+      <c r="K161" s="16" t="n">
+        <v>93.44444444444444</v>
       </c>
     </row>
     <row r="162">
@@ -8456,11 +8456,11 @@
         </is>
       </c>
       <c r="G162" s="4" t="n">
-        <v>22639</v>
+        <v>26994</v>
       </c>
       <c r="H162" s="3" t="inlineStr">
         <is>
-          <t>8/30</t>
+          <t>9/30</t>
         </is>
       </c>
       <c r="I162" s="3" t="inlineStr">
@@ -8469,10 +8469,10 @@
         </is>
       </c>
       <c r="J162" s="4" t="n">
-        <v>84896</v>
+        <v>89980</v>
       </c>
       <c r="K162" s="5" t="n">
-        <v>2829.875</v>
+        <v>2999.333333333333</v>
       </c>
     </row>
     <row r="163">
@@ -8770,52 +8770,52 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="13" t="inlineStr">
+      <c r="A169" s="9" t="inlineStr">
         <is>
           <t>SRIVAIKUNTAM</t>
         </is>
       </c>
-      <c r="B169" s="14" t="n">
+      <c r="B169" s="10" t="n">
         <v>216</v>
       </c>
-      <c r="C169" s="14" t="inlineStr">
+      <c r="C169" s="10" t="inlineStr">
         <is>
           <t>SHANMUGANATHAN. S. P</t>
         </is>
       </c>
-      <c r="D169" s="14" t="inlineStr">
+      <c r="D169" s="10" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E169" s="14" t="inlineStr">
+      <c r="E169" s="10" t="inlineStr">
         <is>
           <t>SARAVANAN. G</t>
         </is>
       </c>
-      <c r="F169" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G169" s="15" t="n">
-        <v>544</v>
-      </c>
-      <c r="H169" s="14" t="inlineStr">
-        <is>
-          <t>17/21</t>
-        </is>
-      </c>
-      <c r="I169" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J169" s="15" t="n">
-        <v>672</v>
-      </c>
-      <c r="K169" s="16" t="n">
-        <v>32</v>
+      <c r="F169" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G169" s="11" t="n">
+        <v>177</v>
+      </c>
+      <c r="H169" s="10" t="inlineStr">
+        <is>
+          <t>18/21</t>
+        </is>
+      </c>
+      <c r="I169" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J169" s="11" t="n">
+        <v>206</v>
+      </c>
+      <c r="K169" s="12" t="n">
+        <v>9.833333333333334</v>
       </c>
     </row>
     <row r="170">
@@ -8848,11 +8848,11 @@
         </is>
       </c>
       <c r="G170" s="7" t="n">
-        <v>5099</v>
+        <v>5324</v>
       </c>
       <c r="H170" s="6" t="inlineStr">
         <is>
-          <t>8/22</t>
+          <t>9/22</t>
         </is>
       </c>
       <c r="I170" s="6" t="inlineStr">
@@ -8861,10 +8861,10 @@
         </is>
       </c>
       <c r="J170" s="7" t="n">
-        <v>14022</v>
+        <v>13014</v>
       </c>
       <c r="K170" s="8" t="n">
-        <v>637.375</v>
+        <v>591.5555555555555</v>
       </c>
     </row>
     <row r="171">
@@ -8897,11 +8897,11 @@
         </is>
       </c>
       <c r="G171" s="7" t="n">
-        <v>8538</v>
+        <v>8516</v>
       </c>
       <c r="H171" s="6" t="inlineStr">
         <is>
-          <t>13/28</t>
+          <t>14/28</t>
         </is>
       </c>
       <c r="I171" s="6" t="inlineStr">
@@ -8910,10 +8910,10 @@
         </is>
       </c>
       <c r="J171" s="7" t="n">
-        <v>18390</v>
+        <v>17032</v>
       </c>
       <c r="K171" s="8" t="n">
-        <v>656.7692307692307</v>
+        <v>608.2857142857143</v>
       </c>
     </row>
     <row r="172">
@@ -8946,11 +8946,11 @@
         </is>
       </c>
       <c r="G172" s="4" t="n">
-        <v>17063</v>
+        <v>18325</v>
       </c>
       <c r="H172" s="3" t="inlineStr">
         <is>
-          <t>20/34</t>
+          <t>21/34</t>
         </is>
       </c>
       <c r="I172" s="3" t="inlineStr">
@@ -8959,10 +8959,10 @@
         </is>
       </c>
       <c r="J172" s="4" t="n">
-        <v>29007</v>
+        <v>29669</v>
       </c>
       <c r="K172" s="5" t="n">
-        <v>853.15</v>
+        <v>872.6190476190476</v>
       </c>
     </row>
     <row r="173">
@@ -9044,11 +9044,11 @@
         </is>
       </c>
       <c r="G174" s="15" t="n">
-        <v>298</v>
+        <v>1235</v>
       </c>
       <c r="H174" s="14" t="inlineStr">
         <is>
-          <t>10/24</t>
+          <t>11/24</t>
         </is>
       </c>
       <c r="I174" s="14" t="inlineStr">
@@ -9057,10 +9057,10 @@
         </is>
       </c>
       <c r="J174" s="15" t="n">
-        <v>715</v>
+        <v>2695</v>
       </c>
       <c r="K174" s="16" t="n">
-        <v>29.8</v>
+        <v>112.2727272727273</v>
       </c>
     </row>
     <row r="175">
@@ -9093,11 +9093,11 @@
         </is>
       </c>
       <c r="G175" s="4" t="n">
-        <v>16692</v>
+        <v>16972</v>
       </c>
       <c r="H175" s="3" t="inlineStr">
         <is>
-          <t>21/23</t>
+          <t>22/23</t>
         </is>
       </c>
       <c r="I175" s="3" t="inlineStr">
@@ -9106,10 +9106,10 @@
         </is>
       </c>
       <c r="J175" s="4" t="n">
-        <v>18282</v>
+        <v>17743</v>
       </c>
       <c r="K175" s="5" t="n">
-        <v>794.8571428571429</v>
+        <v>771.4545454545455</v>
       </c>
     </row>
     <row r="176">
@@ -9142,11 +9142,11 @@
         </is>
       </c>
       <c r="G176" s="4" t="n">
-        <v>18505</v>
+        <v>18298</v>
       </c>
       <c r="H176" s="3" t="inlineStr">
         <is>
-          <t>13/17</t>
+          <t>14/17</t>
         </is>
       </c>
       <c r="I176" s="3" t="inlineStr">
@@ -9155,10 +9155,10 @@
         </is>
       </c>
       <c r="J176" s="4" t="n">
-        <v>24199</v>
+        <v>22219</v>
       </c>
       <c r="K176" s="5" t="n">
-        <v>1423.461538461539</v>
+        <v>1307</v>
       </c>
     </row>
     <row r="177">
@@ -9338,11 +9338,11 @@
         </is>
       </c>
       <c r="G180" s="4" t="n">
-        <v>22118</v>
+        <v>24214</v>
       </c>
       <c r="H180" s="3" t="inlineStr">
         <is>
-          <t>12/29</t>
+          <t>13/29</t>
         </is>
       </c>
       <c r="I180" s="3" t="inlineStr">
@@ -9351,10 +9351,10 @@
         </is>
       </c>
       <c r="J180" s="4" t="n">
-        <v>53452</v>
+        <v>54016</v>
       </c>
       <c r="K180" s="5" t="n">
-        <v>1843.166666666667</v>
+        <v>1862.615384615385</v>
       </c>
     </row>
     <row r="181">
@@ -9485,11 +9485,11 @@
         </is>
       </c>
       <c r="G183" s="7" t="n">
-        <v>10304</v>
+        <v>11905</v>
       </c>
       <c r="H183" s="6" t="inlineStr">
         <is>
-          <t>14/24</t>
+          <t>15/24</t>
         </is>
       </c>
       <c r="I183" s="6" t="inlineStr">
@@ -9498,10 +9498,10 @@
         </is>
       </c>
       <c r="J183" s="7" t="n">
-        <v>17664</v>
+        <v>19048</v>
       </c>
       <c r="K183" s="8" t="n">
-        <v>736</v>
+        <v>793.6666666666666</v>
       </c>
     </row>
     <row r="184">
@@ -9583,11 +9583,11 @@
         </is>
       </c>
       <c r="G185" s="7" t="n">
-        <v>1077</v>
+        <v>1906</v>
       </c>
       <c r="H185" s="6" t="inlineStr">
         <is>
-          <t>8/23</t>
+          <t>9/23</t>
         </is>
       </c>
       <c r="I185" s="6" t="inlineStr">
@@ -9596,10 +9596,10 @@
         </is>
       </c>
       <c r="J185" s="7" t="n">
-        <v>3096</v>
+        <v>4871</v>
       </c>
       <c r="K185" s="8" t="n">
-        <v>134.625</v>
+        <v>211.7777777777778</v>
       </c>
     </row>
     <row r="186">
@@ -9681,11 +9681,11 @@
         </is>
       </c>
       <c r="G187" s="4" t="n">
-        <v>33635</v>
+        <v>35989</v>
       </c>
       <c r="H187" s="3" t="inlineStr">
         <is>
-          <t>14/25</t>
+          <t>15/25</t>
         </is>
       </c>
       <c r="I187" s="3" t="inlineStr">
@@ -9694,10 +9694,10 @@
         </is>
       </c>
       <c r="J187" s="4" t="n">
-        <v>60062</v>
+        <v>59982</v>
       </c>
       <c r="K187" s="5" t="n">
-        <v>2402.5</v>
+        <v>2399.266666666667</v>
       </c>
     </row>
     <row r="188">
@@ -9828,11 +9828,11 @@
         </is>
       </c>
       <c r="G190" s="4" t="n">
-        <v>24123</v>
+        <v>26334</v>
       </c>
       <c r="H190" s="3" t="inlineStr">
         <is>
-          <t>15/26</t>
+          <t>16/26</t>
         </is>
       </c>
       <c r="I190" s="3" t="inlineStr">
@@ -9841,10 +9841,10 @@
         </is>
       </c>
       <c r="J190" s="4" t="n">
-        <v>41813</v>
+        <v>42793</v>
       </c>
       <c r="K190" s="5" t="n">
-        <v>1608.2</v>
+        <v>1645.875</v>
       </c>
     </row>
     <row r="191">
@@ -9926,11 +9926,11 @@
         </is>
       </c>
       <c r="G192" s="7" t="n">
-        <v>3801</v>
+        <v>5085</v>
       </c>
       <c r="H192" s="6" t="inlineStr">
         <is>
-          <t>13/22</t>
+          <t>14/22</t>
         </is>
       </c>
       <c r="I192" s="6" t="inlineStr">
@@ -9939,59 +9939,59 @@
         </is>
       </c>
       <c r="J192" s="7" t="n">
-        <v>6432</v>
+        <v>7991</v>
       </c>
       <c r="K192" s="8" t="n">
-        <v>292.3846153846154</v>
+        <v>363.2142857142857</v>
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="9" t="inlineStr">
+      <c r="A193" s="13" t="inlineStr">
         <is>
           <t>TINDIVANAM</t>
         </is>
       </c>
-      <c r="B193" s="10" t="n">
+      <c r="B193" s="14" t="n">
         <v>72</v>
       </c>
-      <c r="C193" s="10" t="inlineStr">
+      <c r="C193" s="14" t="inlineStr">
+        <is>
+          <t>VANNI ARASU</t>
+        </is>
+      </c>
+      <c r="D193" s="14" t="inlineStr">
+        <is>
+          <t>Viduthalai Chiruthaigal Katchi</t>
+        </is>
+      </c>
+      <c r="E193" s="14" t="inlineStr">
         <is>
           <t>ARJUNAN. P</t>
         </is>
       </c>
-      <c r="D193" s="10" t="inlineStr">
+      <c r="F193" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E193" s="10" t="inlineStr">
-        <is>
-          <t>VANNI ARASU</t>
-        </is>
-      </c>
-      <c r="F193" s="10" t="inlineStr">
-        <is>
-          <t>Viduthalai Chiruthaigal Katchi</t>
-        </is>
-      </c>
-      <c r="G193" s="11" t="n">
-        <v>144</v>
-      </c>
-      <c r="H193" s="10" t="inlineStr">
-        <is>
-          <t>10/21</t>
-        </is>
-      </c>
-      <c r="I193" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J193" s="11" t="n">
-        <v>302</v>
-      </c>
-      <c r="K193" s="12" t="n">
-        <v>14.4</v>
+      <c r="G193" s="15" t="n">
+        <v>620</v>
+      </c>
+      <c r="H193" s="14" t="inlineStr">
+        <is>
+          <t>11/21</t>
+        </is>
+      </c>
+      <c r="I193" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J193" s="15" t="n">
+        <v>1184</v>
+      </c>
+      <c r="K193" s="16" t="n">
+        <v>56.36363636363637</v>
       </c>
     </row>
     <row r="194">
@@ -10073,11 +10073,11 @@
         </is>
       </c>
       <c r="G195" s="7" t="n">
-        <v>4810</v>
+        <v>6465</v>
       </c>
       <c r="H195" s="6" t="inlineStr">
         <is>
-          <t>9/21</t>
+          <t>10/21</t>
         </is>
       </c>
       <c r="I195" s="6" t="inlineStr">
@@ -10086,10 +10086,10 @@
         </is>
       </c>
       <c r="J195" s="7" t="n">
-        <v>11223</v>
+        <v>13576</v>
       </c>
       <c r="K195" s="8" t="n">
-        <v>534.4444444444445</v>
+        <v>646.5</v>
       </c>
     </row>
     <row r="196">
@@ -10220,11 +10220,11 @@
         </is>
       </c>
       <c r="G198" s="7" t="n">
-        <v>1914</v>
+        <v>2341</v>
       </c>
       <c r="H198" s="6" t="inlineStr">
         <is>
-          <t>7/21</t>
+          <t>8/21</t>
         </is>
       </c>
       <c r="I198" s="6" t="inlineStr">
@@ -10233,10 +10233,10 @@
         </is>
       </c>
       <c r="J198" s="7" t="n">
-        <v>5742</v>
+        <v>6145</v>
       </c>
       <c r="K198" s="8" t="n">
-        <v>273.4285714285714</v>
+        <v>292.625</v>
       </c>
     </row>
     <row r="199">
@@ -10250,30 +10250,30 @@
       </c>
       <c r="C199" s="14" t="inlineStr">
         <is>
+          <t>VIJAY R BARANIBALAAJI</t>
+        </is>
+      </c>
+      <c r="D199" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E199" s="14" t="inlineStr">
+        <is>
           <t>PALANISAMY S</t>
         </is>
       </c>
-      <c r="D199" s="14" t="inlineStr">
+      <c r="F199" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E199" s="14" t="inlineStr">
-        <is>
-          <t>VIJAY R BARANIBALAAJI</t>
-        </is>
-      </c>
-      <c r="F199" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
       <c r="G199" s="15" t="n">
-        <v>279</v>
+        <v>385</v>
       </c>
       <c r="H199" s="14" t="inlineStr">
         <is>
-          <t>12/24</t>
+          <t>13/24</t>
         </is>
       </c>
       <c r="I199" s="14" t="inlineStr">
@@ -10282,10 +10282,10 @@
         </is>
       </c>
       <c r="J199" s="15" t="n">
-        <v>558</v>
+        <v>711</v>
       </c>
       <c r="K199" s="16" t="n">
-        <v>23.25</v>
+        <v>29.61538461538462</v>
       </c>
     </row>
     <row r="200">
@@ -10416,11 +10416,11 @@
         </is>
       </c>
       <c r="G202" s="7" t="n">
-        <v>4157</v>
+        <v>3904</v>
       </c>
       <c r="H202" s="6" t="inlineStr">
         <is>
-          <t>11/27</t>
+          <t>12/27</t>
         </is>
       </c>
       <c r="I202" s="6" t="inlineStr">
@@ -10429,10 +10429,10 @@
         </is>
       </c>
       <c r="J202" s="7" t="n">
-        <v>10204</v>
+        <v>8784</v>
       </c>
       <c r="K202" s="8" t="n">
-        <v>377.9090909090909</v>
+        <v>325.3333333333333</v>
       </c>
     </row>
     <row r="203">
@@ -10465,11 +10465,11 @@
         </is>
       </c>
       <c r="G203" s="4" t="n">
-        <v>31637</v>
+        <v>35105</v>
       </c>
       <c r="H203" s="3" t="inlineStr">
         <is>
-          <t>13/32</t>
+          <t>14/32</t>
         </is>
       </c>
       <c r="I203" s="3" t="inlineStr">
@@ -10478,10 +10478,10 @@
         </is>
       </c>
       <c r="J203" s="4" t="n">
-        <v>77876</v>
+        <v>80240</v>
       </c>
       <c r="K203" s="5" t="n">
-        <v>2433.615384615385</v>
+        <v>2507.5</v>
       </c>
     </row>
     <row r="204">
@@ -10603,20 +10603,20 @@
       </c>
       <c r="E206" s="10" t="inlineStr">
         <is>
-          <t>M.KEERTHIKA</t>
+          <t>RM. KARUMANICKAM</t>
         </is>
       </c>
       <c r="F206" s="10" t="inlineStr">
         <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
+          <t>Indian National Congress</t>
         </is>
       </c>
       <c r="G206" s="11" t="n">
-        <v>119</v>
+        <v>17</v>
       </c>
       <c r="H206" s="10" t="inlineStr">
         <is>
-          <t>18/27</t>
+          <t>19/27</t>
         </is>
       </c>
       <c r="I206" s="10" t="inlineStr">
@@ -10625,10 +10625,10 @@
         </is>
       </c>
       <c r="J206" s="11" t="n">
-        <v>178</v>
+        <v>24</v>
       </c>
       <c r="K206" s="12" t="n">
-        <v>6.611111111111111</v>
+        <v>0.8947368421052632</v>
       </c>
     </row>
     <row r="207">
@@ -10759,7 +10759,7 @@
         </is>
       </c>
       <c r="G209" s="11" t="n">
-        <v>189</v>
+        <v>433</v>
       </c>
       <c r="H209" s="10" t="inlineStr">
         <is>
@@ -10772,10 +10772,10 @@
         </is>
       </c>
       <c r="J209" s="11" t="n">
-        <v>211</v>
+        <v>484</v>
       </c>
       <c r="K209" s="12" t="n">
-        <v>11.11764705882353</v>
+        <v>25.47058823529412</v>
       </c>
     </row>
     <row r="210">
@@ -10808,11 +10808,11 @@
         </is>
       </c>
       <c r="G210" s="7" t="n">
-        <v>3857</v>
+        <v>4023</v>
       </c>
       <c r="H210" s="6" t="inlineStr">
         <is>
-          <t>14/22</t>
+          <t>15/22</t>
         </is>
       </c>
       <c r="I210" s="6" t="inlineStr">
@@ -10821,10 +10821,10 @@
         </is>
       </c>
       <c r="J210" s="7" t="n">
-        <v>6061</v>
+        <v>5900</v>
       </c>
       <c r="K210" s="8" t="n">
-        <v>275.5</v>
+        <v>268.2</v>
       </c>
     </row>
     <row r="211">
@@ -10857,11 +10857,11 @@
         </is>
       </c>
       <c r="G211" s="15" t="n">
-        <v>913</v>
+        <v>1100</v>
       </c>
       <c r="H211" s="14" t="inlineStr">
         <is>
-          <t>11/27</t>
+          <t>12/27</t>
         </is>
       </c>
       <c r="I211" s="14" t="inlineStr">
@@ -10870,10 +10870,10 @@
         </is>
       </c>
       <c r="J211" s="15" t="n">
-        <v>2241</v>
+        <v>2475</v>
       </c>
       <c r="K211" s="16" t="n">
-        <v>83</v>
+        <v>91.66666666666667</v>
       </c>
     </row>
     <row r="212">
@@ -10906,11 +10906,11 @@
         </is>
       </c>
       <c r="G212" s="7" t="n">
-        <v>2777</v>
+        <v>2187</v>
       </c>
       <c r="H212" s="6" t="inlineStr">
         <is>
-          <t>9/25</t>
+          <t>10/25</t>
         </is>
       </c>
       <c r="I212" s="6" t="inlineStr">
@@ -10919,108 +10919,108 @@
         </is>
       </c>
       <c r="J212" s="7" t="n">
-        <v>7714</v>
+        <v>5468</v>
       </c>
       <c r="K212" s="8" t="n">
-        <v>308.5555555555555</v>
+        <v>218.7</v>
       </c>
     </row>
     <row r="213">
-      <c r="A213" s="6" t="inlineStr">
+      <c r="A213" s="2" t="inlineStr">
         <is>
           <t>UTHANGARAI</t>
         </is>
       </c>
-      <c r="B213" s="6" t="n">
+      <c r="B213" s="3" t="n">
         <v>51</v>
       </c>
-      <c r="C213" s="6" t="inlineStr">
+      <c r="C213" s="3" t="inlineStr">
         <is>
           <t>N ELAIYARAJA</t>
         </is>
       </c>
-      <c r="D213" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E213" s="6" t="inlineStr">
+      <c r="D213" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E213" s="3" t="inlineStr">
         <is>
           <t>T M TAMILSELVAM</t>
         </is>
       </c>
-      <c r="F213" s="6" t="inlineStr">
+      <c r="F213" s="3" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G213" s="7" t="n">
-        <v>4544</v>
-      </c>
-      <c r="H213" s="6" t="inlineStr">
-        <is>
-          <t>17/23</t>
-        </is>
-      </c>
-      <c r="I213" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J213" s="7" t="n">
-        <v>6148</v>
-      </c>
-      <c r="K213" s="8" t="n">
-        <v>267.2941176470588</v>
+      <c r="G213" s="4" t="n">
+        <v>5701</v>
+      </c>
+      <c r="H213" s="3" t="inlineStr">
+        <is>
+          <t>18/23</t>
+        </is>
+      </c>
+      <c r="I213" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J213" s="4" t="n">
+        <v>7285</v>
+      </c>
+      <c r="K213" s="5" t="n">
+        <v>316.7222222222222</v>
       </c>
     </row>
     <row r="214">
-      <c r="A214" s="2" t="inlineStr">
+      <c r="A214" s="6" t="inlineStr">
         <is>
           <t>UTHIRAMERUR</t>
         </is>
       </c>
-      <c r="B214" s="3" t="n">
+      <c r="B214" s="6" t="n">
         <v>36</v>
       </c>
-      <c r="C214" s="3" t="inlineStr">
+      <c r="C214" s="6" t="inlineStr">
         <is>
           <t>MUNIRATHINAM.J</t>
         </is>
       </c>
-      <c r="D214" s="3" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E214" s="3" t="inlineStr">
+      <c r="D214" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E214" s="6" t="inlineStr">
         <is>
           <t>SUNDAR.K</t>
         </is>
       </c>
-      <c r="F214" s="3" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G214" s="4" t="n">
-        <v>13510</v>
-      </c>
-      <c r="H214" s="3" t="inlineStr">
-        <is>
-          <t>15/23</t>
-        </is>
-      </c>
-      <c r="I214" s="3" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J214" s="4" t="n">
-        <v>20715</v>
-      </c>
-      <c r="K214" s="5" t="n">
-        <v>900.6666666666666</v>
+      <c r="F214" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G214" s="7" t="n">
+        <v>13873</v>
+      </c>
+      <c r="H214" s="6" t="inlineStr">
+        <is>
+          <t>16/23</t>
+        </is>
+      </c>
+      <c r="I214" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J214" s="7" t="n">
+        <v>19942</v>
+      </c>
+      <c r="K214" s="8" t="n">
+        <v>867.0625</v>
       </c>
     </row>
     <row r="215">
@@ -11102,11 +11102,11 @@
         </is>
       </c>
       <c r="G216" s="7" t="n">
-        <v>3787</v>
+        <v>3547</v>
       </c>
       <c r="H216" s="6" t="inlineStr">
         <is>
-          <t>12/21</t>
+          <t>13/21</t>
         </is>
       </c>
       <c r="I216" s="6" t="inlineStr">
@@ -11115,10 +11115,10 @@
         </is>
       </c>
       <c r="J216" s="7" t="n">
-        <v>6627</v>
+        <v>5730</v>
       </c>
       <c r="K216" s="8" t="n">
-        <v>315.5833333333333</v>
+        <v>272.8461538461539</v>
       </c>
     </row>
     <row r="217">
@@ -11151,11 +11151,11 @@
         </is>
       </c>
       <c r="G217" s="4" t="n">
-        <v>8280</v>
+        <v>5010</v>
       </c>
       <c r="H217" s="3" t="inlineStr">
         <is>
-          <t>19/23</t>
+          <t>21/23</t>
         </is>
       </c>
       <c r="I217" s="3" t="inlineStr">
@@ -11164,10 +11164,10 @@
         </is>
       </c>
       <c r="J217" s="4" t="n">
-        <v>10023</v>
+        <v>5487</v>
       </c>
       <c r="K217" s="5" t="n">
-        <v>435.7894736842105</v>
+        <v>238.5714285714286</v>
       </c>
     </row>
     <row r="218">
@@ -11200,11 +11200,11 @@
         </is>
       </c>
       <c r="G218" s="7" t="n">
-        <v>2378</v>
+        <v>2733</v>
       </c>
       <c r="H218" s="6" t="inlineStr">
         <is>
-          <t>11/22</t>
+          <t>12/22</t>
         </is>
       </c>
       <c r="I218" s="6" t="inlineStr">
@@ -11213,10 +11213,10 @@
         </is>
       </c>
       <c r="J218" s="7" t="n">
-        <v>4756</v>
+        <v>5010</v>
       </c>
       <c r="K218" s="8" t="n">
-        <v>216.1818181818182</v>
+        <v>227.75</v>
       </c>
     </row>
     <row r="219">
@@ -11249,11 +11249,11 @@
         </is>
       </c>
       <c r="G219" s="7" t="n">
-        <v>6212</v>
+        <v>6198</v>
       </c>
       <c r="H219" s="6" t="inlineStr">
         <is>
-          <t>14/23</t>
+          <t>15/23</t>
         </is>
       </c>
       <c r="I219" s="6" t="inlineStr">
@@ -11262,10 +11262,10 @@
         </is>
       </c>
       <c r="J219" s="7" t="n">
-        <v>10205</v>
+        <v>9504</v>
       </c>
       <c r="K219" s="8" t="n">
-        <v>443.7142857142857</v>
+        <v>413.2</v>
       </c>
     </row>
     <row r="220">
@@ -11298,11 +11298,11 @@
         </is>
       </c>
       <c r="G220" s="7" t="n">
-        <v>5705</v>
+        <v>5392</v>
       </c>
       <c r="H220" s="6" t="inlineStr">
         <is>
-          <t>11/18</t>
+          <t>12/18</t>
         </is>
       </c>
       <c r="I220" s="6" t="inlineStr">
@@ -11311,10 +11311,10 @@
         </is>
       </c>
       <c r="J220" s="7" t="n">
-        <v>9335</v>
+        <v>8088</v>
       </c>
       <c r="K220" s="8" t="n">
-        <v>518.6363636363636</v>
+        <v>449.3333333333333</v>
       </c>
     </row>
     <row r="221">
@@ -11347,11 +11347,11 @@
         </is>
       </c>
       <c r="G221" s="7" t="n">
-        <v>5936</v>
+        <v>7238</v>
       </c>
       <c r="H221" s="6" t="inlineStr">
         <is>
-          <t>12/24</t>
+          <t>13/24</t>
         </is>
       </c>
       <c r="I221" s="6" t="inlineStr">
@@ -11360,10 +11360,10 @@
         </is>
       </c>
       <c r="J221" s="7" t="n">
-        <v>11872</v>
+        <v>13362</v>
       </c>
       <c r="K221" s="8" t="n">
-        <v>494.6666666666667</v>
+        <v>556.7692307692307</v>
       </c>
     </row>
     <row r="222">
@@ -11514,52 +11514,52 @@
       </c>
     </row>
     <row r="225">
-      <c r="A225" s="6" t="inlineStr">
+      <c r="A225" s="13" t="inlineStr">
         <is>
           <t>VEPPANAHALLI</t>
         </is>
       </c>
-      <c r="B225" s="6" t="n">
+      <c r="B225" s="14" t="n">
         <v>54</v>
       </c>
-      <c r="C225" s="6" t="inlineStr">
+      <c r="C225" s="14" t="inlineStr">
         <is>
           <t>MUNUSAMY.K.P</t>
         </is>
       </c>
-      <c r="D225" s="6" t="inlineStr">
+      <c r="D225" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E225" s="6" t="inlineStr">
+      <c r="E225" s="14" t="inlineStr">
         <is>
           <t>SRINIVASAN.P.S</t>
         </is>
       </c>
-      <c r="F225" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G225" s="7" t="n">
-        <v>2927</v>
-      </c>
-      <c r="H225" s="6" t="inlineStr">
-        <is>
-          <t>14/25</t>
-        </is>
-      </c>
-      <c r="I225" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J225" s="7" t="n">
-        <v>5227</v>
-      </c>
-      <c r="K225" s="8" t="n">
-        <v>209.0714285714286</v>
+      <c r="F225" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G225" s="15" t="n">
+        <v>1623</v>
+      </c>
+      <c r="H225" s="14" t="inlineStr">
+        <is>
+          <t>15/25</t>
+        </is>
+      </c>
+      <c r="I225" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J225" s="15" t="n">
+        <v>2705</v>
+      </c>
+      <c r="K225" s="16" t="n">
+        <v>108.2</v>
       </c>
     </row>
     <row r="226">
@@ -11739,11 +11739,11 @@
         </is>
       </c>
       <c r="G229" s="7" t="n">
-        <v>11163</v>
+        <v>12310</v>
       </c>
       <c r="H229" s="6" t="inlineStr">
         <is>
-          <t>12/19</t>
+          <t>13/19</t>
         </is>
       </c>
       <c r="I229" s="6" t="inlineStr">
@@ -11752,10 +11752,10 @@
         </is>
       </c>
       <c r="J229" s="7" t="n">
-        <v>17675</v>
+        <v>17992</v>
       </c>
       <c r="K229" s="8" t="n">
-        <v>930.25</v>
+        <v>946.9230769230769</v>
       </c>
     </row>
     <row r="230">
@@ -11788,11 +11788,11 @@
         </is>
       </c>
       <c r="G230" s="15" t="n">
-        <v>1148</v>
+        <v>1426</v>
       </c>
       <c r="H230" s="14" t="inlineStr">
         <is>
-          <t>14/24</t>
+          <t>15/24</t>
         </is>
       </c>
       <c r="I230" s="14" t="inlineStr">
@@ -11801,10 +11801,10 @@
         </is>
       </c>
       <c r="J230" s="15" t="n">
-        <v>1968</v>
+        <v>2282</v>
       </c>
       <c r="K230" s="16" t="n">
-        <v>82</v>
+        <v>95.06666666666666</v>
       </c>
     </row>
     <row r="231">
@@ -11935,11 +11935,11 @@
         </is>
       </c>
       <c r="G233" s="4" t="n">
-        <v>9977</v>
+        <v>11348</v>
       </c>
       <c r="H233" s="3" t="inlineStr">
         <is>
-          <t>10/23</t>
+          <t>11/23</t>
         </is>
       </c>
       <c r="I233" s="3" t="inlineStr">
@@ -11948,10 +11948,10 @@
         </is>
       </c>
       <c r="J233" s="4" t="n">
-        <v>22947</v>
+        <v>23728</v>
       </c>
       <c r="K233" s="5" t="n">
-        <v>997.7</v>
+        <v>1031.636363636364</v>
       </c>
     </row>
     <row r="234">
@@ -11984,11 +11984,11 @@
         </is>
       </c>
       <c r="G234" s="7" t="n">
-        <v>2466</v>
+        <v>3008</v>
       </c>
       <c r="H234" s="6" t="inlineStr">
         <is>
-          <t>13/23</t>
+          <t>14/23</t>
         </is>
       </c>
       <c r="I234" s="6" t="inlineStr">
@@ -11997,10 +11997,10 @@
         </is>
       </c>
       <c r="J234" s="7" t="n">
-        <v>4363</v>
+        <v>4942</v>
       </c>
       <c r="K234" s="8" t="n">
-        <v>189.6923076923077</v>
+        <v>214.8571428571429</v>
       </c>
     </row>
     <row r="235">

</xml_diff>

<commit_message>
Update election results snapshot (64.9% counted)
TVK 105, DMK 59, AIADMK 48. 12 lead changes. SHOLAVANDAN settled (TVK).
MANAPPARAI at 31-vote TVK lead, THALLI at 24-vote BJP lead. 10 knife-edge.

https://claude.ai/code/session_01MizbUy44JG5sXyvaf3Wekb
</commit_message>
<xml_diff>
--- a/tn_election_results_may2026.xlsx
+++ b/tn_election_results_may2026.xlsx
@@ -685,52 +685,52 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>ALANGULAM</t>
         </is>
       </c>
-      <c r="B4" s="10" t="n">
+      <c r="B4" s="6" t="n">
         <v>223</v>
       </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>PAUL MANOJ PANDIAN</t>
         </is>
       </c>
-      <c r="D4" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>K R P PRABAKARAN</t>
         </is>
       </c>
-      <c r="F4" s="10" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G4" s="11" t="n">
-        <v>2048</v>
-      </c>
-      <c r="H4" s="10" t="inlineStr">
-        <is>
-          <t>17/24</t>
-        </is>
-      </c>
-      <c r="I4" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J4" s="11" t="n">
-        <v>2891</v>
-      </c>
-      <c r="K4" s="12" t="n">
-        <v>120.4705882352941</v>
+      <c r="G4" s="7" t="n">
+        <v>3679</v>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>18/24</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J4" s="7" t="n">
+        <v>4905</v>
+      </c>
+      <c r="K4" s="8" t="n">
+        <v>204.3888888888889</v>
       </c>
     </row>
     <row r="5">
@@ -754,20 +754,20 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>S.RAJAGOPAL</t>
+          <t>V.P.DURAI</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Tamilaga Vettri Kazhagam</t>
+          <t>Indian National Congress</t>
         </is>
       </c>
       <c r="G5" s="4" t="n">
-        <v>9368</v>
+        <v>10632</v>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>20/23</t>
+          <t>21/23</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -776,10 +776,10 @@
         </is>
       </c>
       <c r="J5" s="4" t="n">
-        <v>10773</v>
+        <v>11645</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>468.4</v>
+        <v>506.2857142857143</v>
       </c>
     </row>
     <row r="6">
@@ -812,11 +812,11 @@
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>38162</v>
+        <v>38522</v>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>15/27</t>
+          <t>16/27</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -825,10 +825,10 @@
         </is>
       </c>
       <c r="J6" s="4" t="n">
-        <v>68692</v>
+        <v>65006</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>2544.133333333333</v>
+        <v>2407.625</v>
       </c>
     </row>
     <row r="7">
@@ -861,11 +861,11 @@
         </is>
       </c>
       <c r="G7" s="7" t="n">
-        <v>6012</v>
+        <v>2928</v>
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>10/22</t>
+          <t>11/22</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
@@ -874,10 +874,10 @@
         </is>
       </c>
       <c r="J7" s="7" t="n">
-        <v>13226</v>
+        <v>5856</v>
       </c>
       <c r="K7" s="8" t="n">
-        <v>601.2</v>
+        <v>266.1818181818182</v>
       </c>
     </row>
     <row r="8">
@@ -1155,11 +1155,11 @@
         </is>
       </c>
       <c r="G13" s="7" t="n">
-        <v>2912</v>
+        <v>3291</v>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>19/24</t>
+          <t>20/24</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
@@ -1168,10 +1168,10 @@
         </is>
       </c>
       <c r="J13" s="7" t="n">
-        <v>3678</v>
+        <v>3949</v>
       </c>
       <c r="K13" s="8" t="n">
-        <v>153.2631578947368</v>
+        <v>164.55</v>
       </c>
     </row>
     <row r="14">
@@ -1204,11 +1204,11 @@
         </is>
       </c>
       <c r="G14" s="7" t="n">
-        <v>11610</v>
+        <v>11861</v>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>14/22</t>
+          <t>15/22</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
@@ -1217,10 +1217,10 @@
         </is>
       </c>
       <c r="J14" s="7" t="n">
-        <v>18244</v>
+        <v>17396</v>
       </c>
       <c r="K14" s="8" t="n">
-        <v>829.2857142857143</v>
+        <v>790.7333333333335</v>
       </c>
     </row>
     <row r="15">
@@ -1302,11 +1302,11 @@
         </is>
       </c>
       <c r="G16" s="4" t="n">
-        <v>14495</v>
+        <v>15837</v>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>10/23</t>
+          <t>11/23</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
@@ -1315,10 +1315,10 @@
         </is>
       </c>
       <c r="J16" s="4" t="n">
-        <v>33338</v>
+        <v>33114</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>1449.5</v>
+        <v>1439.727272727273</v>
       </c>
     </row>
     <row r="17">
@@ -1351,11 +1351,11 @@
         </is>
       </c>
       <c r="G17" s="4" t="n">
-        <v>13335</v>
+        <v>16268</v>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>19/24</t>
+          <t>20/24</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -1364,10 +1364,10 @@
         </is>
       </c>
       <c r="J17" s="4" t="n">
-        <v>16844</v>
+        <v>19522</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>701.8421052631579</v>
+        <v>813.4</v>
       </c>
     </row>
     <row r="18">
@@ -1547,11 +1547,11 @@
         </is>
       </c>
       <c r="G21" s="4" t="n">
-        <v>36289</v>
+        <v>39060</v>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>13/26</t>
+          <t>14/26</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -1560,10 +1560,10 @@
         </is>
       </c>
       <c r="J21" s="4" t="n">
-        <v>72578</v>
+        <v>72540</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>2791.461538461539</v>
+        <v>2790</v>
       </c>
     </row>
     <row r="22">
@@ -1616,52 +1616,52 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t>BARGUR</t>
         </is>
       </c>
-      <c r="B23" s="6" t="n">
+      <c r="B23" s="10" t="n">
         <v>52</v>
       </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C23" s="10" t="inlineStr">
         <is>
           <t>E. MURALIDHARAN</t>
         </is>
       </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="inlineStr">
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E23" s="10" t="inlineStr">
         <is>
           <t>E.C. GOVINDARASAN</t>
         </is>
       </c>
-      <c r="F23" s="6" t="inlineStr">
+      <c r="F23" s="10" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G23" s="7" t="n">
-        <v>1877</v>
-      </c>
-      <c r="H23" s="6" t="inlineStr">
-        <is>
-          <t>13/24</t>
-        </is>
-      </c>
-      <c r="I23" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J23" s="7" t="n">
-        <v>3465</v>
-      </c>
-      <c r="K23" s="8" t="n">
-        <v>144.3846153846154</v>
+      <c r="G23" s="11" t="n">
+        <v>1440</v>
+      </c>
+      <c r="H23" s="10" t="inlineStr">
+        <is>
+          <t>14/24</t>
+        </is>
+      </c>
+      <c r="I23" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J23" s="11" t="n">
+        <v>2469</v>
+      </c>
+      <c r="K23" s="12" t="n">
+        <v>102.8571428571429</v>
       </c>
     </row>
     <row r="24">
@@ -1714,52 +1714,52 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="9" t="inlineStr">
+      <c r="A25" s="13" t="inlineStr">
         <is>
           <t>BHAVANISAGAR</t>
         </is>
       </c>
-      <c r="B25" s="10" t="n">
+      <c r="B25" s="14" t="n">
         <v>107</v>
       </c>
-      <c r="C25" s="10" t="inlineStr">
+      <c r="C25" s="14" t="inlineStr">
         <is>
           <t>A.BANNARI</t>
         </is>
       </c>
-      <c r="D25" s="10" t="inlineStr">
+      <c r="D25" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E25" s="10" t="inlineStr">
+      <c r="E25" s="14" t="inlineStr">
         <is>
           <t>V.P.TAMILSELVI</t>
         </is>
       </c>
-      <c r="F25" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G25" s="11" t="n">
-        <v>1161</v>
-      </c>
-      <c r="H25" s="10" t="inlineStr">
-        <is>
-          <t>15/24</t>
-        </is>
-      </c>
-      <c r="I25" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J25" s="11" t="n">
-        <v>1858</v>
-      </c>
-      <c r="K25" s="12" t="n">
-        <v>77.40000000000001</v>
+      <c r="F25" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G25" s="15" t="n">
+        <v>71</v>
+      </c>
+      <c r="H25" s="14" t="inlineStr">
+        <is>
+          <t>16/24</t>
+        </is>
+      </c>
+      <c r="I25" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J25" s="15" t="n">
+        <v>106</v>
+      </c>
+      <c r="K25" s="16" t="n">
+        <v>4.4375</v>
       </c>
     </row>
     <row r="26">
@@ -1792,11 +1792,11 @@
         </is>
       </c>
       <c r="G26" s="7" t="n">
-        <v>6810</v>
+        <v>6062</v>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>12/22</t>
+          <t>13/22</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
@@ -1805,10 +1805,10 @@
         </is>
       </c>
       <c r="J26" s="7" t="n">
-        <v>12485</v>
+        <v>10259</v>
       </c>
       <c r="K26" s="8" t="n">
-        <v>567.5</v>
+        <v>466.3076923076923</v>
       </c>
     </row>
     <row r="27">
@@ -1890,11 +1890,11 @@
         </is>
       </c>
       <c r="G28" s="4" t="n">
-        <v>15424</v>
+        <v>15264</v>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>11/36</t>
+          <t>12/36</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
@@ -1903,10 +1903,10 @@
         </is>
       </c>
       <c r="J28" s="4" t="n">
-        <v>50479</v>
+        <v>45792</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>1402.181818181818</v>
+        <v>1272</v>
       </c>
     </row>
     <row r="29">
@@ -2086,11 +2086,11 @@
         </is>
       </c>
       <c r="G32" s="7" t="n">
-        <v>3193</v>
+        <v>3784</v>
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>18/21</t>
+          <t>19/21</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
@@ -2099,10 +2099,10 @@
         </is>
       </c>
       <c r="J32" s="7" t="n">
-        <v>3725</v>
+        <v>4182</v>
       </c>
       <c r="K32" s="8" t="n">
-        <v>177.3888888888889</v>
+        <v>199.1578947368421</v>
       </c>
     </row>
     <row r="33">
@@ -2380,11 +2380,11 @@
         </is>
       </c>
       <c r="G38" s="7" t="n">
-        <v>7310</v>
+        <v>8464</v>
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>12/19</t>
+          <t>13/19</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr">
@@ -2393,10 +2393,10 @@
         </is>
       </c>
       <c r="J38" s="7" t="n">
-        <v>11574</v>
+        <v>12370</v>
       </c>
       <c r="K38" s="8" t="n">
-        <v>609.1666666666666</v>
+        <v>651.0769230769231</v>
       </c>
     </row>
     <row r="39">
@@ -2478,11 +2478,11 @@
         </is>
       </c>
       <c r="G40" s="4" t="n">
-        <v>13132</v>
+        <v>14301</v>
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>20/23</t>
+          <t>21/23</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
@@ -2491,10 +2491,10 @@
         </is>
       </c>
       <c r="J40" s="4" t="n">
-        <v>15102</v>
+        <v>15663</v>
       </c>
       <c r="K40" s="5" t="n">
-        <v>656.6</v>
+        <v>681</v>
       </c>
     </row>
     <row r="41">
@@ -2527,11 +2527,11 @@
         </is>
       </c>
       <c r="G41" s="4" t="n">
-        <v>13571</v>
+        <v>15176</v>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>19/23</t>
+          <t>20/23</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
@@ -2540,10 +2540,10 @@
         </is>
       </c>
       <c r="J41" s="4" t="n">
-        <v>16428</v>
+        <v>17452</v>
       </c>
       <c r="K41" s="5" t="n">
-        <v>714.2631578947369</v>
+        <v>758.8</v>
       </c>
     </row>
     <row r="42">
@@ -2576,11 +2576,11 @@
         </is>
       </c>
       <c r="G42" s="11" t="n">
-        <v>1079</v>
+        <v>449</v>
       </c>
       <c r="H42" s="10" t="inlineStr">
         <is>
-          <t>17/24</t>
+          <t>18/24</t>
         </is>
       </c>
       <c r="I42" s="10" t="inlineStr">
@@ -2589,10 +2589,10 @@
         </is>
       </c>
       <c r="J42" s="11" t="n">
-        <v>1523</v>
+        <v>599</v>
       </c>
       <c r="K42" s="12" t="n">
-        <v>63.47058823529412</v>
+        <v>24.94444444444444</v>
       </c>
     </row>
     <row r="43">
@@ -2772,11 +2772,11 @@
         </is>
       </c>
       <c r="G46" s="4" t="n">
-        <v>21444</v>
+        <v>22453</v>
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>16/19</t>
+          <t>17/19</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
@@ -2785,10 +2785,10 @@
         </is>
       </c>
       <c r="J46" s="4" t="n">
-        <v>25465</v>
+        <v>25095</v>
       </c>
       <c r="K46" s="5" t="n">
-        <v>1340.25</v>
+        <v>1320.764705882353</v>
       </c>
     </row>
     <row r="47">
@@ -2821,11 +2821,11 @@
         </is>
       </c>
       <c r="G47" s="4" t="n">
-        <v>16032</v>
+        <v>17047</v>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>13/24</t>
+          <t>14/24</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
@@ -2834,10 +2834,10 @@
         </is>
       </c>
       <c r="J47" s="4" t="n">
-        <v>29598</v>
+        <v>29223</v>
       </c>
       <c r="K47" s="5" t="n">
-        <v>1233.230769230769</v>
+        <v>1217.642857142857</v>
       </c>
     </row>
     <row r="48">
@@ -2919,11 +2919,11 @@
         </is>
       </c>
       <c r="G49" s="4" t="n">
-        <v>13557</v>
+        <v>13359</v>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>12/20</t>
+          <t>13/20</t>
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr">
@@ -2932,10 +2932,10 @@
         </is>
       </c>
       <c r="J49" s="4" t="n">
-        <v>22595</v>
+        <v>20552</v>
       </c>
       <c r="K49" s="5" t="n">
-        <v>1129.75</v>
+        <v>1027.615384615385</v>
       </c>
     </row>
     <row r="50">
@@ -2968,11 +2968,11 @@
         </is>
       </c>
       <c r="G50" s="7" t="n">
-        <v>5587</v>
+        <v>6363</v>
       </c>
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>8/23</t>
+          <t>9/23</t>
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr">
@@ -2981,10 +2981,10 @@
         </is>
       </c>
       <c r="J50" s="7" t="n">
-        <v>16063</v>
+        <v>16261</v>
       </c>
       <c r="K50" s="8" t="n">
-        <v>698.375</v>
+        <v>707</v>
       </c>
     </row>
     <row r="51">
@@ -3017,11 +3017,11 @@
         </is>
       </c>
       <c r="G51" s="4" t="n">
-        <v>15616</v>
+        <v>15852</v>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>18/23</t>
+          <t>19/23</t>
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr">
@@ -3030,10 +3030,10 @@
         </is>
       </c>
       <c r="J51" s="4" t="n">
-        <v>19954</v>
+        <v>19189</v>
       </c>
       <c r="K51" s="5" t="n">
-        <v>867.5555555555555</v>
+        <v>834.3157894736842</v>
       </c>
     </row>
     <row r="52">
@@ -3096,30 +3096,30 @@
       </c>
       <c r="C53" s="10" t="inlineStr">
         <is>
+          <t>K.SINDU</t>
+        </is>
+      </c>
+      <c r="D53" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E53" s="10" t="inlineStr">
+        <is>
           <t>K.B.PRADAP</t>
         </is>
       </c>
-      <c r="D53" s="10" t="inlineStr">
+      <c r="F53" s="10" t="inlineStr">
         <is>
           <t>Desiya Murpokku Dravida Kazhagam</t>
         </is>
       </c>
-      <c r="E53" s="10" t="inlineStr">
-        <is>
-          <t>K.SINDU</t>
-        </is>
-      </c>
-      <c r="F53" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
       <c r="G53" s="11" t="n">
-        <v>920</v>
+        <v>1637</v>
       </c>
       <c r="H53" s="10" t="inlineStr">
         <is>
-          <t>14/23</t>
+          <t>15/23</t>
         </is>
       </c>
       <c r="I53" s="10" t="inlineStr">
@@ -3128,10 +3128,10 @@
         </is>
       </c>
       <c r="J53" s="11" t="n">
-        <v>1511</v>
+        <v>2510</v>
       </c>
       <c r="K53" s="12" t="n">
-        <v>65.71428571428571</v>
+        <v>109.1333333333333</v>
       </c>
     </row>
     <row r="54">
@@ -3164,11 +3164,11 @@
         </is>
       </c>
       <c r="G54" s="4" t="n">
-        <v>15549</v>
+        <v>17456</v>
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>13/25</t>
+          <t>14/25</t>
         </is>
       </c>
       <c r="I54" s="3" t="inlineStr">
@@ -3177,10 +3177,10 @@
         </is>
       </c>
       <c r="J54" s="4" t="n">
-        <v>29902</v>
+        <v>31171</v>
       </c>
       <c r="K54" s="5" t="n">
-        <v>1196.076923076923</v>
+        <v>1246.857142857143</v>
       </c>
     </row>
     <row r="55">
@@ -3262,11 +3262,11 @@
         </is>
       </c>
       <c r="G56" s="7" t="n">
-        <v>4248</v>
+        <v>4450</v>
       </c>
       <c r="H56" s="6" t="inlineStr">
         <is>
-          <t>19/23</t>
+          <t>20/23</t>
         </is>
       </c>
       <c r="I56" s="6" t="inlineStr">
@@ -3275,10 +3275,10 @@
         </is>
       </c>
       <c r="J56" s="7" t="n">
-        <v>5142</v>
+        <v>5118</v>
       </c>
       <c r="K56" s="8" t="n">
-        <v>223.578947368421</v>
+        <v>222.5</v>
       </c>
     </row>
     <row r="57">
@@ -3311,11 +3311,11 @@
         </is>
       </c>
       <c r="G57" s="4" t="n">
-        <v>24891</v>
+        <v>24189</v>
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>15/34</t>
+          <t>16/34</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr">
@@ -3324,10 +3324,10 @@
         </is>
       </c>
       <c r="J57" s="4" t="n">
-        <v>56420</v>
+        <v>51402</v>
       </c>
       <c r="K57" s="5" t="n">
-        <v>1659.4</v>
+        <v>1511.8125</v>
       </c>
     </row>
     <row r="58">
@@ -3360,11 +3360,11 @@
         </is>
       </c>
       <c r="G58" s="7" t="n">
-        <v>10437</v>
+        <v>11496</v>
       </c>
       <c r="H58" s="6" t="inlineStr">
         <is>
-          <t>15/23</t>
+          <t>16/23</t>
         </is>
       </c>
       <c r="I58" s="6" t="inlineStr">
@@ -3373,10 +3373,10 @@
         </is>
       </c>
       <c r="J58" s="7" t="n">
-        <v>16003</v>
+        <v>16526</v>
       </c>
       <c r="K58" s="8" t="n">
-        <v>695.8</v>
+        <v>718.5</v>
       </c>
     </row>
     <row r="59">
@@ -3429,52 +3429,52 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="9" t="inlineStr">
+      <c r="A60" s="13" t="inlineStr">
         <is>
           <t>KADAYANALLUR</t>
         </is>
       </c>
-      <c r="B60" s="10" t="n">
+      <c r="B60" s="14" t="n">
         <v>221</v>
       </c>
-      <c r="C60" s="10" t="inlineStr">
+      <c r="C60" s="14" t="inlineStr">
         <is>
           <t>RAJENDRAN. T. M</t>
         </is>
       </c>
-      <c r="D60" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E60" s="10" t="inlineStr">
+      <c r="D60" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E60" s="14" t="inlineStr">
         <is>
           <t>C. KRISHNAMURALI</t>
         </is>
       </c>
-      <c r="F60" s="10" t="inlineStr">
+      <c r="F60" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G60" s="11" t="n">
-        <v>1162</v>
-      </c>
-      <c r="H60" s="10" t="inlineStr">
-        <is>
-          <t>13/26</t>
-        </is>
-      </c>
-      <c r="I60" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J60" s="11" t="n">
-        <v>2324</v>
-      </c>
-      <c r="K60" s="12" t="n">
-        <v>89.38461538461539</v>
+      <c r="G60" s="15" t="n">
+        <v>193</v>
+      </c>
+      <c r="H60" s="14" t="inlineStr">
+        <is>
+          <t>14/26</t>
+        </is>
+      </c>
+      <c r="I60" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J60" s="15" t="n">
+        <v>358</v>
+      </c>
+      <c r="K60" s="16" t="n">
+        <v>13.78571428571429</v>
       </c>
     </row>
     <row r="61">
@@ -3556,11 +3556,11 @@
         </is>
       </c>
       <c r="G62" s="7" t="n">
-        <v>3444</v>
+        <v>3031</v>
       </c>
       <c r="H62" s="6" t="inlineStr">
         <is>
-          <t>13/27</t>
+          <t>14/27</t>
         </is>
       </c>
       <c r="I62" s="6" t="inlineStr">
@@ -3569,10 +3569,10 @@
         </is>
       </c>
       <c r="J62" s="7" t="n">
-        <v>7153</v>
+        <v>5846</v>
       </c>
       <c r="K62" s="8" t="n">
-        <v>264.9230769230769</v>
+        <v>216.5</v>
       </c>
     </row>
     <row r="63">
@@ -3605,11 +3605,11 @@
         </is>
       </c>
       <c r="G63" s="7" t="n">
-        <v>3500</v>
+        <v>5188</v>
       </c>
       <c r="H63" s="6" t="inlineStr">
         <is>
-          <t>12/26</t>
+          <t>13/26</t>
         </is>
       </c>
       <c r="I63" s="6" t="inlineStr">
@@ -3618,10 +3618,10 @@
         </is>
       </c>
       <c r="J63" s="7" t="n">
-        <v>7583</v>
+        <v>10376</v>
       </c>
       <c r="K63" s="8" t="n">
-        <v>291.6666666666667</v>
+        <v>399.0769230769231</v>
       </c>
     </row>
     <row r="64">
@@ -3703,11 +3703,11 @@
         </is>
       </c>
       <c r="G65" s="7" t="n">
-        <v>5167</v>
+        <v>5180</v>
       </c>
       <c r="H65" s="6" t="inlineStr">
         <is>
-          <t>14/26</t>
+          <t>15/26</t>
         </is>
       </c>
       <c r="I65" s="6" t="inlineStr">
@@ -3716,10 +3716,10 @@
         </is>
       </c>
       <c r="J65" s="7" t="n">
-        <v>9596</v>
+        <v>8979</v>
       </c>
       <c r="K65" s="8" t="n">
-        <v>369.0714285714286</v>
+        <v>345.3333333333334</v>
       </c>
     </row>
     <row r="66">
@@ -3978,30 +3978,30 @@
       </c>
       <c r="C71" s="14" t="inlineStr">
         <is>
+          <t>RAJESH KUMAR. S</t>
+        </is>
+      </c>
+      <c r="D71" s="14" t="inlineStr">
+        <is>
+          <t>Indian National Congress</t>
+        </is>
+      </c>
+      <c r="E71" s="14" t="inlineStr">
+        <is>
           <t>SABIN. S</t>
         </is>
       </c>
-      <c r="D71" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E71" s="14" t="inlineStr">
-        <is>
-          <t>RAJESH KUMAR. S</t>
-        </is>
-      </c>
       <c r="F71" s="14" t="inlineStr">
         <is>
-          <t>Indian National Congress</t>
+          <t>Tamilaga Vettri Kazhagam</t>
         </is>
       </c>
       <c r="G71" s="15" t="n">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="H71" s="14" t="inlineStr">
         <is>
-          <t>13/22</t>
+          <t>14/22</t>
         </is>
       </c>
       <c r="I71" s="14" t="inlineStr">
@@ -4010,10 +4010,10 @@
         </is>
       </c>
       <c r="J71" s="15" t="n">
-        <v>256</v>
+        <v>225</v>
       </c>
       <c r="K71" s="16" t="n">
-        <v>11.61538461538461</v>
+        <v>10.21428571428571</v>
       </c>
     </row>
     <row r="72">
@@ -4046,11 +4046,11 @@
         </is>
       </c>
       <c r="G72" s="4" t="n">
-        <v>28935</v>
+        <v>27814</v>
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>16/22</t>
+          <t>17/22</t>
         </is>
       </c>
       <c r="I72" s="3" t="inlineStr">
@@ -4059,10 +4059,10 @@
         </is>
       </c>
       <c r="J72" s="4" t="n">
-        <v>39786</v>
+        <v>35995</v>
       </c>
       <c r="K72" s="5" t="n">
-        <v>1808.4375</v>
+        <v>1636.117647058823</v>
       </c>
     </row>
     <row r="73">
@@ -4144,11 +4144,11 @@
         </is>
       </c>
       <c r="G74" s="11" t="n">
-        <v>1667</v>
+        <v>425</v>
       </c>
       <c r="H74" s="10" t="inlineStr">
         <is>
-          <t>9/16</t>
+          <t>10/16</t>
         </is>
       </c>
       <c r="I74" s="10" t="inlineStr">
@@ -4157,10 +4157,10 @@
         </is>
       </c>
       <c r="J74" s="11" t="n">
-        <v>2964</v>
+        <v>680</v>
       </c>
       <c r="K74" s="12" t="n">
-        <v>185.2222222222222</v>
+        <v>42.5</v>
       </c>
     </row>
     <row r="75">
@@ -4193,11 +4193,11 @@
         </is>
       </c>
       <c r="G75" s="4" t="n">
-        <v>12501</v>
+        <v>13039</v>
       </c>
       <c r="H75" s="3" t="inlineStr">
         <is>
-          <t>25/28</t>
+          <t>26/28</t>
         </is>
       </c>
       <c r="I75" s="3" t="inlineStr">
@@ -4206,10 +4206,10 @@
         </is>
       </c>
       <c r="J75" s="4" t="n">
-        <v>14001</v>
+        <v>14042</v>
       </c>
       <c r="K75" s="5" t="n">
-        <v>500.04</v>
+        <v>501.5</v>
       </c>
     </row>
     <row r="76">
@@ -4242,11 +4242,11 @@
         </is>
       </c>
       <c r="G76" s="7" t="n">
-        <v>7074</v>
+        <v>7544</v>
       </c>
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>15/22</t>
+          <t>16/22</t>
         </is>
       </c>
       <c r="I76" s="6" t="inlineStr">
@@ -4255,10 +4255,10 @@
         </is>
       </c>
       <c r="J76" s="7" t="n">
-        <v>10375</v>
+        <v>10373</v>
       </c>
       <c r="K76" s="8" t="n">
-        <v>471.6000000000001</v>
+        <v>471.5</v>
       </c>
     </row>
     <row r="77">
@@ -4340,11 +4340,11 @@
         </is>
       </c>
       <c r="G78" s="4" t="n">
-        <v>18131</v>
+        <v>18582</v>
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
-          <t>19/25</t>
+          <t>20/25</t>
         </is>
       </c>
       <c r="I78" s="3" t="inlineStr">
@@ -4353,10 +4353,10 @@
         </is>
       </c>
       <c r="J78" s="4" t="n">
-        <v>23857</v>
+        <v>23228</v>
       </c>
       <c r="K78" s="5" t="n">
-        <v>954.2631578947369</v>
+        <v>929.1</v>
       </c>
     </row>
     <row r="79">
@@ -4409,52 +4409,52 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="9" t="inlineStr">
+      <c r="A80" s="6" t="inlineStr">
         <is>
           <t>KULITHALAI</t>
         </is>
       </c>
-      <c r="B80" s="10" t="n">
+      <c r="B80" s="6" t="n">
         <v>137</v>
       </c>
-      <c r="C80" s="10" t="inlineStr">
+      <c r="C80" s="6" t="inlineStr">
         <is>
           <t>G.BALASUBRAMANI</t>
         </is>
       </c>
-      <c r="D80" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E80" s="10" t="inlineStr">
+      <c r="D80" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E80" s="6" t="inlineStr">
         <is>
           <t>SURIYANUR. A. CHANDRAN</t>
         </is>
       </c>
-      <c r="F80" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G80" s="11" t="n">
-        <v>1825</v>
-      </c>
-      <c r="H80" s="10" t="inlineStr">
-        <is>
-          <t>13/21</t>
-        </is>
-      </c>
-      <c r="I80" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J80" s="11" t="n">
-        <v>2948</v>
-      </c>
-      <c r="K80" s="12" t="n">
-        <v>140.3846153846154</v>
+      <c r="F80" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G80" s="7" t="n">
+        <v>2256</v>
+      </c>
+      <c r="H80" s="6" t="inlineStr">
+        <is>
+          <t>14/21</t>
+        </is>
+      </c>
+      <c r="I80" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J80" s="7" t="n">
+        <v>3384</v>
+      </c>
+      <c r="K80" s="8" t="n">
+        <v>161.1428571428571</v>
       </c>
     </row>
     <row r="81">
@@ -4487,11 +4487,11 @@
         </is>
       </c>
       <c r="G81" s="7" t="n">
-        <v>2093</v>
+        <v>1927</v>
       </c>
       <c r="H81" s="6" t="inlineStr">
         <is>
-          <t>12/24</t>
+          <t>13/24</t>
         </is>
       </c>
       <c r="I81" s="6" t="inlineStr">
@@ -4500,10 +4500,10 @@
         </is>
       </c>
       <c r="J81" s="7" t="n">
-        <v>4186</v>
+        <v>3558</v>
       </c>
       <c r="K81" s="8" t="n">
-        <v>174.4166666666667</v>
+        <v>148.2307692307692</v>
       </c>
     </row>
     <row r="82">
@@ -4585,11 +4585,11 @@
         </is>
       </c>
       <c r="G83" s="4" t="n">
-        <v>14893</v>
+        <v>15608</v>
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
-          <t>16/25</t>
+          <t>17/25</t>
         </is>
       </c>
       <c r="I83" s="3" t="inlineStr">
@@ -4598,10 +4598,10 @@
         </is>
       </c>
       <c r="J83" s="4" t="n">
-        <v>23270</v>
+        <v>22953</v>
       </c>
       <c r="K83" s="5" t="n">
-        <v>930.8125</v>
+        <v>918.1176470588235</v>
       </c>
     </row>
     <row r="84">
@@ -4634,11 +4634,11 @@
         </is>
       </c>
       <c r="G84" s="7" t="n">
-        <v>2195</v>
+        <v>2732</v>
       </c>
       <c r="H84" s="6" t="inlineStr">
         <is>
-          <t>14/20</t>
+          <t>15/20</t>
         </is>
       </c>
       <c r="I84" s="6" t="inlineStr">
@@ -4647,10 +4647,10 @@
         </is>
       </c>
       <c r="J84" s="7" t="n">
-        <v>3136</v>
+        <v>3643</v>
       </c>
       <c r="K84" s="8" t="n">
-        <v>156.7857142857143</v>
+        <v>182.1333333333333</v>
       </c>
     </row>
     <row r="85">
@@ -4683,11 +4683,11 @@
         </is>
       </c>
       <c r="G85" s="11" t="n">
-        <v>974</v>
+        <v>1174</v>
       </c>
       <c r="H85" s="10" t="inlineStr">
         <is>
-          <t>13/20</t>
+          <t>14/20</t>
         </is>
       </c>
       <c r="I85" s="10" t="inlineStr">
@@ -4696,10 +4696,10 @@
         </is>
       </c>
       <c r="J85" s="11" t="n">
-        <v>1498</v>
+        <v>1677</v>
       </c>
       <c r="K85" s="12" t="n">
-        <v>74.92307692307692</v>
+        <v>83.85714285714286</v>
       </c>
     </row>
     <row r="86">
@@ -4732,11 +4732,11 @@
         </is>
       </c>
       <c r="G86" s="7" t="n">
-        <v>3678</v>
+        <v>4567</v>
       </c>
       <c r="H86" s="6" t="inlineStr">
         <is>
-          <t>11/21</t>
+          <t>12/21</t>
         </is>
       </c>
       <c r="I86" s="6" t="inlineStr">
@@ -4745,10 +4745,10 @@
         </is>
       </c>
       <c r="J86" s="7" t="n">
-        <v>7022</v>
+        <v>7992</v>
       </c>
       <c r="K86" s="8" t="n">
-        <v>334.3636363636364</v>
+        <v>380.5833333333333</v>
       </c>
     </row>
     <row r="87">
@@ -4781,11 +4781,11 @@
         </is>
       </c>
       <c r="G87" s="4" t="n">
-        <v>79885</v>
+        <v>86172</v>
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
-          <t>16/19</t>
+          <t>17/19</t>
         </is>
       </c>
       <c r="I87" s="3" t="inlineStr">
@@ -4794,10 +4794,10 @@
         </is>
       </c>
       <c r="J87" s="4" t="n">
-        <v>94863</v>
+        <v>96310</v>
       </c>
       <c r="K87" s="5" t="n">
-        <v>4992.8125</v>
+        <v>5068.941176470588</v>
       </c>
     </row>
     <row r="88">
@@ -4830,11 +4830,11 @@
         </is>
       </c>
       <c r="G88" s="4" t="n">
-        <v>16020</v>
+        <v>15901</v>
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>10/19</t>
+          <t>11/19</t>
         </is>
       </c>
       <c r="I88" s="3" t="inlineStr">
@@ -4843,10 +4843,10 @@
         </is>
       </c>
       <c r="J88" s="4" t="n">
-        <v>30438</v>
+        <v>27465</v>
       </c>
       <c r="K88" s="5" t="n">
-        <v>1602</v>
+        <v>1445.545454545455</v>
       </c>
     </row>
     <row r="89">
@@ -4928,11 +4928,11 @@
         </is>
       </c>
       <c r="G90" s="4" t="n">
-        <v>14435</v>
+        <v>14739</v>
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>13/19</t>
+          <t>14/19</t>
         </is>
       </c>
       <c r="I90" s="3" t="inlineStr">
@@ -4941,10 +4941,10 @@
         </is>
       </c>
       <c r="J90" s="4" t="n">
-        <v>21097</v>
+        <v>20003</v>
       </c>
       <c r="K90" s="5" t="n">
-        <v>1110.384615384615</v>
+        <v>1052.785714285714</v>
       </c>
     </row>
     <row r="91">
@@ -4977,11 +4977,11 @@
         </is>
       </c>
       <c r="G91" s="4" t="n">
-        <v>20023</v>
+        <v>21529</v>
       </c>
       <c r="H91" s="3" t="inlineStr">
         <is>
-          <t>16/17</t>
+          <t>17/17</t>
         </is>
       </c>
       <c r="I91" s="3" t="inlineStr">
@@ -4990,10 +4990,10 @@
         </is>
       </c>
       <c r="J91" s="4" t="n">
-        <v>21274</v>
+        <v>21529</v>
       </c>
       <c r="K91" s="5" t="n">
-        <v>1251.4375</v>
+        <v>1266.411764705882</v>
       </c>
     </row>
     <row r="92">
@@ -5124,11 +5124,11 @@
         </is>
       </c>
       <c r="G94" s="4" t="n">
-        <v>26286</v>
+        <v>29024</v>
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
-          <t>9/25</t>
+          <t>10/25</t>
         </is>
       </c>
       <c r="I94" s="3" t="inlineStr">
@@ -5137,10 +5137,10 @@
         </is>
       </c>
       <c r="J94" s="4" t="n">
-        <v>73017</v>
+        <v>72560</v>
       </c>
       <c r="K94" s="5" t="n">
-        <v>2920.666666666667</v>
+        <v>2902.4</v>
       </c>
     </row>
     <row r="95">
@@ -5222,11 +5222,11 @@
         </is>
       </c>
       <c r="G96" s="4" t="n">
-        <v>9716</v>
+        <v>10155</v>
       </c>
       <c r="H96" s="3" t="inlineStr">
         <is>
-          <t>18/22</t>
+          <t>19/22</t>
         </is>
       </c>
       <c r="I96" s="3" t="inlineStr">
@@ -5235,10 +5235,10 @@
         </is>
       </c>
       <c r="J96" s="4" t="n">
-        <v>11875</v>
+        <v>11758</v>
       </c>
       <c r="K96" s="5" t="n">
-        <v>539.7777777777778</v>
+        <v>534.4736842105264</v>
       </c>
     </row>
     <row r="97">
@@ -5301,30 +5301,30 @@
       </c>
       <c r="C98" s="14" t="inlineStr">
         <is>
+          <t>R. KATHIRAVAN</t>
+        </is>
+      </c>
+      <c r="D98" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E98" s="14" t="inlineStr">
+        <is>
           <t>DR. PL. VIJAYAKUMAR</t>
         </is>
       </c>
-      <c r="D98" s="14" t="inlineStr">
+      <c r="F98" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E98" s="14" t="inlineStr">
-        <is>
-          <t>R. KATHIRAVAN</t>
-        </is>
-      </c>
-      <c r="F98" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
       <c r="G98" s="15" t="n">
-        <v>293</v>
+        <v>31</v>
       </c>
       <c r="H98" s="14" t="inlineStr">
         <is>
-          <t>19/25</t>
+          <t>20/25</t>
         </is>
       </c>
       <c r="I98" s="14" t="inlineStr">
@@ -5333,10 +5333,10 @@
         </is>
       </c>
       <c r="J98" s="15" t="n">
-        <v>386</v>
+        <v>39</v>
       </c>
       <c r="K98" s="16" t="n">
-        <v>15.42105263157895</v>
+        <v>1.55</v>
       </c>
     </row>
     <row r="99">
@@ -5418,11 +5418,11 @@
         </is>
       </c>
       <c r="G100" s="7" t="n">
-        <v>7147</v>
+        <v>8004</v>
       </c>
       <c r="H100" s="6" t="inlineStr">
         <is>
-          <t>13/22</t>
+          <t>14/22</t>
         </is>
       </c>
       <c r="I100" s="6" t="inlineStr">
@@ -5431,10 +5431,10 @@
         </is>
       </c>
       <c r="J100" s="7" t="n">
-        <v>12095</v>
+        <v>12578</v>
       </c>
       <c r="K100" s="8" t="n">
-        <v>549.7692307692307</v>
+        <v>571.7142857142857</v>
       </c>
     </row>
     <row r="101">
@@ -5487,101 +5487,101 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="13" t="inlineStr">
+      <c r="A102" s="9" t="inlineStr">
         <is>
           <t>METTUPPALAYAM</t>
         </is>
       </c>
-      <c r="B102" s="14" t="n">
+      <c r="B102" s="10" t="n">
         <v>111</v>
       </c>
-      <c r="C102" s="14" t="inlineStr">
+      <c r="C102" s="10" t="inlineStr">
         <is>
           <t>SUNILANAND</t>
         </is>
       </c>
-      <c r="D102" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E102" s="14" t="inlineStr">
+      <c r="D102" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E102" s="10" t="inlineStr">
         <is>
           <t>SMT.KAVITHA KALYANASUNDARAM</t>
         </is>
       </c>
-      <c r="F102" s="14" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G102" s="15" t="n">
-        <v>52</v>
-      </c>
-      <c r="H102" s="14" t="inlineStr">
-        <is>
-          <t>14/26</t>
-        </is>
-      </c>
-      <c r="I102" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J102" s="15" t="n">
-        <v>97</v>
-      </c>
-      <c r="K102" s="16" t="n">
-        <v>3.714285714285714</v>
+      <c r="F102" s="10" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G102" s="11" t="n">
+        <v>637</v>
+      </c>
+      <c r="H102" s="10" t="inlineStr">
+        <is>
+          <t>15/26</t>
+        </is>
+      </c>
+      <c r="I102" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J102" s="11" t="n">
+        <v>1104</v>
+      </c>
+      <c r="K102" s="12" t="n">
+        <v>42.46666666666667</v>
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="9" t="inlineStr">
+      <c r="A103" s="13" t="inlineStr">
         <is>
           <t>METTUR</t>
         </is>
       </c>
-      <c r="B103" s="10" t="n">
+      <c r="B103" s="14" t="n">
         <v>85</v>
       </c>
-      <c r="C103" s="10" t="inlineStr">
+      <c r="C103" s="14" t="inlineStr">
+        <is>
+          <t>VENKATACHALAM. G</t>
+        </is>
+      </c>
+      <c r="D103" s="14" t="inlineStr">
+        <is>
+          <t>All India Anna Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E103" s="14" t="inlineStr">
         <is>
           <t>MIDHUN CHAKRAVARTHY. M</t>
         </is>
       </c>
-      <c r="D103" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E103" s="10" t="inlineStr">
-        <is>
-          <t>VENKATACHALAM. G</t>
-        </is>
-      </c>
-      <c r="F103" s="10" t="inlineStr">
-        <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G103" s="11" t="n">
-        <v>869</v>
-      </c>
-      <c r="H103" s="10" t="inlineStr">
-        <is>
-          <t>11/24</t>
-        </is>
-      </c>
-      <c r="I103" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J103" s="11" t="n">
-        <v>1896</v>
-      </c>
-      <c r="K103" s="12" t="n">
-        <v>79</v>
+      <c r="F103" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G103" s="15" t="n">
+        <v>161</v>
+      </c>
+      <c r="H103" s="14" t="inlineStr">
+        <is>
+          <t>12/24</t>
+        </is>
+      </c>
+      <c r="I103" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J103" s="15" t="n">
+        <v>322</v>
+      </c>
+      <c r="K103" s="16" t="n">
+        <v>13.41666666666667</v>
       </c>
     </row>
     <row r="104">
@@ -5614,11 +5614,11 @@
         </is>
       </c>
       <c r="G104" s="7" t="n">
-        <v>3383</v>
+        <v>3563</v>
       </c>
       <c r="H104" s="6" t="inlineStr">
         <is>
-          <t>15/21</t>
+          <t>16/21</t>
         </is>
       </c>
       <c r="I104" s="6" t="inlineStr">
@@ -5627,10 +5627,10 @@
         </is>
       </c>
       <c r="J104" s="7" t="n">
-        <v>4736</v>
+        <v>4676</v>
       </c>
       <c r="K104" s="8" t="n">
-        <v>225.5333333333333</v>
+        <v>222.6875</v>
       </c>
     </row>
     <row r="105">
@@ -5654,20 +5654,20 @@
       </c>
       <c r="E105" s="6" t="inlineStr">
         <is>
-          <t>S.PANDI</t>
+          <t>MALARVIZHI. B</t>
         </is>
       </c>
       <c r="F105" s="6" t="inlineStr">
         <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
+          <t>Tamilaga Vettri Kazhagam</t>
         </is>
       </c>
       <c r="G105" s="7" t="n">
-        <v>9495</v>
+        <v>11364</v>
       </c>
       <c r="H105" s="6" t="inlineStr">
         <is>
-          <t>18/30</t>
+          <t>19/30</t>
         </is>
       </c>
       <c r="I105" s="6" t="inlineStr">
@@ -5676,10 +5676,10 @@
         </is>
       </c>
       <c r="J105" s="7" t="n">
-        <v>15825</v>
+        <v>17943</v>
       </c>
       <c r="K105" s="8" t="n">
-        <v>527.5</v>
+        <v>598.1052631578947</v>
       </c>
     </row>
     <row r="106">
@@ -5761,11 +5761,11 @@
         </is>
       </c>
       <c r="G107" s="4" t="n">
-        <v>23844</v>
+        <v>25547</v>
       </c>
       <c r="H107" s="3" t="inlineStr">
         <is>
-          <t>16/20</t>
+          <t>17/20</t>
         </is>
       </c>
       <c r="I107" s="3" t="inlineStr">
@@ -5774,59 +5774,59 @@
         </is>
       </c>
       <c r="J107" s="4" t="n">
-        <v>29805</v>
+        <v>30055</v>
       </c>
       <c r="K107" s="5" t="n">
-        <v>1490.25</v>
+        <v>1502.764705882353</v>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="6" t="inlineStr">
+      <c r="A108" s="2" t="inlineStr">
         <is>
           <t>NAGAPATTINAM</t>
         </is>
       </c>
-      <c r="B108" s="6" t="n">
+      <c r="B108" s="3" t="n">
         <v>163</v>
       </c>
-      <c r="C108" s="6" t="inlineStr">
+      <c r="C108" s="3" t="inlineStr">
         <is>
           <t>M.H.JAWAHIRULLAH</t>
         </is>
       </c>
-      <c r="D108" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E108" s="6" t="inlineStr">
+      <c r="D108" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E108" s="3" t="inlineStr">
         <is>
           <t>THANKA.KATHIRAVAN</t>
         </is>
       </c>
-      <c r="F108" s="6" t="inlineStr">
+      <c r="F108" s="3" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G108" s="7" t="n">
-        <v>8201</v>
-      </c>
-      <c r="H108" s="6" t="inlineStr">
-        <is>
-          <t>8/18</t>
-        </is>
-      </c>
-      <c r="I108" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J108" s="7" t="n">
-        <v>18452</v>
-      </c>
-      <c r="K108" s="8" t="n">
-        <v>1025.125</v>
+      <c r="G108" s="4" t="n">
+        <v>11757</v>
+      </c>
+      <c r="H108" s="3" t="inlineStr">
+        <is>
+          <t>9/18</t>
+        </is>
+      </c>
+      <c r="I108" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J108" s="4" t="n">
+        <v>23514</v>
+      </c>
+      <c r="K108" s="5" t="n">
+        <v>1306.333333333333</v>
       </c>
     </row>
     <row r="109">
@@ -5859,11 +5859,11 @@
         </is>
       </c>
       <c r="G109" s="7" t="n">
-        <v>4175</v>
+        <v>4719</v>
       </c>
       <c r="H109" s="6" t="inlineStr">
         <is>
-          <t>16/23</t>
+          <t>17/23</t>
         </is>
       </c>
       <c r="I109" s="6" t="inlineStr">
@@ -5872,10 +5872,10 @@
         </is>
       </c>
       <c r="J109" s="7" t="n">
-        <v>6002</v>
+        <v>6385</v>
       </c>
       <c r="K109" s="8" t="n">
-        <v>260.9375</v>
+        <v>277.5882352941176</v>
       </c>
     </row>
     <row r="110">
@@ -5889,30 +5889,30 @@
       </c>
       <c r="C110" s="10" t="inlineStr">
         <is>
+          <t>DILIP C S</t>
+        </is>
+      </c>
+      <c r="D110" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E110" s="10" t="inlineStr">
+        <is>
           <t>SRIDEVI MOHAN P S</t>
         </is>
       </c>
-      <c r="D110" s="10" t="inlineStr">
+      <c r="F110" s="10" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E110" s="10" t="inlineStr">
-        <is>
-          <t>DILIP C S</t>
-        </is>
-      </c>
-      <c r="F110" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
       <c r="G110" s="11" t="n">
-        <v>502</v>
+        <v>446</v>
       </c>
       <c r="H110" s="10" t="inlineStr">
         <is>
-          <t>9/23</t>
+          <t>10/23</t>
         </is>
       </c>
       <c r="I110" s="10" t="inlineStr">
@@ -5921,10 +5921,10 @@
         </is>
       </c>
       <c r="J110" s="11" t="n">
-        <v>1283</v>
+        <v>1026</v>
       </c>
       <c r="K110" s="12" t="n">
-        <v>55.77777777777778</v>
+        <v>44.6</v>
       </c>
     </row>
     <row r="111">
@@ -5957,11 +5957,11 @@
         </is>
       </c>
       <c r="G111" s="4" t="n">
-        <v>14216</v>
+        <v>15331</v>
       </c>
       <c r="H111" s="3" t="inlineStr">
         <is>
-          <t>23/25</t>
+          <t>24/25</t>
         </is>
       </c>
       <c r="I111" s="3" t="inlineStr">
@@ -5970,10 +5970,10 @@
         </is>
       </c>
       <c r="J111" s="4" t="n">
-        <v>15452</v>
+        <v>15970</v>
       </c>
       <c r="K111" s="5" t="n">
-        <v>618.0869565217391</v>
+        <v>638.7916666666666</v>
       </c>
     </row>
     <row r="112">
@@ -6046,20 +6046,20 @@
       </c>
       <c r="E113" s="6" t="inlineStr">
         <is>
-          <t>RAMESH L N</t>
+          <t>SELVAKUMAR K</t>
         </is>
       </c>
       <c r="F113" s="6" t="inlineStr">
         <is>
-          <t>Tamilaga Vettri Kazhagam</t>
+          <t>Dravida Munnetra Kazhagam</t>
         </is>
       </c>
       <c r="G113" s="7" t="n">
-        <v>8937</v>
+        <v>10382</v>
       </c>
       <c r="H113" s="6" t="inlineStr">
         <is>
-          <t>16/26</t>
+          <t>17/26</t>
         </is>
       </c>
       <c r="I113" s="6" t="inlineStr">
@@ -6068,10 +6068,10 @@
         </is>
       </c>
       <c r="J113" s="7" t="n">
-        <v>14523</v>
+        <v>15878</v>
       </c>
       <c r="K113" s="8" t="n">
-        <v>558.5625</v>
+        <v>610.7058823529412</v>
       </c>
     </row>
     <row r="114">
@@ -6104,11 +6104,11 @@
         </is>
       </c>
       <c r="G114" s="4" t="n">
-        <v>11169</v>
+        <v>11002</v>
       </c>
       <c r="H114" s="3" t="inlineStr">
         <is>
-          <t>15/19</t>
+          <t>16/19</t>
         </is>
       </c>
       <c r="I114" s="3" t="inlineStr">
@@ -6117,10 +6117,10 @@
         </is>
       </c>
       <c r="J114" s="4" t="n">
-        <v>14147</v>
+        <v>13065</v>
       </c>
       <c r="K114" s="5" t="n">
-        <v>744.6</v>
+        <v>687.625</v>
       </c>
     </row>
     <row r="115">
@@ -6202,11 +6202,11 @@
         </is>
       </c>
       <c r="G116" s="4" t="n">
-        <v>26282</v>
+        <v>28835</v>
       </c>
       <c r="H116" s="3" t="inlineStr">
         <is>
-          <t>15/24</t>
+          <t>16/24</t>
         </is>
       </c>
       <c r="I116" s="3" t="inlineStr">
@@ -6215,10 +6215,10 @@
         </is>
       </c>
       <c r="J116" s="4" t="n">
-        <v>42051</v>
+        <v>43252</v>
       </c>
       <c r="K116" s="5" t="n">
-        <v>1752.133333333333</v>
+        <v>1802.1875</v>
       </c>
     </row>
     <row r="117">
@@ -6251,11 +6251,11 @@
         </is>
       </c>
       <c r="G117" s="7" t="n">
-        <v>5630</v>
+        <v>7988</v>
       </c>
       <c r="H117" s="6" t="inlineStr">
         <is>
-          <t>16/26</t>
+          <t>17/26</t>
         </is>
       </c>
       <c r="I117" s="6" t="inlineStr">
@@ -6264,10 +6264,10 @@
         </is>
       </c>
       <c r="J117" s="7" t="n">
-        <v>9149</v>
+        <v>12217</v>
       </c>
       <c r="K117" s="8" t="n">
-        <v>351.875</v>
+        <v>469.8823529411765</v>
       </c>
     </row>
     <row r="118">
@@ -6300,11 +6300,11 @@
         </is>
       </c>
       <c r="G118" s="4" t="n">
-        <v>28750</v>
+        <v>30266</v>
       </c>
       <c r="H118" s="3" t="inlineStr">
         <is>
-          <t>19/23</t>
+          <t>20/23</t>
         </is>
       </c>
       <c r="I118" s="3" t="inlineStr">
@@ -6313,10 +6313,10 @@
         </is>
       </c>
       <c r="J118" s="4" t="n">
-        <v>34803</v>
+        <v>34806</v>
       </c>
       <c r="K118" s="5" t="n">
-        <v>1513.157894736842</v>
+        <v>1513.3</v>
       </c>
     </row>
     <row r="119">
@@ -6398,11 +6398,11 @@
         </is>
       </c>
       <c r="G120" s="7" t="n">
-        <v>9725</v>
+        <v>10209</v>
       </c>
       <c r="H120" s="6" t="inlineStr">
         <is>
-          <t>14/23</t>
+          <t>15/23</t>
         </is>
       </c>
       <c r="I120" s="6" t="inlineStr">
@@ -6411,10 +6411,10 @@
         </is>
       </c>
       <c r="J120" s="7" t="n">
-        <v>15977</v>
+        <v>15654</v>
       </c>
       <c r="K120" s="8" t="n">
-        <v>694.6428571428571</v>
+        <v>680.6</v>
       </c>
     </row>
     <row r="121">
@@ -6496,11 +6496,11 @@
         </is>
       </c>
       <c r="G122" s="7" t="n">
-        <v>3336</v>
+        <v>2886</v>
       </c>
       <c r="H122" s="6" t="inlineStr">
         <is>
-          <t>16/25</t>
+          <t>17/25</t>
         </is>
       </c>
       <c r="I122" s="6" t="inlineStr">
@@ -6509,59 +6509,59 @@
         </is>
       </c>
       <c r="J122" s="7" t="n">
-        <v>5212</v>
+        <v>4244</v>
       </c>
       <c r="K122" s="8" t="n">
-        <v>208.5</v>
+        <v>169.7647058823529</v>
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="6" t="inlineStr">
+      <c r="A123" s="2" t="inlineStr">
         <is>
           <t>PALAYAMKOTTAI</t>
         </is>
       </c>
-      <c r="B123" s="6" t="n">
+      <c r="B123" s="3" t="n">
         <v>226</v>
       </c>
-      <c r="C123" s="6" t="inlineStr">
+      <c r="C123" s="3" t="inlineStr">
         <is>
           <t>M.ABDUL WAHAB</t>
         </is>
       </c>
-      <c r="D123" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E123" s="6" t="inlineStr">
+      <c r="D123" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E123" s="3" t="inlineStr">
         <is>
           <t>MARIA JOHN</t>
         </is>
       </c>
-      <c r="F123" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G123" s="7" t="n">
-        <v>4845</v>
-      </c>
-      <c r="H123" s="6" t="inlineStr">
-        <is>
-          <t>19/22</t>
-        </is>
-      </c>
-      <c r="I123" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J123" s="7" t="n">
-        <v>5610</v>
-      </c>
-      <c r="K123" s="8" t="n">
-        <v>255</v>
+      <c r="F123" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G123" s="4" t="n">
+        <v>8903</v>
+      </c>
+      <c r="H123" s="3" t="inlineStr">
+        <is>
+          <t>20/22</t>
+        </is>
+      </c>
+      <c r="I123" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J123" s="4" t="n">
+        <v>9793</v>
+      </c>
+      <c r="K123" s="5" t="n">
+        <v>445.15</v>
       </c>
     </row>
     <row r="124">
@@ -6594,11 +6594,11 @@
         </is>
       </c>
       <c r="G124" s="4" t="n">
-        <v>27678</v>
+        <v>30529</v>
       </c>
       <c r="H124" s="3" t="inlineStr">
         <is>
-          <t>21/35</t>
+          <t>22/35</t>
         </is>
       </c>
       <c r="I124" s="3" t="inlineStr">
@@ -6607,10 +6607,10 @@
         </is>
       </c>
       <c r="J124" s="4" t="n">
-        <v>46130</v>
+        <v>48569</v>
       </c>
       <c r="K124" s="5" t="n">
-        <v>1318</v>
+        <v>1387.681818181818</v>
       </c>
     </row>
     <row r="125">
@@ -6790,11 +6790,11 @@
         </is>
       </c>
       <c r="G128" s="4" t="n">
-        <v>35159</v>
+        <v>34889</v>
       </c>
       <c r="H128" s="3" t="inlineStr">
         <is>
-          <t>18/23</t>
+          <t>19/23</t>
         </is>
       </c>
       <c r="I128" s="3" t="inlineStr">
@@ -6803,10 +6803,10 @@
         </is>
       </c>
       <c r="J128" s="4" t="n">
-        <v>44925</v>
+        <v>42234</v>
       </c>
       <c r="K128" s="5" t="n">
-        <v>1953.277777777778</v>
+        <v>1836.263157894737</v>
       </c>
     </row>
     <row r="129">
@@ -6928,20 +6928,20 @@
       </c>
       <c r="E131" s="6" t="inlineStr">
         <is>
-          <t>SEKAR C V</t>
+          <t>MATHAN C</t>
         </is>
       </c>
       <c r="F131" s="6" t="inlineStr">
         <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
+          <t>Tamilaga Vettri Kazhagam</t>
         </is>
       </c>
       <c r="G131" s="7" t="n">
-        <v>4737</v>
+        <v>5292</v>
       </c>
       <c r="H131" s="6" t="inlineStr">
         <is>
-          <t>11/23</t>
+          <t>12/23</t>
         </is>
       </c>
       <c r="I131" s="6" t="inlineStr">
@@ -6950,10 +6950,10 @@
         </is>
       </c>
       <c r="J131" s="7" t="n">
-        <v>9905</v>
+        <v>10143</v>
       </c>
       <c r="K131" s="8" t="n">
-        <v>430.6363636363636</v>
+        <v>441</v>
       </c>
     </row>
     <row r="132">
@@ -6986,11 +6986,11 @@
         </is>
       </c>
       <c r="G132" s="7" t="n">
-        <v>2815</v>
+        <v>1933</v>
       </c>
       <c r="H132" s="6" t="inlineStr">
         <is>
-          <t>12/23</t>
+          <t>13/23</t>
         </is>
       </c>
       <c r="I132" s="6" t="inlineStr">
@@ -6999,10 +6999,10 @@
         </is>
       </c>
       <c r="J132" s="7" t="n">
-        <v>5395</v>
+        <v>3420</v>
       </c>
       <c r="K132" s="8" t="n">
-        <v>234.5833333333333</v>
+        <v>148.6923076923077</v>
       </c>
     </row>
     <row r="133">
@@ -7035,11 +7035,11 @@
         </is>
       </c>
       <c r="G133" s="7" t="n">
-        <v>8462</v>
+        <v>9318</v>
       </c>
       <c r="H133" s="6" t="inlineStr">
         <is>
-          <t>18/28</t>
+          <t>19/28</t>
         </is>
       </c>
       <c r="I133" s="6" t="inlineStr">
@@ -7048,10 +7048,10 @@
         </is>
       </c>
       <c r="J133" s="7" t="n">
-        <v>13163</v>
+        <v>13732</v>
       </c>
       <c r="K133" s="8" t="n">
-        <v>470.1111111111111</v>
+        <v>490.421052631579</v>
       </c>
     </row>
     <row r="134">
@@ -7084,11 +7084,11 @@
         </is>
       </c>
       <c r="G134" s="4" t="n">
-        <v>23207</v>
+        <v>25723</v>
       </c>
       <c r="H134" s="3" t="inlineStr">
         <is>
-          <t>10/22</t>
+          <t>11/22</t>
         </is>
       </c>
       <c r="I134" s="3" t="inlineStr">
@@ -7097,10 +7097,10 @@
         </is>
       </c>
       <c r="J134" s="4" t="n">
-        <v>51055</v>
+        <v>51446</v>
       </c>
       <c r="K134" s="5" t="n">
-        <v>2320.7</v>
+        <v>2338.454545454545</v>
       </c>
     </row>
     <row r="135">
@@ -7182,11 +7182,11 @@
         </is>
       </c>
       <c r="G136" s="7" t="n">
-        <v>5279</v>
+        <v>3844</v>
       </c>
       <c r="H136" s="6" t="inlineStr">
         <is>
-          <t>14/26</t>
+          <t>15/26</t>
         </is>
       </c>
       <c r="I136" s="6" t="inlineStr">
@@ -7195,10 +7195,10 @@
         </is>
       </c>
       <c r="J136" s="7" t="n">
-        <v>9804</v>
+        <v>6663</v>
       </c>
       <c r="K136" s="8" t="n">
-        <v>377.0714285714286</v>
+        <v>256.2666666666667</v>
       </c>
     </row>
     <row r="137">
@@ -7231,11 +7231,11 @@
         </is>
       </c>
       <c r="G137" s="7" t="n">
-        <v>4861</v>
+        <v>5236</v>
       </c>
       <c r="H137" s="6" t="inlineStr">
         <is>
-          <t>14/21</t>
+          <t>15/21</t>
         </is>
       </c>
       <c r="I137" s="6" t="inlineStr">
@@ -7244,10 +7244,10 @@
         </is>
       </c>
       <c r="J137" s="7" t="n">
-        <v>7292</v>
+        <v>7330</v>
       </c>
       <c r="K137" s="8" t="n">
-        <v>347.2142857142857</v>
+        <v>349.0666666666667</v>
       </c>
     </row>
     <row r="138">
@@ -7280,11 +7280,11 @@
         </is>
       </c>
       <c r="G138" s="11" t="n">
-        <v>1326</v>
+        <v>2359</v>
       </c>
       <c r="H138" s="10" t="inlineStr">
         <is>
-          <t>16/20</t>
+          <t>17/20</t>
         </is>
       </c>
       <c r="I138" s="10" t="inlineStr">
@@ -7293,10 +7293,10 @@
         </is>
       </c>
       <c r="J138" s="11" t="n">
-        <v>1658</v>
+        <v>2775</v>
       </c>
       <c r="K138" s="12" t="n">
-        <v>82.875</v>
+        <v>138.7647058823529</v>
       </c>
     </row>
     <row r="139">
@@ -7378,11 +7378,11 @@
         </is>
       </c>
       <c r="G140" s="4" t="n">
-        <v>34010</v>
+        <v>36253</v>
       </c>
       <c r="H140" s="3" t="inlineStr">
         <is>
-          <t>15/24</t>
+          <t>16/24</t>
         </is>
       </c>
       <c r="I140" s="3" t="inlineStr">
@@ -7391,10 +7391,10 @@
         </is>
       </c>
       <c r="J140" s="4" t="n">
-        <v>54416</v>
+        <v>54380</v>
       </c>
       <c r="K140" s="5" t="n">
-        <v>2267.333333333333</v>
+        <v>2265.8125</v>
       </c>
     </row>
     <row r="141">
@@ -7427,11 +7427,11 @@
         </is>
       </c>
       <c r="G141" s="7" t="n">
-        <v>3100</v>
+        <v>4011</v>
       </c>
       <c r="H141" s="6" t="inlineStr">
         <is>
-          <t>13/25</t>
+          <t>14/25</t>
         </is>
       </c>
       <c r="I141" s="6" t="inlineStr">
@@ -7440,10 +7440,10 @@
         </is>
       </c>
       <c r="J141" s="7" t="n">
-        <v>5962</v>
+        <v>7162</v>
       </c>
       <c r="K141" s="8" t="n">
-        <v>238.4615384615385</v>
+        <v>286.4999999999999</v>
       </c>
     </row>
     <row r="142">
@@ -7574,11 +7574,11 @@
         </is>
       </c>
       <c r="G144" s="4" t="n">
-        <v>9821</v>
+        <v>11385</v>
       </c>
       <c r="H144" s="3" t="inlineStr">
         <is>
-          <t>22/24</t>
+          <t>23/24</t>
         </is>
       </c>
       <c r="I144" s="3" t="inlineStr">
@@ -7587,10 +7587,10 @@
         </is>
       </c>
       <c r="J144" s="4" t="n">
-        <v>10714</v>
+        <v>11880</v>
       </c>
       <c r="K144" s="5" t="n">
-        <v>446.4090909090909</v>
+        <v>495</v>
       </c>
     </row>
     <row r="145">
@@ -7623,11 +7623,11 @@
         </is>
       </c>
       <c r="G145" s="4" t="n">
-        <v>10507</v>
+        <v>9970</v>
       </c>
       <c r="H145" s="3" t="inlineStr">
         <is>
-          <t>15/20</t>
+          <t>16/20</t>
         </is>
       </c>
       <c r="I145" s="3" t="inlineStr">
@@ -7636,10 +7636,10 @@
         </is>
       </c>
       <c r="J145" s="4" t="n">
-        <v>14009</v>
+        <v>12462</v>
       </c>
       <c r="K145" s="5" t="n">
-        <v>700.4666666666667</v>
+        <v>623.125</v>
       </c>
     </row>
     <row r="146">
@@ -7672,11 +7672,11 @@
         </is>
       </c>
       <c r="G146" s="4" t="n">
-        <v>14962</v>
+        <v>14383</v>
       </c>
       <c r="H146" s="3" t="inlineStr">
         <is>
-          <t>23/29</t>
+          <t>24/29</t>
         </is>
       </c>
       <c r="I146" s="3" t="inlineStr">
@@ -7685,59 +7685,59 @@
         </is>
       </c>
       <c r="J146" s="4" t="n">
-        <v>18865</v>
+        <v>17379</v>
       </c>
       <c r="K146" s="5" t="n">
-        <v>650.5217391304348</v>
+        <v>599.2916666666666</v>
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="6" t="inlineStr">
+      <c r="A147" s="9" t="inlineStr">
         <is>
           <t>RANIPET</t>
         </is>
       </c>
-      <c r="B147" s="6" t="n">
+      <c r="B147" s="10" t="n">
         <v>41</v>
       </c>
-      <c r="C147" s="6" t="inlineStr">
+      <c r="C147" s="10" t="inlineStr">
         <is>
           <t>R. GANDHI</t>
         </is>
       </c>
-      <c r="D147" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E147" s="6" t="inlineStr">
+      <c r="D147" s="10" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E147" s="10" t="inlineStr">
         <is>
           <t>THAHIRA</t>
         </is>
       </c>
-      <c r="F147" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G147" s="7" t="n">
-        <v>2137</v>
-      </c>
-      <c r="H147" s="6" t="inlineStr">
-        <is>
-          <t>13/22</t>
-        </is>
-      </c>
-      <c r="I147" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J147" s="7" t="n">
-        <v>3616</v>
-      </c>
-      <c r="K147" s="8" t="n">
-        <v>164.3846153846154</v>
+      <c r="F147" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G147" s="11" t="n">
+        <v>1569</v>
+      </c>
+      <c r="H147" s="10" t="inlineStr">
+        <is>
+          <t>14/22</t>
+        </is>
+      </c>
+      <c r="I147" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J147" s="11" t="n">
+        <v>2466</v>
+      </c>
+      <c r="K147" s="12" t="n">
+        <v>112.0714285714286</v>
       </c>
     </row>
     <row r="148">
@@ -7868,7 +7868,7 @@
         </is>
       </c>
       <c r="G150" s="4" t="n">
-        <v>11815</v>
+        <v>11868</v>
       </c>
       <c r="H150" s="3" t="inlineStr">
         <is>
@@ -7881,10 +7881,10 @@
         </is>
       </c>
       <c r="J150" s="4" t="n">
-        <v>13784</v>
+        <v>13846</v>
       </c>
       <c r="K150" s="5" t="n">
-        <v>984.5833333333334</v>
+        <v>989</v>
       </c>
     </row>
     <row r="151">
@@ -7966,11 +7966,11 @@
         </is>
       </c>
       <c r="G152" s="7" t="n">
-        <v>7892</v>
+        <v>6821</v>
       </c>
       <c r="H152" s="6" t="inlineStr">
         <is>
-          <t>13/21</t>
+          <t>14/21</t>
         </is>
       </c>
       <c r="I152" s="6" t="inlineStr">
@@ -7979,10 +7979,10 @@
         </is>
       </c>
       <c r="J152" s="7" t="n">
-        <v>12749</v>
+        <v>10232</v>
       </c>
       <c r="K152" s="8" t="n">
-        <v>607.0769230769231</v>
+        <v>487.2142857142857</v>
       </c>
     </row>
     <row r="153">
@@ -8015,11 +8015,11 @@
         </is>
       </c>
       <c r="G153" s="4" t="n">
-        <v>27504</v>
+        <v>28406</v>
       </c>
       <c r="H153" s="3" t="inlineStr">
         <is>
-          <t>14/20</t>
+          <t>15/20</t>
         </is>
       </c>
       <c r="I153" s="3" t="inlineStr">
@@ -8028,10 +8028,10 @@
         </is>
       </c>
       <c r="J153" s="4" t="n">
-        <v>39291</v>
+        <v>37875</v>
       </c>
       <c r="K153" s="5" t="n">
-        <v>1964.571428571429</v>
+        <v>1893.733333333333</v>
       </c>
     </row>
     <row r="154">
@@ -8064,11 +8064,11 @@
         </is>
       </c>
       <c r="G154" s="4" t="n">
-        <v>35110</v>
+        <v>39014</v>
       </c>
       <c r="H154" s="3" t="inlineStr">
         <is>
-          <t>11/23</t>
+          <t>12/23</t>
         </is>
       </c>
       <c r="I154" s="3" t="inlineStr">
@@ -8077,10 +8077,10 @@
         </is>
       </c>
       <c r="J154" s="4" t="n">
-        <v>73412</v>
+        <v>74777</v>
       </c>
       <c r="K154" s="5" t="n">
-        <v>3191.818181818182</v>
+        <v>3251.166666666667</v>
       </c>
     </row>
     <row r="155">
@@ -8231,52 +8231,52 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="13" t="inlineStr">
+      <c r="A158" s="9" t="inlineStr">
         <is>
           <t>SATTUR</t>
         </is>
       </c>
-      <c r="B158" s="14" t="n">
+      <c r="B158" s="10" t="n">
         <v>204</v>
       </c>
-      <c r="C158" s="14" t="inlineStr">
+      <c r="C158" s="10" t="inlineStr">
+        <is>
+          <t>NAINAR NAGENTHRAN</t>
+        </is>
+      </c>
+      <c r="D158" s="10" t="inlineStr">
+        <is>
+          <t>Bharatiya Janata Party</t>
+        </is>
+      </c>
+      <c r="E158" s="10" t="inlineStr">
         <is>
           <t>KADARKARAIRAJ. A</t>
         </is>
       </c>
-      <c r="D158" s="14" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E158" s="14" t="inlineStr">
-        <is>
-          <t>AJITH. M</t>
-        </is>
-      </c>
-      <c r="F158" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G158" s="15" t="n">
-        <v>46</v>
-      </c>
-      <c r="H158" s="14" t="inlineStr">
-        <is>
-          <t>6/21</t>
-        </is>
-      </c>
-      <c r="I158" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J158" s="15" t="n">
-        <v>161</v>
-      </c>
-      <c r="K158" s="16" t="n">
-        <v>7.666666666666667</v>
+      <c r="F158" s="10" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G158" s="11" t="n">
+        <v>563</v>
+      </c>
+      <c r="H158" s="10" t="inlineStr">
+        <is>
+          <t>7/21</t>
+        </is>
+      </c>
+      <c r="I158" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J158" s="11" t="n">
+        <v>1689</v>
+      </c>
+      <c r="K158" s="12" t="n">
+        <v>80.42857142857143</v>
       </c>
     </row>
     <row r="159">
@@ -8329,52 +8329,52 @@
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="13" t="inlineStr">
+      <c r="A160" s="9" t="inlineStr">
         <is>
           <t>SHOLAVANDAN</t>
         </is>
       </c>
-      <c r="B160" s="14" t="n">
+      <c r="B160" s="10" t="n">
         <v>190</v>
       </c>
-      <c r="C160" s="14" t="inlineStr">
+      <c r="C160" s="10" t="inlineStr">
+        <is>
+          <t>KARUPPAIAH.M.V</t>
+        </is>
+      </c>
+      <c r="D160" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E160" s="10" t="inlineStr">
         <is>
           <t>VENKATESAN.A</t>
         </is>
       </c>
-      <c r="D160" s="14" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E160" s="14" t="inlineStr">
-        <is>
-          <t>KARUPPAIAH.M.V</t>
-        </is>
-      </c>
-      <c r="F160" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G160" s="15" t="n">
-        <v>15</v>
-      </c>
-      <c r="H160" s="14" t="inlineStr">
-        <is>
-          <t>8/19</t>
-        </is>
-      </c>
-      <c r="I160" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J160" s="15" t="n">
-        <v>36</v>
-      </c>
-      <c r="K160" s="16" t="n">
-        <v>1.875</v>
+      <c r="F160" s="10" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G160" s="11" t="n">
+        <v>701</v>
+      </c>
+      <c r="H160" s="10" t="inlineStr">
+        <is>
+          <t>9/19</t>
+        </is>
+      </c>
+      <c r="I160" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J160" s="11" t="n">
+        <v>1480</v>
+      </c>
+      <c r="K160" s="12" t="n">
+        <v>77.88888888888889</v>
       </c>
     </row>
     <row r="161">
@@ -8407,11 +8407,11 @@
         </is>
       </c>
       <c r="G161" s="11" t="n">
-        <v>841</v>
+        <v>437</v>
       </c>
       <c r="H161" s="10" t="inlineStr">
         <is>
-          <t>9/25</t>
+          <t>10/25</t>
         </is>
       </c>
       <c r="I161" s="10" t="inlineStr">
@@ -8420,10 +8420,10 @@
         </is>
       </c>
       <c r="J161" s="11" t="n">
-        <v>2336</v>
+        <v>1092</v>
       </c>
       <c r="K161" s="12" t="n">
-        <v>93.44444444444444</v>
+        <v>43.7</v>
       </c>
     </row>
     <row r="162">
@@ -8456,11 +8456,11 @@
         </is>
       </c>
       <c r="G162" s="4" t="n">
-        <v>30277</v>
+        <v>31634</v>
       </c>
       <c r="H162" s="3" t="inlineStr">
         <is>
-          <t>10/30</t>
+          <t>11/30</t>
         </is>
       </c>
       <c r="I162" s="3" t="inlineStr">
@@ -8469,10 +8469,10 @@
         </is>
       </c>
       <c r="J162" s="4" t="n">
-        <v>90831</v>
+        <v>86275</v>
       </c>
       <c r="K162" s="5" t="n">
-        <v>3027.7</v>
+        <v>2875.818181818182</v>
       </c>
     </row>
     <row r="163">
@@ -8505,11 +8505,11 @@
         </is>
       </c>
       <c r="G163" s="4" t="n">
-        <v>12853</v>
+        <v>13494</v>
       </c>
       <c r="H163" s="3" t="inlineStr">
         <is>
-          <t>13/26</t>
+          <t>14/26</t>
         </is>
       </c>
       <c r="I163" s="3" t="inlineStr">
@@ -8518,10 +8518,10 @@
         </is>
       </c>
       <c r="J163" s="4" t="n">
-        <v>25706</v>
+        <v>25060</v>
       </c>
       <c r="K163" s="5" t="n">
-        <v>988.6923076923077</v>
+        <v>963.8571428571429</v>
       </c>
     </row>
     <row r="164">
@@ -8652,11 +8652,11 @@
         </is>
       </c>
       <c r="G166" s="7" t="n">
-        <v>1572</v>
+        <v>2334</v>
       </c>
       <c r="H166" s="6" t="inlineStr">
         <is>
-          <t>7/21</t>
+          <t>8/21</t>
         </is>
       </c>
       <c r="I166" s="6" t="inlineStr">
@@ -8665,10 +8665,10 @@
         </is>
       </c>
       <c r="J166" s="7" t="n">
-        <v>4716</v>
+        <v>6127</v>
       </c>
       <c r="K166" s="8" t="n">
-        <v>224.5714285714286</v>
+        <v>291.75</v>
       </c>
     </row>
     <row r="167">
@@ -8780,26 +8780,26 @@
       </c>
       <c r="C169" s="14" t="inlineStr">
         <is>
+          <t>SHANMUGANATHAN. S. P</t>
+        </is>
+      </c>
+      <c r="D169" s="14" t="inlineStr">
+        <is>
+          <t>All India Anna Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E169" s="14" t="inlineStr">
+        <is>
           <t>SARAVANAN. G</t>
         </is>
       </c>
-      <c r="D169" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E169" s="14" t="inlineStr">
-        <is>
-          <t>SHANMUGANATHAN. S. P</t>
-        </is>
-      </c>
       <c r="F169" s="14" t="inlineStr">
         <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
+          <t>Tamilaga Vettri Kazhagam</t>
         </is>
       </c>
       <c r="G169" s="15" t="n">
-        <v>38</v>
+        <v>207</v>
       </c>
       <c r="H169" s="14" t="inlineStr">
         <is>
@@ -8812,10 +8812,10 @@
         </is>
       </c>
       <c r="J169" s="15" t="n">
-        <v>42</v>
+        <v>229</v>
       </c>
       <c r="K169" s="16" t="n">
-        <v>2</v>
+        <v>10.89473684210526</v>
       </c>
     </row>
     <row r="170">
@@ -8848,11 +8848,11 @@
         </is>
       </c>
       <c r="G170" s="7" t="n">
-        <v>3737</v>
+        <v>2412</v>
       </c>
       <c r="H170" s="6" t="inlineStr">
         <is>
-          <t>10/22</t>
+          <t>11/22</t>
         </is>
       </c>
       <c r="I170" s="6" t="inlineStr">
@@ -8861,10 +8861,10 @@
         </is>
       </c>
       <c r="J170" s="7" t="n">
-        <v>8221</v>
+        <v>4824</v>
       </c>
       <c r="K170" s="8" t="n">
-        <v>373.7</v>
+        <v>219.2727272727273</v>
       </c>
     </row>
     <row r="171">
@@ -8897,11 +8897,11 @@
         </is>
       </c>
       <c r="G171" s="7" t="n">
-        <v>8837</v>
+        <v>9240</v>
       </c>
       <c r="H171" s="6" t="inlineStr">
         <is>
-          <t>16/28</t>
+          <t>17/28</t>
         </is>
       </c>
       <c r="I171" s="6" t="inlineStr">
@@ -8910,10 +8910,10 @@
         </is>
       </c>
       <c r="J171" s="7" t="n">
-        <v>15465</v>
+        <v>15219</v>
       </c>
       <c r="K171" s="8" t="n">
-        <v>552.3125</v>
+        <v>543.5294117647059</v>
       </c>
     </row>
     <row r="172">
@@ -8995,11 +8995,11 @@
         </is>
       </c>
       <c r="G173" s="7" t="n">
-        <v>6597</v>
+        <v>5825</v>
       </c>
       <c r="H173" s="6" t="inlineStr">
         <is>
-          <t>13/26</t>
+          <t>14/26</t>
         </is>
       </c>
       <c r="I173" s="6" t="inlineStr">
@@ -9008,10 +9008,10 @@
         </is>
       </c>
       <c r="J173" s="7" t="n">
-        <v>13194</v>
+        <v>10818</v>
       </c>
       <c r="K173" s="8" t="n">
-        <v>507.4615384615385</v>
+        <v>416.0714285714286</v>
       </c>
     </row>
     <row r="174">
@@ -9044,11 +9044,11 @@
         </is>
       </c>
       <c r="G174" s="15" t="n">
-        <v>237</v>
+        <v>24</v>
       </c>
       <c r="H174" s="14" t="inlineStr">
         <is>
-          <t>12/24</t>
+          <t>13/24</t>
         </is>
       </c>
       <c r="I174" s="14" t="inlineStr">
@@ -9057,10 +9057,10 @@
         </is>
       </c>
       <c r="J174" s="15" t="n">
-        <v>474</v>
+        <v>44</v>
       </c>
       <c r="K174" s="16" t="n">
-        <v>19.75</v>
+        <v>1.846153846153846</v>
       </c>
     </row>
     <row r="175">
@@ -9142,11 +9142,11 @@
         </is>
       </c>
       <c r="G176" s="4" t="n">
-        <v>20636</v>
+        <v>22164</v>
       </c>
       <c r="H176" s="3" t="inlineStr">
         <is>
-          <t>15/17</t>
+          <t>16/17</t>
         </is>
       </c>
       <c r="I176" s="3" t="inlineStr">
@@ -9155,10 +9155,10 @@
         </is>
       </c>
       <c r="J176" s="4" t="n">
-        <v>23387</v>
+        <v>23549</v>
       </c>
       <c r="K176" s="5" t="n">
-        <v>1375.733333333333</v>
+        <v>1385.25</v>
       </c>
     </row>
     <row r="177">
@@ -9191,11 +9191,11 @@
         </is>
       </c>
       <c r="G177" s="4" t="n">
-        <v>14259</v>
+        <v>15762</v>
       </c>
       <c r="H177" s="3" t="inlineStr">
         <is>
-          <t>18/26</t>
+          <t>19/26</t>
         </is>
       </c>
       <c r="I177" s="3" t="inlineStr">
@@ -9204,10 +9204,10 @@
         </is>
       </c>
       <c r="J177" s="4" t="n">
-        <v>20596</v>
+        <v>21569</v>
       </c>
       <c r="K177" s="5" t="n">
-        <v>792.1666666666666</v>
+        <v>829.578947368421</v>
       </c>
     </row>
     <row r="178">
@@ -9231,20 +9231,20 @@
       </c>
       <c r="E178" s="6" t="inlineStr">
         <is>
-          <t>CHINTHAMANI.C</t>
+          <t>VAIRAMUTHU.PK</t>
         </is>
       </c>
       <c r="F178" s="6" t="inlineStr">
         <is>
-          <t>Tamilaga Vettri Kazhagam</t>
+          <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
       <c r="G178" s="7" t="n">
-        <v>1713</v>
+        <v>1357</v>
       </c>
       <c r="H178" s="6" t="inlineStr">
         <is>
-          <t>8/22</t>
+          <t>9/22</t>
         </is>
       </c>
       <c r="I178" s="6" t="inlineStr">
@@ -9253,10 +9253,10 @@
         </is>
       </c>
       <c r="J178" s="7" t="n">
-        <v>4711</v>
+        <v>3317</v>
       </c>
       <c r="K178" s="8" t="n">
-        <v>214.125</v>
+        <v>150.7777777777778</v>
       </c>
     </row>
     <row r="179">
@@ -9338,11 +9338,11 @@
         </is>
       </c>
       <c r="G180" s="4" t="n">
-        <v>24214</v>
+        <v>25891</v>
       </c>
       <c r="H180" s="3" t="inlineStr">
         <is>
-          <t>13/29</t>
+          <t>14/29</t>
         </is>
       </c>
       <c r="I180" s="3" t="inlineStr">
@@ -9351,10 +9351,10 @@
         </is>
       </c>
       <c r="J180" s="4" t="n">
-        <v>54016</v>
+        <v>53631</v>
       </c>
       <c r="K180" s="5" t="n">
-        <v>1862.615384615385</v>
+        <v>1849.357142857143</v>
       </c>
     </row>
     <row r="181">
@@ -9436,11 +9436,11 @@
         </is>
       </c>
       <c r="G182" s="7" t="n">
-        <v>7160</v>
+        <v>8121</v>
       </c>
       <c r="H182" s="6" t="inlineStr">
         <is>
-          <t>11/25</t>
+          <t>12/25</t>
         </is>
       </c>
       <c r="I182" s="6" t="inlineStr">
@@ -9449,10 +9449,10 @@
         </is>
       </c>
       <c r="J182" s="7" t="n">
-        <v>16273</v>
+        <v>16919</v>
       </c>
       <c r="K182" s="8" t="n">
-        <v>650.9090909090909</v>
+        <v>676.75</v>
       </c>
     </row>
     <row r="183">
@@ -9632,11 +9632,11 @@
         </is>
       </c>
       <c r="G186" s="7" t="n">
-        <v>7694</v>
+        <v>7957</v>
       </c>
       <c r="H186" s="6" t="inlineStr">
         <is>
-          <t>13/24</t>
+          <t>14/24</t>
         </is>
       </c>
       <c r="I186" s="6" t="inlineStr">
@@ -9645,10 +9645,10 @@
         </is>
       </c>
       <c r="J186" s="7" t="n">
-        <v>14204</v>
+        <v>13641</v>
       </c>
       <c r="K186" s="8" t="n">
-        <v>591.8461538461538</v>
+        <v>568.3571428571429</v>
       </c>
     </row>
     <row r="187">
@@ -9750,52 +9750,52 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="2" t="inlineStr">
+      <c r="A189" s="6" t="inlineStr">
         <is>
           <t>THONDAMUTHUR</t>
         </is>
       </c>
-      <c r="B189" s="3" t="n">
+      <c r="B189" s="6" t="n">
         <v>119</v>
       </c>
-      <c r="C189" s="3" t="inlineStr">
+      <c r="C189" s="6" t="inlineStr">
         <is>
           <t>S.P.VELUMANI</t>
         </is>
       </c>
-      <c r="D189" s="3" t="inlineStr">
+      <c r="D189" s="6" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E189" s="3" t="inlineStr">
-        <is>
-          <t>SATHISH RAJU (ALIAS) K.P.R. SATHISH</t>
-        </is>
-      </c>
-      <c r="F189" s="3" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G189" s="4" t="n">
-        <v>13894</v>
-      </c>
-      <c r="H189" s="3" t="inlineStr">
-        <is>
-          <t>12/27</t>
-        </is>
-      </c>
-      <c r="I189" s="3" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J189" s="4" t="n">
-        <v>31261</v>
-      </c>
-      <c r="K189" s="5" t="n">
-        <v>1157.833333333333</v>
+      <c r="E189" s="6" t="inlineStr">
+        <is>
+          <t>N.R.KARTHIKEYAN</t>
+        </is>
+      </c>
+      <c r="F189" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G189" s="7" t="n">
+        <v>9220</v>
+      </c>
+      <c r="H189" s="6" t="inlineStr">
+        <is>
+          <t>13/27</t>
+        </is>
+      </c>
+      <c r="I189" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J189" s="7" t="n">
+        <v>19149</v>
+      </c>
+      <c r="K189" s="8" t="n">
+        <v>709.2307692307693</v>
       </c>
     </row>
     <row r="190">
@@ -9877,11 +9877,11 @@
         </is>
       </c>
       <c r="G191" s="7" t="n">
-        <v>6025</v>
+        <v>7536</v>
       </c>
       <c r="H191" s="6" t="inlineStr">
         <is>
-          <t>10/18</t>
+          <t>11/18</t>
         </is>
       </c>
       <c r="I191" s="6" t="inlineStr">
@@ -9890,10 +9890,10 @@
         </is>
       </c>
       <c r="J191" s="7" t="n">
-        <v>10845</v>
+        <v>12332</v>
       </c>
       <c r="K191" s="8" t="n">
-        <v>602.5</v>
+        <v>685.0909090909091</v>
       </c>
     </row>
     <row r="192">
@@ -9975,11 +9975,11 @@
         </is>
       </c>
       <c r="G193" s="11" t="n">
-        <v>620</v>
+        <v>1560</v>
       </c>
       <c r="H193" s="10" t="inlineStr">
         <is>
-          <t>11/21</t>
+          <t>12/22</t>
         </is>
       </c>
       <c r="I193" s="10" t="inlineStr">
@@ -9988,59 +9988,59 @@
         </is>
       </c>
       <c r="J193" s="11" t="n">
-        <v>1184</v>
+        <v>2860</v>
       </c>
       <c r="K193" s="12" t="n">
-        <v>56.36363636363637</v>
+        <v>130</v>
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="6" t="inlineStr">
+      <c r="A194" s="2" t="inlineStr">
         <is>
           <t>TIRUCHENDUR</t>
         </is>
       </c>
-      <c r="B194" s="6" t="n">
+      <c r="B194" s="3" t="n">
         <v>215</v>
       </c>
-      <c r="C194" s="6" t="inlineStr">
+      <c r="C194" s="3" t="inlineStr">
         <is>
           <t>ANITHA R. RADHAKRISHNAN</t>
         </is>
       </c>
-      <c r="D194" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E194" s="6" t="inlineStr">
+      <c r="D194" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E194" s="3" t="inlineStr">
         <is>
           <t>J. MURUGAN</t>
         </is>
       </c>
-      <c r="F194" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G194" s="7" t="n">
-        <v>6600</v>
-      </c>
-      <c r="H194" s="6" t="inlineStr">
-        <is>
-          <t>16/22</t>
-        </is>
-      </c>
-      <c r="I194" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J194" s="7" t="n">
-        <v>9075</v>
-      </c>
-      <c r="K194" s="8" t="n">
-        <v>412.5</v>
+      <c r="F194" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G194" s="4" t="n">
+        <v>5302</v>
+      </c>
+      <c r="H194" s="3" t="inlineStr">
+        <is>
+          <t>17/22</t>
+        </is>
+      </c>
+      <c r="I194" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J194" s="4" t="n">
+        <v>6861</v>
+      </c>
+      <c r="K194" s="5" t="n">
+        <v>311.8823529411765</v>
       </c>
     </row>
     <row r="195">
@@ -10269,11 +10269,11 @@
         </is>
       </c>
       <c r="G199" s="11" t="n">
-        <v>385</v>
+        <v>972</v>
       </c>
       <c r="H199" s="10" t="inlineStr">
         <is>
-          <t>13/24</t>
+          <t>14/24</t>
         </is>
       </c>
       <c r="I199" s="10" t="inlineStr">
@@ -10282,10 +10282,10 @@
         </is>
       </c>
       <c r="J199" s="11" t="n">
-        <v>711</v>
+        <v>1666</v>
       </c>
       <c r="K199" s="12" t="n">
-        <v>29.61538461538462</v>
+        <v>69.42857142857143</v>
       </c>
     </row>
     <row r="200">
@@ -10367,11 +10367,11 @@
         </is>
       </c>
       <c r="G201" s="4" t="n">
-        <v>15344</v>
+        <v>17070</v>
       </c>
       <c r="H201" s="3" t="inlineStr">
         <is>
-          <t>9/22</t>
+          <t>10/22</t>
         </is>
       </c>
       <c r="I201" s="3" t="inlineStr">
@@ -10380,10 +10380,10 @@
         </is>
       </c>
       <c r="J201" s="4" t="n">
-        <v>37508</v>
+        <v>37554</v>
       </c>
       <c r="K201" s="5" t="n">
-        <v>1704.888888888889</v>
+        <v>1707</v>
       </c>
     </row>
     <row r="202">
@@ -10416,11 +10416,11 @@
         </is>
       </c>
       <c r="G202" s="7" t="n">
-        <v>3904</v>
+        <v>4109</v>
       </c>
       <c r="H202" s="6" t="inlineStr">
         <is>
-          <t>12/27</t>
+          <t>13/27</t>
         </is>
       </c>
       <c r="I202" s="6" t="inlineStr">
@@ -10429,10 +10429,10 @@
         </is>
       </c>
       <c r="J202" s="7" t="n">
-        <v>8784</v>
+        <v>8534</v>
       </c>
       <c r="K202" s="8" t="n">
-        <v>325.3333333333333</v>
+        <v>316.0769230769231</v>
       </c>
     </row>
     <row r="203">
@@ -10485,52 +10485,52 @@
       </c>
     </row>
     <row r="204">
-      <c r="A204" s="2" t="inlineStr">
+      <c r="A204" s="6" t="inlineStr">
         <is>
           <t>TIRUPPUR (SOUTH)</t>
         </is>
       </c>
-      <c r="B204" s="3" t="n">
+      <c r="B204" s="6" t="n">
         <v>114</v>
       </c>
-      <c r="C204" s="3" t="inlineStr">
+      <c r="C204" s="6" t="inlineStr">
         <is>
           <t>BALAMURUGAN. S</t>
         </is>
       </c>
-      <c r="D204" s="3" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E204" s="3" t="inlineStr">
+      <c r="D204" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E204" s="6" t="inlineStr">
         <is>
           <t>DINESHKUMAR. N</t>
         </is>
       </c>
-      <c r="F204" s="3" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G204" s="4" t="n">
-        <v>13479</v>
-      </c>
-      <c r="H204" s="3" t="inlineStr">
-        <is>
-          <t>11/21</t>
-        </is>
-      </c>
-      <c r="I204" s="3" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J204" s="4" t="n">
-        <v>25733</v>
-      </c>
-      <c r="K204" s="5" t="n">
-        <v>1225.363636363636</v>
+      <c r="F204" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G204" s="7" t="n">
+        <v>9409</v>
+      </c>
+      <c r="H204" s="6" t="inlineStr">
+        <is>
+          <t>12/21</t>
+        </is>
+      </c>
+      <c r="I204" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J204" s="7" t="n">
+        <v>16466</v>
+      </c>
+      <c r="K204" s="8" t="n">
+        <v>784.0833333333334</v>
       </c>
     </row>
     <row r="205">
@@ -10612,11 +10612,11 @@
         </is>
       </c>
       <c r="G206" s="15" t="n">
-        <v>17</v>
+        <v>345</v>
       </c>
       <c r="H206" s="14" t="inlineStr">
         <is>
-          <t>19/27</t>
+          <t>20/27</t>
         </is>
       </c>
       <c r="I206" s="14" t="inlineStr">
@@ -10625,10 +10625,10 @@
         </is>
       </c>
       <c r="J206" s="15" t="n">
-        <v>24</v>
+        <v>466</v>
       </c>
       <c r="K206" s="16" t="n">
-        <v>0.8947368421052632</v>
+        <v>17.25</v>
       </c>
     </row>
     <row r="207">
@@ -10710,11 +10710,11 @@
         </is>
       </c>
       <c r="G208" s="11" t="n">
-        <v>1366</v>
+        <v>1004</v>
       </c>
       <c r="H208" s="10" t="inlineStr">
         <is>
-          <t>10/20</t>
+          <t>11/20</t>
         </is>
       </c>
       <c r="I208" s="10" t="inlineStr">
@@ -10723,10 +10723,10 @@
         </is>
       </c>
       <c r="J208" s="11" t="n">
-        <v>2732</v>
+        <v>1825</v>
       </c>
       <c r="K208" s="12" t="n">
-        <v>136.6</v>
+        <v>91.27272727272727</v>
       </c>
     </row>
     <row r="209">
@@ -10759,11 +10759,11 @@
         </is>
       </c>
       <c r="G209" s="11" t="n">
-        <v>986</v>
+        <v>1231</v>
       </c>
       <c r="H209" s="10" t="inlineStr">
         <is>
-          <t>18/19</t>
+          <t>19/21</t>
         </is>
       </c>
       <c r="I209" s="10" t="inlineStr">
@@ -10772,10 +10772,10 @@
         </is>
       </c>
       <c r="J209" s="11" t="n">
-        <v>1041</v>
+        <v>1361</v>
       </c>
       <c r="K209" s="12" t="n">
-        <v>54.77777777777778</v>
+        <v>64.78947368421052</v>
       </c>
     </row>
     <row r="210">
@@ -10808,11 +10808,11 @@
         </is>
       </c>
       <c r="G210" s="7" t="n">
-        <v>4487</v>
+        <v>4020</v>
       </c>
       <c r="H210" s="6" t="inlineStr">
         <is>
-          <t>16/22</t>
+          <t>17/22</t>
         </is>
       </c>
       <c r="I210" s="6" t="inlineStr">
@@ -10821,10 +10821,10 @@
         </is>
       </c>
       <c r="J210" s="7" t="n">
-        <v>6170</v>
+        <v>5202</v>
       </c>
       <c r="K210" s="8" t="n">
-        <v>280.4375</v>
+        <v>236.4705882352941</v>
       </c>
     </row>
     <row r="211">
@@ -10857,11 +10857,11 @@
         </is>
       </c>
       <c r="G211" s="11" t="n">
-        <v>1290</v>
+        <v>1448</v>
       </c>
       <c r="H211" s="10" t="inlineStr">
         <is>
-          <t>13/27</t>
+          <t>14/27</t>
         </is>
       </c>
       <c r="I211" s="10" t="inlineStr">
@@ -10870,10 +10870,10 @@
         </is>
       </c>
       <c r="J211" s="11" t="n">
-        <v>2679</v>
+        <v>2793</v>
       </c>
       <c r="K211" s="12" t="n">
-        <v>99.23076923076923</v>
+        <v>103.4285714285714</v>
       </c>
     </row>
     <row r="212">
@@ -10906,11 +10906,11 @@
         </is>
       </c>
       <c r="G212" s="7" t="n">
-        <v>2187</v>
+        <v>2132</v>
       </c>
       <c r="H212" s="6" t="inlineStr">
         <is>
-          <t>10/25</t>
+          <t>11/25</t>
         </is>
       </c>
       <c r="I212" s="6" t="inlineStr">
@@ -10919,59 +10919,59 @@
         </is>
       </c>
       <c r="J212" s="7" t="n">
-        <v>5468</v>
+        <v>4845</v>
       </c>
       <c r="K212" s="8" t="n">
-        <v>218.7</v>
+        <v>193.8181818181818</v>
       </c>
     </row>
     <row r="213">
-      <c r="A213" s="2" t="inlineStr">
+      <c r="A213" s="6" t="inlineStr">
         <is>
           <t>UTHANGARAI</t>
         </is>
       </c>
-      <c r="B213" s="3" t="n">
+      <c r="B213" s="6" t="n">
         <v>51</v>
       </c>
-      <c r="C213" s="3" t="inlineStr">
+      <c r="C213" s="6" t="inlineStr">
         <is>
           <t>N ELAIYARAJA</t>
         </is>
       </c>
-      <c r="D213" s="3" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E213" s="3" t="inlineStr">
+      <c r="D213" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E213" s="6" t="inlineStr">
         <is>
           <t>T M TAMILSELVAM</t>
         </is>
       </c>
-      <c r="F213" s="3" t="inlineStr">
+      <c r="F213" s="6" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G213" s="4" t="n">
-        <v>5482</v>
-      </c>
-      <c r="H213" s="3" t="inlineStr">
-        <is>
-          <t>19/23</t>
-        </is>
-      </c>
-      <c r="I213" s="3" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J213" s="4" t="n">
-        <v>6636</v>
-      </c>
-      <c r="K213" s="5" t="n">
-        <v>288.5263157894737</v>
+      <c r="G213" s="7" t="n">
+        <v>4888</v>
+      </c>
+      <c r="H213" s="6" t="inlineStr">
+        <is>
+          <t>20/23</t>
+        </is>
+      </c>
+      <c r="I213" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J213" s="7" t="n">
+        <v>5621</v>
+      </c>
+      <c r="K213" s="8" t="n">
+        <v>244.4</v>
       </c>
     </row>
     <row r="214">
@@ -11004,11 +11004,11 @@
         </is>
       </c>
       <c r="G214" s="7" t="n">
-        <v>13873</v>
+        <v>13927</v>
       </c>
       <c r="H214" s="6" t="inlineStr">
         <is>
-          <t>16/23</t>
+          <t>17/23</t>
         </is>
       </c>
       <c r="I214" s="6" t="inlineStr">
@@ -11017,10 +11017,10 @@
         </is>
       </c>
       <c r="J214" s="7" t="n">
-        <v>19942</v>
+        <v>18842</v>
       </c>
       <c r="K214" s="8" t="n">
-        <v>867.0625</v>
+        <v>819.2352941176471</v>
       </c>
     </row>
     <row r="215">
@@ -11102,11 +11102,11 @@
         </is>
       </c>
       <c r="G216" s="7" t="n">
-        <v>2516</v>
+        <v>3617</v>
       </c>
       <c r="H216" s="6" t="inlineStr">
         <is>
-          <t>14/21</t>
+          <t>15/21</t>
         </is>
       </c>
       <c r="I216" s="6" t="inlineStr">
@@ -11115,10 +11115,10 @@
         </is>
       </c>
       <c r="J216" s="7" t="n">
-        <v>3774</v>
+        <v>5064</v>
       </c>
       <c r="K216" s="8" t="n">
-        <v>179.7142857142857</v>
+        <v>241.1333333333333</v>
       </c>
     </row>
     <row r="217">
@@ -11151,7 +11151,7 @@
         </is>
       </c>
       <c r="G217" s="4" t="n">
-        <v>5010</v>
+        <v>5073</v>
       </c>
       <c r="H217" s="3" t="inlineStr">
         <is>
@@ -11164,10 +11164,10 @@
         </is>
       </c>
       <c r="J217" s="4" t="n">
-        <v>5487</v>
+        <v>5556</v>
       </c>
       <c r="K217" s="5" t="n">
-        <v>238.5714285714286</v>
+        <v>241.5714285714286</v>
       </c>
     </row>
     <row r="218">
@@ -11200,11 +11200,11 @@
         </is>
       </c>
       <c r="G218" s="7" t="n">
-        <v>2845</v>
+        <v>3645</v>
       </c>
       <c r="H218" s="6" t="inlineStr">
         <is>
-          <t>13/22</t>
+          <t>14/22</t>
         </is>
       </c>
       <c r="I218" s="6" t="inlineStr">
@@ -11213,10 +11213,10 @@
         </is>
       </c>
       <c r="J218" s="7" t="n">
-        <v>4815</v>
+        <v>5728</v>
       </c>
       <c r="K218" s="8" t="n">
-        <v>218.8461538461538</v>
+        <v>260.3571428571428</v>
       </c>
     </row>
     <row r="219">
@@ -11298,11 +11298,11 @@
         </is>
       </c>
       <c r="G220" s="7" t="n">
-        <v>5392</v>
+        <v>5884</v>
       </c>
       <c r="H220" s="6" t="inlineStr">
         <is>
-          <t>12/18</t>
+          <t>13/18</t>
         </is>
       </c>
       <c r="I220" s="6" t="inlineStr">
@@ -11311,10 +11311,10 @@
         </is>
       </c>
       <c r="J220" s="7" t="n">
-        <v>8088</v>
+        <v>8147</v>
       </c>
       <c r="K220" s="8" t="n">
-        <v>449.3333333333333</v>
+        <v>452.6153846153846</v>
       </c>
     </row>
     <row r="221">
@@ -11347,11 +11347,11 @@
         </is>
       </c>
       <c r="G221" s="7" t="n">
-        <v>8038</v>
+        <v>8170</v>
       </c>
       <c r="H221" s="6" t="inlineStr">
         <is>
-          <t>14/24</t>
+          <t>15/24</t>
         </is>
       </c>
       <c r="I221" s="6" t="inlineStr">
@@ -11360,10 +11360,10 @@
         </is>
       </c>
       <c r="J221" s="7" t="n">
-        <v>13779</v>
+        <v>13072</v>
       </c>
       <c r="K221" s="8" t="n">
-        <v>574.1428571428571</v>
+        <v>544.6666666666666</v>
       </c>
     </row>
     <row r="222">
@@ -11445,11 +11445,11 @@
         </is>
       </c>
       <c r="G223" s="4" t="n">
-        <v>23805</v>
+        <v>26684</v>
       </c>
       <c r="H223" s="3" t="inlineStr">
         <is>
-          <t>15/23</t>
+          <t>17/23</t>
         </is>
       </c>
       <c r="I223" s="3" t="inlineStr">
@@ -11458,59 +11458,59 @@
         </is>
       </c>
       <c r="J223" s="4" t="n">
-        <v>36501</v>
+        <v>36102</v>
       </c>
       <c r="K223" s="5" t="n">
-        <v>1587</v>
+        <v>1569.64705882353</v>
       </c>
     </row>
     <row r="224">
-      <c r="A224" s="13" t="inlineStr">
+      <c r="A224" s="6" t="inlineStr">
         <is>
           <t>VELLORE</t>
         </is>
       </c>
-      <c r="B224" s="14" t="n">
+      <c r="B224" s="6" t="n">
         <v>43</v>
       </c>
-      <c r="C224" s="14" t="inlineStr">
+      <c r="C224" s="6" t="inlineStr">
+        <is>
+          <t>M.M.VINOTH KANNAN</t>
+        </is>
+      </c>
+      <c r="D224" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E224" s="6" t="inlineStr">
         <is>
           <t>P.KARTHIKEYAN</t>
         </is>
       </c>
-      <c r="D224" s="14" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E224" s="14" t="inlineStr">
-        <is>
-          <t>M.M.VINOTH KANNAN</t>
-        </is>
-      </c>
-      <c r="F224" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G224" s="15" t="n">
-        <v>40</v>
-      </c>
-      <c r="H224" s="14" t="inlineStr">
-        <is>
-          <t>13/20</t>
-        </is>
-      </c>
-      <c r="I224" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J224" s="15" t="n">
-        <v>62</v>
-      </c>
-      <c r="K224" s="16" t="n">
-        <v>3.076923076923077</v>
+      <c r="F224" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G224" s="7" t="n">
+        <v>2395</v>
+      </c>
+      <c r="H224" s="6" t="inlineStr">
+        <is>
+          <t>15/20</t>
+        </is>
+      </c>
+      <c r="I224" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J224" s="7" t="n">
+        <v>3193</v>
+      </c>
+      <c r="K224" s="8" t="n">
+        <v>159.6666666666667</v>
       </c>
     </row>
     <row r="225">
@@ -11524,30 +11524,30 @@
       </c>
       <c r="C225" s="10" t="inlineStr">
         <is>
+          <t>SRINIVASAN.P.S</t>
+        </is>
+      </c>
+      <c r="D225" s="10" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E225" s="10" t="inlineStr">
+        <is>
           <t>MUNUSAMY.K.P</t>
         </is>
       </c>
-      <c r="D225" s="10" t="inlineStr">
+      <c r="F225" s="10" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E225" s="10" t="inlineStr">
-        <is>
-          <t>SRINIVASAN.P.S</t>
-        </is>
-      </c>
-      <c r="F225" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
       <c r="G225" s="11" t="n">
-        <v>983</v>
+        <v>361</v>
       </c>
       <c r="H225" s="10" t="inlineStr">
         <is>
-          <t>17/25</t>
+          <t>18/25</t>
         </is>
       </c>
       <c r="I225" s="10" t="inlineStr">
@@ -11556,10 +11556,10 @@
         </is>
       </c>
       <c r="J225" s="11" t="n">
-        <v>1446</v>
+        <v>501</v>
       </c>
       <c r="K225" s="12" t="n">
-        <v>57.8235294117647</v>
+        <v>20.05555555555556</v>
       </c>
     </row>
     <row r="226">
@@ -11641,11 +11641,11 @@
         </is>
       </c>
       <c r="G227" s="4" t="n">
-        <v>5595</v>
+        <v>6909</v>
       </c>
       <c r="H227" s="3" t="inlineStr">
         <is>
-          <t>16/20</t>
+          <t>17/20</t>
         </is>
       </c>
       <c r="I227" s="3" t="inlineStr">
@@ -11654,10 +11654,10 @@
         </is>
       </c>
       <c r="J227" s="4" t="n">
-        <v>6994</v>
+        <v>8128</v>
       </c>
       <c r="K227" s="5" t="n">
-        <v>349.6875</v>
+        <v>406.4117647058824</v>
       </c>
     </row>
     <row r="228">
@@ -11690,11 +11690,11 @@
         </is>
       </c>
       <c r="G228" s="4" t="n">
-        <v>14796</v>
+        <v>15814</v>
       </c>
       <c r="H228" s="3" t="inlineStr">
         <is>
-          <t>13/22</t>
+          <t>14/22</t>
         </is>
       </c>
       <c r="I228" s="3" t="inlineStr">
@@ -11703,10 +11703,10 @@
         </is>
       </c>
       <c r="J228" s="4" t="n">
-        <v>25039</v>
+        <v>24851</v>
       </c>
       <c r="K228" s="5" t="n">
-        <v>1138.153846153846</v>
+        <v>1129.571428571429</v>
       </c>
     </row>
     <row r="229">
@@ -11788,11 +11788,11 @@
         </is>
       </c>
       <c r="G230" s="11" t="n">
-        <v>1840</v>
+        <v>1745</v>
       </c>
       <c r="H230" s="10" t="inlineStr">
         <is>
-          <t>16/24</t>
+          <t>17/24</t>
         </is>
       </c>
       <c r="I230" s="10" t="inlineStr">
@@ -11801,10 +11801,10 @@
         </is>
       </c>
       <c r="J230" s="11" t="n">
-        <v>2760</v>
+        <v>2464</v>
       </c>
       <c r="K230" s="12" t="n">
-        <v>115</v>
+        <v>102.6470588235294</v>
       </c>
     </row>
     <row r="231">
@@ -11837,11 +11837,11 @@
         </is>
       </c>
       <c r="G231" s="4" t="n">
-        <v>33402</v>
+        <v>37214</v>
       </c>
       <c r="H231" s="3" t="inlineStr">
         <is>
-          <t>11/20</t>
+          <t>12/20</t>
         </is>
       </c>
       <c r="I231" s="3" t="inlineStr">
@@ -11850,10 +11850,10 @@
         </is>
       </c>
       <c r="J231" s="4" t="n">
-        <v>60731</v>
+        <v>62023</v>
       </c>
       <c r="K231" s="5" t="n">
-        <v>3036.545454545455</v>
+        <v>3101.166666666667</v>
       </c>
     </row>
     <row r="232">
@@ -11886,11 +11886,11 @@
         </is>
       </c>
       <c r="G232" s="7" t="n">
-        <v>2769</v>
+        <v>4064</v>
       </c>
       <c r="H232" s="6" t="inlineStr">
         <is>
-          <t>11/21</t>
+          <t>12/21</t>
         </is>
       </c>
       <c r="I232" s="6" t="inlineStr">
@@ -11899,10 +11899,10 @@
         </is>
       </c>
       <c r="J232" s="7" t="n">
-        <v>5286</v>
+        <v>7112</v>
       </c>
       <c r="K232" s="8" t="n">
-        <v>251.7272727272727</v>
+        <v>338.6666666666667</v>
       </c>
     </row>
     <row r="233">
@@ -11935,11 +11935,11 @@
         </is>
       </c>
       <c r="G233" s="4" t="n">
-        <v>11348</v>
+        <v>12406</v>
       </c>
       <c r="H233" s="3" t="inlineStr">
         <is>
-          <t>11/23</t>
+          <t>12/23</t>
         </is>
       </c>
       <c r="I233" s="3" t="inlineStr">
@@ -11948,10 +11948,10 @@
         </is>
       </c>
       <c r="J233" s="4" t="n">
-        <v>23728</v>
+        <v>23778</v>
       </c>
       <c r="K233" s="5" t="n">
-        <v>1031.636363636364</v>
+        <v>1033.833333333333</v>
       </c>
     </row>
     <row r="234">
@@ -12004,52 +12004,52 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="9" t="inlineStr">
+      <c r="A235" s="6" t="inlineStr">
         <is>
           <t>YERCAUD</t>
         </is>
       </c>
-      <c r="B235" s="10" t="n">
+      <c r="B235" s="6" t="n">
         <v>83</v>
       </c>
-      <c r="C235" s="10" t="inlineStr">
+      <c r="C235" s="6" t="inlineStr">
         <is>
           <t>LAKSHMI JANARTHANAN. J</t>
         </is>
       </c>
-      <c r="D235" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E235" s="10" t="inlineStr">
+      <c r="D235" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E235" s="6" t="inlineStr">
         <is>
           <t>USHARANI. P</t>
         </is>
       </c>
-      <c r="F235" s="10" t="inlineStr">
+      <c r="F235" s="6" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G235" s="11" t="n">
-        <v>973</v>
-      </c>
-      <c r="H235" s="10" t="inlineStr">
-        <is>
-          <t>11/24</t>
-        </is>
-      </c>
-      <c r="I235" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J235" s="11" t="n">
-        <v>2123</v>
-      </c>
-      <c r="K235" s="12" t="n">
-        <v>88.45454545454545</v>
+      <c r="G235" s="7" t="n">
+        <v>1558</v>
+      </c>
+      <c r="H235" s="6" t="inlineStr">
+        <is>
+          <t>12/24</t>
+        </is>
+      </c>
+      <c r="I235" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J235" s="7" t="n">
+        <v>3116</v>
+      </c>
+      <c r="K235" s="8" t="n">
+        <v>129.8333333333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update election results snapshot (66.7% counted)
TVK 107, DMK 59, AIADMK 47. VIKRAVANDI flipped back to TVK by 169 votes.
9 knife-edge seats; THALLI at 24 (BJP), MANAPPARAI at 31 (TVK). 5 declared.

https://claude.ai/code/session_01MizbUy44JG5sXyvaf3Wekb
</commit_message>
<xml_diff>
--- a/tn_election_results_may2026.xlsx
+++ b/tn_election_results_may2026.xlsx
@@ -616,11 +616,11 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>17087</v>
+        <v>18967</v>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>12/31</t>
+          <t>13/31</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -629,10 +629,10 @@
         </is>
       </c>
       <c r="J2" s="4" t="n">
-        <v>44141</v>
+        <v>45229</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>1423.916666666667</v>
+        <v>1459</v>
       </c>
     </row>
     <row r="3">
@@ -665,11 +665,11 @@
         </is>
       </c>
       <c r="G3" s="7" t="n">
-        <v>4654</v>
+        <v>4796</v>
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
-          <t>9/20</t>
+          <t>10/20</t>
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr">
@@ -678,10 +678,10 @@
         </is>
       </c>
       <c r="J3" s="7" t="n">
-        <v>10342</v>
+        <v>9592</v>
       </c>
       <c r="K3" s="8" t="n">
-        <v>517.1111111111111</v>
+        <v>479.6</v>
       </c>
     </row>
     <row r="4">
@@ -930,52 +930,52 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>ANDIPATTI</t>
         </is>
       </c>
-      <c r="B9" s="10" t="n">
+      <c r="B9" s="6" t="n">
         <v>198</v>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>MAHARAJAN.A</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>LOGIRAJAN.A</t>
         </is>
       </c>
-      <c r="F9" s="10" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G9" s="11" t="n">
-        <v>1774</v>
-      </c>
-      <c r="H9" s="10" t="inlineStr">
-        <is>
-          <t>15/25</t>
-        </is>
-      </c>
-      <c r="I9" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J9" s="11" t="n">
-        <v>2957</v>
-      </c>
-      <c r="K9" s="12" t="n">
-        <v>118.2666666666667</v>
+      <c r="G9" s="7" t="n">
+        <v>2398</v>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>16/25</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="n">
+        <v>3747</v>
+      </c>
+      <c r="K9" s="8" t="n">
+        <v>149.875</v>
       </c>
     </row>
     <row r="10">
@@ -1204,11 +1204,11 @@
         </is>
       </c>
       <c r="G14" s="7" t="n">
-        <v>11861</v>
+        <v>11595</v>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>15/22</t>
+          <t>16/22</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
@@ -1217,10 +1217,10 @@
         </is>
       </c>
       <c r="J14" s="7" t="n">
-        <v>17396</v>
+        <v>15943</v>
       </c>
       <c r="K14" s="8" t="n">
-        <v>790.7333333333335</v>
+        <v>724.6875</v>
       </c>
     </row>
     <row r="15">
@@ -1351,11 +1351,11 @@
         </is>
       </c>
       <c r="G17" s="4" t="n">
-        <v>16268</v>
+        <v>17842</v>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>20/24</t>
+          <t>21/24</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -1364,10 +1364,10 @@
         </is>
       </c>
       <c r="J17" s="4" t="n">
-        <v>19522</v>
+        <v>20391</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>813.4</v>
+        <v>849.6190476190476</v>
       </c>
     </row>
     <row r="18">
@@ -1400,11 +1400,11 @@
         </is>
       </c>
       <c r="G18" s="7" t="n">
-        <v>3652</v>
+        <v>3083</v>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>12/20</t>
+          <t>13/20</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr">
@@ -1413,10 +1413,10 @@
         </is>
       </c>
       <c r="J18" s="7" t="n">
-        <v>6087</v>
+        <v>4743</v>
       </c>
       <c r="K18" s="8" t="n">
-        <v>304.3333333333333</v>
+        <v>237.1538461538462</v>
       </c>
     </row>
     <row r="19">
@@ -1449,11 +1449,11 @@
         </is>
       </c>
       <c r="G19" s="4" t="n">
-        <v>15139</v>
+        <v>18038</v>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>15/25</t>
+          <t>16/25</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -1462,10 +1462,10 @@
         </is>
       </c>
       <c r="J19" s="4" t="n">
-        <v>25232</v>
+        <v>28184</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>1009.266666666667</v>
+        <v>1127.375</v>
       </c>
     </row>
     <row r="20">
@@ -1596,11 +1596,11 @@
         </is>
       </c>
       <c r="G22" s="7" t="n">
-        <v>7484</v>
+        <v>8442</v>
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>18/27</t>
+          <t>19/27</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr">
@@ -1609,10 +1609,10 @@
         </is>
       </c>
       <c r="J22" s="7" t="n">
-        <v>11226</v>
+        <v>11997</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>415.7777777777778</v>
+        <v>444.3157894736842</v>
       </c>
     </row>
     <row r="23">
@@ -1645,11 +1645,11 @@
         </is>
       </c>
       <c r="G23" s="11" t="n">
-        <v>1440</v>
+        <v>954</v>
       </c>
       <c r="H23" s="10" t="inlineStr">
         <is>
-          <t>14/24</t>
+          <t>15/24</t>
         </is>
       </c>
       <c r="I23" s="10" t="inlineStr">
@@ -1658,10 +1658,10 @@
         </is>
       </c>
       <c r="J23" s="11" t="n">
-        <v>2469</v>
+        <v>1526</v>
       </c>
       <c r="K23" s="12" t="n">
-        <v>102.8571428571429</v>
+        <v>63.6</v>
       </c>
     </row>
     <row r="24">
@@ -1724,30 +1724,30 @@
       </c>
       <c r="C25" s="14" t="inlineStr">
         <is>
+          <t>V.P.TAMILSELVI</t>
+        </is>
+      </c>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E25" s="14" t="inlineStr">
+        <is>
           <t>A.BANNARI</t>
         </is>
       </c>
-      <c r="D25" s="14" t="inlineStr">
+      <c r="F25" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E25" s="14" t="inlineStr">
-        <is>
-          <t>V.P.TAMILSELVI</t>
-        </is>
-      </c>
-      <c r="F25" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
       <c r="G25" s="15" t="n">
-        <v>71</v>
+        <v>276</v>
       </c>
       <c r="H25" s="14" t="inlineStr">
         <is>
-          <t>16/24</t>
+          <t>17/24</t>
         </is>
       </c>
       <c r="I25" s="14" t="inlineStr">
@@ -1756,10 +1756,10 @@
         </is>
       </c>
       <c r="J25" s="15" t="n">
-        <v>106</v>
+        <v>390</v>
       </c>
       <c r="K25" s="16" t="n">
-        <v>4.4375</v>
+        <v>16.23529411764706</v>
       </c>
     </row>
     <row r="26">
@@ -1841,11 +1841,11 @@
         </is>
       </c>
       <c r="G27" s="7" t="n">
-        <v>2590</v>
+        <v>2697</v>
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>13/25</t>
+          <t>14/25</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
@@ -1854,10 +1854,10 @@
         </is>
       </c>
       <c r="J27" s="7" t="n">
-        <v>4981</v>
+        <v>4816</v>
       </c>
       <c r="K27" s="8" t="n">
-        <v>199.2307692307692</v>
+        <v>192.6428571428571</v>
       </c>
     </row>
     <row r="28">
@@ -1939,11 +1939,11 @@
         </is>
       </c>
       <c r="G29" s="7" t="n">
-        <v>4987</v>
+        <v>6016</v>
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>10/25</t>
+          <t>11/25</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
@@ -1952,10 +1952,10 @@
         </is>
       </c>
       <c r="J29" s="7" t="n">
-        <v>12468</v>
+        <v>13673</v>
       </c>
       <c r="K29" s="8" t="n">
-        <v>498.7</v>
+        <v>546.9090909090909</v>
       </c>
     </row>
     <row r="30">
@@ -2135,11 +2135,11 @@
         </is>
       </c>
       <c r="G33" s="7" t="n">
-        <v>4179</v>
+        <v>4757</v>
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>14/22</t>
+          <t>15/22</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
@@ -2148,10 +2148,10 @@
         </is>
       </c>
       <c r="J33" s="7" t="n">
-        <v>6567</v>
+        <v>6977</v>
       </c>
       <c r="K33" s="8" t="n">
-        <v>298.5</v>
+        <v>317.1333333333334</v>
       </c>
     </row>
     <row r="34">
@@ -2184,11 +2184,11 @@
         </is>
       </c>
       <c r="G34" s="4" t="n">
-        <v>7846</v>
+        <v>9163</v>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>9/25</t>
+          <t>10/25</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
@@ -2197,10 +2197,10 @@
         </is>
       </c>
       <c r="J34" s="4" t="n">
-        <v>21794</v>
+        <v>22908</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>871.7777777777778</v>
+        <v>916.3</v>
       </c>
     </row>
     <row r="35">
@@ -2429,11 +2429,11 @@
         </is>
       </c>
       <c r="G39" s="7" t="n">
-        <v>3369</v>
+        <v>2832</v>
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>10/25</t>
+          <t>11/25</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr">
@@ -2442,10 +2442,10 @@
         </is>
       </c>
       <c r="J39" s="7" t="n">
-        <v>8422</v>
+        <v>6436</v>
       </c>
       <c r="K39" s="8" t="n">
-        <v>336.9</v>
+        <v>257.4545454545454</v>
       </c>
     </row>
     <row r="40">
@@ -2576,11 +2576,11 @@
         </is>
       </c>
       <c r="G42" s="11" t="n">
-        <v>449</v>
+        <v>1739</v>
       </c>
       <c r="H42" s="10" t="inlineStr">
         <is>
-          <t>18/24</t>
+          <t>19/24</t>
         </is>
       </c>
       <c r="I42" s="10" t="inlineStr">
@@ -2589,10 +2589,10 @@
         </is>
       </c>
       <c r="J42" s="11" t="n">
-        <v>599</v>
+        <v>2197</v>
       </c>
       <c r="K42" s="12" t="n">
-        <v>24.94444444444444</v>
+        <v>91.52631578947368</v>
       </c>
     </row>
     <row r="43">
@@ -2674,11 +2674,11 @@
         </is>
       </c>
       <c r="G44" s="4" t="n">
-        <v>78058</v>
+        <v>82438</v>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>20/25</t>
+          <t>21/25</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
@@ -2687,10 +2687,10 @@
         </is>
       </c>
       <c r="J44" s="4" t="n">
-        <v>97572</v>
+        <v>98140</v>
       </c>
       <c r="K44" s="5" t="n">
-        <v>3902.9</v>
+        <v>3925.619047619048</v>
       </c>
     </row>
     <row r="45">
@@ -2723,11 +2723,11 @@
         </is>
       </c>
       <c r="G45" s="4" t="n">
-        <v>12407</v>
+        <v>13084</v>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>12/15</t>
+          <t>13/15</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
@@ -2736,10 +2736,10 @@
         </is>
       </c>
       <c r="J45" s="4" t="n">
-        <v>15509</v>
+        <v>15097</v>
       </c>
       <c r="K45" s="5" t="n">
-        <v>1033.916666666667</v>
+        <v>1006.461538461538</v>
       </c>
     </row>
     <row r="46">
@@ -2772,7 +2772,7 @@
         </is>
       </c>
       <c r="G46" s="4" t="n">
-        <v>22453</v>
+        <v>22362</v>
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
@@ -2785,10 +2785,10 @@
         </is>
       </c>
       <c r="J46" s="4" t="n">
-        <v>25095</v>
+        <v>24993</v>
       </c>
       <c r="K46" s="5" t="n">
-        <v>1320.764705882353</v>
+        <v>1315.411764705882</v>
       </c>
     </row>
     <row r="47">
@@ -2890,52 +2890,52 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr">
+      <c r="A49" s="6" t="inlineStr">
         <is>
           <t>GANGAVALLI</t>
         </is>
       </c>
-      <c r="B49" s="3" t="n">
+      <c r="B49" s="6" t="n">
         <v>81</v>
       </c>
-      <c r="C49" s="3" t="inlineStr">
+      <c r="C49" s="6" t="inlineStr">
         <is>
           <t>NALLATHAMBI. A</t>
         </is>
       </c>
-      <c r="D49" s="3" t="inlineStr">
+      <c r="D49" s="6" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E49" s="3" t="inlineStr">
+      <c r="E49" s="6" t="inlineStr">
         <is>
           <t>CHINNADURAI. K</t>
         </is>
       </c>
-      <c r="F49" s="3" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G49" s="4" t="n">
-        <v>13359</v>
-      </c>
-      <c r="H49" s="3" t="inlineStr">
-        <is>
-          <t>13/20</t>
-        </is>
-      </c>
-      <c r="I49" s="3" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J49" s="4" t="n">
-        <v>20552</v>
-      </c>
-      <c r="K49" s="5" t="n">
-        <v>1027.615384615385</v>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G49" s="7" t="n">
+        <v>13962</v>
+      </c>
+      <c r="H49" s="6" t="inlineStr">
+        <is>
+          <t>14/20</t>
+        </is>
+      </c>
+      <c r="I49" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J49" s="7" t="n">
+        <v>19946</v>
+      </c>
+      <c r="K49" s="8" t="n">
+        <v>997.2857142857143</v>
       </c>
     </row>
     <row r="50">
@@ -3017,11 +3017,11 @@
         </is>
       </c>
       <c r="G51" s="4" t="n">
-        <v>15852</v>
+        <v>16234</v>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>19/23</t>
+          <t>20/23</t>
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr">
@@ -3030,10 +3030,10 @@
         </is>
       </c>
       <c r="J51" s="4" t="n">
-        <v>19189</v>
+        <v>18669</v>
       </c>
       <c r="K51" s="5" t="n">
-        <v>834.3157894736842</v>
+        <v>811.7</v>
       </c>
     </row>
     <row r="52">
@@ -3164,11 +3164,11 @@
         </is>
       </c>
       <c r="G54" s="4" t="n">
-        <v>17456</v>
+        <v>17793</v>
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>14/25</t>
+          <t>15/25</t>
         </is>
       </c>
       <c r="I54" s="3" t="inlineStr">
@@ -3177,59 +3177,59 @@
         </is>
       </c>
       <c r="J54" s="4" t="n">
-        <v>31171</v>
+        <v>29655</v>
       </c>
       <c r="K54" s="5" t="n">
-        <v>1246.857142857143</v>
+        <v>1186.2</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="6" t="inlineStr">
+      <c r="A55" s="2" t="inlineStr">
         <is>
           <t>HARBOUR</t>
         </is>
       </c>
-      <c r="B55" s="6" t="n">
+      <c r="B55" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="C55" s="6" t="inlineStr">
+      <c r="C55" s="3" t="inlineStr">
         <is>
           <t>P K SEKARBABU</t>
         </is>
       </c>
-      <c r="D55" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E55" s="6" t="inlineStr">
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
         <is>
           <t>SINORA P S ASHOK</t>
         </is>
       </c>
-      <c r="F55" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G55" s="7" t="n">
-        <v>9760</v>
-      </c>
-      <c r="H55" s="6" t="inlineStr">
-        <is>
-          <t>10/14</t>
-        </is>
-      </c>
-      <c r="I55" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J55" s="7" t="n">
-        <v>13664</v>
-      </c>
-      <c r="K55" s="8" t="n">
-        <v>976</v>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="n">
+        <v>10318</v>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>11/14</t>
+        </is>
+      </c>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J55" s="4" t="n">
+        <v>13132</v>
+      </c>
+      <c r="K55" s="5" t="n">
+        <v>938</v>
       </c>
     </row>
     <row r="56">
@@ -3311,11 +3311,11 @@
         </is>
       </c>
       <c r="G57" s="4" t="n">
-        <v>24189</v>
+        <v>24278</v>
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>16/34</t>
+          <t>17/34</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr">
@@ -3324,10 +3324,10 @@
         </is>
       </c>
       <c r="J57" s="4" t="n">
-        <v>51402</v>
+        <v>48556</v>
       </c>
       <c r="K57" s="5" t="n">
-        <v>1511.8125</v>
+        <v>1428.117647058823</v>
       </c>
     </row>
     <row r="58">
@@ -3380,52 +3380,52 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="6" t="inlineStr">
+      <c r="A59" s="2" t="inlineStr">
         <is>
           <t>JOLARPET</t>
         </is>
       </c>
-      <c r="B59" s="6" t="n">
+      <c r="B59" s="3" t="n">
         <v>49</v>
       </c>
-      <c r="C59" s="6" t="inlineStr">
+      <c r="C59" s="3" t="inlineStr">
         <is>
           <t>VEERAMANI K.C.</t>
         </is>
       </c>
-      <c r="D59" s="6" t="inlineStr">
+      <c r="D59" s="3" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E59" s="6" t="inlineStr">
+      <c r="E59" s="3" t="inlineStr">
         <is>
           <t>MUNISAMY C</t>
         </is>
       </c>
-      <c r="F59" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G59" s="7" t="n">
-        <v>9862</v>
-      </c>
-      <c r="H59" s="6" t="inlineStr">
-        <is>
-          <t>14/21</t>
-        </is>
-      </c>
-      <c r="I59" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J59" s="7" t="n">
-        <v>14793</v>
-      </c>
-      <c r="K59" s="8" t="n">
-        <v>704.4285714285714</v>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G59" s="4" t="n">
+        <v>13027</v>
+      </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>16/21</t>
+        </is>
+      </c>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J59" s="4" t="n">
+        <v>17098</v>
+      </c>
+      <c r="K59" s="5" t="n">
+        <v>814.1875</v>
       </c>
     </row>
     <row r="60">
@@ -3556,11 +3556,11 @@
         </is>
       </c>
       <c r="G62" s="7" t="n">
-        <v>3031</v>
+        <v>3152</v>
       </c>
       <c r="H62" s="6" t="inlineStr">
         <is>
-          <t>14/27</t>
+          <t>15/27</t>
         </is>
       </c>
       <c r="I62" s="6" t="inlineStr">
@@ -3569,10 +3569,10 @@
         </is>
       </c>
       <c r="J62" s="7" t="n">
-        <v>5846</v>
+        <v>5674</v>
       </c>
       <c r="K62" s="8" t="n">
-        <v>216.5</v>
+        <v>210.1333333333333</v>
       </c>
     </row>
     <row r="63">
@@ -3605,11 +3605,11 @@
         </is>
       </c>
       <c r="G63" s="7" t="n">
-        <v>5188</v>
+        <v>6289</v>
       </c>
       <c r="H63" s="6" t="inlineStr">
         <is>
-          <t>13/26</t>
+          <t>14/26</t>
         </is>
       </c>
       <c r="I63" s="6" t="inlineStr">
@@ -3618,10 +3618,10 @@
         </is>
       </c>
       <c r="J63" s="7" t="n">
-        <v>10376</v>
+        <v>11680</v>
       </c>
       <c r="K63" s="8" t="n">
-        <v>399.0769230769231</v>
+        <v>449.2142857142857</v>
       </c>
     </row>
     <row r="64">
@@ -3654,11 +3654,11 @@
         </is>
       </c>
       <c r="G64" s="7" t="n">
-        <v>4187</v>
+        <v>5199</v>
       </c>
       <c r="H64" s="6" t="inlineStr">
         <is>
-          <t>14/23</t>
+          <t>15/23</t>
         </is>
       </c>
       <c r="I64" s="6" t="inlineStr">
@@ -3667,10 +3667,10 @@
         </is>
       </c>
       <c r="J64" s="7" t="n">
-        <v>6879</v>
+        <v>7972</v>
       </c>
       <c r="K64" s="8" t="n">
-        <v>299.0714285714286</v>
+        <v>346.6</v>
       </c>
     </row>
     <row r="65">
@@ -3752,11 +3752,11 @@
         </is>
       </c>
       <c r="G66" s="4" t="n">
-        <v>23023</v>
+        <v>24684</v>
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>13/28</t>
+          <t>14/28</t>
         </is>
       </c>
       <c r="I66" s="3" t="inlineStr">
@@ -3765,10 +3765,10 @@
         </is>
       </c>
       <c r="J66" s="4" t="n">
-        <v>49588</v>
+        <v>49368</v>
       </c>
       <c r="K66" s="5" t="n">
-        <v>1771</v>
+        <v>1763.142857142857</v>
       </c>
     </row>
     <row r="67">
@@ -3801,11 +3801,11 @@
         </is>
       </c>
       <c r="G67" s="7" t="n">
-        <v>5843</v>
+        <v>5280</v>
       </c>
       <c r="H67" s="6" t="inlineStr">
         <is>
-          <t>11/21</t>
+          <t>12/21</t>
         </is>
       </c>
       <c r="I67" s="6" t="inlineStr">
@@ -3814,10 +3814,10 @@
         </is>
       </c>
       <c r="J67" s="7" t="n">
-        <v>11155</v>
+        <v>9240</v>
       </c>
       <c r="K67" s="8" t="n">
-        <v>531.1818181818181</v>
+        <v>440</v>
       </c>
     </row>
     <row r="68">
@@ -3899,11 +3899,11 @@
         </is>
       </c>
       <c r="G69" s="4" t="n">
-        <v>16899</v>
+        <v>17932</v>
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
-          <t>12/21</t>
+          <t>13/21</t>
         </is>
       </c>
       <c r="I69" s="3" t="inlineStr">
@@ -3912,10 +3912,10 @@
         </is>
       </c>
       <c r="J69" s="4" t="n">
-        <v>29573</v>
+        <v>28967</v>
       </c>
       <c r="K69" s="5" t="n">
-        <v>1408.25</v>
+        <v>1379.384615384615</v>
       </c>
     </row>
     <row r="70">
@@ -3948,11 +3948,11 @@
         </is>
       </c>
       <c r="G70" s="4" t="n">
-        <v>37275</v>
+        <v>39671</v>
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>23/28</t>
+          <t>24/28</t>
         </is>
       </c>
       <c r="I70" s="3" t="inlineStr">
@@ -3961,10 +3961,10 @@
         </is>
       </c>
       <c r="J70" s="4" t="n">
-        <v>45378</v>
+        <v>46283</v>
       </c>
       <c r="K70" s="5" t="n">
-        <v>1620.652173913043</v>
+        <v>1652.958333333333</v>
       </c>
     </row>
     <row r="71">
@@ -4282,20 +4282,20 @@
       </c>
       <c r="E77" s="6" t="inlineStr">
         <is>
-          <t>KADAMBUR RAJU.C</t>
+          <t>BALASUBRAMANIAN.S</t>
         </is>
       </c>
       <c r="F77" s="6" t="inlineStr">
         <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
+          <t>Tamilaga Vettri Kazhagam</t>
         </is>
       </c>
       <c r="G77" s="7" t="n">
-        <v>4122</v>
+        <v>5265</v>
       </c>
       <c r="H77" s="6" t="inlineStr">
         <is>
-          <t>13/23</t>
+          <t>14/23</t>
         </is>
       </c>
       <c r="I77" s="6" t="inlineStr">
@@ -4304,10 +4304,10 @@
         </is>
       </c>
       <c r="J77" s="7" t="n">
-        <v>7293</v>
+        <v>8650</v>
       </c>
       <c r="K77" s="8" t="n">
-        <v>317.0769230769231</v>
+        <v>376.0714285714286</v>
       </c>
     </row>
     <row r="78">
@@ -4389,11 +4389,11 @@
         </is>
       </c>
       <c r="G79" s="7" t="n">
-        <v>3031</v>
+        <v>2946</v>
       </c>
       <c r="H79" s="6" t="inlineStr">
         <is>
-          <t>12/20</t>
+          <t>13/20</t>
         </is>
       </c>
       <c r="I79" s="6" t="inlineStr">
@@ -4402,10 +4402,10 @@
         </is>
       </c>
       <c r="J79" s="7" t="n">
-        <v>5052</v>
+        <v>4532</v>
       </c>
       <c r="K79" s="8" t="n">
-        <v>252.5833333333333</v>
+        <v>226.6153846153846</v>
       </c>
     </row>
     <row r="80">
@@ -4634,11 +4634,11 @@
         </is>
       </c>
       <c r="G84" s="7" t="n">
-        <v>2732</v>
+        <v>3474</v>
       </c>
       <c r="H84" s="6" t="inlineStr">
         <is>
-          <t>15/20</t>
+          <t>16/20</t>
         </is>
       </c>
       <c r="I84" s="6" t="inlineStr">
@@ -4647,10 +4647,10 @@
         </is>
       </c>
       <c r="J84" s="7" t="n">
-        <v>3643</v>
+        <v>4342</v>
       </c>
       <c r="K84" s="8" t="n">
-        <v>182.1333333333333</v>
+        <v>217.125</v>
       </c>
     </row>
     <row r="85">
@@ -4683,11 +4683,11 @@
         </is>
       </c>
       <c r="G85" s="11" t="n">
-        <v>1174</v>
+        <v>1181</v>
       </c>
       <c r="H85" s="10" t="inlineStr">
         <is>
-          <t>14/20</t>
+          <t>15/20</t>
         </is>
       </c>
       <c r="I85" s="10" t="inlineStr">
@@ -4696,10 +4696,10 @@
         </is>
       </c>
       <c r="J85" s="11" t="n">
-        <v>1677</v>
+        <v>1575</v>
       </c>
       <c r="K85" s="12" t="n">
-        <v>83.85714285714286</v>
+        <v>78.73333333333333</v>
       </c>
     </row>
     <row r="86">
@@ -4781,7 +4781,7 @@
         </is>
       </c>
       <c r="G87" s="4" t="n">
-        <v>86172</v>
+        <v>86155</v>
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
@@ -4794,10 +4794,10 @@
         </is>
       </c>
       <c r="J87" s="4" t="n">
-        <v>96310</v>
+        <v>96291</v>
       </c>
       <c r="K87" s="5" t="n">
-        <v>5068.941176470588</v>
+        <v>5067.941176470588</v>
       </c>
     </row>
     <row r="88">
@@ -4879,11 +4879,11 @@
         </is>
       </c>
       <c r="G89" s="7" t="n">
-        <v>7334</v>
+        <v>8230</v>
       </c>
       <c r="H89" s="6" t="inlineStr">
         <is>
-          <t>19/29</t>
+          <t>20/29</t>
         </is>
       </c>
       <c r="I89" s="6" t="inlineStr">
@@ -4892,10 +4892,10 @@
         </is>
       </c>
       <c r="J89" s="7" t="n">
-        <v>11194</v>
+        <v>11934</v>
       </c>
       <c r="K89" s="8" t="n">
-        <v>386</v>
+        <v>411.5</v>
       </c>
     </row>
     <row r="90">
@@ -4997,52 +4997,52 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="6" t="inlineStr">
+      <c r="A92" s="2" t="inlineStr">
         <is>
           <t>MADURAI WEST</t>
         </is>
       </c>
-      <c r="B92" s="6" t="n">
+      <c r="B92" s="3" t="n">
         <v>194</v>
       </c>
-      <c r="C92" s="6" t="inlineStr">
+      <c r="C92" s="3" t="inlineStr">
         <is>
           <t>THANGAPANDI SR</t>
         </is>
       </c>
-      <c r="D92" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E92" s="6" t="inlineStr">
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E92" s="3" t="inlineStr">
         <is>
           <t>BALAJI R</t>
         </is>
       </c>
-      <c r="F92" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G92" s="7" t="n">
-        <v>4966</v>
-      </c>
-      <c r="H92" s="6" t="inlineStr">
-        <is>
-          <t>17/24</t>
-        </is>
-      </c>
-      <c r="I92" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J92" s="7" t="n">
-        <v>7011</v>
-      </c>
-      <c r="K92" s="8" t="n">
-        <v>292.1176470588235</v>
+      <c r="F92" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G92" s="4" t="n">
+        <v>6006</v>
+      </c>
+      <c r="H92" s="3" t="inlineStr">
+        <is>
+          <t>18/24</t>
+        </is>
+      </c>
+      <c r="I92" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J92" s="4" t="n">
+        <v>8008</v>
+      </c>
+      <c r="K92" s="5" t="n">
+        <v>333.6666666666667</v>
       </c>
     </row>
     <row r="93">
@@ -5075,11 +5075,11 @@
         </is>
       </c>
       <c r="G93" s="7" t="n">
-        <v>4749</v>
+        <v>5429</v>
       </c>
       <c r="H93" s="6" t="inlineStr">
         <is>
-          <t>14/21</t>
+          <t>15/21</t>
         </is>
       </c>
       <c r="I93" s="6" t="inlineStr">
@@ -5088,10 +5088,10 @@
         </is>
       </c>
       <c r="J93" s="7" t="n">
-        <v>7124</v>
+        <v>7601</v>
       </c>
       <c r="K93" s="8" t="n">
-        <v>339.2142857142857</v>
+        <v>361.9333333333333</v>
       </c>
     </row>
     <row r="94">
@@ -5173,11 +5173,11 @@
         </is>
       </c>
       <c r="G95" s="4" t="n">
-        <v>25203</v>
+        <v>26593</v>
       </c>
       <c r="H95" s="3" t="inlineStr">
         <is>
-          <t>15/20</t>
+          <t>16/20</t>
         </is>
       </c>
       <c r="I95" s="3" t="inlineStr">
@@ -5186,10 +5186,10 @@
         </is>
       </c>
       <c r="J95" s="4" t="n">
-        <v>33604</v>
+        <v>33241</v>
       </c>
       <c r="K95" s="5" t="n">
-        <v>1680.2</v>
+        <v>1662.0625</v>
       </c>
     </row>
     <row r="96">
@@ -5271,11 +5271,11 @@
         </is>
       </c>
       <c r="G97" s="7" t="n">
-        <v>4081</v>
+        <v>4247</v>
       </c>
       <c r="H97" s="6" t="inlineStr">
         <is>
-          <t>10/27</t>
+          <t>11/27</t>
         </is>
       </c>
       <c r="I97" s="6" t="inlineStr">
@@ -5284,10 +5284,10 @@
         </is>
       </c>
       <c r="J97" s="7" t="n">
-        <v>11019</v>
+        <v>10424</v>
       </c>
       <c r="K97" s="8" t="n">
-        <v>408.1</v>
+        <v>386.0909090909091</v>
       </c>
     </row>
     <row r="98">
@@ -5369,11 +5369,11 @@
         </is>
       </c>
       <c r="G99" s="11" t="n">
-        <v>2017</v>
+        <v>1198</v>
       </c>
       <c r="H99" s="10" t="inlineStr">
         <is>
-          <t>16/22</t>
+          <t>17/22</t>
         </is>
       </c>
       <c r="I99" s="10" t="inlineStr">
@@ -5382,10 +5382,10 @@
         </is>
       </c>
       <c r="J99" s="11" t="n">
-        <v>2773</v>
+        <v>1550</v>
       </c>
       <c r="K99" s="12" t="n">
-        <v>126.0625</v>
+        <v>70.47058823529412</v>
       </c>
     </row>
     <row r="100">
@@ -5614,11 +5614,11 @@
         </is>
       </c>
       <c r="G104" s="7" t="n">
-        <v>3563</v>
+        <v>3226</v>
       </c>
       <c r="H104" s="6" t="inlineStr">
         <is>
-          <t>16/21</t>
+          <t>17/21</t>
         </is>
       </c>
       <c r="I104" s="6" t="inlineStr">
@@ -5627,10 +5627,10 @@
         </is>
       </c>
       <c r="J104" s="7" t="n">
-        <v>4676</v>
+        <v>3985</v>
       </c>
       <c r="K104" s="8" t="n">
-        <v>222.6875</v>
+        <v>189.7647058823529</v>
       </c>
     </row>
     <row r="105">
@@ -5663,11 +5663,11 @@
         </is>
       </c>
       <c r="G105" s="7" t="n">
-        <v>11364</v>
+        <v>11356</v>
       </c>
       <c r="H105" s="6" t="inlineStr">
         <is>
-          <t>19/30</t>
+          <t>20/30</t>
         </is>
       </c>
       <c r="I105" s="6" t="inlineStr">
@@ -5676,10 +5676,10 @@
         </is>
       </c>
       <c r="J105" s="7" t="n">
-        <v>17943</v>
+        <v>17034</v>
       </c>
       <c r="K105" s="8" t="n">
-        <v>598.1052631578947</v>
+        <v>567.8</v>
       </c>
     </row>
     <row r="106">
@@ -5703,20 +5703,20 @@
       </c>
       <c r="E106" s="3" t="inlineStr">
         <is>
-          <t>N.YOGANATHAN</t>
+          <t>N.S.KARUNAIRAAJA</t>
         </is>
       </c>
       <c r="F106" s="3" t="inlineStr">
         <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
+          <t>Dravida Munnetra Kazhagam</t>
         </is>
       </c>
       <c r="G106" s="4" t="n">
-        <v>16236</v>
+        <v>17883</v>
       </c>
       <c r="H106" s="3" t="inlineStr">
         <is>
-          <t>18/21</t>
+          <t>19/21</t>
         </is>
       </c>
       <c r="I106" s="3" t="inlineStr">
@@ -5725,10 +5725,10 @@
         </is>
       </c>
       <c r="J106" s="4" t="n">
-        <v>18942</v>
+        <v>19765</v>
       </c>
       <c r="K106" s="5" t="n">
-        <v>902</v>
+        <v>941.2105263157895</v>
       </c>
     </row>
     <row r="107">
@@ -5859,11 +5859,11 @@
         </is>
       </c>
       <c r="G109" s="7" t="n">
-        <v>4719</v>
+        <v>3456</v>
       </c>
       <c r="H109" s="6" t="inlineStr">
         <is>
-          <t>17/23</t>
+          <t>18/23</t>
         </is>
       </c>
       <c r="I109" s="6" t="inlineStr">
@@ -5872,10 +5872,10 @@
         </is>
       </c>
       <c r="J109" s="7" t="n">
-        <v>6385</v>
+        <v>4416</v>
       </c>
       <c r="K109" s="8" t="n">
-        <v>277.5882352941176</v>
+        <v>192</v>
       </c>
     </row>
     <row r="110">
@@ -5957,11 +5957,11 @@
         </is>
       </c>
       <c r="G111" s="4" t="n">
-        <v>15331</v>
+        <v>16419</v>
       </c>
       <c r="H111" s="3" t="inlineStr">
         <is>
-          <t>24/25</t>
+          <t>25/25</t>
         </is>
       </c>
       <c r="I111" s="3" t="inlineStr">
@@ -5970,10 +5970,10 @@
         </is>
       </c>
       <c r="J111" s="4" t="n">
-        <v>15970</v>
+        <v>16419</v>
       </c>
       <c r="K111" s="5" t="n">
-        <v>638.7916666666666</v>
+        <v>656.76</v>
       </c>
     </row>
     <row r="112">
@@ -6006,11 +6006,11 @@
         </is>
       </c>
       <c r="G112" s="4" t="n">
-        <v>29643</v>
+        <v>30870</v>
       </c>
       <c r="H112" s="3" t="inlineStr">
         <is>
-          <t>18/25</t>
+          <t>19/25</t>
         </is>
       </c>
       <c r="I112" s="3" t="inlineStr">
@@ -6019,10 +6019,10 @@
         </is>
       </c>
       <c r="J112" s="4" t="n">
-        <v>41171</v>
+        <v>40618</v>
       </c>
       <c r="K112" s="5" t="n">
-        <v>1646.833333333333</v>
+        <v>1624.736842105263</v>
       </c>
     </row>
     <row r="113">
@@ -6124,52 +6124,52 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="6" t="inlineStr">
+      <c r="A115" s="9" t="inlineStr">
         <is>
           <t>NILAKKOTTAI</t>
         </is>
       </c>
-      <c r="B115" s="6" t="n">
+      <c r="B115" s="10" t="n">
         <v>130</v>
       </c>
-      <c r="C115" s="6" t="inlineStr">
+      <c r="C115" s="10" t="inlineStr">
         <is>
           <t>NAGAJOTHI.S</t>
         </is>
       </c>
-      <c r="D115" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E115" s="6" t="inlineStr">
+      <c r="D115" s="10" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E115" s="10" t="inlineStr">
         <is>
           <t>AYYANAR.R</t>
         </is>
       </c>
-      <c r="F115" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G115" s="7" t="n">
-        <v>2008</v>
-      </c>
-      <c r="H115" s="6" t="inlineStr">
-        <is>
-          <t>11/23</t>
-        </is>
-      </c>
-      <c r="I115" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J115" s="7" t="n">
-        <v>4199</v>
-      </c>
-      <c r="K115" s="8" t="n">
-        <v>182.5454545454545</v>
+      <c r="F115" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G115" s="11" t="n">
+        <v>520</v>
+      </c>
+      <c r="H115" s="10" t="inlineStr">
+        <is>
+          <t>12/23</t>
+        </is>
+      </c>
+      <c r="I115" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J115" s="11" t="n">
+        <v>997</v>
+      </c>
+      <c r="K115" s="12" t="n">
+        <v>43.33333333333334</v>
       </c>
     </row>
     <row r="116">
@@ -6349,11 +6349,11 @@
         </is>
       </c>
       <c r="G119" s="4" t="n">
-        <v>22812</v>
+        <v>22447</v>
       </c>
       <c r="H119" s="3" t="inlineStr">
         <is>
-          <t>15/23</t>
+          <t>16/23</t>
         </is>
       </c>
       <c r="I119" s="3" t="inlineStr">
@@ -6362,10 +6362,10 @@
         </is>
       </c>
       <c r="J119" s="4" t="n">
-        <v>34978</v>
+        <v>32268</v>
       </c>
       <c r="K119" s="5" t="n">
-        <v>1520.8</v>
+        <v>1402.9375</v>
       </c>
     </row>
     <row r="120">
@@ -6447,11 +6447,11 @@
         </is>
       </c>
       <c r="G121" s="4" t="n">
-        <v>28586</v>
+        <v>31091</v>
       </c>
       <c r="H121" s="3" t="inlineStr">
         <is>
-          <t>18/23</t>
+          <t>19/23</t>
         </is>
       </c>
       <c r="I121" s="3" t="inlineStr">
@@ -6460,10 +6460,10 @@
         </is>
       </c>
       <c r="J121" s="4" t="n">
-        <v>36527</v>
+        <v>37636</v>
       </c>
       <c r="K121" s="5" t="n">
-        <v>1588.111111111111</v>
+        <v>1636.368421052632</v>
       </c>
     </row>
     <row r="122">
@@ -6487,20 +6487,20 @@
       </c>
       <c r="E122" s="6" t="inlineStr">
         <is>
-          <t>PANDI. N</t>
+          <t>DR. PRAVEEN KUMAR. M</t>
         </is>
       </c>
       <c r="F122" s="6" t="inlineStr">
         <is>
-          <t>Communist Party of India (Marxist)</t>
+          <t>Tamilaga Vettri Kazhagam</t>
         </is>
       </c>
       <c r="G122" s="7" t="n">
-        <v>2886</v>
+        <v>2987</v>
       </c>
       <c r="H122" s="6" t="inlineStr">
         <is>
-          <t>17/25</t>
+          <t>18/25</t>
         </is>
       </c>
       <c r="I122" s="6" t="inlineStr">
@@ -6509,10 +6509,10 @@
         </is>
       </c>
       <c r="J122" s="7" t="n">
-        <v>4244</v>
+        <v>4149</v>
       </c>
       <c r="K122" s="8" t="n">
-        <v>169.7647058823529</v>
+        <v>165.9444444444445</v>
       </c>
     </row>
     <row r="123">
@@ -6594,11 +6594,11 @@
         </is>
       </c>
       <c r="G124" s="4" t="n">
-        <v>30529</v>
+        <v>32307</v>
       </c>
       <c r="H124" s="3" t="inlineStr">
         <is>
-          <t>22/35</t>
+          <t>23/35</t>
         </is>
       </c>
       <c r="I124" s="3" t="inlineStr">
@@ -6607,10 +6607,10 @@
         </is>
       </c>
       <c r="J124" s="4" t="n">
-        <v>48569</v>
+        <v>49163</v>
       </c>
       <c r="K124" s="5" t="n">
-        <v>1387.681818181818</v>
+        <v>1404.652173913043</v>
       </c>
     </row>
     <row r="125">
@@ -6643,11 +6643,11 @@
         </is>
       </c>
       <c r="G125" s="4" t="n">
-        <v>26160</v>
+        <v>27588</v>
       </c>
       <c r="H125" s="3" t="inlineStr">
         <is>
-          <t>16/34</t>
+          <t>17/34</t>
         </is>
       </c>
       <c r="I125" s="3" t="inlineStr">
@@ -6656,10 +6656,10 @@
         </is>
       </c>
       <c r="J125" s="4" t="n">
-        <v>55590</v>
+        <v>55176</v>
       </c>
       <c r="K125" s="5" t="n">
-        <v>1635</v>
+        <v>1622.823529411765</v>
       </c>
     </row>
     <row r="126">
@@ -6741,11 +6741,11 @@
         </is>
       </c>
       <c r="G127" s="7" t="n">
-        <v>6639</v>
+        <v>5554</v>
       </c>
       <c r="H127" s="6" t="inlineStr">
         <is>
-          <t>10/23</t>
+          <t>11/23</t>
         </is>
       </c>
       <c r="I127" s="6" t="inlineStr">
@@ -6754,10 +6754,10 @@
         </is>
       </c>
       <c r="J127" s="7" t="n">
-        <v>15270</v>
+        <v>11613</v>
       </c>
       <c r="K127" s="8" t="n">
-        <v>663.9</v>
+        <v>504.9090909090909</v>
       </c>
     </row>
     <row r="128">
@@ -6790,11 +6790,11 @@
         </is>
       </c>
       <c r="G128" s="4" t="n">
-        <v>34889</v>
+        <v>35402</v>
       </c>
       <c r="H128" s="3" t="inlineStr">
         <is>
-          <t>19/23</t>
+          <t>20/23</t>
         </is>
       </c>
       <c r="I128" s="3" t="inlineStr">
@@ -6803,10 +6803,10 @@
         </is>
       </c>
       <c r="J128" s="4" t="n">
-        <v>42234</v>
+        <v>40712</v>
       </c>
       <c r="K128" s="5" t="n">
-        <v>1836.263157894737</v>
+        <v>1770.1</v>
       </c>
     </row>
     <row r="129">
@@ -6839,11 +6839,11 @@
         </is>
       </c>
       <c r="G129" s="11" t="n">
-        <v>523</v>
+        <v>1341</v>
       </c>
       <c r="H129" s="10" t="inlineStr">
         <is>
-          <t>19/24</t>
+          <t>20/24</t>
         </is>
       </c>
       <c r="I129" s="10" t="inlineStr">
@@ -6852,10 +6852,10 @@
         </is>
       </c>
       <c r="J129" s="11" t="n">
-        <v>661</v>
+        <v>1609</v>
       </c>
       <c r="K129" s="12" t="n">
-        <v>27.52631578947368</v>
+        <v>67.05</v>
       </c>
     </row>
     <row r="130">
@@ -6888,11 +6888,11 @@
         </is>
       </c>
       <c r="G130" s="11" t="n">
-        <v>1116</v>
+        <v>1542</v>
       </c>
       <c r="H130" s="10" t="inlineStr">
         <is>
-          <t>10/20</t>
+          <t>11/20</t>
         </is>
       </c>
       <c r="I130" s="10" t="inlineStr">
@@ -6901,10 +6901,10 @@
         </is>
       </c>
       <c r="J130" s="11" t="n">
-        <v>2232</v>
+        <v>2804</v>
       </c>
       <c r="K130" s="12" t="n">
-        <v>111.6</v>
+        <v>140.1818181818182</v>
       </c>
     </row>
     <row r="131">
@@ -6937,11 +6937,11 @@
         </is>
       </c>
       <c r="G131" s="7" t="n">
-        <v>5292</v>
+        <v>5130</v>
       </c>
       <c r="H131" s="6" t="inlineStr">
         <is>
-          <t>12/23</t>
+          <t>13/23</t>
         </is>
       </c>
       <c r="I131" s="6" t="inlineStr">
@@ -6950,10 +6950,10 @@
         </is>
       </c>
       <c r="J131" s="7" t="n">
-        <v>10143</v>
+        <v>9076</v>
       </c>
       <c r="K131" s="8" t="n">
-        <v>441</v>
+        <v>394.6153846153846</v>
       </c>
     </row>
     <row r="132">
@@ -7035,11 +7035,11 @@
         </is>
       </c>
       <c r="G133" s="7" t="n">
-        <v>9318</v>
+        <v>10019</v>
       </c>
       <c r="H133" s="6" t="inlineStr">
         <is>
-          <t>19/28</t>
+          <t>20/28</t>
         </is>
       </c>
       <c r="I133" s="6" t="inlineStr">
@@ -7048,10 +7048,10 @@
         </is>
       </c>
       <c r="J133" s="7" t="n">
-        <v>13732</v>
+        <v>14027</v>
       </c>
       <c r="K133" s="8" t="n">
-        <v>490.421052631579</v>
+        <v>500.95</v>
       </c>
     </row>
     <row r="134">
@@ -7280,11 +7280,11 @@
         </is>
       </c>
       <c r="G138" s="11" t="n">
-        <v>2359</v>
+        <v>2609</v>
       </c>
       <c r="H138" s="10" t="inlineStr">
         <is>
-          <t>17/20</t>
+          <t>18/20</t>
         </is>
       </c>
       <c r="I138" s="10" t="inlineStr">
@@ -7293,10 +7293,10 @@
         </is>
       </c>
       <c r="J138" s="11" t="n">
-        <v>2775</v>
+        <v>2899</v>
       </c>
       <c r="K138" s="12" t="n">
-        <v>138.7647058823529</v>
+        <v>144.9444444444445</v>
       </c>
     </row>
     <row r="139">
@@ -7378,11 +7378,11 @@
         </is>
       </c>
       <c r="G140" s="4" t="n">
-        <v>36253</v>
+        <v>38889</v>
       </c>
       <c r="H140" s="3" t="inlineStr">
         <is>
-          <t>16/24</t>
+          <t>17/24</t>
         </is>
       </c>
       <c r="I140" s="3" t="inlineStr">
@@ -7391,10 +7391,10 @@
         </is>
       </c>
       <c r="J140" s="4" t="n">
-        <v>54380</v>
+        <v>54902</v>
       </c>
       <c r="K140" s="5" t="n">
-        <v>2265.8125</v>
+        <v>2287.588235294118</v>
       </c>
     </row>
     <row r="141">
@@ -7476,11 +7476,11 @@
         </is>
       </c>
       <c r="G142" s="4" t="n">
-        <v>55671</v>
+        <v>58192</v>
       </c>
       <c r="H142" s="3" t="inlineStr">
         <is>
-          <t>16/23</t>
+          <t>17/23</t>
         </is>
       </c>
       <c r="I142" s="3" t="inlineStr">
@@ -7489,10 +7489,10 @@
         </is>
       </c>
       <c r="J142" s="4" t="n">
-        <v>80027</v>
+        <v>78730</v>
       </c>
       <c r="K142" s="5" t="n">
-        <v>3479.4375</v>
+        <v>3423.058823529412</v>
       </c>
     </row>
     <row r="143">
@@ -7525,11 +7525,11 @@
         </is>
       </c>
       <c r="G143" s="7" t="n">
-        <v>1671</v>
+        <v>2266</v>
       </c>
       <c r="H143" s="6" t="inlineStr">
         <is>
-          <t>12/22</t>
+          <t>13/22</t>
         </is>
       </c>
       <c r="I143" s="6" t="inlineStr">
@@ -7538,10 +7538,10 @@
         </is>
       </c>
       <c r="J143" s="7" t="n">
-        <v>3064</v>
+        <v>3835</v>
       </c>
       <c r="K143" s="8" t="n">
-        <v>139.25</v>
+        <v>174.3076923076923</v>
       </c>
     </row>
     <row r="144">
@@ -7574,11 +7574,11 @@
         </is>
       </c>
       <c r="G144" s="4" t="n">
-        <v>11385</v>
+        <v>12216</v>
       </c>
       <c r="H144" s="3" t="inlineStr">
         <is>
-          <t>23/24</t>
+          <t>24/26</t>
         </is>
       </c>
       <c r="I144" s="3" t="inlineStr">
@@ -7587,10 +7587,10 @@
         </is>
       </c>
       <c r="J144" s="4" t="n">
-        <v>11880</v>
+        <v>13234</v>
       </c>
       <c r="K144" s="5" t="n">
-        <v>495</v>
+        <v>509</v>
       </c>
     </row>
     <row r="145">
@@ -7672,11 +7672,11 @@
         </is>
       </c>
       <c r="G146" s="4" t="n">
-        <v>14383</v>
+        <v>15209</v>
       </c>
       <c r="H146" s="3" t="inlineStr">
         <is>
-          <t>24/29</t>
+          <t>25/29</t>
         </is>
       </c>
       <c r="I146" s="3" t="inlineStr">
@@ -7685,10 +7685,10 @@
         </is>
       </c>
       <c r="J146" s="4" t="n">
-        <v>17379</v>
+        <v>17642</v>
       </c>
       <c r="K146" s="5" t="n">
-        <v>599.2916666666666</v>
+        <v>608.36</v>
       </c>
     </row>
     <row r="147">
@@ -7770,11 +7770,11 @@
         </is>
       </c>
       <c r="G148" s="7" t="n">
-        <v>12816</v>
+        <v>14061</v>
       </c>
       <c r="H148" s="6" t="inlineStr">
         <is>
-          <t>14/21</t>
+          <t>15/21</t>
         </is>
       </c>
       <c r="I148" s="6" t="inlineStr">
@@ -7783,10 +7783,10 @@
         </is>
       </c>
       <c r="J148" s="7" t="n">
-        <v>19224</v>
+        <v>19685</v>
       </c>
       <c r="K148" s="8" t="n">
-        <v>915.4285714285714</v>
+        <v>937.4</v>
       </c>
     </row>
     <row r="149">
@@ -7819,11 +7819,11 @@
         </is>
       </c>
       <c r="G149" s="7" t="n">
-        <v>2647</v>
+        <v>3101</v>
       </c>
       <c r="H149" s="6" t="inlineStr">
         <is>
-          <t>10/25</t>
+          <t>11/25</t>
         </is>
       </c>
       <c r="I149" s="6" t="inlineStr">
@@ -7832,10 +7832,10 @@
         </is>
       </c>
       <c r="J149" s="7" t="n">
-        <v>6618</v>
+        <v>7048</v>
       </c>
       <c r="K149" s="8" t="n">
-        <v>264.7</v>
+        <v>281.9090909090909</v>
       </c>
     </row>
     <row r="150">
@@ -7917,11 +7917,11 @@
         </is>
       </c>
       <c r="G151" s="4" t="n">
-        <v>19587</v>
+        <v>20749</v>
       </c>
       <c r="H151" s="3" t="inlineStr">
         <is>
-          <t>13/21</t>
+          <t>14/21</t>
         </is>
       </c>
       <c r="I151" s="3" t="inlineStr">
@@ -7930,10 +7930,10 @@
         </is>
       </c>
       <c r="J151" s="4" t="n">
-        <v>31641</v>
+        <v>31124</v>
       </c>
       <c r="K151" s="5" t="n">
-        <v>1506.692307692308</v>
+        <v>1482.071428571429</v>
       </c>
     </row>
     <row r="152">
@@ -8015,11 +8015,11 @@
         </is>
       </c>
       <c r="G153" s="4" t="n">
-        <v>28406</v>
+        <v>29324</v>
       </c>
       <c r="H153" s="3" t="inlineStr">
         <is>
-          <t>15/20</t>
+          <t>16/20</t>
         </is>
       </c>
       <c r="I153" s="3" t="inlineStr">
@@ -8028,10 +8028,10 @@
         </is>
       </c>
       <c r="J153" s="4" t="n">
-        <v>37875</v>
+        <v>36655</v>
       </c>
       <c r="K153" s="5" t="n">
-        <v>1893.733333333333</v>
+        <v>1832.75</v>
       </c>
     </row>
     <row r="154">
@@ -8211,11 +8211,11 @@
         </is>
       </c>
       <c r="G157" s="7" t="n">
-        <v>4217</v>
+        <v>4578</v>
       </c>
       <c r="H157" s="6" t="inlineStr">
         <is>
-          <t>17/25</t>
+          <t>18/25</t>
         </is>
       </c>
       <c r="I157" s="6" t="inlineStr">
@@ -8224,10 +8224,10 @@
         </is>
       </c>
       <c r="J157" s="7" t="n">
-        <v>6201</v>
+        <v>6358</v>
       </c>
       <c r="K157" s="8" t="n">
-        <v>248.0588235294118</v>
+        <v>254.3333333333333</v>
       </c>
     </row>
     <row r="158">
@@ -8309,11 +8309,11 @@
         </is>
       </c>
       <c r="G159" s="11" t="n">
-        <v>1231</v>
+        <v>792</v>
       </c>
       <c r="H159" s="10" t="inlineStr">
         <is>
-          <t>17/22</t>
+          <t>18/22</t>
         </is>
       </c>
       <c r="I159" s="10" t="inlineStr">
@@ -8322,10 +8322,10 @@
         </is>
       </c>
       <c r="J159" s="11" t="n">
-        <v>1593</v>
+        <v>968</v>
       </c>
       <c r="K159" s="12" t="n">
-        <v>72.41176470588235</v>
+        <v>44</v>
       </c>
     </row>
     <row r="160">
@@ -8456,11 +8456,11 @@
         </is>
       </c>
       <c r="G162" s="4" t="n">
-        <v>31634</v>
+        <v>35149</v>
       </c>
       <c r="H162" s="3" t="inlineStr">
         <is>
-          <t>11/30</t>
+          <t>12/30</t>
         </is>
       </c>
       <c r="I162" s="3" t="inlineStr">
@@ -8469,10 +8469,10 @@
         </is>
       </c>
       <c r="J162" s="4" t="n">
-        <v>86275</v>
+        <v>87872</v>
       </c>
       <c r="K162" s="5" t="n">
-        <v>2875.818181818182</v>
+        <v>2929.083333333333</v>
       </c>
     </row>
     <row r="163">
@@ -8603,11 +8603,11 @@
         </is>
       </c>
       <c r="G165" s="7" t="n">
-        <v>7271</v>
+        <v>8116</v>
       </c>
       <c r="H165" s="6" t="inlineStr">
         <is>
-          <t>13/29</t>
+          <t>14/29</t>
         </is>
       </c>
       <c r="I165" s="6" t="inlineStr">
@@ -8616,10 +8616,10 @@
         </is>
       </c>
       <c r="J165" s="7" t="n">
-        <v>16220</v>
+        <v>16812</v>
       </c>
       <c r="K165" s="8" t="n">
-        <v>559.3076923076923</v>
+        <v>579.7142857142857</v>
       </c>
     </row>
     <row r="166">
@@ -8701,11 +8701,11 @@
         </is>
       </c>
       <c r="G167" s="4" t="n">
-        <v>23957</v>
+        <v>26478</v>
       </c>
       <c r="H167" s="3" t="inlineStr">
         <is>
-          <t>15/32</t>
+          <t>16/32</t>
         </is>
       </c>
       <c r="I167" s="3" t="inlineStr">
@@ -8714,10 +8714,10 @@
         </is>
       </c>
       <c r="J167" s="4" t="n">
-        <v>51108</v>
+        <v>52956</v>
       </c>
       <c r="K167" s="5" t="n">
-        <v>1597.133333333333</v>
+        <v>1654.875</v>
       </c>
     </row>
     <row r="168">
@@ -8750,11 +8750,11 @@
         </is>
       </c>
       <c r="G168" s="4" t="n">
-        <v>15758</v>
+        <v>16885</v>
       </c>
       <c r="H168" s="3" t="inlineStr">
         <is>
-          <t>12/27</t>
+          <t>13/27</t>
         </is>
       </c>
       <c r="I168" s="3" t="inlineStr">
@@ -8763,10 +8763,10 @@
         </is>
       </c>
       <c r="J168" s="4" t="n">
-        <v>35456</v>
+        <v>35069</v>
       </c>
       <c r="K168" s="5" t="n">
-        <v>1313.166666666667</v>
+        <v>1298.846153846154</v>
       </c>
     </row>
     <row r="169">
@@ -8946,11 +8946,11 @@
         </is>
       </c>
       <c r="G172" s="4" t="n">
-        <v>20177</v>
+        <v>21294</v>
       </c>
       <c r="H172" s="3" t="inlineStr">
         <is>
-          <t>22/34</t>
+          <t>23/34</t>
         </is>
       </c>
       <c r="I172" s="3" t="inlineStr">
@@ -8959,10 +8959,10 @@
         </is>
       </c>
       <c r="J172" s="4" t="n">
-        <v>31183</v>
+        <v>31478</v>
       </c>
       <c r="K172" s="5" t="n">
-        <v>917.1363636363636</v>
+        <v>925.8260869565217</v>
       </c>
     </row>
     <row r="173">
@@ -8995,11 +8995,11 @@
         </is>
       </c>
       <c r="G173" s="7" t="n">
-        <v>5825</v>
+        <v>5709</v>
       </c>
       <c r="H173" s="6" t="inlineStr">
         <is>
-          <t>14/26</t>
+          <t>15/26</t>
         </is>
       </c>
       <c r="I173" s="6" t="inlineStr">
@@ -9008,10 +9008,10 @@
         </is>
       </c>
       <c r="J173" s="7" t="n">
-        <v>10818</v>
+        <v>9896</v>
       </c>
       <c r="K173" s="8" t="n">
-        <v>416.0714285714286</v>
+        <v>380.6</v>
       </c>
     </row>
     <row r="174">
@@ -9142,11 +9142,11 @@
         </is>
       </c>
       <c r="G176" s="4" t="n">
-        <v>22164</v>
+        <v>22333</v>
       </c>
       <c r="H176" s="3" t="inlineStr">
         <is>
-          <t>16/17</t>
+          <t>17/17</t>
         </is>
       </c>
       <c r="I176" s="3" t="inlineStr">
@@ -9155,10 +9155,10 @@
         </is>
       </c>
       <c r="J176" s="4" t="n">
-        <v>23549</v>
+        <v>22333</v>
       </c>
       <c r="K176" s="5" t="n">
-        <v>1385.25</v>
+        <v>1313.705882352941</v>
       </c>
     </row>
     <row r="177">
@@ -9387,11 +9387,11 @@
         </is>
       </c>
       <c r="G181" s="4" t="n">
-        <v>8442</v>
+        <v>8551</v>
       </c>
       <c r="H181" s="3" t="inlineStr">
         <is>
-          <t>16/21</t>
+          <t>17/21</t>
         </is>
       </c>
       <c r="I181" s="3" t="inlineStr">
@@ -9400,10 +9400,10 @@
         </is>
       </c>
       <c r="J181" s="4" t="n">
-        <v>11080</v>
+        <v>10563</v>
       </c>
       <c r="K181" s="5" t="n">
-        <v>527.625</v>
+        <v>503</v>
       </c>
     </row>
     <row r="182">
@@ -9583,11 +9583,11 @@
         </is>
       </c>
       <c r="G185" s="7" t="n">
-        <v>2034</v>
+        <v>2886</v>
       </c>
       <c r="H185" s="6" t="inlineStr">
         <is>
-          <t>10/23</t>
+          <t>11/23</t>
         </is>
       </c>
       <c r="I185" s="6" t="inlineStr">
@@ -9596,10 +9596,10 @@
         </is>
       </c>
       <c r="J185" s="7" t="n">
-        <v>4678</v>
+        <v>6034</v>
       </c>
       <c r="K185" s="8" t="n">
-        <v>203.4</v>
+        <v>262.3636363636364</v>
       </c>
     </row>
     <row r="186">
@@ -9632,11 +9632,11 @@
         </is>
       </c>
       <c r="G186" s="7" t="n">
-        <v>7957</v>
+        <v>7849</v>
       </c>
       <c r="H186" s="6" t="inlineStr">
         <is>
-          <t>14/24</t>
+          <t>15/24</t>
         </is>
       </c>
       <c r="I186" s="6" t="inlineStr">
@@ -9645,10 +9645,10 @@
         </is>
       </c>
       <c r="J186" s="7" t="n">
-        <v>13641</v>
+        <v>12558</v>
       </c>
       <c r="K186" s="8" t="n">
-        <v>568.3571428571429</v>
+        <v>523.2666666666667</v>
       </c>
     </row>
     <row r="187">
@@ -9681,11 +9681,11 @@
         </is>
       </c>
       <c r="G187" s="4" t="n">
-        <v>37800</v>
+        <v>39525</v>
       </c>
       <c r="H187" s="3" t="inlineStr">
         <is>
-          <t>16/25</t>
+          <t>17/25</t>
         </is>
       </c>
       <c r="I187" s="3" t="inlineStr">
@@ -9694,10 +9694,10 @@
         </is>
       </c>
       <c r="J187" s="4" t="n">
-        <v>59062</v>
+        <v>58125</v>
       </c>
       <c r="K187" s="5" t="n">
-        <v>2362.5</v>
+        <v>2325</v>
       </c>
     </row>
     <row r="188">
@@ -9730,11 +9730,11 @@
         </is>
       </c>
       <c r="G188" s="4" t="n">
-        <v>11883</v>
+        <v>12949</v>
       </c>
       <c r="H188" s="3" t="inlineStr">
         <is>
-          <t>14/18</t>
+          <t>15/18</t>
         </is>
       </c>
       <c r="I188" s="3" t="inlineStr">
@@ -9743,10 +9743,10 @@
         </is>
       </c>
       <c r="J188" s="4" t="n">
-        <v>15278</v>
+        <v>15539</v>
       </c>
       <c r="K188" s="5" t="n">
-        <v>848.7857142857143</v>
+        <v>863.2666666666667</v>
       </c>
     </row>
     <row r="189">
@@ -9779,11 +9779,11 @@
         </is>
       </c>
       <c r="G189" s="7" t="n">
-        <v>9220</v>
+        <v>9848</v>
       </c>
       <c r="H189" s="6" t="inlineStr">
         <is>
-          <t>13/27</t>
+          <t>14/27</t>
         </is>
       </c>
       <c r="I189" s="6" t="inlineStr">
@@ -9792,10 +9792,10 @@
         </is>
       </c>
       <c r="J189" s="7" t="n">
-        <v>19149</v>
+        <v>18993</v>
       </c>
       <c r="K189" s="8" t="n">
-        <v>709.2307692307693</v>
+        <v>703.4285714285714</v>
       </c>
     </row>
     <row r="190">
@@ -9828,11 +9828,11 @@
         </is>
       </c>
       <c r="G190" s="4" t="n">
-        <v>26772</v>
+        <v>28169</v>
       </c>
       <c r="H190" s="3" t="inlineStr">
         <is>
-          <t>17/26</t>
+          <t>18/26</t>
         </is>
       </c>
       <c r="I190" s="3" t="inlineStr">
@@ -9841,10 +9841,10 @@
         </is>
       </c>
       <c r="J190" s="4" t="n">
-        <v>40945</v>
+        <v>40689</v>
       </c>
       <c r="K190" s="5" t="n">
-        <v>1574.823529411765</v>
+        <v>1564.944444444444</v>
       </c>
     </row>
     <row r="191">
@@ -9926,11 +9926,11 @@
         </is>
       </c>
       <c r="G192" s="7" t="n">
-        <v>6229</v>
+        <v>7310</v>
       </c>
       <c r="H192" s="6" t="inlineStr">
         <is>
-          <t>15/22</t>
+          <t>16/22</t>
         </is>
       </c>
       <c r="I192" s="6" t="inlineStr">
@@ -9939,10 +9939,10 @@
         </is>
       </c>
       <c r="J192" s="7" t="n">
-        <v>9136</v>
+        <v>10051</v>
       </c>
       <c r="K192" s="8" t="n">
-        <v>415.2666666666667</v>
+        <v>456.875</v>
       </c>
     </row>
     <row r="193">
@@ -10073,11 +10073,11 @@
         </is>
       </c>
       <c r="G195" s="7" t="n">
-        <v>6465</v>
+        <v>9128</v>
       </c>
       <c r="H195" s="6" t="inlineStr">
         <is>
-          <t>10/21</t>
+          <t>11/21</t>
         </is>
       </c>
       <c r="I195" s="6" t="inlineStr">
@@ -10086,10 +10086,10 @@
         </is>
       </c>
       <c r="J195" s="7" t="n">
-        <v>13576</v>
+        <v>17426</v>
       </c>
       <c r="K195" s="8" t="n">
-        <v>646.5</v>
+        <v>829.8181818181819</v>
       </c>
     </row>
     <row r="196">
@@ -10142,52 +10142,52 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" s="2" t="inlineStr">
+      <c r="A197" s="6" t="inlineStr">
         <is>
           <t>TIRUCHIRAPPALLI (WEST)</t>
         </is>
       </c>
-      <c r="B197" s="3" t="n">
+      <c r="B197" s="6" t="n">
         <v>140</v>
       </c>
-      <c r="C197" s="3" t="inlineStr">
+      <c r="C197" s="6" t="inlineStr">
         <is>
           <t>K.N.NEHRU</t>
         </is>
       </c>
-      <c r="D197" s="3" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E197" s="3" t="inlineStr">
+      <c r="D197" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E197" s="6" t="inlineStr">
         <is>
           <t>G.RAMAMOORTHI</t>
         </is>
       </c>
-      <c r="F197" s="3" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G197" s="4" t="n">
-        <v>5375</v>
-      </c>
-      <c r="H197" s="3" t="inlineStr">
-        <is>
-          <t>21/24</t>
-        </is>
-      </c>
-      <c r="I197" s="3" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J197" s="4" t="n">
-        <v>6143</v>
-      </c>
-      <c r="K197" s="5" t="n">
-        <v>255.952380952381</v>
+      <c r="F197" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G197" s="7" t="n">
+        <v>4883</v>
+      </c>
+      <c r="H197" s="6" t="inlineStr">
+        <is>
+          <t>22/24</t>
+        </is>
+      </c>
+      <c r="I197" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J197" s="7" t="n">
+        <v>5327</v>
+      </c>
+      <c r="K197" s="8" t="n">
+        <v>221.9545454545455</v>
       </c>
     </row>
     <row r="198">
@@ -10220,11 +10220,11 @@
         </is>
       </c>
       <c r="G198" s="7" t="n">
-        <v>3317</v>
+        <v>4243</v>
       </c>
       <c r="H198" s="6" t="inlineStr">
         <is>
-          <t>9/21</t>
+          <t>10/21</t>
         </is>
       </c>
       <c r="I198" s="6" t="inlineStr">
@@ -10233,10 +10233,10 @@
         </is>
       </c>
       <c r="J198" s="7" t="n">
-        <v>7740</v>
+        <v>8910</v>
       </c>
       <c r="K198" s="8" t="n">
-        <v>368.5555555555555</v>
+        <v>424.3</v>
       </c>
     </row>
     <row r="199">
@@ -10318,11 +10318,11 @@
         </is>
       </c>
       <c r="G200" s="4" t="n">
-        <v>8461</v>
+        <v>9196</v>
       </c>
       <c r="H200" s="3" t="inlineStr">
         <is>
-          <t>24/28</t>
+          <t>25/28</t>
         </is>
       </c>
       <c r="I200" s="3" t="inlineStr">
@@ -10331,10 +10331,10 @@
         </is>
       </c>
       <c r="J200" s="4" t="n">
-        <v>9871</v>
+        <v>10300</v>
       </c>
       <c r="K200" s="5" t="n">
-        <v>352.5416666666667</v>
+        <v>367.84</v>
       </c>
     </row>
     <row r="201">
@@ -10465,11 +10465,11 @@
         </is>
       </c>
       <c r="G203" s="4" t="n">
-        <v>37991</v>
+        <v>39813</v>
       </c>
       <c r="H203" s="3" t="inlineStr">
         <is>
-          <t>15/32</t>
+          <t>16/32</t>
         </is>
       </c>
       <c r="I203" s="3" t="inlineStr">
@@ -10478,10 +10478,10 @@
         </is>
       </c>
       <c r="J203" s="4" t="n">
-        <v>81047</v>
+        <v>79626</v>
       </c>
       <c r="K203" s="5" t="n">
-        <v>2532.733333333333</v>
+        <v>2488.3125</v>
       </c>
     </row>
     <row r="204">
@@ -10583,52 +10583,52 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="13" t="inlineStr">
+      <c r="A206" s="9" t="inlineStr">
         <is>
           <t>TIRUVADANAI</t>
         </is>
       </c>
-      <c r="B206" s="14" t="n">
+      <c r="B206" s="10" t="n">
         <v>210</v>
       </c>
-      <c r="C206" s="14" t="inlineStr">
+      <c r="C206" s="10" t="inlineStr">
         <is>
           <t>RAJEEV</t>
         </is>
       </c>
-      <c r="D206" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E206" s="14" t="inlineStr">
+      <c r="D206" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E206" s="10" t="inlineStr">
         <is>
           <t>RM. KARUMANICKAM</t>
         </is>
       </c>
-      <c r="F206" s="14" t="inlineStr">
+      <c r="F206" s="10" t="inlineStr">
         <is>
           <t>Indian National Congress</t>
         </is>
       </c>
-      <c r="G206" s="15" t="n">
-        <v>345</v>
-      </c>
-      <c r="H206" s="14" t="inlineStr">
-        <is>
-          <t>20/27</t>
-        </is>
-      </c>
-      <c r="I206" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J206" s="15" t="n">
-        <v>466</v>
-      </c>
-      <c r="K206" s="16" t="n">
-        <v>17.25</v>
+      <c r="G206" s="11" t="n">
+        <v>1875</v>
+      </c>
+      <c r="H206" s="10" t="inlineStr">
+        <is>
+          <t>21/27</t>
+        </is>
+      </c>
+      <c r="I206" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J206" s="11" t="n">
+        <v>2411</v>
+      </c>
+      <c r="K206" s="12" t="n">
+        <v>89.28571428571429</v>
       </c>
     </row>
     <row r="207">
@@ -10710,11 +10710,11 @@
         </is>
       </c>
       <c r="G208" s="11" t="n">
-        <v>1004</v>
+        <v>530</v>
       </c>
       <c r="H208" s="10" t="inlineStr">
         <is>
-          <t>11/20</t>
+          <t>12/20</t>
         </is>
       </c>
       <c r="I208" s="10" t="inlineStr">
@@ -10723,10 +10723,10 @@
         </is>
       </c>
       <c r="J208" s="11" t="n">
-        <v>1825</v>
+        <v>883</v>
       </c>
       <c r="K208" s="12" t="n">
-        <v>91.27272727272727</v>
+        <v>44.16666666666666</v>
       </c>
     </row>
     <row r="209">
@@ -10808,11 +10808,11 @@
         </is>
       </c>
       <c r="G210" s="7" t="n">
-        <v>4020</v>
+        <v>2832</v>
       </c>
       <c r="H210" s="6" t="inlineStr">
         <is>
-          <t>17/22</t>
+          <t>18/22</t>
         </is>
       </c>
       <c r="I210" s="6" t="inlineStr">
@@ -10821,10 +10821,10 @@
         </is>
       </c>
       <c r="J210" s="7" t="n">
-        <v>5202</v>
+        <v>3461</v>
       </c>
       <c r="K210" s="8" t="n">
-        <v>236.4705882352941</v>
+        <v>157.3333333333333</v>
       </c>
     </row>
     <row r="211">
@@ -10906,11 +10906,11 @@
         </is>
       </c>
       <c r="G212" s="7" t="n">
-        <v>2132</v>
+        <v>1858</v>
       </c>
       <c r="H212" s="6" t="inlineStr">
         <is>
-          <t>11/25</t>
+          <t>12/25</t>
         </is>
       </c>
       <c r="I212" s="6" t="inlineStr">
@@ -10919,10 +10919,10 @@
         </is>
       </c>
       <c r="J212" s="7" t="n">
-        <v>4845</v>
+        <v>3871</v>
       </c>
       <c r="K212" s="8" t="n">
-        <v>193.8181818181818</v>
+        <v>154.8333333333333</v>
       </c>
     </row>
     <row r="213">
@@ -11122,52 +11122,52 @@
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="2" t="inlineStr">
+      <c r="A217" s="6" t="inlineStr">
         <is>
           <t>VANIYAMBADI</t>
         </is>
       </c>
-      <c r="B217" s="3" t="n">
+      <c r="B217" s="6" t="n">
         <v>47</v>
       </c>
-      <c r="C217" s="3" t="inlineStr">
+      <c r="C217" s="6" t="inlineStr">
         <is>
           <t>SYED FAROOQ BASHA SSB</t>
         </is>
       </c>
-      <c r="D217" s="3" t="inlineStr">
+      <c r="D217" s="6" t="inlineStr">
         <is>
           <t>Indian Union Muslim League</t>
         </is>
       </c>
-      <c r="E217" s="3" t="inlineStr">
+      <c r="E217" s="6" t="inlineStr">
         <is>
           <t>SYED BHURHANUDEEN</t>
         </is>
       </c>
-      <c r="F217" s="3" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G217" s="4" t="n">
-        <v>5073</v>
-      </c>
-      <c r="H217" s="3" t="inlineStr">
-        <is>
-          <t>21/23</t>
-        </is>
-      </c>
-      <c r="I217" s="3" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J217" s="4" t="n">
-        <v>5556</v>
-      </c>
-      <c r="K217" s="5" t="n">
-        <v>241.5714285714286</v>
+      <c r="F217" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G217" s="7" t="n">
+        <v>3069</v>
+      </c>
+      <c r="H217" s="6" t="inlineStr">
+        <is>
+          <t>22/23</t>
+        </is>
+      </c>
+      <c r="I217" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J217" s="7" t="n">
+        <v>3208</v>
+      </c>
+      <c r="K217" s="8" t="n">
+        <v>139.5</v>
       </c>
     </row>
     <row r="218">
@@ -11347,11 +11347,11 @@
         </is>
       </c>
       <c r="G221" s="7" t="n">
-        <v>8170</v>
+        <v>6926</v>
       </c>
       <c r="H221" s="6" t="inlineStr">
         <is>
-          <t>15/24</t>
+          <t>16/24</t>
         </is>
       </c>
       <c r="I221" s="6" t="inlineStr">
@@ -11360,10 +11360,10 @@
         </is>
       </c>
       <c r="J221" s="7" t="n">
-        <v>13072</v>
+        <v>10389</v>
       </c>
       <c r="K221" s="8" t="n">
-        <v>544.6666666666666</v>
+        <v>432.875</v>
       </c>
     </row>
     <row r="222">
@@ -11396,11 +11396,11 @@
         </is>
       </c>
       <c r="G222" s="7" t="n">
-        <v>4301</v>
+        <v>3899</v>
       </c>
       <c r="H222" s="6" t="inlineStr">
         <is>
-          <t>14/23</t>
+          <t>15/23</t>
         </is>
       </c>
       <c r="I222" s="6" t="inlineStr">
@@ -11409,10 +11409,10 @@
         </is>
       </c>
       <c r="J222" s="7" t="n">
-        <v>7066</v>
+        <v>5978</v>
       </c>
       <c r="K222" s="8" t="n">
-        <v>307.2142857142857</v>
+        <v>259.9333333333333</v>
       </c>
     </row>
     <row r="223">
@@ -11573,30 +11573,30 @@
       </c>
       <c r="C226" s="14" t="inlineStr">
         <is>
+          <t>VIJAI VADIVEL A</t>
+        </is>
+      </c>
+      <c r="D226" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E226" s="14" t="inlineStr">
+        <is>
           <t>SIVAKUMAR C</t>
         </is>
       </c>
-      <c r="D226" s="14" t="inlineStr">
+      <c r="F226" s="14" t="inlineStr">
         <is>
           <t>Pattali Makkal Katchi</t>
         </is>
       </c>
-      <c r="E226" s="14" t="inlineStr">
-        <is>
-          <t>VIJAI VADIVEL A</t>
-        </is>
-      </c>
-      <c r="F226" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
       <c r="G226" s="15" t="n">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="H226" s="14" t="inlineStr">
         <is>
-          <t>8/23</t>
+          <t>9/23</t>
         </is>
       </c>
       <c r="I226" s="14" t="inlineStr">
@@ -11605,10 +11605,10 @@
         </is>
       </c>
       <c r="J226" s="15" t="n">
-        <v>477</v>
+        <v>432</v>
       </c>
       <c r="K226" s="16" t="n">
-        <v>20.75</v>
+        <v>18.77777777777778</v>
       </c>
     </row>
     <row r="227">
@@ -11710,52 +11710,52 @@
       </c>
     </row>
     <row r="229">
-      <c r="A229" s="6" t="inlineStr">
+      <c r="A229" s="2" t="inlineStr">
         <is>
           <t>VILLIVAKKAM</t>
         </is>
       </c>
-      <c r="B229" s="6" t="n">
+      <c r="B229" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="C229" s="6" t="inlineStr">
+      <c r="C229" s="3" t="inlineStr">
         <is>
           <t>AADHAV ARJUNA</t>
         </is>
       </c>
-      <c r="D229" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E229" s="6" t="inlineStr">
+      <c r="D229" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E229" s="3" t="inlineStr">
         <is>
           <t>KARTHIK MOHAN</t>
         </is>
       </c>
-      <c r="F229" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G229" s="7" t="n">
-        <v>13311</v>
-      </c>
-      <c r="H229" s="6" t="inlineStr">
-        <is>
-          <t>14/19</t>
-        </is>
-      </c>
-      <c r="I229" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J229" s="7" t="n">
-        <v>18065</v>
-      </c>
-      <c r="K229" s="8" t="n">
-        <v>950.7857142857143</v>
+      <c r="F229" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G229" s="4" t="n">
+        <v>14495</v>
+      </c>
+      <c r="H229" s="3" t="inlineStr">
+        <is>
+          <t>15/19</t>
+        </is>
+      </c>
+      <c r="I229" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J229" s="4" t="n">
+        <v>18360</v>
+      </c>
+      <c r="K229" s="5" t="n">
+        <v>966.3333333333334</v>
       </c>
     </row>
     <row r="230">

</xml_diff>

<commit_message>
Update election results snapshot (69.2% counted)
TVK 107, DMK 58, AIADMK 47. ANNA NAGAR declared (TVK). NILAKKOTTAI new
tightest at 16-vote TVK lead. THALLI settled to CPI. 9 knife-edge seats.

https://claude.ai/code/session_01MizbUy44JG5sXyvaf3Wekb
</commit_message>
<xml_diff>
--- a/tn_election_results_may2026.xlsx
+++ b/tn_election_results_may2026.xlsx
@@ -714,11 +714,11 @@
         </is>
       </c>
       <c r="G4" s="7" t="n">
-        <v>3679</v>
+        <v>4300</v>
       </c>
       <c r="H4" s="6" t="inlineStr">
         <is>
-          <t>18/24</t>
+          <t>19/24</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
@@ -727,10 +727,10 @@
         </is>
       </c>
       <c r="J4" s="7" t="n">
-        <v>4905</v>
+        <v>5432</v>
       </c>
       <c r="K4" s="8" t="n">
-        <v>204.3888888888889</v>
+        <v>226.3157894736842</v>
       </c>
     </row>
     <row r="5">
@@ -763,11 +763,11 @@
         </is>
       </c>
       <c r="G5" s="4" t="n">
-        <v>10632</v>
+        <v>10245</v>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>21/23</t>
+          <t>23/23</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -776,10 +776,10 @@
         </is>
       </c>
       <c r="J5" s="4" t="n">
-        <v>11645</v>
+        <v>10245</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>506.2857142857143</v>
+        <v>445.4347826086956</v>
       </c>
     </row>
     <row r="6">
@@ -812,11 +812,11 @@
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>38522</v>
+        <v>40258</v>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>16/27</t>
+          <t>17/27</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -825,59 +825,59 @@
         </is>
       </c>
       <c r="J6" s="4" t="n">
-        <v>65006</v>
+        <v>63939</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>2407.625</v>
+        <v>2368.117647058823</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>AMBUR</t>
         </is>
       </c>
-      <c r="B7" s="6" t="n">
+      <c r="B7" s="10" t="n">
         <v>48</v>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>IMTHIYAZ PANDARATTUDU ABDU</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
         <is>
           <t>VILWANATHAN. A.C.</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G7" s="7" t="n">
-        <v>2928</v>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>11/22</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J7" s="7" t="n">
-        <v>5856</v>
-      </c>
-      <c r="K7" s="8" t="n">
-        <v>266.1818181818182</v>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="n">
+        <v>275</v>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>12/22</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J7" s="11" t="n">
+        <v>504</v>
+      </c>
+      <c r="K7" s="12" t="n">
+        <v>22.91666666666667</v>
       </c>
     </row>
     <row r="8">
@@ -910,11 +910,11 @@
         </is>
       </c>
       <c r="G8" s="7" t="n">
-        <v>5762</v>
+        <v>6049</v>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>12/22</t>
+          <t>13/22</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
@@ -923,10 +923,10 @@
         </is>
       </c>
       <c r="J8" s="7" t="n">
-        <v>10564</v>
+        <v>10237</v>
       </c>
       <c r="K8" s="8" t="n">
-        <v>480.1666666666667</v>
+        <v>465.3076923076923</v>
       </c>
     </row>
     <row r="9">
@@ -1017,7 +1017,7 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J10" s="4" t="n">
@@ -1057,11 +1057,11 @@
         </is>
       </c>
       <c r="G11" s="11" t="n">
-        <v>1027</v>
+        <v>1363</v>
       </c>
       <c r="H11" s="10" t="inlineStr">
         <is>
-          <t>18/20</t>
+          <t>20/20</t>
         </is>
       </c>
       <c r="I11" s="10" t="inlineStr">
@@ -1070,10 +1070,10 @@
         </is>
       </c>
       <c r="J11" s="11" t="n">
-        <v>1141</v>
+        <v>1363</v>
       </c>
       <c r="K11" s="12" t="n">
-        <v>57.05555555555556</v>
+        <v>68.15000000000001</v>
       </c>
     </row>
     <row r="12">
@@ -1175,52 +1175,52 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>ARANTHANGI</t>
         </is>
       </c>
-      <c r="B14" s="6" t="n">
+      <c r="B14" s="3" t="n">
         <v>183</v>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>MOHAMED FARVAS. J</t>
         </is>
       </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>RAMACHANDRAN . T</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>Indian National Congress</t>
         </is>
       </c>
-      <c r="G14" s="7" t="n">
-        <v>11595</v>
-      </c>
-      <c r="H14" s="6" t="inlineStr">
-        <is>
-          <t>16/22</t>
-        </is>
-      </c>
-      <c r="I14" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J14" s="7" t="n">
-        <v>15943</v>
-      </c>
-      <c r="K14" s="8" t="n">
-        <v>724.6875</v>
+      <c r="G14" s="4" t="n">
+        <v>12301</v>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>17/22</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>15919</v>
+      </c>
+      <c r="K14" s="5" t="n">
+        <v>723.5882352941177</v>
       </c>
     </row>
     <row r="15">
@@ -1302,11 +1302,11 @@
         </is>
       </c>
       <c r="G16" s="4" t="n">
-        <v>15837</v>
+        <v>16312</v>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>11/23</t>
+          <t>12/23</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
@@ -1315,10 +1315,10 @@
         </is>
       </c>
       <c r="J16" s="4" t="n">
-        <v>33114</v>
+        <v>31265</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>1439.727272727273</v>
+        <v>1359.333333333333</v>
       </c>
     </row>
     <row r="17">
@@ -1498,11 +1498,11 @@
         </is>
       </c>
       <c r="G20" s="4" t="n">
-        <v>11757</v>
+        <v>12052</v>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>18/22</t>
+          <t>19/22</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
@@ -1511,10 +1511,10 @@
         </is>
       </c>
       <c r="J20" s="4" t="n">
-        <v>14370</v>
+        <v>13955</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>653.1666666666666</v>
+        <v>634.3157894736842</v>
       </c>
     </row>
     <row r="21">
@@ -1547,11 +1547,11 @@
         </is>
       </c>
       <c r="G21" s="4" t="n">
-        <v>39060</v>
+        <v>41308</v>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>14/26</t>
+          <t>15/26</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -1560,10 +1560,10 @@
         </is>
       </c>
       <c r="J21" s="4" t="n">
-        <v>72540</v>
+        <v>71601</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>2790</v>
+        <v>2753.866666666667</v>
       </c>
     </row>
     <row r="22">
@@ -1596,11 +1596,11 @@
         </is>
       </c>
       <c r="G22" s="7" t="n">
-        <v>8442</v>
+        <v>8929</v>
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>19/27</t>
+          <t>20/27</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr">
@@ -1609,10 +1609,10 @@
         </is>
       </c>
       <c r="J22" s="7" t="n">
-        <v>11997</v>
+        <v>12054</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>444.3157894736842</v>
+        <v>446.45</v>
       </c>
     </row>
     <row r="23">
@@ -1694,11 +1694,11 @@
         </is>
       </c>
       <c r="G24" s="7" t="n">
-        <v>8437</v>
+        <v>9095</v>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>11/22</t>
+          <t>12/22</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr">
@@ -1707,10 +1707,10 @@
         </is>
       </c>
       <c r="J24" s="7" t="n">
-        <v>16874</v>
+        <v>16674</v>
       </c>
       <c r="K24" s="8" t="n">
-        <v>767</v>
+        <v>757.9166666666666</v>
       </c>
     </row>
     <row r="25">
@@ -1743,11 +1743,11 @@
         </is>
       </c>
       <c r="G25" s="15" t="n">
-        <v>276</v>
+        <v>205</v>
       </c>
       <c r="H25" s="14" t="inlineStr">
         <is>
-          <t>17/24</t>
+          <t>18/24</t>
         </is>
       </c>
       <c r="I25" s="14" t="inlineStr">
@@ -1756,10 +1756,10 @@
         </is>
       </c>
       <c r="J25" s="15" t="n">
-        <v>390</v>
+        <v>273</v>
       </c>
       <c r="K25" s="16" t="n">
-        <v>16.23529411764706</v>
+        <v>11.38888888888889</v>
       </c>
     </row>
     <row r="26">
@@ -1792,11 +1792,11 @@
         </is>
       </c>
       <c r="G26" s="7" t="n">
-        <v>6062</v>
+        <v>6142</v>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>13/22</t>
+          <t>14/22</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
@@ -1805,10 +1805,10 @@
         </is>
       </c>
       <c r="J26" s="7" t="n">
-        <v>10259</v>
+        <v>9652</v>
       </c>
       <c r="K26" s="8" t="n">
-        <v>466.3076923076923</v>
+        <v>438.7142857142857</v>
       </c>
     </row>
     <row r="27">
@@ -1841,11 +1841,11 @@
         </is>
       </c>
       <c r="G27" s="7" t="n">
-        <v>2697</v>
+        <v>4213</v>
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>14/25</t>
+          <t>15/25</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
@@ -1854,10 +1854,10 @@
         </is>
       </c>
       <c r="J27" s="7" t="n">
-        <v>4816</v>
+        <v>7022</v>
       </c>
       <c r="K27" s="8" t="n">
-        <v>192.6428571428571</v>
+        <v>280.8666666666667</v>
       </c>
     </row>
     <row r="28">
@@ -1890,11 +1890,11 @@
         </is>
       </c>
       <c r="G28" s="4" t="n">
-        <v>15264</v>
+        <v>15383</v>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>12/36</t>
+          <t>13/36</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
@@ -1903,10 +1903,10 @@
         </is>
       </c>
       <c r="J28" s="4" t="n">
-        <v>45792</v>
+        <v>42599</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>1272</v>
+        <v>1183.307692307692</v>
       </c>
     </row>
     <row r="29">
@@ -1939,11 +1939,11 @@
         </is>
       </c>
       <c r="G29" s="7" t="n">
-        <v>6016</v>
+        <v>6585</v>
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>11/25</t>
+          <t>12/25</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
@@ -1952,10 +1952,10 @@
         </is>
       </c>
       <c r="J29" s="7" t="n">
-        <v>13673</v>
+        <v>13719</v>
       </c>
       <c r="K29" s="8" t="n">
-        <v>546.9090909090909</v>
+        <v>548.75</v>
       </c>
     </row>
     <row r="30">
@@ -1988,11 +1988,11 @@
         </is>
       </c>
       <c r="G30" s="7" t="n">
-        <v>4319</v>
+        <v>6118</v>
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>11/17</t>
+          <t>12/17</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
@@ -2001,10 +2001,10 @@
         </is>
       </c>
       <c r="J30" s="7" t="n">
-        <v>6675</v>
+        <v>8667</v>
       </c>
       <c r="K30" s="8" t="n">
-        <v>392.6363636363636</v>
+        <v>509.8333333333333</v>
       </c>
     </row>
     <row r="31">
@@ -2037,11 +2037,11 @@
         </is>
       </c>
       <c r="G31" s="4" t="n">
-        <v>19848</v>
+        <v>21081</v>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>23/24</t>
+          <t>24/24</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -2050,10 +2050,10 @@
         </is>
       </c>
       <c r="J31" s="4" t="n">
-        <v>20711</v>
+        <v>21081</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>862.9565217391304</v>
+        <v>878.375</v>
       </c>
     </row>
     <row r="32">
@@ -2184,11 +2184,11 @@
         </is>
       </c>
       <c r="G34" s="4" t="n">
-        <v>9163</v>
+        <v>9884</v>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>10/25</t>
+          <t>11/25</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
@@ -2197,10 +2197,10 @@
         </is>
       </c>
       <c r="J34" s="4" t="n">
-        <v>22908</v>
+        <v>22464</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>916.3</v>
+        <v>898.5454545454545</v>
       </c>
     </row>
     <row r="35">
@@ -2282,11 +2282,11 @@
         </is>
       </c>
       <c r="G36" s="7" t="n">
-        <v>6631</v>
+        <v>6403</v>
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>11/23</t>
+          <t>12/23</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
@@ -2295,10 +2295,10 @@
         </is>
       </c>
       <c r="J36" s="7" t="n">
-        <v>13865</v>
+        <v>12272</v>
       </c>
       <c r="K36" s="8" t="n">
-        <v>602.8181818181819</v>
+        <v>533.5833333333334</v>
       </c>
     </row>
     <row r="37">
@@ -2380,11 +2380,11 @@
         </is>
       </c>
       <c r="G38" s="7" t="n">
-        <v>8464</v>
+        <v>10137</v>
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>13/19</t>
+          <t>14/19</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr">
@@ -2393,10 +2393,10 @@
         </is>
       </c>
       <c r="J38" s="7" t="n">
-        <v>12370</v>
+        <v>13757</v>
       </c>
       <c r="K38" s="8" t="n">
-        <v>651.0769230769231</v>
+        <v>724.0714285714286</v>
       </c>
     </row>
     <row r="39">
@@ -2429,11 +2429,11 @@
         </is>
       </c>
       <c r="G39" s="7" t="n">
-        <v>2832</v>
+        <v>2637</v>
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>11/25</t>
+          <t>12/25</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr">
@@ -2442,10 +2442,10 @@
         </is>
       </c>
       <c r="J39" s="7" t="n">
-        <v>6436</v>
+        <v>5494</v>
       </c>
       <c r="K39" s="8" t="n">
-        <v>257.4545454545454</v>
+        <v>219.75</v>
       </c>
     </row>
     <row r="40">
@@ -2527,7 +2527,7 @@
         </is>
       </c>
       <c r="G41" s="4" t="n">
-        <v>15176</v>
+        <v>16090</v>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
@@ -2540,10 +2540,10 @@
         </is>
       </c>
       <c r="J41" s="4" t="n">
-        <v>17452</v>
+        <v>18504</v>
       </c>
       <c r="K41" s="5" t="n">
-        <v>758.8</v>
+        <v>804.5</v>
       </c>
     </row>
     <row r="42">
@@ -2576,11 +2576,11 @@
         </is>
       </c>
       <c r="G42" s="11" t="n">
-        <v>1739</v>
+        <v>1471</v>
       </c>
       <c r="H42" s="10" t="inlineStr">
         <is>
-          <t>19/24</t>
+          <t>20/24</t>
         </is>
       </c>
       <c r="I42" s="10" t="inlineStr">
@@ -2589,10 +2589,10 @@
         </is>
       </c>
       <c r="J42" s="11" t="n">
-        <v>2197</v>
+        <v>1765</v>
       </c>
       <c r="K42" s="12" t="n">
-        <v>91.52631578947368</v>
+        <v>73.55</v>
       </c>
     </row>
     <row r="43">
@@ -2625,11 +2625,11 @@
         </is>
       </c>
       <c r="G43" s="4" t="n">
-        <v>18861</v>
+        <v>21650</v>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>8/18</t>
+          <t>9/18</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
@@ -2638,10 +2638,10 @@
         </is>
       </c>
       <c r="J43" s="4" t="n">
-        <v>42437</v>
+        <v>43300</v>
       </c>
       <c r="K43" s="5" t="n">
-        <v>2357.625</v>
+        <v>2405.555555555556</v>
       </c>
     </row>
     <row r="44">
@@ -2674,11 +2674,11 @@
         </is>
       </c>
       <c r="G44" s="4" t="n">
-        <v>82438</v>
+        <v>86286</v>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>21/25</t>
+          <t>22/25</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
@@ -2687,10 +2687,10 @@
         </is>
       </c>
       <c r="J44" s="4" t="n">
-        <v>98140</v>
+        <v>98052</v>
       </c>
       <c r="K44" s="5" t="n">
-        <v>3925.619047619048</v>
+        <v>3922.090909090909</v>
       </c>
     </row>
     <row r="45">
@@ -2821,11 +2821,11 @@
         </is>
       </c>
       <c r="G47" s="4" t="n">
-        <v>17047</v>
+        <v>19123</v>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>14/24</t>
+          <t>15/24</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
@@ -2834,10 +2834,10 @@
         </is>
       </c>
       <c r="J47" s="4" t="n">
-        <v>29223</v>
+        <v>30597</v>
       </c>
       <c r="K47" s="5" t="n">
-        <v>1217.642857142857</v>
+        <v>1274.866666666667</v>
       </c>
     </row>
     <row r="48">
@@ -2870,11 +2870,11 @@
         </is>
       </c>
       <c r="G48" s="7" t="n">
-        <v>5580</v>
+        <v>6344</v>
       </c>
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>9/18</t>
+          <t>10/18</t>
         </is>
       </c>
       <c r="I48" s="6" t="inlineStr">
@@ -2883,59 +2883,59 @@
         </is>
       </c>
       <c r="J48" s="7" t="n">
-        <v>11160</v>
+        <v>11419</v>
       </c>
       <c r="K48" s="8" t="n">
-        <v>620</v>
+        <v>634.4</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="6" t="inlineStr">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>GANGAVALLI</t>
         </is>
       </c>
-      <c r="B49" s="6" t="n">
+      <c r="B49" s="3" t="n">
         <v>81</v>
       </c>
-      <c r="C49" s="6" t="inlineStr">
+      <c r="C49" s="3" t="inlineStr">
         <is>
           <t>NALLATHAMBI. A</t>
         </is>
       </c>
-      <c r="D49" s="6" t="inlineStr">
+      <c r="D49" s="3" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E49" s="6" t="inlineStr">
+      <c r="E49" s="3" t="inlineStr">
         <is>
           <t>CHINNADURAI. K</t>
         </is>
       </c>
-      <c r="F49" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G49" s="7" t="n">
-        <v>13962</v>
-      </c>
-      <c r="H49" s="6" t="inlineStr">
-        <is>
-          <t>14/20</t>
-        </is>
-      </c>
-      <c r="I49" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J49" s="7" t="n">
-        <v>19946</v>
-      </c>
-      <c r="K49" s="8" t="n">
-        <v>997.2857142857143</v>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="n">
+        <v>14359</v>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>15/20</t>
+        </is>
+      </c>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J49" s="4" t="n">
+        <v>19145</v>
+      </c>
+      <c r="K49" s="5" t="n">
+        <v>957.2666666666667</v>
       </c>
     </row>
     <row r="50">
@@ -3017,11 +3017,11 @@
         </is>
       </c>
       <c r="G51" s="4" t="n">
-        <v>16234</v>
+        <v>16494</v>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>20/23</t>
+          <t>21/23</t>
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr">
@@ -3030,10 +3030,10 @@
         </is>
       </c>
       <c r="J51" s="4" t="n">
-        <v>18669</v>
+        <v>18065</v>
       </c>
       <c r="K51" s="5" t="n">
-        <v>811.7</v>
+        <v>785.4285714285714</v>
       </c>
     </row>
     <row r="52">
@@ -3115,11 +3115,11 @@
         </is>
       </c>
       <c r="G53" s="11" t="n">
-        <v>1637</v>
+        <v>1682</v>
       </c>
       <c r="H53" s="10" t="inlineStr">
         <is>
-          <t>15/23</t>
+          <t>16/23</t>
         </is>
       </c>
       <c r="I53" s="10" t="inlineStr">
@@ -3128,10 +3128,10 @@
         </is>
       </c>
       <c r="J53" s="11" t="n">
-        <v>2510</v>
+        <v>2418</v>
       </c>
       <c r="K53" s="12" t="n">
-        <v>109.1333333333333</v>
+        <v>105.125</v>
       </c>
     </row>
     <row r="54">
@@ -3164,11 +3164,11 @@
         </is>
       </c>
       <c r="G54" s="4" t="n">
-        <v>17793</v>
+        <v>19483</v>
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>15/25</t>
+          <t>16/25</t>
         </is>
       </c>
       <c r="I54" s="3" t="inlineStr">
@@ -3177,10 +3177,10 @@
         </is>
       </c>
       <c r="J54" s="4" t="n">
-        <v>29655</v>
+        <v>30442</v>
       </c>
       <c r="K54" s="5" t="n">
-        <v>1186.2</v>
+        <v>1217.6875</v>
       </c>
     </row>
     <row r="55">
@@ -3262,11 +3262,11 @@
         </is>
       </c>
       <c r="G56" s="7" t="n">
-        <v>4450</v>
+        <v>4400</v>
       </c>
       <c r="H56" s="6" t="inlineStr">
         <is>
-          <t>20/23</t>
+          <t>21/23</t>
         </is>
       </c>
       <c r="I56" s="6" t="inlineStr">
@@ -3275,10 +3275,10 @@
         </is>
       </c>
       <c r="J56" s="7" t="n">
-        <v>5118</v>
+        <v>4819</v>
       </c>
       <c r="K56" s="8" t="n">
-        <v>222.5</v>
+        <v>209.5238095238095</v>
       </c>
     </row>
     <row r="57">
@@ -3360,11 +3360,11 @@
         </is>
       </c>
       <c r="G58" s="7" t="n">
-        <v>11496</v>
+        <v>10939</v>
       </c>
       <c r="H58" s="6" t="inlineStr">
         <is>
-          <t>16/23</t>
+          <t>17/23</t>
         </is>
       </c>
       <c r="I58" s="6" t="inlineStr">
@@ -3373,10 +3373,10 @@
         </is>
       </c>
       <c r="J58" s="7" t="n">
-        <v>16526</v>
+        <v>14800</v>
       </c>
       <c r="K58" s="8" t="n">
-        <v>718.5</v>
+        <v>643.4705882352941</v>
       </c>
     </row>
     <row r="59">
@@ -3409,11 +3409,11 @@
         </is>
       </c>
       <c r="G59" s="4" t="n">
-        <v>13027</v>
+        <v>14827</v>
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>16/21</t>
+          <t>17/21</t>
         </is>
       </c>
       <c r="I59" s="3" t="inlineStr">
@@ -3422,10 +3422,10 @@
         </is>
       </c>
       <c r="J59" s="4" t="n">
-        <v>17098</v>
+        <v>18316</v>
       </c>
       <c r="K59" s="5" t="n">
-        <v>814.1875</v>
+        <v>872.1764705882352</v>
       </c>
     </row>
     <row r="60">
@@ -3439,30 +3439,30 @@
       </c>
       <c r="C60" s="14" t="inlineStr">
         <is>
+          <t>C. KRISHNAMURALI</t>
+        </is>
+      </c>
+      <c r="D60" s="14" t="inlineStr">
+        <is>
+          <t>All India Anna Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E60" s="14" t="inlineStr">
+        <is>
           <t>RAJENDRAN. T. M</t>
         </is>
       </c>
-      <c r="D60" s="14" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E60" s="14" t="inlineStr">
-        <is>
-          <t>C. KRISHNAMURALI</t>
-        </is>
-      </c>
       <c r="F60" s="14" t="inlineStr">
         <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
+          <t>Dravida Munnetra Kazhagam</t>
         </is>
       </c>
       <c r="G60" s="15" t="n">
-        <v>193</v>
+        <v>232</v>
       </c>
       <c r="H60" s="14" t="inlineStr">
         <is>
-          <t>14/26</t>
+          <t>15/26</t>
         </is>
       </c>
       <c r="I60" s="14" t="inlineStr">
@@ -3471,10 +3471,10 @@
         </is>
       </c>
       <c r="J60" s="15" t="n">
-        <v>358</v>
+        <v>402</v>
       </c>
       <c r="K60" s="16" t="n">
-        <v>13.78571428571429</v>
+        <v>15.46666666666667</v>
       </c>
     </row>
     <row r="61">
@@ -3556,11 +3556,11 @@
         </is>
       </c>
       <c r="G62" s="7" t="n">
-        <v>3152</v>
+        <v>2185</v>
       </c>
       <c r="H62" s="6" t="inlineStr">
         <is>
-          <t>15/27</t>
+          <t>16/27</t>
         </is>
       </c>
       <c r="I62" s="6" t="inlineStr">
@@ -3569,10 +3569,10 @@
         </is>
       </c>
       <c r="J62" s="7" t="n">
-        <v>5674</v>
+        <v>3687</v>
       </c>
       <c r="K62" s="8" t="n">
-        <v>210.1333333333333</v>
+        <v>136.5625</v>
       </c>
     </row>
     <row r="63">
@@ -3821,52 +3821,52 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="9" t="inlineStr">
+      <c r="A68" s="13" t="inlineStr">
         <is>
           <t>KATPADI</t>
         </is>
       </c>
-      <c r="B68" s="10" t="n">
+      <c r="B68" s="14" t="n">
         <v>40</v>
       </c>
-      <c r="C68" s="10" t="inlineStr">
+      <c r="C68" s="14" t="inlineStr">
         <is>
           <t>V. RAMU</t>
         </is>
       </c>
-      <c r="D68" s="10" t="inlineStr">
+      <c r="D68" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E68" s="10" t="inlineStr">
+      <c r="E68" s="14" t="inlineStr">
         <is>
           <t>DR M SUDHAKAR</t>
         </is>
       </c>
-      <c r="F68" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G68" s="11" t="n">
-        <v>1313</v>
-      </c>
-      <c r="H68" s="10" t="inlineStr">
-        <is>
-          <t>10/20</t>
-        </is>
-      </c>
-      <c r="I68" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J68" s="11" t="n">
-        <v>2626</v>
-      </c>
-      <c r="K68" s="12" t="n">
-        <v>131.3</v>
+      <c r="F68" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G68" s="15" t="n">
+        <v>141</v>
+      </c>
+      <c r="H68" s="14" t="inlineStr">
+        <is>
+          <t>11/20</t>
+        </is>
+      </c>
+      <c r="I68" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J68" s="15" t="n">
+        <v>256</v>
+      </c>
+      <c r="K68" s="16" t="n">
+        <v>12.81818181818182</v>
       </c>
     </row>
     <row r="69">
@@ -3948,11 +3948,11 @@
         </is>
       </c>
       <c r="G70" s="4" t="n">
-        <v>39671</v>
+        <v>41243</v>
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>24/28</t>
+          <t>25/28</t>
         </is>
       </c>
       <c r="I70" s="3" t="inlineStr">
@@ -3961,59 +3961,59 @@
         </is>
       </c>
       <c r="J70" s="4" t="n">
-        <v>46283</v>
+        <v>46192</v>
       </c>
       <c r="K70" s="5" t="n">
-        <v>1652.958333333333</v>
+        <v>1649.72</v>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="13" t="inlineStr">
+      <c r="A71" s="9" t="inlineStr">
         <is>
           <t>KILLIYOOR</t>
         </is>
       </c>
-      <c r="B71" s="14" t="n">
+      <c r="B71" s="10" t="n">
         <v>234</v>
       </c>
-      <c r="C71" s="14" t="inlineStr">
+      <c r="C71" s="10" t="inlineStr">
         <is>
           <t>RAJESH KUMAR. S</t>
         </is>
       </c>
-      <c r="D71" s="14" t="inlineStr">
+      <c r="D71" s="10" t="inlineStr">
         <is>
           <t>Indian National Congress</t>
         </is>
       </c>
-      <c r="E71" s="14" t="inlineStr">
+      <c r="E71" s="10" t="inlineStr">
         <is>
           <t>SABIN. S</t>
         </is>
       </c>
-      <c r="F71" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G71" s="15" t="n">
-        <v>143</v>
-      </c>
-      <c r="H71" s="14" t="inlineStr">
-        <is>
-          <t>14/22</t>
-        </is>
-      </c>
-      <c r="I71" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J71" s="15" t="n">
-        <v>225</v>
-      </c>
-      <c r="K71" s="16" t="n">
-        <v>10.21428571428571</v>
+      <c r="F71" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G71" s="11" t="n">
+        <v>910</v>
+      </c>
+      <c r="H71" s="10" t="inlineStr">
+        <is>
+          <t>15/22</t>
+        </is>
+      </c>
+      <c r="I71" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J71" s="11" t="n">
+        <v>1335</v>
+      </c>
+      <c r="K71" s="12" t="n">
+        <v>60.66666666666667</v>
       </c>
     </row>
     <row r="72">
@@ -4046,11 +4046,11 @@
         </is>
       </c>
       <c r="G72" s="4" t="n">
-        <v>27814</v>
+        <v>28382</v>
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>17/22</t>
+          <t>18/22</t>
         </is>
       </c>
       <c r="I72" s="3" t="inlineStr">
@@ -4059,59 +4059,59 @@
         </is>
       </c>
       <c r="J72" s="4" t="n">
-        <v>35995</v>
+        <v>34689</v>
       </c>
       <c r="K72" s="5" t="n">
-        <v>1636.117647058823</v>
+        <v>1576.777777777778</v>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="6" t="inlineStr">
+      <c r="A73" s="2" t="inlineStr">
         <is>
           <t>KILVAITHINANKUPPAM</t>
         </is>
       </c>
-      <c r="B73" s="6" t="n">
+      <c r="B73" s="3" t="n">
         <v>45</v>
       </c>
-      <c r="C73" s="6" t="inlineStr">
+      <c r="C73" s="3" t="inlineStr">
         <is>
           <t>THENRAL KUMAR. E</t>
         </is>
       </c>
-      <c r="D73" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E73" s="6" t="inlineStr">
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
         <is>
           <t>DR. RAJESWARI. R</t>
         </is>
       </c>
-      <c r="F73" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G73" s="7" t="n">
-        <v>8083</v>
-      </c>
-      <c r="H73" s="6" t="inlineStr">
-        <is>
-          <t>8/19</t>
-        </is>
-      </c>
-      <c r="I73" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J73" s="7" t="n">
-        <v>19197</v>
-      </c>
-      <c r="K73" s="8" t="n">
-        <v>1010.375</v>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G73" s="4" t="n">
+        <v>9794</v>
+      </c>
+      <c r="H73" s="3" t="inlineStr">
+        <is>
+          <t>9/19</t>
+        </is>
+      </c>
+      <c r="I73" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J73" s="4" t="n">
+        <v>20676</v>
+      </c>
+      <c r="K73" s="5" t="n">
+        <v>1088.222222222222</v>
       </c>
     </row>
     <row r="74">
@@ -4125,30 +4125,30 @@
       </c>
       <c r="C74" s="10" t="inlineStr">
         <is>
+          <t>LATHA. T</t>
+        </is>
+      </c>
+      <c r="D74" s="10" t="inlineStr">
+        <is>
+          <t>Communist Party of India (Marxist)</t>
+        </is>
+      </c>
+      <c r="E74" s="10" t="inlineStr">
+        <is>
           <t>SENTHIL PANDIAN. P</t>
         </is>
       </c>
-      <c r="D74" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E74" s="10" t="inlineStr">
-        <is>
-          <t>LATHA. T</t>
-        </is>
-      </c>
       <c r="F74" s="10" t="inlineStr">
         <is>
-          <t>Communist Party of India (Marxist)</t>
+          <t>Tamilaga Vettri Kazhagam</t>
         </is>
       </c>
       <c r="G74" s="11" t="n">
-        <v>425</v>
+        <v>663</v>
       </c>
       <c r="H74" s="10" t="inlineStr">
         <is>
-          <t>10/16</t>
+          <t>11/16</t>
         </is>
       </c>
       <c r="I74" s="10" t="inlineStr">
@@ -4157,10 +4157,10 @@
         </is>
       </c>
       <c r="J74" s="11" t="n">
-        <v>680</v>
+        <v>964</v>
       </c>
       <c r="K74" s="12" t="n">
-        <v>42.5</v>
+        <v>60.27272727272727</v>
       </c>
     </row>
     <row r="75">
@@ -4213,52 +4213,52 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="6" t="inlineStr">
+      <c r="A76" s="2" t="inlineStr">
         <is>
           <t>KOLATHUR</t>
         </is>
       </c>
-      <c r="B76" s="6" t="n">
+      <c r="B76" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="C76" s="6" t="inlineStr">
+      <c r="C76" s="3" t="inlineStr">
         <is>
           <t>V. S. BABU</t>
         </is>
       </c>
-      <c r="D76" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E76" s="6" t="inlineStr">
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
         <is>
           <t>M. K. STALIN</t>
         </is>
       </c>
-      <c r="F76" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G76" s="7" t="n">
-        <v>7544</v>
-      </c>
-      <c r="H76" s="6" t="inlineStr">
-        <is>
-          <t>16/22</t>
-        </is>
-      </c>
-      <c r="I76" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J76" s="7" t="n">
-        <v>10373</v>
-      </c>
-      <c r="K76" s="8" t="n">
-        <v>471.5</v>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G76" s="4" t="n">
+        <v>7731</v>
+      </c>
+      <c r="H76" s="3" t="inlineStr">
+        <is>
+          <t>17/22</t>
+        </is>
+      </c>
+      <c r="I76" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J76" s="4" t="n">
+        <v>10005</v>
+      </c>
+      <c r="K76" s="5" t="n">
+        <v>454.7647058823529</v>
       </c>
     </row>
     <row r="77">
@@ -4291,11 +4291,11 @@
         </is>
       </c>
       <c r="G77" s="7" t="n">
-        <v>5265</v>
+        <v>4605</v>
       </c>
       <c r="H77" s="6" t="inlineStr">
         <is>
-          <t>14/23</t>
+          <t>15/23</t>
         </is>
       </c>
       <c r="I77" s="6" t="inlineStr">
@@ -4304,10 +4304,10 @@
         </is>
       </c>
       <c r="J77" s="7" t="n">
-        <v>8650</v>
+        <v>7061</v>
       </c>
       <c r="K77" s="8" t="n">
-        <v>376.0714285714286</v>
+        <v>307</v>
       </c>
     </row>
     <row r="78">
@@ -4340,11 +4340,11 @@
         </is>
       </c>
       <c r="G78" s="4" t="n">
-        <v>18582</v>
+        <v>19141</v>
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
-          <t>20/25</t>
+          <t>21/25</t>
         </is>
       </c>
       <c r="I78" s="3" t="inlineStr">
@@ -4353,10 +4353,10 @@
         </is>
       </c>
       <c r="J78" s="4" t="n">
-        <v>23228</v>
+        <v>22787</v>
       </c>
       <c r="K78" s="5" t="n">
-        <v>929.1</v>
+        <v>911.4761904761905</v>
       </c>
     </row>
     <row r="79">
@@ -4438,11 +4438,11 @@
         </is>
       </c>
       <c r="G80" s="7" t="n">
-        <v>2256</v>
+        <v>2207</v>
       </c>
       <c r="H80" s="6" t="inlineStr">
         <is>
-          <t>14/21</t>
+          <t>15/21</t>
         </is>
       </c>
       <c r="I80" s="6" t="inlineStr">
@@ -4451,10 +4451,10 @@
         </is>
       </c>
       <c r="J80" s="7" t="n">
-        <v>3384</v>
+        <v>3090</v>
       </c>
       <c r="K80" s="8" t="n">
-        <v>161.1428571428571</v>
+        <v>147.1333333333333</v>
       </c>
     </row>
     <row r="81">
@@ -4487,11 +4487,11 @@
         </is>
       </c>
       <c r="G81" s="7" t="n">
-        <v>1927</v>
+        <v>3029</v>
       </c>
       <c r="H81" s="6" t="inlineStr">
         <is>
-          <t>13/24</t>
+          <t>14/24</t>
         </is>
       </c>
       <c r="I81" s="6" t="inlineStr">
@@ -4500,10 +4500,10 @@
         </is>
       </c>
       <c r="J81" s="7" t="n">
-        <v>3558</v>
+        <v>5193</v>
       </c>
       <c r="K81" s="8" t="n">
-        <v>148.2307692307692</v>
+        <v>216.3571428571429</v>
       </c>
     </row>
     <row r="82">
@@ -4585,11 +4585,11 @@
         </is>
       </c>
       <c r="G83" s="4" t="n">
-        <v>15608</v>
+        <v>15601</v>
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
-          <t>17/25</t>
+          <t>18/25</t>
         </is>
       </c>
       <c r="I83" s="3" t="inlineStr">
@@ -4598,10 +4598,10 @@
         </is>
       </c>
       <c r="J83" s="4" t="n">
-        <v>22953</v>
+        <v>21668</v>
       </c>
       <c r="K83" s="5" t="n">
-        <v>918.1176470588235</v>
+        <v>866.7222222222222</v>
       </c>
     </row>
     <row r="84">
@@ -4732,11 +4732,11 @@
         </is>
       </c>
       <c r="G86" s="7" t="n">
-        <v>4567</v>
+        <v>5807</v>
       </c>
       <c r="H86" s="6" t="inlineStr">
         <is>
-          <t>12/21</t>
+          <t>13/21</t>
         </is>
       </c>
       <c r="I86" s="6" t="inlineStr">
@@ -4745,10 +4745,10 @@
         </is>
       </c>
       <c r="J86" s="7" t="n">
-        <v>7992</v>
+        <v>9381</v>
       </c>
       <c r="K86" s="8" t="n">
-        <v>380.5833333333333</v>
+        <v>446.6923076923077</v>
       </c>
     </row>
     <row r="87">
@@ -4781,11 +4781,11 @@
         </is>
       </c>
       <c r="G87" s="4" t="n">
-        <v>86155</v>
+        <v>91600</v>
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
-          <t>17/19</t>
+          <t>18/19</t>
         </is>
       </c>
       <c r="I87" s="3" t="inlineStr">
@@ -4794,10 +4794,10 @@
         </is>
       </c>
       <c r="J87" s="4" t="n">
-        <v>96291</v>
+        <v>96689</v>
       </c>
       <c r="K87" s="5" t="n">
-        <v>5067.941176470588</v>
+        <v>5088.888888888889</v>
       </c>
     </row>
     <row r="88">
@@ -4830,11 +4830,11 @@
         </is>
       </c>
       <c r="G88" s="4" t="n">
-        <v>15901</v>
+        <v>15374</v>
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>11/19</t>
+          <t>12/19</t>
         </is>
       </c>
       <c r="I88" s="3" t="inlineStr">
@@ -4843,10 +4843,10 @@
         </is>
       </c>
       <c r="J88" s="4" t="n">
-        <v>27465</v>
+        <v>24342</v>
       </c>
       <c r="K88" s="5" t="n">
-        <v>1445.545454545455</v>
+        <v>1281.166666666667</v>
       </c>
     </row>
     <row r="89">
@@ -4879,11 +4879,11 @@
         </is>
       </c>
       <c r="G89" s="7" t="n">
-        <v>8230</v>
+        <v>9621</v>
       </c>
       <c r="H89" s="6" t="inlineStr">
         <is>
-          <t>20/29</t>
+          <t>21/29</t>
         </is>
       </c>
       <c r="I89" s="6" t="inlineStr">
@@ -4892,10 +4892,10 @@
         </is>
       </c>
       <c r="J89" s="7" t="n">
-        <v>11934</v>
+        <v>13286</v>
       </c>
       <c r="K89" s="8" t="n">
-        <v>411.5</v>
+        <v>458.1428571428572</v>
       </c>
     </row>
     <row r="90">
@@ -5026,11 +5026,11 @@
         </is>
       </c>
       <c r="G92" s="4" t="n">
-        <v>6006</v>
+        <v>7147</v>
       </c>
       <c r="H92" s="3" t="inlineStr">
         <is>
-          <t>18/24</t>
+          <t>19/24</t>
         </is>
       </c>
       <c r="I92" s="3" t="inlineStr">
@@ -5039,59 +5039,59 @@
         </is>
       </c>
       <c r="J92" s="4" t="n">
-        <v>8008</v>
+        <v>9028</v>
       </c>
       <c r="K92" s="5" t="n">
-        <v>333.6666666666667</v>
+        <v>376.1578947368421</v>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="6" t="inlineStr">
+      <c r="A93" s="2" t="inlineStr">
         <is>
           <t>MADURANTAKAM</t>
         </is>
       </c>
-      <c r="B93" s="6" t="n">
+      <c r="B93" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="C93" s="6" t="inlineStr">
+      <c r="C93" s="3" t="inlineStr">
         <is>
           <t>MARAGATHAM KUMARAVEL.K</t>
         </is>
       </c>
-      <c r="D93" s="6" t="inlineStr">
+      <c r="D93" s="3" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E93" s="6" t="inlineStr">
+      <c r="E93" s="3" t="inlineStr">
         <is>
           <t>EZHIL KATHARINE EZHILMALAI</t>
         </is>
       </c>
-      <c r="F93" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G93" s="7" t="n">
-        <v>5429</v>
-      </c>
-      <c r="H93" s="6" t="inlineStr">
-        <is>
-          <t>15/21</t>
-        </is>
-      </c>
-      <c r="I93" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J93" s="7" t="n">
-        <v>7601</v>
-      </c>
-      <c r="K93" s="8" t="n">
-        <v>361.9333333333333</v>
+      <c r="F93" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G93" s="4" t="n">
+        <v>5157</v>
+      </c>
+      <c r="H93" s="3" t="inlineStr">
+        <is>
+          <t>16/21</t>
+        </is>
+      </c>
+      <c r="I93" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J93" s="4" t="n">
+        <v>6769</v>
+      </c>
+      <c r="K93" s="5" t="n">
+        <v>322.3125</v>
       </c>
     </row>
     <row r="94">
@@ -5124,11 +5124,11 @@
         </is>
       </c>
       <c r="G94" s="4" t="n">
-        <v>29024</v>
+        <v>31121</v>
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
-          <t>10/25</t>
+          <t>11/25</t>
         </is>
       </c>
       <c r="I94" s="3" t="inlineStr">
@@ -5137,10 +5137,10 @@
         </is>
       </c>
       <c r="J94" s="4" t="n">
-        <v>72560</v>
+        <v>70730</v>
       </c>
       <c r="K94" s="5" t="n">
-        <v>2902.4</v>
+        <v>2829.181818181818</v>
       </c>
     </row>
     <row r="95">
@@ -5320,11 +5320,11 @@
         </is>
       </c>
       <c r="G98" s="15" t="n">
-        <v>31</v>
+        <v>369</v>
       </c>
       <c r="H98" s="14" t="inlineStr">
         <is>
-          <t>20/25</t>
+          <t>21/25</t>
         </is>
       </c>
       <c r="I98" s="14" t="inlineStr">
@@ -5333,10 +5333,10 @@
         </is>
       </c>
       <c r="J98" s="15" t="n">
-        <v>39</v>
+        <v>439</v>
       </c>
       <c r="K98" s="16" t="n">
-        <v>1.55</v>
+        <v>17.57142857142857</v>
       </c>
     </row>
     <row r="99">
@@ -5418,11 +5418,11 @@
         </is>
       </c>
       <c r="G100" s="7" t="n">
-        <v>8004</v>
+        <v>8440</v>
       </c>
       <c r="H100" s="6" t="inlineStr">
         <is>
-          <t>14/22</t>
+          <t>15/22</t>
         </is>
       </c>
       <c r="I100" s="6" t="inlineStr">
@@ -5431,10 +5431,10 @@
         </is>
       </c>
       <c r="J100" s="7" t="n">
-        <v>12578</v>
+        <v>12379</v>
       </c>
       <c r="K100" s="8" t="n">
-        <v>571.7142857142857</v>
+        <v>562.6666666666667</v>
       </c>
     </row>
     <row r="101">
@@ -5516,11 +5516,11 @@
         </is>
       </c>
       <c r="G102" s="11" t="n">
-        <v>637</v>
+        <v>1597</v>
       </c>
       <c r="H102" s="10" t="inlineStr">
         <is>
-          <t>15/26</t>
+          <t>16/26</t>
         </is>
       </c>
       <c r="I102" s="10" t="inlineStr">
@@ -5529,10 +5529,10 @@
         </is>
       </c>
       <c r="J102" s="11" t="n">
-        <v>1104</v>
+        <v>2595</v>
       </c>
       <c r="K102" s="12" t="n">
-        <v>42.46666666666667</v>
+        <v>99.8125</v>
       </c>
     </row>
     <row r="103">
@@ -5546,30 +5546,30 @@
       </c>
       <c r="C103" s="14" t="inlineStr">
         <is>
+          <t>MIDHUN CHAKRAVARTHY. M</t>
+        </is>
+      </c>
+      <c r="D103" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E103" s="14" t="inlineStr">
+        <is>
           <t>VENKATACHALAM. G</t>
         </is>
       </c>
-      <c r="D103" s="14" t="inlineStr">
+      <c r="F103" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E103" s="14" t="inlineStr">
-        <is>
-          <t>MIDHUN CHAKRAVARTHY. M</t>
-        </is>
-      </c>
-      <c r="F103" s="14" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
       <c r="G103" s="15" t="n">
-        <v>161</v>
+        <v>32</v>
       </c>
       <c r="H103" s="14" t="inlineStr">
         <is>
-          <t>12/24</t>
+          <t>13/24</t>
         </is>
       </c>
       <c r="I103" s="14" t="inlineStr">
@@ -5578,10 +5578,10 @@
         </is>
       </c>
       <c r="J103" s="15" t="n">
-        <v>322</v>
+        <v>59</v>
       </c>
       <c r="K103" s="16" t="n">
-        <v>13.41666666666667</v>
+        <v>2.461538461538462</v>
       </c>
     </row>
     <row r="104">
@@ -5663,11 +5663,11 @@
         </is>
       </c>
       <c r="G105" s="7" t="n">
-        <v>11356</v>
+        <v>11994</v>
       </c>
       <c r="H105" s="6" t="inlineStr">
         <is>
-          <t>20/30</t>
+          <t>21/30</t>
         </is>
       </c>
       <c r="I105" s="6" t="inlineStr">
@@ -5676,10 +5676,10 @@
         </is>
       </c>
       <c r="J105" s="7" t="n">
-        <v>17034</v>
+        <v>17134</v>
       </c>
       <c r="K105" s="8" t="n">
-        <v>567.8</v>
+        <v>571.1428571428571</v>
       </c>
     </row>
     <row r="106">
@@ -5761,11 +5761,11 @@
         </is>
       </c>
       <c r="G107" s="4" t="n">
-        <v>25547</v>
+        <v>26853</v>
       </c>
       <c r="H107" s="3" t="inlineStr">
         <is>
-          <t>17/20</t>
+          <t>18/20</t>
         </is>
       </c>
       <c r="I107" s="3" t="inlineStr">
@@ -5774,10 +5774,10 @@
         </is>
       </c>
       <c r="J107" s="4" t="n">
-        <v>30055</v>
+        <v>29837</v>
       </c>
       <c r="K107" s="5" t="n">
-        <v>1502.764705882353</v>
+        <v>1491.833333333333</v>
       </c>
     </row>
     <row r="108">
@@ -5801,20 +5801,20 @@
       </c>
       <c r="E108" s="3" t="inlineStr">
         <is>
-          <t>THANKA.KATHIRAVAN</t>
+          <t>M.SUGUMAR</t>
         </is>
       </c>
       <c r="F108" s="3" t="inlineStr">
         <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
+          <t>Tamilaga Vettri Kazhagam</t>
         </is>
       </c>
       <c r="G108" s="4" t="n">
-        <v>11757</v>
+        <v>11123</v>
       </c>
       <c r="H108" s="3" t="inlineStr">
         <is>
-          <t>9/18</t>
+          <t>10/18</t>
         </is>
       </c>
       <c r="I108" s="3" t="inlineStr">
@@ -5823,10 +5823,10 @@
         </is>
       </c>
       <c r="J108" s="4" t="n">
-        <v>23514</v>
+        <v>20021</v>
       </c>
       <c r="K108" s="5" t="n">
-        <v>1306.333333333333</v>
+        <v>1112.3</v>
       </c>
     </row>
     <row r="109">
@@ -5859,11 +5859,11 @@
         </is>
       </c>
       <c r="G109" s="7" t="n">
-        <v>3456</v>
+        <v>3260</v>
       </c>
       <c r="H109" s="6" t="inlineStr">
         <is>
-          <t>18/23</t>
+          <t>19/23</t>
         </is>
       </c>
       <c r="I109" s="6" t="inlineStr">
@@ -5872,10 +5872,10 @@
         </is>
       </c>
       <c r="J109" s="7" t="n">
-        <v>4416</v>
+        <v>3946</v>
       </c>
       <c r="K109" s="8" t="n">
-        <v>192</v>
+        <v>171.578947368421</v>
       </c>
     </row>
     <row r="110">
@@ -6124,52 +6124,52 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="9" t="inlineStr">
+      <c r="A115" s="13" t="inlineStr">
         <is>
           <t>NILAKKOTTAI</t>
         </is>
       </c>
-      <c r="B115" s="10" t="n">
+      <c r="B115" s="14" t="n">
         <v>130</v>
       </c>
-      <c r="C115" s="10" t="inlineStr">
+      <c r="C115" s="14" t="inlineStr">
+        <is>
+          <t>AYYANAR.R</t>
+        </is>
+      </c>
+      <c r="D115" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E115" s="14" t="inlineStr">
         <is>
           <t>NAGAJOTHI.S</t>
         </is>
       </c>
-      <c r="D115" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E115" s="10" t="inlineStr">
-        <is>
-          <t>AYYANAR.R</t>
-        </is>
-      </c>
-      <c r="F115" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G115" s="11" t="n">
-        <v>520</v>
-      </c>
-      <c r="H115" s="10" t="inlineStr">
-        <is>
-          <t>12/23</t>
-        </is>
-      </c>
-      <c r="I115" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J115" s="11" t="n">
-        <v>997</v>
-      </c>
-      <c r="K115" s="12" t="n">
-        <v>43.33333333333334</v>
+      <c r="F115" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G115" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="H115" s="14" t="inlineStr">
+        <is>
+          <t>13/23</t>
+        </is>
+      </c>
+      <c r="I115" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J115" s="15" t="n">
+        <v>28</v>
+      </c>
+      <c r="K115" s="16" t="n">
+        <v>1.230769230769231</v>
       </c>
     </row>
     <row r="116">
@@ -6202,11 +6202,11 @@
         </is>
       </c>
       <c r="G116" s="4" t="n">
-        <v>28835</v>
+        <v>31339</v>
       </c>
       <c r="H116" s="3" t="inlineStr">
         <is>
-          <t>16/24</t>
+          <t>17/24</t>
         </is>
       </c>
       <c r="I116" s="3" t="inlineStr">
@@ -6215,10 +6215,10 @@
         </is>
       </c>
       <c r="J116" s="4" t="n">
-        <v>43252</v>
+        <v>44243</v>
       </c>
       <c r="K116" s="5" t="n">
-        <v>1802.1875</v>
+        <v>1843.470588235294</v>
       </c>
     </row>
     <row r="117">
@@ -6251,11 +6251,11 @@
         </is>
       </c>
       <c r="G117" s="7" t="n">
-        <v>7988</v>
+        <v>10754</v>
       </c>
       <c r="H117" s="6" t="inlineStr">
         <is>
-          <t>17/26</t>
+          <t>18/26</t>
         </is>
       </c>
       <c r="I117" s="6" t="inlineStr">
@@ -6264,10 +6264,10 @@
         </is>
       </c>
       <c r="J117" s="7" t="n">
-        <v>12217</v>
+        <v>15534</v>
       </c>
       <c r="K117" s="8" t="n">
-        <v>469.8823529411765</v>
+        <v>597.4444444444445</v>
       </c>
     </row>
     <row r="118">
@@ -6300,11 +6300,11 @@
         </is>
       </c>
       <c r="G118" s="4" t="n">
-        <v>30266</v>
+        <v>31686</v>
       </c>
       <c r="H118" s="3" t="inlineStr">
         <is>
-          <t>20/23</t>
+          <t>21/24</t>
         </is>
       </c>
       <c r="I118" s="3" t="inlineStr">
@@ -6313,10 +6313,10 @@
         </is>
       </c>
       <c r="J118" s="4" t="n">
-        <v>34806</v>
+        <v>36213</v>
       </c>
       <c r="K118" s="5" t="n">
-        <v>1513.3</v>
+        <v>1508.857142857143</v>
       </c>
     </row>
     <row r="119">
@@ -6349,11 +6349,11 @@
         </is>
       </c>
       <c r="G119" s="4" t="n">
-        <v>22447</v>
+        <v>22678</v>
       </c>
       <c r="H119" s="3" t="inlineStr">
         <is>
-          <t>16/23</t>
+          <t>17/23</t>
         </is>
       </c>
       <c r="I119" s="3" t="inlineStr">
@@ -6362,10 +6362,10 @@
         </is>
       </c>
       <c r="J119" s="4" t="n">
-        <v>32268</v>
+        <v>30682</v>
       </c>
       <c r="K119" s="5" t="n">
-        <v>1402.9375</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="120">
@@ -6398,11 +6398,11 @@
         </is>
       </c>
       <c r="G120" s="7" t="n">
-        <v>10209</v>
+        <v>12036</v>
       </c>
       <c r="H120" s="6" t="inlineStr">
         <is>
-          <t>15/23</t>
+          <t>16/23</t>
         </is>
       </c>
       <c r="I120" s="6" t="inlineStr">
@@ -6411,10 +6411,10 @@
         </is>
       </c>
       <c r="J120" s="7" t="n">
-        <v>15654</v>
+        <v>17302</v>
       </c>
       <c r="K120" s="8" t="n">
-        <v>680.6</v>
+        <v>752.25</v>
       </c>
     </row>
     <row r="121">
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="G123" s="4" t="n">
-        <v>8903</v>
+        <v>9359</v>
       </c>
       <c r="H123" s="3" t="inlineStr">
         <is>
@@ -6558,10 +6558,10 @@
         </is>
       </c>
       <c r="J123" s="4" t="n">
-        <v>9793</v>
+        <v>10295</v>
       </c>
       <c r="K123" s="5" t="n">
-        <v>445.15</v>
+        <v>467.95</v>
       </c>
     </row>
     <row r="124">
@@ -6594,11 +6594,11 @@
         </is>
       </c>
       <c r="G124" s="4" t="n">
-        <v>32307</v>
+        <v>34719</v>
       </c>
       <c r="H124" s="3" t="inlineStr">
         <is>
-          <t>23/35</t>
+          <t>24/35</t>
         </is>
       </c>
       <c r="I124" s="3" t="inlineStr">
@@ -6607,10 +6607,10 @@
         </is>
       </c>
       <c r="J124" s="4" t="n">
-        <v>49163</v>
+        <v>50632</v>
       </c>
       <c r="K124" s="5" t="n">
-        <v>1404.652173913043</v>
+        <v>1446.625</v>
       </c>
     </row>
     <row r="125">
@@ -6643,11 +6643,11 @@
         </is>
       </c>
       <c r="G125" s="4" t="n">
-        <v>27588</v>
+        <v>29315</v>
       </c>
       <c r="H125" s="3" t="inlineStr">
         <is>
-          <t>17/34</t>
+          <t>18/34</t>
         </is>
       </c>
       <c r="I125" s="3" t="inlineStr">
@@ -6656,10 +6656,10 @@
         </is>
       </c>
       <c r="J125" s="4" t="n">
-        <v>55176</v>
+        <v>55373</v>
       </c>
       <c r="K125" s="5" t="n">
-        <v>1622.823529411765</v>
+        <v>1628.611111111111</v>
       </c>
     </row>
     <row r="126">
@@ -6839,11 +6839,11 @@
         </is>
       </c>
       <c r="G129" s="11" t="n">
-        <v>1341</v>
+        <v>1132</v>
       </c>
       <c r="H129" s="10" t="inlineStr">
         <is>
-          <t>20/24</t>
+          <t>21/24</t>
         </is>
       </c>
       <c r="I129" s="10" t="inlineStr">
@@ -6852,10 +6852,10 @@
         </is>
       </c>
       <c r="J129" s="11" t="n">
-        <v>1609</v>
+        <v>1294</v>
       </c>
       <c r="K129" s="12" t="n">
-        <v>67.05</v>
+        <v>53.90476190476191</v>
       </c>
     </row>
     <row r="130">
@@ -6957,101 +6957,101 @@
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="6" t="inlineStr">
+      <c r="A132" s="9" t="inlineStr">
         <is>
           <t>PENNAGARAM</t>
         </is>
       </c>
-      <c r="B132" s="6" t="n">
+      <c r="B132" s="10" t="n">
         <v>58</v>
       </c>
-      <c r="C132" s="6" t="inlineStr">
+      <c r="C132" s="10" t="inlineStr">
+        <is>
+          <t>GAJENDRAN. S.</t>
+        </is>
+      </c>
+      <c r="D132" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E132" s="10" t="inlineStr">
         <is>
           <t>SELVAM. V.</t>
         </is>
       </c>
-      <c r="D132" s="6" t="inlineStr">
+      <c r="F132" s="10" t="inlineStr">
         <is>
           <t>Pattali Makkal Katchi</t>
         </is>
       </c>
-      <c r="E132" s="6" t="inlineStr">
-        <is>
-          <t>GAJENDRAN. S.</t>
-        </is>
-      </c>
-      <c r="F132" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G132" s="7" t="n">
-        <v>1933</v>
-      </c>
-      <c r="H132" s="6" t="inlineStr">
-        <is>
-          <t>13/23</t>
-        </is>
-      </c>
-      <c r="I132" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J132" s="7" t="n">
-        <v>3420</v>
-      </c>
-      <c r="K132" s="8" t="n">
-        <v>148.6923076923077</v>
+      <c r="G132" s="11" t="n">
+        <v>1576</v>
+      </c>
+      <c r="H132" s="10" t="inlineStr">
+        <is>
+          <t>15/23</t>
+        </is>
+      </c>
+      <c r="I132" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J132" s="11" t="n">
+        <v>2417</v>
+      </c>
+      <c r="K132" s="12" t="n">
+        <v>105.0666666666667</v>
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="6" t="inlineStr">
+      <c r="A133" s="2" t="inlineStr">
         <is>
           <t>PERAMBALUR</t>
         </is>
       </c>
-      <c r="B133" s="6" t="n">
+      <c r="B133" s="3" t="n">
         <v>147</v>
       </c>
-      <c r="C133" s="6" t="inlineStr">
+      <c r="C133" s="3" t="inlineStr">
         <is>
           <t>SIVAKUMAR. K</t>
         </is>
       </c>
-      <c r="D133" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E133" s="6" t="inlineStr">
+      <c r="D133" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E133" s="3" t="inlineStr">
         <is>
           <t>DR. JAYALAKSHMI. S.T</t>
         </is>
       </c>
-      <c r="F133" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G133" s="7" t="n">
-        <v>10019</v>
-      </c>
-      <c r="H133" s="6" t="inlineStr">
-        <is>
-          <t>20/28</t>
-        </is>
-      </c>
-      <c r="I133" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J133" s="7" t="n">
-        <v>14027</v>
-      </c>
-      <c r="K133" s="8" t="n">
-        <v>500.95</v>
+      <c r="F133" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G133" s="4" t="n">
+        <v>9859</v>
+      </c>
+      <c r="H133" s="3" t="inlineStr">
+        <is>
+          <t>21/28</t>
+        </is>
+      </c>
+      <c r="I133" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J133" s="4" t="n">
+        <v>13145</v>
+      </c>
+      <c r="K133" s="5" t="n">
+        <v>469.4761904761905</v>
       </c>
     </row>
     <row r="134">
@@ -7202,52 +7202,52 @@
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="6" t="inlineStr">
+      <c r="A137" s="2" t="inlineStr">
         <is>
           <t>PERUNDURAI</t>
         </is>
       </c>
-      <c r="B137" s="6" t="n">
+      <c r="B137" s="3" t="n">
         <v>103</v>
       </c>
-      <c r="C137" s="6" t="inlineStr">
+      <c r="C137" s="3" t="inlineStr">
         <is>
           <t>JAYAKUMAR. S</t>
         </is>
       </c>
-      <c r="D137" s="6" t="inlineStr">
+      <c r="D137" s="3" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E137" s="6" t="inlineStr">
+      <c r="E137" s="3" t="inlineStr">
         <is>
           <t>THOPPU VENKATACHALAM (ALIAS) N.D. VENKATACHALAM</t>
         </is>
       </c>
-      <c r="F137" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G137" s="7" t="n">
-        <v>5236</v>
-      </c>
-      <c r="H137" s="6" t="inlineStr">
-        <is>
-          <t>15/21</t>
-        </is>
-      </c>
-      <c r="I137" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J137" s="7" t="n">
-        <v>7330</v>
-      </c>
-      <c r="K137" s="8" t="n">
-        <v>349.0666666666667</v>
+      <c r="F137" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G137" s="4" t="n">
+        <v>6709</v>
+      </c>
+      <c r="H137" s="3" t="inlineStr">
+        <is>
+          <t>16/21</t>
+        </is>
+      </c>
+      <c r="I137" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J137" s="4" t="n">
+        <v>8806</v>
+      </c>
+      <c r="K137" s="5" t="n">
+        <v>419.3125</v>
       </c>
     </row>
     <row r="138">
@@ -7427,11 +7427,11 @@
         </is>
       </c>
       <c r="G141" s="7" t="n">
-        <v>4011</v>
+        <v>5021</v>
       </c>
       <c r="H141" s="6" t="inlineStr">
         <is>
-          <t>14/25</t>
+          <t>15/25</t>
         </is>
       </c>
       <c r="I141" s="6" t="inlineStr">
@@ -7440,10 +7440,10 @@
         </is>
       </c>
       <c r="J141" s="7" t="n">
-        <v>7162</v>
+        <v>8368</v>
       </c>
       <c r="K141" s="8" t="n">
-        <v>286.4999999999999</v>
+        <v>334.7333333333333</v>
       </c>
     </row>
     <row r="142">
@@ -7623,11 +7623,11 @@
         </is>
       </c>
       <c r="G145" s="4" t="n">
-        <v>9970</v>
+        <v>10912</v>
       </c>
       <c r="H145" s="3" t="inlineStr">
         <is>
-          <t>16/20</t>
+          <t>17/20</t>
         </is>
       </c>
       <c r="I145" s="3" t="inlineStr">
@@ -7636,10 +7636,10 @@
         </is>
       </c>
       <c r="J145" s="4" t="n">
-        <v>12462</v>
+        <v>12838</v>
       </c>
       <c r="K145" s="5" t="n">
-        <v>623.125</v>
+        <v>641.8823529411765</v>
       </c>
     </row>
     <row r="146">
@@ -7672,11 +7672,11 @@
         </is>
       </c>
       <c r="G146" s="4" t="n">
-        <v>15209</v>
+        <v>14803</v>
       </c>
       <c r="H146" s="3" t="inlineStr">
         <is>
-          <t>25/29</t>
+          <t>26/29</t>
         </is>
       </c>
       <c r="I146" s="3" t="inlineStr">
@@ -7685,10 +7685,10 @@
         </is>
       </c>
       <c r="J146" s="4" t="n">
-        <v>17642</v>
+        <v>16511</v>
       </c>
       <c r="K146" s="5" t="n">
-        <v>608.36</v>
+        <v>569.3461538461538</v>
       </c>
     </row>
     <row r="147">
@@ -7741,52 +7741,52 @@
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="6" t="inlineStr">
+      <c r="A148" s="2" t="inlineStr">
         <is>
           <t>RASIPURAM</t>
         </is>
       </c>
-      <c r="B148" s="6" t="n">
+      <c r="B148" s="3" t="n">
         <v>92</v>
       </c>
-      <c r="C148" s="6" t="inlineStr">
+      <c r="C148" s="3" t="inlineStr">
         <is>
           <t>LOGESH TAMILSELVAN D</t>
         </is>
       </c>
-      <c r="D148" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E148" s="6" t="inlineStr">
+      <c r="D148" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E148" s="3" t="inlineStr">
         <is>
           <t>MATHIVENTHAN M DR</t>
         </is>
       </c>
-      <c r="F148" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G148" s="7" t="n">
-        <v>14061</v>
-      </c>
-      <c r="H148" s="6" t="inlineStr">
-        <is>
-          <t>15/21</t>
-        </is>
-      </c>
-      <c r="I148" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J148" s="7" t="n">
-        <v>19685</v>
-      </c>
-      <c r="K148" s="8" t="n">
-        <v>937.4</v>
+      <c r="F148" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G148" s="4" t="n">
+        <v>15193</v>
+      </c>
+      <c r="H148" s="3" t="inlineStr">
+        <is>
+          <t>16/21</t>
+        </is>
+      </c>
+      <c r="I148" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J148" s="4" t="n">
+        <v>19941</v>
+      </c>
+      <c r="K148" s="5" t="n">
+        <v>949.5625</v>
       </c>
     </row>
     <row r="149">
@@ -7868,11 +7868,11 @@
         </is>
       </c>
       <c r="G150" s="4" t="n">
-        <v>11868</v>
+        <v>14227</v>
       </c>
       <c r="H150" s="3" t="inlineStr">
         <is>
-          <t>12/14</t>
+          <t>13/14</t>
         </is>
       </c>
       <c r="I150" s="3" t="inlineStr">
@@ -7881,10 +7881,10 @@
         </is>
       </c>
       <c r="J150" s="4" t="n">
-        <v>13846</v>
+        <v>15321</v>
       </c>
       <c r="K150" s="5" t="n">
-        <v>989</v>
+        <v>1094.384615384615</v>
       </c>
     </row>
     <row r="151">
@@ -8064,11 +8064,11 @@
         </is>
       </c>
       <c r="G154" s="4" t="n">
-        <v>39014</v>
+        <v>41826</v>
       </c>
       <c r="H154" s="3" t="inlineStr">
         <is>
-          <t>12/23</t>
+          <t>13/23</t>
         </is>
       </c>
       <c r="I154" s="3" t="inlineStr">
@@ -8077,10 +8077,10 @@
         </is>
       </c>
       <c r="J154" s="4" t="n">
-        <v>74777</v>
+        <v>74000</v>
       </c>
       <c r="K154" s="5" t="n">
-        <v>3251.166666666667</v>
+        <v>3217.384615384616</v>
       </c>
     </row>
     <row r="155">
@@ -8133,52 +8133,52 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="9" t="inlineStr">
+      <c r="A156" s="6" t="inlineStr">
         <is>
           <t>SANKARAPURAM</t>
         </is>
       </c>
-      <c r="B156" s="10" t="n">
+      <c r="B156" s="6" t="n">
         <v>79</v>
       </c>
-      <c r="C156" s="10" t="inlineStr">
+      <c r="C156" s="6" t="inlineStr">
         <is>
           <t>UDHAYASURIYAN T</t>
         </is>
       </c>
-      <c r="D156" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E156" s="10" t="inlineStr">
+      <c r="D156" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E156" s="6" t="inlineStr">
         <is>
           <t>RAKESH R</t>
         </is>
       </c>
-      <c r="F156" s="10" t="inlineStr">
+      <c r="F156" s="6" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G156" s="11" t="n">
-        <v>969</v>
-      </c>
-      <c r="H156" s="10" t="inlineStr">
-        <is>
-          <t>9/25</t>
-        </is>
-      </c>
-      <c r="I156" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J156" s="11" t="n">
-        <v>2692</v>
-      </c>
-      <c r="K156" s="12" t="n">
-        <v>107.6666666666667</v>
+      <c r="G156" s="7" t="n">
+        <v>2254</v>
+      </c>
+      <c r="H156" s="6" t="inlineStr">
+        <is>
+          <t>10/25</t>
+        </is>
+      </c>
+      <c r="I156" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J156" s="7" t="n">
+        <v>5635</v>
+      </c>
+      <c r="K156" s="8" t="n">
+        <v>225.4</v>
       </c>
     </row>
     <row r="157">
@@ -8309,11 +8309,11 @@
         </is>
       </c>
       <c r="G159" s="11" t="n">
-        <v>792</v>
+        <v>458</v>
       </c>
       <c r="H159" s="10" t="inlineStr">
         <is>
-          <t>18/22</t>
+          <t>19/22</t>
         </is>
       </c>
       <c r="I159" s="10" t="inlineStr">
@@ -8322,10 +8322,10 @@
         </is>
       </c>
       <c r="J159" s="11" t="n">
-        <v>968</v>
+        <v>530</v>
       </c>
       <c r="K159" s="12" t="n">
-        <v>44</v>
+        <v>24.10526315789474</v>
       </c>
     </row>
     <row r="160">
@@ -8358,11 +8358,11 @@
         </is>
       </c>
       <c r="G160" s="11" t="n">
-        <v>701</v>
+        <v>628</v>
       </c>
       <c r="H160" s="10" t="inlineStr">
         <is>
-          <t>9/19</t>
+          <t>10/19</t>
         </is>
       </c>
       <c r="I160" s="10" t="inlineStr">
@@ -8371,10 +8371,10 @@
         </is>
       </c>
       <c r="J160" s="11" t="n">
-        <v>1480</v>
+        <v>1193</v>
       </c>
       <c r="K160" s="12" t="n">
-        <v>77.88888888888889</v>
+        <v>62.8</v>
       </c>
     </row>
     <row r="161">
@@ -8505,11 +8505,11 @@
         </is>
       </c>
       <c r="G163" s="4" t="n">
-        <v>13494</v>
+        <v>14442</v>
       </c>
       <c r="H163" s="3" t="inlineStr">
         <is>
-          <t>14/26</t>
+          <t>15/26</t>
         </is>
       </c>
       <c r="I163" s="3" t="inlineStr">
@@ -8518,10 +8518,10 @@
         </is>
       </c>
       <c r="J163" s="4" t="n">
-        <v>25060</v>
+        <v>25033</v>
       </c>
       <c r="K163" s="5" t="n">
-        <v>963.8571428571429</v>
+        <v>962.8000000000001</v>
       </c>
     </row>
     <row r="164">
@@ -8603,11 +8603,11 @@
         </is>
       </c>
       <c r="G165" s="7" t="n">
-        <v>8116</v>
+        <v>8547</v>
       </c>
       <c r="H165" s="6" t="inlineStr">
         <is>
-          <t>14/29</t>
+          <t>15/29</t>
         </is>
       </c>
       <c r="I165" s="6" t="inlineStr">
@@ -8616,10 +8616,10 @@
         </is>
       </c>
       <c r="J165" s="7" t="n">
-        <v>16812</v>
+        <v>16524</v>
       </c>
       <c r="K165" s="8" t="n">
-        <v>579.7142857142857</v>
+        <v>569.8</v>
       </c>
     </row>
     <row r="166">
@@ -8701,11 +8701,11 @@
         </is>
       </c>
       <c r="G167" s="4" t="n">
-        <v>26478</v>
+        <v>28623</v>
       </c>
       <c r="H167" s="3" t="inlineStr">
         <is>
-          <t>16/32</t>
+          <t>17/32</t>
         </is>
       </c>
       <c r="I167" s="3" t="inlineStr">
@@ -8714,10 +8714,10 @@
         </is>
       </c>
       <c r="J167" s="4" t="n">
-        <v>52956</v>
+        <v>53879</v>
       </c>
       <c r="K167" s="5" t="n">
-        <v>1654.875</v>
+        <v>1683.705882352941</v>
       </c>
     </row>
     <row r="168">
@@ -8799,11 +8799,11 @@
         </is>
       </c>
       <c r="G169" s="15" t="n">
-        <v>207</v>
+        <v>136</v>
       </c>
       <c r="H169" s="14" t="inlineStr">
         <is>
-          <t>19/21</t>
+          <t>20/21</t>
         </is>
       </c>
       <c r="I169" s="14" t="inlineStr">
@@ -8812,10 +8812,10 @@
         </is>
       </c>
       <c r="J169" s="15" t="n">
-        <v>229</v>
+        <v>143</v>
       </c>
       <c r="K169" s="16" t="n">
-        <v>10.89473684210526</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="170">
@@ -8848,11 +8848,11 @@
         </is>
       </c>
       <c r="G170" s="7" t="n">
-        <v>2412</v>
+        <v>2260</v>
       </c>
       <c r="H170" s="6" t="inlineStr">
         <is>
-          <t>11/22</t>
+          <t>12/22</t>
         </is>
       </c>
       <c r="I170" s="6" t="inlineStr">
@@ -8861,10 +8861,10 @@
         </is>
       </c>
       <c r="J170" s="7" t="n">
-        <v>4824</v>
+        <v>4143</v>
       </c>
       <c r="K170" s="8" t="n">
-        <v>219.2727272727273</v>
+        <v>188.3333333333333</v>
       </c>
     </row>
     <row r="171">
@@ -8897,11 +8897,11 @@
         </is>
       </c>
       <c r="G171" s="7" t="n">
-        <v>9240</v>
+        <v>9889</v>
       </c>
       <c r="H171" s="6" t="inlineStr">
         <is>
-          <t>17/28</t>
+          <t>18/28</t>
         </is>
       </c>
       <c r="I171" s="6" t="inlineStr">
@@ -8910,10 +8910,10 @@
         </is>
       </c>
       <c r="J171" s="7" t="n">
-        <v>15219</v>
+        <v>15383</v>
       </c>
       <c r="K171" s="8" t="n">
-        <v>543.5294117647059</v>
+        <v>549.3888888888889</v>
       </c>
     </row>
     <row r="172">
@@ -8946,11 +8946,11 @@
         </is>
       </c>
       <c r="G172" s="4" t="n">
-        <v>21294</v>
+        <v>22484</v>
       </c>
       <c r="H172" s="3" t="inlineStr">
         <is>
-          <t>23/34</t>
+          <t>24/34</t>
         </is>
       </c>
       <c r="I172" s="3" t="inlineStr">
@@ -8959,10 +8959,10 @@
         </is>
       </c>
       <c r="J172" s="4" t="n">
-        <v>31478</v>
+        <v>31852</v>
       </c>
       <c r="K172" s="5" t="n">
-        <v>925.8260869565217</v>
+        <v>936.8333333333334</v>
       </c>
     </row>
     <row r="173">
@@ -9015,52 +9015,52 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="13" t="inlineStr">
+      <c r="A174" s="9" t="inlineStr">
         <is>
           <t>THALLI</t>
         </is>
       </c>
-      <c r="B174" s="14" t="n">
+      <c r="B174" s="10" t="n">
         <v>56</v>
       </c>
-      <c r="C174" s="14" t="inlineStr">
+      <c r="C174" s="10" t="inlineStr">
+        <is>
+          <t>RAMACHANDRAN. T</t>
+        </is>
+      </c>
+      <c r="D174" s="10" t="inlineStr">
+        <is>
+          <t>Communist Party of India</t>
+        </is>
+      </c>
+      <c r="E174" s="10" t="inlineStr">
         <is>
           <t>DR.NAGESH KUMAR. C</t>
         </is>
       </c>
-      <c r="D174" s="14" t="inlineStr">
+      <c r="F174" s="10" t="inlineStr">
         <is>
           <t>Bharatiya Janata Party</t>
         </is>
       </c>
-      <c r="E174" s="14" t="inlineStr">
-        <is>
-          <t>RAMACHANDRAN. T</t>
-        </is>
-      </c>
-      <c r="F174" s="14" t="inlineStr">
-        <is>
-          <t>Communist Party of India</t>
-        </is>
-      </c>
-      <c r="G174" s="15" t="n">
-        <v>24</v>
-      </c>
-      <c r="H174" s="14" t="inlineStr">
-        <is>
-          <t>13/24</t>
-        </is>
-      </c>
-      <c r="I174" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J174" s="15" t="n">
-        <v>44</v>
-      </c>
-      <c r="K174" s="16" t="n">
-        <v>1.846153846153846</v>
+      <c r="G174" s="11" t="n">
+        <v>477</v>
+      </c>
+      <c r="H174" s="10" t="inlineStr">
+        <is>
+          <t>14/24</t>
+        </is>
+      </c>
+      <c r="I174" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J174" s="11" t="n">
+        <v>818</v>
+      </c>
+      <c r="K174" s="12" t="n">
+        <v>34.07142857142857</v>
       </c>
     </row>
     <row r="175">
@@ -9182,20 +9182,20 @@
       </c>
       <c r="E177" s="3" t="inlineStr">
         <is>
-          <t>SATHISHKUMAR.N</t>
+          <t>UDHAYAKUMAR.R.B</t>
         </is>
       </c>
       <c r="F177" s="3" t="inlineStr">
         <is>
-          <t>Tamilaga Vettri Kazhagam</t>
+          <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
       <c r="G177" s="4" t="n">
-        <v>15762</v>
+        <v>16179</v>
       </c>
       <c r="H177" s="3" t="inlineStr">
         <is>
-          <t>19/26</t>
+          <t>20/26</t>
         </is>
       </c>
       <c r="I177" s="3" t="inlineStr">
@@ -9204,59 +9204,59 @@
         </is>
       </c>
       <c r="J177" s="4" t="n">
-        <v>21569</v>
+        <v>21033</v>
       </c>
       <c r="K177" s="5" t="n">
-        <v>829.578947368421</v>
+        <v>808.95</v>
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="6" t="inlineStr">
+      <c r="A178" s="9" t="inlineStr">
         <is>
           <t>THIRUMAYAM</t>
         </is>
       </c>
-      <c r="B178" s="6" t="n">
+      <c r="B178" s="10" t="n">
         <v>181</v>
       </c>
-      <c r="C178" s="6" t="inlineStr">
+      <c r="C178" s="10" t="inlineStr">
         <is>
           <t>REGUPATHY.S</t>
         </is>
       </c>
-      <c r="D178" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E178" s="6" t="inlineStr">
+      <c r="D178" s="10" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E178" s="10" t="inlineStr">
         <is>
           <t>VAIRAMUTHU.PK</t>
         </is>
       </c>
-      <c r="F178" s="6" t="inlineStr">
+      <c r="F178" s="10" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G178" s="7" t="n">
-        <v>1357</v>
-      </c>
-      <c r="H178" s="6" t="inlineStr">
-        <is>
-          <t>9/22</t>
-        </is>
-      </c>
-      <c r="I178" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J178" s="7" t="n">
-        <v>3317</v>
-      </c>
-      <c r="K178" s="8" t="n">
-        <v>150.7777777777778</v>
+      <c r="G178" s="11" t="n">
+        <v>547</v>
+      </c>
+      <c r="H178" s="10" t="inlineStr">
+        <is>
+          <t>10/22</t>
+        </is>
+      </c>
+      <c r="I178" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J178" s="11" t="n">
+        <v>1203</v>
+      </c>
+      <c r="K178" s="12" t="n">
+        <v>54.7</v>
       </c>
     </row>
     <row r="179">
@@ -9338,11 +9338,11 @@
         </is>
       </c>
       <c r="G180" s="4" t="n">
-        <v>25891</v>
+        <v>27550</v>
       </c>
       <c r="H180" s="3" t="inlineStr">
         <is>
-          <t>14/29</t>
+          <t>15/29</t>
         </is>
       </c>
       <c r="I180" s="3" t="inlineStr">
@@ -9351,10 +9351,10 @@
         </is>
       </c>
       <c r="J180" s="4" t="n">
-        <v>53631</v>
+        <v>53263</v>
       </c>
       <c r="K180" s="5" t="n">
-        <v>1849.357142857143</v>
+        <v>1836.666666666667</v>
       </c>
     </row>
     <row r="181">
@@ -9387,11 +9387,11 @@
         </is>
       </c>
       <c r="G181" s="4" t="n">
-        <v>8551</v>
+        <v>9690</v>
       </c>
       <c r="H181" s="3" t="inlineStr">
         <is>
-          <t>17/21</t>
+          <t>18/21</t>
         </is>
       </c>
       <c r="I181" s="3" t="inlineStr">
@@ -9400,10 +9400,10 @@
         </is>
       </c>
       <c r="J181" s="4" t="n">
-        <v>10563</v>
+        <v>11305</v>
       </c>
       <c r="K181" s="5" t="n">
-        <v>503</v>
+        <v>538.3333333333334</v>
       </c>
     </row>
     <row r="182">
@@ -9436,11 +9436,11 @@
         </is>
       </c>
       <c r="G182" s="7" t="n">
-        <v>8121</v>
+        <v>7803</v>
       </c>
       <c r="H182" s="6" t="inlineStr">
         <is>
-          <t>12/25</t>
+          <t>13/25</t>
         </is>
       </c>
       <c r="I182" s="6" t="inlineStr">
@@ -9449,10 +9449,10 @@
         </is>
       </c>
       <c r="J182" s="7" t="n">
-        <v>16919</v>
+        <v>15006</v>
       </c>
       <c r="K182" s="8" t="n">
-        <v>676.75</v>
+        <v>600.2307692307693</v>
       </c>
     </row>
     <row r="183">
@@ -9485,11 +9485,11 @@
         </is>
       </c>
       <c r="G183" s="4" t="n">
-        <v>13729</v>
+        <v>15578</v>
       </c>
       <c r="H183" s="3" t="inlineStr">
         <is>
-          <t>16/24</t>
+          <t>17/24</t>
         </is>
       </c>
       <c r="I183" s="3" t="inlineStr">
@@ -9498,10 +9498,10 @@
         </is>
       </c>
       <c r="J183" s="4" t="n">
-        <v>20594</v>
+        <v>21992</v>
       </c>
       <c r="K183" s="5" t="n">
-        <v>858.0625</v>
+        <v>916.3529411764706</v>
       </c>
     </row>
     <row r="184">
@@ -9534,11 +9534,11 @@
         </is>
       </c>
       <c r="G184" s="4" t="n">
-        <v>16401</v>
+        <v>17876</v>
       </c>
       <c r="H184" s="3" t="inlineStr">
         <is>
-          <t>22/24</t>
+          <t>23/24</t>
         </is>
       </c>
       <c r="I184" s="3" t="inlineStr">
@@ -9547,10 +9547,10 @@
         </is>
       </c>
       <c r="J184" s="4" t="n">
-        <v>17892</v>
+        <v>18653</v>
       </c>
       <c r="K184" s="5" t="n">
-        <v>745.5</v>
+        <v>777.2173913043479</v>
       </c>
     </row>
     <row r="185">
@@ -9632,11 +9632,11 @@
         </is>
       </c>
       <c r="G186" s="7" t="n">
-        <v>7849</v>
+        <v>9876</v>
       </c>
       <c r="H186" s="6" t="inlineStr">
         <is>
-          <t>15/24</t>
+          <t>16/24</t>
         </is>
       </c>
       <c r="I186" s="6" t="inlineStr">
@@ -9645,10 +9645,10 @@
         </is>
       </c>
       <c r="J186" s="7" t="n">
-        <v>12558</v>
+        <v>14814</v>
       </c>
       <c r="K186" s="8" t="n">
-        <v>523.2666666666667</v>
+        <v>617.25</v>
       </c>
     </row>
     <row r="187">
@@ -9681,11 +9681,11 @@
         </is>
       </c>
       <c r="G187" s="4" t="n">
-        <v>39525</v>
+        <v>41496</v>
       </c>
       <c r="H187" s="3" t="inlineStr">
         <is>
-          <t>17/25</t>
+          <t>18/25</t>
         </is>
       </c>
       <c r="I187" s="3" t="inlineStr">
@@ -9694,10 +9694,10 @@
         </is>
       </c>
       <c r="J187" s="4" t="n">
-        <v>58125</v>
+        <v>57633</v>
       </c>
       <c r="K187" s="5" t="n">
-        <v>2325</v>
+        <v>2305.333333333333</v>
       </c>
     </row>
     <row r="188">
@@ -9770,20 +9770,20 @@
       </c>
       <c r="E189" s="6" t="inlineStr">
         <is>
-          <t>N.R.KARTHIKEYAN</t>
+          <t>SATHISH RAJU (ALIAS) K.P.R. SATHISH</t>
         </is>
       </c>
       <c r="F189" s="6" t="inlineStr">
         <is>
-          <t>Dravida Munnetra Kazhagam</t>
+          <t>Tamilaga Vettri Kazhagam</t>
         </is>
       </c>
       <c r="G189" s="7" t="n">
-        <v>9848</v>
+        <v>10598</v>
       </c>
       <c r="H189" s="6" t="inlineStr">
         <is>
-          <t>14/27</t>
+          <t>15/27</t>
         </is>
       </c>
       <c r="I189" s="6" t="inlineStr">
@@ -9792,10 +9792,10 @@
         </is>
       </c>
       <c r="J189" s="7" t="n">
-        <v>18993</v>
+        <v>19076</v>
       </c>
       <c r="K189" s="8" t="n">
-        <v>703.4285714285714</v>
+        <v>706.5333333333333</v>
       </c>
     </row>
     <row r="190">
@@ -9828,11 +9828,11 @@
         </is>
       </c>
       <c r="G190" s="4" t="n">
-        <v>28169</v>
+        <v>29857</v>
       </c>
       <c r="H190" s="3" t="inlineStr">
         <is>
-          <t>18/26</t>
+          <t>19/26</t>
         </is>
       </c>
       <c r="I190" s="3" t="inlineStr">
@@ -9841,10 +9841,10 @@
         </is>
       </c>
       <c r="J190" s="4" t="n">
-        <v>40689</v>
+        <v>40857</v>
       </c>
       <c r="K190" s="5" t="n">
-        <v>1564.944444444444</v>
+        <v>1571.421052631579</v>
       </c>
     </row>
     <row r="191">
@@ -9877,11 +9877,11 @@
         </is>
       </c>
       <c r="G191" s="7" t="n">
-        <v>7536</v>
+        <v>9024</v>
       </c>
       <c r="H191" s="6" t="inlineStr">
         <is>
-          <t>11/18</t>
+          <t>12/18</t>
         </is>
       </c>
       <c r="I191" s="6" t="inlineStr">
@@ -9890,10 +9890,10 @@
         </is>
       </c>
       <c r="J191" s="7" t="n">
-        <v>12332</v>
+        <v>13536</v>
       </c>
       <c r="K191" s="8" t="n">
-        <v>685.0909090909091</v>
+        <v>752</v>
       </c>
     </row>
     <row r="192">
@@ -9946,52 +9946,52 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="9" t="inlineStr">
+      <c r="A193" s="6" t="inlineStr">
         <is>
           <t>TINDIVANAM</t>
         </is>
       </c>
-      <c r="B193" s="10" t="n">
+      <c r="B193" s="6" t="n">
         <v>72</v>
       </c>
-      <c r="C193" s="10" t="inlineStr">
+      <c r="C193" s="6" t="inlineStr">
         <is>
           <t>VANNI ARASU</t>
         </is>
       </c>
-      <c r="D193" s="10" t="inlineStr">
+      <c r="D193" s="6" t="inlineStr">
         <is>
           <t>Viduthalai Chiruthaigal Katchi</t>
         </is>
       </c>
-      <c r="E193" s="10" t="inlineStr">
+      <c r="E193" s="6" t="inlineStr">
         <is>
           <t>ARJUNAN. P</t>
         </is>
       </c>
-      <c r="F193" s="10" t="inlineStr">
+      <c r="F193" s="6" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G193" s="11" t="n">
-        <v>1560</v>
-      </c>
-      <c r="H193" s="10" t="inlineStr">
-        <is>
-          <t>12/22</t>
-        </is>
-      </c>
-      <c r="I193" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J193" s="11" t="n">
-        <v>2860</v>
-      </c>
-      <c r="K193" s="12" t="n">
-        <v>130</v>
+      <c r="G193" s="7" t="n">
+        <v>1947</v>
+      </c>
+      <c r="H193" s="6" t="inlineStr">
+        <is>
+          <t>13/22</t>
+        </is>
+      </c>
+      <c r="I193" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J193" s="7" t="n">
+        <v>3295</v>
+      </c>
+      <c r="K193" s="8" t="n">
+        <v>149.7692307692308</v>
       </c>
     </row>
     <row r="194">
@@ -10024,11 +10024,11 @@
         </is>
       </c>
       <c r="G194" s="4" t="n">
-        <v>5302</v>
+        <v>5601</v>
       </c>
       <c r="H194" s="3" t="inlineStr">
         <is>
-          <t>17/22</t>
+          <t>18/22</t>
         </is>
       </c>
       <c r="I194" s="3" t="inlineStr">
@@ -10037,10 +10037,10 @@
         </is>
       </c>
       <c r="J194" s="4" t="n">
-        <v>6861</v>
+        <v>6846</v>
       </c>
       <c r="K194" s="5" t="n">
-        <v>311.8823529411765</v>
+        <v>311.1666666666667</v>
       </c>
     </row>
     <row r="195">
@@ -10269,11 +10269,11 @@
         </is>
       </c>
       <c r="G199" s="11" t="n">
-        <v>972</v>
+        <v>1703</v>
       </c>
       <c r="H199" s="10" t="inlineStr">
         <is>
-          <t>14/24</t>
+          <t>15/24</t>
         </is>
       </c>
       <c r="I199" s="10" t="inlineStr">
@@ -10282,10 +10282,10 @@
         </is>
       </c>
       <c r="J199" s="11" t="n">
-        <v>1666</v>
+        <v>2725</v>
       </c>
       <c r="K199" s="12" t="n">
-        <v>69.42857142857143</v>
+        <v>113.5333333333333</v>
       </c>
     </row>
     <row r="200">
@@ -10318,11 +10318,11 @@
         </is>
       </c>
       <c r="G200" s="4" t="n">
-        <v>9196</v>
+        <v>9959</v>
       </c>
       <c r="H200" s="3" t="inlineStr">
         <is>
-          <t>25/28</t>
+          <t>26/28</t>
         </is>
       </c>
       <c r="I200" s="3" t="inlineStr">
@@ -10331,10 +10331,10 @@
         </is>
       </c>
       <c r="J200" s="4" t="n">
-        <v>10300</v>
+        <v>10725</v>
       </c>
       <c r="K200" s="5" t="n">
-        <v>367.84</v>
+        <v>383.0384615384615</v>
       </c>
     </row>
     <row r="201">
@@ -10367,11 +10367,11 @@
         </is>
       </c>
       <c r="G201" s="4" t="n">
-        <v>17070</v>
+        <v>21129</v>
       </c>
       <c r="H201" s="3" t="inlineStr">
         <is>
-          <t>10/22</t>
+          <t>11/22</t>
         </is>
       </c>
       <c r="I201" s="3" t="inlineStr">
@@ -10380,10 +10380,10 @@
         </is>
       </c>
       <c r="J201" s="4" t="n">
-        <v>37554</v>
+        <v>42258</v>
       </c>
       <c r="K201" s="5" t="n">
-        <v>1707</v>
+        <v>1920.818181818182</v>
       </c>
     </row>
     <row r="202">
@@ -10563,11 +10563,11 @@
         </is>
       </c>
       <c r="G205" s="7" t="n">
-        <v>7944</v>
+        <v>7682</v>
       </c>
       <c r="H205" s="6" t="inlineStr">
         <is>
-          <t>12/25</t>
+          <t>13/25</t>
         </is>
       </c>
       <c r="I205" s="6" t="inlineStr">
@@ -10576,10 +10576,10 @@
         </is>
       </c>
       <c r="J205" s="7" t="n">
-        <v>16550</v>
+        <v>14773</v>
       </c>
       <c r="K205" s="8" t="n">
-        <v>662</v>
+        <v>590.9230769230769</v>
       </c>
     </row>
     <row r="206">
@@ -10779,52 +10779,52 @@
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="6" t="inlineStr">
+      <c r="A210" s="9" t="inlineStr">
         <is>
           <t>UDUMALAIPETTAI</t>
         </is>
       </c>
-      <c r="B210" s="6" t="n">
+      <c r="B210" s="10" t="n">
         <v>125</v>
       </c>
-      <c r="C210" s="6" t="inlineStr">
+      <c r="C210" s="10" t="inlineStr">
         <is>
           <t>RADHAKRISHNAN K.</t>
         </is>
       </c>
-      <c r="D210" s="6" t="inlineStr">
+      <c r="D210" s="10" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E210" s="6" t="inlineStr">
+      <c r="E210" s="10" t="inlineStr">
         <is>
           <t>JAYAKUMAR M.</t>
         </is>
       </c>
-      <c r="F210" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G210" s="7" t="n">
-        <v>2832</v>
-      </c>
-      <c r="H210" s="6" t="inlineStr">
-        <is>
-          <t>18/22</t>
-        </is>
-      </c>
-      <c r="I210" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J210" s="7" t="n">
-        <v>3461</v>
-      </c>
-      <c r="K210" s="8" t="n">
-        <v>157.3333333333333</v>
+      <c r="F210" s="10" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G210" s="11" t="n">
+        <v>1602</v>
+      </c>
+      <c r="H210" s="10" t="inlineStr">
+        <is>
+          <t>19/22</t>
+        </is>
+      </c>
+      <c r="I210" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J210" s="11" t="n">
+        <v>1855</v>
+      </c>
+      <c r="K210" s="12" t="n">
+        <v>84.31578947368421</v>
       </c>
     </row>
     <row r="211">
@@ -10857,11 +10857,11 @@
         </is>
       </c>
       <c r="G211" s="11" t="n">
-        <v>1448</v>
+        <v>644</v>
       </c>
       <c r="H211" s="10" t="inlineStr">
         <is>
-          <t>14/27</t>
+          <t>15/27</t>
         </is>
       </c>
       <c r="I211" s="10" t="inlineStr">
@@ -10870,10 +10870,10 @@
         </is>
       </c>
       <c r="J211" s="11" t="n">
-        <v>2793</v>
+        <v>1159</v>
       </c>
       <c r="K211" s="12" t="n">
-        <v>103.4285714285714</v>
+        <v>42.93333333333333</v>
       </c>
     </row>
     <row r="212">
@@ -10955,11 +10955,11 @@
         </is>
       </c>
       <c r="G213" s="7" t="n">
-        <v>4888</v>
+        <v>4604</v>
       </c>
       <c r="H213" s="6" t="inlineStr">
         <is>
-          <t>20/23</t>
+          <t>21/23</t>
         </is>
       </c>
       <c r="I213" s="6" t="inlineStr">
@@ -10968,59 +10968,59 @@
         </is>
       </c>
       <c r="J213" s="7" t="n">
-        <v>5621</v>
+        <v>5042</v>
       </c>
       <c r="K213" s="8" t="n">
-        <v>244.4</v>
+        <v>219.2380952380952</v>
       </c>
     </row>
     <row r="214">
-      <c r="A214" s="6" t="inlineStr">
+      <c r="A214" s="2" t="inlineStr">
         <is>
           <t>UTHIRAMERUR</t>
         </is>
       </c>
-      <c r="B214" s="6" t="n">
+      <c r="B214" s="3" t="n">
         <v>36</v>
       </c>
-      <c r="C214" s="6" t="inlineStr">
+      <c r="C214" s="3" t="inlineStr">
         <is>
           <t>MUNIRATHINAM.J</t>
         </is>
       </c>
-      <c r="D214" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E214" s="6" t="inlineStr">
+      <c r="D214" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E214" s="3" t="inlineStr">
         <is>
           <t>SUNDAR.K</t>
         </is>
       </c>
-      <c r="F214" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G214" s="7" t="n">
-        <v>13927</v>
-      </c>
-      <c r="H214" s="6" t="inlineStr">
-        <is>
-          <t>17/23</t>
-        </is>
-      </c>
-      <c r="I214" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J214" s="7" t="n">
-        <v>18842</v>
-      </c>
-      <c r="K214" s="8" t="n">
-        <v>819.2352941176471</v>
+      <c r="F214" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G214" s="4" t="n">
+        <v>14118</v>
+      </c>
+      <c r="H214" s="3" t="inlineStr">
+        <is>
+          <t>18/23</t>
+        </is>
+      </c>
+      <c r="I214" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J214" s="4" t="n">
+        <v>18040</v>
+      </c>
+      <c r="K214" s="5" t="n">
+        <v>784.3333333333334</v>
       </c>
     </row>
     <row r="215">
@@ -11102,11 +11102,11 @@
         </is>
       </c>
       <c r="G216" s="7" t="n">
-        <v>3617</v>
+        <v>3346</v>
       </c>
       <c r="H216" s="6" t="inlineStr">
         <is>
-          <t>15/21</t>
+          <t>16/21</t>
         </is>
       </c>
       <c r="I216" s="6" t="inlineStr">
@@ -11115,59 +11115,59 @@
         </is>
       </c>
       <c r="J216" s="7" t="n">
-        <v>5064</v>
+        <v>4392</v>
       </c>
       <c r="K216" s="8" t="n">
-        <v>241.1333333333333</v>
+        <v>209.125</v>
       </c>
     </row>
     <row r="217">
-      <c r="A217" s="6" t="inlineStr">
+      <c r="A217" s="9" t="inlineStr">
         <is>
           <t>VANIYAMBADI</t>
         </is>
       </c>
-      <c r="B217" s="6" t="n">
+      <c r="B217" s="10" t="n">
         <v>47</v>
       </c>
-      <c r="C217" s="6" t="inlineStr">
+      <c r="C217" s="10" t="inlineStr">
         <is>
           <t>SYED FAROOQ BASHA SSB</t>
         </is>
       </c>
-      <c r="D217" s="6" t="inlineStr">
+      <c r="D217" s="10" t="inlineStr">
         <is>
           <t>Indian Union Muslim League</t>
         </is>
       </c>
-      <c r="E217" s="6" t="inlineStr">
+      <c r="E217" s="10" t="inlineStr">
         <is>
           <t>SYED BHURHANUDEEN</t>
         </is>
       </c>
-      <c r="F217" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G217" s="7" t="n">
-        <v>3069</v>
-      </c>
-      <c r="H217" s="6" t="inlineStr">
-        <is>
-          <t>22/23</t>
-        </is>
-      </c>
-      <c r="I217" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J217" s="7" t="n">
-        <v>3208</v>
-      </c>
-      <c r="K217" s="8" t="n">
-        <v>139.5</v>
+      <c r="F217" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G217" s="11" t="n">
+        <v>2572</v>
+      </c>
+      <c r="H217" s="10" t="inlineStr">
+        <is>
+          <t>23/24</t>
+        </is>
+      </c>
+      <c r="I217" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J217" s="11" t="n">
+        <v>2684</v>
+      </c>
+      <c r="K217" s="12" t="n">
+        <v>111.8260869565217</v>
       </c>
     </row>
     <row r="218">
@@ -11200,11 +11200,11 @@
         </is>
       </c>
       <c r="G218" s="7" t="n">
-        <v>3645</v>
+        <v>3884</v>
       </c>
       <c r="H218" s="6" t="inlineStr">
         <is>
-          <t>14/22</t>
+          <t>15/22</t>
         </is>
       </c>
       <c r="I218" s="6" t="inlineStr">
@@ -11213,10 +11213,10 @@
         </is>
       </c>
       <c r="J218" s="7" t="n">
-        <v>5728</v>
+        <v>5697</v>
       </c>
       <c r="K218" s="8" t="n">
-        <v>260.3571428571428</v>
+        <v>258.9333333333333</v>
       </c>
     </row>
     <row r="219">
@@ -11249,11 +11249,11 @@
         </is>
       </c>
       <c r="G219" s="7" t="n">
-        <v>6198</v>
+        <v>6449</v>
       </c>
       <c r="H219" s="6" t="inlineStr">
         <is>
-          <t>15/23</t>
+          <t>16/23</t>
         </is>
       </c>
       <c r="I219" s="6" t="inlineStr">
@@ -11262,10 +11262,10 @@
         </is>
       </c>
       <c r="J219" s="7" t="n">
-        <v>9504</v>
+        <v>9270</v>
       </c>
       <c r="K219" s="8" t="n">
-        <v>413.2</v>
+        <v>403.0625</v>
       </c>
     </row>
     <row r="220">
@@ -11445,11 +11445,11 @@
         </is>
       </c>
       <c r="G223" s="4" t="n">
-        <v>26684</v>
+        <v>27350</v>
       </c>
       <c r="H223" s="3" t="inlineStr">
         <is>
-          <t>17/23</t>
+          <t>18/23</t>
         </is>
       </c>
       <c r="I223" s="3" t="inlineStr">
@@ -11458,10 +11458,10 @@
         </is>
       </c>
       <c r="J223" s="4" t="n">
-        <v>36102</v>
+        <v>34947</v>
       </c>
       <c r="K223" s="5" t="n">
-        <v>1569.64705882353</v>
+        <v>1519.444444444444</v>
       </c>
     </row>
     <row r="224">
@@ -11494,11 +11494,11 @@
         </is>
       </c>
       <c r="G224" s="7" t="n">
-        <v>2395</v>
+        <v>3229</v>
       </c>
       <c r="H224" s="6" t="inlineStr">
         <is>
-          <t>15/20</t>
+          <t>16/20</t>
         </is>
       </c>
       <c r="I224" s="6" t="inlineStr">
@@ -11507,108 +11507,108 @@
         </is>
       </c>
       <c r="J224" s="7" t="n">
-        <v>3193</v>
+        <v>4036</v>
       </c>
       <c r="K224" s="8" t="n">
-        <v>159.6666666666667</v>
+        <v>201.8125</v>
       </c>
     </row>
     <row r="225">
-      <c r="A225" s="9" t="inlineStr">
+      <c r="A225" s="13" t="inlineStr">
         <is>
           <t>VEPPANAHALLI</t>
         </is>
       </c>
-      <c r="B225" s="10" t="n">
+      <c r="B225" s="14" t="n">
         <v>54</v>
       </c>
-      <c r="C225" s="10" t="inlineStr">
+      <c r="C225" s="14" t="inlineStr">
         <is>
           <t>SRINIVASAN.P.S</t>
         </is>
       </c>
-      <c r="D225" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E225" s="10" t="inlineStr">
+      <c r="D225" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E225" s="14" t="inlineStr">
         <is>
           <t>MUNUSAMY.K.P</t>
         </is>
       </c>
-      <c r="F225" s="10" t="inlineStr">
+      <c r="F225" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G225" s="11" t="n">
-        <v>361</v>
-      </c>
-      <c r="H225" s="10" t="inlineStr">
-        <is>
-          <t>18/25</t>
-        </is>
-      </c>
-      <c r="I225" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J225" s="11" t="n">
-        <v>501</v>
-      </c>
-      <c r="K225" s="12" t="n">
-        <v>20.05555555555556</v>
+      <c r="G225" s="15" t="n">
+        <v>333</v>
+      </c>
+      <c r="H225" s="14" t="inlineStr">
+        <is>
+          <t>19/25</t>
+        </is>
+      </c>
+      <c r="I225" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J225" s="15" t="n">
+        <v>438</v>
+      </c>
+      <c r="K225" s="16" t="n">
+        <v>17.52631578947368</v>
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="13" t="inlineStr">
+      <c r="A226" s="9" t="inlineStr">
         <is>
           <t>VIKRAVANDI</t>
         </is>
       </c>
-      <c r="B226" s="14" t="n">
+      <c r="B226" s="10" t="n">
         <v>75</v>
       </c>
-      <c r="C226" s="14" t="inlineStr">
+      <c r="C226" s="10" t="inlineStr">
+        <is>
+          <t>SIVAKUMAR C</t>
+        </is>
+      </c>
+      <c r="D226" s="10" t="inlineStr">
+        <is>
+          <t>Pattali Makkal Katchi</t>
+        </is>
+      </c>
+      <c r="E226" s="10" t="inlineStr">
         <is>
           <t>VIJAI VADIVEL A</t>
         </is>
       </c>
-      <c r="D226" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E226" s="14" t="inlineStr">
-        <is>
-          <t>SIVAKUMAR C</t>
-        </is>
-      </c>
-      <c r="F226" s="14" t="inlineStr">
-        <is>
-          <t>Pattali Makkal Katchi</t>
-        </is>
-      </c>
-      <c r="G226" s="15" t="n">
-        <v>169</v>
-      </c>
-      <c r="H226" s="14" t="inlineStr">
-        <is>
-          <t>9/23</t>
-        </is>
-      </c>
-      <c r="I226" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J226" s="15" t="n">
-        <v>432</v>
-      </c>
-      <c r="K226" s="16" t="n">
-        <v>18.77777777777778</v>
+      <c r="F226" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G226" s="11" t="n">
+        <v>730</v>
+      </c>
+      <c r="H226" s="10" t="inlineStr">
+        <is>
+          <t>10/23</t>
+        </is>
+      </c>
+      <c r="I226" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J226" s="11" t="n">
+        <v>1679</v>
+      </c>
+      <c r="K226" s="12" t="n">
+        <v>73</v>
       </c>
     </row>
     <row r="227">
@@ -11641,11 +11641,11 @@
         </is>
       </c>
       <c r="G227" s="4" t="n">
-        <v>6909</v>
+        <v>7697</v>
       </c>
       <c r="H227" s="3" t="inlineStr">
         <is>
-          <t>17/20</t>
+          <t>18/20</t>
         </is>
       </c>
       <c r="I227" s="3" t="inlineStr">
@@ -11654,10 +11654,10 @@
         </is>
       </c>
       <c r="J227" s="4" t="n">
-        <v>8128</v>
+        <v>8552</v>
       </c>
       <c r="K227" s="5" t="n">
-        <v>406.4117647058824</v>
+        <v>427.6111111111111</v>
       </c>
     </row>
     <row r="228">
@@ -11690,11 +11690,11 @@
         </is>
       </c>
       <c r="G228" s="4" t="n">
-        <v>15814</v>
+        <v>16292</v>
       </c>
       <c r="H228" s="3" t="inlineStr">
         <is>
-          <t>14/22</t>
+          <t>15/22</t>
         </is>
       </c>
       <c r="I228" s="3" t="inlineStr">
@@ -11703,10 +11703,10 @@
         </is>
       </c>
       <c r="J228" s="4" t="n">
-        <v>24851</v>
+        <v>23895</v>
       </c>
       <c r="K228" s="5" t="n">
-        <v>1129.571428571429</v>
+        <v>1086.133333333333</v>
       </c>
     </row>
     <row r="229">
@@ -11788,11 +11788,11 @@
         </is>
       </c>
       <c r="G230" s="11" t="n">
-        <v>1745</v>
+        <v>1491</v>
       </c>
       <c r="H230" s="10" t="inlineStr">
         <is>
-          <t>17/24</t>
+          <t>18/24</t>
         </is>
       </c>
       <c r="I230" s="10" t="inlineStr">
@@ -11801,10 +11801,10 @@
         </is>
       </c>
       <c r="J230" s="11" t="n">
-        <v>2464</v>
+        <v>1988</v>
       </c>
       <c r="K230" s="12" t="n">
-        <v>102.6470588235294</v>
+        <v>82.83333333333333</v>
       </c>
     </row>
     <row r="231">
@@ -11837,11 +11837,11 @@
         </is>
       </c>
       <c r="G231" s="4" t="n">
-        <v>37214</v>
+        <v>40612</v>
       </c>
       <c r="H231" s="3" t="inlineStr">
         <is>
-          <t>12/20</t>
+          <t>13/20</t>
         </is>
       </c>
       <c r="I231" s="3" t="inlineStr">
@@ -11850,10 +11850,10 @@
         </is>
       </c>
       <c r="J231" s="4" t="n">
-        <v>62023</v>
+        <v>62480</v>
       </c>
       <c r="K231" s="5" t="n">
-        <v>3101.166666666667</v>
+        <v>3124</v>
       </c>
     </row>
     <row r="232">
@@ -11935,11 +11935,11 @@
         </is>
       </c>
       <c r="G233" s="4" t="n">
-        <v>12406</v>
+        <v>14433</v>
       </c>
       <c r="H233" s="3" t="inlineStr">
         <is>
-          <t>12/23</t>
+          <t>13/23</t>
         </is>
       </c>
       <c r="I233" s="3" t="inlineStr">
@@ -11948,10 +11948,10 @@
         </is>
       </c>
       <c r="J233" s="4" t="n">
-        <v>23778</v>
+        <v>25535</v>
       </c>
       <c r="K233" s="5" t="n">
-        <v>1033.833333333333</v>
+        <v>1110.230769230769</v>
       </c>
     </row>
     <row r="234">
@@ -12004,52 +12004,52 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="6" t="inlineStr">
+      <c r="A235" s="9" t="inlineStr">
         <is>
           <t>YERCAUD</t>
         </is>
       </c>
-      <c r="B235" s="6" t="n">
+      <c r="B235" s="10" t="n">
         <v>83</v>
       </c>
-      <c r="C235" s="6" t="inlineStr">
+      <c r="C235" s="10" t="inlineStr">
         <is>
           <t>LAKSHMI JANARTHANAN. J</t>
         </is>
       </c>
-      <c r="D235" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E235" s="6" t="inlineStr">
+      <c r="D235" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E235" s="10" t="inlineStr">
         <is>
           <t>USHARANI. P</t>
         </is>
       </c>
-      <c r="F235" s="6" t="inlineStr">
+      <c r="F235" s="10" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G235" s="7" t="n">
-        <v>1558</v>
-      </c>
-      <c r="H235" s="6" t="inlineStr">
-        <is>
-          <t>12/24</t>
-        </is>
-      </c>
-      <c r="I235" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J235" s="7" t="n">
-        <v>3116</v>
-      </c>
-      <c r="K235" s="8" t="n">
-        <v>129.8333333333333</v>
+      <c r="G235" s="11" t="n">
+        <v>1480</v>
+      </c>
+      <c r="H235" s="10" t="inlineStr">
+        <is>
+          <t>13/24</t>
+        </is>
+      </c>
+      <c r="I235" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J235" s="11" t="n">
+        <v>2732</v>
+      </c>
+      <c r="K235" s="12" t="n">
+        <v>113.8461538461538</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update election results snapshot (71.5% counted)
TVK 109, DMK 56, AIADMK 47. NILAKKOTTAI still at 16-vote TVK lead.
SRIVAIKUNTAM AIADMK last round pending. 7 knife-edge, 6 declared total.

https://claude.ai/code/session_01MizbUy44JG5sXyvaf3Wekb
</commit_message>
<xml_diff>
--- a/tn_election_results_may2026.xlsx
+++ b/tn_election_results_may2026.xlsx
@@ -616,11 +616,11 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>18967</v>
+        <v>20291</v>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>13/31</t>
+          <t>14/31</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -629,10 +629,10 @@
         </is>
       </c>
       <c r="J2" s="4" t="n">
-        <v>45229</v>
+        <v>44930</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>1459</v>
+        <v>1449.357142857143</v>
       </c>
     </row>
     <row r="3">
@@ -665,11 +665,11 @@
         </is>
       </c>
       <c r="G3" s="7" t="n">
-        <v>4796</v>
+        <v>5727</v>
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
-          <t>10/20</t>
+          <t>11/20</t>
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr">
@@ -678,59 +678,59 @@
         </is>
       </c>
       <c r="J3" s="7" t="n">
-        <v>9592</v>
+        <v>10413</v>
       </c>
       <c r="K3" s="8" t="n">
-        <v>479.6</v>
+        <v>520.6363636363636</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>ALANGULAM</t>
         </is>
       </c>
-      <c r="B4" s="6" t="n">
+      <c r="B4" s="3" t="n">
         <v>223</v>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>PAUL MANOJ PANDIAN</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>K R P PRABAKARAN</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G4" s="7" t="n">
-        <v>4300</v>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>19/24</t>
-        </is>
-      </c>
-      <c r="I4" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J4" s="7" t="n">
-        <v>5432</v>
-      </c>
-      <c r="K4" s="8" t="n">
-        <v>226.3157894736842</v>
+      <c r="G4" s="4" t="n">
+        <v>6654</v>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>20/24</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>7985</v>
+      </c>
+      <c r="K4" s="5" t="n">
+        <v>332.7</v>
       </c>
     </row>
     <row r="5">
@@ -812,11 +812,11 @@
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>40258</v>
+        <v>43424</v>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>17/27</t>
+          <t>18/27</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -825,10 +825,10 @@
         </is>
       </c>
       <c r="J6" s="4" t="n">
-        <v>63939</v>
+        <v>65136</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>2368.117647058823</v>
+        <v>2412.444444444444</v>
       </c>
     </row>
     <row r="7">
@@ -959,11 +959,11 @@
         </is>
       </c>
       <c r="G9" s="7" t="n">
-        <v>2398</v>
+        <v>3571</v>
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>16/25</t>
+          <t>17/25</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
@@ -972,10 +972,10 @@
         </is>
       </c>
       <c r="J9" s="7" t="n">
-        <v>3747</v>
+        <v>5251</v>
       </c>
       <c r="K9" s="8" t="n">
-        <v>149.875</v>
+        <v>210.0588235294118</v>
       </c>
     </row>
     <row r="10">
@@ -1155,11 +1155,11 @@
         </is>
       </c>
       <c r="G13" s="7" t="n">
-        <v>3291</v>
+        <v>4020</v>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>20/24</t>
+          <t>21/24</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
@@ -1168,10 +1168,10 @@
         </is>
       </c>
       <c r="J13" s="7" t="n">
-        <v>3949</v>
+        <v>4594</v>
       </c>
       <c r="K13" s="8" t="n">
-        <v>164.55</v>
+        <v>191.4285714285714</v>
       </c>
     </row>
     <row r="14">
@@ -1204,11 +1204,11 @@
         </is>
       </c>
       <c r="G14" s="4" t="n">
-        <v>12301</v>
+        <v>12730</v>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>17/22</t>
+          <t>18/22</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
@@ -1217,10 +1217,10 @@
         </is>
       </c>
       <c r="J14" s="4" t="n">
-        <v>15919</v>
+        <v>15559</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>723.5882352941177</v>
+        <v>707.2222222222222</v>
       </c>
     </row>
     <row r="15">
@@ -1351,11 +1351,11 @@
         </is>
       </c>
       <c r="G17" s="4" t="n">
-        <v>17842</v>
+        <v>22502</v>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>21/24</t>
+          <t>23/25</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -1364,10 +1364,10 @@
         </is>
       </c>
       <c r="J17" s="4" t="n">
-        <v>20391</v>
+        <v>24459</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>849.6190476190476</v>
+        <v>978.3478260869565</v>
       </c>
     </row>
     <row r="18">
@@ -1400,11 +1400,11 @@
         </is>
       </c>
       <c r="G18" s="7" t="n">
-        <v>3083</v>
+        <v>2479</v>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>13/20</t>
+          <t>14/20</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr">
@@ -1413,10 +1413,10 @@
         </is>
       </c>
       <c r="J18" s="7" t="n">
-        <v>4743</v>
+        <v>3541</v>
       </c>
       <c r="K18" s="8" t="n">
-        <v>237.1538461538462</v>
+        <v>177.0714285714286</v>
       </c>
     </row>
     <row r="19">
@@ -1449,11 +1449,11 @@
         </is>
       </c>
       <c r="G19" s="4" t="n">
-        <v>18038</v>
+        <v>20123</v>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>16/25</t>
+          <t>17/25</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -1462,10 +1462,10 @@
         </is>
       </c>
       <c r="J19" s="4" t="n">
-        <v>28184</v>
+        <v>29593</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>1127.375</v>
+        <v>1183.705882352941</v>
       </c>
     </row>
     <row r="20">
@@ -1498,11 +1498,11 @@
         </is>
       </c>
       <c r="G20" s="4" t="n">
-        <v>12052</v>
+        <v>13481</v>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>19/22</t>
+          <t>20/22</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
@@ -1511,10 +1511,10 @@
         </is>
       </c>
       <c r="J20" s="4" t="n">
-        <v>13955</v>
+        <v>14829</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>634.3157894736842</v>
+        <v>674.05</v>
       </c>
     </row>
     <row r="21">
@@ -1714,52 +1714,52 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="inlineStr">
+      <c r="A25" s="9" t="inlineStr">
         <is>
           <t>BHAVANISAGAR</t>
         </is>
       </c>
-      <c r="B25" s="14" t="n">
+      <c r="B25" s="10" t="n">
         <v>107</v>
       </c>
-      <c r="C25" s="14" t="inlineStr">
+      <c r="C25" s="10" t="inlineStr">
         <is>
           <t>V.P.TAMILSELVI</t>
         </is>
       </c>
-      <c r="D25" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E25" s="14" t="inlineStr">
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="inlineStr">
         <is>
           <t>A.BANNARI</t>
         </is>
       </c>
-      <c r="F25" s="14" t="inlineStr">
+      <c r="F25" s="10" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G25" s="15" t="n">
-        <v>205</v>
-      </c>
-      <c r="H25" s="14" t="inlineStr">
-        <is>
-          <t>18/24</t>
-        </is>
-      </c>
-      <c r="I25" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J25" s="15" t="n">
-        <v>273</v>
-      </c>
-      <c r="K25" s="16" t="n">
-        <v>11.38888888888889</v>
+      <c r="G25" s="11" t="n">
+        <v>1195</v>
+      </c>
+      <c r="H25" s="10" t="inlineStr">
+        <is>
+          <t>19/24</t>
+        </is>
+      </c>
+      <c r="I25" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J25" s="11" t="n">
+        <v>1509</v>
+      </c>
+      <c r="K25" s="12" t="n">
+        <v>62.89473684210526</v>
       </c>
     </row>
     <row r="26">
@@ -1841,11 +1841,11 @@
         </is>
       </c>
       <c r="G27" s="7" t="n">
-        <v>4213</v>
+        <v>4502</v>
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>15/25</t>
+          <t>16/25</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
@@ -1854,10 +1854,10 @@
         </is>
       </c>
       <c r="J27" s="7" t="n">
-        <v>7022</v>
+        <v>7034</v>
       </c>
       <c r="K27" s="8" t="n">
-        <v>280.8666666666667</v>
+        <v>281.375</v>
       </c>
     </row>
     <row r="28">
@@ -1890,11 +1890,11 @@
         </is>
       </c>
       <c r="G28" s="4" t="n">
-        <v>15383</v>
+        <v>15321</v>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>13/36</t>
+          <t>14/36</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
@@ -1903,10 +1903,10 @@
         </is>
       </c>
       <c r="J28" s="4" t="n">
-        <v>42599</v>
+        <v>39397</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>1183.307692307692</v>
+        <v>1094.357142857143</v>
       </c>
     </row>
     <row r="29">
@@ -1939,11 +1939,11 @@
         </is>
       </c>
       <c r="G29" s="7" t="n">
-        <v>6585</v>
+        <v>7659</v>
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>12/25</t>
+          <t>13/25</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
@@ -1952,59 +1952,59 @@
         </is>
       </c>
       <c r="J29" s="7" t="n">
-        <v>13719</v>
+        <v>14729</v>
       </c>
       <c r="K29" s="8" t="n">
-        <v>548.75</v>
+        <v>589.1538461538462</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>CHEPAUK-THIRUVALLIKENI</t>
         </is>
       </c>
-      <c r="B30" s="6" t="n">
+      <c r="B30" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="C30" s="6" t="inlineStr">
+      <c r="C30" s="3" t="inlineStr">
         <is>
           <t>UDHAYANIDHI STALIN</t>
         </is>
       </c>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="inlineStr">
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
         <is>
           <t>SELVAM. D</t>
         </is>
       </c>
-      <c r="F30" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G30" s="7" t="n">
-        <v>6118</v>
-      </c>
-      <c r="H30" s="6" t="inlineStr">
-        <is>
-          <t>12/17</t>
-        </is>
-      </c>
-      <c r="I30" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J30" s="7" t="n">
-        <v>8667</v>
-      </c>
-      <c r="K30" s="8" t="n">
-        <v>509.8333333333333</v>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="n">
+        <v>9881</v>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>13/17</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J30" s="4" t="n">
+        <v>12921</v>
+      </c>
+      <c r="K30" s="5" t="n">
+        <v>760.0769230769231</v>
       </c>
     </row>
     <row r="31">
@@ -2233,11 +2233,11 @@
         </is>
       </c>
       <c r="G35" s="11" t="n">
-        <v>1198</v>
+        <v>1231</v>
       </c>
       <c r="H35" s="10" t="inlineStr">
         <is>
-          <t>11/20</t>
+          <t>12/20</t>
         </is>
       </c>
       <c r="I35" s="10" t="inlineStr">
@@ -2246,10 +2246,10 @@
         </is>
       </c>
       <c r="J35" s="11" t="n">
-        <v>2178</v>
+        <v>2052</v>
       </c>
       <c r="K35" s="12" t="n">
-        <v>108.9090909090909</v>
+        <v>102.5833333333333</v>
       </c>
     </row>
     <row r="36">
@@ -2282,11 +2282,11 @@
         </is>
       </c>
       <c r="G36" s="7" t="n">
-        <v>6403</v>
+        <v>4409</v>
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>12/23</t>
+          <t>13/23</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
@@ -2295,10 +2295,10 @@
         </is>
       </c>
       <c r="J36" s="7" t="n">
-        <v>12272</v>
+        <v>7801</v>
       </c>
       <c r="K36" s="8" t="n">
-        <v>533.5833333333334</v>
+        <v>339.1538461538462</v>
       </c>
     </row>
     <row r="37">
@@ -2527,11 +2527,11 @@
         </is>
       </c>
       <c r="G41" s="4" t="n">
-        <v>16090</v>
+        <v>17366</v>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>20/23</t>
+          <t>21/23</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
@@ -2540,10 +2540,10 @@
         </is>
       </c>
       <c r="J41" s="4" t="n">
-        <v>18504</v>
+        <v>19020</v>
       </c>
       <c r="K41" s="5" t="n">
-        <v>804.5</v>
+        <v>826.952380952381</v>
       </c>
     </row>
     <row r="42">
@@ -2674,11 +2674,11 @@
         </is>
       </c>
       <c r="G44" s="4" t="n">
-        <v>86286</v>
+        <v>90278</v>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>22/25</t>
+          <t>23/25</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
@@ -2687,10 +2687,10 @@
         </is>
       </c>
       <c r="J44" s="4" t="n">
-        <v>98052</v>
+        <v>98128</v>
       </c>
       <c r="K44" s="5" t="n">
-        <v>3922.090909090909</v>
+        <v>3925.130434782609</v>
       </c>
     </row>
     <row r="45">
@@ -2723,7 +2723,7 @@
         </is>
       </c>
       <c r="G45" s="4" t="n">
-        <v>13084</v>
+        <v>13096</v>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
@@ -2736,10 +2736,10 @@
         </is>
       </c>
       <c r="J45" s="4" t="n">
-        <v>15097</v>
+        <v>15111</v>
       </c>
       <c r="K45" s="5" t="n">
-        <v>1006.461538461538</v>
+        <v>1007.384615384615</v>
       </c>
     </row>
     <row r="46">
@@ -2772,11 +2772,11 @@
         </is>
       </c>
       <c r="G46" s="4" t="n">
-        <v>22362</v>
+        <v>23372</v>
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>17/19</t>
+          <t>18/20</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
@@ -2785,10 +2785,10 @@
         </is>
       </c>
       <c r="J46" s="4" t="n">
-        <v>24993</v>
+        <v>25969</v>
       </c>
       <c r="K46" s="5" t="n">
-        <v>1315.411764705882</v>
+        <v>1298.444444444444</v>
       </c>
     </row>
     <row r="47">
@@ -2821,11 +2821,11 @@
         </is>
       </c>
       <c r="G47" s="4" t="n">
-        <v>19123</v>
+        <v>20799</v>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>15/24</t>
+          <t>16/24</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
@@ -2834,10 +2834,10 @@
         </is>
       </c>
       <c r="J47" s="4" t="n">
-        <v>30597</v>
+        <v>31198</v>
       </c>
       <c r="K47" s="5" t="n">
-        <v>1274.866666666667</v>
+        <v>1299.9375</v>
       </c>
     </row>
     <row r="48">
@@ -2870,11 +2870,11 @@
         </is>
       </c>
       <c r="G48" s="7" t="n">
-        <v>6344</v>
+        <v>7531</v>
       </c>
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>10/18</t>
+          <t>11/18</t>
         </is>
       </c>
       <c r="I48" s="6" t="inlineStr">
@@ -2883,10 +2883,10 @@
         </is>
       </c>
       <c r="J48" s="7" t="n">
-        <v>11419</v>
+        <v>12323</v>
       </c>
       <c r="K48" s="8" t="n">
-        <v>634.4</v>
+        <v>684.6363636363636</v>
       </c>
     </row>
     <row r="49">
@@ -2968,11 +2968,11 @@
         </is>
       </c>
       <c r="G50" s="7" t="n">
-        <v>6363</v>
+        <v>8430</v>
       </c>
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>9/23</t>
+          <t>10/23</t>
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr">
@@ -2981,10 +2981,10 @@
         </is>
       </c>
       <c r="J50" s="7" t="n">
-        <v>16261</v>
+        <v>19389</v>
       </c>
       <c r="K50" s="8" t="n">
-        <v>707</v>
+        <v>843</v>
       </c>
     </row>
     <row r="51">
@@ -3017,11 +3017,11 @@
         </is>
       </c>
       <c r="G51" s="4" t="n">
-        <v>16494</v>
+        <v>16620</v>
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>21/23</t>
+          <t>23/23</t>
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr">
@@ -3030,10 +3030,10 @@
         </is>
       </c>
       <c r="J51" s="4" t="n">
-        <v>18065</v>
+        <v>16620</v>
       </c>
       <c r="K51" s="5" t="n">
-        <v>785.4285714285714</v>
+        <v>722.6086956521739</v>
       </c>
     </row>
     <row r="52">
@@ -3086,52 +3086,52 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="9" t="inlineStr">
+      <c r="A53" s="6" t="inlineStr">
         <is>
           <t>GUDIYATTAM</t>
         </is>
       </c>
-      <c r="B53" s="10" t="n">
+      <c r="B53" s="6" t="n">
         <v>46</v>
       </c>
-      <c r="C53" s="10" t="inlineStr">
+      <c r="C53" s="6" t="inlineStr">
         <is>
           <t>K.SINDU</t>
         </is>
       </c>
-      <c r="D53" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E53" s="10" t="inlineStr">
+      <c r="D53" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E53" s="6" t="inlineStr">
         <is>
           <t>K.B.PRADAP</t>
         </is>
       </c>
-      <c r="F53" s="10" t="inlineStr">
+      <c r="F53" s="6" t="inlineStr">
         <is>
           <t>Desiya Murpokku Dravida Kazhagam</t>
         </is>
       </c>
-      <c r="G53" s="11" t="n">
-        <v>1682</v>
-      </c>
-      <c r="H53" s="10" t="inlineStr">
-        <is>
-          <t>16/23</t>
-        </is>
-      </c>
-      <c r="I53" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J53" s="11" t="n">
-        <v>2418</v>
-      </c>
-      <c r="K53" s="12" t="n">
-        <v>105.125</v>
+      <c r="G53" s="7" t="n">
+        <v>2770</v>
+      </c>
+      <c r="H53" s="6" t="inlineStr">
+        <is>
+          <t>17/23</t>
+        </is>
+      </c>
+      <c r="I53" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J53" s="7" t="n">
+        <v>3748</v>
+      </c>
+      <c r="K53" s="8" t="n">
+        <v>162.9411764705882</v>
       </c>
     </row>
     <row r="54">
@@ -3213,11 +3213,11 @@
         </is>
       </c>
       <c r="G55" s="4" t="n">
-        <v>10318</v>
+        <v>10639</v>
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>11/14</t>
+          <t>12/14</t>
         </is>
       </c>
       <c r="I55" s="3" t="inlineStr">
@@ -3226,10 +3226,10 @@
         </is>
       </c>
       <c r="J55" s="4" t="n">
-        <v>13132</v>
+        <v>12412</v>
       </c>
       <c r="K55" s="5" t="n">
-        <v>938</v>
+        <v>886.5833333333334</v>
       </c>
     </row>
     <row r="56">
@@ -3311,11 +3311,11 @@
         </is>
       </c>
       <c r="G57" s="4" t="n">
-        <v>24278</v>
+        <v>24038</v>
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>17/34</t>
+          <t>18/34</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr">
@@ -3324,59 +3324,59 @@
         </is>
       </c>
       <c r="J57" s="4" t="n">
-        <v>48556</v>
+        <v>45405</v>
       </c>
       <c r="K57" s="5" t="n">
-        <v>1428.117647058823</v>
+        <v>1335.444444444444</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="6" t="inlineStr">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>JAYANKONDAM</t>
         </is>
       </c>
-      <c r="B58" s="6" t="n">
+      <c r="B58" s="3" t="n">
         <v>150</v>
       </c>
-      <c r="C58" s="6" t="inlineStr">
+      <c r="C58" s="3" t="inlineStr">
         <is>
           <t>VAITHILINGAM G.</t>
         </is>
       </c>
-      <c r="D58" s="6" t="inlineStr">
+      <c r="D58" s="3" t="inlineStr">
         <is>
           <t>Pattali Makkal Katchi</t>
         </is>
       </c>
-      <c r="E58" s="6" t="inlineStr">
+      <c r="E58" s="3" t="inlineStr">
         <is>
           <t>KANNAN KA.SO.KA.</t>
         </is>
       </c>
-      <c r="F58" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G58" s="7" t="n">
-        <v>10939</v>
-      </c>
-      <c r="H58" s="6" t="inlineStr">
-        <is>
-          <t>17/23</t>
-        </is>
-      </c>
-      <c r="I58" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J58" s="7" t="n">
-        <v>14800</v>
-      </c>
-      <c r="K58" s="8" t="n">
-        <v>643.4705882352941</v>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G58" s="4" t="n">
+        <v>10651</v>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>18/23</t>
+        </is>
+      </c>
+      <c r="I58" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J58" s="4" t="n">
+        <v>13610</v>
+      </c>
+      <c r="K58" s="5" t="n">
+        <v>591.7222222222222</v>
       </c>
     </row>
     <row r="59">
@@ -3605,11 +3605,11 @@
         </is>
       </c>
       <c r="G63" s="7" t="n">
-        <v>6289</v>
+        <v>7578</v>
       </c>
       <c r="H63" s="6" t="inlineStr">
         <is>
-          <t>14/26</t>
+          <t>15/26</t>
         </is>
       </c>
       <c r="I63" s="6" t="inlineStr">
@@ -3618,10 +3618,10 @@
         </is>
       </c>
       <c r="J63" s="7" t="n">
-        <v>11680</v>
+        <v>13135</v>
       </c>
       <c r="K63" s="8" t="n">
-        <v>449.2142857142857</v>
+        <v>505.2</v>
       </c>
     </row>
     <row r="64">
@@ -3654,11 +3654,11 @@
         </is>
       </c>
       <c r="G64" s="7" t="n">
-        <v>5199</v>
+        <v>6410</v>
       </c>
       <c r="H64" s="6" t="inlineStr">
         <is>
-          <t>15/23</t>
+          <t>16/23</t>
         </is>
       </c>
       <c r="I64" s="6" t="inlineStr">
@@ -3667,10 +3667,10 @@
         </is>
       </c>
       <c r="J64" s="7" t="n">
-        <v>7972</v>
+        <v>9214</v>
       </c>
       <c r="K64" s="8" t="n">
-        <v>346.6</v>
+        <v>400.625</v>
       </c>
     </row>
     <row r="65">
@@ -3703,11 +3703,11 @@
         </is>
       </c>
       <c r="G65" s="7" t="n">
-        <v>5180</v>
+        <v>4989</v>
       </c>
       <c r="H65" s="6" t="inlineStr">
         <is>
-          <t>15/26</t>
+          <t>16/26</t>
         </is>
       </c>
       <c r="I65" s="6" t="inlineStr">
@@ -3716,10 +3716,10 @@
         </is>
       </c>
       <c r="J65" s="7" t="n">
-        <v>8979</v>
+        <v>8107</v>
       </c>
       <c r="K65" s="8" t="n">
-        <v>345.3333333333334</v>
+        <v>311.8125</v>
       </c>
     </row>
     <row r="66">
@@ -3752,11 +3752,11 @@
         </is>
       </c>
       <c r="G66" s="4" t="n">
-        <v>24684</v>
+        <v>26481</v>
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>14/28</t>
+          <t>15/28</t>
         </is>
       </c>
       <c r="I66" s="3" t="inlineStr">
@@ -3765,10 +3765,10 @@
         </is>
       </c>
       <c r="J66" s="4" t="n">
-        <v>49368</v>
+        <v>49431</v>
       </c>
       <c r="K66" s="5" t="n">
-        <v>1763.142857142857</v>
+        <v>1765.4</v>
       </c>
     </row>
     <row r="67">
@@ -3801,11 +3801,11 @@
         </is>
       </c>
       <c r="G67" s="7" t="n">
-        <v>5280</v>
+        <v>5447</v>
       </c>
       <c r="H67" s="6" t="inlineStr">
         <is>
-          <t>12/21</t>
+          <t>13/21</t>
         </is>
       </c>
       <c r="I67" s="6" t="inlineStr">
@@ -3814,10 +3814,10 @@
         </is>
       </c>
       <c r="J67" s="7" t="n">
-        <v>9240</v>
+        <v>8799</v>
       </c>
       <c r="K67" s="8" t="n">
-        <v>440</v>
+        <v>419</v>
       </c>
     </row>
     <row r="68">
@@ -3948,11 +3948,11 @@
         </is>
       </c>
       <c r="G70" s="4" t="n">
-        <v>41243</v>
+        <v>41613</v>
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>25/28</t>
+          <t>26/28</t>
         </is>
       </c>
       <c r="I70" s="3" t="inlineStr">
@@ -3961,10 +3961,10 @@
         </is>
       </c>
       <c r="J70" s="4" t="n">
-        <v>46192</v>
+        <v>44814</v>
       </c>
       <c r="K70" s="5" t="n">
-        <v>1649.72</v>
+        <v>1600.5</v>
       </c>
     </row>
     <row r="71">
@@ -4193,7 +4193,7 @@
         </is>
       </c>
       <c r="G75" s="4" t="n">
-        <v>13039</v>
+        <v>12635</v>
       </c>
       <c r="H75" s="3" t="inlineStr">
         <is>
@@ -4206,10 +4206,10 @@
         </is>
       </c>
       <c r="J75" s="4" t="n">
-        <v>14042</v>
+        <v>13607</v>
       </c>
       <c r="K75" s="5" t="n">
-        <v>501.5</v>
+        <v>485.9615384615385</v>
       </c>
     </row>
     <row r="76">
@@ -4242,11 +4242,11 @@
         </is>
       </c>
       <c r="G76" s="4" t="n">
-        <v>7731</v>
+        <v>8539</v>
       </c>
       <c r="H76" s="3" t="inlineStr">
         <is>
-          <t>17/22</t>
+          <t>18/22</t>
         </is>
       </c>
       <c r="I76" s="3" t="inlineStr">
@@ -4255,10 +4255,10 @@
         </is>
       </c>
       <c r="J76" s="4" t="n">
-        <v>10005</v>
+        <v>10437</v>
       </c>
       <c r="K76" s="5" t="n">
-        <v>454.7647058823529</v>
+        <v>474.3888888888889</v>
       </c>
     </row>
     <row r="77">
@@ -4409,52 +4409,52 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="6" t="inlineStr">
+      <c r="A80" s="9" t="inlineStr">
         <is>
           <t>KULITHALAI</t>
         </is>
       </c>
-      <c r="B80" s="6" t="n">
+      <c r="B80" s="10" t="n">
         <v>137</v>
       </c>
-      <c r="C80" s="6" t="inlineStr">
+      <c r="C80" s="10" t="inlineStr">
         <is>
           <t>G.BALASUBRAMANI</t>
         </is>
       </c>
-      <c r="D80" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E80" s="6" t="inlineStr">
+      <c r="D80" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E80" s="10" t="inlineStr">
         <is>
           <t>SURIYANUR. A. CHANDRAN</t>
         </is>
       </c>
-      <c r="F80" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G80" s="7" t="n">
-        <v>2207</v>
-      </c>
-      <c r="H80" s="6" t="inlineStr">
-        <is>
-          <t>15/21</t>
-        </is>
-      </c>
-      <c r="I80" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J80" s="7" t="n">
-        <v>3090</v>
-      </c>
-      <c r="K80" s="8" t="n">
-        <v>147.1333333333333</v>
+      <c r="F80" s="10" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G80" s="11" t="n">
+        <v>1748</v>
+      </c>
+      <c r="H80" s="10" t="inlineStr">
+        <is>
+          <t>16/21</t>
+        </is>
+      </c>
+      <c r="I80" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J80" s="11" t="n">
+        <v>2294</v>
+      </c>
+      <c r="K80" s="12" t="n">
+        <v>109.25</v>
       </c>
     </row>
     <row r="81">
@@ -4487,11 +4487,11 @@
         </is>
       </c>
       <c r="G81" s="7" t="n">
-        <v>3029</v>
+        <v>3579</v>
       </c>
       <c r="H81" s="6" t="inlineStr">
         <is>
-          <t>14/24</t>
+          <t>15/24</t>
         </is>
       </c>
       <c r="I81" s="6" t="inlineStr">
@@ -4500,10 +4500,10 @@
         </is>
       </c>
       <c r="J81" s="7" t="n">
-        <v>5193</v>
+        <v>5726</v>
       </c>
       <c r="K81" s="8" t="n">
-        <v>216.3571428571429</v>
+        <v>238.6</v>
       </c>
     </row>
     <row r="82">
@@ -4634,11 +4634,11 @@
         </is>
       </c>
       <c r="G84" s="7" t="n">
-        <v>3474</v>
+        <v>3661</v>
       </c>
       <c r="H84" s="6" t="inlineStr">
         <is>
-          <t>16/20</t>
+          <t>17/20</t>
         </is>
       </c>
       <c r="I84" s="6" t="inlineStr">
@@ -4647,10 +4647,10 @@
         </is>
       </c>
       <c r="J84" s="7" t="n">
-        <v>4342</v>
+        <v>4307</v>
       </c>
       <c r="K84" s="8" t="n">
-        <v>217.125</v>
+        <v>215.3529411764706</v>
       </c>
     </row>
     <row r="85">
@@ -4683,11 +4683,11 @@
         </is>
       </c>
       <c r="G85" s="11" t="n">
-        <v>1181</v>
+        <v>1368</v>
       </c>
       <c r="H85" s="10" t="inlineStr">
         <is>
-          <t>15/20</t>
+          <t>16/20</t>
         </is>
       </c>
       <c r="I85" s="10" t="inlineStr">
@@ -4696,10 +4696,10 @@
         </is>
       </c>
       <c r="J85" s="11" t="n">
-        <v>1575</v>
+        <v>1710</v>
       </c>
       <c r="K85" s="12" t="n">
-        <v>78.73333333333333</v>
+        <v>85.5</v>
       </c>
     </row>
     <row r="86">
@@ -4830,11 +4830,11 @@
         </is>
       </c>
       <c r="G88" s="4" t="n">
-        <v>15374</v>
+        <v>16592</v>
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>12/19</t>
+          <t>13/19</t>
         </is>
       </c>
       <c r="I88" s="3" t="inlineStr">
@@ -4843,59 +4843,59 @@
         </is>
       </c>
       <c r="J88" s="4" t="n">
-        <v>24342</v>
+        <v>24250</v>
       </c>
       <c r="K88" s="5" t="n">
-        <v>1281.166666666667</v>
+        <v>1276.307692307692</v>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="6" t="inlineStr">
+      <c r="A89" s="2" t="inlineStr">
         <is>
           <t>MADURAI EAST</t>
         </is>
       </c>
-      <c r="B89" s="6" t="n">
+      <c r="B89" s="3" t="n">
         <v>189</v>
       </c>
-      <c r="C89" s="6" t="inlineStr">
+      <c r="C89" s="3" t="inlineStr">
         <is>
           <t>KARTHIKEYAN S</t>
         </is>
       </c>
-      <c r="D89" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E89" s="6" t="inlineStr">
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E89" s="3" t="inlineStr">
         <is>
           <t>MOORTHY P</t>
         </is>
       </c>
-      <c r="F89" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G89" s="7" t="n">
-        <v>9621</v>
-      </c>
-      <c r="H89" s="6" t="inlineStr">
-        <is>
-          <t>21/29</t>
-        </is>
-      </c>
-      <c r="I89" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J89" s="7" t="n">
-        <v>13286</v>
-      </c>
-      <c r="K89" s="8" t="n">
-        <v>458.1428571428572</v>
+      <c r="F89" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G89" s="4" t="n">
+        <v>9851</v>
+      </c>
+      <c r="H89" s="3" t="inlineStr">
+        <is>
+          <t>22/29</t>
+        </is>
+      </c>
+      <c r="I89" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J89" s="4" t="n">
+        <v>12985</v>
+      </c>
+      <c r="K89" s="5" t="n">
+        <v>447.7727272727273</v>
       </c>
     </row>
     <row r="90">
@@ -4928,11 +4928,11 @@
         </is>
       </c>
       <c r="G90" s="4" t="n">
-        <v>14739</v>
+        <v>15112</v>
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>14/19</t>
+          <t>15/19</t>
         </is>
       </c>
       <c r="I90" s="3" t="inlineStr">
@@ -4941,10 +4941,10 @@
         </is>
       </c>
       <c r="J90" s="4" t="n">
-        <v>20003</v>
+        <v>19142</v>
       </c>
       <c r="K90" s="5" t="n">
-        <v>1052.785714285714</v>
+        <v>1007.466666666667</v>
       </c>
     </row>
     <row r="91">
@@ -5075,11 +5075,11 @@
         </is>
       </c>
       <c r="G93" s="4" t="n">
-        <v>5157</v>
+        <v>6138</v>
       </c>
       <c r="H93" s="3" t="inlineStr">
         <is>
-          <t>16/21</t>
+          <t>17/21</t>
         </is>
       </c>
       <c r="I93" s="3" t="inlineStr">
@@ -5088,10 +5088,10 @@
         </is>
       </c>
       <c r="J93" s="4" t="n">
-        <v>6769</v>
+        <v>7582</v>
       </c>
       <c r="K93" s="5" t="n">
-        <v>322.3125</v>
+        <v>361.0588235294118</v>
       </c>
     </row>
     <row r="94">
@@ -5124,11 +5124,11 @@
         </is>
       </c>
       <c r="G94" s="4" t="n">
-        <v>31121</v>
+        <v>33498</v>
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
-          <t>11/25</t>
+          <t>12/25</t>
         </is>
       </c>
       <c r="I94" s="3" t="inlineStr">
@@ -5137,10 +5137,10 @@
         </is>
       </c>
       <c r="J94" s="4" t="n">
-        <v>70730</v>
+        <v>69788</v>
       </c>
       <c r="K94" s="5" t="n">
-        <v>2829.181818181818</v>
+        <v>2791.5</v>
       </c>
     </row>
     <row r="95">
@@ -5173,11 +5173,11 @@
         </is>
       </c>
       <c r="G95" s="4" t="n">
-        <v>26593</v>
+        <v>27214</v>
       </c>
       <c r="H95" s="3" t="inlineStr">
         <is>
-          <t>16/20</t>
+          <t>17/20</t>
         </is>
       </c>
       <c r="I95" s="3" t="inlineStr">
@@ -5186,10 +5186,10 @@
         </is>
       </c>
       <c r="J95" s="4" t="n">
-        <v>33241</v>
+        <v>32016</v>
       </c>
       <c r="K95" s="5" t="n">
-        <v>1662.0625</v>
+        <v>1600.823529411765</v>
       </c>
     </row>
     <row r="96">
@@ -5369,11 +5369,11 @@
         </is>
       </c>
       <c r="G99" s="11" t="n">
-        <v>1198</v>
+        <v>1591</v>
       </c>
       <c r="H99" s="10" t="inlineStr">
         <is>
-          <t>17/22</t>
+          <t>18/22</t>
         </is>
       </c>
       <c r="I99" s="10" t="inlineStr">
@@ -5382,10 +5382,10 @@
         </is>
       </c>
       <c r="J99" s="11" t="n">
-        <v>1550</v>
+        <v>1945</v>
       </c>
       <c r="K99" s="12" t="n">
-        <v>70.47058823529412</v>
+        <v>88.38888888888889</v>
       </c>
     </row>
     <row r="100">
@@ -5418,11 +5418,11 @@
         </is>
       </c>
       <c r="G100" s="7" t="n">
-        <v>8440</v>
+        <v>8341</v>
       </c>
       <c r="H100" s="6" t="inlineStr">
         <is>
-          <t>15/22</t>
+          <t>16/22</t>
         </is>
       </c>
       <c r="I100" s="6" t="inlineStr">
@@ -5431,10 +5431,10 @@
         </is>
       </c>
       <c r="J100" s="7" t="n">
-        <v>12379</v>
+        <v>11469</v>
       </c>
       <c r="K100" s="8" t="n">
-        <v>562.6666666666667</v>
+        <v>521.3125</v>
       </c>
     </row>
     <row r="101">
@@ -5536,101 +5536,101 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="13" t="inlineStr">
+      <c r="A103" s="9" t="inlineStr">
         <is>
           <t>METTUR</t>
         </is>
       </c>
-      <c r="B103" s="14" t="n">
+      <c r="B103" s="10" t="n">
         <v>85</v>
       </c>
-      <c r="C103" s="14" t="inlineStr">
+      <c r="C103" s="10" t="inlineStr">
+        <is>
+          <t>VENKATACHALAM. G</t>
+        </is>
+      </c>
+      <c r="D103" s="10" t="inlineStr">
+        <is>
+          <t>All India Anna Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E103" s="10" t="inlineStr">
         <is>
           <t>MIDHUN CHAKRAVARTHY. M</t>
         </is>
       </c>
-      <c r="D103" s="14" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E103" s="14" t="inlineStr">
-        <is>
-          <t>VENKATACHALAM. G</t>
-        </is>
-      </c>
-      <c r="F103" s="14" t="inlineStr">
-        <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G103" s="15" t="n">
-        <v>32</v>
-      </c>
-      <c r="H103" s="14" t="inlineStr">
-        <is>
-          <t>13/24</t>
-        </is>
-      </c>
-      <c r="I103" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J103" s="15" t="n">
-        <v>59</v>
-      </c>
-      <c r="K103" s="16" t="n">
-        <v>2.461538461538462</v>
+      <c r="F103" s="10" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G103" s="11" t="n">
+        <v>328</v>
+      </c>
+      <c r="H103" s="10" t="inlineStr">
+        <is>
+          <t>14/24</t>
+        </is>
+      </c>
+      <c r="I103" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J103" s="11" t="n">
+        <v>562</v>
+      </c>
+      <c r="K103" s="12" t="n">
+        <v>23.42857142857143</v>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="6" t="inlineStr">
+      <c r="A104" s="9" t="inlineStr">
         <is>
           <t>MODAKKURICHI</t>
         </is>
       </c>
-      <c r="B104" s="6" t="n">
+      <c r="B104" s="10" t="n">
         <v>100</v>
       </c>
-      <c r="C104" s="6" t="inlineStr">
+      <c r="C104" s="10" t="inlineStr">
         <is>
           <t>D.SHANMUGAN</t>
         </is>
       </c>
-      <c r="D104" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E104" s="6" t="inlineStr">
+      <c r="D104" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E104" s="10" t="inlineStr">
         <is>
           <t>S.KIRTHIKA</t>
         </is>
       </c>
-      <c r="F104" s="6" t="inlineStr">
+      <c r="F104" s="10" t="inlineStr">
         <is>
           <t>Bharatiya Janata Party</t>
         </is>
       </c>
-      <c r="G104" s="7" t="n">
-        <v>3226</v>
-      </c>
-      <c r="H104" s="6" t="inlineStr">
-        <is>
-          <t>17/21</t>
-        </is>
-      </c>
-      <c r="I104" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J104" s="7" t="n">
-        <v>3985</v>
-      </c>
-      <c r="K104" s="8" t="n">
-        <v>189.7647058823529</v>
+      <c r="G104" s="11" t="n">
+        <v>2242</v>
+      </c>
+      <c r="H104" s="10" t="inlineStr">
+        <is>
+          <t>18/21</t>
+        </is>
+      </c>
+      <c r="I104" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J104" s="11" t="n">
+        <v>2616</v>
+      </c>
+      <c r="K104" s="12" t="n">
+        <v>124.5555555555556</v>
       </c>
     </row>
     <row r="105">
@@ -5663,11 +5663,11 @@
         </is>
       </c>
       <c r="G105" s="7" t="n">
-        <v>11994</v>
+        <v>12125</v>
       </c>
       <c r="H105" s="6" t="inlineStr">
         <is>
-          <t>21/30</t>
+          <t>22/30</t>
         </is>
       </c>
       <c r="I105" s="6" t="inlineStr">
@@ -5676,10 +5676,10 @@
         </is>
       </c>
       <c r="J105" s="7" t="n">
-        <v>17134</v>
+        <v>16534</v>
       </c>
       <c r="K105" s="8" t="n">
-        <v>571.1428571428571</v>
+        <v>551.1363636363636</v>
       </c>
     </row>
     <row r="106">
@@ -5712,7 +5712,7 @@
         </is>
       </c>
       <c r="G106" s="4" t="n">
-        <v>17883</v>
+        <v>17353</v>
       </c>
       <c r="H106" s="3" t="inlineStr">
         <is>
@@ -5725,10 +5725,10 @@
         </is>
       </c>
       <c r="J106" s="4" t="n">
-        <v>19765</v>
+        <v>19180</v>
       </c>
       <c r="K106" s="5" t="n">
-        <v>941.2105263157895</v>
+        <v>913.3157894736842</v>
       </c>
     </row>
     <row r="107">
@@ -5761,7 +5761,7 @@
         </is>
       </c>
       <c r="G107" s="4" t="n">
-        <v>26853</v>
+        <v>26724</v>
       </c>
       <c r="H107" s="3" t="inlineStr">
         <is>
@@ -5774,10 +5774,10 @@
         </is>
       </c>
       <c r="J107" s="4" t="n">
-        <v>29837</v>
+        <v>29693</v>
       </c>
       <c r="K107" s="5" t="n">
-        <v>1491.833333333333</v>
+        <v>1484.666666666667</v>
       </c>
     </row>
     <row r="108">
@@ -5830,52 +5830,52 @@
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="6" t="inlineStr">
+      <c r="A109" s="2" t="inlineStr">
         <is>
           <t>NAGERCOIL</t>
         </is>
       </c>
-      <c r="B109" s="6" t="n">
+      <c r="B109" s="3" t="n">
         <v>230</v>
       </c>
-      <c r="C109" s="6" t="inlineStr">
+      <c r="C109" s="3" t="inlineStr">
         <is>
           <t>AUSTIN</t>
         </is>
       </c>
-      <c r="D109" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E109" s="6" t="inlineStr">
+      <c r="D109" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E109" s="3" t="inlineStr">
         <is>
           <t>BERVIN KINGS G</t>
         </is>
       </c>
-      <c r="F109" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G109" s="7" t="n">
-        <v>3260</v>
-      </c>
-      <c r="H109" s="6" t="inlineStr">
-        <is>
-          <t>19/23</t>
-        </is>
-      </c>
-      <c r="I109" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J109" s="7" t="n">
-        <v>3946</v>
-      </c>
-      <c r="K109" s="8" t="n">
-        <v>171.578947368421</v>
+      <c r="F109" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G109" s="4" t="n">
+        <v>6139</v>
+      </c>
+      <c r="H109" s="3" t="inlineStr">
+        <is>
+          <t>20/23</t>
+        </is>
+      </c>
+      <c r="I109" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J109" s="4" t="n">
+        <v>7060</v>
+      </c>
+      <c r="K109" s="5" t="n">
+        <v>306.95</v>
       </c>
     </row>
     <row r="110">
@@ -5908,11 +5908,11 @@
         </is>
       </c>
       <c r="G110" s="11" t="n">
-        <v>446</v>
+        <v>1325</v>
       </c>
       <c r="H110" s="10" t="inlineStr">
         <is>
-          <t>10/23</t>
+          <t>11/23</t>
         </is>
       </c>
       <c r="I110" s="10" t="inlineStr">
@@ -5921,10 +5921,10 @@
         </is>
       </c>
       <c r="J110" s="11" t="n">
-        <v>1026</v>
+        <v>2770</v>
       </c>
       <c r="K110" s="12" t="n">
-        <v>44.6</v>
+        <v>120.4545454545455</v>
       </c>
     </row>
     <row r="111">
@@ -6006,11 +6006,11 @@
         </is>
       </c>
       <c r="G112" s="4" t="n">
-        <v>30870</v>
+        <v>32382</v>
       </c>
       <c r="H112" s="3" t="inlineStr">
         <is>
-          <t>19/25</t>
+          <t>20/25</t>
         </is>
       </c>
       <c r="I112" s="3" t="inlineStr">
@@ -6019,10 +6019,10 @@
         </is>
       </c>
       <c r="J112" s="4" t="n">
-        <v>40618</v>
+        <v>40478</v>
       </c>
       <c r="K112" s="5" t="n">
-        <v>1624.736842105263</v>
+        <v>1619.1</v>
       </c>
     </row>
     <row r="113">
@@ -6251,11 +6251,11 @@
         </is>
       </c>
       <c r="G117" s="7" t="n">
-        <v>10754</v>
+        <v>11448</v>
       </c>
       <c r="H117" s="6" t="inlineStr">
         <is>
-          <t>18/26</t>
+          <t>19/26</t>
         </is>
       </c>
       <c r="I117" s="6" t="inlineStr">
@@ -6264,10 +6264,10 @@
         </is>
       </c>
       <c r="J117" s="7" t="n">
-        <v>15534</v>
+        <v>15666</v>
       </c>
       <c r="K117" s="8" t="n">
-        <v>597.4444444444445</v>
+        <v>602.5263157894736</v>
       </c>
     </row>
     <row r="118">
@@ -6300,11 +6300,11 @@
         </is>
       </c>
       <c r="G118" s="4" t="n">
-        <v>31686</v>
+        <v>34116</v>
       </c>
       <c r="H118" s="3" t="inlineStr">
         <is>
-          <t>21/24</t>
+          <t>22/24</t>
         </is>
       </c>
       <c r="I118" s="3" t="inlineStr">
@@ -6313,10 +6313,10 @@
         </is>
       </c>
       <c r="J118" s="4" t="n">
-        <v>36213</v>
+        <v>37217</v>
       </c>
       <c r="K118" s="5" t="n">
-        <v>1508.857142857143</v>
+        <v>1550.727272727273</v>
       </c>
     </row>
     <row r="119">
@@ -6447,11 +6447,11 @@
         </is>
       </c>
       <c r="G121" s="4" t="n">
-        <v>31091</v>
+        <v>34305</v>
       </c>
       <c r="H121" s="3" t="inlineStr">
         <is>
-          <t>19/23</t>
+          <t>20/23</t>
         </is>
       </c>
       <c r="I121" s="3" t="inlineStr">
@@ -6460,10 +6460,10 @@
         </is>
       </c>
       <c r="J121" s="4" t="n">
-        <v>37636</v>
+        <v>39451</v>
       </c>
       <c r="K121" s="5" t="n">
-        <v>1636.368421052632</v>
+        <v>1715.25</v>
       </c>
     </row>
     <row r="122">
@@ -6496,11 +6496,11 @@
         </is>
       </c>
       <c r="G122" s="7" t="n">
-        <v>2987</v>
+        <v>3448</v>
       </c>
       <c r="H122" s="6" t="inlineStr">
         <is>
-          <t>18/25</t>
+          <t>19/25</t>
         </is>
       </c>
       <c r="I122" s="6" t="inlineStr">
@@ -6509,10 +6509,10 @@
         </is>
       </c>
       <c r="J122" s="7" t="n">
-        <v>4149</v>
+        <v>4537</v>
       </c>
       <c r="K122" s="8" t="n">
-        <v>165.9444444444445</v>
+        <v>181.4736842105263</v>
       </c>
     </row>
     <row r="123">
@@ -6545,11 +6545,11 @@
         </is>
       </c>
       <c r="G123" s="4" t="n">
-        <v>9359</v>
+        <v>13897</v>
       </c>
       <c r="H123" s="3" t="inlineStr">
         <is>
-          <t>20/22</t>
+          <t>21/22</t>
         </is>
       </c>
       <c r="I123" s="3" t="inlineStr">
@@ -6558,10 +6558,10 @@
         </is>
       </c>
       <c r="J123" s="4" t="n">
-        <v>10295</v>
+        <v>14559</v>
       </c>
       <c r="K123" s="5" t="n">
-        <v>467.95</v>
+        <v>661.7619047619048</v>
       </c>
     </row>
     <row r="124">
@@ -6594,11 +6594,11 @@
         </is>
       </c>
       <c r="G124" s="4" t="n">
-        <v>34719</v>
+        <v>36952</v>
       </c>
       <c r="H124" s="3" t="inlineStr">
         <is>
-          <t>24/35</t>
+          <t>25/35</t>
         </is>
       </c>
       <c r="I124" s="3" t="inlineStr">
@@ -6607,10 +6607,10 @@
         </is>
       </c>
       <c r="J124" s="4" t="n">
-        <v>50632</v>
+        <v>51733</v>
       </c>
       <c r="K124" s="5" t="n">
-        <v>1446.625</v>
+        <v>1478.08</v>
       </c>
     </row>
     <row r="125">
@@ -6790,11 +6790,11 @@
         </is>
       </c>
       <c r="G128" s="4" t="n">
-        <v>35402</v>
+        <v>35472</v>
       </c>
       <c r="H128" s="3" t="inlineStr">
         <is>
-          <t>20/23</t>
+          <t>21/23</t>
         </is>
       </c>
       <c r="I128" s="3" t="inlineStr">
@@ -6803,10 +6803,10 @@
         </is>
       </c>
       <c r="J128" s="4" t="n">
-        <v>40712</v>
+        <v>38850</v>
       </c>
       <c r="K128" s="5" t="n">
-        <v>1770.1</v>
+        <v>1689.142857142857</v>
       </c>
     </row>
     <row r="129">
@@ -6937,11 +6937,11 @@
         </is>
       </c>
       <c r="G131" s="7" t="n">
-        <v>5130</v>
+        <v>4657</v>
       </c>
       <c r="H131" s="6" t="inlineStr">
         <is>
-          <t>13/23</t>
+          <t>14/23</t>
         </is>
       </c>
       <c r="I131" s="6" t="inlineStr">
@@ -6950,59 +6950,59 @@
         </is>
       </c>
       <c r="J131" s="7" t="n">
-        <v>9076</v>
+        <v>7651</v>
       </c>
       <c r="K131" s="8" t="n">
-        <v>394.6153846153846</v>
+        <v>332.6428571428572</v>
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="9" t="inlineStr">
+      <c r="A132" s="6" t="inlineStr">
         <is>
           <t>PENNAGARAM</t>
         </is>
       </c>
-      <c r="B132" s="10" t="n">
+      <c r="B132" s="6" t="n">
         <v>58</v>
       </c>
-      <c r="C132" s="10" t="inlineStr">
+      <c r="C132" s="6" t="inlineStr">
         <is>
           <t>GAJENDRAN. S.</t>
         </is>
       </c>
-      <c r="D132" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E132" s="10" t="inlineStr">
+      <c r="D132" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E132" s="6" t="inlineStr">
         <is>
           <t>SELVAM. V.</t>
         </is>
       </c>
-      <c r="F132" s="10" t="inlineStr">
+      <c r="F132" s="6" t="inlineStr">
         <is>
           <t>Pattali Makkal Katchi</t>
         </is>
       </c>
-      <c r="G132" s="11" t="n">
-        <v>1576</v>
-      </c>
-      <c r="H132" s="10" t="inlineStr">
-        <is>
-          <t>15/23</t>
-        </is>
-      </c>
-      <c r="I132" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J132" s="11" t="n">
-        <v>2417</v>
-      </c>
-      <c r="K132" s="12" t="n">
-        <v>105.0666666666667</v>
+      <c r="G132" s="7" t="n">
+        <v>2117</v>
+      </c>
+      <c r="H132" s="6" t="inlineStr">
+        <is>
+          <t>16/23</t>
+        </is>
+      </c>
+      <c r="I132" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J132" s="7" t="n">
+        <v>3043</v>
+      </c>
+      <c r="K132" s="8" t="n">
+        <v>132.3125</v>
       </c>
     </row>
     <row r="133">
@@ -7084,11 +7084,11 @@
         </is>
       </c>
       <c r="G134" s="4" t="n">
-        <v>25723</v>
+        <v>29031</v>
       </c>
       <c r="H134" s="3" t="inlineStr">
         <is>
-          <t>11/22</t>
+          <t>12/22</t>
         </is>
       </c>
       <c r="I134" s="3" t="inlineStr">
@@ -7097,10 +7097,10 @@
         </is>
       </c>
       <c r="J134" s="4" t="n">
-        <v>51446</v>
+        <v>53224</v>
       </c>
       <c r="K134" s="5" t="n">
-        <v>2338.454545454545</v>
+        <v>2419.25</v>
       </c>
     </row>
     <row r="135">
@@ -7133,11 +7133,11 @@
         </is>
       </c>
       <c r="G135" s="11" t="n">
-        <v>546</v>
+        <v>428</v>
       </c>
       <c r="H135" s="10" t="inlineStr">
         <is>
-          <t>6/21</t>
+          <t>7/21</t>
         </is>
       </c>
       <c r="I135" s="10" t="inlineStr">
@@ -7146,10 +7146,10 @@
         </is>
       </c>
       <c r="J135" s="11" t="n">
-        <v>1911</v>
+        <v>1284</v>
       </c>
       <c r="K135" s="12" t="n">
-        <v>91</v>
+        <v>61.14285714285715</v>
       </c>
     </row>
     <row r="136">
@@ -7182,11 +7182,11 @@
         </is>
       </c>
       <c r="G136" s="7" t="n">
-        <v>3844</v>
+        <v>4107</v>
       </c>
       <c r="H136" s="6" t="inlineStr">
         <is>
-          <t>15/26</t>
+          <t>16/26</t>
         </is>
       </c>
       <c r="I136" s="6" t="inlineStr">
@@ -7195,10 +7195,10 @@
         </is>
       </c>
       <c r="J136" s="7" t="n">
-        <v>6663</v>
+        <v>6674</v>
       </c>
       <c r="K136" s="8" t="n">
-        <v>256.2666666666667</v>
+        <v>256.6875</v>
       </c>
     </row>
     <row r="137">
@@ -7251,101 +7251,101 @@
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="9" t="inlineStr">
+      <c r="A138" s="6" t="inlineStr">
         <is>
           <t>POLLACHI</t>
         </is>
       </c>
-      <c r="B138" s="10" t="n">
+      <c r="B138" s="6" t="n">
         <v>123</v>
       </c>
-      <c r="C138" s="10" t="inlineStr">
+      <c r="C138" s="6" t="inlineStr">
         <is>
           <t>K. NITHYANANDHAN</t>
         </is>
       </c>
-      <c r="D138" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E138" s="10" t="inlineStr">
+      <c r="D138" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E138" s="6" t="inlineStr">
         <is>
           <t>POLLACHI V. JAYARAMAN</t>
         </is>
       </c>
-      <c r="F138" s="10" t="inlineStr">
+      <c r="F138" s="6" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G138" s="11" t="n">
-        <v>2609</v>
-      </c>
-      <c r="H138" s="10" t="inlineStr">
+      <c r="G138" s="7" t="n">
+        <v>2731</v>
+      </c>
+      <c r="H138" s="6" t="inlineStr">
         <is>
           <t>18/20</t>
         </is>
       </c>
-      <c r="I138" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J138" s="11" t="n">
-        <v>2899</v>
-      </c>
-      <c r="K138" s="12" t="n">
-        <v>144.9444444444445</v>
+      <c r="I138" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J138" s="7" t="n">
+        <v>3034</v>
+      </c>
+      <c r="K138" s="8" t="n">
+        <v>151.7222222222222</v>
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="6" t="inlineStr">
+      <c r="A139" s="9" t="inlineStr">
         <is>
           <t>POLUR</t>
         </is>
       </c>
-      <c r="B139" s="6" t="n">
+      <c r="B139" s="10" t="n">
         <v>66</v>
       </c>
-      <c r="C139" s="6" t="inlineStr">
+      <c r="C139" s="10" t="inlineStr">
         <is>
           <t>ABISHEK. R</t>
         </is>
       </c>
-      <c r="D139" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E139" s="6" t="inlineStr">
+      <c r="D139" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E139" s="10" t="inlineStr">
         <is>
           <t>SARAVANAN. P</t>
         </is>
       </c>
-      <c r="F139" s="6" t="inlineStr">
+      <c r="F139" s="10" t="inlineStr">
         <is>
           <t>Desiya Murpokku Dravida Kazhagam</t>
         </is>
       </c>
-      <c r="G139" s="7" t="n">
-        <v>1431</v>
-      </c>
-      <c r="H139" s="6" t="inlineStr">
-        <is>
-          <t>8/22</t>
-        </is>
-      </c>
-      <c r="I139" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J139" s="7" t="n">
-        <v>3935</v>
-      </c>
-      <c r="K139" s="8" t="n">
-        <v>178.875</v>
+      <c r="G139" s="11" t="n">
+        <v>1085</v>
+      </c>
+      <c r="H139" s="10" t="inlineStr">
+        <is>
+          <t>9/22</t>
+        </is>
+      </c>
+      <c r="I139" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J139" s="11" t="n">
+        <v>2652</v>
+      </c>
+      <c r="K139" s="12" t="n">
+        <v>120.5555555555556</v>
       </c>
     </row>
     <row r="140">
@@ -7378,11 +7378,11 @@
         </is>
       </c>
       <c r="G140" s="4" t="n">
-        <v>38889</v>
+        <v>41638</v>
       </c>
       <c r="H140" s="3" t="inlineStr">
         <is>
-          <t>17/24</t>
+          <t>18/24</t>
         </is>
       </c>
       <c r="I140" s="3" t="inlineStr">
@@ -7391,10 +7391,10 @@
         </is>
       </c>
       <c r="J140" s="4" t="n">
-        <v>54902</v>
+        <v>55517</v>
       </c>
       <c r="K140" s="5" t="n">
-        <v>2287.588235294118</v>
+        <v>2313.222222222222</v>
       </c>
     </row>
     <row r="141">
@@ -7476,11 +7476,11 @@
         </is>
       </c>
       <c r="G142" s="4" t="n">
-        <v>58192</v>
+        <v>60593</v>
       </c>
       <c r="H142" s="3" t="inlineStr">
         <is>
-          <t>17/23</t>
+          <t>18/23</t>
         </is>
       </c>
       <c r="I142" s="3" t="inlineStr">
@@ -7489,10 +7489,10 @@
         </is>
       </c>
       <c r="J142" s="4" t="n">
-        <v>78730</v>
+        <v>77424</v>
       </c>
       <c r="K142" s="5" t="n">
-        <v>3423.058823529412</v>
+        <v>3366.277777777778</v>
       </c>
     </row>
     <row r="143">
@@ -7525,11 +7525,11 @@
         </is>
       </c>
       <c r="G143" s="7" t="n">
-        <v>2266</v>
+        <v>2376</v>
       </c>
       <c r="H143" s="6" t="inlineStr">
         <is>
-          <t>13/22</t>
+          <t>14/22</t>
         </is>
       </c>
       <c r="I143" s="6" t="inlineStr">
@@ -7538,10 +7538,10 @@
         </is>
       </c>
       <c r="J143" s="7" t="n">
-        <v>3835</v>
+        <v>3734</v>
       </c>
       <c r="K143" s="8" t="n">
-        <v>174.3076923076923</v>
+        <v>169.7142857142857</v>
       </c>
     </row>
     <row r="144">
@@ -7574,11 +7574,11 @@
         </is>
       </c>
       <c r="G144" s="4" t="n">
-        <v>12216</v>
+        <v>12193</v>
       </c>
       <c r="H144" s="3" t="inlineStr">
         <is>
-          <t>24/26</t>
+          <t>25/26</t>
         </is>
       </c>
       <c r="I144" s="3" t="inlineStr">
@@ -7587,10 +7587,10 @@
         </is>
       </c>
       <c r="J144" s="4" t="n">
-        <v>13234</v>
+        <v>12681</v>
       </c>
       <c r="K144" s="5" t="n">
-        <v>509</v>
+        <v>487.72</v>
       </c>
     </row>
     <row r="145">
@@ -7623,11 +7623,11 @@
         </is>
       </c>
       <c r="G145" s="4" t="n">
-        <v>10912</v>
+        <v>10807</v>
       </c>
       <c r="H145" s="3" t="inlineStr">
         <is>
-          <t>17/20</t>
+          <t>18/20</t>
         </is>
       </c>
       <c r="I145" s="3" t="inlineStr">
@@ -7636,10 +7636,10 @@
         </is>
       </c>
       <c r="J145" s="4" t="n">
-        <v>12838</v>
+        <v>12008</v>
       </c>
       <c r="K145" s="5" t="n">
-        <v>641.8823529411765</v>
+        <v>600.3888888888889</v>
       </c>
     </row>
     <row r="146">
@@ -7672,11 +7672,11 @@
         </is>
       </c>
       <c r="G146" s="4" t="n">
-        <v>14803</v>
+        <v>13664</v>
       </c>
       <c r="H146" s="3" t="inlineStr">
         <is>
-          <t>26/29</t>
+          <t>27/29</t>
         </is>
       </c>
       <c r="I146" s="3" t="inlineStr">
@@ -7685,10 +7685,10 @@
         </is>
       </c>
       <c r="J146" s="4" t="n">
-        <v>16511</v>
+        <v>14676</v>
       </c>
       <c r="K146" s="5" t="n">
-        <v>569.3461538461538</v>
+        <v>506.0740740740741</v>
       </c>
     </row>
     <row r="147">
@@ -7702,30 +7702,30 @@
       </c>
       <c r="C147" s="10" t="inlineStr">
         <is>
+          <t>THAHIRA</t>
+        </is>
+      </c>
+      <c r="D147" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E147" s="10" t="inlineStr">
+        <is>
           <t>R. GANDHI</t>
         </is>
       </c>
-      <c r="D147" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E147" s="10" t="inlineStr">
-        <is>
-          <t>THAHIRA</t>
-        </is>
-      </c>
       <c r="F147" s="10" t="inlineStr">
         <is>
-          <t>Tamilaga Vettri Kazhagam</t>
+          <t>Dravida Munnetra Kazhagam</t>
         </is>
       </c>
       <c r="G147" s="11" t="n">
-        <v>1569</v>
+        <v>843</v>
       </c>
       <c r="H147" s="10" t="inlineStr">
         <is>
-          <t>14/22</t>
+          <t>16/22</t>
         </is>
       </c>
       <c r="I147" s="10" t="inlineStr">
@@ -7734,10 +7734,10 @@
         </is>
       </c>
       <c r="J147" s="11" t="n">
-        <v>2466</v>
+        <v>1159</v>
       </c>
       <c r="K147" s="12" t="n">
-        <v>112.0714285714286</v>
+        <v>52.6875</v>
       </c>
     </row>
     <row r="148">
@@ -7819,11 +7819,11 @@
         </is>
       </c>
       <c r="G149" s="7" t="n">
-        <v>3101</v>
+        <v>2802</v>
       </c>
       <c r="H149" s="6" t="inlineStr">
         <is>
-          <t>11/25</t>
+          <t>12/25</t>
         </is>
       </c>
       <c r="I149" s="6" t="inlineStr">
@@ -7832,10 +7832,10 @@
         </is>
       </c>
       <c r="J149" s="7" t="n">
-        <v>7048</v>
+        <v>5838</v>
       </c>
       <c r="K149" s="8" t="n">
-        <v>281.9090909090909</v>
+        <v>233.5</v>
       </c>
     </row>
     <row r="150">
@@ -7868,11 +7868,11 @@
         </is>
       </c>
       <c r="G150" s="4" t="n">
-        <v>14227</v>
+        <v>14129</v>
       </c>
       <c r="H150" s="3" t="inlineStr">
         <is>
-          <t>13/14</t>
+          <t>14/14</t>
         </is>
       </c>
       <c r="I150" s="3" t="inlineStr">
@@ -7881,10 +7881,10 @@
         </is>
       </c>
       <c r="J150" s="4" t="n">
-        <v>15321</v>
+        <v>14129</v>
       </c>
       <c r="K150" s="5" t="n">
-        <v>1094.384615384615</v>
+        <v>1009.214285714286</v>
       </c>
     </row>
     <row r="151">
@@ -7917,11 +7917,11 @@
         </is>
       </c>
       <c r="G151" s="4" t="n">
-        <v>20749</v>
+        <v>21064</v>
       </c>
       <c r="H151" s="3" t="inlineStr">
         <is>
-          <t>14/21</t>
+          <t>15/21</t>
         </is>
       </c>
       <c r="I151" s="3" t="inlineStr">
@@ -7930,10 +7930,10 @@
         </is>
       </c>
       <c r="J151" s="4" t="n">
-        <v>31124</v>
+        <v>29490</v>
       </c>
       <c r="K151" s="5" t="n">
-        <v>1482.071428571429</v>
+        <v>1404.266666666667</v>
       </c>
     </row>
     <row r="152">
@@ -7966,11 +7966,11 @@
         </is>
       </c>
       <c r="G152" s="7" t="n">
-        <v>6821</v>
+        <v>6041</v>
       </c>
       <c r="H152" s="6" t="inlineStr">
         <is>
-          <t>14/21</t>
+          <t>15/21</t>
         </is>
       </c>
       <c r="I152" s="6" t="inlineStr">
@@ -7979,10 +7979,10 @@
         </is>
       </c>
       <c r="J152" s="7" t="n">
-        <v>10232</v>
+        <v>8457</v>
       </c>
       <c r="K152" s="8" t="n">
-        <v>487.2142857142857</v>
+        <v>402.7333333333333</v>
       </c>
     </row>
     <row r="153">
@@ -8015,11 +8015,11 @@
         </is>
       </c>
       <c r="G153" s="4" t="n">
-        <v>29324</v>
+        <v>30634</v>
       </c>
       <c r="H153" s="3" t="inlineStr">
         <is>
-          <t>16/20</t>
+          <t>17/20</t>
         </is>
       </c>
       <c r="I153" s="3" t="inlineStr">
@@ -8028,10 +8028,10 @@
         </is>
       </c>
       <c r="J153" s="4" t="n">
-        <v>36655</v>
+        <v>36040</v>
       </c>
       <c r="K153" s="5" t="n">
-        <v>1832.75</v>
+        <v>1802</v>
       </c>
     </row>
     <row r="154">
@@ -8064,11 +8064,11 @@
         </is>
       </c>
       <c r="G154" s="4" t="n">
-        <v>41826</v>
+        <v>44746</v>
       </c>
       <c r="H154" s="3" t="inlineStr">
         <is>
-          <t>13/23</t>
+          <t>14/23</t>
         </is>
       </c>
       <c r="I154" s="3" t="inlineStr">
@@ -8077,10 +8077,10 @@
         </is>
       </c>
       <c r="J154" s="4" t="n">
-        <v>74000</v>
+        <v>73511</v>
       </c>
       <c r="K154" s="5" t="n">
-        <v>3217.384615384616</v>
+        <v>3196.142857142857</v>
       </c>
     </row>
     <row r="155">
@@ -8113,11 +8113,11 @@
         </is>
       </c>
       <c r="G155" s="7" t="n">
-        <v>3318</v>
+        <v>3338</v>
       </c>
       <c r="H155" s="6" t="inlineStr">
         <is>
-          <t>15/23</t>
+          <t>16/23</t>
         </is>
       </c>
       <c r="I155" s="6" t="inlineStr">
@@ -8126,10 +8126,10 @@
         </is>
       </c>
       <c r="J155" s="7" t="n">
-        <v>5088</v>
+        <v>4798</v>
       </c>
       <c r="K155" s="8" t="n">
-        <v>221.2</v>
+        <v>208.625</v>
       </c>
     </row>
     <row r="156">
@@ -8182,52 +8182,52 @@
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="6" t="inlineStr">
+      <c r="A157" s="2" t="inlineStr">
         <is>
           <t>SANKARI</t>
         </is>
       </c>
-      <c r="B157" s="6" t="n">
+      <c r="B157" s="3" t="n">
         <v>87</v>
       </c>
-      <c r="C157" s="6" t="inlineStr">
+      <c r="C157" s="3" t="inlineStr">
         <is>
           <t>VETRIVEL. S</t>
         </is>
       </c>
-      <c r="D157" s="6" t="inlineStr">
+      <c r="D157" s="3" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E157" s="6" t="inlineStr">
+      <c r="E157" s="3" t="inlineStr">
         <is>
           <t>SENTHILKUMAR. K</t>
         </is>
       </c>
-      <c r="F157" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G157" s="7" t="n">
-        <v>4578</v>
-      </c>
-      <c r="H157" s="6" t="inlineStr">
-        <is>
-          <t>18/25</t>
-        </is>
-      </c>
-      <c r="I157" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J157" s="7" t="n">
-        <v>6358</v>
-      </c>
-      <c r="K157" s="8" t="n">
-        <v>254.3333333333333</v>
+      <c r="F157" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G157" s="4" t="n">
+        <v>5906</v>
+      </c>
+      <c r="H157" s="3" t="inlineStr">
+        <is>
+          <t>19/25</t>
+        </is>
+      </c>
+      <c r="I157" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J157" s="4" t="n">
+        <v>7771</v>
+      </c>
+      <c r="K157" s="5" t="n">
+        <v>310.8421052631579</v>
       </c>
     </row>
     <row r="158">
@@ -8260,11 +8260,11 @@
         </is>
       </c>
       <c r="G158" s="11" t="n">
-        <v>563</v>
+        <v>741</v>
       </c>
       <c r="H158" s="10" t="inlineStr">
         <is>
-          <t>7/21</t>
+          <t>8/21</t>
         </is>
       </c>
       <c r="I158" s="10" t="inlineStr">
@@ -8273,10 +8273,10 @@
         </is>
       </c>
       <c r="J158" s="11" t="n">
-        <v>1689</v>
+        <v>1945</v>
       </c>
       <c r="K158" s="12" t="n">
-        <v>80.42857142857143</v>
+        <v>92.625</v>
       </c>
     </row>
     <row r="159">
@@ -8290,30 +8290,30 @@
       </c>
       <c r="C159" s="10" t="inlineStr">
         <is>
+          <t>P CHANDRASEKAR</t>
+        </is>
+      </c>
+      <c r="D159" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E159" s="10" t="inlineStr">
+        <is>
           <t>C CHANDRASEKARAN</t>
         </is>
       </c>
-      <c r="D159" s="10" t="inlineStr">
+      <c r="F159" s="10" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E159" s="10" t="inlineStr">
-        <is>
-          <t>P CHANDRASEKAR</t>
-        </is>
-      </c>
-      <c r="F159" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
       <c r="G159" s="11" t="n">
-        <v>458</v>
+        <v>760</v>
       </c>
       <c r="H159" s="10" t="inlineStr">
         <is>
-          <t>19/22</t>
+          <t>20/22</t>
         </is>
       </c>
       <c r="I159" s="10" t="inlineStr">
@@ -8322,10 +8322,10 @@
         </is>
       </c>
       <c r="J159" s="11" t="n">
-        <v>530</v>
+        <v>836</v>
       </c>
       <c r="K159" s="12" t="n">
-        <v>24.10526315789474</v>
+        <v>38</v>
       </c>
     </row>
     <row r="160">
@@ -8456,11 +8456,11 @@
         </is>
       </c>
       <c r="G162" s="4" t="n">
-        <v>35149</v>
+        <v>38323</v>
       </c>
       <c r="H162" s="3" t="inlineStr">
         <is>
-          <t>12/30</t>
+          <t>13/30</t>
         </is>
       </c>
       <c r="I162" s="3" t="inlineStr">
@@ -8469,10 +8469,10 @@
         </is>
       </c>
       <c r="J162" s="4" t="n">
-        <v>87872</v>
+        <v>88438</v>
       </c>
       <c r="K162" s="5" t="n">
-        <v>2929.083333333333</v>
+        <v>2947.923076923077</v>
       </c>
     </row>
     <row r="163">
@@ -8505,11 +8505,11 @@
         </is>
       </c>
       <c r="G163" s="4" t="n">
-        <v>14442</v>
+        <v>16388</v>
       </c>
       <c r="H163" s="3" t="inlineStr">
         <is>
-          <t>15/26</t>
+          <t>16/26</t>
         </is>
       </c>
       <c r="I163" s="3" t="inlineStr">
@@ -8518,10 +8518,10 @@
         </is>
       </c>
       <c r="J163" s="4" t="n">
-        <v>25033</v>
+        <v>26630</v>
       </c>
       <c r="K163" s="5" t="n">
-        <v>962.8000000000001</v>
+        <v>1024.25</v>
       </c>
     </row>
     <row r="164">
@@ -8603,11 +8603,11 @@
         </is>
       </c>
       <c r="G165" s="7" t="n">
-        <v>8547</v>
+        <v>10459</v>
       </c>
       <c r="H165" s="6" t="inlineStr">
         <is>
-          <t>15/29</t>
+          <t>16/29</t>
         </is>
       </c>
       <c r="I165" s="6" t="inlineStr">
@@ -8616,10 +8616,10 @@
         </is>
       </c>
       <c r="J165" s="7" t="n">
-        <v>16524</v>
+        <v>18957</v>
       </c>
       <c r="K165" s="8" t="n">
-        <v>569.8</v>
+        <v>653.6875</v>
       </c>
     </row>
     <row r="166">
@@ -8750,11 +8750,11 @@
         </is>
       </c>
       <c r="G168" s="4" t="n">
-        <v>16885</v>
+        <v>18542</v>
       </c>
       <c r="H168" s="3" t="inlineStr">
         <is>
-          <t>13/27</t>
+          <t>14/27</t>
         </is>
       </c>
       <c r="I168" s="3" t="inlineStr">
@@ -8763,10 +8763,10 @@
         </is>
       </c>
       <c r="J168" s="4" t="n">
-        <v>35069</v>
+        <v>35760</v>
       </c>
       <c r="K168" s="5" t="n">
-        <v>1298.846153846154</v>
+        <v>1324.428571428571</v>
       </c>
     </row>
     <row r="169">
@@ -8848,11 +8848,11 @@
         </is>
       </c>
       <c r="G170" s="7" t="n">
-        <v>2260</v>
+        <v>2791</v>
       </c>
       <c r="H170" s="6" t="inlineStr">
         <is>
-          <t>12/22</t>
+          <t>13/22</t>
         </is>
       </c>
       <c r="I170" s="6" t="inlineStr">
@@ -8861,10 +8861,10 @@
         </is>
       </c>
       <c r="J170" s="7" t="n">
-        <v>4143</v>
+        <v>4723</v>
       </c>
       <c r="K170" s="8" t="n">
-        <v>188.3333333333333</v>
+        <v>214.6923076923077</v>
       </c>
     </row>
     <row r="171">
@@ -8897,11 +8897,11 @@
         </is>
       </c>
       <c r="G171" s="7" t="n">
-        <v>9889</v>
+        <v>10928</v>
       </c>
       <c r="H171" s="6" t="inlineStr">
         <is>
-          <t>18/28</t>
+          <t>19/28</t>
         </is>
       </c>
       <c r="I171" s="6" t="inlineStr">
@@ -8910,10 +8910,10 @@
         </is>
       </c>
       <c r="J171" s="7" t="n">
-        <v>15383</v>
+        <v>16104</v>
       </c>
       <c r="K171" s="8" t="n">
-        <v>549.3888888888889</v>
+        <v>575.1578947368421</v>
       </c>
     </row>
     <row r="172">
@@ -8946,11 +8946,11 @@
         </is>
       </c>
       <c r="G172" s="4" t="n">
-        <v>22484</v>
+        <v>23858</v>
       </c>
       <c r="H172" s="3" t="inlineStr">
         <is>
-          <t>24/34</t>
+          <t>25/34</t>
         </is>
       </c>
       <c r="I172" s="3" t="inlineStr">
@@ -8959,10 +8959,10 @@
         </is>
       </c>
       <c r="J172" s="4" t="n">
-        <v>31852</v>
+        <v>32447</v>
       </c>
       <c r="K172" s="5" t="n">
-        <v>936.8333333333334</v>
+        <v>954.3200000000001</v>
       </c>
     </row>
     <row r="173">
@@ -9044,11 +9044,11 @@
         </is>
       </c>
       <c r="G174" s="11" t="n">
-        <v>477</v>
+        <v>413</v>
       </c>
       <c r="H174" s="10" t="inlineStr">
         <is>
-          <t>14/24</t>
+          <t>15/24</t>
         </is>
       </c>
       <c r="I174" s="10" t="inlineStr">
@@ -9057,10 +9057,10 @@
         </is>
       </c>
       <c r="J174" s="11" t="n">
-        <v>818</v>
+        <v>661</v>
       </c>
       <c r="K174" s="12" t="n">
-        <v>34.07142857142857</v>
+        <v>27.53333333333333</v>
       </c>
     </row>
     <row r="175">
@@ -9191,11 +9191,11 @@
         </is>
       </c>
       <c r="G177" s="4" t="n">
-        <v>16179</v>
+        <v>17629</v>
       </c>
       <c r="H177" s="3" t="inlineStr">
         <is>
-          <t>20/26</t>
+          <t>21/26</t>
         </is>
       </c>
       <c r="I177" s="3" t="inlineStr">
@@ -9204,10 +9204,10 @@
         </is>
       </c>
       <c r="J177" s="4" t="n">
-        <v>21033</v>
+        <v>21826</v>
       </c>
       <c r="K177" s="5" t="n">
-        <v>808.95</v>
+        <v>839.4761904761905</v>
       </c>
     </row>
     <row r="178">
@@ -9221,30 +9221,30 @@
       </c>
       <c r="C178" s="10" t="inlineStr">
         <is>
+          <t>VAIRAMUTHU.PK</t>
+        </is>
+      </c>
+      <c r="D178" s="10" t="inlineStr">
+        <is>
+          <t>All India Anna Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E178" s="10" t="inlineStr">
+        <is>
           <t>REGUPATHY.S</t>
         </is>
       </c>
-      <c r="D178" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E178" s="10" t="inlineStr">
-        <is>
-          <t>VAIRAMUTHU.PK</t>
-        </is>
-      </c>
       <c r="F178" s="10" t="inlineStr">
         <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
+          <t>Dravida Munnetra Kazhagam</t>
         </is>
       </c>
       <c r="G178" s="11" t="n">
-        <v>547</v>
+        <v>275</v>
       </c>
       <c r="H178" s="10" t="inlineStr">
         <is>
-          <t>10/22</t>
+          <t>11/22</t>
         </is>
       </c>
       <c r="I178" s="10" t="inlineStr">
@@ -9253,10 +9253,10 @@
         </is>
       </c>
       <c r="J178" s="11" t="n">
-        <v>1203</v>
+        <v>550</v>
       </c>
       <c r="K178" s="12" t="n">
-        <v>54.7</v>
+        <v>25</v>
       </c>
     </row>
     <row r="179">
@@ -9289,11 +9289,11 @@
         </is>
       </c>
       <c r="G179" s="4" t="n">
-        <v>17607</v>
+        <v>18994</v>
       </c>
       <c r="H179" s="3" t="inlineStr">
         <is>
-          <t>13/26</t>
+          <t>14/26</t>
         </is>
       </c>
       <c r="I179" s="3" t="inlineStr">
@@ -9302,10 +9302,10 @@
         </is>
       </c>
       <c r="J179" s="4" t="n">
-        <v>35214</v>
+        <v>35275</v>
       </c>
       <c r="K179" s="5" t="n">
-        <v>1354.384615384615</v>
+        <v>1356.714285714286</v>
       </c>
     </row>
     <row r="180">
@@ -9485,11 +9485,11 @@
         </is>
       </c>
       <c r="G183" s="4" t="n">
-        <v>15578</v>
+        <v>17740</v>
       </c>
       <c r="H183" s="3" t="inlineStr">
         <is>
-          <t>17/24</t>
+          <t>18/24</t>
         </is>
       </c>
       <c r="I183" s="3" t="inlineStr">
@@ -9498,10 +9498,10 @@
         </is>
       </c>
       <c r="J183" s="4" t="n">
-        <v>21992</v>
+        <v>23653</v>
       </c>
       <c r="K183" s="5" t="n">
-        <v>916.3529411764706</v>
+        <v>985.5555555555555</v>
       </c>
     </row>
     <row r="184">
@@ -9534,11 +9534,11 @@
         </is>
       </c>
       <c r="G184" s="4" t="n">
-        <v>17876</v>
+        <v>18148</v>
       </c>
       <c r="H184" s="3" t="inlineStr">
         <is>
-          <t>23/24</t>
+          <t>25/25</t>
         </is>
       </c>
       <c r="I184" s="3" t="inlineStr">
@@ -9547,10 +9547,10 @@
         </is>
       </c>
       <c r="J184" s="4" t="n">
-        <v>18653</v>
+        <v>18148</v>
       </c>
       <c r="K184" s="5" t="n">
-        <v>777.2173913043479</v>
+        <v>725.92</v>
       </c>
     </row>
     <row r="185">
@@ -9583,11 +9583,11 @@
         </is>
       </c>
       <c r="G185" s="7" t="n">
-        <v>2886</v>
+        <v>4021</v>
       </c>
       <c r="H185" s="6" t="inlineStr">
         <is>
-          <t>11/23</t>
+          <t>12/23</t>
         </is>
       </c>
       <c r="I185" s="6" t="inlineStr">
@@ -9596,10 +9596,10 @@
         </is>
       </c>
       <c r="J185" s="7" t="n">
-        <v>6034</v>
+        <v>7707</v>
       </c>
       <c r="K185" s="8" t="n">
-        <v>262.3636363636364</v>
+        <v>335.0833333333333</v>
       </c>
     </row>
     <row r="186">
@@ -9632,11 +9632,11 @@
         </is>
       </c>
       <c r="G186" s="7" t="n">
-        <v>9876</v>
+        <v>10311</v>
       </c>
       <c r="H186" s="6" t="inlineStr">
         <is>
-          <t>16/24</t>
+          <t>17/24</t>
         </is>
       </c>
       <c r="I186" s="6" t="inlineStr">
@@ -9645,10 +9645,10 @@
         </is>
       </c>
       <c r="J186" s="7" t="n">
-        <v>14814</v>
+        <v>14557</v>
       </c>
       <c r="K186" s="8" t="n">
-        <v>617.25</v>
+        <v>606.5294117647059</v>
       </c>
     </row>
     <row r="187">
@@ -9730,7 +9730,7 @@
         </is>
       </c>
       <c r="G188" s="4" t="n">
-        <v>12949</v>
+        <v>12783</v>
       </c>
       <c r="H188" s="3" t="inlineStr">
         <is>
@@ -9743,10 +9743,10 @@
         </is>
       </c>
       <c r="J188" s="4" t="n">
-        <v>15539</v>
+        <v>15340</v>
       </c>
       <c r="K188" s="5" t="n">
-        <v>863.2666666666667</v>
+        <v>852.2</v>
       </c>
     </row>
     <row r="189">
@@ -9897,52 +9897,52 @@
       </c>
     </row>
     <row r="192">
-      <c r="A192" s="6" t="inlineStr">
+      <c r="A192" s="2" t="inlineStr">
         <is>
           <t>THURAIYUR</t>
         </is>
       </c>
-      <c r="B192" s="6" t="n">
+      <c r="B192" s="3" t="n">
         <v>146</v>
       </c>
-      <c r="C192" s="6" t="inlineStr">
+      <c r="C192" s="3" t="inlineStr">
         <is>
           <t>RAVISANKAR.M</t>
         </is>
       </c>
-      <c r="D192" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E192" s="6" t="inlineStr">
+      <c r="D192" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E192" s="3" t="inlineStr">
         <is>
           <t>E.SAROJA</t>
         </is>
       </c>
-      <c r="F192" s="6" t="inlineStr">
+      <c r="F192" s="3" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G192" s="7" t="n">
-        <v>7310</v>
-      </c>
-      <c r="H192" s="6" t="inlineStr">
-        <is>
-          <t>16/22</t>
-        </is>
-      </c>
-      <c r="I192" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J192" s="7" t="n">
-        <v>10051</v>
-      </c>
-      <c r="K192" s="8" t="n">
-        <v>456.875</v>
+      <c r="G192" s="4" t="n">
+        <v>7558</v>
+      </c>
+      <c r="H192" s="3" t="inlineStr">
+        <is>
+          <t>17/22</t>
+        </is>
+      </c>
+      <c r="I192" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J192" s="4" t="n">
+        <v>9781</v>
+      </c>
+      <c r="K192" s="5" t="n">
+        <v>444.5882352941176</v>
       </c>
     </row>
     <row r="193">
@@ -10024,11 +10024,11 @@
         </is>
       </c>
       <c r="G194" s="4" t="n">
-        <v>5601</v>
+        <v>6228</v>
       </c>
       <c r="H194" s="3" t="inlineStr">
         <is>
-          <t>18/22</t>
+          <t>19/22</t>
         </is>
       </c>
       <c r="I194" s="3" t="inlineStr">
@@ -10037,10 +10037,10 @@
         </is>
       </c>
       <c r="J194" s="4" t="n">
-        <v>6846</v>
+        <v>7211</v>
       </c>
       <c r="K194" s="5" t="n">
-        <v>311.1666666666667</v>
+        <v>327.7894736842105</v>
       </c>
     </row>
     <row r="195">
@@ -10073,11 +10073,11 @@
         </is>
       </c>
       <c r="G195" s="7" t="n">
-        <v>9128</v>
+        <v>11181</v>
       </c>
       <c r="H195" s="6" t="inlineStr">
         <is>
-          <t>11/21</t>
+          <t>12/21</t>
         </is>
       </c>
       <c r="I195" s="6" t="inlineStr">
@@ -10086,10 +10086,10 @@
         </is>
       </c>
       <c r="J195" s="7" t="n">
-        <v>17426</v>
+        <v>19567</v>
       </c>
       <c r="K195" s="8" t="n">
-        <v>829.8181818181819</v>
+        <v>931.75</v>
       </c>
     </row>
     <row r="196">
@@ -10122,11 +10122,11 @@
         </is>
       </c>
       <c r="G196" s="4" t="n">
-        <v>13879</v>
+        <v>15707</v>
       </c>
       <c r="H196" s="3" t="inlineStr">
         <is>
-          <t>11/22</t>
+          <t>12/22</t>
         </is>
       </c>
       <c r="I196" s="3" t="inlineStr">
@@ -10135,10 +10135,10 @@
         </is>
       </c>
       <c r="J196" s="4" t="n">
-        <v>27758</v>
+        <v>28796</v>
       </c>
       <c r="K196" s="5" t="n">
-        <v>1261.727272727273</v>
+        <v>1308.916666666667</v>
       </c>
     </row>
     <row r="197">
@@ -10171,11 +10171,11 @@
         </is>
       </c>
       <c r="G197" s="7" t="n">
-        <v>4883</v>
+        <v>4786</v>
       </c>
       <c r="H197" s="6" t="inlineStr">
         <is>
-          <t>22/24</t>
+          <t>24/24</t>
         </is>
       </c>
       <c r="I197" s="6" t="inlineStr">
@@ -10184,10 +10184,10 @@
         </is>
       </c>
       <c r="J197" s="7" t="n">
-        <v>5327</v>
+        <v>4786</v>
       </c>
       <c r="K197" s="8" t="n">
-        <v>221.9545454545455</v>
+        <v>199.4166666666667</v>
       </c>
     </row>
     <row r="198">
@@ -10220,11 +10220,11 @@
         </is>
       </c>
       <c r="G198" s="7" t="n">
-        <v>4243</v>
+        <v>5128</v>
       </c>
       <c r="H198" s="6" t="inlineStr">
         <is>
-          <t>10/21</t>
+          <t>11/21</t>
         </is>
       </c>
       <c r="I198" s="6" t="inlineStr">
@@ -10233,10 +10233,10 @@
         </is>
       </c>
       <c r="J198" s="7" t="n">
-        <v>8910</v>
+        <v>9790</v>
       </c>
       <c r="K198" s="8" t="n">
-        <v>424.3</v>
+        <v>466.1818181818182</v>
       </c>
     </row>
     <row r="199">
@@ -10318,11 +10318,11 @@
         </is>
       </c>
       <c r="G200" s="4" t="n">
-        <v>9959</v>
+        <v>11123</v>
       </c>
       <c r="H200" s="3" t="inlineStr">
         <is>
-          <t>26/28</t>
+          <t>27/28</t>
         </is>
       </c>
       <c r="I200" s="3" t="inlineStr">
@@ -10331,10 +10331,10 @@
         </is>
       </c>
       <c r="J200" s="4" t="n">
-        <v>10725</v>
+        <v>11535</v>
       </c>
       <c r="K200" s="5" t="n">
-        <v>383.0384615384615</v>
+        <v>411.962962962963</v>
       </c>
     </row>
     <row r="201">
@@ -10416,11 +10416,11 @@
         </is>
       </c>
       <c r="G202" s="7" t="n">
-        <v>4109</v>
+        <v>3663</v>
       </c>
       <c r="H202" s="6" t="inlineStr">
         <is>
-          <t>13/27</t>
+          <t>14/27</t>
         </is>
       </c>
       <c r="I202" s="6" t="inlineStr">
@@ -10429,10 +10429,10 @@
         </is>
       </c>
       <c r="J202" s="7" t="n">
-        <v>8534</v>
+        <v>7064</v>
       </c>
       <c r="K202" s="8" t="n">
-        <v>316.0769230769231</v>
+        <v>261.6428571428572</v>
       </c>
     </row>
     <row r="203">
@@ -10465,11 +10465,11 @@
         </is>
       </c>
       <c r="G203" s="4" t="n">
-        <v>39813</v>
+        <v>41023</v>
       </c>
       <c r="H203" s="3" t="inlineStr">
         <is>
-          <t>16/32</t>
+          <t>17/32</t>
         </is>
       </c>
       <c r="I203" s="3" t="inlineStr">
@@ -10478,10 +10478,10 @@
         </is>
       </c>
       <c r="J203" s="4" t="n">
-        <v>79626</v>
+        <v>77220</v>
       </c>
       <c r="K203" s="5" t="n">
-        <v>2488.3125</v>
+        <v>2413.117647058823</v>
       </c>
     </row>
     <row r="204">
@@ -10514,11 +10514,11 @@
         </is>
       </c>
       <c r="G204" s="7" t="n">
-        <v>9409</v>
+        <v>10976</v>
       </c>
       <c r="H204" s="6" t="inlineStr">
         <is>
-          <t>12/21</t>
+          <t>13/21</t>
         </is>
       </c>
       <c r="I204" s="6" t="inlineStr">
@@ -10527,10 +10527,10 @@
         </is>
       </c>
       <c r="J204" s="7" t="n">
-        <v>16466</v>
+        <v>17730</v>
       </c>
       <c r="K204" s="8" t="n">
-        <v>784.0833333333334</v>
+        <v>844.3076923076923</v>
       </c>
     </row>
     <row r="205">
@@ -10583,52 +10583,52 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="9" t="inlineStr">
+      <c r="A206" s="6" t="inlineStr">
         <is>
           <t>TIRUVADANAI</t>
         </is>
       </c>
-      <c r="B206" s="10" t="n">
+      <c r="B206" s="6" t="n">
         <v>210</v>
       </c>
-      <c r="C206" s="10" t="inlineStr">
+      <c r="C206" s="6" t="inlineStr">
         <is>
           <t>RAJEEV</t>
         </is>
       </c>
-      <c r="D206" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E206" s="10" t="inlineStr">
+      <c r="D206" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E206" s="6" t="inlineStr">
         <is>
           <t>RM. KARUMANICKAM</t>
         </is>
       </c>
-      <c r="F206" s="10" t="inlineStr">
+      <c r="F206" s="6" t="inlineStr">
         <is>
           <t>Indian National Congress</t>
         </is>
       </c>
-      <c r="G206" s="11" t="n">
-        <v>1875</v>
-      </c>
-      <c r="H206" s="10" t="inlineStr">
-        <is>
-          <t>21/27</t>
-        </is>
-      </c>
-      <c r="I206" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J206" s="11" t="n">
-        <v>2411</v>
-      </c>
-      <c r="K206" s="12" t="n">
-        <v>89.28571428571429</v>
+      <c r="G206" s="7" t="n">
+        <v>2533</v>
+      </c>
+      <c r="H206" s="6" t="inlineStr">
+        <is>
+          <t>22/27</t>
+        </is>
+      </c>
+      <c r="I206" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J206" s="7" t="n">
+        <v>3109</v>
+      </c>
+      <c r="K206" s="8" t="n">
+        <v>115.1363636363636</v>
       </c>
     </row>
     <row r="207">
@@ -10789,30 +10789,30 @@
       </c>
       <c r="C210" s="10" t="inlineStr">
         <is>
+          <t>JAYAKUMAR M.</t>
+        </is>
+      </c>
+      <c r="D210" s="10" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E210" s="10" t="inlineStr">
+        <is>
           <t>RADHAKRISHNAN K.</t>
         </is>
       </c>
-      <c r="D210" s="10" t="inlineStr">
+      <c r="F210" s="10" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E210" s="10" t="inlineStr">
-        <is>
-          <t>JAYAKUMAR M.</t>
-        </is>
-      </c>
-      <c r="F210" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
       <c r="G210" s="11" t="n">
-        <v>1602</v>
+        <v>542</v>
       </c>
       <c r="H210" s="10" t="inlineStr">
         <is>
-          <t>19/22</t>
+          <t>20/22</t>
         </is>
       </c>
       <c r="I210" s="10" t="inlineStr">
@@ -10821,59 +10821,59 @@
         </is>
       </c>
       <c r="J210" s="11" t="n">
-        <v>1855</v>
+        <v>596</v>
       </c>
       <c r="K210" s="12" t="n">
-        <v>84.31578947368421</v>
+        <v>27.1</v>
       </c>
     </row>
     <row r="211">
-      <c r="A211" s="9" t="inlineStr">
+      <c r="A211" s="13" t="inlineStr">
         <is>
           <t>ULUNDURPETTAI</t>
         </is>
       </c>
-      <c r="B211" s="10" t="n">
+      <c r="B211" s="14" t="n">
         <v>77</v>
       </c>
-      <c r="C211" s="10" t="inlineStr">
+      <c r="C211" s="14" t="inlineStr">
         <is>
           <t>VASANTHAVEL G R</t>
         </is>
       </c>
-      <c r="D211" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E211" s="10" t="inlineStr">
+      <c r="D211" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E211" s="14" t="inlineStr">
         <is>
           <t>KUMARAGURU R</t>
         </is>
       </c>
-      <c r="F211" s="10" t="inlineStr">
+      <c r="F211" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G211" s="11" t="n">
-        <v>644</v>
-      </c>
-      <c r="H211" s="10" t="inlineStr">
-        <is>
-          <t>15/27</t>
-        </is>
-      </c>
-      <c r="I211" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J211" s="11" t="n">
-        <v>1159</v>
-      </c>
-      <c r="K211" s="12" t="n">
-        <v>42.93333333333333</v>
+      <c r="G211" s="15" t="n">
+        <v>42</v>
+      </c>
+      <c r="H211" s="14" t="inlineStr">
+        <is>
+          <t>16/27</t>
+        </is>
+      </c>
+      <c r="I211" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J211" s="15" t="n">
+        <v>71</v>
+      </c>
+      <c r="K211" s="16" t="n">
+        <v>2.625</v>
       </c>
     </row>
     <row r="212">
@@ -10906,11 +10906,11 @@
         </is>
       </c>
       <c r="G212" s="7" t="n">
-        <v>1858</v>
+        <v>1828</v>
       </c>
       <c r="H212" s="6" t="inlineStr">
         <is>
-          <t>12/25</t>
+          <t>13/25</t>
         </is>
       </c>
       <c r="I212" s="6" t="inlineStr">
@@ -10919,10 +10919,10 @@
         </is>
       </c>
       <c r="J212" s="7" t="n">
-        <v>3871</v>
+        <v>3515</v>
       </c>
       <c r="K212" s="8" t="n">
-        <v>154.8333333333333</v>
+        <v>140.6153846153846</v>
       </c>
     </row>
     <row r="213">
@@ -11200,11 +11200,11 @@
         </is>
       </c>
       <c r="G218" s="7" t="n">
-        <v>3884</v>
+        <v>4254</v>
       </c>
       <c r="H218" s="6" t="inlineStr">
         <is>
-          <t>15/22</t>
+          <t>16/22</t>
         </is>
       </c>
       <c r="I218" s="6" t="inlineStr">
@@ -11213,10 +11213,10 @@
         </is>
       </c>
       <c r="J218" s="7" t="n">
-        <v>5697</v>
+        <v>5849</v>
       </c>
       <c r="K218" s="8" t="n">
-        <v>258.9333333333333</v>
+        <v>265.875</v>
       </c>
     </row>
     <row r="219">
@@ -11249,11 +11249,11 @@
         </is>
       </c>
       <c r="G219" s="7" t="n">
-        <v>6449</v>
+        <v>7074</v>
       </c>
       <c r="H219" s="6" t="inlineStr">
         <is>
-          <t>16/23</t>
+          <t>17/23</t>
         </is>
       </c>
       <c r="I219" s="6" t="inlineStr">
@@ -11262,59 +11262,59 @@
         </is>
       </c>
       <c r="J219" s="7" t="n">
-        <v>9270</v>
+        <v>9571</v>
       </c>
       <c r="K219" s="8" t="n">
-        <v>403.0625</v>
+        <v>416.1176470588235</v>
       </c>
     </row>
     <row r="220">
-      <c r="A220" s="6" t="inlineStr">
+      <c r="A220" s="2" t="inlineStr">
         <is>
           <t>VEDARANYAM</t>
         </is>
       </c>
-      <c r="B220" s="6" t="n">
+      <c r="B220" s="3" t="n">
         <v>165</v>
       </c>
-      <c r="C220" s="6" t="inlineStr">
+      <c r="C220" s="3" t="inlineStr">
         <is>
           <t>MANIAN. O.S</t>
         </is>
       </c>
-      <c r="D220" s="6" t="inlineStr">
+      <c r="D220" s="3" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E220" s="6" t="inlineStr">
+      <c r="E220" s="3" t="inlineStr">
         <is>
           <t>PUGAZHENDI. M</t>
         </is>
       </c>
-      <c r="F220" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G220" s="7" t="n">
-        <v>5884</v>
-      </c>
-      <c r="H220" s="6" t="inlineStr">
-        <is>
-          <t>13/18</t>
-        </is>
-      </c>
-      <c r="I220" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J220" s="7" t="n">
-        <v>8147</v>
-      </c>
-      <c r="K220" s="8" t="n">
-        <v>452.6153846153846</v>
+      <c r="F220" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G220" s="4" t="n">
+        <v>6721</v>
+      </c>
+      <c r="H220" s="3" t="inlineStr">
+        <is>
+          <t>14/18</t>
+        </is>
+      </c>
+      <c r="I220" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J220" s="4" t="n">
+        <v>8641</v>
+      </c>
+      <c r="K220" s="5" t="n">
+        <v>480.0714285714286</v>
       </c>
     </row>
     <row r="221">
@@ -11347,11 +11347,11 @@
         </is>
       </c>
       <c r="G221" s="7" t="n">
-        <v>6926</v>
+        <v>7314</v>
       </c>
       <c r="H221" s="6" t="inlineStr">
         <is>
-          <t>16/24</t>
+          <t>17/24</t>
         </is>
       </c>
       <c r="I221" s="6" t="inlineStr">
@@ -11360,10 +11360,10 @@
         </is>
       </c>
       <c r="J221" s="7" t="n">
-        <v>10389</v>
+        <v>10326</v>
       </c>
       <c r="K221" s="8" t="n">
-        <v>432.875</v>
+        <v>430.2352941176471</v>
       </c>
     </row>
     <row r="222">
@@ -11396,11 +11396,11 @@
         </is>
       </c>
       <c r="G222" s="7" t="n">
-        <v>3899</v>
+        <v>3700</v>
       </c>
       <c r="H222" s="6" t="inlineStr">
         <is>
-          <t>15/23</t>
+          <t>16/23</t>
         </is>
       </c>
       <c r="I222" s="6" t="inlineStr">
@@ -11409,10 +11409,10 @@
         </is>
       </c>
       <c r="J222" s="7" t="n">
-        <v>5978</v>
+        <v>5319</v>
       </c>
       <c r="K222" s="8" t="n">
-        <v>259.9333333333333</v>
+        <v>231.25</v>
       </c>
     </row>
     <row r="223">
@@ -11445,11 +11445,11 @@
         </is>
       </c>
       <c r="G223" s="4" t="n">
-        <v>27350</v>
+        <v>28238</v>
       </c>
       <c r="H223" s="3" t="inlineStr">
         <is>
-          <t>18/23</t>
+          <t>19/23</t>
         </is>
       </c>
       <c r="I223" s="3" t="inlineStr">
@@ -11458,10 +11458,10 @@
         </is>
       </c>
       <c r="J223" s="4" t="n">
-        <v>34947</v>
+        <v>34183</v>
       </c>
       <c r="K223" s="5" t="n">
-        <v>1519.444444444444</v>
+        <v>1486.210526315789</v>
       </c>
     </row>
     <row r="224">
@@ -11494,11 +11494,11 @@
         </is>
       </c>
       <c r="G224" s="7" t="n">
-        <v>3229</v>
+        <v>4141</v>
       </c>
       <c r="H224" s="6" t="inlineStr">
         <is>
-          <t>16/20</t>
+          <t>17/20</t>
         </is>
       </c>
       <c r="I224" s="6" t="inlineStr">
@@ -11507,59 +11507,59 @@
         </is>
       </c>
       <c r="J224" s="7" t="n">
-        <v>4036</v>
+        <v>4872</v>
       </c>
       <c r="K224" s="8" t="n">
-        <v>201.8125</v>
+        <v>243.5882352941177</v>
       </c>
     </row>
     <row r="225">
-      <c r="A225" s="13" t="inlineStr">
+      <c r="A225" s="9" t="inlineStr">
         <is>
           <t>VEPPANAHALLI</t>
         </is>
       </c>
-      <c r="B225" s="14" t="n">
+      <c r="B225" s="10" t="n">
         <v>54</v>
       </c>
-      <c r="C225" s="14" t="inlineStr">
+      <c r="C225" s="10" t="inlineStr">
         <is>
           <t>SRINIVASAN.P.S</t>
         </is>
       </c>
-      <c r="D225" s="14" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E225" s="14" t="inlineStr">
+      <c r="D225" s="10" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E225" s="10" t="inlineStr">
         <is>
           <t>MUNUSAMY.K.P</t>
         </is>
       </c>
-      <c r="F225" s="14" t="inlineStr">
+      <c r="F225" s="10" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G225" s="15" t="n">
-        <v>333</v>
-      </c>
-      <c r="H225" s="14" t="inlineStr">
-        <is>
-          <t>19/25</t>
-        </is>
-      </c>
-      <c r="I225" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J225" s="15" t="n">
-        <v>438</v>
-      </c>
-      <c r="K225" s="16" t="n">
-        <v>17.52631578947368</v>
+      <c r="G225" s="11" t="n">
+        <v>688</v>
+      </c>
+      <c r="H225" s="10" t="inlineStr">
+        <is>
+          <t>20/25</t>
+        </is>
+      </c>
+      <c r="I225" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J225" s="11" t="n">
+        <v>860</v>
+      </c>
+      <c r="K225" s="12" t="n">
+        <v>34.4</v>
       </c>
     </row>
     <row r="226">
@@ -11641,7 +11641,7 @@
         </is>
       </c>
       <c r="G227" s="4" t="n">
-        <v>7697</v>
+        <v>8216</v>
       </c>
       <c r="H227" s="3" t="inlineStr">
         <is>
@@ -11654,10 +11654,10 @@
         </is>
       </c>
       <c r="J227" s="4" t="n">
-        <v>8552</v>
+        <v>9129</v>
       </c>
       <c r="K227" s="5" t="n">
-        <v>427.6111111111111</v>
+        <v>456.4444444444445</v>
       </c>
     </row>
     <row r="228">
@@ -11739,11 +11739,11 @@
         </is>
       </c>
       <c r="G229" s="4" t="n">
-        <v>14495</v>
+        <v>15461</v>
       </c>
       <c r="H229" s="3" t="inlineStr">
         <is>
-          <t>15/19</t>
+          <t>16/19</t>
         </is>
       </c>
       <c r="I229" s="3" t="inlineStr">
@@ -11755,7 +11755,7 @@
         <v>18360</v>
       </c>
       <c r="K229" s="5" t="n">
-        <v>966.3333333333334</v>
+        <v>966.3125</v>
       </c>
     </row>
     <row r="230">
@@ -11837,11 +11837,11 @@
         </is>
       </c>
       <c r="G231" s="4" t="n">
-        <v>40612</v>
+        <v>44006</v>
       </c>
       <c r="H231" s="3" t="inlineStr">
         <is>
-          <t>13/20</t>
+          <t>14/20</t>
         </is>
       </c>
       <c r="I231" s="3" t="inlineStr">
@@ -11850,10 +11850,10 @@
         </is>
       </c>
       <c r="J231" s="4" t="n">
-        <v>62480</v>
+        <v>62866</v>
       </c>
       <c r="K231" s="5" t="n">
-        <v>3124</v>
+        <v>3143.285714285714</v>
       </c>
     </row>
     <row r="232">
@@ -11886,11 +11886,11 @@
         </is>
       </c>
       <c r="G232" s="7" t="n">
-        <v>4064</v>
+        <v>5677</v>
       </c>
       <c r="H232" s="6" t="inlineStr">
         <is>
-          <t>12/21</t>
+          <t>13/21</t>
         </is>
       </c>
       <c r="I232" s="6" t="inlineStr">
@@ -11899,10 +11899,10 @@
         </is>
       </c>
       <c r="J232" s="7" t="n">
-        <v>7112</v>
+        <v>9171</v>
       </c>
       <c r="K232" s="8" t="n">
-        <v>338.6666666666667</v>
+        <v>436.6923076923077</v>
       </c>
     </row>
     <row r="233">
@@ -11984,11 +11984,11 @@
         </is>
       </c>
       <c r="G234" s="7" t="n">
-        <v>3301</v>
+        <v>3327</v>
       </c>
       <c r="H234" s="6" t="inlineStr">
         <is>
-          <t>15/23</t>
+          <t>16/23</t>
         </is>
       </c>
       <c r="I234" s="6" t="inlineStr">
@@ -11997,10 +11997,10 @@
         </is>
       </c>
       <c r="J234" s="7" t="n">
-        <v>5062</v>
+        <v>4783</v>
       </c>
       <c r="K234" s="8" t="n">
-        <v>220.0666666666667</v>
+        <v>207.9375</v>
       </c>
     </row>
     <row r="235">
@@ -12033,11 +12033,11 @@
         </is>
       </c>
       <c r="G235" s="11" t="n">
-        <v>1480</v>
+        <v>1190</v>
       </c>
       <c r="H235" s="10" t="inlineStr">
         <is>
-          <t>13/24</t>
+          <t>14/24</t>
         </is>
       </c>
       <c r="I235" s="10" t="inlineStr">
@@ -12046,10 +12046,10 @@
         </is>
       </c>
       <c r="J235" s="11" t="n">
-        <v>2732</v>
+        <v>2040</v>
       </c>
       <c r="K235" s="12" t="n">
-        <v>113.8461538461538</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update election results snapshot (76.2% counted)
TVK 108, DMK 59, AIADMK 44. 14 declared total — 6 this round including
SRIVAIKUNTAM (TVK), TIRUNELVELI (TVK), TIRUCHIRAPPALLI WEST (DMK).
KUMBAKONAM last true knife-edge at 86 votes with 3 rounds left.

https://claude.ai/code/session_01MizbUy44JG5sXyvaf3Wekb
</commit_message>
<xml_diff>
--- a/tn_election_results_may2026.xlsx
+++ b/tn_election_results_may2026.xlsx
@@ -616,11 +616,11 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>20771</v>
+        <v>21617</v>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>15/31</t>
+          <t>16/31</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -629,10 +629,10 @@
         </is>
       </c>
       <c r="J2" s="4" t="n">
-        <v>42927</v>
+        <v>41883</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>1384.733333333333</v>
+        <v>1351.0625</v>
       </c>
     </row>
     <row r="3">
@@ -665,11 +665,11 @@
         </is>
       </c>
       <c r="G3" s="7" t="n">
-        <v>5727</v>
+        <v>6581</v>
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
-          <t>11/20</t>
+          <t>12/20</t>
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr">
@@ -678,10 +678,10 @@
         </is>
       </c>
       <c r="J3" s="7" t="n">
-        <v>10413</v>
+        <v>10968</v>
       </c>
       <c r="K3" s="8" t="n">
-        <v>520.6363636363636</v>
+        <v>548.4166666666666</v>
       </c>
     </row>
     <row r="4">
@@ -714,11 +714,11 @@
         </is>
       </c>
       <c r="G4" s="4" t="n">
-        <v>6654</v>
+        <v>6721</v>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>20/24</t>
+          <t>21/24</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -727,10 +727,10 @@
         </is>
       </c>
       <c r="J4" s="4" t="n">
-        <v>7985</v>
+        <v>7681</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>332.7</v>
+        <v>320.047619047619</v>
       </c>
     </row>
     <row r="5">
@@ -861,11 +861,11 @@
         </is>
       </c>
       <c r="G7" s="7" t="n">
-        <v>3750</v>
+        <v>9595</v>
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>13/22</t>
+          <t>14/22</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
@@ -874,10 +874,10 @@
         </is>
       </c>
       <c r="J7" s="7" t="n">
-        <v>6346</v>
+        <v>15078</v>
       </c>
       <c r="K7" s="8" t="n">
-        <v>288.4615384615385</v>
+        <v>685.3571428571429</v>
       </c>
     </row>
     <row r="8">
@@ -910,11 +910,11 @@
         </is>
       </c>
       <c r="G8" s="7" t="n">
-        <v>7584</v>
+        <v>7134</v>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>14/22</t>
+          <t>15/22</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
@@ -923,10 +923,10 @@
         </is>
       </c>
       <c r="J8" s="7" t="n">
-        <v>11918</v>
+        <v>10463</v>
       </c>
       <c r="K8" s="8" t="n">
-        <v>541.7142857142857</v>
+        <v>475.6000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -959,11 +959,11 @@
         </is>
       </c>
       <c r="G9" s="7" t="n">
-        <v>3571</v>
+        <v>4266</v>
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>17/25</t>
+          <t>18/25</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
@@ -972,10 +972,10 @@
         </is>
       </c>
       <c r="J9" s="7" t="n">
-        <v>5251</v>
+        <v>5925</v>
       </c>
       <c r="K9" s="8" t="n">
-        <v>210.0588235294118</v>
+        <v>237</v>
       </c>
     </row>
     <row r="10">
@@ -1302,11 +1302,11 @@
         </is>
       </c>
       <c r="G16" s="4" t="n">
-        <v>16312</v>
+        <v>18192</v>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>12/23</t>
+          <t>13/23</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
@@ -1315,10 +1315,10 @@
         </is>
       </c>
       <c r="J16" s="4" t="n">
-        <v>31265</v>
+        <v>32186</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>1359.333333333333</v>
+        <v>1399.384615384615</v>
       </c>
     </row>
     <row r="17">
@@ -1449,11 +1449,11 @@
         </is>
       </c>
       <c r="G19" s="4" t="n">
-        <v>20123</v>
+        <v>21702</v>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>17/25</t>
+          <t>18/25</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -1462,10 +1462,10 @@
         </is>
       </c>
       <c r="J19" s="4" t="n">
-        <v>29593</v>
+        <v>30142</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>1183.705882352941</v>
+        <v>1205.666666666667</v>
       </c>
     </row>
     <row r="20">
@@ -1498,11 +1498,11 @@
         </is>
       </c>
       <c r="G20" s="4" t="n">
-        <v>13481</v>
+        <v>13950</v>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>20/22</t>
+          <t>21/23</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
@@ -1511,10 +1511,10 @@
         </is>
       </c>
       <c r="J20" s="4" t="n">
-        <v>14829</v>
+        <v>15279</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>674.05</v>
+        <v>664.2857142857143</v>
       </c>
     </row>
     <row r="21">
@@ -1694,11 +1694,11 @@
         </is>
       </c>
       <c r="G24" s="7" t="n">
-        <v>8409</v>
+        <v>7238</v>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>13/22</t>
+          <t>14/22</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr">
@@ -1707,59 +1707,59 @@
         </is>
       </c>
       <c r="J24" s="7" t="n">
-        <v>14231</v>
+        <v>11374</v>
       </c>
       <c r="K24" s="8" t="n">
-        <v>646.8461538461538</v>
+        <v>517</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="9" t="inlineStr">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>BHAVANISAGAR</t>
         </is>
       </c>
-      <c r="B25" s="10" t="n">
+      <c r="B25" s="6" t="n">
         <v>107</v>
       </c>
-      <c r="C25" s="10" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>V.P.TAMILSELVI</t>
         </is>
       </c>
-      <c r="D25" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E25" s="10" t="inlineStr">
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
         <is>
           <t>A.BANNARI</t>
         </is>
       </c>
-      <c r="F25" s="10" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G25" s="11" t="n">
-        <v>2483</v>
-      </c>
-      <c r="H25" s="10" t="inlineStr">
-        <is>
-          <t>20/24</t>
-        </is>
-      </c>
-      <c r="I25" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J25" s="11" t="n">
-        <v>2980</v>
-      </c>
-      <c r="K25" s="12" t="n">
-        <v>124.15</v>
+      <c r="G25" s="7" t="n">
+        <v>2720</v>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>21/24</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J25" s="7" t="n">
+        <v>3109</v>
+      </c>
+      <c r="K25" s="8" t="n">
+        <v>129.5238095238095</v>
       </c>
     </row>
     <row r="26">
@@ -1792,11 +1792,11 @@
         </is>
       </c>
       <c r="G26" s="7" t="n">
-        <v>5797</v>
+        <v>7166</v>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>15/22</t>
+          <t>16/22</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
@@ -1805,10 +1805,10 @@
         </is>
       </c>
       <c r="J26" s="7" t="n">
-        <v>8502</v>
+        <v>9853</v>
       </c>
       <c r="K26" s="8" t="n">
-        <v>386.4666666666667</v>
+        <v>447.875</v>
       </c>
     </row>
     <row r="27">
@@ -1841,11 +1841,11 @@
         </is>
       </c>
       <c r="G27" s="7" t="n">
-        <v>3589</v>
+        <v>3697</v>
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>17/25</t>
+          <t>18/25</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
@@ -1854,10 +1854,10 @@
         </is>
       </c>
       <c r="J27" s="7" t="n">
-        <v>5278</v>
+        <v>5135</v>
       </c>
       <c r="K27" s="8" t="n">
-        <v>211.1176470588235</v>
+        <v>205.3888888888889</v>
       </c>
     </row>
     <row r="28">
@@ -1890,11 +1890,11 @@
         </is>
       </c>
       <c r="G28" s="4" t="n">
-        <v>15321</v>
+        <v>15969</v>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>14/36</t>
+          <t>15/36</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
@@ -1903,10 +1903,10 @@
         </is>
       </c>
       <c r="J28" s="4" t="n">
-        <v>39397</v>
+        <v>38326</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>1094.357142857143</v>
+        <v>1064.6</v>
       </c>
     </row>
     <row r="29">
@@ -2135,11 +2135,11 @@
         </is>
       </c>
       <c r="G33" s="7" t="n">
-        <v>4757</v>
+        <v>5033</v>
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>15/22</t>
+          <t>16/22</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
@@ -2148,10 +2148,10 @@
         </is>
       </c>
       <c r="J33" s="7" t="n">
-        <v>6977</v>
+        <v>6920</v>
       </c>
       <c r="K33" s="8" t="n">
-        <v>317.1333333333334</v>
+        <v>314.5625</v>
       </c>
     </row>
     <row r="34">
@@ -2204,52 +2204,52 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="9" t="inlineStr">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t>COIMBATORE (SOUTH)</t>
         </is>
       </c>
-      <c r="B35" s="10" t="n">
+      <c r="B35" s="6" t="n">
         <v>120</v>
       </c>
-      <c r="C35" s="10" t="inlineStr">
+      <c r="C35" s="6" t="inlineStr">
         <is>
           <t>V SENTHILBALAJI</t>
         </is>
       </c>
-      <c r="D35" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E35" s="10" t="inlineStr">
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="inlineStr">
         <is>
           <t>V. SENTHILKUMAR</t>
         </is>
       </c>
-      <c r="F35" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G35" s="11" t="n">
-        <v>1231</v>
-      </c>
-      <c r="H35" s="10" t="inlineStr">
-        <is>
-          <t>12/20</t>
-        </is>
-      </c>
-      <c r="I35" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J35" s="11" t="n">
-        <v>2052</v>
-      </c>
-      <c r="K35" s="12" t="n">
-        <v>102.5833333333333</v>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="n">
+        <v>2675</v>
+      </c>
+      <c r="H35" s="6" t="inlineStr">
+        <is>
+          <t>13/20</t>
+        </is>
+      </c>
+      <c r="I35" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J35" s="7" t="n">
+        <v>4115</v>
+      </c>
+      <c r="K35" s="8" t="n">
+        <v>205.7692307692308</v>
       </c>
     </row>
     <row r="36">
@@ -2380,11 +2380,11 @@
         </is>
       </c>
       <c r="G38" s="4" t="n">
-        <v>11355</v>
+        <v>13034</v>
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>15/19</t>
+          <t>16/19</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
@@ -2393,59 +2393,59 @@
         </is>
       </c>
       <c r="J38" s="4" t="n">
-        <v>14383</v>
+        <v>15478</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>757</v>
+        <v>814.625</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="6" t="inlineStr">
+      <c r="A39" s="9" t="inlineStr">
         <is>
           <t>CUMBUM</t>
         </is>
       </c>
-      <c r="B39" s="6" t="n">
+      <c r="B39" s="10" t="n">
         <v>201</v>
       </c>
-      <c r="C39" s="6" t="inlineStr">
+      <c r="C39" s="10" t="inlineStr">
         <is>
           <t>JEGANATHMISHRA PLA</t>
         </is>
       </c>
-      <c r="D39" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E39" s="6" t="inlineStr">
+      <c r="D39" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E39" s="10" t="inlineStr">
         <is>
           <t>ERAMAKRISHNAN N</t>
         </is>
       </c>
-      <c r="F39" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G39" s="7" t="n">
-        <v>2099</v>
-      </c>
-      <c r="H39" s="6" t="inlineStr">
-        <is>
-          <t>13/25</t>
-        </is>
-      </c>
-      <c r="I39" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J39" s="7" t="n">
-        <v>4037</v>
-      </c>
-      <c r="K39" s="8" t="n">
-        <v>161.4615384615385</v>
+      <c r="F39" s="10" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G39" s="11" t="n">
+        <v>1605</v>
+      </c>
+      <c r="H39" s="10" t="inlineStr">
+        <is>
+          <t>14/25</t>
+        </is>
+      </c>
+      <c r="I39" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J39" s="11" t="n">
+        <v>2866</v>
+      </c>
+      <c r="K39" s="12" t="n">
+        <v>114.6428571428571</v>
       </c>
     </row>
     <row r="40">
@@ -2478,11 +2478,11 @@
         </is>
       </c>
       <c r="G40" s="4" t="n">
-        <v>14116</v>
+        <v>15442</v>
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>21/23</t>
+          <t>22/23</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
@@ -2491,10 +2491,10 @@
         </is>
       </c>
       <c r="J40" s="4" t="n">
-        <v>15460</v>
+        <v>16144</v>
       </c>
       <c r="K40" s="5" t="n">
-        <v>672.1904761904761</v>
+        <v>701.9090909090909</v>
       </c>
     </row>
     <row r="41">
@@ -2547,52 +2547,52 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="9" t="inlineStr">
+      <c r="A42" s="13" t="inlineStr">
         <is>
           <t>DINDIGUL</t>
         </is>
       </c>
-      <c r="B42" s="10" t="n">
+      <c r="B42" s="14" t="n">
         <v>132</v>
       </c>
-      <c r="C42" s="10" t="inlineStr">
+      <c r="C42" s="14" t="inlineStr">
         <is>
           <t>SENTHILKUMAR. I.P</t>
         </is>
       </c>
-      <c r="D42" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E42" s="10" t="inlineStr">
+      <c r="D42" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E42" s="14" t="inlineStr">
         <is>
           <t>NAZEER RAJA. G</t>
         </is>
       </c>
-      <c r="F42" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G42" s="11" t="n">
-        <v>838</v>
-      </c>
-      <c r="H42" s="10" t="inlineStr">
-        <is>
-          <t>21/24</t>
-        </is>
-      </c>
-      <c r="I42" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J42" s="11" t="n">
-        <v>958</v>
-      </c>
-      <c r="K42" s="12" t="n">
-        <v>39.90476190476191</v>
+      <c r="F42" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G42" s="15" t="n">
+        <v>279</v>
+      </c>
+      <c r="H42" s="14" t="inlineStr">
+        <is>
+          <t>22/26</t>
+        </is>
+      </c>
+      <c r="I42" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J42" s="15" t="n">
+        <v>330</v>
+      </c>
+      <c r="K42" s="16" t="n">
+        <v>12.68181818181818</v>
       </c>
     </row>
     <row r="43">
@@ -2625,11 +2625,11 @@
         </is>
       </c>
       <c r="G43" s="4" t="n">
-        <v>21650</v>
+        <v>24744</v>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>9/18</t>
+          <t>10/18</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
@@ -2638,10 +2638,10 @@
         </is>
       </c>
       <c r="J43" s="4" t="n">
-        <v>43300</v>
+        <v>44539</v>
       </c>
       <c r="K43" s="5" t="n">
-        <v>2405.555555555556</v>
+        <v>2474.4</v>
       </c>
     </row>
     <row r="44">
@@ -2674,7 +2674,7 @@
         </is>
       </c>
       <c r="G44" s="4" t="n">
-        <v>90278</v>
+        <v>92619</v>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
@@ -2687,10 +2687,10 @@
         </is>
       </c>
       <c r="J44" s="4" t="n">
-        <v>98128</v>
+        <v>100673</v>
       </c>
       <c r="K44" s="5" t="n">
-        <v>3925.130434782609</v>
+        <v>4026.913043478261</v>
       </c>
     </row>
     <row r="45">
@@ -2723,11 +2723,11 @@
         </is>
       </c>
       <c r="G45" s="4" t="n">
-        <v>13096</v>
+        <v>11336</v>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>13/15</t>
+          <t>14/15</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
@@ -2736,10 +2736,10 @@
         </is>
       </c>
       <c r="J45" s="4" t="n">
-        <v>15111</v>
+        <v>12146</v>
       </c>
       <c r="K45" s="5" t="n">
-        <v>1007.384615384615</v>
+        <v>809.7142857142857</v>
       </c>
     </row>
     <row r="46">
@@ -2772,11 +2772,11 @@
         </is>
       </c>
       <c r="G46" s="4" t="n">
-        <v>23678</v>
+        <v>23966</v>
       </c>
       <c r="H46" s="3" t="inlineStr">
         <is>
-          <t>19/20</t>
+          <t>20/20</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
@@ -2785,10 +2785,10 @@
         </is>
       </c>
       <c r="J46" s="4" t="n">
-        <v>24924</v>
+        <v>23966</v>
       </c>
       <c r="K46" s="5" t="n">
-        <v>1246.210526315789</v>
+        <v>1198.3</v>
       </c>
     </row>
     <row r="47">
@@ -2821,11 +2821,11 @@
         </is>
       </c>
       <c r="G47" s="4" t="n">
-        <v>21263</v>
+        <v>21517</v>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>17/24</t>
+          <t>18/24</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
@@ -2834,10 +2834,10 @@
         </is>
       </c>
       <c r="J47" s="4" t="n">
-        <v>30018</v>
+        <v>28689</v>
       </c>
       <c r="K47" s="5" t="n">
-        <v>1250.764705882353</v>
+        <v>1195.388888888889</v>
       </c>
     </row>
     <row r="48">
@@ -2968,11 +2968,11 @@
         </is>
       </c>
       <c r="G50" s="7" t="n">
-        <v>8430</v>
+        <v>9208</v>
       </c>
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>10/23</t>
+          <t>11/23</t>
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr">
@@ -2981,10 +2981,10 @@
         </is>
       </c>
       <c r="J50" s="7" t="n">
-        <v>19389</v>
+        <v>19253</v>
       </c>
       <c r="K50" s="8" t="n">
-        <v>843</v>
+        <v>837.0909090909091</v>
       </c>
     </row>
     <row r="51">
@@ -3026,7 +3026,7 @@
       </c>
       <c r="I51" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J51" s="4" t="n">
@@ -3086,52 +3086,52 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="6" t="inlineStr">
+      <c r="A53" s="2" t="inlineStr">
         <is>
           <t>GUDIYATTAM</t>
         </is>
       </c>
-      <c r="B53" s="6" t="n">
+      <c r="B53" s="3" t="n">
         <v>46</v>
       </c>
-      <c r="C53" s="6" t="inlineStr">
+      <c r="C53" s="3" t="inlineStr">
         <is>
           <t>K.SINDU</t>
         </is>
       </c>
-      <c r="D53" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E53" s="6" t="inlineStr">
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
         <is>
           <t>K.B.PRADAP</t>
         </is>
       </c>
-      <c r="F53" s="6" t="inlineStr">
+      <c r="F53" s="3" t="inlineStr">
         <is>
           <t>Desiya Murpokku Dravida Kazhagam</t>
         </is>
       </c>
-      <c r="G53" s="7" t="n">
-        <v>4847</v>
-      </c>
-      <c r="H53" s="6" t="inlineStr">
-        <is>
-          <t>18/23</t>
-        </is>
-      </c>
-      <c r="I53" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J53" s="7" t="n">
-        <v>6193</v>
-      </c>
-      <c r="K53" s="8" t="n">
-        <v>269.2777777777778</v>
+      <c r="G53" s="4" t="n">
+        <v>6105</v>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>19/23</t>
+        </is>
+      </c>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J53" s="4" t="n">
+        <v>7390</v>
+      </c>
+      <c r="K53" s="5" t="n">
+        <v>321.3157894736842</v>
       </c>
     </row>
     <row r="54">
@@ -3164,11 +3164,11 @@
         </is>
       </c>
       <c r="G54" s="4" t="n">
-        <v>21752</v>
+        <v>22596</v>
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>17/25</t>
+          <t>18/25</t>
         </is>
       </c>
       <c r="I54" s="3" t="inlineStr">
@@ -3177,10 +3177,10 @@
         </is>
       </c>
       <c r="J54" s="4" t="n">
-        <v>31988</v>
+        <v>31383</v>
       </c>
       <c r="K54" s="5" t="n">
-        <v>1279.529411764706</v>
+        <v>1255.333333333333</v>
       </c>
     </row>
     <row r="55">
@@ -3360,11 +3360,11 @@
         </is>
       </c>
       <c r="G58" s="4" t="n">
-        <v>13449</v>
+        <v>14778</v>
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>19/23</t>
+          <t>20/23</t>
         </is>
       </c>
       <c r="I58" s="3" t="inlineStr">
@@ -3373,10 +3373,10 @@
         </is>
       </c>
       <c r="J58" s="4" t="n">
-        <v>16280</v>
+        <v>16995</v>
       </c>
       <c r="K58" s="5" t="n">
-        <v>707.8421052631579</v>
+        <v>738.9</v>
       </c>
     </row>
     <row r="59">
@@ -3409,11 +3409,11 @@
         </is>
       </c>
       <c r="G59" s="4" t="n">
-        <v>14669</v>
+        <v>15081</v>
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>18/21</t>
+          <t>19/21</t>
         </is>
       </c>
       <c r="I59" s="3" t="inlineStr">
@@ -3422,10 +3422,10 @@
         </is>
       </c>
       <c r="J59" s="4" t="n">
-        <v>17114</v>
+        <v>16668</v>
       </c>
       <c r="K59" s="5" t="n">
-        <v>814.9444444444445</v>
+        <v>793.7368421052631</v>
       </c>
     </row>
     <row r="60">
@@ -3458,11 +3458,11 @@
         </is>
       </c>
       <c r="G60" s="11" t="n">
-        <v>1600</v>
+        <v>1459</v>
       </c>
       <c r="H60" s="10" t="inlineStr">
         <is>
-          <t>16/26</t>
+          <t>17/26</t>
         </is>
       </c>
       <c r="I60" s="10" t="inlineStr">
@@ -3471,10 +3471,10 @@
         </is>
       </c>
       <c r="J60" s="11" t="n">
-        <v>2600</v>
+        <v>2231</v>
       </c>
       <c r="K60" s="12" t="n">
-        <v>100</v>
+        <v>85.82352941176471</v>
       </c>
     </row>
     <row r="61">
@@ -3556,11 +3556,11 @@
         </is>
       </c>
       <c r="G62" s="7" t="n">
-        <v>2185</v>
+        <v>2180</v>
       </c>
       <c r="H62" s="6" t="inlineStr">
         <is>
-          <t>16/27</t>
+          <t>17/27</t>
         </is>
       </c>
       <c r="I62" s="6" t="inlineStr">
@@ -3569,10 +3569,10 @@
         </is>
       </c>
       <c r="J62" s="7" t="n">
-        <v>3687</v>
+        <v>3462</v>
       </c>
       <c r="K62" s="8" t="n">
-        <v>136.5625</v>
+        <v>128.2352941176471</v>
       </c>
     </row>
     <row r="63">
@@ -3752,11 +3752,11 @@
         </is>
       </c>
       <c r="G66" s="4" t="n">
-        <v>26481</v>
+        <v>28296</v>
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>15/28</t>
+          <t>16/28</t>
         </is>
       </c>
       <c r="I66" s="3" t="inlineStr">
@@ -3765,10 +3765,10 @@
         </is>
       </c>
       <c r="J66" s="4" t="n">
-        <v>49431</v>
+        <v>49518</v>
       </c>
       <c r="K66" s="5" t="n">
-        <v>1765.4</v>
+        <v>1768.5</v>
       </c>
     </row>
     <row r="67">
@@ -3801,11 +3801,11 @@
         </is>
       </c>
       <c r="G67" s="7" t="n">
-        <v>5447</v>
+        <v>4677</v>
       </c>
       <c r="H67" s="6" t="inlineStr">
         <is>
-          <t>13/21</t>
+          <t>14/21</t>
         </is>
       </c>
       <c r="I67" s="6" t="inlineStr">
@@ -3814,10 +3814,10 @@
         </is>
       </c>
       <c r="J67" s="7" t="n">
-        <v>8799</v>
+        <v>7016</v>
       </c>
       <c r="K67" s="8" t="n">
-        <v>419</v>
+        <v>334.0714285714286</v>
       </c>
     </row>
     <row r="68">
@@ -3997,11 +3997,11 @@
         </is>
       </c>
       <c r="G71" s="11" t="n">
-        <v>959</v>
+        <v>1987</v>
       </c>
       <c r="H71" s="10" t="inlineStr">
         <is>
-          <t>16/22</t>
+          <t>17/22</t>
         </is>
       </c>
       <c r="I71" s="10" t="inlineStr">
@@ -4010,10 +4010,10 @@
         </is>
       </c>
       <c r="J71" s="11" t="n">
-        <v>1319</v>
+        <v>2571</v>
       </c>
       <c r="K71" s="12" t="n">
-        <v>59.9375</v>
+        <v>116.8823529411765</v>
       </c>
     </row>
     <row r="72">
@@ -4144,11 +4144,11 @@
         </is>
       </c>
       <c r="G74" s="11" t="n">
-        <v>996</v>
+        <v>1679</v>
       </c>
       <c r="H74" s="10" t="inlineStr">
         <is>
-          <t>12/16</t>
+          <t>13/16</t>
         </is>
       </c>
       <c r="I74" s="10" t="inlineStr">
@@ -4157,10 +4157,10 @@
         </is>
       </c>
       <c r="J74" s="11" t="n">
-        <v>1328</v>
+        <v>2066</v>
       </c>
       <c r="K74" s="12" t="n">
-        <v>83</v>
+        <v>129.1538461538462</v>
       </c>
     </row>
     <row r="75">
@@ -4291,11 +4291,11 @@
         </is>
       </c>
       <c r="G77" s="7" t="n">
-        <v>3845</v>
+        <v>2862</v>
       </c>
       <c r="H77" s="6" t="inlineStr">
         <is>
-          <t>16/23</t>
+          <t>17/23</t>
         </is>
       </c>
       <c r="I77" s="6" t="inlineStr">
@@ -4304,10 +4304,10 @@
         </is>
       </c>
       <c r="J77" s="7" t="n">
-        <v>5527</v>
+        <v>3872</v>
       </c>
       <c r="K77" s="8" t="n">
-        <v>240.3125</v>
+        <v>168.3529411764706</v>
       </c>
     </row>
     <row r="78">
@@ -4487,11 +4487,11 @@
         </is>
       </c>
       <c r="G81" s="7" t="n">
-        <v>3579</v>
+        <v>4558</v>
       </c>
       <c r="H81" s="6" t="inlineStr">
         <is>
-          <t>15/24</t>
+          <t>16/24</t>
         </is>
       </c>
       <c r="I81" s="6" t="inlineStr">
@@ -4500,10 +4500,10 @@
         </is>
       </c>
       <c r="J81" s="7" t="n">
-        <v>5726</v>
+        <v>6837</v>
       </c>
       <c r="K81" s="8" t="n">
-        <v>238.6</v>
+        <v>284.875</v>
       </c>
     </row>
     <row r="82">
@@ -4683,11 +4683,11 @@
         </is>
       </c>
       <c r="G85" s="11" t="n">
-        <v>1160</v>
+        <v>1101</v>
       </c>
       <c r="H85" s="10" t="inlineStr">
         <is>
-          <t>17/20</t>
+          <t>18/20</t>
         </is>
       </c>
       <c r="I85" s="10" t="inlineStr">
@@ -4696,10 +4696,10 @@
         </is>
       </c>
       <c r="J85" s="11" t="n">
-        <v>1365</v>
+        <v>1223</v>
       </c>
       <c r="K85" s="12" t="n">
-        <v>68.23529411764706</v>
+        <v>61.16666666666666</v>
       </c>
     </row>
     <row r="86">
@@ -4732,11 +4732,11 @@
         </is>
       </c>
       <c r="G86" s="7" t="n">
-        <v>5807</v>
+        <v>5632</v>
       </c>
       <c r="H86" s="6" t="inlineStr">
         <is>
-          <t>13/21</t>
+          <t>14/21</t>
         </is>
       </c>
       <c r="I86" s="6" t="inlineStr">
@@ -4745,10 +4745,10 @@
         </is>
       </c>
       <c r="J86" s="7" t="n">
-        <v>9381</v>
+        <v>8448</v>
       </c>
       <c r="K86" s="8" t="n">
-        <v>446.6923076923077</v>
+        <v>402.2857142857143</v>
       </c>
     </row>
     <row r="87">
@@ -4830,11 +4830,11 @@
         </is>
       </c>
       <c r="G88" s="4" t="n">
-        <v>17069</v>
+        <v>18028</v>
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>14/19</t>
+          <t>15/19</t>
         </is>
       </c>
       <c r="I88" s="3" t="inlineStr">
@@ -4843,10 +4843,10 @@
         </is>
       </c>
       <c r="J88" s="4" t="n">
-        <v>23165</v>
+        <v>22835</v>
       </c>
       <c r="K88" s="5" t="n">
-        <v>1219.214285714286</v>
+        <v>1201.866666666667</v>
       </c>
     </row>
     <row r="89">
@@ -5026,11 +5026,11 @@
         </is>
       </c>
       <c r="G92" s="4" t="n">
-        <v>8628</v>
+        <v>9773</v>
       </c>
       <c r="H92" s="3" t="inlineStr">
         <is>
-          <t>20/24</t>
+          <t>21/24</t>
         </is>
       </c>
       <c r="I92" s="3" t="inlineStr">
@@ -5039,10 +5039,10 @@
         </is>
       </c>
       <c r="J92" s="4" t="n">
-        <v>10354</v>
+        <v>11169</v>
       </c>
       <c r="K92" s="5" t="n">
-        <v>431.4</v>
+        <v>465.3809523809524</v>
       </c>
     </row>
     <row r="93">
@@ -5124,11 +5124,11 @@
         </is>
       </c>
       <c r="G94" s="4" t="n">
-        <v>36223</v>
+        <v>38848</v>
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
-          <t>13/25</t>
+          <t>14/25</t>
         </is>
       </c>
       <c r="I94" s="3" t="inlineStr">
@@ -5137,10 +5137,10 @@
         </is>
       </c>
       <c r="J94" s="4" t="n">
-        <v>69660</v>
+        <v>69371</v>
       </c>
       <c r="K94" s="5" t="n">
-        <v>2786.384615384615</v>
+        <v>2774.857142857143</v>
       </c>
     </row>
     <row r="95">
@@ -5271,11 +5271,11 @@
         </is>
       </c>
       <c r="G97" s="7" t="n">
-        <v>3526</v>
+        <v>3848</v>
       </c>
       <c r="H97" s="6" t="inlineStr">
         <is>
-          <t>12/27</t>
+          <t>13/27</t>
         </is>
       </c>
       <c r="I97" s="6" t="inlineStr">
@@ -5284,10 +5284,10 @@
         </is>
       </c>
       <c r="J97" s="7" t="n">
-        <v>7933</v>
+        <v>7992</v>
       </c>
       <c r="K97" s="8" t="n">
-        <v>293.8333333333333</v>
+        <v>296</v>
       </c>
     </row>
     <row r="98">
@@ -5369,11 +5369,11 @@
         </is>
       </c>
       <c r="G99" s="11" t="n">
-        <v>1591</v>
+        <v>1367</v>
       </c>
       <c r="H99" s="10" t="inlineStr">
         <is>
-          <t>18/22</t>
+          <t>19/22</t>
         </is>
       </c>
       <c r="I99" s="10" t="inlineStr">
@@ -5382,10 +5382,10 @@
         </is>
       </c>
       <c r="J99" s="11" t="n">
-        <v>1945</v>
+        <v>1583</v>
       </c>
       <c r="K99" s="12" t="n">
-        <v>88.38888888888889</v>
+        <v>71.94736842105263</v>
       </c>
     </row>
     <row r="100">
@@ -5565,11 +5565,11 @@
         </is>
       </c>
       <c r="G103" s="11" t="n">
-        <v>328</v>
+        <v>360</v>
       </c>
       <c r="H103" s="10" t="inlineStr">
         <is>
-          <t>14/24</t>
+          <t>15/24</t>
         </is>
       </c>
       <c r="I103" s="10" t="inlineStr">
@@ -5578,10 +5578,10 @@
         </is>
       </c>
       <c r="J103" s="11" t="n">
-        <v>562</v>
+        <v>576</v>
       </c>
       <c r="K103" s="12" t="n">
-        <v>23.42857142857143</v>
+        <v>24</v>
       </c>
     </row>
     <row r="104">
@@ -5614,7 +5614,7 @@
         </is>
       </c>
       <c r="G104" s="11" t="n">
-        <v>2132</v>
+        <v>1890</v>
       </c>
       <c r="H104" s="10" t="inlineStr">
         <is>
@@ -5627,10 +5627,10 @@
         </is>
       </c>
       <c r="J104" s="11" t="n">
-        <v>2356</v>
+        <v>2089</v>
       </c>
       <c r="K104" s="12" t="n">
-        <v>112.2105263157895</v>
+        <v>99.47368421052632</v>
       </c>
     </row>
     <row r="105">
@@ -5663,11 +5663,11 @@
         </is>
       </c>
       <c r="G105" s="4" t="n">
-        <v>12922</v>
+        <v>14509</v>
       </c>
       <c r="H105" s="3" t="inlineStr">
         <is>
-          <t>23/30</t>
+          <t>24/30</t>
         </is>
       </c>
       <c r="I105" s="3" t="inlineStr">
@@ -5676,10 +5676,10 @@
         </is>
       </c>
       <c r="J105" s="4" t="n">
-        <v>16855</v>
+        <v>18136</v>
       </c>
       <c r="K105" s="5" t="n">
-        <v>561.8260869565217</v>
+        <v>604.5416666666666</v>
       </c>
     </row>
     <row r="106">
@@ -5712,11 +5712,11 @@
         </is>
       </c>
       <c r="G106" s="4" t="n">
-        <v>17525</v>
+        <v>17442</v>
       </c>
       <c r="H106" s="3" t="inlineStr">
         <is>
-          <t>20/21</t>
+          <t>21/21</t>
         </is>
       </c>
       <c r="I106" s="3" t="inlineStr">
@@ -5725,10 +5725,10 @@
         </is>
       </c>
       <c r="J106" s="4" t="n">
-        <v>18401</v>
+        <v>17442</v>
       </c>
       <c r="K106" s="5" t="n">
-        <v>876.25</v>
+        <v>830.5714285714286</v>
       </c>
     </row>
     <row r="107">
@@ -5761,11 +5761,11 @@
         </is>
       </c>
       <c r="G107" s="4" t="n">
-        <v>27874</v>
+        <v>28928</v>
       </c>
       <c r="H107" s="3" t="inlineStr">
         <is>
-          <t>19/21</t>
+          <t>20/21</t>
         </is>
       </c>
       <c r="I107" s="3" t="inlineStr">
@@ -5774,59 +5774,59 @@
         </is>
       </c>
       <c r="J107" s="4" t="n">
-        <v>30808</v>
+        <v>30374</v>
       </c>
       <c r="K107" s="5" t="n">
-        <v>1467.052631578947</v>
+        <v>1446.4</v>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="inlineStr">
+      <c r="A108" s="6" t="inlineStr">
         <is>
           <t>NAGAPATTINAM</t>
         </is>
       </c>
-      <c r="B108" s="3" t="n">
+      <c r="B108" s="6" t="n">
         <v>163</v>
       </c>
-      <c r="C108" s="3" t="inlineStr">
+      <c r="C108" s="6" t="inlineStr">
         <is>
           <t>M.H.JAWAHIRULLAH</t>
         </is>
       </c>
-      <c r="D108" s="3" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E108" s="3" t="inlineStr">
+      <c r="D108" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E108" s="6" t="inlineStr">
         <is>
           <t>M.SUGUMAR</t>
         </is>
       </c>
-      <c r="F108" s="3" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G108" s="4" t="n">
-        <v>11123</v>
-      </c>
-      <c r="H108" s="3" t="inlineStr">
-        <is>
-          <t>10/18</t>
-        </is>
-      </c>
-      <c r="I108" s="3" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J108" s="4" t="n">
-        <v>20021</v>
-      </c>
-      <c r="K108" s="5" t="n">
-        <v>1112.3</v>
+      <c r="F108" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G108" s="7" t="n">
+        <v>9638</v>
+      </c>
+      <c r="H108" s="6" t="inlineStr">
+        <is>
+          <t>11/18</t>
+        </is>
+      </c>
+      <c r="I108" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J108" s="7" t="n">
+        <v>15771</v>
+      </c>
+      <c r="K108" s="8" t="n">
+        <v>876.1818181818181</v>
       </c>
     </row>
     <row r="109">
@@ -5966,7 +5966,7 @@
       </c>
       <c r="I111" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J111" s="4" t="n">
@@ -6251,11 +6251,11 @@
         </is>
       </c>
       <c r="G117" s="4" t="n">
-        <v>14081</v>
+        <v>15797</v>
       </c>
       <c r="H117" s="3" t="inlineStr">
         <is>
-          <t>20/26</t>
+          <t>21/26</t>
         </is>
       </c>
       <c r="I117" s="3" t="inlineStr">
@@ -6264,10 +6264,10 @@
         </is>
       </c>
       <c r="J117" s="4" t="n">
-        <v>18305</v>
+        <v>19558</v>
       </c>
       <c r="K117" s="5" t="n">
-        <v>704.05</v>
+        <v>752.2380952380952</v>
       </c>
     </row>
     <row r="118">
@@ -6369,52 +6369,52 @@
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="6" t="inlineStr">
+      <c r="A120" s="2" t="inlineStr">
         <is>
           <t>PADMANABHAPURAM</t>
         </is>
       </c>
-      <c r="B120" s="6" t="n">
+      <c r="B120" s="3" t="n">
         <v>232</v>
       </c>
-      <c r="C120" s="6" t="inlineStr">
+      <c r="C120" s="3" t="inlineStr">
         <is>
           <t>CHELLASWAMY. R</t>
         </is>
       </c>
-      <c r="D120" s="6" t="inlineStr">
+      <c r="D120" s="3" t="inlineStr">
         <is>
           <t>Communist Party of India (Marxist)</t>
         </is>
       </c>
-      <c r="E120" s="6" t="inlineStr">
+      <c r="E120" s="3" t="inlineStr">
         <is>
           <t>KRISHNA KUMAR. S</t>
         </is>
       </c>
-      <c r="F120" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G120" s="7" t="n">
-        <v>12302</v>
-      </c>
-      <c r="H120" s="6" t="inlineStr">
-        <is>
-          <t>17/23</t>
-        </is>
-      </c>
-      <c r="I120" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J120" s="7" t="n">
-        <v>16644</v>
-      </c>
-      <c r="K120" s="8" t="n">
-        <v>723.6470588235294</v>
+      <c r="F120" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G120" s="4" t="n">
+        <v>13869</v>
+      </c>
+      <c r="H120" s="3" t="inlineStr">
+        <is>
+          <t>18/23</t>
+        </is>
+      </c>
+      <c r="I120" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J120" s="4" t="n">
+        <v>17722</v>
+      </c>
+      <c r="K120" s="5" t="n">
+        <v>770.5</v>
       </c>
     </row>
     <row r="121">
@@ -6447,11 +6447,11 @@
         </is>
       </c>
       <c r="G121" s="4" t="n">
-        <v>35025</v>
+        <v>36153</v>
       </c>
       <c r="H121" s="3" t="inlineStr">
         <is>
-          <t>20/23</t>
+          <t>21/23</t>
         </is>
       </c>
       <c r="I121" s="3" t="inlineStr">
@@ -6460,59 +6460,59 @@
         </is>
       </c>
       <c r="J121" s="4" t="n">
-        <v>40279</v>
+        <v>39596</v>
       </c>
       <c r="K121" s="5" t="n">
-        <v>1751.25</v>
+        <v>1721.571428571429</v>
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="6" t="inlineStr">
+      <c r="A122" s="9" t="inlineStr">
         <is>
           <t>PALANI</t>
         </is>
       </c>
-      <c r="B122" s="6" t="n">
+      <c r="B122" s="10" t="n">
         <v>127</v>
       </c>
-      <c r="C122" s="6" t="inlineStr">
+      <c r="C122" s="10" t="inlineStr">
         <is>
           <t>RAVIMANOHARAN. K</t>
         </is>
       </c>
-      <c r="D122" s="6" t="inlineStr">
+      <c r="D122" s="10" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E122" s="6" t="inlineStr">
+      <c r="E122" s="10" t="inlineStr">
         <is>
           <t>DR. PRAVEEN KUMAR. M</t>
         </is>
       </c>
-      <c r="F122" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G122" s="7" t="n">
-        <v>2932</v>
-      </c>
-      <c r="H122" s="6" t="inlineStr">
-        <is>
-          <t>20/25</t>
-        </is>
-      </c>
-      <c r="I122" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J122" s="7" t="n">
-        <v>3665</v>
-      </c>
-      <c r="K122" s="8" t="n">
-        <v>146.6</v>
+      <c r="F122" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G122" s="11" t="n">
+        <v>1246</v>
+      </c>
+      <c r="H122" s="10" t="inlineStr">
+        <is>
+          <t>21/25</t>
+        </is>
+      </c>
+      <c r="I122" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J122" s="11" t="n">
+        <v>1483</v>
+      </c>
+      <c r="K122" s="12" t="n">
+        <v>59.33333333333334</v>
       </c>
     </row>
     <row r="123">
@@ -6594,11 +6594,11 @@
         </is>
       </c>
       <c r="G124" s="4" t="n">
-        <v>39315</v>
+        <v>39962</v>
       </c>
       <c r="H124" s="3" t="inlineStr">
         <is>
-          <t>27/35</t>
+          <t>28/35</t>
         </is>
       </c>
       <c r="I124" s="3" t="inlineStr">
@@ -6607,10 +6607,10 @@
         </is>
       </c>
       <c r="J124" s="4" t="n">
-        <v>50964</v>
+        <v>49952</v>
       </c>
       <c r="K124" s="5" t="n">
-        <v>1456.111111111111</v>
+        <v>1427.214285714286</v>
       </c>
     </row>
     <row r="125">
@@ -6643,11 +6643,11 @@
         </is>
       </c>
       <c r="G125" s="4" t="n">
-        <v>29315</v>
+        <v>31435</v>
       </c>
       <c r="H125" s="3" t="inlineStr">
         <is>
-          <t>18/34</t>
+          <t>19/34</t>
         </is>
       </c>
       <c r="I125" s="3" t="inlineStr">
@@ -6656,10 +6656,10 @@
         </is>
       </c>
       <c r="J125" s="4" t="n">
-        <v>55373</v>
+        <v>56252</v>
       </c>
       <c r="K125" s="5" t="n">
-        <v>1628.611111111111</v>
+        <v>1654.473684210526</v>
       </c>
     </row>
     <row r="126">
@@ -6937,11 +6937,11 @@
         </is>
       </c>
       <c r="G131" s="7" t="n">
-        <v>4180</v>
+        <v>4695</v>
       </c>
       <c r="H131" s="6" t="inlineStr">
         <is>
-          <t>15/23</t>
+          <t>16/23</t>
         </is>
       </c>
       <c r="I131" s="6" t="inlineStr">
@@ -6950,10 +6950,10 @@
         </is>
       </c>
       <c r="J131" s="7" t="n">
-        <v>6409</v>
+        <v>6749</v>
       </c>
       <c r="K131" s="8" t="n">
-        <v>278.6666666666667</v>
+        <v>293.4375</v>
       </c>
     </row>
     <row r="132">
@@ -6986,11 +6986,11 @@
         </is>
       </c>
       <c r="G132" s="7" t="n">
-        <v>2790</v>
+        <v>4603</v>
       </c>
       <c r="H132" s="6" t="inlineStr">
         <is>
-          <t>17/23</t>
+          <t>18/23</t>
         </is>
       </c>
       <c r="I132" s="6" t="inlineStr">
@@ -6999,10 +6999,10 @@
         </is>
       </c>
       <c r="J132" s="7" t="n">
-        <v>3775</v>
+        <v>5882</v>
       </c>
       <c r="K132" s="8" t="n">
-        <v>164.1176470588235</v>
+        <v>255.7222222222222</v>
       </c>
     </row>
     <row r="133">
@@ -7035,11 +7035,11 @@
         </is>
       </c>
       <c r="G133" s="4" t="n">
-        <v>9914</v>
+        <v>11310</v>
       </c>
       <c r="H133" s="3" t="inlineStr">
         <is>
-          <t>22/28</t>
+          <t>23/28</t>
         </is>
       </c>
       <c r="I133" s="3" t="inlineStr">
@@ -7048,10 +7048,10 @@
         </is>
       </c>
       <c r="J133" s="4" t="n">
-        <v>12618</v>
+        <v>13769</v>
       </c>
       <c r="K133" s="5" t="n">
-        <v>450.6363636363636</v>
+        <v>491.7391304347826</v>
       </c>
     </row>
     <row r="134">
@@ -7084,11 +7084,11 @@
         </is>
       </c>
       <c r="G134" s="4" t="n">
-        <v>29031</v>
+        <v>31766</v>
       </c>
       <c r="H134" s="3" t="inlineStr">
         <is>
-          <t>12/22</t>
+          <t>13/22</t>
         </is>
       </c>
       <c r="I134" s="3" t="inlineStr">
@@ -7097,59 +7097,59 @@
         </is>
       </c>
       <c r="J134" s="4" t="n">
-        <v>53224</v>
+        <v>53758</v>
       </c>
       <c r="K134" s="5" t="n">
-        <v>2419.25</v>
+        <v>2443.538461538461</v>
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="9" t="inlineStr">
+      <c r="A135" s="6" t="inlineStr">
         <is>
           <t>PERAVURANI</t>
         </is>
       </c>
-      <c r="B135" s="10" t="n">
+      <c r="B135" s="6" t="n">
         <v>177</v>
       </c>
-      <c r="C135" s="10" t="inlineStr">
+      <c r="C135" s="6" t="inlineStr">
+        <is>
+          <t>ASHOKKUMAR. N</t>
+        </is>
+      </c>
+      <c r="D135" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E135" s="6" t="inlineStr">
         <is>
           <t>GOVI.ELANGO</t>
         </is>
       </c>
-      <c r="D135" s="10" t="inlineStr">
+      <c r="F135" s="6" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E135" s="10" t="inlineStr">
-        <is>
-          <t>ASHOKKUMAR. N</t>
-        </is>
-      </c>
-      <c r="F135" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G135" s="11" t="n">
-        <v>428</v>
-      </c>
-      <c r="H135" s="10" t="inlineStr">
-        <is>
-          <t>7/21</t>
-        </is>
-      </c>
-      <c r="I135" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J135" s="11" t="n">
-        <v>1284</v>
-      </c>
-      <c r="K135" s="12" t="n">
-        <v>61.14285714285715</v>
+      <c r="G135" s="7" t="n">
+        <v>1691</v>
+      </c>
+      <c r="H135" s="6" t="inlineStr">
+        <is>
+          <t>8/21</t>
+        </is>
+      </c>
+      <c r="I135" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J135" s="7" t="n">
+        <v>4439</v>
+      </c>
+      <c r="K135" s="8" t="n">
+        <v>211.375</v>
       </c>
     </row>
     <row r="136">
@@ -7182,11 +7182,11 @@
         </is>
       </c>
       <c r="G136" s="7" t="n">
-        <v>4931</v>
+        <v>6271</v>
       </c>
       <c r="H136" s="6" t="inlineStr">
         <is>
-          <t>17/26</t>
+          <t>18/26</t>
         </is>
       </c>
       <c r="I136" s="6" t="inlineStr">
@@ -7195,10 +7195,10 @@
         </is>
       </c>
       <c r="J136" s="7" t="n">
-        <v>7542</v>
+        <v>9058</v>
       </c>
       <c r="K136" s="8" t="n">
-        <v>290.0588235294118</v>
+        <v>348.3888888888889</v>
       </c>
     </row>
     <row r="137">
@@ -7231,11 +7231,11 @@
         </is>
       </c>
       <c r="G137" s="4" t="n">
-        <v>7516</v>
+        <v>8384</v>
       </c>
       <c r="H137" s="3" t="inlineStr">
         <is>
-          <t>17/21</t>
+          <t>18/21</t>
         </is>
       </c>
       <c r="I137" s="3" t="inlineStr">
@@ -7244,10 +7244,10 @@
         </is>
       </c>
       <c r="J137" s="4" t="n">
-        <v>9284</v>
+        <v>9781</v>
       </c>
       <c r="K137" s="5" t="n">
-        <v>442.1176470588235</v>
+        <v>465.7777777777778</v>
       </c>
     </row>
     <row r="138">
@@ -7280,11 +7280,11 @@
         </is>
       </c>
       <c r="G138" s="7" t="n">
-        <v>2731</v>
+        <v>3917</v>
       </c>
       <c r="H138" s="6" t="inlineStr">
         <is>
-          <t>18/22</t>
+          <t>19/22</t>
         </is>
       </c>
       <c r="I138" s="6" t="inlineStr">
@@ -7293,10 +7293,10 @@
         </is>
       </c>
       <c r="J138" s="7" t="n">
-        <v>3338</v>
+        <v>4535</v>
       </c>
       <c r="K138" s="8" t="n">
-        <v>151.7222222222222</v>
+        <v>206.1578947368421</v>
       </c>
     </row>
     <row r="139">
@@ -7378,11 +7378,11 @@
         </is>
       </c>
       <c r="G140" s="4" t="n">
-        <v>44586</v>
+        <v>46942</v>
       </c>
       <c r="H140" s="3" t="inlineStr">
         <is>
-          <t>19/24</t>
+          <t>20/24</t>
         </is>
       </c>
       <c r="I140" s="3" t="inlineStr">
@@ -7391,10 +7391,10 @@
         </is>
       </c>
       <c r="J140" s="4" t="n">
-        <v>56319</v>
+        <v>56330</v>
       </c>
       <c r="K140" s="5" t="n">
-        <v>2346.631578947368</v>
+        <v>2347.1</v>
       </c>
     </row>
     <row r="141">
@@ -7476,11 +7476,11 @@
         </is>
       </c>
       <c r="G142" s="4" t="n">
-        <v>61989</v>
+        <v>63006</v>
       </c>
       <c r="H142" s="3" t="inlineStr">
         <is>
-          <t>19/23</t>
+          <t>20/23</t>
         </is>
       </c>
       <c r="I142" s="3" t="inlineStr">
@@ -7489,10 +7489,10 @@
         </is>
       </c>
       <c r="J142" s="4" t="n">
-        <v>75039</v>
+        <v>72457</v>
       </c>
       <c r="K142" s="5" t="n">
-        <v>3262.578947368421</v>
+        <v>3150.3</v>
       </c>
     </row>
     <row r="143">
@@ -7525,11 +7525,11 @@
         </is>
       </c>
       <c r="G143" s="7" t="n">
-        <v>2376</v>
+        <v>2920</v>
       </c>
       <c r="H143" s="6" t="inlineStr">
         <is>
-          <t>14/22</t>
+          <t>15/22</t>
         </is>
       </c>
       <c r="I143" s="6" t="inlineStr">
@@ -7538,10 +7538,10 @@
         </is>
       </c>
       <c r="J143" s="7" t="n">
-        <v>3734</v>
+        <v>4283</v>
       </c>
       <c r="K143" s="8" t="n">
-        <v>169.7142857142857</v>
+        <v>194.6666666666667</v>
       </c>
     </row>
     <row r="144">
@@ -7672,11 +7672,11 @@
         </is>
       </c>
       <c r="G146" s="4" t="n">
-        <v>14012</v>
+        <v>13101</v>
       </c>
       <c r="H146" s="3" t="inlineStr">
         <is>
-          <t>27/29</t>
+          <t>28/29</t>
         </is>
       </c>
       <c r="I146" s="3" t="inlineStr">
@@ -7685,10 +7685,10 @@
         </is>
       </c>
       <c r="J146" s="4" t="n">
-        <v>15050</v>
+        <v>13569</v>
       </c>
       <c r="K146" s="5" t="n">
-        <v>518.9629629629629</v>
+        <v>467.8928571428572</v>
       </c>
     </row>
     <row r="147">
@@ -7721,11 +7721,11 @@
         </is>
       </c>
       <c r="G147" s="7" t="n">
-        <v>2416</v>
+        <v>3162</v>
       </c>
       <c r="H147" s="6" t="inlineStr">
         <is>
-          <t>17/22</t>
+          <t>18/22</t>
         </is>
       </c>
       <c r="I147" s="6" t="inlineStr">
@@ -7734,10 +7734,10 @@
         </is>
       </c>
       <c r="J147" s="7" t="n">
-        <v>3127</v>
+        <v>3865</v>
       </c>
       <c r="K147" s="8" t="n">
-        <v>142.1176470588235</v>
+        <v>175.6666666666667</v>
       </c>
     </row>
     <row r="148">
@@ -7761,20 +7761,20 @@
       </c>
       <c r="E148" s="3" t="inlineStr">
         <is>
-          <t>MATHIVENTHAN M DR</t>
+          <t>PREMKUMAR S D</t>
         </is>
       </c>
       <c r="F148" s="3" t="inlineStr">
         <is>
-          <t>Dravida Munnetra Kazhagam</t>
+          <t>Bharatiya Janata Party</t>
         </is>
       </c>
       <c r="G148" s="4" t="n">
-        <v>15314</v>
+        <v>14196</v>
       </c>
       <c r="H148" s="3" t="inlineStr">
         <is>
-          <t>17/21</t>
+          <t>18/21</t>
         </is>
       </c>
       <c r="I148" s="3" t="inlineStr">
@@ -7783,10 +7783,10 @@
         </is>
       </c>
       <c r="J148" s="4" t="n">
-        <v>18917</v>
+        <v>16562</v>
       </c>
       <c r="K148" s="5" t="n">
-        <v>900.8235294117648</v>
+        <v>788.6666666666666</v>
       </c>
     </row>
     <row r="149">
@@ -7819,11 +7819,11 @@
         </is>
       </c>
       <c r="G149" s="7" t="n">
-        <v>3740</v>
+        <v>3368</v>
       </c>
       <c r="H149" s="6" t="inlineStr">
         <is>
-          <t>13/25</t>
+          <t>14/25</t>
         </is>
       </c>
       <c r="I149" s="6" t="inlineStr">
@@ -7832,10 +7832,10 @@
         </is>
       </c>
       <c r="J149" s="7" t="n">
-        <v>7192</v>
+        <v>6014</v>
       </c>
       <c r="K149" s="8" t="n">
-        <v>287.6923076923077</v>
+        <v>240.5714285714285</v>
       </c>
     </row>
     <row r="150">
@@ -7937,52 +7937,52 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="6" t="inlineStr">
+      <c r="A152" s="2" t="inlineStr">
         <is>
           <t>SALEM (NORTH)</t>
         </is>
       </c>
-      <c r="B152" s="6" t="n">
+      <c r="B152" s="3" t="n">
         <v>89</v>
       </c>
-      <c r="C152" s="6" t="inlineStr">
+      <c r="C152" s="3" t="inlineStr">
         <is>
           <t>SIVAKUMAR. K</t>
         </is>
       </c>
-      <c r="D152" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E152" s="6" t="inlineStr">
+      <c r="D152" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E152" s="3" t="inlineStr">
         <is>
           <t>RAJENDRAN. R</t>
         </is>
       </c>
-      <c r="F152" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G152" s="7" t="n">
-        <v>6041</v>
-      </c>
-      <c r="H152" s="6" t="inlineStr">
-        <is>
-          <t>15/21</t>
-        </is>
-      </c>
-      <c r="I152" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J152" s="7" t="n">
-        <v>8457</v>
-      </c>
-      <c r="K152" s="8" t="n">
-        <v>402.7333333333333</v>
+      <c r="F152" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G152" s="4" t="n">
+        <v>7752</v>
+      </c>
+      <c r="H152" s="3" t="inlineStr">
+        <is>
+          <t>16/21</t>
+        </is>
+      </c>
+      <c r="I152" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J152" s="4" t="n">
+        <v>10174</v>
+      </c>
+      <c r="K152" s="5" t="n">
+        <v>484.5</v>
       </c>
     </row>
     <row r="153">
@@ -8015,11 +8015,11 @@
         </is>
       </c>
       <c r="G153" s="4" t="n">
-        <v>31731</v>
+        <v>33203</v>
       </c>
       <c r="H153" s="3" t="inlineStr">
         <is>
-          <t>18/20</t>
+          <t>19/20</t>
         </is>
       </c>
       <c r="I153" s="3" t="inlineStr">
@@ -8028,10 +8028,10 @@
         </is>
       </c>
       <c r="J153" s="4" t="n">
-        <v>35257</v>
+        <v>34951</v>
       </c>
       <c r="K153" s="5" t="n">
-        <v>1762.833333333333</v>
+        <v>1747.526315789474</v>
       </c>
     </row>
     <row r="154">
@@ -8064,11 +8064,11 @@
         </is>
       </c>
       <c r="G154" s="4" t="n">
-        <v>47352</v>
+        <v>50943</v>
       </c>
       <c r="H154" s="3" t="inlineStr">
         <is>
-          <t>15/23</t>
+          <t>16/23</t>
         </is>
       </c>
       <c r="I154" s="3" t="inlineStr">
@@ -8077,10 +8077,10 @@
         </is>
       </c>
       <c r="J154" s="4" t="n">
-        <v>72606</v>
+        <v>73231</v>
       </c>
       <c r="K154" s="5" t="n">
-        <v>3156.8</v>
+        <v>3183.9375</v>
       </c>
     </row>
     <row r="155">
@@ -8162,11 +8162,11 @@
         </is>
       </c>
       <c r="G156" s="7" t="n">
-        <v>2467</v>
+        <v>2436</v>
       </c>
       <c r="H156" s="6" t="inlineStr">
         <is>
-          <t>11/25</t>
+          <t>12/25</t>
         </is>
       </c>
       <c r="I156" s="6" t="inlineStr">
@@ -8175,10 +8175,10 @@
         </is>
       </c>
       <c r="J156" s="7" t="n">
-        <v>5607</v>
+        <v>5075</v>
       </c>
       <c r="K156" s="8" t="n">
-        <v>224.2727272727273</v>
+        <v>203</v>
       </c>
     </row>
     <row r="157">
@@ -8211,11 +8211,11 @@
         </is>
       </c>
       <c r="G157" s="4" t="n">
-        <v>6318</v>
+        <v>6282</v>
       </c>
       <c r="H157" s="3" t="inlineStr">
         <is>
-          <t>20/25</t>
+          <t>21/25</t>
         </is>
       </c>
       <c r="I157" s="3" t="inlineStr">
@@ -8224,10 +8224,10 @@
         </is>
       </c>
       <c r="J157" s="4" t="n">
-        <v>7897</v>
+        <v>7479</v>
       </c>
       <c r="K157" s="5" t="n">
-        <v>315.9</v>
+        <v>299.1428571428572</v>
       </c>
     </row>
     <row r="158">
@@ -8309,11 +8309,11 @@
         </is>
       </c>
       <c r="G159" s="11" t="n">
-        <v>452</v>
+        <v>1466</v>
       </c>
       <c r="H159" s="10" t="inlineStr">
         <is>
-          <t>20/23</t>
+          <t>21/23</t>
         </is>
       </c>
       <c r="I159" s="10" t="inlineStr">
@@ -8322,10 +8322,10 @@
         </is>
       </c>
       <c r="J159" s="11" t="n">
-        <v>520</v>
+        <v>1606</v>
       </c>
       <c r="K159" s="12" t="n">
-        <v>22.6</v>
+        <v>69.80952380952381</v>
       </c>
     </row>
     <row r="160">
@@ -8358,11 +8358,11 @@
         </is>
       </c>
       <c r="G160" s="11" t="n">
-        <v>1180</v>
+        <v>1504</v>
       </c>
       <c r="H160" s="10" t="inlineStr">
         <is>
-          <t>11/19</t>
+          <t>12/19</t>
         </is>
       </c>
       <c r="I160" s="10" t="inlineStr">
@@ -8371,10 +8371,10 @@
         </is>
       </c>
       <c r="J160" s="11" t="n">
-        <v>2038</v>
+        <v>2381</v>
       </c>
       <c r="K160" s="12" t="n">
-        <v>107.2727272727273</v>
+        <v>125.3333333333333</v>
       </c>
     </row>
     <row r="161">
@@ -8456,11 +8456,11 @@
         </is>
       </c>
       <c r="G162" s="4" t="n">
-        <v>41159</v>
+        <v>45482</v>
       </c>
       <c r="H162" s="3" t="inlineStr">
         <is>
-          <t>14/30</t>
+          <t>15/30</t>
         </is>
       </c>
       <c r="I162" s="3" t="inlineStr">
@@ -8469,10 +8469,10 @@
         </is>
       </c>
       <c r="J162" s="4" t="n">
-        <v>88198</v>
+        <v>90964</v>
       </c>
       <c r="K162" s="5" t="n">
-        <v>2939.928571428572</v>
+        <v>3032.133333333333</v>
       </c>
     </row>
     <row r="163">
@@ -8505,11 +8505,11 @@
         </is>
       </c>
       <c r="G163" s="4" t="n">
-        <v>16388</v>
+        <v>17997</v>
       </c>
       <c r="H163" s="3" t="inlineStr">
         <is>
-          <t>16/26</t>
+          <t>17/26</t>
         </is>
       </c>
       <c r="I163" s="3" t="inlineStr">
@@ -8518,10 +8518,10 @@
         </is>
       </c>
       <c r="J163" s="4" t="n">
-        <v>26630</v>
+        <v>27525</v>
       </c>
       <c r="K163" s="5" t="n">
-        <v>1024.25</v>
+        <v>1058.64705882353</v>
       </c>
     </row>
     <row r="164">
@@ -8603,11 +8603,11 @@
         </is>
       </c>
       <c r="G165" s="7" t="n">
-        <v>11975</v>
+        <v>12382</v>
       </c>
       <c r="H165" s="6" t="inlineStr">
         <is>
-          <t>18/29</t>
+          <t>19/29</t>
         </is>
       </c>
       <c r="I165" s="6" t="inlineStr">
@@ -8616,10 +8616,10 @@
         </is>
       </c>
       <c r="J165" s="7" t="n">
-        <v>19293</v>
+        <v>18899</v>
       </c>
       <c r="K165" s="8" t="n">
-        <v>665.2777777777778</v>
+        <v>651.6842105263158</v>
       </c>
     </row>
     <row r="166">
@@ -8701,11 +8701,11 @@
         </is>
       </c>
       <c r="G167" s="4" t="n">
-        <v>30598</v>
+        <v>32853</v>
       </c>
       <c r="H167" s="3" t="inlineStr">
         <is>
-          <t>18/32</t>
+          <t>19/32</t>
         </is>
       </c>
       <c r="I167" s="3" t="inlineStr">
@@ -8714,10 +8714,10 @@
         </is>
       </c>
       <c r="J167" s="4" t="n">
-        <v>54396</v>
+        <v>55331</v>
       </c>
       <c r="K167" s="5" t="n">
-        <v>1699.888888888889</v>
+        <v>1729.105263157895</v>
       </c>
     </row>
     <row r="168">
@@ -8808,7 +8808,7 @@
       </c>
       <c r="I169" s="10" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J169" s="11" t="n">
@@ -8897,11 +8897,11 @@
         </is>
       </c>
       <c r="G171" s="4" t="n">
-        <v>11712</v>
+        <v>12326</v>
       </c>
       <c r="H171" s="3" t="inlineStr">
         <is>
-          <t>21/28</t>
+          <t>22/28</t>
         </is>
       </c>
       <c r="I171" s="3" t="inlineStr">
@@ -8910,10 +8910,10 @@
         </is>
       </c>
       <c r="J171" s="4" t="n">
-        <v>15616</v>
+        <v>15688</v>
       </c>
       <c r="K171" s="5" t="n">
-        <v>557.7142857142857</v>
+        <v>560.2727272727273</v>
       </c>
     </row>
     <row r="172">
@@ -9025,30 +9025,30 @@
       </c>
       <c r="C174" s="10" t="inlineStr">
         <is>
+          <t>DR.NAGESH KUMAR. C</t>
+        </is>
+      </c>
+      <c r="D174" s="10" t="inlineStr">
+        <is>
+          <t>Bharatiya Janata Party</t>
+        </is>
+      </c>
+      <c r="E174" s="10" t="inlineStr">
+        <is>
           <t>RAMACHANDRAN. T</t>
         </is>
       </c>
-      <c r="D174" s="10" t="inlineStr">
+      <c r="F174" s="10" t="inlineStr">
         <is>
           <t>Communist Party of India</t>
         </is>
       </c>
-      <c r="E174" s="10" t="inlineStr">
-        <is>
-          <t>DR.NAGESH KUMAR. C</t>
-        </is>
-      </c>
-      <c r="F174" s="10" t="inlineStr">
-        <is>
-          <t>Bharatiya Janata Party</t>
-        </is>
-      </c>
       <c r="G174" s="11" t="n">
-        <v>413</v>
+        <v>354</v>
       </c>
       <c r="H174" s="10" t="inlineStr">
         <is>
-          <t>15/24</t>
+          <t>16/24</t>
         </is>
       </c>
       <c r="I174" s="10" t="inlineStr">
@@ -9057,10 +9057,10 @@
         </is>
       </c>
       <c r="J174" s="11" t="n">
-        <v>661</v>
+        <v>531</v>
       </c>
       <c r="K174" s="12" t="n">
-        <v>27.53333333333333</v>
+        <v>22.125</v>
       </c>
     </row>
     <row r="175">
@@ -9191,11 +9191,11 @@
         </is>
       </c>
       <c r="G177" s="4" t="n">
-        <v>18858</v>
+        <v>20577</v>
       </c>
       <c r="H177" s="3" t="inlineStr">
         <is>
-          <t>22/26</t>
+          <t>23/26</t>
         </is>
       </c>
       <c r="I177" s="3" t="inlineStr">
@@ -9204,10 +9204,10 @@
         </is>
       </c>
       <c r="J177" s="4" t="n">
-        <v>22287</v>
+        <v>23261</v>
       </c>
       <c r="K177" s="5" t="n">
-        <v>857.1818181818181</v>
+        <v>894.6521739130435</v>
       </c>
     </row>
     <row r="178">
@@ -9240,11 +9240,11 @@
         </is>
       </c>
       <c r="G178" s="11" t="n">
-        <v>275</v>
+        <v>1598</v>
       </c>
       <c r="H178" s="10" t="inlineStr">
         <is>
-          <t>11/22</t>
+          <t>12/22</t>
         </is>
       </c>
       <c r="I178" s="10" t="inlineStr">
@@ -9253,10 +9253,10 @@
         </is>
       </c>
       <c r="J178" s="11" t="n">
-        <v>550</v>
+        <v>2930</v>
       </c>
       <c r="K178" s="12" t="n">
-        <v>25</v>
+        <v>133.1666666666667</v>
       </c>
     </row>
     <row r="179">
@@ -9289,11 +9289,11 @@
         </is>
       </c>
       <c r="G179" s="4" t="n">
-        <v>21796</v>
+        <v>24910</v>
       </c>
       <c r="H179" s="3" t="inlineStr">
         <is>
-          <t>15/26</t>
+          <t>16/26</t>
         </is>
       </c>
       <c r="I179" s="3" t="inlineStr">
@@ -9302,10 +9302,10 @@
         </is>
       </c>
       <c r="J179" s="4" t="n">
-        <v>37780</v>
+        <v>40479</v>
       </c>
       <c r="K179" s="5" t="n">
-        <v>1453.066666666667</v>
+        <v>1556.875</v>
       </c>
     </row>
     <row r="180">
@@ -9338,11 +9338,11 @@
         </is>
       </c>
       <c r="G180" s="4" t="n">
-        <v>27550</v>
+        <v>28156</v>
       </c>
       <c r="H180" s="3" t="inlineStr">
         <is>
-          <t>15/29</t>
+          <t>16/29</t>
         </is>
       </c>
       <c r="I180" s="3" t="inlineStr">
@@ -9351,10 +9351,10 @@
         </is>
       </c>
       <c r="J180" s="4" t="n">
-        <v>53263</v>
+        <v>51033</v>
       </c>
       <c r="K180" s="5" t="n">
-        <v>1836.666666666667</v>
+        <v>1759.75</v>
       </c>
     </row>
     <row r="181">
@@ -9387,11 +9387,11 @@
         </is>
       </c>
       <c r="G181" s="4" t="n">
-        <v>12941</v>
+        <v>12731</v>
       </c>
       <c r="H181" s="3" t="inlineStr">
         <is>
-          <t>19/21</t>
+          <t>20/21</t>
         </is>
       </c>
       <c r="I181" s="3" t="inlineStr">
@@ -9400,10 +9400,10 @@
         </is>
       </c>
       <c r="J181" s="4" t="n">
-        <v>14303</v>
+        <v>13368</v>
       </c>
       <c r="K181" s="5" t="n">
-        <v>681.1052631578947</v>
+        <v>636.55</v>
       </c>
     </row>
     <row r="182">
@@ -9583,11 +9583,11 @@
         </is>
       </c>
       <c r="G185" s="7" t="n">
-        <v>5048</v>
+        <v>5346</v>
       </c>
       <c r="H185" s="6" t="inlineStr">
         <is>
-          <t>13/23</t>
+          <t>14/23</t>
         </is>
       </c>
       <c r="I185" s="6" t="inlineStr">
@@ -9596,59 +9596,59 @@
         </is>
       </c>
       <c r="J185" s="7" t="n">
-        <v>8931</v>
+        <v>8783</v>
       </c>
       <c r="K185" s="8" t="n">
-        <v>388.3076923076924</v>
+        <v>381.8571428571428</v>
       </c>
     </row>
     <row r="186">
-      <c r="A186" s="6" t="inlineStr">
+      <c r="A186" s="2" t="inlineStr">
         <is>
           <t>THIRUVIDAIMARUDUR</t>
         </is>
       </c>
-      <c r="B186" s="6" t="n">
+      <c r="B186" s="3" t="n">
         <v>170</v>
       </c>
-      <c r="C186" s="6" t="inlineStr">
+      <c r="C186" s="3" t="inlineStr">
         <is>
           <t>GOVI.CHEZHIAAN</t>
         </is>
       </c>
-      <c r="D186" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E186" s="6" t="inlineStr">
+      <c r="D186" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E186" s="3" t="inlineStr">
         <is>
           <t>S.PRABAKARAN</t>
         </is>
       </c>
-      <c r="F186" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G186" s="7" t="n">
-        <v>10311</v>
-      </c>
-      <c r="H186" s="6" t="inlineStr">
-        <is>
-          <t>17/24</t>
-        </is>
-      </c>
-      <c r="I186" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J186" s="7" t="n">
-        <v>14557</v>
-      </c>
-      <c r="K186" s="8" t="n">
-        <v>606.5294117647059</v>
+      <c r="F186" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G186" s="4" t="n">
+        <v>10733</v>
+      </c>
+      <c r="H186" s="3" t="inlineStr">
+        <is>
+          <t>18/24</t>
+        </is>
+      </c>
+      <c r="I186" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J186" s="4" t="n">
+        <v>14311</v>
+      </c>
+      <c r="K186" s="5" t="n">
+        <v>596.2777777777778</v>
       </c>
     </row>
     <row r="187">
@@ -9681,11 +9681,11 @@
         </is>
       </c>
       <c r="G187" s="4" t="n">
-        <v>43236</v>
+        <v>44951</v>
       </c>
       <c r="H187" s="3" t="inlineStr">
         <is>
-          <t>19/25</t>
+          <t>20/25</t>
         </is>
       </c>
       <c r="I187" s="3" t="inlineStr">
@@ -9694,10 +9694,10 @@
         </is>
       </c>
       <c r="J187" s="4" t="n">
-        <v>56889</v>
+        <v>56189</v>
       </c>
       <c r="K187" s="5" t="n">
-        <v>2275.578947368421</v>
+        <v>2247.55</v>
       </c>
     </row>
     <row r="188">
@@ -9730,11 +9730,11 @@
         </is>
       </c>
       <c r="G188" s="4" t="n">
-        <v>12157</v>
+        <v>12127</v>
       </c>
       <c r="H188" s="3" t="inlineStr">
         <is>
-          <t>16/18</t>
+          <t>17/18</t>
         </is>
       </c>
       <c r="I188" s="3" t="inlineStr">
@@ -9743,10 +9743,10 @@
         </is>
       </c>
       <c r="J188" s="4" t="n">
-        <v>13677</v>
+        <v>12840</v>
       </c>
       <c r="K188" s="5" t="n">
-        <v>759.8125</v>
+        <v>713.3529411764706</v>
       </c>
     </row>
     <row r="189">
@@ -9828,11 +9828,11 @@
         </is>
       </c>
       <c r="G190" s="4" t="n">
-        <v>31251</v>
+        <v>32566</v>
       </c>
       <c r="H190" s="3" t="inlineStr">
         <is>
-          <t>20/26</t>
+          <t>21/26</t>
         </is>
       </c>
       <c r="I190" s="3" t="inlineStr">
@@ -9841,59 +9841,59 @@
         </is>
       </c>
       <c r="J190" s="4" t="n">
-        <v>40626</v>
+        <v>40320</v>
       </c>
       <c r="K190" s="5" t="n">
-        <v>1562.55</v>
+        <v>1550.761904761905</v>
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="6" t="inlineStr">
+      <c r="A191" s="2" t="inlineStr">
         <is>
           <t>THOUSAND LIGHTS</t>
         </is>
       </c>
-      <c r="B191" s="6" t="n">
+      <c r="B191" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="C191" s="6" t="inlineStr">
+      <c r="C191" s="3" t="inlineStr">
         <is>
           <t>PRABHAKAR.J.C.D</t>
         </is>
       </c>
-      <c r="D191" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E191" s="6" t="inlineStr">
+      <c r="D191" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E191" s="3" t="inlineStr">
         <is>
           <t>EZHILAN NAGANATHAN</t>
         </is>
       </c>
-      <c r="F191" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G191" s="7" t="n">
-        <v>9977</v>
-      </c>
-      <c r="H191" s="6" t="inlineStr">
-        <is>
-          <t>13/18</t>
-        </is>
-      </c>
-      <c r="I191" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J191" s="7" t="n">
-        <v>13814</v>
-      </c>
-      <c r="K191" s="8" t="n">
-        <v>767.4615384615385</v>
+      <c r="F191" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G191" s="4" t="n">
+        <v>11140</v>
+      </c>
+      <c r="H191" s="3" t="inlineStr">
+        <is>
+          <t>14/18</t>
+        </is>
+      </c>
+      <c r="I191" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J191" s="4" t="n">
+        <v>14323</v>
+      </c>
+      <c r="K191" s="5" t="n">
+        <v>795.7142857142857</v>
       </c>
     </row>
     <row r="192">
@@ -9926,11 +9926,11 @@
         </is>
       </c>
       <c r="G192" s="4" t="n">
-        <v>7558</v>
+        <v>7885</v>
       </c>
       <c r="H192" s="3" t="inlineStr">
         <is>
-          <t>17/22</t>
+          <t>18/22</t>
         </is>
       </c>
       <c r="I192" s="3" t="inlineStr">
@@ -9939,10 +9939,10 @@
         </is>
       </c>
       <c r="J192" s="4" t="n">
-        <v>9781</v>
+        <v>9637</v>
       </c>
       <c r="K192" s="5" t="n">
-        <v>444.5882352941176</v>
+        <v>438.0555555555555</v>
       </c>
     </row>
     <row r="193">
@@ -10180,7 +10180,7 @@
       </c>
       <c r="I197" s="6" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J197" s="7" t="n">
@@ -10240,52 +10240,52 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="9" t="inlineStr">
+      <c r="A199" s="6" t="inlineStr">
         <is>
           <t>TIRUKKOYILUR</t>
         </is>
       </c>
-      <c r="B199" s="10" t="n">
+      <c r="B199" s="6" t="n">
         <v>76</v>
       </c>
-      <c r="C199" s="10" t="inlineStr">
+      <c r="C199" s="6" t="inlineStr">
         <is>
           <t>VIJAY R BARANIBALAAJI</t>
         </is>
       </c>
-      <c r="D199" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E199" s="10" t="inlineStr">
+      <c r="D199" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E199" s="6" t="inlineStr">
         <is>
           <t>PALANISAMY S</t>
         </is>
       </c>
-      <c r="F199" s="10" t="inlineStr">
+      <c r="F199" s="6" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G199" s="11" t="n">
-        <v>1545</v>
-      </c>
-      <c r="H199" s="10" t="inlineStr">
-        <is>
-          <t>16/24</t>
-        </is>
-      </c>
-      <c r="I199" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J199" s="11" t="n">
-        <v>2318</v>
-      </c>
-      <c r="K199" s="12" t="n">
-        <v>96.5625</v>
+      <c r="G199" s="7" t="n">
+        <v>2405</v>
+      </c>
+      <c r="H199" s="6" t="inlineStr">
+        <is>
+          <t>17/24</t>
+        </is>
+      </c>
+      <c r="I199" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J199" s="7" t="n">
+        <v>3395</v>
+      </c>
+      <c r="K199" s="8" t="n">
+        <v>141.4705882352941</v>
       </c>
     </row>
     <row r="200">
@@ -10327,7 +10327,7 @@
       </c>
       <c r="I200" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J200" s="4" t="n">
@@ -10367,11 +10367,11 @@
         </is>
       </c>
       <c r="G201" s="4" t="n">
-        <v>24232</v>
+        <v>27872</v>
       </c>
       <c r="H201" s="3" t="inlineStr">
         <is>
-          <t>12/22</t>
+          <t>13/22</t>
         </is>
       </c>
       <c r="I201" s="3" t="inlineStr">
@@ -10380,10 +10380,10 @@
         </is>
       </c>
       <c r="J201" s="4" t="n">
-        <v>44425</v>
+        <v>47168</v>
       </c>
       <c r="K201" s="5" t="n">
-        <v>2019.333333333333</v>
+        <v>2144</v>
       </c>
     </row>
     <row r="202">
@@ -10465,11 +10465,11 @@
         </is>
       </c>
       <c r="G203" s="4" t="n">
-        <v>42469</v>
+        <v>44545</v>
       </c>
       <c r="H203" s="3" t="inlineStr">
         <is>
-          <t>18/32</t>
+          <t>19/32</t>
         </is>
       </c>
       <c r="I203" s="3" t="inlineStr">
@@ -10478,10 +10478,10 @@
         </is>
       </c>
       <c r="J203" s="4" t="n">
-        <v>75500</v>
+        <v>75023</v>
       </c>
       <c r="K203" s="5" t="n">
-        <v>2359.388888888889</v>
+        <v>2344.473684210526</v>
       </c>
     </row>
     <row r="204">
@@ -10817,7 +10817,7 @@
       </c>
       <c r="I210" s="10" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J210" s="11" t="n">
@@ -10857,11 +10857,11 @@
         </is>
       </c>
       <c r="G211" s="11" t="n">
-        <v>460</v>
+        <v>529</v>
       </c>
       <c r="H211" s="10" t="inlineStr">
         <is>
-          <t>17/27</t>
+          <t>18/27</t>
         </is>
       </c>
       <c r="I211" s="10" t="inlineStr">
@@ -10870,108 +10870,108 @@
         </is>
       </c>
       <c r="J211" s="11" t="n">
-        <v>731</v>
+        <v>794</v>
       </c>
       <c r="K211" s="12" t="n">
-        <v>27.05882352941176</v>
+        <v>29.38888888888889</v>
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="6" t="inlineStr">
+      <c r="A212" s="9" t="inlineStr">
         <is>
           <t>USILAMPATTI</t>
         </is>
       </c>
-      <c r="B212" s="6" t="n">
+      <c r="B212" s="10" t="n">
         <v>197</v>
       </c>
-      <c r="C212" s="6" t="inlineStr">
+      <c r="C212" s="10" t="inlineStr">
         <is>
           <t>VIJAY. M</t>
         </is>
       </c>
-      <c r="D212" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E212" s="6" t="inlineStr">
+      <c r="D212" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E212" s="10" t="inlineStr">
         <is>
           <t>MAHENDRAN. I</t>
         </is>
       </c>
-      <c r="F212" s="6" t="inlineStr">
+      <c r="F212" s="10" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G212" s="7" t="n">
-        <v>1828</v>
-      </c>
-      <c r="H212" s="6" t="inlineStr">
-        <is>
-          <t>13/25</t>
-        </is>
-      </c>
-      <c r="I212" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J212" s="7" t="n">
-        <v>3515</v>
-      </c>
-      <c r="K212" s="8" t="n">
-        <v>140.6153846153846</v>
+      <c r="G212" s="11" t="n">
+        <v>1605</v>
+      </c>
+      <c r="H212" s="10" t="inlineStr">
+        <is>
+          <t>14/25</t>
+        </is>
+      </c>
+      <c r="I212" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J212" s="11" t="n">
+        <v>2866</v>
+      </c>
+      <c r="K212" s="12" t="n">
+        <v>114.6428571428571</v>
       </c>
     </row>
     <row r="213">
-      <c r="A213" s="6" t="inlineStr">
+      <c r="A213" s="2" t="inlineStr">
         <is>
           <t>UTHANGARAI</t>
         </is>
       </c>
-      <c r="B213" s="6" t="n">
+      <c r="B213" s="3" t="n">
         <v>51</v>
       </c>
-      <c r="C213" s="6" t="inlineStr">
+      <c r="C213" s="3" t="inlineStr">
         <is>
           <t>N ELAIYARAJA</t>
         </is>
       </c>
-      <c r="D213" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E213" s="6" t="inlineStr">
+      <c r="D213" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E213" s="3" t="inlineStr">
         <is>
           <t>T M TAMILSELVAM</t>
         </is>
       </c>
-      <c r="F213" s="6" t="inlineStr">
+      <c r="F213" s="3" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G213" s="7" t="n">
-        <v>4435</v>
-      </c>
-      <c r="H213" s="6" t="inlineStr">
-        <is>
-          <t>21/23</t>
-        </is>
-      </c>
-      <c r="I213" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J213" s="7" t="n">
-        <v>4857</v>
-      </c>
-      <c r="K213" s="8" t="n">
-        <v>211.1904761904762</v>
+      <c r="G213" s="4" t="n">
+        <v>5236</v>
+      </c>
+      <c r="H213" s="3" t="inlineStr">
+        <is>
+          <t>22/25</t>
+        </is>
+      </c>
+      <c r="I213" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J213" s="4" t="n">
+        <v>5950</v>
+      </c>
+      <c r="K213" s="5" t="n">
+        <v>238</v>
       </c>
     </row>
     <row r="214">
@@ -11249,11 +11249,11 @@
         </is>
       </c>
       <c r="G219" s="4" t="n">
-        <v>7509</v>
+        <v>8369</v>
       </c>
       <c r="H219" s="3" t="inlineStr">
         <is>
-          <t>18/23</t>
+          <t>19/23</t>
         </is>
       </c>
       <c r="I219" s="3" t="inlineStr">
@@ -11262,10 +11262,10 @@
         </is>
       </c>
       <c r="J219" s="4" t="n">
-        <v>9595</v>
+        <v>10131</v>
       </c>
       <c r="K219" s="5" t="n">
-        <v>417.1666666666667</v>
+        <v>440.4736842105263</v>
       </c>
     </row>
     <row r="220">
@@ -11298,11 +11298,11 @@
         </is>
       </c>
       <c r="G220" s="4" t="n">
-        <v>6721</v>
+        <v>6688</v>
       </c>
       <c r="H220" s="3" t="inlineStr">
         <is>
-          <t>14/18</t>
+          <t>15/18</t>
         </is>
       </c>
       <c r="I220" s="3" t="inlineStr">
@@ -11311,10 +11311,10 @@
         </is>
       </c>
       <c r="J220" s="4" t="n">
-        <v>8641</v>
+        <v>8026</v>
       </c>
       <c r="K220" s="5" t="n">
-        <v>480.0714285714286</v>
+        <v>445.8666666666667</v>
       </c>
     </row>
     <row r="221">
@@ -11347,11 +11347,11 @@
         </is>
       </c>
       <c r="G221" s="4" t="n">
-        <v>8515</v>
+        <v>9353</v>
       </c>
       <c r="H221" s="3" t="inlineStr">
         <is>
-          <t>18/24</t>
+          <t>19/24</t>
         </is>
       </c>
       <c r="I221" s="3" t="inlineStr">
@@ -11360,10 +11360,10 @@
         </is>
       </c>
       <c r="J221" s="4" t="n">
-        <v>11353</v>
+        <v>11814</v>
       </c>
       <c r="K221" s="5" t="n">
-        <v>473.0555555555555</v>
+        <v>492.2631578947368</v>
       </c>
     </row>
     <row r="222">
@@ -11543,11 +11543,11 @@
         </is>
       </c>
       <c r="G225" s="11" t="n">
-        <v>1058</v>
+        <v>787</v>
       </c>
       <c r="H225" s="10" t="inlineStr">
         <is>
-          <t>21/25</t>
+          <t>22/25</t>
         </is>
       </c>
       <c r="I225" s="10" t="inlineStr">
@@ -11556,10 +11556,10 @@
         </is>
       </c>
       <c r="J225" s="11" t="n">
-        <v>1260</v>
+        <v>894</v>
       </c>
       <c r="K225" s="12" t="n">
-        <v>50.38095238095238</v>
+        <v>35.77272727272727</v>
       </c>
     </row>
     <row r="226">
@@ -11690,11 +11690,11 @@
         </is>
       </c>
       <c r="G228" s="4" t="n">
-        <v>16705</v>
+        <v>17410</v>
       </c>
       <c r="H228" s="3" t="inlineStr">
         <is>
-          <t>16/22</t>
+          <t>17/22</t>
         </is>
       </c>
       <c r="I228" s="3" t="inlineStr">
@@ -11703,10 +11703,10 @@
         </is>
       </c>
       <c r="J228" s="4" t="n">
-        <v>22969</v>
+        <v>22531</v>
       </c>
       <c r="K228" s="5" t="n">
-        <v>1044.0625</v>
+        <v>1024.117647058823</v>
       </c>
     </row>
     <row r="229">
@@ -11759,52 +11759,52 @@
       </c>
     </row>
     <row r="230">
-      <c r="A230" s="9" t="inlineStr">
+      <c r="A230" s="6" t="inlineStr">
         <is>
           <t>VILUPPURAM</t>
         </is>
       </c>
-      <c r="B230" s="10" t="n">
+      <c r="B230" s="6" t="n">
         <v>74</v>
       </c>
-      <c r="C230" s="10" t="inlineStr">
+      <c r="C230" s="6" t="inlineStr">
         <is>
           <t>LAKSHMANAN R</t>
         </is>
       </c>
-      <c r="D230" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E230" s="10" t="inlineStr">
+      <c r="D230" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E230" s="6" t="inlineStr">
         <is>
           <t>MOHANRAJ N</t>
         </is>
       </c>
-      <c r="F230" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G230" s="11" t="n">
-        <v>2054</v>
-      </c>
-      <c r="H230" s="10" t="inlineStr">
-        <is>
-          <t>19/24</t>
-        </is>
-      </c>
-      <c r="I230" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J230" s="11" t="n">
-        <v>2595</v>
-      </c>
-      <c r="K230" s="12" t="n">
-        <v>108.1052631578947</v>
+      <c r="F230" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G230" s="7" t="n">
+        <v>2856</v>
+      </c>
+      <c r="H230" s="6" t="inlineStr">
+        <is>
+          <t>20/24</t>
+        </is>
+      </c>
+      <c r="I230" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J230" s="7" t="n">
+        <v>3427</v>
+      </c>
+      <c r="K230" s="8" t="n">
+        <v>142.8</v>
       </c>
     </row>
     <row r="231">
@@ -12004,52 +12004,52 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="9" t="inlineStr">
+      <c r="A235" s="6" t="inlineStr">
         <is>
           <t>YERCAUD</t>
         </is>
       </c>
-      <c r="B235" s="10" t="n">
+      <c r="B235" s="6" t="n">
         <v>83</v>
       </c>
-      <c r="C235" s="10" t="inlineStr">
+      <c r="C235" s="6" t="inlineStr">
         <is>
           <t>LAKSHMI JANARTHANAN. J</t>
         </is>
       </c>
-      <c r="D235" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E235" s="10" t="inlineStr">
+      <c r="D235" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E235" s="6" t="inlineStr">
         <is>
           <t>USHARANI. P</t>
         </is>
       </c>
-      <c r="F235" s="10" t="inlineStr">
+      <c r="F235" s="6" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G235" s="11" t="n">
-        <v>1190</v>
-      </c>
-      <c r="H235" s="10" t="inlineStr">
-        <is>
-          <t>14/24</t>
-        </is>
-      </c>
-      <c r="I235" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J235" s="11" t="n">
-        <v>2040</v>
-      </c>
-      <c r="K235" s="12" t="n">
-        <v>85</v>
+      <c r="G235" s="7" t="n">
+        <v>1936</v>
+      </c>
+      <c r="H235" s="6" t="inlineStr">
+        <is>
+          <t>15/24</t>
+        </is>
+      </c>
+      <c r="I235" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J235" s="7" t="n">
+        <v>3098</v>
+      </c>
+      <c r="K235" s="8" t="n">
+        <v>129.0666666666667</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update election results snapshot (78.6% counted)
TVK 109, DMK 59, AIADMK 44. 15 declared total. KUMBAKONAM last knife-edge
at 86-vote DMK lead with 3 rounds left. NILAKKOTTAI flipped to TVK again.

https://claude.ai/code/session_01MizbUy44JG5sXyvaf3Wekb
</commit_message>
<xml_diff>
--- a/tn_election_results_may2026.xlsx
+++ b/tn_election_results_may2026.xlsx
@@ -665,11 +665,11 @@
         </is>
       </c>
       <c r="G3" s="7" t="n">
-        <v>6581</v>
+        <v>7210</v>
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
-          <t>12/20</t>
+          <t>13/20</t>
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr">
@@ -678,10 +678,10 @@
         </is>
       </c>
       <c r="J3" s="7" t="n">
-        <v>10968</v>
+        <v>11092</v>
       </c>
       <c r="K3" s="8" t="n">
-        <v>548.4166666666666</v>
+        <v>554.6153846153846</v>
       </c>
     </row>
     <row r="4">
@@ -812,11 +812,11 @@
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>44693</v>
+        <v>46605</v>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>19/27</t>
+          <t>20/27</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -825,10 +825,10 @@
         </is>
       </c>
       <c r="J6" s="4" t="n">
-        <v>63511</v>
+        <v>62917</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>2352.263157894737</v>
+        <v>2330.25</v>
       </c>
     </row>
     <row r="7">
@@ -910,11 +910,11 @@
         </is>
       </c>
       <c r="G8" s="7" t="n">
-        <v>7134</v>
+        <v>6436</v>
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>15/22</t>
+          <t>16/22</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
@@ -923,59 +923,59 @@
         </is>
       </c>
       <c r="J8" s="7" t="n">
-        <v>10463</v>
+        <v>8850</v>
       </c>
       <c r="K8" s="8" t="n">
-        <v>475.6000000000001</v>
+        <v>402.25</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>ANDIPATTI</t>
         </is>
       </c>
-      <c r="B9" s="6" t="n">
+      <c r="B9" s="3" t="n">
         <v>198</v>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>MAHARAJAN.A</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>LOGIRAJAN.A</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G9" s="7" t="n">
-        <v>4266</v>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>18/25</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J9" s="7" t="n">
-        <v>5925</v>
-      </c>
-      <c r="K9" s="8" t="n">
-        <v>237</v>
+      <c r="G9" s="4" t="n">
+        <v>5250</v>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>19/25</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>6908</v>
+      </c>
+      <c r="K9" s="5" t="n">
+        <v>276.3157894736842</v>
       </c>
     </row>
     <row r="10">
@@ -1302,11 +1302,11 @@
         </is>
       </c>
       <c r="G16" s="4" t="n">
-        <v>18192</v>
+        <v>21465</v>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>13/23</t>
+          <t>14/23</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
@@ -1315,10 +1315,10 @@
         </is>
       </c>
       <c r="J16" s="4" t="n">
-        <v>32186</v>
+        <v>35264</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>1399.384615384615</v>
+        <v>1533.214285714286</v>
       </c>
     </row>
     <row r="17">
@@ -1351,11 +1351,11 @@
         </is>
       </c>
       <c r="G17" s="4" t="n">
-        <v>24326</v>
+        <v>24498</v>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>24/25</t>
+          <t>25/25</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -1364,59 +1364,59 @@
         </is>
       </c>
       <c r="J17" s="4" t="n">
-        <v>25340</v>
+        <v>24498</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>1013.583333333333</v>
+        <v>979.92</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="inlineStr">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>ARUPPUKKOTTAI</t>
         </is>
       </c>
-      <c r="B18" s="14" t="n">
+      <c r="B18" s="10" t="n">
         <v>207</v>
       </c>
-      <c r="C18" s="14" t="inlineStr">
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>RAMACHANDRAN. K.K.S.S.R</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
         <is>
           <t>KARTHIK KUMAR. K</t>
         </is>
       </c>
-      <c r="D18" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E18" s="14" t="inlineStr">
-        <is>
-          <t>RAMACHANDRAN. K.K.S.S.R</t>
-        </is>
-      </c>
-      <c r="F18" s="14" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G18" s="15" t="n">
-        <v>278</v>
-      </c>
-      <c r="H18" s="14" t="inlineStr">
-        <is>
-          <t>15/20</t>
-        </is>
-      </c>
-      <c r="I18" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J18" s="15" t="n">
-        <v>371</v>
-      </c>
-      <c r="K18" s="16" t="n">
-        <v>18.53333333333333</v>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="n">
+        <v>1217</v>
+      </c>
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t>16/20</t>
+        </is>
+      </c>
+      <c r="I18" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J18" s="11" t="n">
+        <v>1521</v>
+      </c>
+      <c r="K18" s="12" t="n">
+        <v>76.0625</v>
       </c>
     </row>
     <row r="19">
@@ -1449,11 +1449,11 @@
         </is>
       </c>
       <c r="G19" s="4" t="n">
-        <v>21702</v>
+        <v>21944</v>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>18/25</t>
+          <t>19/25</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -1462,10 +1462,10 @@
         </is>
       </c>
       <c r="J19" s="4" t="n">
-        <v>30142</v>
+        <v>28874</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>1205.666666666667</v>
+        <v>1154.947368421053</v>
       </c>
     </row>
     <row r="20">
@@ -1547,11 +1547,11 @@
         </is>
       </c>
       <c r="G21" s="4" t="n">
-        <v>44512</v>
+        <v>48013</v>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>16/26</t>
+          <t>17/26</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -1560,59 +1560,59 @@
         </is>
       </c>
       <c r="J21" s="4" t="n">
-        <v>72332</v>
+        <v>73432</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>2782</v>
+        <v>2824.294117647059</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>AVANASHI</t>
         </is>
       </c>
-      <c r="B22" s="6" t="n">
+      <c r="B22" s="3" t="n">
         <v>112</v>
       </c>
-      <c r="C22" s="6" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>KAMALI.S</t>
         </is>
       </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>DR. L. MURUGAN</t>
         </is>
       </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>Bharatiya Janata Party</t>
         </is>
       </c>
-      <c r="G22" s="7" t="n">
-        <v>8929</v>
-      </c>
-      <c r="H22" s="6" t="inlineStr">
-        <is>
-          <t>20/27</t>
-        </is>
-      </c>
-      <c r="I22" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J22" s="7" t="n">
-        <v>12054</v>
-      </c>
-      <c r="K22" s="8" t="n">
-        <v>446.45</v>
+      <c r="G22" s="4" t="n">
+        <v>8737</v>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>21/27</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>11233</v>
+      </c>
+      <c r="K22" s="5" t="n">
+        <v>416.047619047619</v>
       </c>
     </row>
     <row r="23">
@@ -1694,11 +1694,11 @@
         </is>
       </c>
       <c r="G24" s="7" t="n">
-        <v>7238</v>
+        <v>5949</v>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>14/22</t>
+          <t>15/22</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr">
@@ -1707,10 +1707,10 @@
         </is>
       </c>
       <c r="J24" s="7" t="n">
-        <v>11374</v>
+        <v>8725</v>
       </c>
       <c r="K24" s="8" t="n">
-        <v>517</v>
+        <v>396.6</v>
       </c>
     </row>
     <row r="25">
@@ -1743,11 +1743,11 @@
         </is>
       </c>
       <c r="G25" s="7" t="n">
-        <v>2720</v>
+        <v>4257</v>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>21/24</t>
+          <t>22/24</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
@@ -1756,10 +1756,10 @@
         </is>
       </c>
       <c r="J25" s="7" t="n">
-        <v>3109</v>
+        <v>4644</v>
       </c>
       <c r="K25" s="8" t="n">
-        <v>129.5238095238095</v>
+        <v>193.5</v>
       </c>
     </row>
     <row r="26">
@@ -1841,11 +1841,11 @@
         </is>
       </c>
       <c r="G27" s="7" t="n">
-        <v>3697</v>
+        <v>3567</v>
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>18/25</t>
+          <t>19/25</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
@@ -1854,10 +1854,10 @@
         </is>
       </c>
       <c r="J27" s="7" t="n">
-        <v>5135</v>
+        <v>4693</v>
       </c>
       <c r="K27" s="8" t="n">
-        <v>205.3888888888889</v>
+        <v>187.7368421052632</v>
       </c>
     </row>
     <row r="28">
@@ -1890,11 +1890,11 @@
         </is>
       </c>
       <c r="G28" s="4" t="n">
-        <v>15969</v>
+        <v>17527</v>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>15/36</t>
+          <t>16/36</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
@@ -1903,10 +1903,10 @@
         </is>
       </c>
       <c r="J28" s="4" t="n">
-        <v>38326</v>
+        <v>39436</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>1064.6</v>
+        <v>1095.4375</v>
       </c>
     </row>
     <row r="29">
@@ -1939,11 +1939,11 @@
         </is>
       </c>
       <c r="G29" s="7" t="n">
-        <v>8143</v>
+        <v>9030</v>
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>14/25</t>
+          <t>15/25</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
@@ -1952,10 +1952,10 @@
         </is>
       </c>
       <c r="J29" s="7" t="n">
-        <v>14541</v>
+        <v>15050</v>
       </c>
       <c r="K29" s="8" t="n">
-        <v>581.6428571428571</v>
+        <v>602</v>
       </c>
     </row>
     <row r="30">
@@ -1988,11 +1988,11 @@
         </is>
       </c>
       <c r="G30" s="4" t="n">
-        <v>9881</v>
+        <v>10209</v>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>13/17</t>
+          <t>14/17</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
@@ -2001,10 +2001,10 @@
         </is>
       </c>
       <c r="J30" s="4" t="n">
-        <v>12921</v>
+        <v>12397</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>760.0769230769231</v>
+        <v>729.2142857142857</v>
       </c>
     </row>
     <row r="31">
@@ -2057,52 +2057,52 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="inlineStr">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>CHEYYUR</t>
         </is>
       </c>
-      <c r="B32" s="6" t="n">
+      <c r="B32" s="3" t="n">
         <v>34</v>
       </c>
-      <c r="C32" s="6" t="inlineStr">
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>RAJASEKAR. E</t>
         </is>
       </c>
-      <c r="D32" s="6" t="inlineStr">
+      <c r="D32" s="3" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E32" s="6" t="inlineStr">
+      <c r="E32" s="3" t="inlineStr">
         <is>
           <t>MOHAN RAJA.M.G.K</t>
         </is>
       </c>
-      <c r="F32" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G32" s="7" t="n">
-        <v>3784</v>
-      </c>
-      <c r="H32" s="6" t="inlineStr">
-        <is>
-          <t>19/21</t>
-        </is>
-      </c>
-      <c r="I32" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J32" s="7" t="n">
-        <v>4182</v>
-      </c>
-      <c r="K32" s="8" t="n">
-        <v>199.1578947368421</v>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="n">
+        <v>5539</v>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>20/21</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J32" s="4" t="n">
+        <v>5816</v>
+      </c>
+      <c r="K32" s="5" t="n">
+        <v>276.95</v>
       </c>
     </row>
     <row r="33">
@@ -2184,11 +2184,11 @@
         </is>
       </c>
       <c r="G34" s="4" t="n">
-        <v>11586</v>
+        <v>12478</v>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>12/25</t>
+          <t>13/25</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
@@ -2197,10 +2197,10 @@
         </is>
       </c>
       <c r="J34" s="4" t="n">
-        <v>24138</v>
+        <v>23996</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>965.5</v>
+        <v>959.8461538461538</v>
       </c>
     </row>
     <row r="35">
@@ -2233,11 +2233,11 @@
         </is>
       </c>
       <c r="G35" s="7" t="n">
-        <v>2675</v>
+        <v>6167</v>
       </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>13/20</t>
+          <t>14/20</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
@@ -2246,10 +2246,10 @@
         </is>
       </c>
       <c r="J35" s="7" t="n">
-        <v>4115</v>
+        <v>8810</v>
       </c>
       <c r="K35" s="8" t="n">
-        <v>205.7692307692308</v>
+        <v>440.5</v>
       </c>
     </row>
     <row r="36">
@@ -2282,11 +2282,11 @@
         </is>
       </c>
       <c r="G36" s="7" t="n">
-        <v>3138</v>
+        <v>2570</v>
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>14/23</t>
+          <t>15/23</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
@@ -2295,10 +2295,10 @@
         </is>
       </c>
       <c r="J36" s="7" t="n">
-        <v>5155</v>
+        <v>3941</v>
       </c>
       <c r="K36" s="8" t="n">
-        <v>224.1428571428571</v>
+        <v>171.3333333333333</v>
       </c>
     </row>
     <row r="37">
@@ -2380,11 +2380,11 @@
         </is>
       </c>
       <c r="G38" s="4" t="n">
-        <v>13034</v>
+        <v>14659</v>
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>16/19</t>
+          <t>17/19</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
@@ -2393,10 +2393,10 @@
         </is>
       </c>
       <c r="J38" s="4" t="n">
-        <v>15478</v>
+        <v>16384</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>814.625</v>
+        <v>862.2941176470588</v>
       </c>
     </row>
     <row r="39">
@@ -2478,11 +2478,11 @@
         </is>
       </c>
       <c r="G40" s="4" t="n">
-        <v>15442</v>
+        <v>16579</v>
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>22/23</t>
+          <t>23/24</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
@@ -2491,10 +2491,10 @@
         </is>
       </c>
       <c r="J40" s="4" t="n">
-        <v>16144</v>
+        <v>17300</v>
       </c>
       <c r="K40" s="5" t="n">
-        <v>701.9090909090909</v>
+        <v>720.8260869565217</v>
       </c>
     </row>
     <row r="41">
@@ -2527,11 +2527,11 @@
         </is>
       </c>
       <c r="G41" s="4" t="n">
-        <v>17366</v>
+        <v>20301</v>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>21/23</t>
+          <t>22/23</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
@@ -2540,59 +2540,59 @@
         </is>
       </c>
       <c r="J41" s="4" t="n">
-        <v>19020</v>
+        <v>21224</v>
       </c>
       <c r="K41" s="5" t="n">
-        <v>826.952380952381</v>
+        <v>922.7727272727273</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="13" t="inlineStr">
+      <c r="A42" s="9" t="inlineStr">
         <is>
           <t>DINDIGUL</t>
         </is>
       </c>
-      <c r="B42" s="14" t="n">
+      <c r="B42" s="10" t="n">
         <v>132</v>
       </c>
-      <c r="C42" s="14" t="inlineStr">
+      <c r="C42" s="10" t="inlineStr">
         <is>
           <t>SENTHILKUMAR. I.P</t>
         </is>
       </c>
-      <c r="D42" s="14" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E42" s="14" t="inlineStr">
+      <c r="D42" s="10" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E42" s="10" t="inlineStr">
         <is>
           <t>NAZEER RAJA. G</t>
         </is>
       </c>
-      <c r="F42" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G42" s="15" t="n">
-        <v>279</v>
-      </c>
-      <c r="H42" s="14" t="inlineStr">
-        <is>
-          <t>22/26</t>
-        </is>
-      </c>
-      <c r="I42" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J42" s="15" t="n">
-        <v>330</v>
-      </c>
-      <c r="K42" s="16" t="n">
-        <v>12.68181818181818</v>
+      <c r="F42" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G42" s="11" t="n">
+        <v>574</v>
+      </c>
+      <c r="H42" s="10" t="inlineStr">
+        <is>
+          <t>24/26</t>
+        </is>
+      </c>
+      <c r="I42" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J42" s="11" t="n">
+        <v>622</v>
+      </c>
+      <c r="K42" s="12" t="n">
+        <v>23.91666666666667</v>
       </c>
     </row>
     <row r="43">
@@ -2625,11 +2625,11 @@
         </is>
       </c>
       <c r="G43" s="4" t="n">
-        <v>24744</v>
+        <v>29688</v>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>10/18</t>
+          <t>11/18</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
@@ -2638,10 +2638,10 @@
         </is>
       </c>
       <c r="J43" s="4" t="n">
-        <v>44539</v>
+        <v>48580</v>
       </c>
       <c r="K43" s="5" t="n">
-        <v>2474.4</v>
+        <v>2698.909090909091</v>
       </c>
     </row>
     <row r="44">
@@ -2674,11 +2674,11 @@
         </is>
       </c>
       <c r="G44" s="4" t="n">
-        <v>92619</v>
+        <v>96471</v>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
-          <t>23/25</t>
+          <t>24/25</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
@@ -2687,10 +2687,10 @@
         </is>
       </c>
       <c r="J44" s="4" t="n">
-        <v>100673</v>
+        <v>100491</v>
       </c>
       <c r="K44" s="5" t="n">
-        <v>4026.913043478261</v>
+        <v>4019.625</v>
       </c>
     </row>
     <row r="45">
@@ -2723,11 +2723,11 @@
         </is>
       </c>
       <c r="G45" s="4" t="n">
-        <v>11336</v>
+        <v>10804</v>
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>14/15</t>
+          <t>15/15</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
@@ -2736,10 +2736,10 @@
         </is>
       </c>
       <c r="J45" s="4" t="n">
-        <v>12146</v>
+        <v>10804</v>
       </c>
       <c r="K45" s="5" t="n">
-        <v>809.7142857142857</v>
+        <v>720.2666666666667</v>
       </c>
     </row>
     <row r="46">
@@ -2821,11 +2821,11 @@
         </is>
       </c>
       <c r="G47" s="4" t="n">
-        <v>21517</v>
+        <v>21643</v>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>18/24</t>
+          <t>19/24</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
@@ -2834,10 +2834,10 @@
         </is>
       </c>
       <c r="J47" s="4" t="n">
-        <v>28689</v>
+        <v>27339</v>
       </c>
       <c r="K47" s="5" t="n">
-        <v>1195.388888888889</v>
+        <v>1139.105263157895</v>
       </c>
     </row>
     <row r="48">
@@ -2870,11 +2870,11 @@
         </is>
       </c>
       <c r="G48" s="7" t="n">
-        <v>7935</v>
+        <v>7970</v>
       </c>
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>12/18</t>
+          <t>13/18</t>
         </is>
       </c>
       <c r="I48" s="6" t="inlineStr">
@@ -2883,10 +2883,10 @@
         </is>
       </c>
       <c r="J48" s="7" t="n">
-        <v>11902</v>
+        <v>11035</v>
       </c>
       <c r="K48" s="8" t="n">
-        <v>661.25</v>
+        <v>613.0769230769231</v>
       </c>
     </row>
     <row r="49">
@@ -2919,11 +2919,11 @@
         </is>
       </c>
       <c r="G49" s="4" t="n">
-        <v>14379</v>
+        <v>14772</v>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>16/20</t>
+          <t>17/20</t>
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr">
@@ -2932,10 +2932,10 @@
         </is>
       </c>
       <c r="J49" s="4" t="n">
-        <v>17974</v>
+        <v>17379</v>
       </c>
       <c r="K49" s="5" t="n">
-        <v>898.6875</v>
+        <v>868.9411764705883</v>
       </c>
     </row>
     <row r="50">
@@ -3115,11 +3115,11 @@
         </is>
       </c>
       <c r="G53" s="4" t="n">
-        <v>6105</v>
+        <v>6580</v>
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>19/23</t>
+          <t>20/23</t>
         </is>
       </c>
       <c r="I53" s="3" t="inlineStr">
@@ -3128,10 +3128,10 @@
         </is>
       </c>
       <c r="J53" s="4" t="n">
-        <v>7390</v>
+        <v>7567</v>
       </c>
       <c r="K53" s="5" t="n">
-        <v>321.3157894736842</v>
+        <v>329</v>
       </c>
     </row>
     <row r="54">
@@ -3213,11 +3213,11 @@
         </is>
       </c>
       <c r="G55" s="4" t="n">
-        <v>10639</v>
+        <v>10520</v>
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>12/14</t>
+          <t>13/14</t>
         </is>
       </c>
       <c r="I55" s="3" t="inlineStr">
@@ -3226,10 +3226,10 @@
         </is>
       </c>
       <c r="J55" s="4" t="n">
-        <v>12412</v>
+        <v>11329</v>
       </c>
       <c r="K55" s="5" t="n">
-        <v>886.5833333333334</v>
+        <v>809.2307692307693</v>
       </c>
     </row>
     <row r="56">
@@ -3311,11 +3311,11 @@
         </is>
       </c>
       <c r="G57" s="4" t="n">
-        <v>24817</v>
+        <v>24775</v>
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>20/34</t>
+          <t>21/34</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr">
@@ -3324,10 +3324,10 @@
         </is>
       </c>
       <c r="J57" s="4" t="n">
-        <v>42189</v>
+        <v>40112</v>
       </c>
       <c r="K57" s="5" t="n">
-        <v>1240.85</v>
+        <v>1179.761904761905</v>
       </c>
     </row>
     <row r="58">
@@ -3360,11 +3360,11 @@
         </is>
       </c>
       <c r="G58" s="4" t="n">
-        <v>14778</v>
+        <v>16273</v>
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>20/23</t>
+          <t>21/23</t>
         </is>
       </c>
       <c r="I58" s="3" t="inlineStr">
@@ -3373,10 +3373,10 @@
         </is>
       </c>
       <c r="J58" s="4" t="n">
-        <v>16995</v>
+        <v>17823</v>
       </c>
       <c r="K58" s="5" t="n">
-        <v>738.9</v>
+        <v>774.9047619047619</v>
       </c>
     </row>
     <row r="59">
@@ -3556,11 +3556,11 @@
         </is>
       </c>
       <c r="G62" s="7" t="n">
-        <v>2180</v>
+        <v>2319</v>
       </c>
       <c r="H62" s="6" t="inlineStr">
         <is>
-          <t>17/27</t>
+          <t>18/27</t>
         </is>
       </c>
       <c r="I62" s="6" t="inlineStr">
@@ -3569,10 +3569,10 @@
         </is>
       </c>
       <c r="J62" s="7" t="n">
-        <v>3462</v>
+        <v>3479</v>
       </c>
       <c r="K62" s="8" t="n">
-        <v>128.2352941176471</v>
+        <v>128.8333333333333</v>
       </c>
     </row>
     <row r="63">
@@ -3605,11 +3605,11 @@
         </is>
       </c>
       <c r="G63" s="7" t="n">
-        <v>9005</v>
+        <v>9922</v>
       </c>
       <c r="H63" s="6" t="inlineStr">
         <is>
-          <t>16/26</t>
+          <t>17/26</t>
         </is>
       </c>
       <c r="I63" s="6" t="inlineStr">
@@ -3618,10 +3618,10 @@
         </is>
       </c>
       <c r="J63" s="7" t="n">
-        <v>14633</v>
+        <v>15175</v>
       </c>
       <c r="K63" s="8" t="n">
-        <v>562.8125</v>
+        <v>583.6470588235294</v>
       </c>
     </row>
     <row r="64">
@@ -3654,11 +3654,11 @@
         </is>
       </c>
       <c r="G64" s="7" t="n">
-        <v>6410</v>
+        <v>8009</v>
       </c>
       <c r="H64" s="6" t="inlineStr">
         <is>
-          <t>16/23</t>
+          <t>17/23</t>
         </is>
       </c>
       <c r="I64" s="6" t="inlineStr">
@@ -3667,10 +3667,10 @@
         </is>
       </c>
       <c r="J64" s="7" t="n">
-        <v>9214</v>
+        <v>10836</v>
       </c>
       <c r="K64" s="8" t="n">
-        <v>400.625</v>
+        <v>471.1176470588235</v>
       </c>
     </row>
     <row r="65">
@@ -3703,11 +3703,11 @@
         </is>
       </c>
       <c r="G65" s="7" t="n">
-        <v>4874</v>
+        <v>5147</v>
       </c>
       <c r="H65" s="6" t="inlineStr">
         <is>
-          <t>17/26</t>
+          <t>18/26</t>
         </is>
       </c>
       <c r="I65" s="6" t="inlineStr">
@@ -3716,10 +3716,10 @@
         </is>
       </c>
       <c r="J65" s="7" t="n">
-        <v>7454</v>
+        <v>7435</v>
       </c>
       <c r="K65" s="8" t="n">
-        <v>286.7058823529412</v>
+        <v>285.9444444444445</v>
       </c>
     </row>
     <row r="66">
@@ -3821,52 +3821,52 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="9" t="inlineStr">
+      <c r="A68" s="6" t="inlineStr">
         <is>
           <t>KATPADI</t>
         </is>
       </c>
-      <c r="B68" s="10" t="n">
+      <c r="B68" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="C68" s="10" t="inlineStr">
+      <c r="C68" s="6" t="inlineStr">
         <is>
           <t>DR M SUDHAKAR</t>
         </is>
       </c>
-      <c r="D68" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E68" s="10" t="inlineStr">
+      <c r="D68" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E68" s="6" t="inlineStr">
         <is>
           <t>V. RAMU</t>
         </is>
       </c>
-      <c r="F68" s="10" t="inlineStr">
+      <c r="F68" s="6" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G68" s="11" t="n">
-        <v>1266</v>
-      </c>
-      <c r="H68" s="10" t="inlineStr">
-        <is>
-          <t>12/20</t>
-        </is>
-      </c>
-      <c r="I68" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J68" s="11" t="n">
-        <v>2110</v>
-      </c>
-      <c r="K68" s="12" t="n">
-        <v>105.5</v>
+      <c r="G68" s="7" t="n">
+        <v>2736</v>
+      </c>
+      <c r="H68" s="6" t="inlineStr">
+        <is>
+          <t>13/20</t>
+        </is>
+      </c>
+      <c r="I68" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J68" s="7" t="n">
+        <v>4209</v>
+      </c>
+      <c r="K68" s="8" t="n">
+        <v>210.4615384615385</v>
       </c>
     </row>
     <row r="69">
@@ -3899,11 +3899,11 @@
         </is>
       </c>
       <c r="G69" s="4" t="n">
-        <v>19630</v>
+        <v>21992</v>
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
-          <t>14/21</t>
+          <t>15/21</t>
         </is>
       </c>
       <c r="I69" s="3" t="inlineStr">
@@ -3912,10 +3912,10 @@
         </is>
       </c>
       <c r="J69" s="4" t="n">
-        <v>29445</v>
+        <v>30789</v>
       </c>
       <c r="K69" s="5" t="n">
-        <v>1402.142857142857</v>
+        <v>1466.133333333333</v>
       </c>
     </row>
     <row r="70">
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="G70" s="4" t="n">
-        <v>41613</v>
+        <v>41054</v>
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
@@ -3961,59 +3961,59 @@
         </is>
       </c>
       <c r="J70" s="4" t="n">
-        <v>44814</v>
+        <v>44212</v>
       </c>
       <c r="K70" s="5" t="n">
-        <v>1600.5</v>
+        <v>1579</v>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="9" t="inlineStr">
+      <c r="A71" s="6" t="inlineStr">
         <is>
           <t>KILLIYOOR</t>
         </is>
       </c>
-      <c r="B71" s="10" t="n">
+      <c r="B71" s="6" t="n">
         <v>234</v>
       </c>
-      <c r="C71" s="10" t="inlineStr">
+      <c r="C71" s="6" t="inlineStr">
         <is>
           <t>RAJESH KUMAR. S</t>
         </is>
       </c>
-      <c r="D71" s="10" t="inlineStr">
+      <c r="D71" s="6" t="inlineStr">
         <is>
           <t>Indian National Congress</t>
         </is>
       </c>
-      <c r="E71" s="10" t="inlineStr">
+      <c r="E71" s="6" t="inlineStr">
         <is>
           <t>SABIN. S</t>
         </is>
       </c>
-      <c r="F71" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G71" s="11" t="n">
-        <v>1987</v>
-      </c>
-      <c r="H71" s="10" t="inlineStr">
-        <is>
-          <t>17/22</t>
-        </is>
-      </c>
-      <c r="I71" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J71" s="11" t="n">
-        <v>2571</v>
-      </c>
-      <c r="K71" s="12" t="n">
-        <v>116.8823529411765</v>
+      <c r="F71" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G71" s="7" t="n">
+        <v>2764</v>
+      </c>
+      <c r="H71" s="6" t="inlineStr">
+        <is>
+          <t>18/22</t>
+        </is>
+      </c>
+      <c r="I71" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J71" s="7" t="n">
+        <v>3378</v>
+      </c>
+      <c r="K71" s="8" t="n">
+        <v>153.5555555555555</v>
       </c>
     </row>
     <row r="72">
@@ -4046,11 +4046,11 @@
         </is>
       </c>
       <c r="G72" s="4" t="n">
-        <v>28382</v>
+        <v>29935</v>
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>18/22</t>
+          <t>19/22</t>
         </is>
       </c>
       <c r="I72" s="3" t="inlineStr">
@@ -4059,10 +4059,10 @@
         </is>
       </c>
       <c r="J72" s="4" t="n">
-        <v>34689</v>
+        <v>34662</v>
       </c>
       <c r="K72" s="5" t="n">
-        <v>1576.777777777778</v>
+        <v>1575.526315789474</v>
       </c>
     </row>
     <row r="73">
@@ -4095,11 +4095,11 @@
         </is>
       </c>
       <c r="G73" s="4" t="n">
-        <v>9794</v>
+        <v>11436</v>
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
-          <t>9/19</t>
+          <t>10/19</t>
         </is>
       </c>
       <c r="I73" s="3" t="inlineStr">
@@ -4108,10 +4108,10 @@
         </is>
       </c>
       <c r="J73" s="4" t="n">
-        <v>20676</v>
+        <v>21728</v>
       </c>
       <c r="K73" s="5" t="n">
-        <v>1088.222222222222</v>
+        <v>1143.6</v>
       </c>
     </row>
     <row r="74">
@@ -4144,11 +4144,11 @@
         </is>
       </c>
       <c r="G74" s="11" t="n">
-        <v>1679</v>
+        <v>1524</v>
       </c>
       <c r="H74" s="10" t="inlineStr">
         <is>
-          <t>13/16</t>
+          <t>14/16</t>
         </is>
       </c>
       <c r="I74" s="10" t="inlineStr">
@@ -4157,10 +4157,10 @@
         </is>
       </c>
       <c r="J74" s="11" t="n">
-        <v>2066</v>
+        <v>1742</v>
       </c>
       <c r="K74" s="12" t="n">
-        <v>129.1538461538462</v>
+        <v>108.8571428571429</v>
       </c>
     </row>
     <row r="75">
@@ -4193,11 +4193,11 @@
         </is>
       </c>
       <c r="G75" s="4" t="n">
-        <v>11720</v>
+        <v>11783</v>
       </c>
       <c r="H75" s="3" t="inlineStr">
         <is>
-          <t>28/31</t>
+          <t>29/31</t>
         </is>
       </c>
       <c r="I75" s="3" t="inlineStr">
@@ -4206,10 +4206,10 @@
         </is>
       </c>
       <c r="J75" s="4" t="n">
-        <v>12976</v>
+        <v>12596</v>
       </c>
       <c r="K75" s="5" t="n">
-        <v>418.5714285714286</v>
+        <v>406.3103448275862</v>
       </c>
     </row>
     <row r="76">
@@ -4262,52 +4262,52 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="6" t="inlineStr">
+      <c r="A77" s="9" t="inlineStr">
         <is>
           <t>KOVILPATTI</t>
         </is>
       </c>
-      <c r="B77" s="6" t="n">
+      <c r="B77" s="10" t="n">
         <v>218</v>
       </c>
-      <c r="C77" s="6" t="inlineStr">
+      <c r="C77" s="10" t="inlineStr">
         <is>
           <t>KARUNANITHI.K</t>
         </is>
       </c>
-      <c r="D77" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E77" s="6" t="inlineStr">
+      <c r="D77" s="10" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E77" s="10" t="inlineStr">
         <is>
           <t>BALASUBRAMANIAN.S</t>
         </is>
       </c>
-      <c r="F77" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G77" s="7" t="n">
-        <v>2862</v>
-      </c>
-      <c r="H77" s="6" t="inlineStr">
-        <is>
-          <t>17/23</t>
-        </is>
-      </c>
-      <c r="I77" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J77" s="7" t="n">
-        <v>3872</v>
-      </c>
-      <c r="K77" s="8" t="n">
-        <v>168.3529411764706</v>
+      <c r="F77" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G77" s="11" t="n">
+        <v>1968</v>
+      </c>
+      <c r="H77" s="10" t="inlineStr">
+        <is>
+          <t>18/23</t>
+        </is>
+      </c>
+      <c r="I77" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J77" s="11" t="n">
+        <v>2515</v>
+      </c>
+      <c r="K77" s="12" t="n">
+        <v>109.3333333333333</v>
       </c>
     </row>
     <row r="78">
@@ -4487,11 +4487,11 @@
         </is>
       </c>
       <c r="G81" s="7" t="n">
-        <v>4558</v>
+        <v>5624</v>
       </c>
       <c r="H81" s="6" t="inlineStr">
         <is>
-          <t>16/24</t>
+          <t>17/24</t>
         </is>
       </c>
       <c r="I81" s="6" t="inlineStr">
@@ -4500,10 +4500,10 @@
         </is>
       </c>
       <c r="J81" s="7" t="n">
-        <v>6837</v>
+        <v>7940</v>
       </c>
       <c r="K81" s="8" t="n">
-        <v>284.875</v>
+        <v>330.8235294117647</v>
       </c>
     </row>
     <row r="82">
@@ -4585,11 +4585,11 @@
         </is>
       </c>
       <c r="G83" s="4" t="n">
-        <v>16332</v>
+        <v>16747</v>
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
-          <t>19/25</t>
+          <t>21/25</t>
         </is>
       </c>
       <c r="I83" s="3" t="inlineStr">
@@ -4598,10 +4598,10 @@
         </is>
       </c>
       <c r="J83" s="4" t="n">
-        <v>21489</v>
+        <v>19937</v>
       </c>
       <c r="K83" s="5" t="n">
-        <v>859.578947368421</v>
+        <v>797.4761904761905</v>
       </c>
     </row>
     <row r="84">
@@ -4687,7 +4687,7 @@
       </c>
       <c r="H85" s="10" t="inlineStr">
         <is>
-          <t>18/20</t>
+          <t>18/21</t>
         </is>
       </c>
       <c r="I85" s="10" t="inlineStr">
@@ -4696,7 +4696,7 @@
         </is>
       </c>
       <c r="J85" s="11" t="n">
-        <v>1223</v>
+        <v>1284</v>
       </c>
       <c r="K85" s="12" t="n">
         <v>61.16666666666666</v>
@@ -4732,11 +4732,11 @@
         </is>
       </c>
       <c r="G86" s="7" t="n">
-        <v>5632</v>
+        <v>6444</v>
       </c>
       <c r="H86" s="6" t="inlineStr">
         <is>
-          <t>14/21</t>
+          <t>15/21</t>
         </is>
       </c>
       <c r="I86" s="6" t="inlineStr">
@@ -4745,10 +4745,10 @@
         </is>
       </c>
       <c r="J86" s="7" t="n">
-        <v>8448</v>
+        <v>9022</v>
       </c>
       <c r="K86" s="8" t="n">
-        <v>402.2857142857143</v>
+        <v>429.6</v>
       </c>
     </row>
     <row r="87">
@@ -4830,11 +4830,11 @@
         </is>
       </c>
       <c r="G88" s="4" t="n">
-        <v>18028</v>
+        <v>18320</v>
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>15/19</t>
+          <t>16/19</t>
         </is>
       </c>
       <c r="I88" s="3" t="inlineStr">
@@ -4843,10 +4843,10 @@
         </is>
       </c>
       <c r="J88" s="4" t="n">
-        <v>22835</v>
+        <v>21755</v>
       </c>
       <c r="K88" s="5" t="n">
-        <v>1201.866666666667</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="89">
@@ -4879,11 +4879,11 @@
         </is>
       </c>
       <c r="G89" s="4" t="n">
-        <v>11523</v>
+        <v>14048</v>
       </c>
       <c r="H89" s="3" t="inlineStr">
         <is>
-          <t>23/29</t>
+          <t>24/29</t>
         </is>
       </c>
       <c r="I89" s="3" t="inlineStr">
@@ -4892,10 +4892,10 @@
         </is>
       </c>
       <c r="J89" s="4" t="n">
-        <v>14529</v>
+        <v>16975</v>
       </c>
       <c r="K89" s="5" t="n">
-        <v>501</v>
+        <v>585.3333333333334</v>
       </c>
     </row>
     <row r="90">
@@ -4928,11 +4928,11 @@
         </is>
       </c>
       <c r="G90" s="4" t="n">
-        <v>16203</v>
+        <v>16521</v>
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>16/19</t>
+          <t>17/19</t>
         </is>
       </c>
       <c r="I90" s="3" t="inlineStr">
@@ -4941,10 +4941,10 @@
         </is>
       </c>
       <c r="J90" s="4" t="n">
-        <v>19241</v>
+        <v>18465</v>
       </c>
       <c r="K90" s="5" t="n">
-        <v>1012.6875</v>
+        <v>971.8235294117648</v>
       </c>
     </row>
     <row r="91">
@@ -5075,11 +5075,11 @@
         </is>
       </c>
       <c r="G93" s="4" t="n">
-        <v>6611</v>
+        <v>6572</v>
       </c>
       <c r="H93" s="3" t="inlineStr">
         <is>
-          <t>18/21</t>
+          <t>19/21</t>
         </is>
       </c>
       <c r="I93" s="3" t="inlineStr">
@@ -5088,10 +5088,10 @@
         </is>
       </c>
       <c r="J93" s="4" t="n">
-        <v>7713</v>
+        <v>7264</v>
       </c>
       <c r="K93" s="5" t="n">
-        <v>367.2777777777778</v>
+        <v>345.8947368421053</v>
       </c>
     </row>
     <row r="94">
@@ -5124,11 +5124,11 @@
         </is>
       </c>
       <c r="G94" s="4" t="n">
-        <v>38848</v>
+        <v>42657</v>
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
-          <t>14/25</t>
+          <t>15/25</t>
         </is>
       </c>
       <c r="I94" s="3" t="inlineStr">
@@ -5137,10 +5137,10 @@
         </is>
       </c>
       <c r="J94" s="4" t="n">
-        <v>69371</v>
+        <v>71095</v>
       </c>
       <c r="K94" s="5" t="n">
-        <v>2774.857142857143</v>
+        <v>2843.8</v>
       </c>
     </row>
     <row r="95">
@@ -5222,11 +5222,11 @@
         </is>
       </c>
       <c r="G96" s="4" t="n">
-        <v>10155</v>
+        <v>10930</v>
       </c>
       <c r="H96" s="3" t="inlineStr">
         <is>
-          <t>19/22</t>
+          <t>20/22</t>
         </is>
       </c>
       <c r="I96" s="3" t="inlineStr">
@@ -5235,10 +5235,10 @@
         </is>
       </c>
       <c r="J96" s="4" t="n">
-        <v>11758</v>
+        <v>12023</v>
       </c>
       <c r="K96" s="5" t="n">
-        <v>534.4736842105264</v>
+        <v>546.5</v>
       </c>
     </row>
     <row r="97">
@@ -5320,11 +5320,11 @@
         </is>
       </c>
       <c r="G98" s="11" t="n">
-        <v>561</v>
+        <v>1360</v>
       </c>
       <c r="H98" s="10" t="inlineStr">
         <is>
-          <t>22/25</t>
+          <t>23/25</t>
         </is>
       </c>
       <c r="I98" s="10" t="inlineStr">
@@ -5333,10 +5333,10 @@
         </is>
       </c>
       <c r="J98" s="11" t="n">
-        <v>638</v>
+        <v>1478</v>
       </c>
       <c r="K98" s="12" t="n">
-        <v>25.5</v>
+        <v>59.1304347826087</v>
       </c>
     </row>
     <row r="99">
@@ -5369,11 +5369,11 @@
         </is>
       </c>
       <c r="G99" s="11" t="n">
-        <v>1367</v>
+        <v>1840</v>
       </c>
       <c r="H99" s="10" t="inlineStr">
         <is>
-          <t>19/22</t>
+          <t>20/22</t>
         </is>
       </c>
       <c r="I99" s="10" t="inlineStr">
@@ -5382,10 +5382,10 @@
         </is>
       </c>
       <c r="J99" s="11" t="n">
-        <v>1583</v>
+        <v>2024</v>
       </c>
       <c r="K99" s="12" t="n">
-        <v>71.94736842105263</v>
+        <v>92</v>
       </c>
     </row>
     <row r="100">
@@ -5418,11 +5418,11 @@
         </is>
       </c>
       <c r="G100" s="4" t="n">
-        <v>8336</v>
+        <v>8541</v>
       </c>
       <c r="H100" s="3" t="inlineStr">
         <is>
-          <t>17/22</t>
+          <t>18/22</t>
         </is>
       </c>
       <c r="I100" s="3" t="inlineStr">
@@ -5431,10 +5431,10 @@
         </is>
       </c>
       <c r="J100" s="4" t="n">
-        <v>10788</v>
+        <v>10439</v>
       </c>
       <c r="K100" s="5" t="n">
-        <v>490.3529411764706</v>
+        <v>474.5</v>
       </c>
     </row>
     <row r="101">
@@ -5516,11 +5516,11 @@
         </is>
       </c>
       <c r="G102" s="7" t="n">
-        <v>2349</v>
+        <v>2351</v>
       </c>
       <c r="H102" s="6" t="inlineStr">
         <is>
-          <t>17/26</t>
+          <t>18/26</t>
         </is>
       </c>
       <c r="I102" s="6" t="inlineStr">
@@ -5529,10 +5529,10 @@
         </is>
       </c>
       <c r="J102" s="7" t="n">
-        <v>3593</v>
+        <v>3396</v>
       </c>
       <c r="K102" s="8" t="n">
-        <v>138.1764705882353</v>
+        <v>130.6111111111111</v>
       </c>
     </row>
     <row r="103">
@@ -5565,11 +5565,11 @@
         </is>
       </c>
       <c r="G103" s="11" t="n">
-        <v>360</v>
+        <v>1968</v>
       </c>
       <c r="H103" s="10" t="inlineStr">
         <is>
-          <t>15/24</t>
+          <t>16/24</t>
         </is>
       </c>
       <c r="I103" s="10" t="inlineStr">
@@ -5578,10 +5578,10 @@
         </is>
       </c>
       <c r="J103" s="11" t="n">
-        <v>576</v>
+        <v>2952</v>
       </c>
       <c r="K103" s="12" t="n">
-        <v>24</v>
+        <v>123</v>
       </c>
     </row>
     <row r="104">
@@ -5663,11 +5663,11 @@
         </is>
       </c>
       <c r="G105" s="4" t="n">
-        <v>14509</v>
+        <v>15247</v>
       </c>
       <c r="H105" s="3" t="inlineStr">
         <is>
-          <t>24/30</t>
+          <t>25/30</t>
         </is>
       </c>
       <c r="I105" s="3" t="inlineStr">
@@ -5676,10 +5676,10 @@
         </is>
       </c>
       <c r="J105" s="4" t="n">
-        <v>18136</v>
+        <v>18296</v>
       </c>
       <c r="K105" s="5" t="n">
-        <v>604.5416666666666</v>
+        <v>609.88</v>
       </c>
     </row>
     <row r="106">
@@ -5761,11 +5761,11 @@
         </is>
       </c>
       <c r="G107" s="4" t="n">
-        <v>28928</v>
+        <v>28972</v>
       </c>
       <c r="H107" s="3" t="inlineStr">
         <is>
-          <t>20/21</t>
+          <t>21/21</t>
         </is>
       </c>
       <c r="I107" s="3" t="inlineStr">
@@ -5774,10 +5774,10 @@
         </is>
       </c>
       <c r="J107" s="4" t="n">
-        <v>30374</v>
+        <v>28972</v>
       </c>
       <c r="K107" s="5" t="n">
-        <v>1446.4</v>
+        <v>1379.619047619048</v>
       </c>
     </row>
     <row r="108">
@@ -5810,11 +5810,11 @@
         </is>
       </c>
       <c r="G108" s="7" t="n">
-        <v>9638</v>
+        <v>9313</v>
       </c>
       <c r="H108" s="6" t="inlineStr">
         <is>
-          <t>11/18</t>
+          <t>12/18</t>
         </is>
       </c>
       <c r="I108" s="6" t="inlineStr">
@@ -5823,10 +5823,10 @@
         </is>
       </c>
       <c r="J108" s="7" t="n">
-        <v>15771</v>
+        <v>13970</v>
       </c>
       <c r="K108" s="8" t="n">
-        <v>876.1818181818181</v>
+        <v>776.0833333333334</v>
       </c>
     </row>
     <row r="109">
@@ -5859,7 +5859,7 @@
         </is>
       </c>
       <c r="G109" s="4" t="n">
-        <v>6254</v>
+        <v>6972</v>
       </c>
       <c r="H109" s="3" t="inlineStr">
         <is>
@@ -5872,10 +5872,10 @@
         </is>
       </c>
       <c r="J109" s="4" t="n">
-        <v>6850</v>
+        <v>7636</v>
       </c>
       <c r="K109" s="5" t="n">
-        <v>297.8095238095238</v>
+        <v>332</v>
       </c>
     </row>
     <row r="110">
@@ -6006,11 +6006,11 @@
         </is>
       </c>
       <c r="G112" s="4" t="n">
-        <v>34574</v>
+        <v>36538</v>
       </c>
       <c r="H112" s="3" t="inlineStr">
         <is>
-          <t>21/25</t>
+          <t>22/25</t>
         </is>
       </c>
       <c r="I112" s="3" t="inlineStr">
@@ -6019,59 +6019,59 @@
         </is>
       </c>
       <c r="J112" s="4" t="n">
-        <v>41160</v>
+        <v>41520</v>
       </c>
       <c r="K112" s="5" t="n">
-        <v>1646.380952380952</v>
+        <v>1660.818181818182</v>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="6" t="inlineStr">
+      <c r="A113" s="2" t="inlineStr">
         <is>
           <t>NATHAM</t>
         </is>
       </c>
-      <c r="B113" s="6" t="n">
+      <c r="B113" s="3" t="n">
         <v>131</v>
       </c>
-      <c r="C113" s="6" t="inlineStr">
+      <c r="C113" s="3" t="inlineStr">
         <is>
           <t>NATHAM VISWANATHAN R</t>
         </is>
       </c>
-      <c r="D113" s="6" t="inlineStr">
+      <c r="D113" s="3" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E113" s="6" t="inlineStr">
+      <c r="E113" s="3" t="inlineStr">
         <is>
           <t>SELVAKUMAR K</t>
         </is>
       </c>
-      <c r="F113" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G113" s="7" t="n">
-        <v>11008</v>
-      </c>
-      <c r="H113" s="6" t="inlineStr">
-        <is>
-          <t>19/26</t>
-        </is>
-      </c>
-      <c r="I113" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J113" s="7" t="n">
-        <v>15064</v>
-      </c>
-      <c r="K113" s="8" t="n">
-        <v>579.3684210526316</v>
+      <c r="F113" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G113" s="4" t="n">
+        <v>10719</v>
+      </c>
+      <c r="H113" s="3" t="inlineStr">
+        <is>
+          <t>20/26</t>
+        </is>
+      </c>
+      <c r="I113" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J113" s="4" t="n">
+        <v>13935</v>
+      </c>
+      <c r="K113" s="5" t="n">
+        <v>535.95</v>
       </c>
     </row>
     <row r="114">
@@ -6134,30 +6134,30 @@
       </c>
       <c r="C115" s="10" t="inlineStr">
         <is>
+          <t>AYYANAR.R</t>
+        </is>
+      </c>
+      <c r="D115" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E115" s="10" t="inlineStr">
+        <is>
           <t>NAGAJOTHI.S</t>
         </is>
       </c>
-      <c r="D115" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E115" s="10" t="inlineStr">
-        <is>
-          <t>AYYANAR.R</t>
-        </is>
-      </c>
       <c r="F115" s="10" t="inlineStr">
         <is>
-          <t>Tamilaga Vettri Kazhagam</t>
+          <t>Dravida Munnetra Kazhagam</t>
         </is>
       </c>
       <c r="G115" s="11" t="n">
-        <v>513</v>
+        <v>1246</v>
       </c>
       <c r="H115" s="10" t="inlineStr">
         <is>
-          <t>14/23</t>
+          <t>15/23</t>
         </is>
       </c>
       <c r="I115" s="10" t="inlineStr">
@@ -6166,10 +6166,10 @@
         </is>
       </c>
       <c r="J115" s="11" t="n">
-        <v>843</v>
+        <v>1911</v>
       </c>
       <c r="K115" s="12" t="n">
-        <v>36.64285714285715</v>
+        <v>83.06666666666666</v>
       </c>
     </row>
     <row r="116">
@@ -6202,11 +6202,11 @@
         </is>
       </c>
       <c r="G116" s="4" t="n">
-        <v>35011</v>
+        <v>36954</v>
       </c>
       <c r="H116" s="3" t="inlineStr">
         <is>
-          <t>19/24</t>
+          <t>20/24</t>
         </is>
       </c>
       <c r="I116" s="3" t="inlineStr">
@@ -6215,10 +6215,10 @@
         </is>
       </c>
       <c r="J116" s="4" t="n">
-        <v>44224</v>
+        <v>44345</v>
       </c>
       <c r="K116" s="5" t="n">
-        <v>1842.684210526316</v>
+        <v>1847.7</v>
       </c>
     </row>
     <row r="117">
@@ -6251,11 +6251,11 @@
         </is>
       </c>
       <c r="G117" s="4" t="n">
-        <v>15797</v>
+        <v>15482</v>
       </c>
       <c r="H117" s="3" t="inlineStr">
         <is>
-          <t>21/26</t>
+          <t>22/26</t>
         </is>
       </c>
       <c r="I117" s="3" t="inlineStr">
@@ -6264,10 +6264,10 @@
         </is>
       </c>
       <c r="J117" s="4" t="n">
-        <v>19558</v>
+        <v>18297</v>
       </c>
       <c r="K117" s="5" t="n">
-        <v>752.2380952380952</v>
+        <v>703.7272727272727</v>
       </c>
     </row>
     <row r="118">
@@ -6300,11 +6300,11 @@
         </is>
       </c>
       <c r="G118" s="4" t="n">
-        <v>34977</v>
+        <v>35028</v>
       </c>
       <c r="H118" s="3" t="inlineStr">
         <is>
-          <t>23/24</t>
+          <t>24/24</t>
         </is>
       </c>
       <c r="I118" s="3" t="inlineStr">
@@ -6313,10 +6313,10 @@
         </is>
       </c>
       <c r="J118" s="4" t="n">
-        <v>36498</v>
+        <v>35028</v>
       </c>
       <c r="K118" s="5" t="n">
-        <v>1520.739130434783</v>
+        <v>1459.5</v>
       </c>
     </row>
     <row r="119">
@@ -6349,11 +6349,11 @@
         </is>
       </c>
       <c r="G119" s="4" t="n">
-        <v>23872</v>
+        <v>25087</v>
       </c>
       <c r="H119" s="3" t="inlineStr">
         <is>
-          <t>19/23</t>
+          <t>20/23</t>
         </is>
       </c>
       <c r="I119" s="3" t="inlineStr">
@@ -6362,10 +6362,10 @@
         </is>
       </c>
       <c r="J119" s="4" t="n">
-        <v>28898</v>
+        <v>28850</v>
       </c>
       <c r="K119" s="5" t="n">
-        <v>1256.421052631579</v>
+        <v>1254.35</v>
       </c>
     </row>
     <row r="120">
@@ -6398,11 +6398,11 @@
         </is>
       </c>
       <c r="G120" s="4" t="n">
-        <v>13869</v>
+        <v>13228</v>
       </c>
       <c r="H120" s="3" t="inlineStr">
         <is>
-          <t>18/23</t>
+          <t>19/23</t>
         </is>
       </c>
       <c r="I120" s="3" t="inlineStr">
@@ -6411,10 +6411,10 @@
         </is>
       </c>
       <c r="J120" s="4" t="n">
-        <v>17722</v>
+        <v>16013</v>
       </c>
       <c r="K120" s="5" t="n">
-        <v>770.5</v>
+        <v>696.2105263157895</v>
       </c>
     </row>
     <row r="121">
@@ -6643,11 +6643,11 @@
         </is>
       </c>
       <c r="G125" s="4" t="n">
-        <v>31435</v>
+        <v>33381</v>
       </c>
       <c r="H125" s="3" t="inlineStr">
         <is>
-          <t>19/34</t>
+          <t>20/34</t>
         </is>
       </c>
       <c r="I125" s="3" t="inlineStr">
@@ -6656,10 +6656,10 @@
         </is>
       </c>
       <c r="J125" s="4" t="n">
-        <v>56252</v>
+        <v>56748</v>
       </c>
       <c r="K125" s="5" t="n">
-        <v>1654.473684210526</v>
+        <v>1669.05</v>
       </c>
     </row>
     <row r="126">
@@ -6888,11 +6888,11 @@
         </is>
       </c>
       <c r="G130" s="11" t="n">
-        <v>1172</v>
+        <v>1009</v>
       </c>
       <c r="H130" s="10" t="inlineStr">
         <is>
-          <t>12/20</t>
+          <t>13/20</t>
         </is>
       </c>
       <c r="I130" s="10" t="inlineStr">
@@ -6901,10 +6901,10 @@
         </is>
       </c>
       <c r="J130" s="11" t="n">
-        <v>1953</v>
+        <v>1552</v>
       </c>
       <c r="K130" s="12" t="n">
-        <v>97.66666666666667</v>
+        <v>77.61538461538461</v>
       </c>
     </row>
     <row r="131">
@@ -6986,11 +6986,11 @@
         </is>
       </c>
       <c r="G132" s="7" t="n">
-        <v>4603</v>
+        <v>4797</v>
       </c>
       <c r="H132" s="6" t="inlineStr">
         <is>
-          <t>18/23</t>
+          <t>19/23</t>
         </is>
       </c>
       <c r="I132" s="6" t="inlineStr">
@@ -6999,10 +6999,10 @@
         </is>
       </c>
       <c r="J132" s="7" t="n">
-        <v>5882</v>
+        <v>5807</v>
       </c>
       <c r="K132" s="8" t="n">
-        <v>255.7222222222222</v>
+        <v>252.4736842105263</v>
       </c>
     </row>
     <row r="133">
@@ -7035,11 +7035,11 @@
         </is>
       </c>
       <c r="G133" s="4" t="n">
-        <v>11310</v>
+        <v>12826</v>
       </c>
       <c r="H133" s="3" t="inlineStr">
         <is>
-          <t>23/28</t>
+          <t>24/28</t>
         </is>
       </c>
       <c r="I133" s="3" t="inlineStr">
@@ -7048,10 +7048,10 @@
         </is>
       </c>
       <c r="J133" s="4" t="n">
-        <v>13769</v>
+        <v>14964</v>
       </c>
       <c r="K133" s="5" t="n">
-        <v>491.7391304347826</v>
+        <v>534.4166666666666</v>
       </c>
     </row>
     <row r="134">
@@ -7084,11 +7084,11 @@
         </is>
       </c>
       <c r="G134" s="4" t="n">
-        <v>31766</v>
+        <v>34744</v>
       </c>
       <c r="H134" s="3" t="inlineStr">
         <is>
-          <t>13/22</t>
+          <t>14/22</t>
         </is>
       </c>
       <c r="I134" s="3" t="inlineStr">
@@ -7097,10 +7097,10 @@
         </is>
       </c>
       <c r="J134" s="4" t="n">
-        <v>53758</v>
+        <v>54598</v>
       </c>
       <c r="K134" s="5" t="n">
-        <v>2443.538461538461</v>
+        <v>2481.714285714286</v>
       </c>
     </row>
     <row r="135">
@@ -7231,11 +7231,11 @@
         </is>
       </c>
       <c r="G137" s="4" t="n">
-        <v>8384</v>
+        <v>8907</v>
       </c>
       <c r="H137" s="3" t="inlineStr">
         <is>
-          <t>18/21</t>
+          <t>19/21</t>
         </is>
       </c>
       <c r="I137" s="3" t="inlineStr">
@@ -7244,10 +7244,10 @@
         </is>
       </c>
       <c r="J137" s="4" t="n">
-        <v>9781</v>
+        <v>9845</v>
       </c>
       <c r="K137" s="5" t="n">
-        <v>465.7777777777778</v>
+        <v>468.7894736842105</v>
       </c>
     </row>
     <row r="138">
@@ -7280,11 +7280,11 @@
         </is>
       </c>
       <c r="G138" s="7" t="n">
-        <v>3917</v>
+        <v>4779</v>
       </c>
       <c r="H138" s="6" t="inlineStr">
         <is>
-          <t>19/22</t>
+          <t>20/22</t>
         </is>
       </c>
       <c r="I138" s="6" t="inlineStr">
@@ -7293,10 +7293,10 @@
         </is>
       </c>
       <c r="J138" s="7" t="n">
-        <v>4535</v>
+        <v>5257</v>
       </c>
       <c r="K138" s="8" t="n">
-        <v>206.1578947368421</v>
+        <v>238.95</v>
       </c>
     </row>
     <row r="139">
@@ -7378,11 +7378,11 @@
         </is>
       </c>
       <c r="G140" s="4" t="n">
-        <v>46942</v>
+        <v>49607</v>
       </c>
       <c r="H140" s="3" t="inlineStr">
         <is>
-          <t>20/24</t>
+          <t>21/24</t>
         </is>
       </c>
       <c r="I140" s="3" t="inlineStr">
@@ -7391,10 +7391,10 @@
         </is>
       </c>
       <c r="J140" s="4" t="n">
-        <v>56330</v>
+        <v>56694</v>
       </c>
       <c r="K140" s="5" t="n">
-        <v>2347.1</v>
+        <v>2362.238095238095</v>
       </c>
     </row>
     <row r="141">
@@ -7476,11 +7476,11 @@
         </is>
       </c>
       <c r="G142" s="4" t="n">
-        <v>63006</v>
+        <v>62906</v>
       </c>
       <c r="H142" s="3" t="inlineStr">
         <is>
-          <t>20/23</t>
+          <t>20/25</t>
         </is>
       </c>
       <c r="I142" s="3" t="inlineStr">
@@ -7489,10 +7489,10 @@
         </is>
       </c>
       <c r="J142" s="4" t="n">
-        <v>72457</v>
+        <v>78632</v>
       </c>
       <c r="K142" s="5" t="n">
-        <v>3150.3</v>
+        <v>3145.3</v>
       </c>
     </row>
     <row r="143">
@@ -7583,7 +7583,7 @@
       </c>
       <c r="I144" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J144" s="4" t="n">
@@ -7623,11 +7623,11 @@
         </is>
       </c>
       <c r="G145" s="4" t="n">
-        <v>10807</v>
+        <v>10654</v>
       </c>
       <c r="H145" s="3" t="inlineStr">
         <is>
-          <t>18/20</t>
+          <t>18/21</t>
         </is>
       </c>
       <c r="I145" s="3" t="inlineStr">
@@ -7636,10 +7636,10 @@
         </is>
       </c>
       <c r="J145" s="4" t="n">
-        <v>12008</v>
+        <v>12430</v>
       </c>
       <c r="K145" s="5" t="n">
-        <v>600.3888888888889</v>
+        <v>591.8888888888889</v>
       </c>
     </row>
     <row r="146">
@@ -7672,11 +7672,11 @@
         </is>
       </c>
       <c r="G146" s="4" t="n">
-        <v>13101</v>
+        <v>12560</v>
       </c>
       <c r="H146" s="3" t="inlineStr">
         <is>
-          <t>28/29</t>
+          <t>30/31</t>
         </is>
       </c>
       <c r="I146" s="3" t="inlineStr">
@@ -7685,59 +7685,59 @@
         </is>
       </c>
       <c r="J146" s="4" t="n">
-        <v>13569</v>
+        <v>12979</v>
       </c>
       <c r="K146" s="5" t="n">
-        <v>467.8928571428572</v>
+        <v>418.6666666666667</v>
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="6" t="inlineStr">
+      <c r="A147" s="2" t="inlineStr">
         <is>
           <t>RANIPET</t>
         </is>
       </c>
-      <c r="B147" s="6" t="n">
+      <c r="B147" s="3" t="n">
         <v>41</v>
       </c>
-      <c r="C147" s="6" t="inlineStr">
+      <c r="C147" s="3" t="inlineStr">
         <is>
           <t>THAHIRA</t>
         </is>
       </c>
-      <c r="D147" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E147" s="6" t="inlineStr">
+      <c r="D147" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E147" s="3" t="inlineStr">
         <is>
           <t>R. GANDHI</t>
         </is>
       </c>
-      <c r="F147" s="6" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G147" s="7" t="n">
-        <v>3162</v>
-      </c>
-      <c r="H147" s="6" t="inlineStr">
-        <is>
-          <t>18/22</t>
-        </is>
-      </c>
-      <c r="I147" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J147" s="7" t="n">
-        <v>3865</v>
-      </c>
-      <c r="K147" s="8" t="n">
-        <v>175.6666666666667</v>
+      <c r="F147" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G147" s="4" t="n">
+        <v>5938</v>
+      </c>
+      <c r="H147" s="3" t="inlineStr">
+        <is>
+          <t>20/22</t>
+        </is>
+      </c>
+      <c r="I147" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J147" s="4" t="n">
+        <v>6532</v>
+      </c>
+      <c r="K147" s="5" t="n">
+        <v>296.9</v>
       </c>
     </row>
     <row r="148">
@@ -7770,11 +7770,11 @@
         </is>
       </c>
       <c r="G148" s="4" t="n">
-        <v>14196</v>
+        <v>14030</v>
       </c>
       <c r="H148" s="3" t="inlineStr">
         <is>
-          <t>18/21</t>
+          <t>19/21</t>
         </is>
       </c>
       <c r="I148" s="3" t="inlineStr">
@@ -7783,10 +7783,10 @@
         </is>
       </c>
       <c r="J148" s="4" t="n">
-        <v>16562</v>
+        <v>15507</v>
       </c>
       <c r="K148" s="5" t="n">
-        <v>788.6666666666666</v>
+        <v>738.421052631579</v>
       </c>
     </row>
     <row r="149">
@@ -7819,11 +7819,11 @@
         </is>
       </c>
       <c r="G149" s="7" t="n">
-        <v>3368</v>
+        <v>3064</v>
       </c>
       <c r="H149" s="6" t="inlineStr">
         <is>
-          <t>14/25</t>
+          <t>15/25</t>
         </is>
       </c>
       <c r="I149" s="6" t="inlineStr">
@@ -7832,10 +7832,10 @@
         </is>
       </c>
       <c r="J149" s="7" t="n">
-        <v>6014</v>
+        <v>5107</v>
       </c>
       <c r="K149" s="8" t="n">
-        <v>240.5714285714285</v>
+        <v>204.2666666666667</v>
       </c>
     </row>
     <row r="150">
@@ -7917,11 +7917,11 @@
         </is>
       </c>
       <c r="G151" s="4" t="n">
-        <v>22708</v>
+        <v>24451</v>
       </c>
       <c r="H151" s="3" t="inlineStr">
         <is>
-          <t>16/21</t>
+          <t>17/21</t>
         </is>
       </c>
       <c r="I151" s="3" t="inlineStr">
@@ -7930,10 +7930,10 @@
         </is>
       </c>
       <c r="J151" s="4" t="n">
-        <v>29804</v>
+        <v>30204</v>
       </c>
       <c r="K151" s="5" t="n">
-        <v>1419.25</v>
+        <v>1438.294117647059</v>
       </c>
     </row>
     <row r="152">
@@ -7966,11 +7966,11 @@
         </is>
       </c>
       <c r="G152" s="4" t="n">
-        <v>7752</v>
+        <v>9067</v>
       </c>
       <c r="H152" s="3" t="inlineStr">
         <is>
-          <t>16/21</t>
+          <t>17/21</t>
         </is>
       </c>
       <c r="I152" s="3" t="inlineStr">
@@ -7979,10 +7979,10 @@
         </is>
       </c>
       <c r="J152" s="4" t="n">
-        <v>10174</v>
+        <v>11200</v>
       </c>
       <c r="K152" s="5" t="n">
-        <v>484.5</v>
+        <v>533.3529411764706</v>
       </c>
     </row>
     <row r="153">
@@ -8064,11 +8064,11 @@
         </is>
       </c>
       <c r="G154" s="4" t="n">
-        <v>50943</v>
+        <v>55827</v>
       </c>
       <c r="H154" s="3" t="inlineStr">
         <is>
-          <t>16/23</t>
+          <t>17/23</t>
         </is>
       </c>
       <c r="I154" s="3" t="inlineStr">
@@ -8077,10 +8077,10 @@
         </is>
       </c>
       <c r="J154" s="4" t="n">
-        <v>73231</v>
+        <v>75531</v>
       </c>
       <c r="K154" s="5" t="n">
-        <v>3183.9375</v>
+        <v>3283.941176470588</v>
       </c>
     </row>
     <row r="155">
@@ -8113,11 +8113,11 @@
         </is>
       </c>
       <c r="G155" s="7" t="n">
-        <v>3616</v>
+        <v>4185</v>
       </c>
       <c r="H155" s="6" t="inlineStr">
         <is>
-          <t>17/23</t>
+          <t>18/23</t>
         </is>
       </c>
       <c r="I155" s="6" t="inlineStr">
@@ -8126,10 +8126,10 @@
         </is>
       </c>
       <c r="J155" s="7" t="n">
-        <v>4892</v>
+        <v>5348</v>
       </c>
       <c r="K155" s="8" t="n">
-        <v>212.7058823529412</v>
+        <v>232.5</v>
       </c>
     </row>
     <row r="156">
@@ -8211,11 +8211,11 @@
         </is>
       </c>
       <c r="G157" s="4" t="n">
-        <v>6282</v>
+        <v>7176</v>
       </c>
       <c r="H157" s="3" t="inlineStr">
         <is>
-          <t>21/25</t>
+          <t>22/25</t>
         </is>
       </c>
       <c r="I157" s="3" t="inlineStr">
@@ -8224,10 +8224,10 @@
         </is>
       </c>
       <c r="J157" s="4" t="n">
-        <v>7479</v>
+        <v>8155</v>
       </c>
       <c r="K157" s="5" t="n">
-        <v>299.1428571428572</v>
+        <v>326.1818181818182</v>
       </c>
     </row>
     <row r="158">
@@ -8260,11 +8260,11 @@
         </is>
       </c>
       <c r="G158" s="11" t="n">
-        <v>741</v>
+        <v>777</v>
       </c>
       <c r="H158" s="10" t="inlineStr">
         <is>
-          <t>8/21</t>
+          <t>9/21</t>
         </is>
       </c>
       <c r="I158" s="10" t="inlineStr">
@@ -8273,10 +8273,10 @@
         </is>
       </c>
       <c r="J158" s="11" t="n">
-        <v>1945</v>
+        <v>1813</v>
       </c>
       <c r="K158" s="12" t="n">
-        <v>92.625</v>
+        <v>86.33333333333333</v>
       </c>
     </row>
     <row r="159">
@@ -8309,11 +8309,11 @@
         </is>
       </c>
       <c r="G159" s="11" t="n">
-        <v>1466</v>
+        <v>2655</v>
       </c>
       <c r="H159" s="10" t="inlineStr">
         <is>
-          <t>21/23</t>
+          <t>23/23</t>
         </is>
       </c>
       <c r="I159" s="10" t="inlineStr">
@@ -8322,10 +8322,10 @@
         </is>
       </c>
       <c r="J159" s="11" t="n">
-        <v>1606</v>
+        <v>2655</v>
       </c>
       <c r="K159" s="12" t="n">
-        <v>69.80952380952381</v>
+        <v>115.4347826086957</v>
       </c>
     </row>
     <row r="160">
@@ -8358,11 +8358,11 @@
         </is>
       </c>
       <c r="G160" s="11" t="n">
-        <v>1504</v>
+        <v>727</v>
       </c>
       <c r="H160" s="10" t="inlineStr">
         <is>
-          <t>12/19</t>
+          <t>13/19</t>
         </is>
       </c>
       <c r="I160" s="10" t="inlineStr">
@@ -8371,10 +8371,10 @@
         </is>
       </c>
       <c r="J160" s="11" t="n">
-        <v>2381</v>
+        <v>1063</v>
       </c>
       <c r="K160" s="12" t="n">
-        <v>125.3333333333333</v>
+        <v>55.92307692307692</v>
       </c>
     </row>
     <row r="161">
@@ -8407,11 +8407,11 @@
         </is>
       </c>
       <c r="G161" s="7" t="n">
-        <v>1561</v>
+        <v>1938</v>
       </c>
       <c r="H161" s="6" t="inlineStr">
         <is>
-          <t>11/25</t>
+          <t>12/25</t>
         </is>
       </c>
       <c r="I161" s="6" t="inlineStr">
@@ -8420,10 +8420,10 @@
         </is>
       </c>
       <c r="J161" s="7" t="n">
-        <v>3548</v>
+        <v>4038</v>
       </c>
       <c r="K161" s="8" t="n">
-        <v>141.9090909090909</v>
+        <v>161.5</v>
       </c>
     </row>
     <row r="162">
@@ -8505,11 +8505,11 @@
         </is>
       </c>
       <c r="G163" s="4" t="n">
-        <v>17997</v>
+        <v>19512</v>
       </c>
       <c r="H163" s="3" t="inlineStr">
         <is>
-          <t>17/26</t>
+          <t>18/26</t>
         </is>
       </c>
       <c r="I163" s="3" t="inlineStr">
@@ -8518,10 +8518,10 @@
         </is>
       </c>
       <c r="J163" s="4" t="n">
-        <v>27525</v>
+        <v>28184</v>
       </c>
       <c r="K163" s="5" t="n">
-        <v>1058.64705882353</v>
+        <v>1084</v>
       </c>
     </row>
     <row r="164">
@@ -8603,11 +8603,11 @@
         </is>
       </c>
       <c r="G165" s="7" t="n">
-        <v>12382</v>
+        <v>13027</v>
       </c>
       <c r="H165" s="6" t="inlineStr">
         <is>
-          <t>19/29</t>
+          <t>20/29</t>
         </is>
       </c>
       <c r="I165" s="6" t="inlineStr">
@@ -8616,10 +8616,10 @@
         </is>
       </c>
       <c r="J165" s="7" t="n">
-        <v>18899</v>
+        <v>18889</v>
       </c>
       <c r="K165" s="8" t="n">
-        <v>651.6842105263158</v>
+        <v>651.35</v>
       </c>
     </row>
     <row r="166">
@@ -8652,11 +8652,11 @@
         </is>
       </c>
       <c r="G166" s="7" t="n">
-        <v>2334</v>
+        <v>2979</v>
       </c>
       <c r="H166" s="6" t="inlineStr">
         <is>
-          <t>8/21</t>
+          <t>9/21</t>
         </is>
       </c>
       <c r="I166" s="6" t="inlineStr">
@@ -8665,10 +8665,10 @@
         </is>
       </c>
       <c r="J166" s="7" t="n">
-        <v>6127</v>
+        <v>6951</v>
       </c>
       <c r="K166" s="8" t="n">
-        <v>291.75</v>
+        <v>331</v>
       </c>
     </row>
     <row r="167">
@@ -8750,11 +8750,11 @@
         </is>
       </c>
       <c r="G168" s="4" t="n">
-        <v>19930</v>
+        <v>22777</v>
       </c>
       <c r="H168" s="3" t="inlineStr">
         <is>
-          <t>15/27</t>
+          <t>16/27</t>
         </is>
       </c>
       <c r="I168" s="3" t="inlineStr">
@@ -8763,10 +8763,10 @@
         </is>
       </c>
       <c r="J168" s="4" t="n">
-        <v>35874</v>
+        <v>38436</v>
       </c>
       <c r="K168" s="5" t="n">
-        <v>1328.666666666667</v>
+        <v>1423.5625</v>
       </c>
     </row>
     <row r="169">
@@ -8819,52 +8819,52 @@
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="6" t="inlineStr">
+      <c r="A170" s="9" t="inlineStr">
         <is>
           <t>SRIVILLIPUTHUR</t>
         </is>
       </c>
-      <c r="B170" s="6" t="n">
+      <c r="B170" s="10" t="n">
         <v>203</v>
       </c>
-      <c r="C170" s="6" t="inlineStr">
+      <c r="C170" s="10" t="inlineStr">
+        <is>
+          <t>KARTHIK.A</t>
+        </is>
+      </c>
+      <c r="D170" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E170" s="10" t="inlineStr">
         <is>
           <t>MAHALINGAM.P</t>
         </is>
       </c>
-      <c r="D170" s="6" t="inlineStr">
+      <c r="F170" s="10" t="inlineStr">
         <is>
           <t>Communist Party of India</t>
         </is>
       </c>
-      <c r="E170" s="6" t="inlineStr">
-        <is>
-          <t>KARTHIK.A</t>
-        </is>
-      </c>
-      <c r="F170" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G170" s="7" t="n">
-        <v>2515</v>
-      </c>
-      <c r="H170" s="6" t="inlineStr">
-        <is>
-          <t>14/22</t>
-        </is>
-      </c>
-      <c r="I170" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J170" s="7" t="n">
-        <v>3952</v>
-      </c>
-      <c r="K170" s="8" t="n">
-        <v>179.6428571428571</v>
+      <c r="G170" s="11" t="n">
+        <v>1192</v>
+      </c>
+      <c r="H170" s="10" t="inlineStr">
+        <is>
+          <t>16/22</t>
+        </is>
+      </c>
+      <c r="I170" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J170" s="11" t="n">
+        <v>1639</v>
+      </c>
+      <c r="K170" s="12" t="n">
+        <v>74.5</v>
       </c>
     </row>
     <row r="171">
@@ -8995,11 +8995,11 @@
         </is>
       </c>
       <c r="G173" s="7" t="n">
-        <v>5982</v>
+        <v>5503</v>
       </c>
       <c r="H173" s="6" t="inlineStr">
         <is>
-          <t>16/26</t>
+          <t>17/26</t>
         </is>
       </c>
       <c r="I173" s="6" t="inlineStr">
@@ -9008,10 +9008,10 @@
         </is>
       </c>
       <c r="J173" s="7" t="n">
-        <v>9721</v>
+        <v>8416</v>
       </c>
       <c r="K173" s="8" t="n">
-        <v>373.875</v>
+        <v>323.7058823529412</v>
       </c>
     </row>
     <row r="174">
@@ -9191,11 +9191,11 @@
         </is>
       </c>
       <c r="G177" s="4" t="n">
-        <v>20577</v>
+        <v>22494</v>
       </c>
       <c r="H177" s="3" t="inlineStr">
         <is>
-          <t>23/26</t>
+          <t>24/26</t>
         </is>
       </c>
       <c r="I177" s="3" t="inlineStr">
@@ -9204,10 +9204,10 @@
         </is>
       </c>
       <c r="J177" s="4" t="n">
-        <v>23261</v>
+        <v>24368</v>
       </c>
       <c r="K177" s="5" t="n">
-        <v>894.6521739130435</v>
+        <v>937.25</v>
       </c>
     </row>
     <row r="178">
@@ -9240,11 +9240,11 @@
         </is>
       </c>
       <c r="G178" s="11" t="n">
-        <v>1598</v>
+        <v>1695</v>
       </c>
       <c r="H178" s="10" t="inlineStr">
         <is>
-          <t>12/22</t>
+          <t>13/22</t>
         </is>
       </c>
       <c r="I178" s="10" t="inlineStr">
@@ -9253,10 +9253,10 @@
         </is>
       </c>
       <c r="J178" s="11" t="n">
-        <v>2930</v>
+        <v>2868</v>
       </c>
       <c r="K178" s="12" t="n">
-        <v>133.1666666666667</v>
+        <v>130.3846153846154</v>
       </c>
     </row>
     <row r="179">
@@ -9289,11 +9289,11 @@
         </is>
       </c>
       <c r="G179" s="4" t="n">
-        <v>24910</v>
+        <v>26575</v>
       </c>
       <c r="H179" s="3" t="inlineStr">
         <is>
-          <t>16/26</t>
+          <t>17/26</t>
         </is>
       </c>
       <c r="I179" s="3" t="inlineStr">
@@ -9302,10 +9302,10 @@
         </is>
       </c>
       <c r="J179" s="4" t="n">
-        <v>40479</v>
+        <v>40644</v>
       </c>
       <c r="K179" s="5" t="n">
-        <v>1556.875</v>
+        <v>1563.235294117647</v>
       </c>
     </row>
     <row r="180">
@@ -9387,11 +9387,11 @@
         </is>
       </c>
       <c r="G181" s="4" t="n">
-        <v>12731</v>
+        <v>12922</v>
       </c>
       <c r="H181" s="3" t="inlineStr">
         <is>
-          <t>20/21</t>
+          <t>21/21</t>
         </is>
       </c>
       <c r="I181" s="3" t="inlineStr">
@@ -9400,10 +9400,10 @@
         </is>
       </c>
       <c r="J181" s="4" t="n">
-        <v>13368</v>
+        <v>12922</v>
       </c>
       <c r="K181" s="5" t="n">
-        <v>636.55</v>
+        <v>615.3333333333334</v>
       </c>
     </row>
     <row r="182">
@@ -9436,11 +9436,11 @@
         </is>
       </c>
       <c r="G182" s="7" t="n">
-        <v>8895</v>
+        <v>9047</v>
       </c>
       <c r="H182" s="6" t="inlineStr">
         <is>
-          <t>14/25</t>
+          <t>15/25</t>
         </is>
       </c>
       <c r="I182" s="6" t="inlineStr">
@@ -9449,10 +9449,10 @@
         </is>
       </c>
       <c r="J182" s="7" t="n">
-        <v>15884</v>
+        <v>15078</v>
       </c>
       <c r="K182" s="8" t="n">
-        <v>635.3571428571428</v>
+        <v>603.1333333333333</v>
       </c>
     </row>
     <row r="183">
@@ -9485,11 +9485,11 @@
         </is>
       </c>
       <c r="G183" s="4" t="n">
-        <v>19228</v>
+        <v>19690</v>
       </c>
       <c r="H183" s="3" t="inlineStr">
         <is>
-          <t>19/24</t>
+          <t>20/24</t>
         </is>
       </c>
       <c r="I183" s="3" t="inlineStr">
@@ -9498,10 +9498,10 @@
         </is>
       </c>
       <c r="J183" s="4" t="n">
-        <v>24288</v>
+        <v>23628</v>
       </c>
       <c r="K183" s="5" t="n">
-        <v>1012</v>
+        <v>984.5</v>
       </c>
     </row>
     <row r="184">
@@ -9583,11 +9583,11 @@
         </is>
       </c>
       <c r="G185" s="7" t="n">
-        <v>5346</v>
+        <v>6194</v>
       </c>
       <c r="H185" s="6" t="inlineStr">
         <is>
-          <t>14/23</t>
+          <t>15/23</t>
         </is>
       </c>
       <c r="I185" s="6" t="inlineStr">
@@ -9596,10 +9596,10 @@
         </is>
       </c>
       <c r="J185" s="7" t="n">
-        <v>8783</v>
+        <v>9497</v>
       </c>
       <c r="K185" s="8" t="n">
-        <v>381.8571428571428</v>
+        <v>412.9333333333333</v>
       </c>
     </row>
     <row r="186">
@@ -9681,11 +9681,11 @@
         </is>
       </c>
       <c r="G187" s="4" t="n">
-        <v>44951</v>
+        <v>45921</v>
       </c>
       <c r="H187" s="3" t="inlineStr">
         <is>
-          <t>20/25</t>
+          <t>21/25</t>
         </is>
       </c>
       <c r="I187" s="3" t="inlineStr">
@@ -9694,10 +9694,10 @@
         </is>
       </c>
       <c r="J187" s="4" t="n">
-        <v>56189</v>
+        <v>54668</v>
       </c>
       <c r="K187" s="5" t="n">
-        <v>2247.55</v>
+        <v>2186.714285714286</v>
       </c>
     </row>
     <row r="188">
@@ -9730,11 +9730,11 @@
         </is>
       </c>
       <c r="G188" s="4" t="n">
-        <v>12127</v>
+        <v>13027</v>
       </c>
       <c r="H188" s="3" t="inlineStr">
         <is>
-          <t>17/18</t>
+          <t>18/18</t>
         </is>
       </c>
       <c r="I188" s="3" t="inlineStr">
@@ -9743,10 +9743,10 @@
         </is>
       </c>
       <c r="J188" s="4" t="n">
-        <v>12840</v>
+        <v>13027</v>
       </c>
       <c r="K188" s="5" t="n">
-        <v>713.3529411764706</v>
+        <v>723.7222222222222</v>
       </c>
     </row>
     <row r="189">
@@ -9828,11 +9828,11 @@
         </is>
       </c>
       <c r="G190" s="4" t="n">
-        <v>32566</v>
+        <v>33620</v>
       </c>
       <c r="H190" s="3" t="inlineStr">
         <is>
-          <t>21/26</t>
+          <t>22/26</t>
         </is>
       </c>
       <c r="I190" s="3" t="inlineStr">
@@ -9841,10 +9841,10 @@
         </is>
       </c>
       <c r="J190" s="4" t="n">
-        <v>40320</v>
+        <v>39733</v>
       </c>
       <c r="K190" s="5" t="n">
-        <v>1550.761904761905</v>
+        <v>1528.181818181818</v>
       </c>
     </row>
     <row r="191">
@@ -9926,11 +9926,11 @@
         </is>
       </c>
       <c r="G192" s="4" t="n">
-        <v>7885</v>
+        <v>8558</v>
       </c>
       <c r="H192" s="3" t="inlineStr">
         <is>
-          <t>18/22</t>
+          <t>19/22</t>
         </is>
       </c>
       <c r="I192" s="3" t="inlineStr">
@@ -9939,59 +9939,59 @@
         </is>
       </c>
       <c r="J192" s="4" t="n">
-        <v>9637</v>
+        <v>9909</v>
       </c>
       <c r="K192" s="5" t="n">
-        <v>438.0555555555555</v>
+        <v>450.421052631579</v>
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="6" t="inlineStr">
+      <c r="A193" s="13" t="inlineStr">
         <is>
           <t>TINDIVANAM</t>
         </is>
       </c>
-      <c r="B193" s="6" t="n">
+      <c r="B193" s="14" t="n">
         <v>72</v>
       </c>
-      <c r="C193" s="6" t="inlineStr">
+      <c r="C193" s="14" t="inlineStr">
         <is>
           <t>VANNI ARASU</t>
         </is>
       </c>
-      <c r="D193" s="6" t="inlineStr">
+      <c r="D193" s="14" t="inlineStr">
         <is>
           <t>Viduthalai Chiruthaigal Katchi</t>
         </is>
       </c>
-      <c r="E193" s="6" t="inlineStr">
+      <c r="E193" s="14" t="inlineStr">
         <is>
           <t>ARJUNAN. P</t>
         </is>
       </c>
-      <c r="F193" s="6" t="inlineStr">
+      <c r="F193" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G193" s="7" t="n">
-        <v>1989</v>
-      </c>
-      <c r="H193" s="6" t="inlineStr">
-        <is>
-          <t>14/22</t>
-        </is>
-      </c>
-      <c r="I193" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J193" s="7" t="n">
-        <v>3126</v>
-      </c>
-      <c r="K193" s="8" t="n">
-        <v>142.0714285714286</v>
+      <c r="G193" s="15" t="n">
+        <v>149</v>
+      </c>
+      <c r="H193" s="14" t="inlineStr">
+        <is>
+          <t>15/22</t>
+        </is>
+      </c>
+      <c r="I193" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J193" s="15" t="n">
+        <v>219</v>
+      </c>
+      <c r="K193" s="16" t="n">
+        <v>9.933333333333335</v>
       </c>
     </row>
     <row r="194">
@@ -10073,11 +10073,11 @@
         </is>
       </c>
       <c r="G195" s="4" t="n">
-        <v>14188</v>
+        <v>16892</v>
       </c>
       <c r="H195" s="3" t="inlineStr">
         <is>
-          <t>13/21</t>
+          <t>14/21</t>
         </is>
       </c>
       <c r="I195" s="3" t="inlineStr">
@@ -10086,10 +10086,10 @@
         </is>
       </c>
       <c r="J195" s="4" t="n">
-        <v>22919</v>
+        <v>25338</v>
       </c>
       <c r="K195" s="5" t="n">
-        <v>1091.384615384615</v>
+        <v>1206.571428571429</v>
       </c>
     </row>
     <row r="196">
@@ -10122,11 +10122,11 @@
         </is>
       </c>
       <c r="G196" s="4" t="n">
-        <v>15707</v>
+        <v>17733</v>
       </c>
       <c r="H196" s="3" t="inlineStr">
         <is>
-          <t>12/22</t>
+          <t>13/22</t>
         </is>
       </c>
       <c r="I196" s="3" t="inlineStr">
@@ -10135,10 +10135,10 @@
         </is>
       </c>
       <c r="J196" s="4" t="n">
-        <v>28796</v>
+        <v>30010</v>
       </c>
       <c r="K196" s="5" t="n">
-        <v>1308.916666666667</v>
+        <v>1364.076923076923</v>
       </c>
     </row>
     <row r="197">
@@ -10220,11 +10220,11 @@
         </is>
       </c>
       <c r="G198" s="7" t="n">
-        <v>5847</v>
+        <v>6865</v>
       </c>
       <c r="H198" s="6" t="inlineStr">
         <is>
-          <t>12/21</t>
+          <t>13/21</t>
         </is>
       </c>
       <c r="I198" s="6" t="inlineStr">
@@ -10233,10 +10233,10 @@
         </is>
       </c>
       <c r="J198" s="7" t="n">
-        <v>10232</v>
+        <v>11090</v>
       </c>
       <c r="K198" s="8" t="n">
-        <v>487.25</v>
+        <v>528.0769230769231</v>
       </c>
     </row>
     <row r="199">
@@ -10416,11 +10416,11 @@
         </is>
       </c>
       <c r="G202" s="7" t="n">
-        <v>3086</v>
+        <v>3885</v>
       </c>
       <c r="H202" s="6" t="inlineStr">
         <is>
-          <t>15/27</t>
+          <t>16/27</t>
         </is>
       </c>
       <c r="I202" s="6" t="inlineStr">
@@ -10429,10 +10429,10 @@
         </is>
       </c>
       <c r="J202" s="7" t="n">
-        <v>5555</v>
+        <v>6556</v>
       </c>
       <c r="K202" s="8" t="n">
-        <v>205.7333333333333</v>
+        <v>242.8125</v>
       </c>
     </row>
     <row r="203">
@@ -10465,11 +10465,11 @@
         </is>
       </c>
       <c r="G203" s="4" t="n">
-        <v>44545</v>
+        <v>46377</v>
       </c>
       <c r="H203" s="3" t="inlineStr">
         <is>
-          <t>19/32</t>
+          <t>20/32</t>
         </is>
       </c>
       <c r="I203" s="3" t="inlineStr">
@@ -10478,10 +10478,10 @@
         </is>
       </c>
       <c r="J203" s="4" t="n">
-        <v>75023</v>
+        <v>74203</v>
       </c>
       <c r="K203" s="5" t="n">
-        <v>2344.473684210526</v>
+        <v>2318.85</v>
       </c>
     </row>
     <row r="204">
@@ -10514,11 +10514,11 @@
         </is>
       </c>
       <c r="G204" s="7" t="n">
-        <v>10976</v>
+        <v>12574</v>
       </c>
       <c r="H204" s="6" t="inlineStr">
         <is>
-          <t>13/21</t>
+          <t>14/21</t>
         </is>
       </c>
       <c r="I204" s="6" t="inlineStr">
@@ -10527,10 +10527,10 @@
         </is>
       </c>
       <c r="J204" s="7" t="n">
-        <v>17730</v>
+        <v>18861</v>
       </c>
       <c r="K204" s="8" t="n">
-        <v>844.3076923076923</v>
+        <v>898.1428571428571</v>
       </c>
     </row>
     <row r="205">
@@ -10563,11 +10563,11 @@
         </is>
       </c>
       <c r="G205" s="7" t="n">
-        <v>8642</v>
+        <v>9688</v>
       </c>
       <c r="H205" s="6" t="inlineStr">
         <is>
-          <t>14/25</t>
+          <t>15/25</t>
         </is>
       </c>
       <c r="I205" s="6" t="inlineStr">
@@ -10576,10 +10576,10 @@
         </is>
       </c>
       <c r="J205" s="7" t="n">
-        <v>15432</v>
+        <v>16147</v>
       </c>
       <c r="K205" s="8" t="n">
-        <v>617.2857142857142</v>
+        <v>645.8666666666667</v>
       </c>
     </row>
     <row r="206">
@@ -10612,11 +10612,11 @@
         </is>
       </c>
       <c r="G206" s="7" t="n">
-        <v>2941</v>
+        <v>3111</v>
       </c>
       <c r="H206" s="6" t="inlineStr">
         <is>
-          <t>23/27</t>
+          <t>24/27</t>
         </is>
       </c>
       <c r="I206" s="6" t="inlineStr">
@@ -10625,10 +10625,10 @@
         </is>
       </c>
       <c r="J206" s="7" t="n">
-        <v>3452</v>
+        <v>3500</v>
       </c>
       <c r="K206" s="8" t="n">
-        <v>127.8695652173913</v>
+        <v>129.625</v>
       </c>
     </row>
     <row r="207">
@@ -10661,11 +10661,11 @@
         </is>
       </c>
       <c r="G207" s="11" t="n">
-        <v>1074</v>
+        <v>1417</v>
       </c>
       <c r="H207" s="10" t="inlineStr">
         <is>
-          <t>12/23</t>
+          <t>13/23</t>
         </is>
       </c>
       <c r="I207" s="10" t="inlineStr">
@@ -10674,10 +10674,10 @@
         </is>
       </c>
       <c r="J207" s="11" t="n">
-        <v>2058</v>
+        <v>2507</v>
       </c>
       <c r="K207" s="12" t="n">
-        <v>89.5</v>
+        <v>109</v>
       </c>
     </row>
     <row r="208">
@@ -10857,11 +10857,11 @@
         </is>
       </c>
       <c r="G211" s="11" t="n">
-        <v>529</v>
+        <v>1402</v>
       </c>
       <c r="H211" s="10" t="inlineStr">
         <is>
-          <t>18/27</t>
+          <t>19/27</t>
         </is>
       </c>
       <c r="I211" s="10" t="inlineStr">
@@ -10870,59 +10870,59 @@
         </is>
       </c>
       <c r="J211" s="11" t="n">
-        <v>794</v>
+        <v>1992</v>
       </c>
       <c r="K211" s="12" t="n">
-        <v>29.38888888888889</v>
+        <v>73.78947368421052</v>
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="9" t="inlineStr">
+      <c r="A212" s="6" t="inlineStr">
         <is>
           <t>USILAMPATTI</t>
         </is>
       </c>
-      <c r="B212" s="10" t="n">
+      <c r="B212" s="6" t="n">
         <v>197</v>
       </c>
-      <c r="C212" s="10" t="inlineStr">
+      <c r="C212" s="6" t="inlineStr">
         <is>
           <t>VIJAY. M</t>
         </is>
       </c>
-      <c r="D212" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E212" s="10" t="inlineStr">
+      <c r="D212" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E212" s="6" t="inlineStr">
         <is>
           <t>MAHENDRAN. I</t>
         </is>
       </c>
-      <c r="F212" s="10" t="inlineStr">
+      <c r="F212" s="6" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G212" s="11" t="n">
-        <v>1605</v>
-      </c>
-      <c r="H212" s="10" t="inlineStr">
-        <is>
-          <t>14/25</t>
-        </is>
-      </c>
-      <c r="I212" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J212" s="11" t="n">
-        <v>2866</v>
-      </c>
-      <c r="K212" s="12" t="n">
-        <v>114.6428571428571</v>
+      <c r="G212" s="7" t="n">
+        <v>1973</v>
+      </c>
+      <c r="H212" s="6" t="inlineStr">
+        <is>
+          <t>15/25</t>
+        </is>
+      </c>
+      <c r="I212" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J212" s="7" t="n">
+        <v>3288</v>
+      </c>
+      <c r="K212" s="8" t="n">
+        <v>131.5333333333333</v>
       </c>
     </row>
     <row r="213">
@@ -11004,11 +11004,11 @@
         </is>
       </c>
       <c r="G214" s="4" t="n">
-        <v>13999</v>
+        <v>14215</v>
       </c>
       <c r="H214" s="3" t="inlineStr">
         <is>
-          <t>19/23</t>
+          <t>20/23</t>
         </is>
       </c>
       <c r="I214" s="3" t="inlineStr">
@@ -11017,10 +11017,10 @@
         </is>
       </c>
       <c r="J214" s="4" t="n">
-        <v>16946</v>
+        <v>16347</v>
       </c>
       <c r="K214" s="5" t="n">
-        <v>736.7894736842105</v>
+        <v>710.75</v>
       </c>
     </row>
     <row r="215">
@@ -11200,11 +11200,11 @@
         </is>
       </c>
       <c r="G218" s="7" t="n">
-        <v>4496</v>
+        <v>3922</v>
       </c>
       <c r="H218" s="6" t="inlineStr">
         <is>
-          <t>17/22</t>
+          <t>18/22</t>
         </is>
       </c>
       <c r="I218" s="6" t="inlineStr">
@@ -11213,10 +11213,10 @@
         </is>
       </c>
       <c r="J218" s="7" t="n">
-        <v>5818</v>
+        <v>4794</v>
       </c>
       <c r="K218" s="8" t="n">
-        <v>264.4705882352941</v>
+        <v>217.8888888888889</v>
       </c>
     </row>
     <row r="219">
@@ -11249,11 +11249,11 @@
         </is>
       </c>
       <c r="G219" s="4" t="n">
-        <v>8369</v>
+        <v>7095</v>
       </c>
       <c r="H219" s="3" t="inlineStr">
         <is>
-          <t>19/23</t>
+          <t>20/23</t>
         </is>
       </c>
       <c r="I219" s="3" t="inlineStr">
@@ -11262,10 +11262,10 @@
         </is>
       </c>
       <c r="J219" s="4" t="n">
-        <v>10131</v>
+        <v>8159</v>
       </c>
       <c r="K219" s="5" t="n">
-        <v>440.4736842105263</v>
+        <v>354.75</v>
       </c>
     </row>
     <row r="220">
@@ -11347,11 +11347,11 @@
         </is>
       </c>
       <c r="G221" s="4" t="n">
-        <v>9353</v>
+        <v>9993</v>
       </c>
       <c r="H221" s="3" t="inlineStr">
         <is>
-          <t>19/24</t>
+          <t>20/24</t>
         </is>
       </c>
       <c r="I221" s="3" t="inlineStr">
@@ -11360,10 +11360,10 @@
         </is>
       </c>
       <c r="J221" s="4" t="n">
-        <v>11814</v>
+        <v>11992</v>
       </c>
       <c r="K221" s="5" t="n">
-        <v>492.2631578947368</v>
+        <v>499.65</v>
       </c>
     </row>
     <row r="222">
@@ -11445,11 +11445,11 @@
         </is>
       </c>
       <c r="G223" s="4" t="n">
-        <v>29825</v>
+        <v>30683</v>
       </c>
       <c r="H223" s="3" t="inlineStr">
         <is>
-          <t>20/23</t>
+          <t>21/23</t>
         </is>
       </c>
       <c r="I223" s="3" t="inlineStr">
@@ -11458,59 +11458,59 @@
         </is>
       </c>
       <c r="J223" s="4" t="n">
-        <v>34299</v>
+        <v>33605</v>
       </c>
       <c r="K223" s="5" t="n">
-        <v>1491.25</v>
+        <v>1461.095238095238</v>
       </c>
     </row>
     <row r="224">
-      <c r="A224" s="2" t="inlineStr">
+      <c r="A224" s="6" t="inlineStr">
         <is>
           <t>VELLORE</t>
         </is>
       </c>
-      <c r="B224" s="3" t="n">
+      <c r="B224" s="6" t="n">
         <v>43</v>
       </c>
-      <c r="C224" s="3" t="inlineStr">
+      <c r="C224" s="6" t="inlineStr">
         <is>
           <t>M.M.VINOTH KANNAN</t>
         </is>
       </c>
-      <c r="D224" s="3" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E224" s="3" t="inlineStr">
+      <c r="D224" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E224" s="6" t="inlineStr">
         <is>
           <t>P.KARTHIKEYAN</t>
         </is>
       </c>
-      <c r="F224" s="3" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G224" s="4" t="n">
-        <v>5153</v>
-      </c>
-      <c r="H224" s="3" t="inlineStr">
+      <c r="F224" s="6" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G224" s="7" t="n">
+        <v>4954</v>
+      </c>
+      <c r="H224" s="6" t="inlineStr">
         <is>
           <t>18/20</t>
         </is>
       </c>
-      <c r="I224" s="3" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J224" s="4" t="n">
-        <v>5726</v>
-      </c>
-      <c r="K224" s="5" t="n">
-        <v>286.2777777777778</v>
+      <c r="I224" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J224" s="7" t="n">
+        <v>5504</v>
+      </c>
+      <c r="K224" s="8" t="n">
+        <v>275.2222222222222</v>
       </c>
     </row>
     <row r="225">
@@ -11543,11 +11543,11 @@
         </is>
       </c>
       <c r="G225" s="11" t="n">
-        <v>787</v>
+        <v>696</v>
       </c>
       <c r="H225" s="10" t="inlineStr">
         <is>
-          <t>22/25</t>
+          <t>23/25</t>
         </is>
       </c>
       <c r="I225" s="10" t="inlineStr">
@@ -11556,59 +11556,59 @@
         </is>
       </c>
       <c r="J225" s="11" t="n">
-        <v>894</v>
+        <v>757</v>
       </c>
       <c r="K225" s="12" t="n">
-        <v>35.77272727272727</v>
+        <v>30.26086956521739</v>
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="9" t="inlineStr">
+      <c r="A226" s="6" t="inlineStr">
         <is>
           <t>VIKRAVANDI</t>
         </is>
       </c>
-      <c r="B226" s="10" t="n">
+      <c r="B226" s="6" t="n">
         <v>75</v>
       </c>
-      <c r="C226" s="10" t="inlineStr">
+      <c r="C226" s="6" t="inlineStr">
         <is>
           <t>SIVAKUMAR C</t>
         </is>
       </c>
-      <c r="D226" s="10" t="inlineStr">
+      <c r="D226" s="6" t="inlineStr">
         <is>
           <t>Pattali Makkal Katchi</t>
         </is>
       </c>
-      <c r="E226" s="10" t="inlineStr">
+      <c r="E226" s="6" t="inlineStr">
         <is>
           <t>VIJAI VADIVEL A</t>
         </is>
       </c>
-      <c r="F226" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G226" s="11" t="n">
-        <v>1075</v>
-      </c>
-      <c r="H226" s="10" t="inlineStr">
-        <is>
-          <t>11/23</t>
-        </is>
-      </c>
-      <c r="I226" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J226" s="11" t="n">
-        <v>2248</v>
-      </c>
-      <c r="K226" s="12" t="n">
-        <v>97.72727272727273</v>
+      <c r="F226" s="6" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G226" s="7" t="n">
+        <v>1726</v>
+      </c>
+      <c r="H226" s="6" t="inlineStr">
+        <is>
+          <t>12/23</t>
+        </is>
+      </c>
+      <c r="I226" s="6" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J226" s="7" t="n">
+        <v>3308</v>
+      </c>
+      <c r="K226" s="8" t="n">
+        <v>143.8333333333333</v>
       </c>
     </row>
     <row r="227">
@@ -11690,11 +11690,11 @@
         </is>
       </c>
       <c r="G228" s="4" t="n">
-        <v>17410</v>
+        <v>17852</v>
       </c>
       <c r="H228" s="3" t="inlineStr">
         <is>
-          <t>17/22</t>
+          <t>18/22</t>
         </is>
       </c>
       <c r="I228" s="3" t="inlineStr">
@@ -11703,10 +11703,10 @@
         </is>
       </c>
       <c r="J228" s="4" t="n">
-        <v>22531</v>
+        <v>21819</v>
       </c>
       <c r="K228" s="5" t="n">
-        <v>1024.117647058823</v>
+        <v>991.7777777777778</v>
       </c>
     </row>
     <row r="229">
@@ -11886,11 +11886,11 @@
         </is>
       </c>
       <c r="G232" s="7" t="n">
-        <v>5677</v>
+        <v>7675</v>
       </c>
       <c r="H232" s="6" t="inlineStr">
         <is>
-          <t>13/21</t>
+          <t>14/21</t>
         </is>
       </c>
       <c r="I232" s="6" t="inlineStr">
@@ -11899,10 +11899,10 @@
         </is>
       </c>
       <c r="J232" s="7" t="n">
-        <v>9171</v>
+        <v>11512</v>
       </c>
       <c r="K232" s="8" t="n">
-        <v>436.6923076923077</v>
+        <v>548.2142857142857</v>
       </c>
     </row>
     <row r="233">
@@ -11955,52 +11955,52 @@
       </c>
     </row>
     <row r="234">
-      <c r="A234" s="6" t="inlineStr">
+      <c r="A234" s="9" t="inlineStr">
         <is>
           <t>VRIDDHACHALAM</t>
         </is>
       </c>
-      <c r="B234" s="6" t="n">
+      <c r="B234" s="10" t="n">
         <v>152</v>
       </c>
-      <c r="C234" s="6" t="inlineStr">
+      <c r="C234" s="10" t="inlineStr">
         <is>
           <t>PREMALLATHA VIJAYAKANT</t>
         </is>
       </c>
-      <c r="D234" s="6" t="inlineStr">
+      <c r="D234" s="10" t="inlineStr">
         <is>
           <t>Desiya Murpokku Dravida Kazhagam</t>
         </is>
       </c>
-      <c r="E234" s="6" t="inlineStr">
+      <c r="E234" s="10" t="inlineStr">
         <is>
           <t>VIJAY.S</t>
         </is>
       </c>
-      <c r="F234" s="6" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G234" s="7" t="n">
-        <v>2611</v>
-      </c>
-      <c r="H234" s="6" t="inlineStr">
-        <is>
-          <t>18/23</t>
-        </is>
-      </c>
-      <c r="I234" s="6" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J234" s="7" t="n">
-        <v>3336</v>
-      </c>
-      <c r="K234" s="8" t="n">
-        <v>145.0555555555555</v>
+      <c r="F234" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G234" s="11" t="n">
+        <v>2283</v>
+      </c>
+      <c r="H234" s="10" t="inlineStr">
+        <is>
+          <t>19/23</t>
+        </is>
+      </c>
+      <c r="I234" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J234" s="11" t="n">
+        <v>2764</v>
+      </c>
+      <c r="K234" s="12" t="n">
+        <v>120.1578947368421</v>
       </c>
     </row>
     <row r="235">

</xml_diff>

<commit_message>
Election snapshot: 92.2% counted — TVK 108, DMK 61, AIADMK 45, 56 declared
THIRUMAYAM down to 3-vote DMK lead (19/22 rounds); 7 knife-edge seats remain.

https://claude.ai/code/session_01MizbUy44JG5sXyvaf3Wekb
</commit_message>
<xml_diff>
--- a/tn_election_results_may2026.xlsx
+++ b/tn_election_results_may2026.xlsx
@@ -616,11 +616,11 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>23127</v>
+        <v>23883</v>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>20/31</t>
+          <t>21/31</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -629,10 +629,10 @@
         </is>
       </c>
       <c r="J2" s="4" t="n">
-        <v>35847</v>
+        <v>35256</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>1156.35</v>
+        <v>1137.285714285714</v>
       </c>
     </row>
     <row r="3">
@@ -665,11 +665,11 @@
         </is>
       </c>
       <c r="G3" s="4" t="n">
-        <v>12580</v>
+        <v>12977</v>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>18/21</t>
+          <t>21/21</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -678,10 +678,10 @@
         </is>
       </c>
       <c r="J3" s="4" t="n">
-        <v>14677</v>
+        <v>12977</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>698.8888888888889</v>
+        <v>617.952380952381</v>
       </c>
     </row>
     <row r="4">
@@ -714,11 +714,11 @@
         </is>
       </c>
       <c r="G4" s="4" t="n">
-        <v>7471</v>
+        <v>7798</v>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>23/24</t>
+          <t>25/25</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -727,10 +727,10 @@
         </is>
       </c>
       <c r="J4" s="4" t="n">
-        <v>7796</v>
+        <v>7798</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>324.8260869565217</v>
+        <v>311.92</v>
       </c>
     </row>
     <row r="5">
@@ -812,11 +812,11 @@
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>53856</v>
+        <v>56253</v>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>24/27</t>
+          <t>25/27</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -825,10 +825,10 @@
         </is>
       </c>
       <c r="J6" s="4" t="n">
-        <v>60588</v>
+        <v>60753</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>2244</v>
+        <v>2250.12</v>
       </c>
     </row>
     <row r="7">
@@ -861,11 +861,11 @@
         </is>
       </c>
       <c r="G7" s="4" t="n">
-        <v>12411</v>
+        <v>10774</v>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>17/22</t>
+          <t>18/22</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -874,10 +874,10 @@
         </is>
       </c>
       <c r="J7" s="4" t="n">
-        <v>16061</v>
+        <v>13168</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>730.0588235294117</v>
+        <v>598.5555555555555</v>
       </c>
     </row>
     <row r="8">
@@ -910,11 +910,11 @@
         </is>
       </c>
       <c r="G8" s="4" t="n">
-        <v>5213</v>
+        <v>7081</v>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>20/23</t>
+          <t>23/23</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
@@ -923,10 +923,10 @@
         </is>
       </c>
       <c r="J8" s="4" t="n">
-        <v>5995</v>
+        <v>7081</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>260.65</v>
+        <v>307.8695652173913</v>
       </c>
     </row>
     <row r="9">
@@ -959,11 +959,11 @@
         </is>
       </c>
       <c r="G9" s="4" t="n">
-        <v>8944</v>
+        <v>9554</v>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>23/25</t>
+          <t>25/25</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -972,10 +972,10 @@
         </is>
       </c>
       <c r="J9" s="4" t="n">
-        <v>9722</v>
+        <v>9554</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>388.8695652173913</v>
+        <v>382.16</v>
       </c>
     </row>
     <row r="10">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J11" s="8" t="n">
@@ -1155,7 +1155,7 @@
         </is>
       </c>
       <c r="G13" s="4" t="n">
-        <v>5094</v>
+        <v>5057</v>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
@@ -1168,10 +1168,10 @@
         </is>
       </c>
       <c r="J13" s="4" t="n">
-        <v>5557</v>
+        <v>5517</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>231.5454545454545</v>
+        <v>229.8636363636364</v>
       </c>
     </row>
     <row r="14">
@@ -1253,11 +1253,11 @@
         </is>
       </c>
       <c r="G15" s="4" t="n">
-        <v>19353</v>
+        <v>19378</v>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>19/20</t>
+          <t>20/20</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
@@ -1266,10 +1266,10 @@
         </is>
       </c>
       <c r="J15" s="4" t="n">
-        <v>20372</v>
+        <v>19378</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>1018.578947368421</v>
+        <v>968.9</v>
       </c>
     </row>
     <row r="16">
@@ -1302,11 +1302,11 @@
         </is>
       </c>
       <c r="G16" s="4" t="n">
-        <v>28884</v>
+        <v>33962</v>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>17/23</t>
+          <t>19/23</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
@@ -1315,10 +1315,10 @@
         </is>
       </c>
       <c r="J16" s="4" t="n">
-        <v>39078</v>
+        <v>41112</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>1699.058823529412</v>
+        <v>1787.473684210526</v>
       </c>
     </row>
     <row r="17">
@@ -1449,11 +1449,11 @@
         </is>
       </c>
       <c r="G19" s="4" t="n">
-        <v>22613</v>
+        <v>22240</v>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>23/25</t>
+          <t>25/26</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -1462,10 +1462,10 @@
         </is>
       </c>
       <c r="J19" s="4" t="n">
-        <v>24579</v>
+        <v>23130</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>983.1739130434783</v>
+        <v>889.6</v>
       </c>
     </row>
     <row r="20">
@@ -1547,11 +1547,11 @@
         </is>
       </c>
       <c r="G21" s="4" t="n">
-        <v>55915</v>
+        <v>60189</v>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>20/26</t>
+          <t>21/26</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -1560,10 +1560,10 @@
         </is>
       </c>
       <c r="J21" s="4" t="n">
-        <v>72690</v>
+        <v>74520</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>2795.75</v>
+        <v>2866.142857142857</v>
       </c>
     </row>
     <row r="22">
@@ -1596,11 +1596,11 @@
         </is>
       </c>
       <c r="G22" s="4" t="n">
-        <v>12527</v>
+        <v>15373</v>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>25/27</t>
+          <t>28/28</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
@@ -1609,59 +1609,59 @@
         </is>
       </c>
       <c r="J22" s="4" t="n">
-        <v>13529</v>
+        <v>15373</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>501.08</v>
+        <v>549.0357142857143</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+      <c r="A23" s="10" t="inlineStr">
         <is>
           <t>BARGUR</t>
         </is>
       </c>
-      <c r="B23" s="7" t="n">
+      <c r="B23" s="10" t="n">
         <v>52</v>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C23" s="10" t="inlineStr">
         <is>
           <t>E.C. GOVINDARASAN</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D23" s="10" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr">
+      <c r="E23" s="10" t="inlineStr">
         <is>
           <t>E. MURALIDHARAN</t>
         </is>
       </c>
-      <c r="F23" s="7" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G23" s="8" t="n">
-        <v>882</v>
-      </c>
-      <c r="H23" s="7" t="inlineStr">
-        <is>
-          <t>19/24</t>
-        </is>
-      </c>
-      <c r="I23" s="7" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J23" s="8" t="n">
-        <v>1114</v>
-      </c>
-      <c r="K23" s="9" t="n">
-        <v>46.42105263157895</v>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="n">
+        <v>3076</v>
+      </c>
+      <c r="H23" s="10" t="inlineStr">
+        <is>
+          <t>21/24</t>
+        </is>
+      </c>
+      <c r="I23" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J23" s="11" t="n">
+        <v>3515</v>
+      </c>
+      <c r="K23" s="12" t="n">
+        <v>146.4761904761905</v>
       </c>
     </row>
     <row r="24">
@@ -1694,11 +1694,11 @@
         </is>
       </c>
       <c r="G24" s="4" t="n">
-        <v>7281</v>
+        <v>7396</v>
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>21/22</t>
+          <t>22/22</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
@@ -1707,10 +1707,10 @@
         </is>
       </c>
       <c r="J24" s="4" t="n">
-        <v>7628</v>
+        <v>7396</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>346.7142857142857</v>
+        <v>336.1818181818182</v>
       </c>
     </row>
     <row r="25">
@@ -1841,7 +1841,7 @@
         </is>
       </c>
       <c r="G27" s="4" t="n">
-        <v>5335</v>
+        <v>5483</v>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
@@ -1854,10 +1854,10 @@
         </is>
       </c>
       <c r="J27" s="4" t="n">
-        <v>5799</v>
+        <v>5960</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>231.9565217391304</v>
+        <v>238.3913043478261</v>
       </c>
     </row>
     <row r="28">
@@ -1890,11 +1890,11 @@
         </is>
       </c>
       <c r="G28" s="4" t="n">
-        <v>23910</v>
+        <v>25958</v>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>21/36</t>
+          <t>23/36</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
@@ -1903,10 +1903,10 @@
         </is>
       </c>
       <c r="J28" s="4" t="n">
-        <v>40989</v>
+        <v>40630</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>1138.571428571429</v>
+        <v>1128.608695652174</v>
       </c>
     </row>
     <row r="29">
@@ -2135,11 +2135,11 @@
         </is>
       </c>
       <c r="G33" s="4" t="n">
-        <v>6722</v>
+        <v>7503</v>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>18/22</t>
+          <t>19/22</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -2148,10 +2148,10 @@
         </is>
       </c>
       <c r="J33" s="4" t="n">
-        <v>8216</v>
+        <v>8688</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>373.4444444444445</v>
+        <v>394.8947368421053</v>
       </c>
     </row>
     <row r="34">
@@ -2184,11 +2184,11 @@
         </is>
       </c>
       <c r="G34" s="4" t="n">
-        <v>15247</v>
+        <v>17084</v>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>18/25</t>
+          <t>20/25</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
@@ -2197,59 +2197,59 @@
         </is>
       </c>
       <c r="J34" s="4" t="n">
-        <v>21176</v>
+        <v>21355</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>847.0555555555555</v>
+        <v>854.2</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="10" t="inlineStr">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t>COIMBATORE (SOUTH)</t>
         </is>
       </c>
-      <c r="B35" s="10" t="n">
+      <c r="B35" s="7" t="n">
         <v>120</v>
       </c>
-      <c r="C35" s="10" t="inlineStr">
+      <c r="C35" s="7" t="inlineStr">
         <is>
           <t>V SENTHILBALAJI</t>
         </is>
       </c>
-      <c r="D35" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E35" s="10" t="inlineStr">
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
         <is>
           <t>V. SENTHILKUMAR</t>
         </is>
       </c>
-      <c r="F35" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G35" s="11" t="n">
-        <v>3365</v>
-      </c>
-      <c r="H35" s="10" t="inlineStr">
-        <is>
-          <t>19/20</t>
-        </is>
-      </c>
-      <c r="I35" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J35" s="11" t="n">
-        <v>3542</v>
-      </c>
-      <c r="K35" s="12" t="n">
-        <v>177.1052631578947</v>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="n">
+        <v>2271</v>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>20/20</t>
+        </is>
+      </c>
+      <c r="I35" s="7" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J35" s="8" t="n">
+        <v>2271</v>
+      </c>
+      <c r="K35" s="9" t="n">
+        <v>113.55</v>
       </c>
     </row>
     <row r="36">
@@ -2380,7 +2380,7 @@
         </is>
       </c>
       <c r="G38" s="4" t="n">
-        <v>14659</v>
+        <v>14394</v>
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
@@ -2393,59 +2393,59 @@
         </is>
       </c>
       <c r="J38" s="4" t="n">
-        <v>16384</v>
+        <v>16087</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>862.2941176470588</v>
+        <v>846.7058823529412</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="6" t="inlineStr">
+      <c r="A39" s="10" t="inlineStr">
         <is>
           <t>CUMBUM</t>
         </is>
       </c>
-      <c r="B39" s="7" t="n">
+      <c r="B39" s="10" t="n">
         <v>201</v>
       </c>
-      <c r="C39" s="7" t="inlineStr">
+      <c r="C39" s="10" t="inlineStr">
         <is>
           <t>ERAMAKRISHNAN N</t>
         </is>
       </c>
-      <c r="D39" s="7" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E39" s="7" t="inlineStr">
+      <c r="D39" s="10" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E39" s="10" t="inlineStr">
         <is>
           <t>JEGANATHMISHRA PLA</t>
         </is>
       </c>
-      <c r="F39" s="7" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G39" s="8" t="n">
-        <v>1873</v>
-      </c>
-      <c r="H39" s="7" t="inlineStr">
-        <is>
-          <t>19/25</t>
-        </is>
-      </c>
-      <c r="I39" s="7" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J39" s="8" t="n">
-        <v>2464</v>
-      </c>
-      <c r="K39" s="9" t="n">
-        <v>98.57894736842105</v>
+      <c r="F39" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G39" s="11" t="n">
+        <v>3354</v>
+      </c>
+      <c r="H39" s="10" t="inlineStr">
+        <is>
+          <t>20/25</t>
+        </is>
+      </c>
+      <c r="I39" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J39" s="11" t="n">
+        <v>4192</v>
+      </c>
+      <c r="K39" s="12" t="n">
+        <v>167.7</v>
       </c>
     </row>
     <row r="40">
@@ -2625,11 +2625,11 @@
         </is>
       </c>
       <c r="G43" s="4" t="n">
-        <v>39106</v>
+        <v>42664</v>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>14/18</t>
+          <t>15/18</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
@@ -2638,10 +2638,10 @@
         </is>
       </c>
       <c r="J43" s="4" t="n">
-        <v>50279</v>
+        <v>51197</v>
       </c>
       <c r="K43" s="5" t="n">
-        <v>2793.285714285714</v>
+        <v>2844.266666666667</v>
       </c>
     </row>
     <row r="44">
@@ -2821,11 +2821,11 @@
         </is>
       </c>
       <c r="G47" s="4" t="n">
-        <v>22615</v>
+        <v>22250</v>
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>22/24</t>
+          <t>24/24</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
@@ -2834,10 +2834,10 @@
         </is>
       </c>
       <c r="J47" s="4" t="n">
-        <v>24671</v>
+        <v>22250</v>
       </c>
       <c r="K47" s="5" t="n">
-        <v>1027.954545454545</v>
+        <v>927.0833333333334</v>
       </c>
     </row>
     <row r="48">
@@ -3115,11 +3115,11 @@
         </is>
       </c>
       <c r="G53" s="4" t="n">
-        <v>8345</v>
+        <v>10097</v>
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>22/23</t>
+          <t>23/23</t>
         </is>
       </c>
       <c r="I53" s="3" t="inlineStr">
@@ -3128,10 +3128,10 @@
         </is>
       </c>
       <c r="J53" s="4" t="n">
-        <v>8724</v>
+        <v>10097</v>
       </c>
       <c r="K53" s="5" t="n">
-        <v>379.3181818181818</v>
+        <v>439</v>
       </c>
     </row>
     <row r="54">
@@ -3168,7 +3168,7 @@
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>23/25</t>
+          <t>23/26</t>
         </is>
       </c>
       <c r="I54" s="3" t="inlineStr">
@@ -3177,7 +3177,7 @@
         </is>
       </c>
       <c r="J54" s="4" t="n">
-        <v>29886</v>
+        <v>31081</v>
       </c>
       <c r="K54" s="5" t="n">
         <v>1195.434782608696</v>
@@ -3271,7 +3271,7 @@
       </c>
       <c r="I56" s="10" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J56" s="11" t="n">
@@ -3311,11 +3311,11 @@
         </is>
       </c>
       <c r="G57" s="4" t="n">
-        <v>21286</v>
+        <v>20706</v>
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>26/32</t>
+          <t>28/32</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr">
@@ -3324,10 +3324,10 @@
         </is>
       </c>
       <c r="J57" s="4" t="n">
-        <v>26198</v>
+        <v>23664</v>
       </c>
       <c r="K57" s="5" t="n">
-        <v>818.6923076923077</v>
+        <v>739.5</v>
       </c>
     </row>
     <row r="58">
@@ -3360,11 +3360,11 @@
         </is>
       </c>
       <c r="G58" s="4" t="n">
-        <v>18347</v>
+        <v>18490</v>
       </c>
       <c r="H58" s="3" t="inlineStr">
         <is>
-          <t>24/25</t>
+          <t>25/25</t>
         </is>
       </c>
       <c r="I58" s="3" t="inlineStr">
@@ -3373,10 +3373,10 @@
         </is>
       </c>
       <c r="J58" s="4" t="n">
-        <v>19111</v>
+        <v>18490</v>
       </c>
       <c r="K58" s="5" t="n">
-        <v>764.4583333333334</v>
+        <v>739.6</v>
       </c>
     </row>
     <row r="59">
@@ -3409,11 +3409,11 @@
         </is>
       </c>
       <c r="G59" s="4" t="n">
-        <v>16202</v>
+        <v>16083</v>
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>21/22</t>
+          <t>22/22</t>
         </is>
       </c>
       <c r="I59" s="3" t="inlineStr">
@@ -3422,10 +3422,10 @@
         </is>
       </c>
       <c r="J59" s="4" t="n">
-        <v>16974</v>
+        <v>16083</v>
       </c>
       <c r="K59" s="5" t="n">
-        <v>771.5238095238095</v>
+        <v>731.0454545454545</v>
       </c>
     </row>
     <row r="60">
@@ -3458,11 +3458,11 @@
         </is>
       </c>
       <c r="G60" s="4" t="n">
-        <v>10906</v>
+        <v>9745</v>
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>21/26</t>
+          <t>22/26</t>
         </is>
       </c>
       <c r="I60" s="3" t="inlineStr">
@@ -3471,10 +3471,10 @@
         </is>
       </c>
       <c r="J60" s="4" t="n">
-        <v>13503</v>
+        <v>11517</v>
       </c>
       <c r="K60" s="5" t="n">
-        <v>519.3333333333334</v>
+        <v>442.9545454545454</v>
       </c>
     </row>
     <row r="61">
@@ -3507,11 +3507,11 @@
         </is>
       </c>
       <c r="G61" s="4" t="n">
-        <v>19812</v>
+        <v>21330</v>
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>17/22</t>
+          <t>18/22</t>
         </is>
       </c>
       <c r="I61" s="3" t="inlineStr">
@@ -3520,10 +3520,10 @@
         </is>
       </c>
       <c r="J61" s="4" t="n">
-        <v>25639</v>
+        <v>26070</v>
       </c>
       <c r="K61" s="5" t="n">
-        <v>1165.411764705882</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="62">
@@ -3556,11 +3556,11 @@
         </is>
       </c>
       <c r="G62" s="15" t="n">
-        <v>390</v>
+        <v>467</v>
       </c>
       <c r="H62" s="14" t="inlineStr">
         <is>
-          <t>24/27</t>
+          <t>26/27</t>
         </is>
       </c>
       <c r="I62" s="14" t="inlineStr">
@@ -3569,10 +3569,10 @@
         </is>
       </c>
       <c r="J62" s="15" t="n">
-        <v>439</v>
+        <v>485</v>
       </c>
       <c r="K62" s="16" t="n">
-        <v>16.25</v>
+        <v>17.96153846153846</v>
       </c>
     </row>
     <row r="63">
@@ -3605,11 +3605,11 @@
         </is>
       </c>
       <c r="G63" s="4" t="n">
-        <v>10451</v>
+        <v>9623</v>
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
-          <t>21/26</t>
+          <t>22/26</t>
         </is>
       </c>
       <c r="I63" s="3" t="inlineStr">
@@ -3618,10 +3618,10 @@
         </is>
       </c>
       <c r="J63" s="4" t="n">
-        <v>12939</v>
+        <v>11373</v>
       </c>
       <c r="K63" s="5" t="n">
-        <v>497.6666666666667</v>
+        <v>437.4090909090909</v>
       </c>
     </row>
     <row r="64">
@@ -3654,11 +3654,11 @@
         </is>
       </c>
       <c r="G64" s="4" t="n">
-        <v>9111</v>
+        <v>7946</v>
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>20/23</t>
+          <t>21/24</t>
         </is>
       </c>
       <c r="I64" s="3" t="inlineStr">
@@ -3667,10 +3667,10 @@
         </is>
       </c>
       <c r="J64" s="4" t="n">
-        <v>10478</v>
+        <v>9081</v>
       </c>
       <c r="K64" s="5" t="n">
-        <v>455.55</v>
+        <v>378.3809523809524</v>
       </c>
     </row>
     <row r="65">
@@ -3703,11 +3703,11 @@
         </is>
       </c>
       <c r="G65" s="11" t="n">
-        <v>3894</v>
+        <v>4265</v>
       </c>
       <c r="H65" s="10" t="inlineStr">
         <is>
-          <t>22/26</t>
+          <t>23/26</t>
         </is>
       </c>
       <c r="I65" s="10" t="inlineStr">
@@ -3716,10 +3716,10 @@
         </is>
       </c>
       <c r="J65" s="11" t="n">
-        <v>4602</v>
+        <v>4821</v>
       </c>
       <c r="K65" s="12" t="n">
-        <v>177</v>
+        <v>185.4347826086957</v>
       </c>
     </row>
     <row r="66">
@@ -3752,11 +3752,11 @@
         </is>
       </c>
       <c r="G66" s="4" t="n">
-        <v>35795</v>
+        <v>36512</v>
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>20/28</t>
+          <t>21/28</t>
         </is>
       </c>
       <c r="I66" s="3" t="inlineStr">
@@ -3765,10 +3765,10 @@
         </is>
       </c>
       <c r="J66" s="4" t="n">
-        <v>50113</v>
+        <v>48683</v>
       </c>
       <c r="K66" s="5" t="n">
-        <v>1789.75</v>
+        <v>1738.666666666667</v>
       </c>
     </row>
     <row r="67">
@@ -3801,11 +3801,11 @@
         </is>
       </c>
       <c r="G67" s="11" t="n">
-        <v>4000</v>
+        <v>2616</v>
       </c>
       <c r="H67" s="10" t="inlineStr">
         <is>
-          <t>16/21</t>
+          <t>17/21</t>
         </is>
       </c>
       <c r="I67" s="10" t="inlineStr">
@@ -3814,59 +3814,59 @@
         </is>
       </c>
       <c r="J67" s="11" t="n">
-        <v>5250</v>
+        <v>3232</v>
       </c>
       <c r="K67" s="12" t="n">
-        <v>250</v>
+        <v>153.8823529411765</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="10" t="inlineStr">
+      <c r="A68" s="2" t="inlineStr">
         <is>
           <t>KATPADI</t>
         </is>
       </c>
-      <c r="B68" s="10" t="n">
+      <c r="B68" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="C68" s="10" t="inlineStr">
+      <c r="C68" s="3" t="inlineStr">
         <is>
           <t>DR M SUDHAKAR</t>
         </is>
       </c>
-      <c r="D68" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E68" s="10" t="inlineStr">
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
         <is>
           <t>DURAIMURUGAN</t>
         </is>
       </c>
-      <c r="F68" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G68" s="11" t="n">
-        <v>4822</v>
-      </c>
-      <c r="H68" s="10" t="inlineStr">
-        <is>
-          <t>15/20</t>
-        </is>
-      </c>
-      <c r="I68" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J68" s="11" t="n">
-        <v>6429</v>
-      </c>
-      <c r="K68" s="12" t="n">
-        <v>321.4666666666666</v>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G68" s="4" t="n">
+        <v>5146</v>
+      </c>
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t>16/20</t>
+        </is>
+      </c>
+      <c r="I68" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J68" s="4" t="n">
+        <v>6432</v>
+      </c>
+      <c r="K68" s="5" t="n">
+        <v>321.625</v>
       </c>
     </row>
     <row r="69">
@@ -3899,11 +3899,11 @@
         </is>
       </c>
       <c r="G69" s="4" t="n">
-        <v>27462</v>
+        <v>31177</v>
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
-          <t>19/21</t>
+          <t>20/21</t>
         </is>
       </c>
       <c r="I69" s="3" t="inlineStr">
@@ -3912,10 +3912,10 @@
         </is>
       </c>
       <c r="J69" s="4" t="n">
-        <v>30353</v>
+        <v>32736</v>
       </c>
       <c r="K69" s="5" t="n">
-        <v>1445.368421052632</v>
+        <v>1558.85</v>
       </c>
     </row>
     <row r="70">
@@ -4046,11 +4046,11 @@
         </is>
       </c>
       <c r="G72" s="4" t="n">
-        <v>29935</v>
+        <v>29639</v>
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>19/22</t>
+          <t>20/22</t>
         </is>
       </c>
       <c r="I72" s="3" t="inlineStr">
@@ -4059,10 +4059,10 @@
         </is>
       </c>
       <c r="J72" s="4" t="n">
-        <v>34662</v>
+        <v>32603</v>
       </c>
       <c r="K72" s="5" t="n">
-        <v>1575.526315789474</v>
+        <v>1481.95</v>
       </c>
     </row>
     <row r="73">
@@ -4095,11 +4095,11 @@
         </is>
       </c>
       <c r="G73" s="4" t="n">
-        <v>15033</v>
+        <v>17544</v>
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
-          <t>15/19</t>
+          <t>17/19</t>
         </is>
       </c>
       <c r="I73" s="3" t="inlineStr">
@@ -4108,10 +4108,10 @@
         </is>
       </c>
       <c r="J73" s="4" t="n">
-        <v>19042</v>
+        <v>19608</v>
       </c>
       <c r="K73" s="5" t="n">
-        <v>1002.2</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="74">
@@ -4262,52 +4262,52 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="13" t="inlineStr">
+      <c r="A77" s="6" t="inlineStr">
         <is>
           <t>KOVILPATTI</t>
         </is>
       </c>
-      <c r="B77" s="14" t="n">
+      <c r="B77" s="7" t="n">
         <v>218</v>
       </c>
-      <c r="C77" s="14" t="inlineStr">
+      <c r="C77" s="7" t="inlineStr">
+        <is>
+          <t>KARUNANITHI.K</t>
+        </is>
+      </c>
+      <c r="D77" s="7" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E77" s="7" t="inlineStr">
         <is>
           <t>BALASUBRAMANIAN.S</t>
         </is>
       </c>
-      <c r="D77" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E77" s="14" t="inlineStr">
-        <is>
-          <t>KARUNANITHI.K</t>
-        </is>
-      </c>
-      <c r="F77" s="14" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G77" s="15" t="n">
-        <v>329</v>
-      </c>
-      <c r="H77" s="14" t="inlineStr">
-        <is>
-          <t>21/23</t>
-        </is>
-      </c>
-      <c r="I77" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J77" s="15" t="n">
-        <v>360</v>
-      </c>
-      <c r="K77" s="16" t="n">
-        <v>15.66666666666667</v>
+      <c r="F77" s="7" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G77" s="8" t="n">
+        <v>509</v>
+      </c>
+      <c r="H77" s="7" t="inlineStr">
+        <is>
+          <t>22/23</t>
+        </is>
+      </c>
+      <c r="I77" s="7" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J77" s="8" t="n">
+        <v>532</v>
+      </c>
+      <c r="K77" s="9" t="n">
+        <v>23.13636363636364</v>
       </c>
     </row>
     <row r="78">
@@ -4340,7 +4340,7 @@
         </is>
       </c>
       <c r="G78" s="4" t="n">
-        <v>19571</v>
+        <v>19650</v>
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
@@ -4353,10 +4353,10 @@
         </is>
       </c>
       <c r="J78" s="4" t="n">
-        <v>21273</v>
+        <v>21359</v>
       </c>
       <c r="K78" s="5" t="n">
-        <v>850.9130434782609</v>
+        <v>854.3478260869565</v>
       </c>
     </row>
     <row r="79">
@@ -4389,11 +4389,11 @@
         </is>
       </c>
       <c r="G79" s="11" t="n">
-        <v>3352</v>
+        <v>3641</v>
       </c>
       <c r="H79" s="10" t="inlineStr">
         <is>
-          <t>17/20</t>
+          <t>18/20</t>
         </is>
       </c>
       <c r="I79" s="10" t="inlineStr">
@@ -4402,10 +4402,10 @@
         </is>
       </c>
       <c r="J79" s="11" t="n">
-        <v>3944</v>
+        <v>4046</v>
       </c>
       <c r="K79" s="12" t="n">
-        <v>197.1764705882353</v>
+        <v>202.2777777777778</v>
       </c>
     </row>
     <row r="80">
@@ -4438,11 +4438,11 @@
         </is>
       </c>
       <c r="G80" s="8" t="n">
-        <v>542</v>
+        <v>560</v>
       </c>
       <c r="H80" s="7" t="inlineStr">
         <is>
-          <t>18/21</t>
+          <t>19/21</t>
         </is>
       </c>
       <c r="I80" s="7" t="inlineStr">
@@ -4451,10 +4451,10 @@
         </is>
       </c>
       <c r="J80" s="8" t="n">
-        <v>632</v>
+        <v>619</v>
       </c>
       <c r="K80" s="9" t="n">
-        <v>30.11111111111111</v>
+        <v>29.47368421052632</v>
       </c>
     </row>
     <row r="81">
@@ -4487,11 +4487,11 @@
         </is>
       </c>
       <c r="G81" s="4" t="n">
-        <v>8039</v>
+        <v>8167</v>
       </c>
       <c r="H81" s="3" t="inlineStr">
         <is>
-          <t>21/24</t>
+          <t>22/24</t>
         </is>
       </c>
       <c r="I81" s="3" t="inlineStr">
@@ -4500,10 +4500,10 @@
         </is>
       </c>
       <c r="J81" s="4" t="n">
-        <v>9187</v>
+        <v>8909</v>
       </c>
       <c r="K81" s="5" t="n">
-        <v>382.8095238095238</v>
+        <v>371.2272727272727</v>
       </c>
     </row>
     <row r="82">
@@ -4585,11 +4585,11 @@
         </is>
       </c>
       <c r="G83" s="4" t="n">
-        <v>16311</v>
+        <v>16141</v>
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
-          <t>23/25</t>
+          <t>24/25</t>
         </is>
       </c>
       <c r="I83" s="3" t="inlineStr">
@@ -4598,10 +4598,10 @@
         </is>
       </c>
       <c r="J83" s="4" t="n">
-        <v>17729</v>
+        <v>16814</v>
       </c>
       <c r="K83" s="5" t="n">
-        <v>709.1739130434783</v>
+        <v>672.5416666666666</v>
       </c>
     </row>
     <row r="84">
@@ -4634,11 +4634,11 @@
         </is>
       </c>
       <c r="G84" s="4" t="n">
-        <v>5651</v>
+        <v>7589</v>
       </c>
       <c r="H84" s="3" t="inlineStr">
         <is>
-          <t>19/20</t>
+          <t>20/20</t>
         </is>
       </c>
       <c r="I84" s="3" t="inlineStr">
@@ -4647,10 +4647,10 @@
         </is>
       </c>
       <c r="J84" s="4" t="n">
-        <v>5948</v>
+        <v>7589</v>
       </c>
       <c r="K84" s="5" t="n">
-        <v>297.421052631579</v>
+        <v>379.45</v>
       </c>
     </row>
     <row r="85">
@@ -4683,11 +4683,11 @@
         </is>
       </c>
       <c r="G85" s="8" t="n">
-        <v>2086</v>
+        <v>2731</v>
       </c>
       <c r="H85" s="7" t="inlineStr">
         <is>
-          <t>19/21</t>
+          <t>20/21</t>
         </is>
       </c>
       <c r="I85" s="7" t="inlineStr">
@@ -4696,10 +4696,10 @@
         </is>
       </c>
       <c r="J85" s="8" t="n">
-        <v>2306</v>
+        <v>2868</v>
       </c>
       <c r="K85" s="9" t="n">
-        <v>109.7894736842105</v>
+        <v>136.55</v>
       </c>
     </row>
     <row r="86">
@@ -4888,7 +4888,7 @@
       </c>
       <c r="I89" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J89" s="4" t="n">
@@ -5075,11 +5075,11 @@
         </is>
       </c>
       <c r="G93" s="4" t="n">
-        <v>7361</v>
+        <v>7194</v>
       </c>
       <c r="H93" s="3" t="inlineStr">
         <is>
-          <t>21/22</t>
+          <t>22/22</t>
         </is>
       </c>
       <c r="I93" s="3" t="inlineStr">
@@ -5088,10 +5088,10 @@
         </is>
       </c>
       <c r="J93" s="4" t="n">
-        <v>7712</v>
+        <v>7194</v>
       </c>
       <c r="K93" s="5" t="n">
-        <v>350.5238095238095</v>
+        <v>327</v>
       </c>
     </row>
     <row r="94">
@@ -5124,11 +5124,11 @@
         </is>
       </c>
       <c r="G94" s="4" t="n">
-        <v>54806</v>
+        <v>56298</v>
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
-          <t>20/25</t>
+          <t>21/25</t>
         </is>
       </c>
       <c r="I94" s="3" t="inlineStr">
@@ -5137,10 +5137,10 @@
         </is>
       </c>
       <c r="J94" s="4" t="n">
-        <v>68508</v>
+        <v>67021</v>
       </c>
       <c r="K94" s="5" t="n">
-        <v>2740.3</v>
+        <v>2680.857142857143</v>
       </c>
     </row>
     <row r="95">
@@ -5271,11 +5271,11 @@
         </is>
       </c>
       <c r="G97" s="11" t="n">
-        <v>7640</v>
+        <v>7263</v>
       </c>
       <c r="H97" s="10" t="inlineStr">
         <is>
-          <t>18/27</t>
+          <t>19/27</t>
         </is>
       </c>
       <c r="I97" s="10" t="inlineStr">
@@ -5284,10 +5284,10 @@
         </is>
       </c>
       <c r="J97" s="11" t="n">
-        <v>11460</v>
+        <v>10321</v>
       </c>
       <c r="K97" s="12" t="n">
-        <v>424.4444444444445</v>
+        <v>382.2631578947368</v>
       </c>
     </row>
     <row r="98">
@@ -5320,11 +5320,11 @@
         </is>
       </c>
       <c r="G98" s="8" t="n">
-        <v>1378</v>
+        <v>1426</v>
       </c>
       <c r="H98" s="7" t="inlineStr">
         <is>
-          <t>25/26</t>
+          <t>26/26</t>
         </is>
       </c>
       <c r="I98" s="7" t="inlineStr">
@@ -5333,10 +5333,10 @@
         </is>
       </c>
       <c r="J98" s="8" t="n">
-        <v>1433</v>
+        <v>1426</v>
       </c>
       <c r="K98" s="9" t="n">
-        <v>55.12</v>
+        <v>54.84615384615385</v>
       </c>
     </row>
     <row r="99">
@@ -5516,11 +5516,11 @@
         </is>
       </c>
       <c r="G102" s="4" t="n">
-        <v>5973</v>
+        <v>6690</v>
       </c>
       <c r="H102" s="3" t="inlineStr">
         <is>
-          <t>23/26</t>
+          <t>24/26</t>
         </is>
       </c>
       <c r="I102" s="3" t="inlineStr">
@@ -5529,10 +5529,10 @@
         </is>
       </c>
       <c r="J102" s="4" t="n">
-        <v>6752</v>
+        <v>7248</v>
       </c>
       <c r="K102" s="5" t="n">
-        <v>259.6956521739131</v>
+        <v>278.75</v>
       </c>
     </row>
     <row r="103">
@@ -5565,11 +5565,11 @@
         </is>
       </c>
       <c r="G103" s="4" t="n">
-        <v>8823</v>
+        <v>13231</v>
       </c>
       <c r="H103" s="3" t="inlineStr">
         <is>
-          <t>19/24</t>
+          <t>21/24</t>
         </is>
       </c>
       <c r="I103" s="3" t="inlineStr">
@@ -5578,10 +5578,10 @@
         </is>
       </c>
       <c r="J103" s="4" t="n">
-        <v>11145</v>
+        <v>15121</v>
       </c>
       <c r="K103" s="5" t="n">
-        <v>464.3684210526316</v>
+        <v>630.047619047619</v>
       </c>
     </row>
     <row r="104">
@@ -5663,11 +5663,11 @@
         </is>
       </c>
       <c r="G105" s="4" t="n">
-        <v>16184</v>
+        <v>17050</v>
       </c>
       <c r="H105" s="3" t="inlineStr">
         <is>
-          <t>28/32</t>
+          <t>29/32</t>
         </is>
       </c>
       <c r="I105" s="3" t="inlineStr">
@@ -5676,10 +5676,10 @@
         </is>
       </c>
       <c r="J105" s="4" t="n">
-        <v>18496</v>
+        <v>18814</v>
       </c>
       <c r="K105" s="5" t="n">
-        <v>578</v>
+        <v>587.9310344827586</v>
       </c>
     </row>
     <row r="106">
@@ -5810,11 +5810,11 @@
         </is>
       </c>
       <c r="G108" s="4" t="n">
-        <v>8774</v>
+        <v>10225</v>
       </c>
       <c r="H108" s="3" t="inlineStr">
         <is>
-          <t>15/18</t>
+          <t>16/18</t>
         </is>
       </c>
       <c r="I108" s="3" t="inlineStr">
@@ -5823,10 +5823,10 @@
         </is>
       </c>
       <c r="J108" s="4" t="n">
-        <v>10529</v>
+        <v>11503</v>
       </c>
       <c r="K108" s="5" t="n">
-        <v>584.9333333333333</v>
+        <v>639.0625</v>
       </c>
     </row>
     <row r="109">
@@ -5908,11 +5908,11 @@
         </is>
       </c>
       <c r="G110" s="11" t="n">
-        <v>5165</v>
+        <v>7284</v>
       </c>
       <c r="H110" s="10" t="inlineStr">
         <is>
-          <t>14/23</t>
+          <t>15/23</t>
         </is>
       </c>
       <c r="I110" s="10" t="inlineStr">
@@ -5921,10 +5921,10 @@
         </is>
       </c>
       <c r="J110" s="11" t="n">
-        <v>8485</v>
+        <v>11169</v>
       </c>
       <c r="K110" s="12" t="n">
-        <v>368.9285714285714</v>
+        <v>485.6</v>
       </c>
     </row>
     <row r="111">
@@ -6059,7 +6059,7 @@
       </c>
       <c r="H113" s="3" t="inlineStr">
         <is>
-          <t>26/26</t>
+          <t>26/27</t>
         </is>
       </c>
       <c r="I113" s="3" t="inlineStr">
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="J113" s="4" t="n">
-        <v>11740</v>
+        <v>12192</v>
       </c>
       <c r="K113" s="5" t="n">
         <v>451.5384615384615</v>
@@ -6104,11 +6104,11 @@
         </is>
       </c>
       <c r="G114" s="4" t="n">
-        <v>11034</v>
+        <v>10962</v>
       </c>
       <c r="H114" s="3" t="inlineStr">
         <is>
-          <t>19/20</t>
+          <t>20/20</t>
         </is>
       </c>
       <c r="I114" s="3" t="inlineStr">
@@ -6117,10 +6117,10 @@
         </is>
       </c>
       <c r="J114" s="4" t="n">
-        <v>11615</v>
+        <v>10962</v>
       </c>
       <c r="K114" s="5" t="n">
-        <v>580.7368421052631</v>
+        <v>548.1</v>
       </c>
     </row>
     <row r="115">
@@ -6153,11 +6153,11 @@
         </is>
       </c>
       <c r="G115" s="11" t="n">
-        <v>3301</v>
+        <v>3794</v>
       </c>
       <c r="H115" s="10" t="inlineStr">
         <is>
-          <t>19/23</t>
+          <t>20/23</t>
         </is>
       </c>
       <c r="I115" s="10" t="inlineStr">
@@ -6166,10 +6166,10 @@
         </is>
       </c>
       <c r="J115" s="11" t="n">
-        <v>3996</v>
+        <v>4363</v>
       </c>
       <c r="K115" s="12" t="n">
-        <v>173.7368421052632</v>
+        <v>189.7</v>
       </c>
     </row>
     <row r="116">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="I116" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J116" s="4" t="n">
@@ -6251,11 +6251,11 @@
         </is>
       </c>
       <c r="G117" s="4" t="n">
-        <v>15792</v>
+        <v>14539</v>
       </c>
       <c r="H117" s="3" t="inlineStr">
         <is>
-          <t>24/26</t>
+          <t>26/26</t>
         </is>
       </c>
       <c r="I117" s="3" t="inlineStr">
@@ -6264,10 +6264,10 @@
         </is>
       </c>
       <c r="J117" s="4" t="n">
-        <v>17108</v>
+        <v>14539</v>
       </c>
       <c r="K117" s="5" t="n">
-        <v>658</v>
+        <v>559.1923076923077</v>
       </c>
     </row>
     <row r="118">
@@ -6398,11 +6398,11 @@
         </is>
       </c>
       <c r="G120" s="4" t="n">
-        <v>15462</v>
+        <v>15569</v>
       </c>
       <c r="H120" s="3" t="inlineStr">
         <is>
-          <t>23/24</t>
+          <t>24/24</t>
         </is>
       </c>
       <c r="I120" s="3" t="inlineStr">
@@ -6411,10 +6411,10 @@
         </is>
       </c>
       <c r="J120" s="4" t="n">
-        <v>16134</v>
+        <v>15569</v>
       </c>
       <c r="K120" s="5" t="n">
-        <v>672.2608695652174</v>
+        <v>648.7083333333334</v>
       </c>
     </row>
     <row r="121">
@@ -6594,11 +6594,11 @@
         </is>
       </c>
       <c r="G124" s="4" t="n">
-        <v>38195</v>
+        <v>37897</v>
       </c>
       <c r="H124" s="3" t="inlineStr">
         <is>
-          <t>34/35</t>
+          <t>35/35</t>
         </is>
       </c>
       <c r="I124" s="3" t="inlineStr">
@@ -6607,10 +6607,10 @@
         </is>
       </c>
       <c r="J124" s="4" t="n">
-        <v>39318</v>
+        <v>37897</v>
       </c>
       <c r="K124" s="5" t="n">
-        <v>1123.382352941177</v>
+        <v>1082.771428571428</v>
       </c>
     </row>
     <row r="125">
@@ -6643,11 +6643,11 @@
         </is>
       </c>
       <c r="G125" s="4" t="n">
-        <v>40846</v>
+        <v>44311</v>
       </c>
       <c r="H125" s="3" t="inlineStr">
         <is>
-          <t>24/34</t>
+          <t>26/34</t>
         </is>
       </c>
       <c r="I125" s="3" t="inlineStr">
@@ -6656,10 +6656,10 @@
         </is>
       </c>
       <c r="J125" s="4" t="n">
-        <v>57865</v>
+        <v>57945</v>
       </c>
       <c r="K125" s="5" t="n">
-        <v>1701.916666666667</v>
+        <v>1704.269230769231</v>
       </c>
     </row>
     <row r="126">
@@ -6692,11 +6692,11 @@
         </is>
       </c>
       <c r="G126" s="4" t="n">
-        <v>10902</v>
+        <v>10663</v>
       </c>
       <c r="H126" s="3" t="inlineStr">
         <is>
-          <t>21/23</t>
+          <t>23/23</t>
         </is>
       </c>
       <c r="I126" s="3" t="inlineStr">
@@ -6705,10 +6705,10 @@
         </is>
       </c>
       <c r="J126" s="4" t="n">
-        <v>11940</v>
+        <v>10663</v>
       </c>
       <c r="K126" s="5" t="n">
-        <v>519.1428571428571</v>
+        <v>463.6086956521739</v>
       </c>
     </row>
     <row r="127">
@@ -6741,11 +6741,11 @@
         </is>
       </c>
       <c r="G127" s="11" t="n">
-        <v>3900</v>
+        <v>2773</v>
       </c>
       <c r="H127" s="10" t="inlineStr">
         <is>
-          <t>16/23</t>
+          <t>18/23</t>
         </is>
       </c>
       <c r="I127" s="10" t="inlineStr">
@@ -6754,10 +6754,10 @@
         </is>
       </c>
       <c r="J127" s="11" t="n">
-        <v>5606</v>
+        <v>3543</v>
       </c>
       <c r="K127" s="12" t="n">
-        <v>243.75</v>
+        <v>154.0555555555555</v>
       </c>
     </row>
     <row r="128">
@@ -6790,11 +6790,11 @@
         </is>
       </c>
       <c r="G128" s="4" t="n">
-        <v>33463</v>
+        <v>33114</v>
       </c>
       <c r="H128" s="3" t="inlineStr">
         <is>
-          <t>24/25</t>
+          <t>25/25</t>
         </is>
       </c>
       <c r="I128" s="3" t="inlineStr">
@@ -6803,10 +6803,10 @@
         </is>
       </c>
       <c r="J128" s="4" t="n">
-        <v>34857</v>
+        <v>33114</v>
       </c>
       <c r="K128" s="5" t="n">
-        <v>1394.291666666667</v>
+        <v>1324.56</v>
       </c>
     </row>
     <row r="129">
@@ -6839,11 +6839,11 @@
         </is>
       </c>
       <c r="G129" s="11" t="n">
-        <v>3509</v>
+        <v>3556</v>
       </c>
       <c r="H129" s="10" t="inlineStr">
         <is>
-          <t>23/24</t>
+          <t>24/25</t>
         </is>
       </c>
       <c r="I129" s="10" t="inlineStr">
@@ -6852,10 +6852,10 @@
         </is>
       </c>
       <c r="J129" s="11" t="n">
-        <v>3662</v>
+        <v>3704</v>
       </c>
       <c r="K129" s="12" t="n">
-        <v>152.5652173913043</v>
+        <v>148.1666666666667</v>
       </c>
     </row>
     <row r="130">
@@ -6888,11 +6888,11 @@
         </is>
       </c>
       <c r="G130" s="15" t="n">
-        <v>47</v>
+        <v>82</v>
       </c>
       <c r="H130" s="14" t="inlineStr">
         <is>
-          <t>16/20</t>
+          <t>17/20</t>
         </is>
       </c>
       <c r="I130" s="14" t="inlineStr">
@@ -6901,10 +6901,10 @@
         </is>
       </c>
       <c r="J130" s="15" t="n">
-        <v>59</v>
+        <v>96</v>
       </c>
       <c r="K130" s="16" t="n">
-        <v>2.9375</v>
+        <v>4.823529411764706</v>
       </c>
     </row>
     <row r="131">
@@ -6937,11 +6937,11 @@
         </is>
       </c>
       <c r="G131" s="4" t="n">
-        <v>6708</v>
+        <v>8035</v>
       </c>
       <c r="H131" s="3" t="inlineStr">
         <is>
-          <t>20/23</t>
+          <t>21/23</t>
         </is>
       </c>
       <c r="I131" s="3" t="inlineStr">
@@ -6950,10 +6950,10 @@
         </is>
       </c>
       <c r="J131" s="4" t="n">
-        <v>7714</v>
+        <v>8800</v>
       </c>
       <c r="K131" s="5" t="n">
-        <v>335.4</v>
+        <v>382.6190476190476</v>
       </c>
     </row>
     <row r="132">
@@ -6986,11 +6986,11 @@
         </is>
       </c>
       <c r="G132" s="11" t="n">
-        <v>3535</v>
+        <v>3165</v>
       </c>
       <c r="H132" s="10" t="inlineStr">
         <is>
-          <t>22/23</t>
+          <t>23/23</t>
         </is>
       </c>
       <c r="I132" s="10" t="inlineStr">
@@ -6999,10 +6999,10 @@
         </is>
       </c>
       <c r="J132" s="11" t="n">
-        <v>3696</v>
+        <v>3165</v>
       </c>
       <c r="K132" s="12" t="n">
-        <v>160.6818181818182</v>
+        <v>137.6086956521739</v>
       </c>
     </row>
     <row r="133">
@@ -7035,11 +7035,11 @@
         </is>
       </c>
       <c r="G133" s="4" t="n">
-        <v>13775</v>
+        <v>13580</v>
       </c>
       <c r="H133" s="3" t="inlineStr">
         <is>
-          <t>26/28</t>
+          <t>27/28</t>
         </is>
       </c>
       <c r="I133" s="3" t="inlineStr">
@@ -7048,10 +7048,10 @@
         </is>
       </c>
       <c r="J133" s="4" t="n">
-        <v>14835</v>
+        <v>14083</v>
       </c>
       <c r="K133" s="5" t="n">
-        <v>529.8076923076923</v>
+        <v>502.962962962963</v>
       </c>
     </row>
     <row r="134">
@@ -7084,11 +7084,11 @@
         </is>
       </c>
       <c r="G134" s="4" t="n">
-        <v>41945</v>
+        <v>44267</v>
       </c>
       <c r="H134" s="3" t="inlineStr">
         <is>
-          <t>17/22</t>
+          <t>18/22</t>
         </is>
       </c>
       <c r="I134" s="3" t="inlineStr">
@@ -7097,10 +7097,10 @@
         </is>
       </c>
       <c r="J134" s="4" t="n">
-        <v>54282</v>
+        <v>54104</v>
       </c>
       <c r="K134" s="5" t="n">
-        <v>2467.352941176471</v>
+        <v>2459.277777777778</v>
       </c>
     </row>
     <row r="135">
@@ -7133,11 +7133,11 @@
         </is>
       </c>
       <c r="G135" s="8" t="n">
-        <v>658</v>
+        <v>573</v>
       </c>
       <c r="H135" s="7" t="inlineStr">
         <is>
-          <t>12/21</t>
+          <t>13/21</t>
         </is>
       </c>
       <c r="I135" s="7" t="inlineStr">
@@ -7146,10 +7146,10 @@
         </is>
       </c>
       <c r="J135" s="8" t="n">
-        <v>1152</v>
+        <v>926</v>
       </c>
       <c r="K135" s="9" t="n">
-        <v>54.83333333333334</v>
+        <v>44.07692307692308</v>
       </c>
     </row>
     <row r="136">
@@ -7182,11 +7182,11 @@
         </is>
       </c>
       <c r="G136" s="4" t="n">
-        <v>11410</v>
+        <v>14416</v>
       </c>
       <c r="H136" s="3" t="inlineStr">
         <is>
-          <t>21/26</t>
+          <t>23/26</t>
         </is>
       </c>
       <c r="I136" s="3" t="inlineStr">
@@ -7195,10 +7195,10 @@
         </is>
       </c>
       <c r="J136" s="4" t="n">
-        <v>14127</v>
+        <v>16296</v>
       </c>
       <c r="K136" s="5" t="n">
-        <v>543.3333333333334</v>
+        <v>626.7826086956521</v>
       </c>
     </row>
     <row r="137">
@@ -7289,7 +7289,7 @@
       </c>
       <c r="I138" s="10" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J138" s="11" t="n">
@@ -7382,7 +7382,7 @@
       </c>
       <c r="H140" s="3" t="inlineStr">
         <is>
-          <t>24/24</t>
+          <t>24/26</t>
         </is>
       </c>
       <c r="I140" s="3" t="inlineStr">
@@ -7391,7 +7391,7 @@
         </is>
       </c>
       <c r="J140" s="4" t="n">
-        <v>55529</v>
+        <v>60156</v>
       </c>
       <c r="K140" s="5" t="n">
         <v>2313.708333333333</v>
@@ -7427,11 +7427,11 @@
         </is>
       </c>
       <c r="G141" s="11" t="n">
-        <v>5512</v>
+        <v>6054</v>
       </c>
       <c r="H141" s="10" t="inlineStr">
         <is>
-          <t>17/25</t>
+          <t>18/25</t>
         </is>
       </c>
       <c r="I141" s="10" t="inlineStr">
@@ -7440,10 +7440,10 @@
         </is>
       </c>
       <c r="J141" s="11" t="n">
-        <v>8106</v>
+        <v>8408</v>
       </c>
       <c r="K141" s="12" t="n">
-        <v>324.2352941176471</v>
+        <v>336.3333333333333</v>
       </c>
     </row>
     <row r="142">
@@ -7496,52 +7496,52 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="10" t="inlineStr">
+      <c r="A143" s="6" t="inlineStr">
         <is>
           <t>PUDUKKOTTAI</t>
         </is>
       </c>
-      <c r="B143" s="10" t="n">
+      <c r="B143" s="7" t="n">
         <v>180</v>
       </c>
-      <c r="C143" s="10" t="inlineStr">
+      <c r="C143" s="7" t="inlineStr">
         <is>
           <t>V. MUTHURAJA</t>
         </is>
       </c>
-      <c r="D143" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E143" s="10" t="inlineStr">
+      <c r="D143" s="7" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E143" s="7" t="inlineStr">
         <is>
           <t>K.M. SHARIFF</t>
         </is>
       </c>
-      <c r="F143" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G143" s="11" t="n">
-        <v>2942</v>
-      </c>
-      <c r="H143" s="10" t="inlineStr">
-        <is>
-          <t>18/22</t>
-        </is>
-      </c>
-      <c r="I143" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J143" s="11" t="n">
-        <v>3596</v>
-      </c>
-      <c r="K143" s="12" t="n">
-        <v>163.4444444444445</v>
+      <c r="F143" s="7" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G143" s="8" t="n">
+        <v>2452</v>
+      </c>
+      <c r="H143" s="7" t="inlineStr">
+        <is>
+          <t>19/22</t>
+        </is>
+      </c>
+      <c r="I143" s="7" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J143" s="8" t="n">
+        <v>2839</v>
+      </c>
+      <c r="K143" s="9" t="n">
+        <v>129.0526315789474</v>
       </c>
     </row>
     <row r="144">
@@ -7681,7 +7681,7 @@
       </c>
       <c r="I146" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J146" s="4" t="n">
@@ -7917,11 +7917,11 @@
         </is>
       </c>
       <c r="G151" s="4" t="n">
-        <v>28344</v>
+        <v>28514</v>
       </c>
       <c r="H151" s="3" t="inlineStr">
         <is>
-          <t>20/21</t>
+          <t>21/21</t>
         </is>
       </c>
       <c r="I151" s="3" t="inlineStr">
@@ -7930,10 +7930,10 @@
         </is>
       </c>
       <c r="J151" s="4" t="n">
-        <v>29761</v>
+        <v>28514</v>
       </c>
       <c r="K151" s="5" t="n">
-        <v>1417.2</v>
+        <v>1357.809523809524</v>
       </c>
     </row>
     <row r="152">
@@ -7966,11 +7966,11 @@
         </is>
       </c>
       <c r="G152" s="4" t="n">
-        <v>11244</v>
+        <v>12741</v>
       </c>
       <c r="H152" s="3" t="inlineStr">
         <is>
-          <t>19/21</t>
+          <t>20/21</t>
         </is>
       </c>
       <c r="I152" s="3" t="inlineStr">
@@ -7979,10 +7979,10 @@
         </is>
       </c>
       <c r="J152" s="4" t="n">
-        <v>12428</v>
+        <v>13378</v>
       </c>
       <c r="K152" s="5" t="n">
-        <v>591.7894736842105</v>
+        <v>637.05</v>
       </c>
     </row>
     <row r="153">
@@ -8113,11 +8113,11 @@
         </is>
       </c>
       <c r="G155" s="4" t="n">
-        <v>5394</v>
+        <v>5456</v>
       </c>
       <c r="H155" s="3" t="inlineStr">
         <is>
-          <t>20/23</t>
+          <t>21/23</t>
         </is>
       </c>
       <c r="I155" s="3" t="inlineStr">
@@ -8126,59 +8126,59 @@
         </is>
       </c>
       <c r="J155" s="4" t="n">
-        <v>6203</v>
+        <v>5976</v>
       </c>
       <c r="K155" s="5" t="n">
-        <v>269.7</v>
+        <v>259.8095238095238</v>
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="13" t="inlineStr">
+      <c r="A156" s="6" t="inlineStr">
         <is>
           <t>SANKARAPURAM</t>
         </is>
       </c>
-      <c r="B156" s="14" t="n">
+      <c r="B156" s="7" t="n">
         <v>79</v>
       </c>
-      <c r="C156" s="14" t="inlineStr">
+      <c r="C156" s="7" t="inlineStr">
+        <is>
+          <t>RAKESH R</t>
+        </is>
+      </c>
+      <c r="D156" s="7" t="inlineStr">
+        <is>
+          <t>All India Anna Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E156" s="7" t="inlineStr">
         <is>
           <t>UDHAYASURIYAN T</t>
         </is>
       </c>
-      <c r="D156" s="14" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E156" s="14" t="inlineStr">
-        <is>
-          <t>RAKESH R</t>
-        </is>
-      </c>
-      <c r="F156" s="14" t="inlineStr">
-        <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G156" s="15" t="n">
-        <v>32</v>
-      </c>
-      <c r="H156" s="14" t="inlineStr">
-        <is>
-          <t>15/25</t>
-        </is>
-      </c>
-      <c r="I156" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J156" s="15" t="n">
-        <v>53</v>
-      </c>
-      <c r="K156" s="16" t="n">
-        <v>2.133333333333333</v>
+      <c r="F156" s="7" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G156" s="8" t="n">
+        <v>636</v>
+      </c>
+      <c r="H156" s="7" t="inlineStr">
+        <is>
+          <t>16/25</t>
+        </is>
+      </c>
+      <c r="I156" s="7" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J156" s="8" t="n">
+        <v>994</v>
+      </c>
+      <c r="K156" s="9" t="n">
+        <v>39.75</v>
       </c>
     </row>
     <row r="157">
@@ -8260,11 +8260,11 @@
         </is>
       </c>
       <c r="G158" s="11" t="n">
-        <v>3031</v>
+        <v>4060</v>
       </c>
       <c r="H158" s="10" t="inlineStr">
         <is>
-          <t>15/21</t>
+          <t>17/21</t>
         </is>
       </c>
       <c r="I158" s="10" t="inlineStr">
@@ -8273,10 +8273,10 @@
         </is>
       </c>
       <c r="J158" s="11" t="n">
-        <v>4243</v>
+        <v>5015</v>
       </c>
       <c r="K158" s="12" t="n">
-        <v>202.0666666666667</v>
+        <v>238.8235294117647</v>
       </c>
     </row>
     <row r="159">
@@ -8358,11 +8358,11 @@
         </is>
       </c>
       <c r="G160" s="8" t="n">
-        <v>499</v>
+        <v>573</v>
       </c>
       <c r="H160" s="7" t="inlineStr">
         <is>
-          <t>16/19</t>
+          <t>17/19</t>
         </is>
       </c>
       <c r="I160" s="7" t="inlineStr">
@@ -8371,10 +8371,10 @@
         </is>
       </c>
       <c r="J160" s="8" t="n">
-        <v>593</v>
+        <v>640</v>
       </c>
       <c r="K160" s="9" t="n">
-        <v>31.1875</v>
+        <v>33.70588235294117</v>
       </c>
     </row>
     <row r="161">
@@ -8407,11 +8407,11 @@
         </is>
       </c>
       <c r="G161" s="11" t="n">
-        <v>4115</v>
+        <v>5058</v>
       </c>
       <c r="H161" s="10" t="inlineStr">
         <is>
-          <t>15/25</t>
+          <t>16/25</t>
         </is>
       </c>
       <c r="I161" s="10" t="inlineStr">
@@ -8420,10 +8420,10 @@
         </is>
       </c>
       <c r="J161" s="11" t="n">
-        <v>6858</v>
+        <v>7903</v>
       </c>
       <c r="K161" s="12" t="n">
-        <v>274.3333333333333</v>
+        <v>316.125</v>
       </c>
     </row>
     <row r="162">
@@ -8456,11 +8456,11 @@
         </is>
       </c>
       <c r="G162" s="4" t="n">
-        <v>61407</v>
+        <v>68669</v>
       </c>
       <c r="H162" s="3" t="inlineStr">
         <is>
-          <t>20/30</t>
+          <t>22/30</t>
         </is>
       </c>
       <c r="I162" s="3" t="inlineStr">
@@ -8469,10 +8469,10 @@
         </is>
       </c>
       <c r="J162" s="4" t="n">
-        <v>92110</v>
+        <v>93640</v>
       </c>
       <c r="K162" s="5" t="n">
-        <v>3070.35</v>
+        <v>3121.318181818182</v>
       </c>
     </row>
     <row r="163">
@@ -8496,20 +8496,20 @@
       </c>
       <c r="E163" s="3" t="inlineStr">
         <is>
-          <t>K.R.JAYARAM</t>
+          <t>V.SRINIDHI</t>
         </is>
       </c>
       <c r="F163" s="3" t="inlineStr">
         <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
+          <t>Indian National Congress</t>
         </is>
       </c>
       <c r="G163" s="4" t="n">
-        <v>22902</v>
+        <v>22396</v>
       </c>
       <c r="H163" s="3" t="inlineStr">
         <is>
-          <t>21/26</t>
+          <t>22/26</t>
         </is>
       </c>
       <c r="I163" s="3" t="inlineStr">
@@ -8518,10 +8518,10 @@
         </is>
       </c>
       <c r="J163" s="4" t="n">
-        <v>28355</v>
+        <v>26468</v>
       </c>
       <c r="K163" s="5" t="n">
-        <v>1090.571428571429</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="164">
@@ -8545,16 +8545,16 @@
       </c>
       <c r="E164" s="3" t="inlineStr">
         <is>
-          <t>GOPINATH.S</t>
+          <t>SAKTHI.M</t>
         </is>
       </c>
       <c r="F164" s="3" t="inlineStr">
         <is>
-          <t>Tamilaga Vettri Kazhagam</t>
+          <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
       <c r="G164" s="4" t="n">
-        <v>10766</v>
+        <v>11119</v>
       </c>
       <c r="H164" s="3" t="inlineStr">
         <is>
@@ -8567,10 +8567,10 @@
         </is>
       </c>
       <c r="J164" s="4" t="n">
-        <v>11843</v>
+        <v>12231</v>
       </c>
       <c r="K164" s="5" t="n">
-        <v>538.3</v>
+        <v>555.95</v>
       </c>
     </row>
     <row r="165">
@@ -8603,7 +8603,7 @@
         </is>
       </c>
       <c r="G165" s="4" t="n">
-        <v>15351</v>
+        <v>15502</v>
       </c>
       <c r="H165" s="3" t="inlineStr">
         <is>
@@ -8616,10 +8616,10 @@
         </is>
       </c>
       <c r="J165" s="4" t="n">
-        <v>16488</v>
+        <v>16650</v>
       </c>
       <c r="K165" s="5" t="n">
-        <v>568.5555555555555</v>
+        <v>574.1481481481482</v>
       </c>
     </row>
     <row r="166">
@@ -8652,11 +8652,11 @@
         </is>
       </c>
       <c r="G166" s="4" t="n">
-        <v>8012</v>
+        <v>8121</v>
       </c>
       <c r="H166" s="3" t="inlineStr">
         <is>
-          <t>16/21</t>
+          <t>18/21</t>
         </is>
       </c>
       <c r="I166" s="3" t="inlineStr">
@@ -8665,10 +8665,10 @@
         </is>
       </c>
       <c r="J166" s="4" t="n">
-        <v>10516</v>
+        <v>9474</v>
       </c>
       <c r="K166" s="5" t="n">
-        <v>500.75</v>
+        <v>451.1666666666667</v>
       </c>
     </row>
     <row r="167">
@@ -8701,11 +8701,11 @@
         </is>
       </c>
       <c r="G167" s="4" t="n">
-        <v>39734</v>
+        <v>42940</v>
       </c>
       <c r="H167" s="3" t="inlineStr">
         <is>
-          <t>23/32</t>
+          <t>25/32</t>
         </is>
       </c>
       <c r="I167" s="3" t="inlineStr">
@@ -8714,10 +8714,10 @@
         </is>
       </c>
       <c r="J167" s="4" t="n">
-        <v>55282</v>
+        <v>54963</v>
       </c>
       <c r="K167" s="5" t="n">
-        <v>1727.565217391304</v>
+        <v>1717.6</v>
       </c>
     </row>
     <row r="168">
@@ -8750,11 +8750,11 @@
         </is>
       </c>
       <c r="G168" s="4" t="n">
-        <v>30746</v>
+        <v>33781</v>
       </c>
       <c r="H168" s="3" t="inlineStr">
         <is>
-          <t>20/27</t>
+          <t>22/27</t>
         </is>
       </c>
       <c r="I168" s="3" t="inlineStr">
@@ -8763,10 +8763,10 @@
         </is>
       </c>
       <c r="J168" s="4" t="n">
-        <v>41507</v>
+        <v>41458</v>
       </c>
       <c r="K168" s="5" t="n">
-        <v>1537.3</v>
+        <v>1535.5</v>
       </c>
     </row>
     <row r="169">
@@ -8946,11 +8946,11 @@
         </is>
       </c>
       <c r="G172" s="4" t="n">
-        <v>32740</v>
+        <v>35540</v>
       </c>
       <c r="H172" s="3" t="inlineStr">
         <is>
-          <t>31/34</t>
+          <t>33/39</t>
         </is>
       </c>
       <c r="I172" s="3" t="inlineStr">
@@ -8959,10 +8959,10 @@
         </is>
       </c>
       <c r="J172" s="4" t="n">
-        <v>35908</v>
+        <v>42002</v>
       </c>
       <c r="K172" s="5" t="n">
-        <v>1056.129032258065</v>
+        <v>1076.969696969697</v>
       </c>
     </row>
     <row r="173">
@@ -8995,11 +8995,11 @@
         </is>
       </c>
       <c r="G173" s="4" t="n">
-        <v>9585</v>
+        <v>10064</v>
       </c>
       <c r="H173" s="3" t="inlineStr">
         <is>
-          <t>22/26</t>
+          <t>23/26</t>
         </is>
       </c>
       <c r="I173" s="3" t="inlineStr">
@@ -9008,10 +9008,10 @@
         </is>
       </c>
       <c r="J173" s="4" t="n">
-        <v>11328</v>
+        <v>11377</v>
       </c>
       <c r="K173" s="5" t="n">
-        <v>435.6818181818182</v>
+        <v>437.5652173913044</v>
       </c>
     </row>
     <row r="174">
@@ -9211,52 +9211,52 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="6" t="inlineStr">
+      <c r="A178" s="13" t="inlineStr">
         <is>
           <t>THIRUMAYAM</t>
         </is>
       </c>
-      <c r="B178" s="7" t="n">
+      <c r="B178" s="14" t="n">
         <v>181</v>
       </c>
-      <c r="C178" s="7" t="inlineStr">
+      <c r="C178" s="14" t="inlineStr">
         <is>
           <t>REGUPATHY.S</t>
         </is>
       </c>
-      <c r="D178" s="7" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E178" s="7" t="inlineStr">
+      <c r="D178" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E178" s="14" t="inlineStr">
         <is>
           <t>CHINTHAMANI.C</t>
         </is>
       </c>
-      <c r="F178" s="7" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G178" s="8" t="n">
-        <v>723</v>
-      </c>
-      <c r="H178" s="7" t="inlineStr">
-        <is>
-          <t>17/22</t>
-        </is>
-      </c>
-      <c r="I178" s="7" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J178" s="8" t="n">
-        <v>936</v>
-      </c>
-      <c r="K178" s="9" t="n">
-        <v>42.52941176470588</v>
+      <c r="F178" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G178" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="H178" s="14" t="inlineStr">
+        <is>
+          <t>19/22</t>
+        </is>
+      </c>
+      <c r="I178" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J178" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K178" s="16" t="n">
+        <v>0.1578947368421053</v>
       </c>
     </row>
     <row r="179">
@@ -9289,11 +9289,11 @@
         </is>
       </c>
       <c r="G179" s="4" t="n">
-        <v>37757</v>
+        <v>37938</v>
       </c>
       <c r="H179" s="3" t="inlineStr">
         <is>
-          <t>22/26</t>
+          <t>23/26</t>
         </is>
       </c>
       <c r="I179" s="3" t="inlineStr">
@@ -9302,10 +9302,10 @@
         </is>
       </c>
       <c r="J179" s="4" t="n">
-        <v>44622</v>
+        <v>42886</v>
       </c>
       <c r="K179" s="5" t="n">
-        <v>1716.227272727273</v>
+        <v>1649.478260869565</v>
       </c>
     </row>
     <row r="180">
@@ -9338,11 +9338,11 @@
         </is>
       </c>
       <c r="G180" s="4" t="n">
-        <v>31033</v>
+        <v>32772</v>
       </c>
       <c r="H180" s="3" t="inlineStr">
         <is>
-          <t>19/29</t>
+          <t>21/29</t>
         </is>
       </c>
       <c r="I180" s="3" t="inlineStr">
@@ -9351,10 +9351,10 @@
         </is>
       </c>
       <c r="J180" s="4" t="n">
-        <v>47366</v>
+        <v>45257</v>
       </c>
       <c r="K180" s="5" t="n">
-        <v>1633.315789473684</v>
+        <v>1560.571428571429</v>
       </c>
     </row>
     <row r="181">
@@ -9407,52 +9407,52 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="10" t="inlineStr">
+      <c r="A182" s="2" t="inlineStr">
         <is>
           <t>THIRUVAIYARU</t>
         </is>
       </c>
-      <c r="B182" s="10" t="n">
+      <c r="B182" s="3" t="n">
         <v>173</v>
       </c>
-      <c r="C182" s="10" t="inlineStr">
+      <c r="C182" s="3" t="inlineStr">
         <is>
           <t>DURAI. CHANDRASEKARAN</t>
         </is>
       </c>
-      <c r="D182" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E182" s="10" t="inlineStr">
+      <c r="D182" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E182" s="3" t="inlineStr">
         <is>
           <t>MATHI. MANIKANDAN</t>
         </is>
       </c>
-      <c r="F182" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G182" s="11" t="n">
-        <v>6741</v>
-      </c>
-      <c r="H182" s="10" t="inlineStr">
-        <is>
-          <t>18/25</t>
-        </is>
-      </c>
-      <c r="I182" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J182" s="11" t="n">
-        <v>9362</v>
-      </c>
-      <c r="K182" s="12" t="n">
-        <v>374.5</v>
+      <c r="F182" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G182" s="4" t="n">
+        <v>6731</v>
+      </c>
+      <c r="H182" s="3" t="inlineStr">
+        <is>
+          <t>19/25</t>
+        </is>
+      </c>
+      <c r="I182" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J182" s="4" t="n">
+        <v>8857</v>
+      </c>
+      <c r="K182" s="5" t="n">
+        <v>354.2631578947368</v>
       </c>
     </row>
     <row r="183">
@@ -9583,11 +9583,11 @@
         </is>
       </c>
       <c r="G185" s="4" t="n">
-        <v>7151</v>
+        <v>7542</v>
       </c>
       <c r="H185" s="3" t="inlineStr">
         <is>
-          <t>19/23</t>
+          <t>20/23</t>
         </is>
       </c>
       <c r="I185" s="3" t="inlineStr">
@@ -9596,10 +9596,10 @@
         </is>
       </c>
       <c r="J185" s="4" t="n">
-        <v>8656</v>
+        <v>8673</v>
       </c>
       <c r="K185" s="5" t="n">
-        <v>376.3684210526316</v>
+        <v>377.1</v>
       </c>
     </row>
     <row r="186">
@@ -9632,23 +9632,23 @@
         </is>
       </c>
       <c r="G186" s="4" t="n">
-        <v>14012</v>
+        <v>14116</v>
       </c>
       <c r="H186" s="3" t="inlineStr">
         <is>
-          <t>23/25</t>
+          <t>25/25</t>
         </is>
       </c>
       <c r="I186" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J186" s="4" t="n">
-        <v>15230</v>
+        <v>14116</v>
       </c>
       <c r="K186" s="5" t="n">
-        <v>609.2173913043479</v>
+        <v>564.64</v>
       </c>
     </row>
     <row r="187">
@@ -9681,11 +9681,11 @@
         </is>
       </c>
       <c r="G187" s="4" t="n">
-        <v>53294</v>
+        <v>53337</v>
       </c>
       <c r="H187" s="3" t="inlineStr">
         <is>
-          <t>25/25</t>
+          <t>26/27</t>
         </is>
       </c>
       <c r="I187" s="3" t="inlineStr">
@@ -9694,10 +9694,10 @@
         </is>
       </c>
       <c r="J187" s="4" t="n">
-        <v>53294</v>
+        <v>55388</v>
       </c>
       <c r="K187" s="5" t="n">
-        <v>2131.76</v>
+        <v>2051.423076923077</v>
       </c>
     </row>
     <row r="188">
@@ -9779,11 +9779,11 @@
         </is>
       </c>
       <c r="G189" s="4" t="n">
-        <v>12216</v>
+        <v>13650</v>
       </c>
       <c r="H189" s="3" t="inlineStr">
         <is>
-          <t>21/27</t>
+          <t>23/27</t>
         </is>
       </c>
       <c r="I189" s="3" t="inlineStr">
@@ -9792,10 +9792,10 @@
         </is>
       </c>
       <c r="J189" s="4" t="n">
-        <v>15706</v>
+        <v>16024</v>
       </c>
       <c r="K189" s="5" t="n">
-        <v>581.7142857142857</v>
+        <v>593.4782608695652</v>
       </c>
     </row>
     <row r="190">
@@ -9886,7 +9886,7 @@
       </c>
       <c r="I191" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J191" s="4" t="n">
@@ -9935,7 +9935,7 @@
       </c>
       <c r="I192" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J192" s="4" t="n">
@@ -9946,52 +9946,52 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="13" t="inlineStr">
+      <c r="A193" s="6" t="inlineStr">
         <is>
           <t>TINDIVANAM</t>
         </is>
       </c>
-      <c r="B193" s="14" t="n">
+      <c r="B193" s="7" t="n">
         <v>72</v>
       </c>
-      <c r="C193" s="14" t="inlineStr">
+      <c r="C193" s="7" t="inlineStr">
+        <is>
+          <t>ARJUNAN. P</t>
+        </is>
+      </c>
+      <c r="D193" s="7" t="inlineStr">
+        <is>
+          <t>All India Anna Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E193" s="7" t="inlineStr">
         <is>
           <t>VANNI ARASU</t>
         </is>
       </c>
-      <c r="D193" s="14" t="inlineStr">
+      <c r="F193" s="7" t="inlineStr">
         <is>
           <t>Viduthalai Chiruthaigal Katchi</t>
         </is>
       </c>
-      <c r="E193" s="14" t="inlineStr">
-        <is>
-          <t>ARJUNAN. P</t>
-        </is>
-      </c>
-      <c r="F193" s="14" t="inlineStr">
-        <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G193" s="15" t="n">
-        <v>27</v>
-      </c>
-      <c r="H193" s="14" t="inlineStr">
-        <is>
-          <t>19/23</t>
-        </is>
-      </c>
-      <c r="I193" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J193" s="15" t="n">
-        <v>33</v>
-      </c>
-      <c r="K193" s="16" t="n">
-        <v>1.421052631578947</v>
+      <c r="G193" s="8" t="n">
+        <v>516</v>
+      </c>
+      <c r="H193" s="7" t="inlineStr">
+        <is>
+          <t>20/23</t>
+        </is>
+      </c>
+      <c r="I193" s="7" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J193" s="8" t="n">
+        <v>593</v>
+      </c>
+      <c r="K193" s="9" t="n">
+        <v>25.8</v>
       </c>
     </row>
     <row r="194">
@@ -10033,7 +10033,7 @@
       </c>
       <c r="I194" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J194" s="4" t="n">
@@ -10073,11 +10073,11 @@
         </is>
       </c>
       <c r="G195" s="4" t="n">
-        <v>24828</v>
+        <v>25962</v>
       </c>
       <c r="H195" s="3" t="inlineStr">
         <is>
-          <t>18/21</t>
+          <t>19/22</t>
         </is>
       </c>
       <c r="I195" s="3" t="inlineStr">
@@ -10086,10 +10086,10 @@
         </is>
       </c>
       <c r="J195" s="4" t="n">
-        <v>28966</v>
+        <v>30061</v>
       </c>
       <c r="K195" s="5" t="n">
-        <v>1379.333333333333</v>
+        <v>1366.421052631579</v>
       </c>
     </row>
     <row r="196">
@@ -10122,11 +10122,11 @@
         </is>
       </c>
       <c r="G196" s="4" t="n">
-        <v>20808</v>
+        <v>22092</v>
       </c>
       <c r="H196" s="3" t="inlineStr">
         <is>
-          <t>16/22</t>
+          <t>17/22</t>
         </is>
       </c>
       <c r="I196" s="3" t="inlineStr">
@@ -10135,10 +10135,10 @@
         </is>
       </c>
       <c r="J196" s="4" t="n">
-        <v>28611</v>
+        <v>28590</v>
       </c>
       <c r="K196" s="5" t="n">
-        <v>1300.5</v>
+        <v>1299.529411764706</v>
       </c>
     </row>
     <row r="197">
@@ -10220,11 +10220,11 @@
         </is>
       </c>
       <c r="G198" s="4" t="n">
-        <v>10172</v>
+        <v>10257</v>
       </c>
       <c r="H198" s="3" t="inlineStr">
         <is>
-          <t>16/21</t>
+          <t>17/21</t>
         </is>
       </c>
       <c r="I198" s="3" t="inlineStr">
@@ -10233,59 +10233,59 @@
         </is>
       </c>
       <c r="J198" s="4" t="n">
-        <v>13351</v>
+        <v>12670</v>
       </c>
       <c r="K198" s="5" t="n">
-        <v>635.75</v>
+        <v>603.3529411764706</v>
       </c>
     </row>
     <row r="199">
-      <c r="A199" s="6" t="inlineStr">
+      <c r="A199" s="13" t="inlineStr">
         <is>
           <t>TIRUKKOYILUR</t>
         </is>
       </c>
-      <c r="B199" s="7" t="n">
+      <c r="B199" s="14" t="n">
         <v>76</v>
       </c>
-      <c r="C199" s="7" t="inlineStr">
+      <c r="C199" s="14" t="inlineStr">
         <is>
           <t>VIJAY R BARANIBALAAJI</t>
         </is>
       </c>
-      <c r="D199" s="7" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E199" s="7" t="inlineStr">
+      <c r="D199" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E199" s="14" t="inlineStr">
         <is>
           <t>PALANISAMY S</t>
         </is>
       </c>
-      <c r="F199" s="7" t="inlineStr">
+      <c r="F199" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G199" s="8" t="n">
-        <v>497</v>
-      </c>
-      <c r="H199" s="7" t="inlineStr">
-        <is>
-          <t>21/24</t>
-        </is>
-      </c>
-      <c r="I199" s="7" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J199" s="8" t="n">
-        <v>568</v>
-      </c>
-      <c r="K199" s="9" t="n">
-        <v>23.66666666666667</v>
+      <c r="G199" s="15" t="n">
+        <v>254</v>
+      </c>
+      <c r="H199" s="14" t="inlineStr">
+        <is>
+          <t>22/24</t>
+        </is>
+      </c>
+      <c r="I199" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J199" s="15" t="n">
+        <v>277</v>
+      </c>
+      <c r="K199" s="16" t="n">
+        <v>11.54545454545454</v>
       </c>
     </row>
     <row r="200">
@@ -10367,11 +10367,11 @@
         </is>
       </c>
       <c r="G201" s="4" t="n">
-        <v>38524</v>
+        <v>42858</v>
       </c>
       <c r="H201" s="3" t="inlineStr">
         <is>
-          <t>17/22</t>
+          <t>19/22</t>
         </is>
       </c>
       <c r="I201" s="3" t="inlineStr">
@@ -10380,10 +10380,10 @@
         </is>
       </c>
       <c r="J201" s="4" t="n">
-        <v>49855</v>
+        <v>49625</v>
       </c>
       <c r="K201" s="5" t="n">
-        <v>2266.117647058823</v>
+        <v>2255.684210526316</v>
       </c>
     </row>
     <row r="202">
@@ -10416,11 +10416,11 @@
         </is>
       </c>
       <c r="G202" s="11" t="n">
-        <v>2907</v>
+        <v>2610</v>
       </c>
       <c r="H202" s="10" t="inlineStr">
         <is>
-          <t>20/27</t>
+          <t>22/27</t>
         </is>
       </c>
       <c r="I202" s="10" t="inlineStr">
@@ -10429,10 +10429,10 @@
         </is>
       </c>
       <c r="J202" s="11" t="n">
-        <v>3924</v>
+        <v>3203</v>
       </c>
       <c r="K202" s="12" t="n">
-        <v>145.35</v>
+        <v>118.6363636363636</v>
       </c>
     </row>
     <row r="203">
@@ -10465,11 +10465,11 @@
         </is>
       </c>
       <c r="G203" s="4" t="n">
-        <v>53481</v>
+        <v>57599</v>
       </c>
       <c r="H203" s="3" t="inlineStr">
         <is>
-          <t>24/32</t>
+          <t>26/32</t>
         </is>
       </c>
       <c r="I203" s="3" t="inlineStr">
@@ -10478,10 +10478,10 @@
         </is>
       </c>
       <c r="J203" s="4" t="n">
-        <v>71308</v>
+        <v>70891</v>
       </c>
       <c r="K203" s="5" t="n">
-        <v>2228.375</v>
+        <v>2215.346153846154</v>
       </c>
     </row>
     <row r="204">
@@ -10514,11 +10514,11 @@
         </is>
       </c>
       <c r="G204" s="4" t="n">
-        <v>9955</v>
+        <v>10748</v>
       </c>
       <c r="H204" s="3" t="inlineStr">
         <is>
-          <t>18/21</t>
+          <t>19/21</t>
         </is>
       </c>
       <c r="I204" s="3" t="inlineStr">
@@ -10527,10 +10527,10 @@
         </is>
       </c>
       <c r="J204" s="4" t="n">
-        <v>11614</v>
+        <v>11879</v>
       </c>
       <c r="K204" s="5" t="n">
-        <v>553.0555555555555</v>
+        <v>565.6842105263158</v>
       </c>
     </row>
     <row r="205">
@@ -10661,11 +10661,11 @@
         </is>
       </c>
       <c r="G207" s="8" t="n">
-        <v>1139</v>
+        <v>402</v>
       </c>
       <c r="H207" s="7" t="inlineStr">
         <is>
-          <t>15/23</t>
+          <t>16/23</t>
         </is>
       </c>
       <c r="I207" s="7" t="inlineStr">
@@ -10674,10 +10674,10 @@
         </is>
       </c>
       <c r="J207" s="8" t="n">
-        <v>1746</v>
+        <v>578</v>
       </c>
       <c r="K207" s="9" t="n">
-        <v>75.93333333333334</v>
+        <v>25.125</v>
       </c>
     </row>
     <row r="208">
@@ -10710,11 +10710,11 @@
         </is>
       </c>
       <c r="G208" s="8" t="n">
-        <v>1416</v>
+        <v>1445</v>
       </c>
       <c r="H208" s="7" t="inlineStr">
         <is>
-          <t>17/20</t>
+          <t>18/20</t>
         </is>
       </c>
       <c r="I208" s="7" t="inlineStr">
@@ -10723,10 +10723,10 @@
         </is>
       </c>
       <c r="J208" s="8" t="n">
-        <v>1666</v>
+        <v>1606</v>
       </c>
       <c r="K208" s="9" t="n">
-        <v>83.29411764705883</v>
+        <v>80.27777777777777</v>
       </c>
     </row>
     <row r="209">
@@ -10877,52 +10877,52 @@
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="10" t="inlineStr">
+      <c r="A212" s="6" t="inlineStr">
         <is>
           <t>USILAMPATTI</t>
         </is>
       </c>
-      <c r="B212" s="10" t="n">
+      <c r="B212" s="7" t="n">
         <v>197</v>
       </c>
-      <c r="C212" s="10" t="inlineStr">
+      <c r="C212" s="7" t="inlineStr">
         <is>
           <t>VIJAY. M</t>
         </is>
       </c>
-      <c r="D212" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E212" s="10" t="inlineStr">
+      <c r="D212" s="7" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E212" s="7" t="inlineStr">
         <is>
           <t>MAHENDRAN. I</t>
         </is>
       </c>
-      <c r="F212" s="10" t="inlineStr">
+      <c r="F212" s="7" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G212" s="11" t="n">
-        <v>2553</v>
-      </c>
-      <c r="H212" s="10" t="inlineStr">
-        <is>
-          <t>18/25</t>
-        </is>
-      </c>
-      <c r="I212" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J212" s="11" t="n">
-        <v>3546</v>
-      </c>
-      <c r="K212" s="12" t="n">
-        <v>141.8333333333333</v>
+      <c r="G212" s="8" t="n">
+        <v>2029</v>
+      </c>
+      <c r="H212" s="7" t="inlineStr">
+        <is>
+          <t>20/25</t>
+        </is>
+      </c>
+      <c r="I212" s="7" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J212" s="8" t="n">
+        <v>2536</v>
+      </c>
+      <c r="K212" s="9" t="n">
+        <v>101.45</v>
       </c>
     </row>
     <row r="213">
@@ -11013,7 +11013,7 @@
       </c>
       <c r="I214" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J214" s="4" t="n">
@@ -11200,11 +11200,11 @@
         </is>
       </c>
       <c r="G218" s="4" t="n">
-        <v>6457</v>
+        <v>6967</v>
       </c>
       <c r="H218" s="3" t="inlineStr">
         <is>
-          <t>21/23</t>
+          <t>22/23</t>
         </is>
       </c>
       <c r="I218" s="3" t="inlineStr">
@@ -11213,10 +11213,10 @@
         </is>
       </c>
       <c r="J218" s="4" t="n">
-        <v>7072</v>
+        <v>7284</v>
       </c>
       <c r="K218" s="5" t="n">
-        <v>307.4761904761905</v>
+        <v>316.6818181818182</v>
       </c>
     </row>
     <row r="219">
@@ -11347,11 +11347,11 @@
         </is>
       </c>
       <c r="G221" s="4" t="n">
-        <v>10142</v>
+        <v>9814</v>
       </c>
       <c r="H221" s="3" t="inlineStr">
         <is>
-          <t>22/24</t>
+          <t>24/27</t>
         </is>
       </c>
       <c r="I221" s="3" t="inlineStr">
@@ -11360,10 +11360,10 @@
         </is>
       </c>
       <c r="J221" s="4" t="n">
-        <v>11064</v>
+        <v>11041</v>
       </c>
       <c r="K221" s="5" t="n">
-        <v>461</v>
+        <v>408.9166666666667</v>
       </c>
     </row>
     <row r="222">
@@ -11396,11 +11396,11 @@
         </is>
       </c>
       <c r="G222" s="11" t="n">
-        <v>4793</v>
+        <v>4236</v>
       </c>
       <c r="H222" s="10" t="inlineStr">
         <is>
-          <t>21/23</t>
+          <t>22/23</t>
         </is>
       </c>
       <c r="I222" s="10" t="inlineStr">
@@ -11409,10 +11409,10 @@
         </is>
       </c>
       <c r="J222" s="11" t="n">
-        <v>5249</v>
+        <v>4429</v>
       </c>
       <c r="K222" s="12" t="n">
-        <v>228.2380952380952</v>
+        <v>192.5454545454545</v>
       </c>
     </row>
     <row r="223">
@@ -11454,7 +11454,7 @@
       </c>
       <c r="I223" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J223" s="4" t="n">
@@ -11592,11 +11592,11 @@
         </is>
       </c>
       <c r="G226" s="11" t="n">
-        <v>2950</v>
+        <v>4004</v>
       </c>
       <c r="H226" s="10" t="inlineStr">
         <is>
-          <t>16/23</t>
+          <t>17/23</t>
         </is>
       </c>
       <c r="I226" s="10" t="inlineStr">
@@ -11605,10 +11605,10 @@
         </is>
       </c>
       <c r="J226" s="11" t="n">
-        <v>4241</v>
+        <v>5417</v>
       </c>
       <c r="K226" s="12" t="n">
-        <v>184.375</v>
+        <v>235.5294117647059</v>
       </c>
     </row>
     <row r="227">
@@ -11690,11 +11690,11 @@
         </is>
       </c>
       <c r="G228" s="4" t="n">
-        <v>20762</v>
+        <v>20970</v>
       </c>
       <c r="H228" s="3" t="inlineStr">
         <is>
-          <t>21/22</t>
+          <t>22/22</t>
         </is>
       </c>
       <c r="I228" s="3" t="inlineStr">
@@ -11703,10 +11703,10 @@
         </is>
       </c>
       <c r="J228" s="4" t="n">
-        <v>21751</v>
+        <v>20970</v>
       </c>
       <c r="K228" s="5" t="n">
-        <v>988.6666666666666</v>
+        <v>953.1818181818181</v>
       </c>
     </row>
     <row r="229">
@@ -11748,7 +11748,7 @@
       </c>
       <c r="I229" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J229" s="4" t="n">
@@ -11788,11 +11788,11 @@
         </is>
       </c>
       <c r="G230" s="11" t="n">
-        <v>4027</v>
+        <v>4119</v>
       </c>
       <c r="H230" s="10" t="inlineStr">
         <is>
-          <t>23/24</t>
+          <t>24/24</t>
         </is>
       </c>
       <c r="I230" s="10" t="inlineStr">
@@ -11801,10 +11801,10 @@
         </is>
       </c>
       <c r="J230" s="11" t="n">
-        <v>4202</v>
+        <v>4119</v>
       </c>
       <c r="K230" s="12" t="n">
-        <v>175.0869565217391</v>
+        <v>171.625</v>
       </c>
     </row>
     <row r="231">
@@ -11886,7 +11886,7 @@
         </is>
       </c>
       <c r="G232" s="4" t="n">
-        <v>9874</v>
+        <v>9884</v>
       </c>
       <c r="H232" s="3" t="inlineStr">
         <is>
@@ -11899,10 +11899,10 @@
         </is>
       </c>
       <c r="J232" s="4" t="n">
-        <v>11953</v>
+        <v>11965</v>
       </c>
       <c r="K232" s="5" t="n">
-        <v>519.6842105263158</v>
+        <v>520.2105263157895</v>
       </c>
     </row>
     <row r="233">
@@ -11935,11 +11935,11 @@
         </is>
       </c>
       <c r="G233" s="4" t="n">
-        <v>20432</v>
+        <v>21468</v>
       </c>
       <c r="H233" s="3" t="inlineStr">
         <is>
-          <t>17/23</t>
+          <t>18/23</t>
         </is>
       </c>
       <c r="I233" s="3" t="inlineStr">
@@ -11948,10 +11948,10 @@
         </is>
       </c>
       <c r="J233" s="4" t="n">
-        <v>27643</v>
+        <v>27431</v>
       </c>
       <c r="K233" s="5" t="n">
-        <v>1201.882352941177</v>
+        <v>1192.666666666667</v>
       </c>
     </row>
     <row r="234">
@@ -11984,11 +11984,11 @@
         </is>
       </c>
       <c r="G234" s="8" t="n">
-        <v>1524</v>
+        <v>2387</v>
       </c>
       <c r="H234" s="7" t="inlineStr">
         <is>
-          <t>22/24</t>
+          <t>24/24</t>
         </is>
       </c>
       <c r="I234" s="7" t="inlineStr">
@@ -11997,59 +11997,59 @@
         </is>
       </c>
       <c r="J234" s="8" t="n">
-        <v>1663</v>
+        <v>2387</v>
       </c>
       <c r="K234" s="9" t="n">
-        <v>69.27272727272727</v>
+        <v>99.45833333333333</v>
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="10" t="inlineStr">
+      <c r="A235" s="6" t="inlineStr">
         <is>
           <t>YERCAUD</t>
         </is>
       </c>
-      <c r="B235" s="10" t="n">
+      <c r="B235" s="7" t="n">
         <v>83</v>
       </c>
-      <c r="C235" s="10" t="inlineStr">
+      <c r="C235" s="7" t="inlineStr">
         <is>
           <t>LAKSHMI JANARTHANAN. J</t>
         </is>
       </c>
-      <c r="D235" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E235" s="10" t="inlineStr">
+      <c r="D235" s="7" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E235" s="7" t="inlineStr">
         <is>
           <t>USHARANI. P</t>
         </is>
       </c>
-      <c r="F235" s="10" t="inlineStr">
+      <c r="F235" s="7" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G235" s="11" t="n">
-        <v>2995</v>
-      </c>
-      <c r="H235" s="10" t="inlineStr">
-        <is>
-          <t>19/24</t>
-        </is>
-      </c>
-      <c r="I235" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J235" s="11" t="n">
-        <v>3783</v>
-      </c>
-      <c r="K235" s="12" t="n">
-        <v>157.6315789473684</v>
+      <c r="G235" s="8" t="n">
+        <v>2079</v>
+      </c>
+      <c r="H235" s="7" t="inlineStr">
+        <is>
+          <t>21/24</t>
+        </is>
+      </c>
+      <c r="I235" s="7" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J235" s="8" t="n">
+        <v>2376</v>
+      </c>
+      <c r="K235" s="9" t="n">
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Election snapshot: 92.5% counted — TVK 108, DMK 61, AIADMK 44, 60 declared
TINDIVANAM flipped AIADMK→VCK; THIRUMAYAM still 3-vote DMK lead (19/22 rounds).

https://claude.ai/code/session_01MizbUy44JG5sXyvaf3Wekb
</commit_message>
<xml_diff>
--- a/tn_election_results_may2026.xlsx
+++ b/tn_election_results_may2026.xlsx
@@ -616,11 +616,11 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>23883</v>
+        <v>23196</v>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>21/31</t>
+          <t>22/31</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -629,10 +629,10 @@
         </is>
       </c>
       <c r="J2" s="4" t="n">
-        <v>35256</v>
+        <v>32685</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>1137.285714285714</v>
+        <v>1054.363636363636</v>
       </c>
     </row>
     <row r="3">
@@ -1507,7 +1507,7 @@
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J20" s="4" t="n">
@@ -1792,7 +1792,7 @@
         </is>
       </c>
       <c r="G26" s="4" t="n">
-        <v>5222</v>
+        <v>5301</v>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
@@ -1805,10 +1805,10 @@
         </is>
       </c>
       <c r="J26" s="4" t="n">
-        <v>5744</v>
+        <v>5831</v>
       </c>
       <c r="K26" s="5" t="n">
-        <v>261.1</v>
+        <v>265.05</v>
       </c>
     </row>
     <row r="27">
@@ -1939,11 +1939,11 @@
         </is>
       </c>
       <c r="G29" s="4" t="n">
-        <v>13027</v>
+        <v>13581</v>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>20/25</t>
+          <t>21/25</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
@@ -1952,10 +1952,10 @@
         </is>
       </c>
       <c r="J29" s="4" t="n">
-        <v>16284</v>
+        <v>16168</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>651.35</v>
+        <v>646.7142857142857</v>
       </c>
     </row>
     <row r="30">
@@ -2184,11 +2184,11 @@
         </is>
       </c>
       <c r="G34" s="4" t="n">
-        <v>17084</v>
+        <v>18183</v>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>20/25</t>
+          <t>21/25</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
@@ -2197,10 +2197,10 @@
         </is>
       </c>
       <c r="J34" s="4" t="n">
-        <v>21355</v>
+        <v>21646</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>854.2</v>
+        <v>865.8571428571429</v>
       </c>
     </row>
     <row r="35">
@@ -2487,7 +2487,7 @@
       </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J40" s="4" t="n">
@@ -2732,7 +2732,7 @@
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J45" s="4" t="n">
@@ -2968,11 +2968,11 @@
         </is>
       </c>
       <c r="G50" s="11" t="n">
-        <v>11061</v>
+        <v>11377</v>
       </c>
       <c r="H50" s="10" t="inlineStr">
         <is>
-          <t>15/23</t>
+          <t>16/23</t>
         </is>
       </c>
       <c r="I50" s="10" t="inlineStr">
@@ -2981,10 +2981,10 @@
         </is>
       </c>
       <c r="J50" s="11" t="n">
-        <v>16960</v>
+        <v>16354</v>
       </c>
       <c r="K50" s="12" t="n">
-        <v>737.4</v>
+        <v>711.0625</v>
       </c>
     </row>
     <row r="51">
@@ -3164,11 +3164,11 @@
         </is>
       </c>
       <c r="G54" s="4" t="n">
-        <v>27495</v>
+        <v>27942</v>
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>23/26</t>
+          <t>24/26</t>
         </is>
       </c>
       <c r="I54" s="3" t="inlineStr">
@@ -3177,10 +3177,10 @@
         </is>
       </c>
       <c r="J54" s="4" t="n">
-        <v>31081</v>
+        <v>30270</v>
       </c>
       <c r="K54" s="5" t="n">
-        <v>1195.434782608696</v>
+        <v>1164.25</v>
       </c>
     </row>
     <row r="55">
@@ -3311,11 +3311,11 @@
         </is>
       </c>
       <c r="G57" s="4" t="n">
-        <v>20706</v>
+        <v>22077</v>
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>28/32</t>
+          <t>29/32</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr">
@@ -3324,10 +3324,10 @@
         </is>
       </c>
       <c r="J57" s="4" t="n">
-        <v>23664</v>
+        <v>24361</v>
       </c>
       <c r="K57" s="5" t="n">
-        <v>739.5</v>
+        <v>761.2758620689655</v>
       </c>
     </row>
     <row r="58">
@@ -3752,11 +3752,11 @@
         </is>
       </c>
       <c r="G66" s="4" t="n">
-        <v>36512</v>
+        <v>38439</v>
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>21/28</t>
+          <t>22/28</t>
         </is>
       </c>
       <c r="I66" s="3" t="inlineStr">
@@ -3765,10 +3765,10 @@
         </is>
       </c>
       <c r="J66" s="4" t="n">
-        <v>48683</v>
+        <v>48922</v>
       </c>
       <c r="K66" s="5" t="n">
-        <v>1738.666666666667</v>
+        <v>1747.227272727273</v>
       </c>
     </row>
     <row r="67">
@@ -5084,7 +5084,7 @@
       </c>
       <c r="I93" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J93" s="4" t="n">
@@ -5124,11 +5124,11 @@
         </is>
       </c>
       <c r="G94" s="4" t="n">
-        <v>56298</v>
+        <v>58691</v>
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
-          <t>21/25</t>
+          <t>22/25</t>
         </is>
       </c>
       <c r="I94" s="3" t="inlineStr">
@@ -5137,10 +5137,10 @@
         </is>
       </c>
       <c r="J94" s="4" t="n">
-        <v>67021</v>
+        <v>66694</v>
       </c>
       <c r="K94" s="5" t="n">
-        <v>2680.857142857143</v>
+        <v>2667.772727272727</v>
       </c>
     </row>
     <row r="95">
@@ -5418,11 +5418,11 @@
         </is>
       </c>
       <c r="G100" s="4" t="n">
-        <v>10694</v>
+        <v>10845</v>
       </c>
       <c r="H100" s="3" t="inlineStr">
         <is>
-          <t>21/22</t>
+          <t>22/22</t>
         </is>
       </c>
       <c r="I100" s="3" t="inlineStr">
@@ -5431,10 +5431,10 @@
         </is>
       </c>
       <c r="J100" s="4" t="n">
-        <v>11203</v>
+        <v>10845</v>
       </c>
       <c r="K100" s="5" t="n">
-        <v>509.2380952380952</v>
+        <v>492.9545454545454</v>
       </c>
     </row>
     <row r="101">
@@ -5663,11 +5663,11 @@
         </is>
       </c>
       <c r="G105" s="4" t="n">
-        <v>17050</v>
+        <v>16527</v>
       </c>
       <c r="H105" s="3" t="inlineStr">
         <is>
-          <t>29/32</t>
+          <t>30/32</t>
         </is>
       </c>
       <c r="I105" s="3" t="inlineStr">
@@ -5676,10 +5676,10 @@
         </is>
       </c>
       <c r="J105" s="4" t="n">
-        <v>18814</v>
+        <v>17629</v>
       </c>
       <c r="K105" s="5" t="n">
-        <v>587.9310344827586</v>
+        <v>550.9</v>
       </c>
     </row>
     <row r="106">
@@ -6349,7 +6349,7 @@
         </is>
       </c>
       <c r="G119" s="4" t="n">
-        <v>25783</v>
+        <v>26232</v>
       </c>
       <c r="H119" s="3" t="inlineStr">
         <is>
@@ -6362,10 +6362,10 @@
         </is>
       </c>
       <c r="J119" s="4" t="n">
-        <v>28239</v>
+        <v>28730</v>
       </c>
       <c r="K119" s="5" t="n">
-        <v>1227.761904761905</v>
+        <v>1249.142857142857</v>
       </c>
     </row>
     <row r="120">
@@ -6937,7 +6937,7 @@
         </is>
       </c>
       <c r="G131" s="4" t="n">
-        <v>8035</v>
+        <v>8454</v>
       </c>
       <c r="H131" s="3" t="inlineStr">
         <is>
@@ -6950,10 +6950,10 @@
         </is>
       </c>
       <c r="J131" s="4" t="n">
-        <v>8800</v>
+        <v>9259</v>
       </c>
       <c r="K131" s="5" t="n">
-        <v>382.6190476190476</v>
+        <v>402.5714285714286</v>
       </c>
     </row>
     <row r="132">
@@ -7035,11 +7035,11 @@
         </is>
       </c>
       <c r="G133" s="4" t="n">
-        <v>13580</v>
+        <v>14393</v>
       </c>
       <c r="H133" s="3" t="inlineStr">
         <is>
-          <t>27/28</t>
+          <t>28/28</t>
         </is>
       </c>
       <c r="I133" s="3" t="inlineStr">
@@ -7048,10 +7048,10 @@
         </is>
       </c>
       <c r="J133" s="4" t="n">
-        <v>14083</v>
+        <v>14393</v>
       </c>
       <c r="K133" s="5" t="n">
-        <v>502.962962962963</v>
+        <v>514.0357142857143</v>
       </c>
     </row>
     <row r="134">
@@ -7084,11 +7084,11 @@
         </is>
       </c>
       <c r="G134" s="4" t="n">
-        <v>44267</v>
+        <v>46624</v>
       </c>
       <c r="H134" s="3" t="inlineStr">
         <is>
-          <t>18/22</t>
+          <t>19/22</t>
         </is>
       </c>
       <c r="I134" s="3" t="inlineStr">
@@ -7097,10 +7097,10 @@
         </is>
       </c>
       <c r="J134" s="4" t="n">
-        <v>54104</v>
+        <v>53986</v>
       </c>
       <c r="K134" s="5" t="n">
-        <v>2459.277777777778</v>
+        <v>2453.894736842105</v>
       </c>
     </row>
     <row r="135">
@@ -8603,11 +8603,11 @@
         </is>
       </c>
       <c r="G165" s="4" t="n">
-        <v>15502</v>
+        <v>15210</v>
       </c>
       <c r="H165" s="3" t="inlineStr">
         <is>
-          <t>27/29</t>
+          <t>28/29</t>
         </is>
       </c>
       <c r="I165" s="3" t="inlineStr">
@@ -8616,10 +8616,10 @@
         </is>
       </c>
       <c r="J165" s="4" t="n">
-        <v>16650</v>
+        <v>15753</v>
       </c>
       <c r="K165" s="5" t="n">
-        <v>574.1481481481482</v>
+        <v>543.2142857142857</v>
       </c>
     </row>
     <row r="166">
@@ -8652,11 +8652,11 @@
         </is>
       </c>
       <c r="G166" s="4" t="n">
-        <v>8121</v>
+        <v>9451</v>
       </c>
       <c r="H166" s="3" t="inlineStr">
         <is>
-          <t>18/21</t>
+          <t>19/21</t>
         </is>
       </c>
       <c r="I166" s="3" t="inlineStr">
@@ -8665,10 +8665,10 @@
         </is>
       </c>
       <c r="J166" s="4" t="n">
-        <v>9474</v>
+        <v>10446</v>
       </c>
       <c r="K166" s="5" t="n">
-        <v>451.1666666666667</v>
+        <v>497.421052631579</v>
       </c>
     </row>
     <row r="167">
@@ -8946,11 +8946,11 @@
         </is>
       </c>
       <c r="G172" s="4" t="n">
-        <v>35540</v>
+        <v>35773</v>
       </c>
       <c r="H172" s="3" t="inlineStr">
         <is>
-          <t>33/39</t>
+          <t>34/39</t>
         </is>
       </c>
       <c r="I172" s="3" t="inlineStr">
@@ -8959,10 +8959,10 @@
         </is>
       </c>
       <c r="J172" s="4" t="n">
-        <v>42002</v>
+        <v>41034</v>
       </c>
       <c r="K172" s="5" t="n">
-        <v>1076.969696969697</v>
+        <v>1052.14705882353</v>
       </c>
     </row>
     <row r="173">
@@ -9946,52 +9946,52 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="6" t="inlineStr">
+      <c r="A193" s="13" t="inlineStr">
         <is>
           <t>TINDIVANAM</t>
         </is>
       </c>
-      <c r="B193" s="7" t="n">
+      <c r="B193" s="14" t="n">
         <v>72</v>
       </c>
-      <c r="C193" s="7" t="inlineStr">
+      <c r="C193" s="14" t="inlineStr">
+        <is>
+          <t>VANNI ARASU</t>
+        </is>
+      </c>
+      <c r="D193" s="14" t="inlineStr">
+        <is>
+          <t>Viduthalai Chiruthaigal Katchi</t>
+        </is>
+      </c>
+      <c r="E193" s="14" t="inlineStr">
         <is>
           <t>ARJUNAN. P</t>
         </is>
       </c>
-      <c r="D193" s="7" t="inlineStr">
+      <c r="F193" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E193" s="7" t="inlineStr">
-        <is>
-          <t>VANNI ARASU</t>
-        </is>
-      </c>
-      <c r="F193" s="7" t="inlineStr">
-        <is>
-          <t>Viduthalai Chiruthaigal Katchi</t>
-        </is>
-      </c>
-      <c r="G193" s="8" t="n">
-        <v>516</v>
-      </c>
-      <c r="H193" s="7" t="inlineStr">
-        <is>
-          <t>20/23</t>
-        </is>
-      </c>
-      <c r="I193" s="7" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J193" s="8" t="n">
-        <v>593</v>
-      </c>
-      <c r="K193" s="9" t="n">
-        <v>25.8</v>
+      <c r="G193" s="15" t="n">
+        <v>349</v>
+      </c>
+      <c r="H193" s="14" t="inlineStr">
+        <is>
+          <t>21/23</t>
+        </is>
+      </c>
+      <c r="I193" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J193" s="15" t="n">
+        <v>382</v>
+      </c>
+      <c r="K193" s="16" t="n">
+        <v>16.61904761904762</v>
       </c>
     </row>
     <row r="194">
@@ -11494,11 +11494,11 @@
         </is>
       </c>
       <c r="G224" s="4" t="n">
-        <v>6689</v>
+        <v>6777</v>
       </c>
       <c r="H224" s="3" t="inlineStr">
         <is>
-          <t>21/22</t>
+          <t>22/22</t>
         </is>
       </c>
       <c r="I224" s="3" t="inlineStr">
@@ -11507,10 +11507,10 @@
         </is>
       </c>
       <c r="J224" s="4" t="n">
-        <v>7008</v>
+        <v>6777</v>
       </c>
       <c r="K224" s="5" t="n">
-        <v>318.5238095238095</v>
+        <v>308.0454545454546</v>
       </c>
     </row>
     <row r="225">
@@ -11886,11 +11886,11 @@
         </is>
       </c>
       <c r="G232" s="4" t="n">
-        <v>9884</v>
+        <v>9288</v>
       </c>
       <c r="H232" s="3" t="inlineStr">
         <is>
-          <t>19/23</t>
+          <t>20/23</t>
         </is>
       </c>
       <c r="I232" s="3" t="inlineStr">
@@ -11899,10 +11899,10 @@
         </is>
       </c>
       <c r="J232" s="4" t="n">
-        <v>11965</v>
+        <v>10681</v>
       </c>
       <c r="K232" s="5" t="n">
-        <v>520.2105263157895</v>
+        <v>464.4</v>
       </c>
     </row>
     <row r="233">

</xml_diff>

<commit_message>
Election snapshot: 93.9% counted — 77 declared, ULUNDURPETTAI down to 72 votes
THIRUMAYAM settled (DMK 507); ULUNDURPETTAI new thriller at 72 votes (25/27 rounds).

https://claude.ai/code/session_01MizbUy44JG5sXyvaf3Wekb
</commit_message>
<xml_diff>
--- a/tn_election_results_may2026.xlsx
+++ b/tn_election_results_may2026.xlsx
@@ -616,11 +616,11 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>23196</v>
+        <v>23273</v>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>22/31</t>
+          <t>23/31</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -629,10 +629,10 @@
         </is>
       </c>
       <c r="J2" s="4" t="n">
-        <v>32685</v>
+        <v>31368</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>1054.363636363636</v>
+        <v>1011.869565217391</v>
       </c>
     </row>
     <row r="3">
@@ -674,7 +674,7 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J3" s="4" t="n">
@@ -723,7 +723,7 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J4" s="4" t="n">
@@ -812,11 +812,11 @@
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>56253</v>
+        <v>57844</v>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>25/27</t>
+          <t>27/27</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -825,10 +825,10 @@
         </is>
       </c>
       <c r="J6" s="4" t="n">
-        <v>60753</v>
+        <v>57844</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>2250.12</v>
+        <v>2142.37037037037</v>
       </c>
     </row>
     <row r="7">
@@ -861,11 +861,11 @@
         </is>
       </c>
       <c r="G7" s="4" t="n">
-        <v>10774</v>
+        <v>9443</v>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>18/22</t>
+          <t>19/22</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -874,10 +874,10 @@
         </is>
       </c>
       <c r="J7" s="4" t="n">
-        <v>13168</v>
+        <v>10934</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>598.5555555555555</v>
+        <v>497</v>
       </c>
     </row>
     <row r="8">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J12" s="4" t="n">
@@ -1155,11 +1155,11 @@
         </is>
       </c>
       <c r="G13" s="4" t="n">
-        <v>5057</v>
+        <v>5508</v>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>22/24</t>
+          <t>23/24</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
@@ -1168,10 +1168,10 @@
         </is>
       </c>
       <c r="J13" s="4" t="n">
-        <v>5517</v>
+        <v>5747</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>229.8636363636364</v>
+        <v>239.4782608695652</v>
       </c>
     </row>
     <row r="14">
@@ -1257,7 +1257,7 @@
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>20/20</t>
+          <t>20/22</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
@@ -1266,7 +1266,7 @@
         </is>
       </c>
       <c r="J15" s="4" t="n">
-        <v>19378</v>
+        <v>21316</v>
       </c>
       <c r="K15" s="5" t="n">
         <v>968.9</v>
@@ -1302,11 +1302,11 @@
         </is>
       </c>
       <c r="G16" s="4" t="n">
-        <v>33962</v>
+        <v>35995</v>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>19/23</t>
+          <t>20/23</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
@@ -1315,10 +1315,10 @@
         </is>
       </c>
       <c r="J16" s="4" t="n">
-        <v>41112</v>
+        <v>41394</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>1787.473684210526</v>
+        <v>1799.75</v>
       </c>
     </row>
     <row r="17">
@@ -1547,11 +1547,11 @@
         </is>
       </c>
       <c r="G21" s="4" t="n">
-        <v>60189</v>
+        <v>65751</v>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>21/26</t>
+          <t>22/26</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -1560,10 +1560,10 @@
         </is>
       </c>
       <c r="J21" s="4" t="n">
-        <v>74520</v>
+        <v>77706</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>2866.142857142857</v>
+        <v>2988.681818181818</v>
       </c>
     </row>
     <row r="22">
@@ -1763,52 +1763,52 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t>BHUVANAGIRI</t>
         </is>
       </c>
-      <c r="B26" s="3" t="n">
+      <c r="B26" s="10" t="n">
         <v>157</v>
       </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="C26" s="10" t="inlineStr">
         <is>
           <t>ARUNMOZHITHEVAN . A</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr">
+      <c r="D26" s="10" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="E26" s="10" t="inlineStr">
         <is>
           <t>SARAVANAN. DURAI . K</t>
         </is>
       </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="n">
-        <v>5301</v>
-      </c>
-      <c r="H26" s="3" t="inlineStr">
-        <is>
-          <t>20/22</t>
-        </is>
-      </c>
-      <c r="I26" s="3" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J26" s="4" t="n">
-        <v>5831</v>
-      </c>
-      <c r="K26" s="5" t="n">
-        <v>265.05</v>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G26" s="11" t="n">
+        <v>3966</v>
+      </c>
+      <c r="H26" s="10" t="inlineStr">
+        <is>
+          <t>21/22</t>
+        </is>
+      </c>
+      <c r="I26" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J26" s="11" t="n">
+        <v>4155</v>
+      </c>
+      <c r="K26" s="12" t="n">
+        <v>188.8571428571429</v>
       </c>
     </row>
     <row r="27">
@@ -1841,11 +1841,11 @@
         </is>
       </c>
       <c r="G27" s="4" t="n">
-        <v>5483</v>
+        <v>6023</v>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>23/25</t>
+          <t>24/25</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
@@ -1854,10 +1854,10 @@
         </is>
       </c>
       <c r="J27" s="4" t="n">
-        <v>5960</v>
+        <v>6274</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>238.3913043478261</v>
+        <v>250.9583333333333</v>
       </c>
     </row>
     <row r="28">
@@ -1939,11 +1939,11 @@
         </is>
       </c>
       <c r="G29" s="4" t="n">
-        <v>13581</v>
+        <v>14170</v>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>21/25</t>
+          <t>22/25</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
@@ -1952,10 +1952,10 @@
         </is>
       </c>
       <c r="J29" s="4" t="n">
-        <v>16168</v>
+        <v>16102</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>646.7142857142857</v>
+        <v>644.0909090909091</v>
       </c>
     </row>
     <row r="30">
@@ -2135,11 +2135,11 @@
         </is>
       </c>
       <c r="G33" s="4" t="n">
-        <v>7503</v>
+        <v>6339</v>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>19/22</t>
+          <t>20/22</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -2148,10 +2148,10 @@
         </is>
       </c>
       <c r="J33" s="4" t="n">
-        <v>8688</v>
+        <v>6973</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>394.8947368421053</v>
+        <v>316.95</v>
       </c>
     </row>
     <row r="34">
@@ -2184,11 +2184,11 @@
         </is>
       </c>
       <c r="G34" s="4" t="n">
-        <v>18183</v>
+        <v>19082</v>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>21/25</t>
+          <t>22/25</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
@@ -2197,10 +2197,10 @@
         </is>
       </c>
       <c r="J34" s="4" t="n">
-        <v>21646</v>
+        <v>21684</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>865.8571428571429</v>
+        <v>867.3636363636364</v>
       </c>
     </row>
     <row r="35">
@@ -2282,11 +2282,11 @@
         </is>
       </c>
       <c r="G36" s="8" t="n">
-        <v>2435</v>
+        <v>2499</v>
       </c>
       <c r="H36" s="7" t="inlineStr">
         <is>
-          <t>20/23</t>
+          <t>21/23</t>
         </is>
       </c>
       <c r="I36" s="7" t="inlineStr">
@@ -2295,10 +2295,10 @@
         </is>
       </c>
       <c r="J36" s="8" t="n">
-        <v>2800</v>
+        <v>2737</v>
       </c>
       <c r="K36" s="9" t="n">
-        <v>121.75</v>
+        <v>119</v>
       </c>
     </row>
     <row r="37">
@@ -2380,11 +2380,11 @@
         </is>
       </c>
       <c r="G38" s="4" t="n">
-        <v>14394</v>
+        <v>15400</v>
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>17/19</t>
+          <t>18/20</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
@@ -2393,59 +2393,59 @@
         </is>
       </c>
       <c r="J38" s="4" t="n">
-        <v>16087</v>
+        <v>17111</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>846.7058823529412</v>
+        <v>855.5555555555555</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="10" t="inlineStr">
+      <c r="A39" s="6" t="inlineStr">
         <is>
           <t>CUMBUM</t>
         </is>
       </c>
-      <c r="B39" s="10" t="n">
+      <c r="B39" s="7" t="n">
         <v>201</v>
       </c>
-      <c r="C39" s="10" t="inlineStr">
+      <c r="C39" s="7" t="inlineStr">
         <is>
           <t>ERAMAKRISHNAN N</t>
         </is>
       </c>
-      <c r="D39" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E39" s="10" t="inlineStr">
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
         <is>
           <t>JEGANATHMISHRA PLA</t>
         </is>
       </c>
-      <c r="F39" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G39" s="11" t="n">
-        <v>3354</v>
-      </c>
-      <c r="H39" s="10" t="inlineStr">
-        <is>
-          <t>20/25</t>
-        </is>
-      </c>
-      <c r="I39" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J39" s="11" t="n">
-        <v>4192</v>
-      </c>
-      <c r="K39" s="12" t="n">
-        <v>167.7</v>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="n">
+        <v>548</v>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>22/25</t>
+        </is>
+      </c>
+      <c r="I39" s="7" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J39" s="8" t="n">
+        <v>623</v>
+      </c>
+      <c r="K39" s="9" t="n">
+        <v>24.90909090909091</v>
       </c>
     </row>
     <row r="40">
@@ -2625,11 +2625,11 @@
         </is>
       </c>
       <c r="G43" s="4" t="n">
-        <v>42664</v>
+        <v>45324</v>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>15/18</t>
+          <t>16/18</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
@@ -2638,10 +2638,10 @@
         </is>
       </c>
       <c r="J43" s="4" t="n">
-        <v>51197</v>
+        <v>50990</v>
       </c>
       <c r="K43" s="5" t="n">
-        <v>2844.266666666667</v>
+        <v>2832.75</v>
       </c>
     </row>
     <row r="44">
@@ -2919,11 +2919,11 @@
         </is>
       </c>
       <c r="G49" s="4" t="n">
-        <v>14141</v>
+        <v>14168</v>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>20/22</t>
+          <t>21/22</t>
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr">
@@ -2932,10 +2932,10 @@
         </is>
       </c>
       <c r="J49" s="4" t="n">
-        <v>15555</v>
+        <v>14843</v>
       </c>
       <c r="K49" s="5" t="n">
-        <v>707.05</v>
+        <v>674.6666666666666</v>
       </c>
     </row>
     <row r="50">
@@ -3164,11 +3164,11 @@
         </is>
       </c>
       <c r="G54" s="4" t="n">
-        <v>27942</v>
+        <v>27906</v>
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>24/26</t>
+          <t>25/26</t>
         </is>
       </c>
       <c r="I54" s="3" t="inlineStr">
@@ -3177,10 +3177,10 @@
         </is>
       </c>
       <c r="J54" s="4" t="n">
-        <v>30270</v>
+        <v>29022</v>
       </c>
       <c r="K54" s="5" t="n">
-        <v>1164.25</v>
+        <v>1116.24</v>
       </c>
     </row>
     <row r="55">
@@ -3311,11 +3311,11 @@
         </is>
       </c>
       <c r="G57" s="4" t="n">
-        <v>22077</v>
+        <v>22532</v>
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>29/32</t>
+          <t>30/32</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr">
@@ -3324,10 +3324,10 @@
         </is>
       </c>
       <c r="J57" s="4" t="n">
-        <v>24361</v>
+        <v>24034</v>
       </c>
       <c r="K57" s="5" t="n">
-        <v>761.2758620689655</v>
+        <v>751.0666666666667</v>
       </c>
     </row>
     <row r="58">
@@ -3369,7 +3369,7 @@
       </c>
       <c r="I58" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J58" s="4" t="n">
@@ -3418,7 +3418,7 @@
       </c>
       <c r="I59" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J59" s="4" t="n">
@@ -3458,11 +3458,11 @@
         </is>
       </c>
       <c r="G60" s="4" t="n">
-        <v>9745</v>
+        <v>8512</v>
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>22/26</t>
+          <t>23/26</t>
         </is>
       </c>
       <c r="I60" s="3" t="inlineStr">
@@ -3471,10 +3471,10 @@
         </is>
       </c>
       <c r="J60" s="4" t="n">
-        <v>11517</v>
+        <v>9622</v>
       </c>
       <c r="K60" s="5" t="n">
-        <v>442.9545454545454</v>
+        <v>370.0869565217391</v>
       </c>
     </row>
     <row r="61">
@@ -3507,11 +3507,11 @@
         </is>
       </c>
       <c r="G61" s="4" t="n">
-        <v>21330</v>
+        <v>21798</v>
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>18/22</t>
+          <t>19/22</t>
         </is>
       </c>
       <c r="I61" s="3" t="inlineStr">
@@ -3520,59 +3520,59 @@
         </is>
       </c>
       <c r="J61" s="4" t="n">
-        <v>26070</v>
+        <v>25240</v>
       </c>
       <c r="K61" s="5" t="n">
-        <v>1185</v>
+        <v>1147.263157894737</v>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="13" t="inlineStr">
+      <c r="A62" s="6" t="inlineStr">
         <is>
           <t>KALLAKURICHI</t>
         </is>
       </c>
-      <c r="B62" s="14" t="n">
+      <c r="B62" s="7" t="n">
         <v>80</v>
       </c>
-      <c r="C62" s="14" t="inlineStr">
+      <c r="C62" s="7" t="inlineStr">
         <is>
           <t>ARUL VIGNESH C</t>
         </is>
       </c>
-      <c r="D62" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E62" s="14" t="inlineStr">
+      <c r="D62" s="7" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="inlineStr">
         <is>
           <t>RAJEEVGANDHI S</t>
         </is>
       </c>
-      <c r="F62" s="14" t="inlineStr">
+      <c r="F62" s="7" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G62" s="15" t="n">
-        <v>467</v>
-      </c>
-      <c r="H62" s="14" t="inlineStr">
-        <is>
-          <t>26/27</t>
-        </is>
-      </c>
-      <c r="I62" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J62" s="15" t="n">
-        <v>485</v>
-      </c>
-      <c r="K62" s="16" t="n">
-        <v>17.96153846153846</v>
+      <c r="G62" s="8" t="n">
+        <v>798</v>
+      </c>
+      <c r="H62" s="7" t="inlineStr">
+        <is>
+          <t>27/27</t>
+        </is>
+      </c>
+      <c r="I62" s="7" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J62" s="8" t="n">
+        <v>798</v>
+      </c>
+      <c r="K62" s="9" t="n">
+        <v>29.55555555555556</v>
       </c>
     </row>
     <row r="63">
@@ -3605,11 +3605,11 @@
         </is>
       </c>
       <c r="G63" s="4" t="n">
-        <v>9623</v>
+        <v>11032</v>
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
-          <t>22/26</t>
+          <t>23/26</t>
         </is>
       </c>
       <c r="I63" s="3" t="inlineStr">
@@ -3618,10 +3618,10 @@
         </is>
       </c>
       <c r="J63" s="4" t="n">
-        <v>11373</v>
+        <v>12471</v>
       </c>
       <c r="K63" s="5" t="n">
-        <v>437.4090909090909</v>
+        <v>479.6521739130435</v>
       </c>
     </row>
     <row r="64">
@@ -3654,11 +3654,11 @@
         </is>
       </c>
       <c r="G64" s="4" t="n">
-        <v>7946</v>
+        <v>7420</v>
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>21/24</t>
+          <t>22/24</t>
         </is>
       </c>
       <c r="I64" s="3" t="inlineStr">
@@ -3667,10 +3667,10 @@
         </is>
       </c>
       <c r="J64" s="4" t="n">
-        <v>9081</v>
+        <v>8095</v>
       </c>
       <c r="K64" s="5" t="n">
-        <v>378.3809523809524</v>
+        <v>337.2727272727273</v>
       </c>
     </row>
     <row r="65">
@@ -3703,11 +3703,11 @@
         </is>
       </c>
       <c r="G65" s="11" t="n">
-        <v>4265</v>
+        <v>3795</v>
       </c>
       <c r="H65" s="10" t="inlineStr">
         <is>
-          <t>23/26</t>
+          <t>24/34</t>
         </is>
       </c>
       <c r="I65" s="10" t="inlineStr">
@@ -3716,10 +3716,10 @@
         </is>
       </c>
       <c r="J65" s="11" t="n">
-        <v>4821</v>
+        <v>5376</v>
       </c>
       <c r="K65" s="12" t="n">
-        <v>185.4347826086957</v>
+        <v>158.125</v>
       </c>
     </row>
     <row r="66">
@@ -3752,11 +3752,11 @@
         </is>
       </c>
       <c r="G66" s="4" t="n">
-        <v>38439</v>
+        <v>40038</v>
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>22/28</t>
+          <t>23/28</t>
         </is>
       </c>
       <c r="I66" s="3" t="inlineStr">
@@ -3765,59 +3765,59 @@
         </is>
       </c>
       <c r="J66" s="4" t="n">
-        <v>48922</v>
+        <v>48742</v>
       </c>
       <c r="K66" s="5" t="n">
-        <v>1747.227272727273</v>
+        <v>1740.782608695652</v>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="10" t="inlineStr">
+      <c r="A67" s="6" t="inlineStr">
         <is>
           <t>KARUR</t>
         </is>
       </c>
-      <c r="B67" s="10" t="n">
+      <c r="B67" s="7" t="n">
         <v>135</v>
       </c>
-      <c r="C67" s="10" t="inlineStr">
+      <c r="C67" s="7" t="inlineStr">
         <is>
           <t>M.R. VIJAYABHASKAR</t>
         </is>
       </c>
-      <c r="D67" s="10" t="inlineStr">
+      <c r="D67" s="7" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E67" s="10" t="inlineStr">
+      <c r="E67" s="7" t="inlineStr">
         <is>
           <t>MATHIYALAGAN V.P</t>
         </is>
       </c>
-      <c r="F67" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G67" s="11" t="n">
-        <v>2616</v>
-      </c>
-      <c r="H67" s="10" t="inlineStr">
-        <is>
-          <t>17/21</t>
-        </is>
-      </c>
-      <c r="I67" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J67" s="11" t="n">
-        <v>3232</v>
-      </c>
-      <c r="K67" s="12" t="n">
-        <v>153.8823529411765</v>
+      <c r="F67" s="7" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G67" s="8" t="n">
+        <v>1856</v>
+      </c>
+      <c r="H67" s="7" t="inlineStr">
+        <is>
+          <t>18/21</t>
+        </is>
+      </c>
+      <c r="I67" s="7" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J67" s="8" t="n">
+        <v>2165</v>
+      </c>
+      <c r="K67" s="9" t="n">
+        <v>103.1111111111111</v>
       </c>
     </row>
     <row r="68">
@@ -3850,11 +3850,11 @@
         </is>
       </c>
       <c r="G68" s="4" t="n">
-        <v>5146</v>
+        <v>5956</v>
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>16/20</t>
+          <t>17/20</t>
         </is>
       </c>
       <c r="I68" s="3" t="inlineStr">
@@ -3863,10 +3863,10 @@
         </is>
       </c>
       <c r="J68" s="4" t="n">
-        <v>6432</v>
+        <v>7007</v>
       </c>
       <c r="K68" s="5" t="n">
-        <v>321.625</v>
+        <v>350.3529411764706</v>
       </c>
     </row>
     <row r="69">
@@ -4046,11 +4046,11 @@
         </is>
       </c>
       <c r="G72" s="4" t="n">
-        <v>29639</v>
+        <v>30213</v>
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>20/22</t>
+          <t>21/22</t>
         </is>
       </c>
       <c r="I72" s="3" t="inlineStr">
@@ -4059,10 +4059,10 @@
         </is>
       </c>
       <c r="J72" s="4" t="n">
-        <v>32603</v>
+        <v>31652</v>
       </c>
       <c r="K72" s="5" t="n">
-        <v>1481.95</v>
+        <v>1438.714285714286</v>
       </c>
     </row>
     <row r="73">
@@ -4095,11 +4095,11 @@
         </is>
       </c>
       <c r="G73" s="4" t="n">
-        <v>17544</v>
+        <v>20255</v>
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
-          <t>17/19</t>
+          <t>19/19</t>
         </is>
       </c>
       <c r="I73" s="3" t="inlineStr">
@@ -4108,10 +4108,10 @@
         </is>
       </c>
       <c r="J73" s="4" t="n">
-        <v>19608</v>
+        <v>20255</v>
       </c>
       <c r="K73" s="5" t="n">
-        <v>1032</v>
+        <v>1066.052631578947</v>
       </c>
     </row>
     <row r="74">
@@ -4291,11 +4291,11 @@
         </is>
       </c>
       <c r="G77" s="8" t="n">
-        <v>509</v>
+        <v>962</v>
       </c>
       <c r="H77" s="7" t="inlineStr">
         <is>
-          <t>22/23</t>
+          <t>23/23</t>
         </is>
       </c>
       <c r="I77" s="7" t="inlineStr">
@@ -4304,10 +4304,10 @@
         </is>
       </c>
       <c r="J77" s="8" t="n">
-        <v>532</v>
+        <v>962</v>
       </c>
       <c r="K77" s="9" t="n">
-        <v>23.13636363636364</v>
+        <v>41.82608695652174</v>
       </c>
     </row>
     <row r="78">
@@ -4340,11 +4340,11 @@
         </is>
       </c>
       <c r="G78" s="4" t="n">
-        <v>19650</v>
+        <v>18844</v>
       </c>
       <c r="H78" s="3" t="inlineStr">
         <is>
-          <t>23/25</t>
+          <t>25/25</t>
         </is>
       </c>
       <c r="I78" s="3" t="inlineStr">
@@ -4353,10 +4353,10 @@
         </is>
       </c>
       <c r="J78" s="4" t="n">
-        <v>21359</v>
+        <v>18844</v>
       </c>
       <c r="K78" s="5" t="n">
-        <v>854.3478260869565</v>
+        <v>753.76</v>
       </c>
     </row>
     <row r="79">
@@ -4389,11 +4389,11 @@
         </is>
       </c>
       <c r="G79" s="11" t="n">
-        <v>3641</v>
+        <v>3528</v>
       </c>
       <c r="H79" s="10" t="inlineStr">
         <is>
-          <t>18/20</t>
+          <t>19/20</t>
         </is>
       </c>
       <c r="I79" s="10" t="inlineStr">
@@ -4402,10 +4402,10 @@
         </is>
       </c>
       <c r="J79" s="11" t="n">
-        <v>4046</v>
+        <v>3714</v>
       </c>
       <c r="K79" s="12" t="n">
-        <v>202.2777777777778</v>
+        <v>185.6842105263158</v>
       </c>
     </row>
     <row r="80">
@@ -4487,7 +4487,7 @@
         </is>
       </c>
       <c r="G81" s="4" t="n">
-        <v>8167</v>
+        <v>7772</v>
       </c>
       <c r="H81" s="3" t="inlineStr">
         <is>
@@ -4500,10 +4500,10 @@
         </is>
       </c>
       <c r="J81" s="4" t="n">
-        <v>8909</v>
+        <v>8479</v>
       </c>
       <c r="K81" s="5" t="n">
-        <v>371.2272727272727</v>
+        <v>353.2727272727273</v>
       </c>
     </row>
     <row r="82">
@@ -4585,11 +4585,11 @@
         </is>
       </c>
       <c r="G83" s="4" t="n">
-        <v>16141</v>
+        <v>15557</v>
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
-          <t>24/25</t>
+          <t>25/25</t>
         </is>
       </c>
       <c r="I83" s="3" t="inlineStr">
@@ -4598,10 +4598,10 @@
         </is>
       </c>
       <c r="J83" s="4" t="n">
-        <v>16814</v>
+        <v>15557</v>
       </c>
       <c r="K83" s="5" t="n">
-        <v>672.5416666666666</v>
+        <v>622.28</v>
       </c>
     </row>
     <row r="84">
@@ -4986,7 +4986,7 @@
       </c>
       <c r="I91" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J91" s="4" t="n">
@@ -5124,11 +5124,11 @@
         </is>
       </c>
       <c r="G94" s="4" t="n">
-        <v>58691</v>
+        <v>59717</v>
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
-          <t>22/25</t>
+          <t>23/25</t>
         </is>
       </c>
       <c r="I94" s="3" t="inlineStr">
@@ -5137,10 +5137,10 @@
         </is>
       </c>
       <c r="J94" s="4" t="n">
-        <v>66694</v>
+        <v>64910</v>
       </c>
       <c r="K94" s="5" t="n">
-        <v>2667.772727272727</v>
+        <v>2596.391304347826</v>
       </c>
     </row>
     <row r="95">
@@ -5182,7 +5182,7 @@
       </c>
       <c r="I95" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J95" s="4" t="n">
@@ -5271,11 +5271,11 @@
         </is>
       </c>
       <c r="G97" s="11" t="n">
-        <v>7263</v>
+        <v>6662</v>
       </c>
       <c r="H97" s="10" t="inlineStr">
         <is>
-          <t>19/27</t>
+          <t>20/27</t>
         </is>
       </c>
       <c r="I97" s="10" t="inlineStr">
@@ -5284,10 +5284,10 @@
         </is>
       </c>
       <c r="J97" s="11" t="n">
-        <v>10321</v>
+        <v>8994</v>
       </c>
       <c r="K97" s="12" t="n">
-        <v>382.2631578947368</v>
+        <v>333.1</v>
       </c>
     </row>
     <row r="98">
@@ -5378,7 +5378,7 @@
       </c>
       <c r="I99" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J99" s="8" t="n">
@@ -5516,7 +5516,7 @@
         </is>
       </c>
       <c r="G102" s="4" t="n">
-        <v>6690</v>
+        <v>6281</v>
       </c>
       <c r="H102" s="3" t="inlineStr">
         <is>
@@ -5529,10 +5529,10 @@
         </is>
       </c>
       <c r="J102" s="4" t="n">
-        <v>7248</v>
+        <v>6804</v>
       </c>
       <c r="K102" s="5" t="n">
-        <v>278.75</v>
+        <v>261.7083333333333</v>
       </c>
     </row>
     <row r="103">
@@ -5565,11 +5565,11 @@
         </is>
       </c>
       <c r="G103" s="4" t="n">
-        <v>13231</v>
+        <v>16100</v>
       </c>
       <c r="H103" s="3" t="inlineStr">
         <is>
-          <t>21/24</t>
+          <t>22/24</t>
         </is>
       </c>
       <c r="I103" s="3" t="inlineStr">
@@ -5578,10 +5578,10 @@
         </is>
       </c>
       <c r="J103" s="4" t="n">
-        <v>15121</v>
+        <v>17564</v>
       </c>
       <c r="K103" s="5" t="n">
-        <v>630.047619047619</v>
+        <v>731.8181818181819</v>
       </c>
     </row>
     <row r="104">
@@ -5667,7 +5667,7 @@
       </c>
       <c r="H105" s="3" t="inlineStr">
         <is>
-          <t>30/32</t>
+          <t>30/31</t>
         </is>
       </c>
       <c r="I105" s="3" t="inlineStr">
@@ -5676,7 +5676,7 @@
         </is>
       </c>
       <c r="J105" s="4" t="n">
-        <v>17629</v>
+        <v>17078</v>
       </c>
       <c r="K105" s="5" t="n">
         <v>550.9</v>
@@ -5810,11 +5810,11 @@
         </is>
       </c>
       <c r="G108" s="4" t="n">
-        <v>10225</v>
+        <v>9781</v>
       </c>
       <c r="H108" s="3" t="inlineStr">
         <is>
-          <t>16/18</t>
+          <t>19/19</t>
         </is>
       </c>
       <c r="I108" s="3" t="inlineStr">
@@ -5823,10 +5823,10 @@
         </is>
       </c>
       <c r="J108" s="4" t="n">
-        <v>11503</v>
+        <v>9781</v>
       </c>
       <c r="K108" s="5" t="n">
-        <v>639.0625</v>
+        <v>514.7894736842105</v>
       </c>
     </row>
     <row r="109">
@@ -6055,11 +6055,11 @@
         </is>
       </c>
       <c r="G113" s="4" t="n">
-        <v>11740</v>
+        <v>11869</v>
       </c>
       <c r="H113" s="3" t="inlineStr">
         <is>
-          <t>26/27</t>
+          <t>27/27</t>
         </is>
       </c>
       <c r="I113" s="3" t="inlineStr">
@@ -6068,10 +6068,10 @@
         </is>
       </c>
       <c r="J113" s="4" t="n">
-        <v>12192</v>
+        <v>11869</v>
       </c>
       <c r="K113" s="5" t="n">
-        <v>451.5384615384615</v>
+        <v>439.5925925925926</v>
       </c>
     </row>
     <row r="114">
@@ -6153,11 +6153,11 @@
         </is>
       </c>
       <c r="G115" s="11" t="n">
-        <v>3794</v>
+        <v>3207</v>
       </c>
       <c r="H115" s="10" t="inlineStr">
         <is>
-          <t>20/23</t>
+          <t>21/25</t>
         </is>
       </c>
       <c r="I115" s="10" t="inlineStr">
@@ -6166,10 +6166,10 @@
         </is>
       </c>
       <c r="J115" s="11" t="n">
-        <v>4363</v>
+        <v>3818</v>
       </c>
       <c r="K115" s="12" t="n">
-        <v>189.7</v>
+        <v>152.7142857142857</v>
       </c>
     </row>
     <row r="116">
@@ -6349,11 +6349,11 @@
         </is>
       </c>
       <c r="G119" s="4" t="n">
-        <v>26232</v>
+        <v>27807</v>
       </c>
       <c r="H119" s="3" t="inlineStr">
         <is>
-          <t>21/23</t>
+          <t>22/24</t>
         </is>
       </c>
       <c r="I119" s="3" t="inlineStr">
@@ -6362,10 +6362,10 @@
         </is>
       </c>
       <c r="J119" s="4" t="n">
-        <v>28730</v>
+        <v>30335</v>
       </c>
       <c r="K119" s="5" t="n">
-        <v>1249.142857142857</v>
+        <v>1263.954545454545</v>
       </c>
     </row>
     <row r="120">
@@ -6407,7 +6407,7 @@
       </c>
       <c r="I120" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J120" s="4" t="n">
@@ -6603,7 +6603,7 @@
       </c>
       <c r="I124" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J124" s="4" t="n">
@@ -6643,11 +6643,11 @@
         </is>
       </c>
       <c r="G125" s="4" t="n">
-        <v>44311</v>
+        <v>45461</v>
       </c>
       <c r="H125" s="3" t="inlineStr">
         <is>
-          <t>26/34</t>
+          <t>27/34</t>
         </is>
       </c>
       <c r="I125" s="3" t="inlineStr">
@@ -6656,10 +6656,10 @@
         </is>
       </c>
       <c r="J125" s="4" t="n">
-        <v>57945</v>
+        <v>57247</v>
       </c>
       <c r="K125" s="5" t="n">
-        <v>1704.269230769231</v>
+        <v>1683.740740740741</v>
       </c>
     </row>
     <row r="126">
@@ -6701,7 +6701,7 @@
       </c>
       <c r="I126" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J126" s="4" t="n">
@@ -6712,52 +6712,52 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="10" t="inlineStr">
+      <c r="A127" s="6" t="inlineStr">
         <is>
           <t>PAPANASAM</t>
         </is>
       </c>
-      <c r="B127" s="10" t="n">
+      <c r="B127" s="7" t="n">
         <v>172</v>
       </c>
-      <c r="C127" s="10" t="inlineStr">
+      <c r="C127" s="7" t="inlineStr">
         <is>
           <t>A.M. SHAHJAHAN</t>
         </is>
       </c>
-      <c r="D127" s="10" t="inlineStr">
+      <c r="D127" s="7" t="inlineStr">
         <is>
           <t>Indian Union Muslim League</t>
         </is>
       </c>
-      <c r="E127" s="10" t="inlineStr">
+      <c r="E127" s="7" t="inlineStr">
         <is>
           <t>AZARUDEEN UDUMAN ALI</t>
         </is>
       </c>
-      <c r="F127" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G127" s="11" t="n">
-        <v>2773</v>
-      </c>
-      <c r="H127" s="10" t="inlineStr">
-        <is>
-          <t>18/23</t>
-        </is>
-      </c>
-      <c r="I127" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J127" s="11" t="n">
-        <v>3543</v>
-      </c>
-      <c r="K127" s="12" t="n">
-        <v>154.0555555555555</v>
+      <c r="F127" s="7" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G127" s="8" t="n">
+        <v>2208</v>
+      </c>
+      <c r="H127" s="7" t="inlineStr">
+        <is>
+          <t>19/23</t>
+        </is>
+      </c>
+      <c r="I127" s="7" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J127" s="8" t="n">
+        <v>2673</v>
+      </c>
+      <c r="K127" s="9" t="n">
+        <v>116.2105263157895</v>
       </c>
     </row>
     <row r="128">
@@ -6799,7 +6799,7 @@
       </c>
       <c r="I128" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J128" s="4" t="n">
@@ -6839,11 +6839,11 @@
         </is>
       </c>
       <c r="G129" s="11" t="n">
-        <v>3556</v>
+        <v>3548</v>
       </c>
       <c r="H129" s="10" t="inlineStr">
         <is>
-          <t>24/25</t>
+          <t>25/25</t>
         </is>
       </c>
       <c r="I129" s="10" t="inlineStr">
@@ -6852,10 +6852,10 @@
         </is>
       </c>
       <c r="J129" s="11" t="n">
-        <v>3704</v>
+        <v>3548</v>
       </c>
       <c r="K129" s="12" t="n">
-        <v>148.1666666666667</v>
+        <v>141.92</v>
       </c>
     </row>
     <row r="130">
@@ -6937,11 +6937,11 @@
         </is>
       </c>
       <c r="G131" s="4" t="n">
-        <v>8454</v>
+        <v>13887</v>
       </c>
       <c r="H131" s="3" t="inlineStr">
         <is>
-          <t>21/23</t>
+          <t>22/24</t>
         </is>
       </c>
       <c r="I131" s="3" t="inlineStr">
@@ -6950,10 +6950,10 @@
         </is>
       </c>
       <c r="J131" s="4" t="n">
-        <v>9259</v>
+        <v>15149</v>
       </c>
       <c r="K131" s="5" t="n">
-        <v>402.5714285714286</v>
+        <v>631.2272727272727</v>
       </c>
     </row>
     <row r="132">
@@ -7133,11 +7133,11 @@
         </is>
       </c>
       <c r="G135" s="8" t="n">
-        <v>573</v>
+        <v>927</v>
       </c>
       <c r="H135" s="7" t="inlineStr">
         <is>
-          <t>13/21</t>
+          <t>14/21</t>
         </is>
       </c>
       <c r="I135" s="7" t="inlineStr">
@@ -7146,10 +7146,10 @@
         </is>
       </c>
       <c r="J135" s="8" t="n">
-        <v>926</v>
+        <v>1390</v>
       </c>
       <c r="K135" s="9" t="n">
-        <v>44.07692307692308</v>
+        <v>66.21428571428571</v>
       </c>
     </row>
     <row r="136">
@@ -7182,11 +7182,11 @@
         </is>
       </c>
       <c r="G136" s="4" t="n">
-        <v>14416</v>
+        <v>16590</v>
       </c>
       <c r="H136" s="3" t="inlineStr">
         <is>
-          <t>23/26</t>
+          <t>24/26</t>
         </is>
       </c>
       <c r="I136" s="3" t="inlineStr">
@@ -7195,10 +7195,10 @@
         </is>
       </c>
       <c r="J136" s="4" t="n">
-        <v>16296</v>
+        <v>17972</v>
       </c>
       <c r="K136" s="5" t="n">
-        <v>626.7826086956521</v>
+        <v>691.25</v>
       </c>
     </row>
     <row r="137">
@@ -7398,52 +7398,52 @@
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="10" t="inlineStr">
+      <c r="A141" s="2" t="inlineStr">
         <is>
           <t>POOMPUHAR</t>
         </is>
       </c>
-      <c r="B141" s="10" t="n">
+      <c r="B141" s="3" t="n">
         <v>162</v>
       </c>
-      <c r="C141" s="10" t="inlineStr">
+      <c r="C141" s="3" t="inlineStr">
         <is>
           <t>NIVEDHA M MURUGAN</t>
         </is>
       </c>
-      <c r="D141" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E141" s="10" t="inlineStr">
+      <c r="D141" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E141" s="3" t="inlineStr">
         <is>
           <t>PAVUNRAJ. S</t>
         </is>
       </c>
-      <c r="F141" s="10" t="inlineStr">
+      <c r="F141" s="3" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G141" s="11" t="n">
-        <v>6054</v>
-      </c>
-      <c r="H141" s="10" t="inlineStr">
-        <is>
-          <t>18/25</t>
-        </is>
-      </c>
-      <c r="I141" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J141" s="11" t="n">
-        <v>8408</v>
-      </c>
-      <c r="K141" s="12" t="n">
-        <v>336.3333333333333</v>
+      <c r="G141" s="4" t="n">
+        <v>5850</v>
+      </c>
+      <c r="H141" s="3" t="inlineStr">
+        <is>
+          <t>19/25</t>
+        </is>
+      </c>
+      <c r="I141" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J141" s="4" t="n">
+        <v>7697</v>
+      </c>
+      <c r="K141" s="5" t="n">
+        <v>307.8947368421053</v>
       </c>
     </row>
     <row r="142">
@@ -7525,11 +7525,11 @@
         </is>
       </c>
       <c r="G143" s="8" t="n">
-        <v>2452</v>
+        <v>2031</v>
       </c>
       <c r="H143" s="7" t="inlineStr">
         <is>
-          <t>19/22</t>
+          <t>20/22</t>
         </is>
       </c>
       <c r="I143" s="7" t="inlineStr">
@@ -7538,10 +7538,10 @@
         </is>
       </c>
       <c r="J143" s="8" t="n">
-        <v>2839</v>
+        <v>2234</v>
       </c>
       <c r="K143" s="9" t="n">
-        <v>129.0526315789474</v>
+        <v>101.55</v>
       </c>
     </row>
     <row r="144">
@@ -7730,7 +7730,7 @@
       </c>
       <c r="I147" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J147" s="4" t="n">
@@ -7819,11 +7819,11 @@
         </is>
       </c>
       <c r="G149" s="11" t="n">
-        <v>4830</v>
+        <v>4870</v>
       </c>
       <c r="H149" s="10" t="inlineStr">
         <is>
-          <t>18/25</t>
+          <t>19/25</t>
         </is>
       </c>
       <c r="I149" s="10" t="inlineStr">
@@ -7832,10 +7832,10 @@
         </is>
       </c>
       <c r="J149" s="11" t="n">
-        <v>6708</v>
+        <v>6408</v>
       </c>
       <c r="K149" s="12" t="n">
-        <v>268.3333333333333</v>
+        <v>256.3157894736842</v>
       </c>
     </row>
     <row r="150">
@@ -7966,11 +7966,11 @@
         </is>
       </c>
       <c r="G152" s="4" t="n">
-        <v>12741</v>
+        <v>13898</v>
       </c>
       <c r="H152" s="3" t="inlineStr">
         <is>
-          <t>20/21</t>
+          <t>21/23</t>
         </is>
       </c>
       <c r="I152" s="3" t="inlineStr">
@@ -7979,10 +7979,10 @@
         </is>
       </c>
       <c r="J152" s="4" t="n">
-        <v>13378</v>
+        <v>15222</v>
       </c>
       <c r="K152" s="5" t="n">
-        <v>637.05</v>
+        <v>661.8095238095239</v>
       </c>
     </row>
     <row r="153">
@@ -8024,7 +8024,7 @@
       </c>
       <c r="I153" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J153" s="4" t="n">
@@ -8162,11 +8162,11 @@
         </is>
       </c>
       <c r="G156" s="8" t="n">
-        <v>636</v>
+        <v>1242</v>
       </c>
       <c r="H156" s="7" t="inlineStr">
         <is>
-          <t>16/25</t>
+          <t>18/25</t>
         </is>
       </c>
       <c r="I156" s="7" t="inlineStr">
@@ -8175,10 +8175,10 @@
         </is>
       </c>
       <c r="J156" s="8" t="n">
-        <v>994</v>
+        <v>1725</v>
       </c>
       <c r="K156" s="9" t="n">
-        <v>39.75</v>
+        <v>69</v>
       </c>
     </row>
     <row r="157">
@@ -8231,52 +8231,52 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="10" t="inlineStr">
+      <c r="A158" s="2" t="inlineStr">
         <is>
           <t>SATTUR</t>
         </is>
       </c>
-      <c r="B158" s="10" t="n">
+      <c r="B158" s="3" t="n">
         <v>204</v>
       </c>
-      <c r="C158" s="10" t="inlineStr">
+      <c r="C158" s="3" t="inlineStr">
         <is>
           <t>KADARKARAIRAJ. A</t>
         </is>
       </c>
-      <c r="D158" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E158" s="10" t="inlineStr">
+      <c r="D158" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E158" s="3" t="inlineStr">
         <is>
           <t>NAINAR NAGENTHRAN</t>
         </is>
       </c>
-      <c r="F158" s="10" t="inlineStr">
+      <c r="F158" s="3" t="inlineStr">
         <is>
           <t>Bharatiya Janata Party</t>
         </is>
       </c>
-      <c r="G158" s="11" t="n">
-        <v>4060</v>
-      </c>
-      <c r="H158" s="10" t="inlineStr">
-        <is>
-          <t>17/21</t>
-        </is>
-      </c>
-      <c r="I158" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J158" s="11" t="n">
-        <v>5015</v>
-      </c>
-      <c r="K158" s="12" t="n">
-        <v>238.8235294117647</v>
+      <c r="G158" s="4" t="n">
+        <v>5111</v>
+      </c>
+      <c r="H158" s="3" t="inlineStr">
+        <is>
+          <t>18/21</t>
+        </is>
+      </c>
+      <c r="I158" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J158" s="4" t="n">
+        <v>5963</v>
+      </c>
+      <c r="K158" s="5" t="n">
+        <v>283.9444444444445</v>
       </c>
     </row>
     <row r="159">
@@ -8358,11 +8358,11 @@
         </is>
       </c>
       <c r="G160" s="8" t="n">
-        <v>573</v>
+        <v>1622</v>
       </c>
       <c r="H160" s="7" t="inlineStr">
         <is>
-          <t>17/19</t>
+          <t>18/19</t>
         </is>
       </c>
       <c r="I160" s="7" t="inlineStr">
@@ -8371,10 +8371,10 @@
         </is>
       </c>
       <c r="J160" s="8" t="n">
-        <v>640</v>
+        <v>1712</v>
       </c>
       <c r="K160" s="9" t="n">
-        <v>33.70588235294117</v>
+        <v>90.11111111111111</v>
       </c>
     </row>
     <row r="161">
@@ -8407,11 +8407,11 @@
         </is>
       </c>
       <c r="G161" s="11" t="n">
-        <v>5058</v>
+        <v>4240</v>
       </c>
       <c r="H161" s="10" t="inlineStr">
         <is>
-          <t>16/25</t>
+          <t>17/25</t>
         </is>
       </c>
       <c r="I161" s="10" t="inlineStr">
@@ -8420,10 +8420,10 @@
         </is>
       </c>
       <c r="J161" s="11" t="n">
-        <v>7903</v>
+        <v>6235</v>
       </c>
       <c r="K161" s="12" t="n">
-        <v>316.125</v>
+        <v>249.4117647058823</v>
       </c>
     </row>
     <row r="162">
@@ -8456,11 +8456,11 @@
         </is>
       </c>
       <c r="G162" s="4" t="n">
-        <v>68669</v>
+        <v>75780</v>
       </c>
       <c r="H162" s="3" t="inlineStr">
         <is>
-          <t>22/30</t>
+          <t>24/30</t>
         </is>
       </c>
       <c r="I162" s="3" t="inlineStr">
@@ -8469,10 +8469,10 @@
         </is>
       </c>
       <c r="J162" s="4" t="n">
-        <v>93640</v>
+        <v>94725</v>
       </c>
       <c r="K162" s="5" t="n">
-        <v>3121.318181818182</v>
+        <v>3157.5</v>
       </c>
     </row>
     <row r="163">
@@ -8505,11 +8505,11 @@
         </is>
       </c>
       <c r="G163" s="4" t="n">
-        <v>22396</v>
+        <v>18219</v>
       </c>
       <c r="H163" s="3" t="inlineStr">
         <is>
-          <t>22/26</t>
+          <t>23/26</t>
         </is>
       </c>
       <c r="I163" s="3" t="inlineStr">
@@ -8518,10 +8518,10 @@
         </is>
       </c>
       <c r="J163" s="4" t="n">
-        <v>26468</v>
+        <v>20595</v>
       </c>
       <c r="K163" s="5" t="n">
-        <v>1018</v>
+        <v>792.1304347826087</v>
       </c>
     </row>
     <row r="164">
@@ -8554,11 +8554,11 @@
         </is>
       </c>
       <c r="G164" s="4" t="n">
-        <v>11119</v>
+        <v>11417</v>
       </c>
       <c r="H164" s="3" t="inlineStr">
         <is>
-          <t>20/22</t>
+          <t>23/23</t>
         </is>
       </c>
       <c r="I164" s="3" t="inlineStr">
@@ -8567,10 +8567,10 @@
         </is>
       </c>
       <c r="J164" s="4" t="n">
-        <v>12231</v>
+        <v>11417</v>
       </c>
       <c r="K164" s="5" t="n">
-        <v>555.95</v>
+        <v>496.3913043478261</v>
       </c>
     </row>
     <row r="165">
@@ -8652,11 +8652,11 @@
         </is>
       </c>
       <c r="G166" s="4" t="n">
-        <v>9451</v>
+        <v>10455</v>
       </c>
       <c r="H166" s="3" t="inlineStr">
         <is>
-          <t>19/21</t>
+          <t>20/21</t>
         </is>
       </c>
       <c r="I166" s="3" t="inlineStr">
@@ -8665,10 +8665,10 @@
         </is>
       </c>
       <c r="J166" s="4" t="n">
-        <v>10446</v>
+        <v>10978</v>
       </c>
       <c r="K166" s="5" t="n">
-        <v>497.421052631579</v>
+        <v>522.75</v>
       </c>
     </row>
     <row r="167">
@@ -8701,11 +8701,11 @@
         </is>
       </c>
       <c r="G167" s="4" t="n">
-        <v>42940</v>
+        <v>44141</v>
       </c>
       <c r="H167" s="3" t="inlineStr">
         <is>
-          <t>25/32</t>
+          <t>26/32</t>
         </is>
       </c>
       <c r="I167" s="3" t="inlineStr">
@@ -8714,10 +8714,10 @@
         </is>
       </c>
       <c r="J167" s="4" t="n">
-        <v>54963</v>
+        <v>54327</v>
       </c>
       <c r="K167" s="5" t="n">
-        <v>1717.6</v>
+        <v>1697.730769230769</v>
       </c>
     </row>
     <row r="168">
@@ -8750,11 +8750,11 @@
         </is>
       </c>
       <c r="G168" s="4" t="n">
-        <v>33781</v>
+        <v>34086</v>
       </c>
       <c r="H168" s="3" t="inlineStr">
         <is>
-          <t>22/27</t>
+          <t>23/28</t>
         </is>
       </c>
       <c r="I168" s="3" t="inlineStr">
@@ -8763,10 +8763,10 @@
         </is>
       </c>
       <c r="J168" s="4" t="n">
-        <v>41458</v>
+        <v>41496</v>
       </c>
       <c r="K168" s="5" t="n">
-        <v>1535.5</v>
+        <v>1482</v>
       </c>
     </row>
     <row r="169">
@@ -8848,11 +8848,11 @@
         </is>
       </c>
       <c r="G170" s="4" t="n">
-        <v>7132</v>
+        <v>7265</v>
       </c>
       <c r="H170" s="3" t="inlineStr">
         <is>
-          <t>20/22</t>
+          <t>20/23</t>
         </is>
       </c>
       <c r="I170" s="3" t="inlineStr">
@@ -8861,10 +8861,10 @@
         </is>
       </c>
       <c r="J170" s="4" t="n">
-        <v>7845</v>
+        <v>8355</v>
       </c>
       <c r="K170" s="5" t="n">
-        <v>356.6</v>
+        <v>363.25</v>
       </c>
     </row>
     <row r="171">
@@ -8897,11 +8897,11 @@
         </is>
       </c>
       <c r="G171" s="4" t="n">
-        <v>5199</v>
+        <v>5267</v>
       </c>
       <c r="H171" s="3" t="inlineStr">
         <is>
-          <t>28/30</t>
+          <t>29/32</t>
         </is>
       </c>
       <c r="I171" s="3" t="inlineStr">
@@ -8910,10 +8910,10 @@
         </is>
       </c>
       <c r="J171" s="4" t="n">
-        <v>5570</v>
+        <v>5812</v>
       </c>
       <c r="K171" s="5" t="n">
-        <v>185.6785714285714</v>
+        <v>181.6206896551724</v>
       </c>
     </row>
     <row r="172">
@@ -8946,11 +8946,11 @@
         </is>
       </c>
       <c r="G172" s="4" t="n">
-        <v>35773</v>
+        <v>35937</v>
       </c>
       <c r="H172" s="3" t="inlineStr">
         <is>
-          <t>34/39</t>
+          <t>37/39</t>
         </is>
       </c>
       <c r="I172" s="3" t="inlineStr">
@@ -8959,10 +8959,10 @@
         </is>
       </c>
       <c r="J172" s="4" t="n">
-        <v>41034</v>
+        <v>37880</v>
       </c>
       <c r="K172" s="5" t="n">
-        <v>1052.14705882353</v>
+        <v>971.2702702702703</v>
       </c>
     </row>
     <row r="173">
@@ -8995,11 +8995,11 @@
         </is>
       </c>
       <c r="G173" s="4" t="n">
-        <v>10064</v>
+        <v>9746</v>
       </c>
       <c r="H173" s="3" t="inlineStr">
         <is>
-          <t>23/26</t>
+          <t>24/26</t>
         </is>
       </c>
       <c r="I173" s="3" t="inlineStr">
@@ -9008,59 +9008,59 @@
         </is>
       </c>
       <c r="J173" s="4" t="n">
-        <v>11377</v>
+        <v>10558</v>
       </c>
       <c r="K173" s="5" t="n">
-        <v>437.5652173913044</v>
+        <v>406.0833333333333</v>
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="6" t="inlineStr">
+      <c r="A174" s="10" t="inlineStr">
         <is>
           <t>THALLI</t>
         </is>
       </c>
-      <c r="B174" s="7" t="n">
+      <c r="B174" s="10" t="n">
         <v>56</v>
       </c>
-      <c r="C174" s="7" t="inlineStr">
+      <c r="C174" s="10" t="inlineStr">
         <is>
           <t>RAMACHANDRAN. T</t>
         </is>
       </c>
-      <c r="D174" s="7" t="inlineStr">
+      <c r="D174" s="10" t="inlineStr">
         <is>
           <t>Communist Party of India</t>
         </is>
       </c>
-      <c r="E174" s="7" t="inlineStr">
+      <c r="E174" s="10" t="inlineStr">
         <is>
           <t>DR.NAGESH KUMAR. C</t>
         </is>
       </c>
-      <c r="F174" s="7" t="inlineStr">
+      <c r="F174" s="10" t="inlineStr">
         <is>
           <t>Bharatiya Janata Party</t>
         </is>
       </c>
-      <c r="G174" s="8" t="n">
-        <v>726</v>
-      </c>
-      <c r="H174" s="7" t="inlineStr">
-        <is>
-          <t>18/24</t>
-        </is>
-      </c>
-      <c r="I174" s="7" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J174" s="8" t="n">
-        <v>968</v>
-      </c>
-      <c r="K174" s="9" t="n">
-        <v>40.33333333333334</v>
+      <c r="G174" s="11" t="n">
+        <v>2856</v>
+      </c>
+      <c r="H174" s="10" t="inlineStr">
+        <is>
+          <t>20/24</t>
+        </is>
+      </c>
+      <c r="I174" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J174" s="11" t="n">
+        <v>3427</v>
+      </c>
+      <c r="K174" s="12" t="n">
+        <v>142.8</v>
       </c>
     </row>
     <row r="175">
@@ -9211,52 +9211,52 @@
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="13" t="inlineStr">
+      <c r="A178" s="6" t="inlineStr">
         <is>
           <t>THIRUMAYAM</t>
         </is>
       </c>
-      <c r="B178" s="14" t="n">
+      <c r="B178" s="7" t="n">
         <v>181</v>
       </c>
-      <c r="C178" s="14" t="inlineStr">
+      <c r="C178" s="7" t="inlineStr">
         <is>
           <t>REGUPATHY.S</t>
         </is>
       </c>
-      <c r="D178" s="14" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E178" s="14" t="inlineStr">
+      <c r="D178" s="7" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E178" s="7" t="inlineStr">
         <is>
           <t>CHINTHAMANI.C</t>
         </is>
       </c>
-      <c r="F178" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G178" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="H178" s="14" t="inlineStr">
-        <is>
-          <t>19/22</t>
-        </is>
-      </c>
-      <c r="I178" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J178" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="K178" s="16" t="n">
-        <v>0.1578947368421053</v>
+      <c r="F178" s="7" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G178" s="8" t="n">
+        <v>507</v>
+      </c>
+      <c r="H178" s="7" t="inlineStr">
+        <is>
+          <t>20/22</t>
+        </is>
+      </c>
+      <c r="I178" s="7" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J178" s="8" t="n">
+        <v>558</v>
+      </c>
+      <c r="K178" s="9" t="n">
+        <v>25.35</v>
       </c>
     </row>
     <row r="179">
@@ -9338,11 +9338,11 @@
         </is>
       </c>
       <c r="G180" s="4" t="n">
-        <v>32772</v>
+        <v>34361</v>
       </c>
       <c r="H180" s="3" t="inlineStr">
         <is>
-          <t>21/29</t>
+          <t>22/29</t>
         </is>
       </c>
       <c r="I180" s="3" t="inlineStr">
@@ -9351,10 +9351,10 @@
         </is>
       </c>
       <c r="J180" s="4" t="n">
-        <v>45257</v>
+        <v>45294</v>
       </c>
       <c r="K180" s="5" t="n">
-        <v>1560.571428571429</v>
+        <v>1561.863636363636</v>
       </c>
     </row>
     <row r="181">
@@ -9436,11 +9436,11 @@
         </is>
       </c>
       <c r="G182" s="4" t="n">
-        <v>6731</v>
+        <v>7361</v>
       </c>
       <c r="H182" s="3" t="inlineStr">
         <is>
-          <t>19/25</t>
+          <t>20/25</t>
         </is>
       </c>
       <c r="I182" s="3" t="inlineStr">
@@ -9449,10 +9449,10 @@
         </is>
       </c>
       <c r="J182" s="4" t="n">
-        <v>8857</v>
+        <v>9201</v>
       </c>
       <c r="K182" s="5" t="n">
-        <v>354.2631578947368</v>
+        <v>368.05</v>
       </c>
     </row>
     <row r="183">
@@ -9494,7 +9494,7 @@
       </c>
       <c r="I183" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J183" s="4" t="n">
@@ -9583,11 +9583,11 @@
         </is>
       </c>
       <c r="G185" s="4" t="n">
-        <v>7542</v>
+        <v>7811</v>
       </c>
       <c r="H185" s="3" t="inlineStr">
         <is>
-          <t>20/23</t>
+          <t>21/23</t>
         </is>
       </c>
       <c r="I185" s="3" t="inlineStr">
@@ -9596,10 +9596,10 @@
         </is>
       </c>
       <c r="J185" s="4" t="n">
-        <v>8673</v>
+        <v>8555</v>
       </c>
       <c r="K185" s="5" t="n">
-        <v>377.1</v>
+        <v>371.952380952381</v>
       </c>
     </row>
     <row r="186">
@@ -9685,7 +9685,7 @@
       </c>
       <c r="H187" s="3" t="inlineStr">
         <is>
-          <t>26/27</t>
+          <t>26/26</t>
         </is>
       </c>
       <c r="I187" s="3" t="inlineStr">
@@ -9694,7 +9694,7 @@
         </is>
       </c>
       <c r="J187" s="4" t="n">
-        <v>55388</v>
+        <v>53337</v>
       </c>
       <c r="K187" s="5" t="n">
         <v>2051.423076923077</v>
@@ -9779,11 +9779,11 @@
         </is>
       </c>
       <c r="G189" s="4" t="n">
-        <v>13650</v>
+        <v>14196</v>
       </c>
       <c r="H189" s="3" t="inlineStr">
         <is>
-          <t>23/27</t>
+          <t>24/27</t>
         </is>
       </c>
       <c r="I189" s="3" t="inlineStr">
@@ -9792,10 +9792,10 @@
         </is>
       </c>
       <c r="J189" s="4" t="n">
-        <v>16024</v>
+        <v>15970</v>
       </c>
       <c r="K189" s="5" t="n">
-        <v>593.4782608695652</v>
+        <v>591.5</v>
       </c>
     </row>
     <row r="190">
@@ -9828,23 +9828,23 @@
         </is>
       </c>
       <c r="G190" s="4" t="n">
-        <v>36921</v>
+        <v>37731</v>
       </c>
       <c r="H190" s="3" t="inlineStr">
         <is>
-          <t>25/26</t>
+          <t>26/26</t>
         </is>
       </c>
       <c r="I190" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J190" s="4" t="n">
-        <v>38398</v>
+        <v>37731</v>
       </c>
       <c r="K190" s="5" t="n">
-        <v>1476.84</v>
+        <v>1451.192307692308</v>
       </c>
     </row>
     <row r="191">
@@ -10073,11 +10073,11 @@
         </is>
       </c>
       <c r="G195" s="4" t="n">
-        <v>25962</v>
+        <v>27265</v>
       </c>
       <c r="H195" s="3" t="inlineStr">
         <is>
-          <t>19/22</t>
+          <t>20/22</t>
         </is>
       </c>
       <c r="I195" s="3" t="inlineStr">
@@ -10086,10 +10086,10 @@
         </is>
       </c>
       <c r="J195" s="4" t="n">
-        <v>30061</v>
+        <v>29992</v>
       </c>
       <c r="K195" s="5" t="n">
-        <v>1366.421052631579</v>
+        <v>1363.25</v>
       </c>
     </row>
     <row r="196">
@@ -10122,11 +10122,11 @@
         </is>
       </c>
       <c r="G196" s="4" t="n">
-        <v>22092</v>
+        <v>22869</v>
       </c>
       <c r="H196" s="3" t="inlineStr">
         <is>
-          <t>17/22</t>
+          <t>18/22</t>
         </is>
       </c>
       <c r="I196" s="3" t="inlineStr">
@@ -10135,10 +10135,10 @@
         </is>
       </c>
       <c r="J196" s="4" t="n">
-        <v>28590</v>
+        <v>27951</v>
       </c>
       <c r="K196" s="5" t="n">
-        <v>1299.529411764706</v>
+        <v>1270.5</v>
       </c>
     </row>
     <row r="197">
@@ -10220,11 +10220,11 @@
         </is>
       </c>
       <c r="G198" s="4" t="n">
-        <v>10257</v>
+        <v>10615</v>
       </c>
       <c r="H198" s="3" t="inlineStr">
         <is>
-          <t>17/21</t>
+          <t>18/21</t>
         </is>
       </c>
       <c r="I198" s="3" t="inlineStr">
@@ -10233,10 +10233,10 @@
         </is>
       </c>
       <c r="J198" s="4" t="n">
-        <v>12670</v>
+        <v>12384</v>
       </c>
       <c r="K198" s="5" t="n">
-        <v>603.3529411764706</v>
+        <v>589.7222222222222</v>
       </c>
     </row>
     <row r="199">
@@ -10387,52 +10387,52 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="10" t="inlineStr">
+      <c r="A202" s="6" t="inlineStr">
         <is>
           <t>TIRUPPATTUR</t>
         </is>
       </c>
-      <c r="B202" s="10" t="n">
+      <c r="B202" s="7" t="n">
         <v>185</v>
       </c>
-      <c r="C202" s="10" t="inlineStr">
+      <c r="C202" s="7" t="inlineStr">
         <is>
           <t>PERIAKARUPPAN. KR</t>
         </is>
       </c>
-      <c r="D202" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E202" s="10" t="inlineStr">
+      <c r="D202" s="7" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E202" s="7" t="inlineStr">
         <is>
           <t>SEENIVASA SETHUPATHY. R</t>
         </is>
       </c>
-      <c r="F202" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G202" s="11" t="n">
-        <v>2610</v>
-      </c>
-      <c r="H202" s="10" t="inlineStr">
-        <is>
-          <t>22/27</t>
-        </is>
-      </c>
-      <c r="I202" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J202" s="11" t="n">
-        <v>3203</v>
-      </c>
-      <c r="K202" s="12" t="n">
-        <v>118.6363636363636</v>
+      <c r="F202" s="7" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G202" s="8" t="n">
+        <v>2237</v>
+      </c>
+      <c r="H202" s="7" t="inlineStr">
+        <is>
+          <t>23/27</t>
+        </is>
+      </c>
+      <c r="I202" s="7" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J202" s="8" t="n">
+        <v>2626</v>
+      </c>
+      <c r="K202" s="9" t="n">
+        <v>97.26086956521739</v>
       </c>
     </row>
     <row r="203">
@@ -10465,11 +10465,11 @@
         </is>
       </c>
       <c r="G203" s="4" t="n">
-        <v>57599</v>
+        <v>60629</v>
       </c>
       <c r="H203" s="3" t="inlineStr">
         <is>
-          <t>26/32</t>
+          <t>27/32</t>
         </is>
       </c>
       <c r="I203" s="3" t="inlineStr">
@@ -10478,10 +10478,10 @@
         </is>
       </c>
       <c r="J203" s="4" t="n">
-        <v>70891</v>
+        <v>71857</v>
       </c>
       <c r="K203" s="5" t="n">
-        <v>2215.346153846154</v>
+        <v>2245.518518518519</v>
       </c>
     </row>
     <row r="204">
@@ -10514,11 +10514,11 @@
         </is>
       </c>
       <c r="G204" s="4" t="n">
-        <v>10748</v>
+        <v>11969</v>
       </c>
       <c r="H204" s="3" t="inlineStr">
         <is>
-          <t>19/21</t>
+          <t>20/21</t>
         </is>
       </c>
       <c r="I204" s="3" t="inlineStr">
@@ -10527,59 +10527,59 @@
         </is>
       </c>
       <c r="J204" s="4" t="n">
-        <v>11879</v>
+        <v>12567</v>
       </c>
       <c r="K204" s="5" t="n">
-        <v>565.6842105263158</v>
+        <v>598.45</v>
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="10" t="inlineStr">
+      <c r="A205" s="2" t="inlineStr">
         <is>
           <t>TIRUTTANI</t>
         </is>
       </c>
-      <c r="B205" s="10" t="n">
+      <c r="B205" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="C205" s="10" t="inlineStr">
+      <c r="C205" s="3" t="inlineStr">
         <is>
           <t>G.HARI</t>
         </is>
       </c>
-      <c r="D205" s="10" t="inlineStr">
+      <c r="D205" s="3" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E205" s="10" t="inlineStr">
+      <c r="E205" s="3" t="inlineStr">
         <is>
           <t>M.SATHYA KUMAR</t>
         </is>
       </c>
-      <c r="F205" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G205" s="11" t="n">
-        <v>8342</v>
-      </c>
-      <c r="H205" s="10" t="inlineStr">
-        <is>
-          <t>18/25</t>
-        </is>
-      </c>
-      <c r="I205" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J205" s="11" t="n">
-        <v>11586</v>
-      </c>
-      <c r="K205" s="12" t="n">
-        <v>463.4444444444445</v>
+      <c r="F205" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G205" s="4" t="n">
+        <v>6905</v>
+      </c>
+      <c r="H205" s="3" t="inlineStr">
+        <is>
+          <t>19/25</t>
+        </is>
+      </c>
+      <c r="I205" s="3" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J205" s="4" t="n">
+        <v>9086</v>
+      </c>
+      <c r="K205" s="5" t="n">
+        <v>363.421052631579</v>
       </c>
     </row>
     <row r="206">
@@ -10857,7 +10857,7 @@
         </is>
       </c>
       <c r="G211" s="15" t="n">
-        <v>365</v>
+        <v>72</v>
       </c>
       <c r="H211" s="14" t="inlineStr">
         <is>
@@ -10870,10 +10870,10 @@
         </is>
       </c>
       <c r="J211" s="15" t="n">
-        <v>394</v>
+        <v>78</v>
       </c>
       <c r="K211" s="16" t="n">
-        <v>14.6</v>
+        <v>2.88</v>
       </c>
     </row>
     <row r="212">
@@ -10906,11 +10906,11 @@
         </is>
       </c>
       <c r="G212" s="8" t="n">
-        <v>2029</v>
+        <v>2374</v>
       </c>
       <c r="H212" s="7" t="inlineStr">
         <is>
-          <t>20/25</t>
+          <t>22/25</t>
         </is>
       </c>
       <c r="I212" s="7" t="inlineStr">
@@ -10919,10 +10919,10 @@
         </is>
       </c>
       <c r="J212" s="8" t="n">
-        <v>2536</v>
+        <v>2698</v>
       </c>
       <c r="K212" s="9" t="n">
-        <v>101.45</v>
+        <v>107.9090909090909</v>
       </c>
     </row>
     <row r="213">
@@ -11200,11 +11200,11 @@
         </is>
       </c>
       <c r="G218" s="4" t="n">
-        <v>6967</v>
+        <v>7034</v>
       </c>
       <c r="H218" s="3" t="inlineStr">
         <is>
-          <t>22/23</t>
+          <t>23/23</t>
         </is>
       </c>
       <c r="I218" s="3" t="inlineStr">
@@ -11213,10 +11213,10 @@
         </is>
       </c>
       <c r="J218" s="4" t="n">
-        <v>7284</v>
+        <v>7034</v>
       </c>
       <c r="K218" s="5" t="n">
-        <v>316.6818181818182</v>
+        <v>305.8260869565217</v>
       </c>
     </row>
     <row r="219">
@@ -11347,11 +11347,11 @@
         </is>
       </c>
       <c r="G221" s="4" t="n">
-        <v>9814</v>
+        <v>9922</v>
       </c>
       <c r="H221" s="3" t="inlineStr">
         <is>
-          <t>24/27</t>
+          <t>25/27</t>
         </is>
       </c>
       <c r="I221" s="3" t="inlineStr">
@@ -11360,10 +11360,10 @@
         </is>
       </c>
       <c r="J221" s="4" t="n">
-        <v>11041</v>
+        <v>10716</v>
       </c>
       <c r="K221" s="5" t="n">
-        <v>408.9166666666667</v>
+        <v>396.88</v>
       </c>
     </row>
     <row r="222">
@@ -11396,11 +11396,11 @@
         </is>
       </c>
       <c r="G222" s="11" t="n">
-        <v>4236</v>
+        <v>4071</v>
       </c>
       <c r="H222" s="10" t="inlineStr">
         <is>
-          <t>22/23</t>
+          <t>23/23</t>
         </is>
       </c>
       <c r="I222" s="10" t="inlineStr">
@@ -11409,10 +11409,10 @@
         </is>
       </c>
       <c r="J222" s="11" t="n">
-        <v>4429</v>
+        <v>4071</v>
       </c>
       <c r="K222" s="12" t="n">
-        <v>192.5454545454545</v>
+        <v>177</v>
       </c>
     </row>
     <row r="223">
@@ -11547,7 +11547,7 @@
       </c>
       <c r="H225" s="14" t="inlineStr">
         <is>
-          <t>25/25</t>
+          <t>25/27</t>
         </is>
       </c>
       <c r="I225" s="14" t="inlineStr">
@@ -11556,7 +11556,7 @@
         </is>
       </c>
       <c r="J225" s="15" t="n">
-        <v>272</v>
+        <v>294</v>
       </c>
       <c r="K225" s="16" t="n">
         <v>10.88</v>
@@ -11592,11 +11592,11 @@
         </is>
       </c>
       <c r="G226" s="11" t="n">
-        <v>4004</v>
+        <v>3046</v>
       </c>
       <c r="H226" s="10" t="inlineStr">
         <is>
-          <t>17/23</t>
+          <t>18/23</t>
         </is>
       </c>
       <c r="I226" s="10" t="inlineStr">
@@ -11605,10 +11605,10 @@
         </is>
       </c>
       <c r="J226" s="11" t="n">
-        <v>5417</v>
+        <v>3892</v>
       </c>
       <c r="K226" s="12" t="n">
-        <v>235.5294117647059</v>
+        <v>169.2222222222222</v>
       </c>
     </row>
     <row r="227">
@@ -11641,23 +11641,23 @@
         </is>
       </c>
       <c r="G227" s="4" t="n">
-        <v>8487</v>
+        <v>8228</v>
       </c>
       <c r="H227" s="3" t="inlineStr">
         <is>
-          <t>19/20</t>
+          <t>20/20</t>
         </is>
       </c>
       <c r="I227" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J227" s="4" t="n">
-        <v>8934</v>
+        <v>8228</v>
       </c>
       <c r="K227" s="5" t="n">
-        <v>446.6842105263158</v>
+        <v>411.4</v>
       </c>
     </row>
     <row r="228">
@@ -11886,11 +11886,11 @@
         </is>
       </c>
       <c r="G232" s="4" t="n">
-        <v>9288</v>
+        <v>9206</v>
       </c>
       <c r="H232" s="3" t="inlineStr">
         <is>
-          <t>20/23</t>
+          <t>21/23</t>
         </is>
       </c>
       <c r="I232" s="3" t="inlineStr">
@@ -11899,10 +11899,10 @@
         </is>
       </c>
       <c r="J232" s="4" t="n">
-        <v>10681</v>
+        <v>10083</v>
       </c>
       <c r="K232" s="5" t="n">
-        <v>464.4</v>
+        <v>438.3809523809524</v>
       </c>
     </row>
     <row r="233">
@@ -11935,11 +11935,11 @@
         </is>
       </c>
       <c r="G233" s="4" t="n">
-        <v>21468</v>
+        <v>22165</v>
       </c>
       <c r="H233" s="3" t="inlineStr">
         <is>
-          <t>18/23</t>
+          <t>19/23</t>
         </is>
       </c>
       <c r="I233" s="3" t="inlineStr">
@@ -11948,10 +11948,10 @@
         </is>
       </c>
       <c r="J233" s="4" t="n">
-        <v>27431</v>
+        <v>26831</v>
       </c>
       <c r="K233" s="5" t="n">
-        <v>1192.666666666667</v>
+        <v>1166.578947368421</v>
       </c>
     </row>
     <row r="234">
@@ -12004,52 +12004,52 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="6" t="inlineStr">
+      <c r="A235" s="13" t="inlineStr">
         <is>
           <t>YERCAUD</t>
         </is>
       </c>
-      <c r="B235" s="7" t="n">
+      <c r="B235" s="14" t="n">
         <v>83</v>
       </c>
-      <c r="C235" s="7" t="inlineStr">
+      <c r="C235" s="14" t="inlineStr">
         <is>
           <t>LAKSHMI JANARTHANAN. J</t>
         </is>
       </c>
-      <c r="D235" s="7" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E235" s="7" t="inlineStr">
+      <c r="D235" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E235" s="14" t="inlineStr">
         <is>
           <t>USHARANI. P</t>
         </is>
       </c>
-      <c r="F235" s="7" t="inlineStr">
+      <c r="F235" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G235" s="8" t="n">
-        <v>2079</v>
-      </c>
-      <c r="H235" s="7" t="inlineStr">
-        <is>
-          <t>21/24</t>
-        </is>
-      </c>
-      <c r="I235" s="7" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J235" s="8" t="n">
-        <v>2376</v>
-      </c>
-      <c r="K235" s="9" t="n">
-        <v>99</v>
+      <c r="G235" s="15" t="n">
+        <v>312</v>
+      </c>
+      <c r="H235" s="14" t="inlineStr">
+        <is>
+          <t>22/24</t>
+        </is>
+      </c>
+      <c r="I235" s="14" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J235" s="15" t="n">
+        <v>340</v>
+      </c>
+      <c r="K235" s="16" t="n">
+        <v>14.18181818181818</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Election snapshot: 95.2% counted — 95 declared, TVK 107, AIADMK 45
TIRUKKOYILUR tightest at 69 votes (TVK, 22/24); ULUNDURPETTAI DMK 72 (25/27).
YERCAUD & PARAMATHI-VELUR flipped to AIADMK; TIRUPPATTUR genuinely flipped to DMK.

https://claude.ai/code/session_01MizbUy44JG5sXyvaf3Wekb
</commit_message>
<xml_diff>
--- a/tn_election_results_may2026.xlsx
+++ b/tn_election_results_may2026.xlsx
@@ -616,11 +616,11 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>23273</v>
+        <v>24195</v>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>23/31</t>
+          <t>24/31</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -629,10 +629,10 @@
         </is>
       </c>
       <c r="J2" s="4" t="n">
-        <v>31368</v>
+        <v>31252</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>1011.869565217391</v>
+        <v>1008.125</v>
       </c>
     </row>
     <row r="3">
@@ -861,11 +861,11 @@
         </is>
       </c>
       <c r="G7" s="4" t="n">
-        <v>9443</v>
+        <v>8610</v>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>19/22</t>
+          <t>20/22</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -874,10 +874,10 @@
         </is>
       </c>
       <c r="J7" s="4" t="n">
-        <v>10934</v>
+        <v>9471</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>497</v>
+        <v>430.5</v>
       </c>
     </row>
     <row r="8">
@@ -919,7 +919,7 @@
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J8" s="4" t="n">
@@ -1155,11 +1155,11 @@
         </is>
       </c>
       <c r="G13" s="4" t="n">
-        <v>5508</v>
+        <v>5631</v>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>23/24</t>
+          <t>25/25</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
@@ -1168,10 +1168,10 @@
         </is>
       </c>
       <c r="J13" s="4" t="n">
-        <v>5747</v>
+        <v>5631</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>239.4782608695652</v>
+        <v>225.24</v>
       </c>
     </row>
     <row r="14">
@@ -1253,11 +1253,11 @@
         </is>
       </c>
       <c r="G15" s="4" t="n">
-        <v>19378</v>
+        <v>19382</v>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>20/22</t>
+          <t>22/22</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
@@ -1266,10 +1266,10 @@
         </is>
       </c>
       <c r="J15" s="4" t="n">
-        <v>21316</v>
+        <v>19382</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>968.9</v>
+        <v>881</v>
       </c>
     </row>
     <row r="16">
@@ -1302,11 +1302,11 @@
         </is>
       </c>
       <c r="G16" s="4" t="n">
-        <v>35995</v>
+        <v>37822</v>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>20/23</t>
+          <t>21/23</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
@@ -1315,10 +1315,10 @@
         </is>
       </c>
       <c r="J16" s="4" t="n">
-        <v>41394</v>
+        <v>41424</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>1799.75</v>
+        <v>1801.047619047619</v>
       </c>
     </row>
     <row r="17">
@@ -1400,7 +1400,7 @@
         </is>
       </c>
       <c r="G18" s="11" t="n">
-        <v>3510</v>
+        <v>3885</v>
       </c>
       <c r="H18" s="10" t="inlineStr">
         <is>
@@ -1413,10 +1413,10 @@
         </is>
       </c>
       <c r="J18" s="11" t="n">
-        <v>3900</v>
+        <v>4317</v>
       </c>
       <c r="K18" s="12" t="n">
-        <v>195</v>
+        <v>215.8333333333333</v>
       </c>
     </row>
     <row r="19">
@@ -1547,11 +1547,11 @@
         </is>
       </c>
       <c r="G21" s="4" t="n">
-        <v>65751</v>
+        <v>70239</v>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>22/26</t>
+          <t>23/26</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -1560,10 +1560,10 @@
         </is>
       </c>
       <c r="J21" s="4" t="n">
-        <v>77706</v>
+        <v>79401</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>2988.681818181818</v>
+        <v>3053.869565217391</v>
       </c>
     </row>
     <row r="22">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J22" s="4" t="n">
@@ -1645,11 +1645,11 @@
         </is>
       </c>
       <c r="G23" s="11" t="n">
-        <v>3076</v>
+        <v>4182</v>
       </c>
       <c r="H23" s="10" t="inlineStr">
         <is>
-          <t>21/24</t>
+          <t>22/24</t>
         </is>
       </c>
       <c r="I23" s="10" t="inlineStr">
@@ -1658,10 +1658,10 @@
         </is>
       </c>
       <c r="J23" s="11" t="n">
-        <v>3515</v>
+        <v>4562</v>
       </c>
       <c r="K23" s="12" t="n">
-        <v>146.4761904761905</v>
+        <v>190.0909090909091</v>
       </c>
     </row>
     <row r="24">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J24" s="4" t="n">
@@ -1841,11 +1841,11 @@
         </is>
       </c>
       <c r="G27" s="4" t="n">
-        <v>6023</v>
+        <v>6805</v>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>24/25</t>
+          <t>25/25</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
@@ -1854,10 +1854,10 @@
         </is>
       </c>
       <c r="J27" s="4" t="n">
-        <v>6274</v>
+        <v>6805</v>
       </c>
       <c r="K27" s="5" t="n">
-        <v>250.9583333333333</v>
+        <v>272.2</v>
       </c>
     </row>
     <row r="28">
@@ -1939,11 +1939,11 @@
         </is>
       </c>
       <c r="G29" s="4" t="n">
-        <v>14170</v>
+        <v>14252</v>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>22/25</t>
+          <t>23/25</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
@@ -1952,10 +1952,10 @@
         </is>
       </c>
       <c r="J29" s="4" t="n">
-        <v>16102</v>
+        <v>15491</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>644.0909090909091</v>
+        <v>619.6521739130435</v>
       </c>
     </row>
     <row r="30">
@@ -1997,7 +1997,7 @@
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J30" s="4" t="n">
@@ -2184,11 +2184,11 @@
         </is>
       </c>
       <c r="G34" s="4" t="n">
-        <v>19082</v>
+        <v>20055</v>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>22/25</t>
+          <t>23/25</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
@@ -2197,10 +2197,10 @@
         </is>
       </c>
       <c r="J34" s="4" t="n">
-        <v>21684</v>
+        <v>21799</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>867.3636363636364</v>
+        <v>871.9565217391304</v>
       </c>
     </row>
     <row r="35">
@@ -2253,52 +2253,52 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="6" t="inlineStr">
+      <c r="A36" s="10" t="inlineStr">
         <is>
           <t>COLACHAL</t>
         </is>
       </c>
-      <c r="B36" s="7" t="n">
+      <c r="B36" s="10" t="n">
         <v>231</v>
       </c>
-      <c r="C36" s="7" t="inlineStr">
+      <c r="C36" s="10" t="inlineStr">
         <is>
           <t>THARAHAI CUTHBERT</t>
         </is>
       </c>
-      <c r="D36" s="7" t="inlineStr">
+      <c r="D36" s="10" t="inlineStr">
         <is>
           <t>Indian National Congress</t>
         </is>
       </c>
-      <c r="E36" s="7" t="inlineStr">
+      <c r="E36" s="10" t="inlineStr">
         <is>
           <t>PREM ALEX LAWRENCE</t>
         </is>
       </c>
-      <c r="F36" s="7" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G36" s="8" t="n">
-        <v>2499</v>
-      </c>
-      <c r="H36" s="7" t="inlineStr">
+      <c r="F36" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G36" s="11" t="n">
+        <v>2943</v>
+      </c>
+      <c r="H36" s="10" t="inlineStr">
         <is>
           <t>21/23</t>
         </is>
       </c>
-      <c r="I36" s="7" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J36" s="8" t="n">
-        <v>2737</v>
-      </c>
-      <c r="K36" s="9" t="n">
-        <v>119</v>
+      <c r="I36" s="10" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J36" s="11" t="n">
+        <v>3223</v>
+      </c>
+      <c r="K36" s="12" t="n">
+        <v>140.1428571428571</v>
       </c>
     </row>
     <row r="37">
@@ -2380,11 +2380,11 @@
         </is>
       </c>
       <c r="G38" s="4" t="n">
-        <v>15400</v>
+        <v>15519</v>
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>18/20</t>
+          <t>20/20</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
@@ -2393,10 +2393,10 @@
         </is>
       </c>
       <c r="J38" s="4" t="n">
-        <v>17111</v>
+        <v>15519</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>855.5555555555555</v>
+        <v>775.95</v>
       </c>
     </row>
     <row r="39">
@@ -2536,7 +2536,7 @@
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J41" s="4" t="n">
@@ -2683,7 +2683,7 @@
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J44" s="4" t="n">
@@ -2830,7 +2830,7 @@
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J47" s="4" t="n">
@@ -2919,11 +2919,11 @@
         </is>
       </c>
       <c r="G49" s="4" t="n">
-        <v>14168</v>
+        <v>14404</v>
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>21/22</t>
+          <t>22/22</t>
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr">
@@ -2932,10 +2932,10 @@
         </is>
       </c>
       <c r="J49" s="4" t="n">
-        <v>14843</v>
+        <v>14404</v>
       </c>
       <c r="K49" s="5" t="n">
-        <v>674.6666666666666</v>
+        <v>654.7272727272727</v>
       </c>
     </row>
     <row r="50">
@@ -2968,11 +2968,11 @@
         </is>
       </c>
       <c r="G50" s="11" t="n">
-        <v>11377</v>
+        <v>12024</v>
       </c>
       <c r="H50" s="10" t="inlineStr">
         <is>
-          <t>16/23</t>
+          <t>17/23</t>
         </is>
       </c>
       <c r="I50" s="10" t="inlineStr">
@@ -2981,10 +2981,10 @@
         </is>
       </c>
       <c r="J50" s="11" t="n">
-        <v>16354</v>
+        <v>16268</v>
       </c>
       <c r="K50" s="12" t="n">
-        <v>711.0625</v>
+        <v>707.2941176470588</v>
       </c>
     </row>
     <row r="51">
@@ -3164,23 +3164,23 @@
         </is>
       </c>
       <c r="G54" s="4" t="n">
-        <v>27906</v>
+        <v>27945</v>
       </c>
       <c r="H54" s="3" t="inlineStr">
         <is>
-          <t>25/26</t>
+          <t>26/26</t>
         </is>
       </c>
       <c r="I54" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J54" s="4" t="n">
-        <v>29022</v>
+        <v>27945</v>
       </c>
       <c r="K54" s="5" t="n">
-        <v>1116.24</v>
+        <v>1074.807692307692</v>
       </c>
     </row>
     <row r="55">
@@ -3311,11 +3311,11 @@
         </is>
       </c>
       <c r="G57" s="4" t="n">
-        <v>22532</v>
+        <v>27803</v>
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>30/32</t>
+          <t>32/32</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr">
@@ -3324,10 +3324,10 @@
         </is>
       </c>
       <c r="J57" s="4" t="n">
-        <v>24034</v>
+        <v>27803</v>
       </c>
       <c r="K57" s="5" t="n">
-        <v>751.0666666666667</v>
+        <v>868.84375</v>
       </c>
     </row>
     <row r="58">
@@ -3458,11 +3458,11 @@
         </is>
       </c>
       <c r="G60" s="4" t="n">
-        <v>8512</v>
+        <v>6063</v>
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>23/26</t>
+          <t>25/26</t>
         </is>
       </c>
       <c r="I60" s="3" t="inlineStr">
@@ -3471,10 +3471,10 @@
         </is>
       </c>
       <c r="J60" s="4" t="n">
-        <v>9622</v>
+        <v>6306</v>
       </c>
       <c r="K60" s="5" t="n">
-        <v>370.0869565217391</v>
+        <v>242.52</v>
       </c>
     </row>
     <row r="61">
@@ -3565,7 +3565,7 @@
       </c>
       <c r="I62" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J62" s="8" t="n">
@@ -3605,11 +3605,11 @@
         </is>
       </c>
       <c r="G63" s="4" t="n">
-        <v>11032</v>
+        <v>13422</v>
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
-          <t>23/26</t>
+          <t>24/26</t>
         </is>
       </c>
       <c r="I63" s="3" t="inlineStr">
@@ -3618,10 +3618,10 @@
         </is>
       </c>
       <c r="J63" s="4" t="n">
-        <v>12471</v>
+        <v>14540</v>
       </c>
       <c r="K63" s="5" t="n">
-        <v>479.6521739130435</v>
+        <v>559.25</v>
       </c>
     </row>
     <row r="64">
@@ -3654,11 +3654,11 @@
         </is>
       </c>
       <c r="G64" s="4" t="n">
-        <v>7420</v>
+        <v>7938</v>
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>22/24</t>
+          <t>23/24</t>
         </is>
       </c>
       <c r="I64" s="3" t="inlineStr">
@@ -3667,59 +3667,59 @@
         </is>
       </c>
       <c r="J64" s="4" t="n">
-        <v>8095</v>
+        <v>8283</v>
       </c>
       <c r="K64" s="5" t="n">
-        <v>337.2727272727273</v>
+        <v>345.1304347826087</v>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="10" t="inlineStr">
+      <c r="A65" s="6" t="inlineStr">
         <is>
           <t>KANNIYAKUMARI</t>
         </is>
       </c>
-      <c r="B65" s="10" t="n">
+      <c r="B65" s="7" t="n">
         <v>229</v>
       </c>
-      <c r="C65" s="10" t="inlineStr">
+      <c r="C65" s="7" t="inlineStr">
         <is>
           <t>THALAVAI SUNDARAM. N</t>
         </is>
       </c>
-      <c r="D65" s="10" t="inlineStr">
+      <c r="D65" s="7" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E65" s="10" t="inlineStr">
+      <c r="E65" s="7" t="inlineStr">
         <is>
           <t>MAHESH.R</t>
         </is>
       </c>
-      <c r="F65" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G65" s="11" t="n">
-        <v>3795</v>
-      </c>
-      <c r="H65" s="10" t="inlineStr">
-        <is>
-          <t>24/34</t>
-        </is>
-      </c>
-      <c r="I65" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J65" s="11" t="n">
-        <v>5376</v>
-      </c>
-      <c r="K65" s="12" t="n">
-        <v>158.125</v>
+      <c r="F65" s="7" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G65" s="8" t="n">
+        <v>1770</v>
+      </c>
+      <c r="H65" s="7" t="inlineStr">
+        <is>
+          <t>25/34</t>
+        </is>
+      </c>
+      <c r="I65" s="7" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J65" s="8" t="n">
+        <v>2407</v>
+      </c>
+      <c r="K65" s="9" t="n">
+        <v>70.8</v>
       </c>
     </row>
     <row r="66">
@@ -3752,11 +3752,11 @@
         </is>
       </c>
       <c r="G66" s="4" t="n">
-        <v>40038</v>
+        <v>41498</v>
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>23/28</t>
+          <t>24/30</t>
         </is>
       </c>
       <c r="I66" s="3" t="inlineStr">
@@ -3765,10 +3765,10 @@
         </is>
       </c>
       <c r="J66" s="4" t="n">
-        <v>48742</v>
+        <v>51872</v>
       </c>
       <c r="K66" s="5" t="n">
-        <v>1740.782608695652</v>
+        <v>1729.083333333333</v>
       </c>
     </row>
     <row r="67">
@@ -3801,11 +3801,11 @@
         </is>
       </c>
       <c r="G67" s="8" t="n">
-        <v>1856</v>
+        <v>1340</v>
       </c>
       <c r="H67" s="7" t="inlineStr">
         <is>
-          <t>18/21</t>
+          <t>19/21</t>
         </is>
       </c>
       <c r="I67" s="7" t="inlineStr">
@@ -3814,10 +3814,10 @@
         </is>
       </c>
       <c r="J67" s="8" t="n">
-        <v>2165</v>
+        <v>1481</v>
       </c>
       <c r="K67" s="9" t="n">
-        <v>103.1111111111111</v>
+        <v>70.52631578947368</v>
       </c>
     </row>
     <row r="68">
@@ -3841,20 +3841,20 @@
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>DURAIMURUGAN</t>
+          <t>V. RAMU</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>Dravida Munnetra Kazhagam</t>
+          <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
       <c r="G68" s="4" t="n">
-        <v>5956</v>
+        <v>6142</v>
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>17/20</t>
+          <t>18/20</t>
         </is>
       </c>
       <c r="I68" s="3" t="inlineStr">
@@ -3863,10 +3863,10 @@
         </is>
       </c>
       <c r="J68" s="4" t="n">
-        <v>7007</v>
+        <v>6824</v>
       </c>
       <c r="K68" s="5" t="n">
-        <v>350.3529411764706</v>
+        <v>341.2222222222222</v>
       </c>
     </row>
     <row r="69">
@@ -3899,11 +3899,11 @@
         </is>
       </c>
       <c r="G69" s="4" t="n">
-        <v>31177</v>
+        <v>33063</v>
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
-          <t>20/21</t>
+          <t>22/22</t>
         </is>
       </c>
       <c r="I69" s="3" t="inlineStr">
@@ -3912,10 +3912,10 @@
         </is>
       </c>
       <c r="J69" s="4" t="n">
-        <v>32736</v>
+        <v>33063</v>
       </c>
       <c r="K69" s="5" t="n">
-        <v>1558.85</v>
+        <v>1502.863636363636</v>
       </c>
     </row>
     <row r="70">
@@ -4046,11 +4046,11 @@
         </is>
       </c>
       <c r="G72" s="4" t="n">
-        <v>30213</v>
+        <v>30465</v>
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>21/22</t>
+          <t>23/23</t>
         </is>
       </c>
       <c r="I72" s="3" t="inlineStr">
@@ -4059,10 +4059,10 @@
         </is>
       </c>
       <c r="J72" s="4" t="n">
-        <v>31652</v>
+        <v>30465</v>
       </c>
       <c r="K72" s="5" t="n">
-        <v>1438.714285714286</v>
+        <v>1324.565217391304</v>
       </c>
     </row>
     <row r="73">
@@ -4104,7 +4104,7 @@
       </c>
       <c r="I73" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J73" s="4" t="n">
@@ -4295,7 +4295,7 @@
       </c>
       <c r="H77" s="7" t="inlineStr">
         <is>
-          <t>23/23</t>
+          <t>23/25</t>
         </is>
       </c>
       <c r="I77" s="7" t="inlineStr">
@@ -4304,7 +4304,7 @@
         </is>
       </c>
       <c r="J77" s="8" t="n">
-        <v>962</v>
+        <v>1046</v>
       </c>
       <c r="K77" s="9" t="n">
         <v>41.82608695652174</v>
@@ -4349,7 +4349,7 @@
       </c>
       <c r="I78" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J78" s="4" t="n">
@@ -4389,11 +4389,11 @@
         </is>
       </c>
       <c r="G79" s="11" t="n">
-        <v>3528</v>
+        <v>3523</v>
       </c>
       <c r="H79" s="10" t="inlineStr">
         <is>
-          <t>19/20</t>
+          <t>20/21</t>
         </is>
       </c>
       <c r="I79" s="10" t="inlineStr">
@@ -4402,10 +4402,10 @@
         </is>
       </c>
       <c r="J79" s="11" t="n">
-        <v>3714</v>
+        <v>3699</v>
       </c>
       <c r="K79" s="12" t="n">
-        <v>185.6842105263158</v>
+        <v>176.15</v>
       </c>
     </row>
     <row r="80">
@@ -4487,11 +4487,11 @@
         </is>
       </c>
       <c r="G81" s="4" t="n">
-        <v>7772</v>
+        <v>7682</v>
       </c>
       <c r="H81" s="3" t="inlineStr">
         <is>
-          <t>22/24</t>
+          <t>23/24</t>
         </is>
       </c>
       <c r="I81" s="3" t="inlineStr">
@@ -4500,10 +4500,10 @@
         </is>
       </c>
       <c r="J81" s="4" t="n">
-        <v>8479</v>
+        <v>8016</v>
       </c>
       <c r="K81" s="5" t="n">
-        <v>353.2727272727273</v>
+        <v>334</v>
       </c>
     </row>
     <row r="82">
@@ -4683,11 +4683,11 @@
         </is>
       </c>
       <c r="G85" s="8" t="n">
-        <v>2731</v>
+        <v>2739</v>
       </c>
       <c r="H85" s="7" t="inlineStr">
         <is>
-          <t>20/21</t>
+          <t>21/21</t>
         </is>
       </c>
       <c r="I85" s="7" t="inlineStr">
@@ -4696,10 +4696,10 @@
         </is>
       </c>
       <c r="J85" s="8" t="n">
-        <v>2868</v>
+        <v>2739</v>
       </c>
       <c r="K85" s="9" t="n">
-        <v>136.55</v>
+        <v>130.4285714285714</v>
       </c>
     </row>
     <row r="86">
@@ -4732,11 +4732,11 @@
         </is>
       </c>
       <c r="G86" s="4" t="n">
-        <v>13089</v>
+        <v>14572</v>
       </c>
       <c r="H86" s="3" t="inlineStr">
         <is>
-          <t>19/21</t>
+          <t>20/21</t>
         </is>
       </c>
       <c r="I86" s="3" t="inlineStr">
@@ -4745,10 +4745,10 @@
         </is>
       </c>
       <c r="J86" s="4" t="n">
-        <v>14467</v>
+        <v>15301</v>
       </c>
       <c r="K86" s="5" t="n">
-        <v>688.8947368421053</v>
+        <v>728.6</v>
       </c>
     </row>
     <row r="87">
@@ -5026,11 +5026,11 @@
         </is>
       </c>
       <c r="G92" s="4" t="n">
-        <v>11291</v>
+        <v>11713</v>
       </c>
       <c r="H92" s="3" t="inlineStr">
         <is>
-          <t>23/24</t>
+          <t>24/24</t>
         </is>
       </c>
       <c r="I92" s="3" t="inlineStr">
@@ -5039,10 +5039,10 @@
         </is>
       </c>
       <c r="J92" s="4" t="n">
-        <v>11782</v>
+        <v>11713</v>
       </c>
       <c r="K92" s="5" t="n">
-        <v>490.9130434782609</v>
+        <v>488.0416666666667</v>
       </c>
     </row>
     <row r="93">
@@ -5124,7 +5124,7 @@
         </is>
       </c>
       <c r="G94" s="4" t="n">
-        <v>59717</v>
+        <v>59470</v>
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
@@ -5137,10 +5137,10 @@
         </is>
       </c>
       <c r="J94" s="4" t="n">
-        <v>64910</v>
+        <v>64641</v>
       </c>
       <c r="K94" s="5" t="n">
-        <v>2596.391304347826</v>
+        <v>2585.652173913043</v>
       </c>
     </row>
     <row r="95">
@@ -5271,11 +5271,11 @@
         </is>
       </c>
       <c r="G97" s="11" t="n">
-        <v>6662</v>
+        <v>2772</v>
       </c>
       <c r="H97" s="10" t="inlineStr">
         <is>
-          <t>20/27</t>
+          <t>21/27</t>
         </is>
       </c>
       <c r="I97" s="10" t="inlineStr">
@@ -5284,10 +5284,10 @@
         </is>
       </c>
       <c r="J97" s="11" t="n">
-        <v>8994</v>
+        <v>3564</v>
       </c>
       <c r="K97" s="12" t="n">
-        <v>333.1</v>
+        <v>132</v>
       </c>
     </row>
     <row r="98">
@@ -5819,7 +5819,7 @@
       </c>
       <c r="I108" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J108" s="4" t="n">
@@ -5908,11 +5908,11 @@
         </is>
       </c>
       <c r="G110" s="11" t="n">
-        <v>7284</v>
+        <v>8865</v>
       </c>
       <c r="H110" s="10" t="inlineStr">
         <is>
-          <t>15/23</t>
+          <t>16/23</t>
         </is>
       </c>
       <c r="I110" s="10" t="inlineStr">
@@ -5921,10 +5921,10 @@
         </is>
       </c>
       <c r="J110" s="11" t="n">
-        <v>11169</v>
+        <v>12743</v>
       </c>
       <c r="K110" s="12" t="n">
-        <v>485.6</v>
+        <v>554.0625</v>
       </c>
     </row>
     <row r="111">
@@ -6153,11 +6153,11 @@
         </is>
       </c>
       <c r="G115" s="11" t="n">
-        <v>3207</v>
+        <v>3038</v>
       </c>
       <c r="H115" s="10" t="inlineStr">
         <is>
-          <t>21/25</t>
+          <t>22/25</t>
         </is>
       </c>
       <c r="I115" s="10" t="inlineStr">
@@ -6166,10 +6166,10 @@
         </is>
       </c>
       <c r="J115" s="11" t="n">
-        <v>3818</v>
+        <v>3452</v>
       </c>
       <c r="K115" s="12" t="n">
-        <v>152.7142857142857</v>
+        <v>138.0909090909091</v>
       </c>
     </row>
     <row r="116">
@@ -6643,11 +6643,11 @@
         </is>
       </c>
       <c r="G125" s="4" t="n">
-        <v>45461</v>
+        <v>46706</v>
       </c>
       <c r="H125" s="3" t="inlineStr">
         <is>
-          <t>27/34</t>
+          <t>28/34</t>
         </is>
       </c>
       <c r="I125" s="3" t="inlineStr">
@@ -6656,10 +6656,10 @@
         </is>
       </c>
       <c r="J125" s="4" t="n">
-        <v>57247</v>
+        <v>56714</v>
       </c>
       <c r="K125" s="5" t="n">
-        <v>1683.740740740741</v>
+        <v>1668.071428571429</v>
       </c>
     </row>
     <row r="126">
@@ -6741,11 +6741,11 @@
         </is>
       </c>
       <c r="G127" s="8" t="n">
-        <v>2208</v>
+        <v>1648</v>
       </c>
       <c r="H127" s="7" t="inlineStr">
         <is>
-          <t>19/23</t>
+          <t>20/23</t>
         </is>
       </c>
       <c r="I127" s="7" t="inlineStr">
@@ -6754,10 +6754,10 @@
         </is>
       </c>
       <c r="J127" s="8" t="n">
-        <v>2673</v>
+        <v>1895</v>
       </c>
       <c r="K127" s="9" t="n">
-        <v>116.2105263157895</v>
+        <v>82.40000000000001</v>
       </c>
     </row>
     <row r="128">
@@ -6848,7 +6848,7 @@
       </c>
       <c r="I129" s="10" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J129" s="11" t="n">
@@ -6859,52 +6859,52 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="13" t="inlineStr">
+      <c r="A130" s="6" t="inlineStr">
         <is>
           <t>PARAMATHI-VELUR</t>
         </is>
       </c>
-      <c r="B130" s="14" t="n">
+      <c r="B130" s="7" t="n">
         <v>95</v>
       </c>
-      <c r="C130" s="14" t="inlineStr">
+      <c r="C130" s="7" t="inlineStr">
+        <is>
+          <t>SEKAR S</t>
+        </is>
+      </c>
+      <c r="D130" s="7" t="inlineStr">
+        <is>
+          <t>All India Anna Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E130" s="7" t="inlineStr">
         <is>
           <t>MOORTHIY K S</t>
         </is>
       </c>
-      <c r="D130" s="14" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E130" s="14" t="inlineStr">
-        <is>
-          <t>SEKAR S</t>
-        </is>
-      </c>
-      <c r="F130" s="14" t="inlineStr">
-        <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G130" s="15" t="n">
-        <v>82</v>
-      </c>
-      <c r="H130" s="14" t="inlineStr">
-        <is>
-          <t>17/20</t>
-        </is>
-      </c>
-      <c r="I130" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J130" s="15" t="n">
-        <v>96</v>
-      </c>
-      <c r="K130" s="16" t="n">
-        <v>4.823529411764706</v>
+      <c r="F130" s="7" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G130" s="8" t="n">
+        <v>665</v>
+      </c>
+      <c r="H130" s="7" t="inlineStr">
+        <is>
+          <t>18/20</t>
+        </is>
+      </c>
+      <c r="I130" s="7" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J130" s="8" t="n">
+        <v>739</v>
+      </c>
+      <c r="K130" s="9" t="n">
+        <v>36.94444444444444</v>
       </c>
     </row>
     <row r="131">
@@ -6937,11 +6937,11 @@
         </is>
       </c>
       <c r="G131" s="4" t="n">
-        <v>13887</v>
+        <v>13754</v>
       </c>
       <c r="H131" s="3" t="inlineStr">
         <is>
-          <t>22/24</t>
+          <t>24/24</t>
         </is>
       </c>
       <c r="I131" s="3" t="inlineStr">
@@ -6950,10 +6950,10 @@
         </is>
       </c>
       <c r="J131" s="4" t="n">
-        <v>15149</v>
+        <v>13754</v>
       </c>
       <c r="K131" s="5" t="n">
-        <v>631.2272727272727</v>
+        <v>573.0833333333334</v>
       </c>
     </row>
     <row r="132">
@@ -7084,11 +7084,11 @@
         </is>
       </c>
       <c r="G134" s="4" t="n">
-        <v>46624</v>
+        <v>49765</v>
       </c>
       <c r="H134" s="3" t="inlineStr">
         <is>
-          <t>19/22</t>
+          <t>20/22</t>
         </is>
       </c>
       <c r="I134" s="3" t="inlineStr">
@@ -7097,10 +7097,10 @@
         </is>
       </c>
       <c r="J134" s="4" t="n">
-        <v>53986</v>
+        <v>54742</v>
       </c>
       <c r="K134" s="5" t="n">
-        <v>2453.894736842105</v>
+        <v>2488.25</v>
       </c>
     </row>
     <row r="135">
@@ -7133,11 +7133,11 @@
         </is>
       </c>
       <c r="G135" s="8" t="n">
-        <v>927</v>
+        <v>415</v>
       </c>
       <c r="H135" s="7" t="inlineStr">
         <is>
-          <t>14/21</t>
+          <t>15/21</t>
         </is>
       </c>
       <c r="I135" s="7" t="inlineStr">
@@ -7146,10 +7146,10 @@
         </is>
       </c>
       <c r="J135" s="8" t="n">
-        <v>1390</v>
+        <v>581</v>
       </c>
       <c r="K135" s="9" t="n">
-        <v>66.21428571428571</v>
+        <v>27.66666666666667</v>
       </c>
     </row>
     <row r="136">
@@ -7378,11 +7378,11 @@
         </is>
       </c>
       <c r="G140" s="4" t="n">
-        <v>55529</v>
+        <v>55627</v>
       </c>
       <c r="H140" s="3" t="inlineStr">
         <is>
-          <t>24/26</t>
+          <t>25/26</t>
         </is>
       </c>
       <c r="I140" s="3" t="inlineStr">
@@ -7391,10 +7391,10 @@
         </is>
       </c>
       <c r="J140" s="4" t="n">
-        <v>60156</v>
+        <v>57852</v>
       </c>
       <c r="K140" s="5" t="n">
-        <v>2313.708333333333</v>
+        <v>2225.08</v>
       </c>
     </row>
     <row r="141">
@@ -7427,11 +7427,11 @@
         </is>
       </c>
       <c r="G141" s="4" t="n">
-        <v>5850</v>
+        <v>5928</v>
       </c>
       <c r="H141" s="3" t="inlineStr">
         <is>
-          <t>19/25</t>
+          <t>20/25</t>
         </is>
       </c>
       <c r="I141" s="3" t="inlineStr">
@@ -7440,10 +7440,10 @@
         </is>
       </c>
       <c r="J141" s="4" t="n">
-        <v>7697</v>
+        <v>7410</v>
       </c>
       <c r="K141" s="5" t="n">
-        <v>307.8947368421053</v>
+        <v>296.4</v>
       </c>
     </row>
     <row r="142">
@@ -7819,11 +7819,11 @@
         </is>
       </c>
       <c r="G149" s="11" t="n">
-        <v>4870</v>
+        <v>4997</v>
       </c>
       <c r="H149" s="10" t="inlineStr">
         <is>
-          <t>19/25</t>
+          <t>20/25</t>
         </is>
       </c>
       <c r="I149" s="10" t="inlineStr">
@@ -7832,10 +7832,10 @@
         </is>
       </c>
       <c r="J149" s="11" t="n">
-        <v>6408</v>
+        <v>6246</v>
       </c>
       <c r="K149" s="12" t="n">
-        <v>256.3157894736842</v>
+        <v>249.85</v>
       </c>
     </row>
     <row r="150">
@@ -7966,23 +7966,23 @@
         </is>
       </c>
       <c r="G152" s="4" t="n">
-        <v>13898</v>
+        <v>14034</v>
       </c>
       <c r="H152" s="3" t="inlineStr">
         <is>
-          <t>21/23</t>
+          <t>23/23</t>
         </is>
       </c>
       <c r="I152" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J152" s="4" t="n">
-        <v>15222</v>
+        <v>14034</v>
       </c>
       <c r="K152" s="5" t="n">
-        <v>661.8095238095239</v>
+        <v>610.1739130434783</v>
       </c>
     </row>
     <row r="153">
@@ -8143,30 +8143,30 @@
       </c>
       <c r="C156" s="7" t="inlineStr">
         <is>
+          <t>UDHAYASURIYAN T</t>
+        </is>
+      </c>
+      <c r="D156" s="7" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E156" s="7" t="inlineStr">
+        <is>
           <t>RAKESH R</t>
         </is>
       </c>
-      <c r="D156" s="7" t="inlineStr">
+      <c r="F156" s="7" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E156" s="7" t="inlineStr">
-        <is>
-          <t>UDHAYASURIYAN T</t>
-        </is>
-      </c>
-      <c r="F156" s="7" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
       <c r="G156" s="8" t="n">
-        <v>1242</v>
+        <v>475</v>
       </c>
       <c r="H156" s="7" t="inlineStr">
         <is>
-          <t>18/25</t>
+          <t>20/25</t>
         </is>
       </c>
       <c r="I156" s="7" t="inlineStr">
@@ -8175,10 +8175,10 @@
         </is>
       </c>
       <c r="J156" s="8" t="n">
-        <v>1725</v>
+        <v>594</v>
       </c>
       <c r="K156" s="9" t="n">
-        <v>69</v>
+        <v>23.75</v>
       </c>
     </row>
     <row r="157">
@@ -8220,7 +8220,7 @@
       </c>
       <c r="I157" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J157" s="4" t="n">
@@ -8260,11 +8260,11 @@
         </is>
       </c>
       <c r="G158" s="4" t="n">
-        <v>5111</v>
+        <v>5443</v>
       </c>
       <c r="H158" s="3" t="inlineStr">
         <is>
-          <t>18/21</t>
+          <t>19/21</t>
         </is>
       </c>
       <c r="I158" s="3" t="inlineStr">
@@ -8273,10 +8273,10 @@
         </is>
       </c>
       <c r="J158" s="4" t="n">
-        <v>5963</v>
+        <v>6016</v>
       </c>
       <c r="K158" s="5" t="n">
-        <v>283.9444444444445</v>
+        <v>286.4736842105263</v>
       </c>
     </row>
     <row r="159">
@@ -8358,23 +8358,23 @@
         </is>
       </c>
       <c r="G160" s="8" t="n">
-        <v>1622</v>
+        <v>2678</v>
       </c>
       <c r="H160" s="7" t="inlineStr">
         <is>
-          <t>18/19</t>
+          <t>19/19</t>
         </is>
       </c>
       <c r="I160" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J160" s="8" t="n">
-        <v>1712</v>
+        <v>2678</v>
       </c>
       <c r="K160" s="9" t="n">
-        <v>90.11111111111111</v>
+        <v>140.9473684210526</v>
       </c>
     </row>
     <row r="161">
@@ -8407,11 +8407,11 @@
         </is>
       </c>
       <c r="G161" s="11" t="n">
-        <v>4240</v>
+        <v>2475</v>
       </c>
       <c r="H161" s="10" t="inlineStr">
         <is>
-          <t>17/25</t>
+          <t>18/25</t>
         </is>
       </c>
       <c r="I161" s="10" t="inlineStr">
@@ -8420,10 +8420,10 @@
         </is>
       </c>
       <c r="J161" s="11" t="n">
-        <v>6235</v>
+        <v>3438</v>
       </c>
       <c r="K161" s="12" t="n">
-        <v>249.4117647058823</v>
+        <v>137.5</v>
       </c>
     </row>
     <row r="162">
@@ -8456,11 +8456,11 @@
         </is>
       </c>
       <c r="G162" s="4" t="n">
-        <v>75780</v>
+        <v>77452</v>
       </c>
       <c r="H162" s="3" t="inlineStr">
         <is>
-          <t>24/30</t>
+          <t>25/30</t>
         </is>
       </c>
       <c r="I162" s="3" t="inlineStr">
@@ -8469,10 +8469,10 @@
         </is>
       </c>
       <c r="J162" s="4" t="n">
-        <v>94725</v>
+        <v>92942</v>
       </c>
       <c r="K162" s="5" t="n">
-        <v>3157.5</v>
+        <v>3098.08</v>
       </c>
     </row>
     <row r="163">
@@ -8505,11 +8505,11 @@
         </is>
       </c>
       <c r="G163" s="4" t="n">
-        <v>18219</v>
+        <v>18965</v>
       </c>
       <c r="H163" s="3" t="inlineStr">
         <is>
-          <t>23/26</t>
+          <t>24/27</t>
         </is>
       </c>
       <c r="I163" s="3" t="inlineStr">
@@ -8518,10 +8518,10 @@
         </is>
       </c>
       <c r="J163" s="4" t="n">
-        <v>20595</v>
+        <v>21336</v>
       </c>
       <c r="K163" s="5" t="n">
-        <v>792.1304347826087</v>
+        <v>790.2083333333334</v>
       </c>
     </row>
     <row r="164">
@@ -8563,7 +8563,7 @@
       </c>
       <c r="I164" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J164" s="4" t="n">
@@ -8652,11 +8652,11 @@
         </is>
       </c>
       <c r="G166" s="4" t="n">
-        <v>10455</v>
+        <v>11670</v>
       </c>
       <c r="H166" s="3" t="inlineStr">
         <is>
-          <t>20/21</t>
+          <t>22/22</t>
         </is>
       </c>
       <c r="I166" s="3" t="inlineStr">
@@ -8665,10 +8665,10 @@
         </is>
       </c>
       <c r="J166" s="4" t="n">
-        <v>10978</v>
+        <v>11670</v>
       </c>
       <c r="K166" s="5" t="n">
-        <v>522.75</v>
+        <v>530.4545454545455</v>
       </c>
     </row>
     <row r="167">
@@ -8701,11 +8701,11 @@
         </is>
       </c>
       <c r="G167" s="4" t="n">
-        <v>44141</v>
+        <v>45556</v>
       </c>
       <c r="H167" s="3" t="inlineStr">
         <is>
-          <t>26/32</t>
+          <t>27/32</t>
         </is>
       </c>
       <c r="I167" s="3" t="inlineStr">
@@ -8714,10 +8714,10 @@
         </is>
       </c>
       <c r="J167" s="4" t="n">
-        <v>54327</v>
+        <v>53992</v>
       </c>
       <c r="K167" s="5" t="n">
-        <v>1697.730769230769</v>
+        <v>1687.259259259259</v>
       </c>
     </row>
     <row r="168">
@@ -8750,11 +8750,11 @@
         </is>
       </c>
       <c r="G168" s="4" t="n">
-        <v>34086</v>
+        <v>33941</v>
       </c>
       <c r="H168" s="3" t="inlineStr">
         <is>
-          <t>23/28</t>
+          <t>24/28</t>
         </is>
       </c>
       <c r="I168" s="3" t="inlineStr">
@@ -8763,10 +8763,10 @@
         </is>
       </c>
       <c r="J168" s="4" t="n">
-        <v>41496</v>
+        <v>39598</v>
       </c>
       <c r="K168" s="5" t="n">
-        <v>1482</v>
+        <v>1414.208333333333</v>
       </c>
     </row>
     <row r="169">
@@ -8848,11 +8848,11 @@
         </is>
       </c>
       <c r="G170" s="4" t="n">
-        <v>7265</v>
+        <v>8097</v>
       </c>
       <c r="H170" s="3" t="inlineStr">
         <is>
-          <t>20/23</t>
+          <t>21/23</t>
         </is>
       </c>
       <c r="I170" s="3" t="inlineStr">
@@ -8861,10 +8861,10 @@
         </is>
       </c>
       <c r="J170" s="4" t="n">
-        <v>8355</v>
+        <v>8868</v>
       </c>
       <c r="K170" s="5" t="n">
-        <v>363.25</v>
+        <v>385.5714285714286</v>
       </c>
     </row>
     <row r="171">
@@ -8897,11 +8897,11 @@
         </is>
       </c>
       <c r="G171" s="4" t="n">
-        <v>5267</v>
+        <v>5248</v>
       </c>
       <c r="H171" s="3" t="inlineStr">
         <is>
-          <t>29/32</t>
+          <t>30/35</t>
         </is>
       </c>
       <c r="I171" s="3" t="inlineStr">
@@ -8910,10 +8910,10 @@
         </is>
       </c>
       <c r="J171" s="4" t="n">
-        <v>5812</v>
+        <v>6123</v>
       </c>
       <c r="K171" s="5" t="n">
-        <v>181.6206896551724</v>
+        <v>174.9333333333333</v>
       </c>
     </row>
     <row r="172">
@@ -8946,11 +8946,11 @@
         </is>
       </c>
       <c r="G172" s="4" t="n">
-        <v>35937</v>
+        <v>35621</v>
       </c>
       <c r="H172" s="3" t="inlineStr">
         <is>
-          <t>37/39</t>
+          <t>39/39</t>
         </is>
       </c>
       <c r="I172" s="3" t="inlineStr">
@@ -8959,10 +8959,10 @@
         </is>
       </c>
       <c r="J172" s="4" t="n">
-        <v>37880</v>
+        <v>35621</v>
       </c>
       <c r="K172" s="5" t="n">
-        <v>971.2702702702703</v>
+        <v>913.3589743589744</v>
       </c>
     </row>
     <row r="173">
@@ -8995,11 +8995,11 @@
         </is>
       </c>
       <c r="G173" s="4" t="n">
-        <v>9746</v>
+        <v>9776</v>
       </c>
       <c r="H173" s="3" t="inlineStr">
         <is>
-          <t>24/26</t>
+          <t>25/26</t>
         </is>
       </c>
       <c r="I173" s="3" t="inlineStr">
@@ -9008,10 +9008,10 @@
         </is>
       </c>
       <c r="J173" s="4" t="n">
-        <v>10558</v>
+        <v>10167</v>
       </c>
       <c r="K173" s="5" t="n">
-        <v>406.0833333333333</v>
+        <v>391.04</v>
       </c>
     </row>
     <row r="174">
@@ -9044,11 +9044,11 @@
         </is>
       </c>
       <c r="G174" s="11" t="n">
-        <v>2856</v>
+        <v>2643</v>
       </c>
       <c r="H174" s="10" t="inlineStr">
         <is>
-          <t>20/24</t>
+          <t>21/24</t>
         </is>
       </c>
       <c r="I174" s="10" t="inlineStr">
@@ -9057,10 +9057,10 @@
         </is>
       </c>
       <c r="J174" s="11" t="n">
-        <v>3427</v>
+        <v>3021</v>
       </c>
       <c r="K174" s="12" t="n">
-        <v>142.8</v>
+        <v>125.8571428571429</v>
       </c>
     </row>
     <row r="175">
@@ -9240,7 +9240,7 @@
         </is>
       </c>
       <c r="G178" s="8" t="n">
-        <v>507</v>
+        <v>786</v>
       </c>
       <c r="H178" s="7" t="inlineStr">
         <is>
@@ -9253,10 +9253,10 @@
         </is>
       </c>
       <c r="J178" s="8" t="n">
-        <v>558</v>
+        <v>865</v>
       </c>
       <c r="K178" s="9" t="n">
-        <v>25.35</v>
+        <v>39.3</v>
       </c>
     </row>
     <row r="179">
@@ -9289,11 +9289,11 @@
         </is>
       </c>
       <c r="G179" s="4" t="n">
-        <v>37938</v>
+        <v>40016</v>
       </c>
       <c r="H179" s="3" t="inlineStr">
         <is>
-          <t>23/26</t>
+          <t>24/26</t>
         </is>
       </c>
       <c r="I179" s="3" t="inlineStr">
@@ -9302,10 +9302,10 @@
         </is>
       </c>
       <c r="J179" s="4" t="n">
-        <v>42886</v>
+        <v>43351</v>
       </c>
       <c r="K179" s="5" t="n">
-        <v>1649.478260869565</v>
+        <v>1667.333333333333</v>
       </c>
     </row>
     <row r="180">
@@ -9338,11 +9338,11 @@
         </is>
       </c>
       <c r="G180" s="4" t="n">
-        <v>34361</v>
+        <v>36383</v>
       </c>
       <c r="H180" s="3" t="inlineStr">
         <is>
-          <t>22/29</t>
+          <t>24/29</t>
         </is>
       </c>
       <c r="I180" s="3" t="inlineStr">
@@ -9351,10 +9351,10 @@
         </is>
       </c>
       <c r="J180" s="4" t="n">
-        <v>45294</v>
+        <v>43963</v>
       </c>
       <c r="K180" s="5" t="n">
-        <v>1561.863636363636</v>
+        <v>1515.958333333333</v>
       </c>
     </row>
     <row r="181">
@@ -9583,11 +9583,11 @@
         </is>
       </c>
       <c r="G185" s="4" t="n">
-        <v>7811</v>
+        <v>8720</v>
       </c>
       <c r="H185" s="3" t="inlineStr">
         <is>
-          <t>21/23</t>
+          <t>22/24</t>
         </is>
       </c>
       <c r="I185" s="3" t="inlineStr">
@@ -9596,10 +9596,10 @@
         </is>
       </c>
       <c r="J185" s="4" t="n">
-        <v>8555</v>
+        <v>9513</v>
       </c>
       <c r="K185" s="5" t="n">
-        <v>371.952380952381</v>
+        <v>396.3636363636364</v>
       </c>
     </row>
     <row r="186">
@@ -9779,11 +9779,11 @@
         </is>
       </c>
       <c r="G189" s="4" t="n">
-        <v>14196</v>
+        <v>14785</v>
       </c>
       <c r="H189" s="3" t="inlineStr">
         <is>
-          <t>24/27</t>
+          <t>25/27</t>
         </is>
       </c>
       <c r="I189" s="3" t="inlineStr">
@@ -9792,10 +9792,10 @@
         </is>
       </c>
       <c r="J189" s="4" t="n">
-        <v>15970</v>
+        <v>15968</v>
       </c>
       <c r="K189" s="5" t="n">
-        <v>591.5</v>
+        <v>591.4</v>
       </c>
     </row>
     <row r="190">
@@ -10073,11 +10073,11 @@
         </is>
       </c>
       <c r="G195" s="4" t="n">
-        <v>27265</v>
+        <v>28172</v>
       </c>
       <c r="H195" s="3" t="inlineStr">
         <is>
-          <t>20/22</t>
+          <t>22/22</t>
         </is>
       </c>
       <c r="I195" s="3" t="inlineStr">
@@ -10086,10 +10086,10 @@
         </is>
       </c>
       <c r="J195" s="4" t="n">
-        <v>29992</v>
+        <v>28172</v>
       </c>
       <c r="K195" s="5" t="n">
-        <v>1363.25</v>
+        <v>1280.545454545455</v>
       </c>
     </row>
     <row r="196">
@@ -10220,11 +10220,11 @@
         </is>
       </c>
       <c r="G198" s="4" t="n">
-        <v>10615</v>
+        <v>11276</v>
       </c>
       <c r="H198" s="3" t="inlineStr">
         <is>
-          <t>18/21</t>
+          <t>19/21</t>
         </is>
       </c>
       <c r="I198" s="3" t="inlineStr">
@@ -10233,10 +10233,10 @@
         </is>
       </c>
       <c r="J198" s="4" t="n">
-        <v>12384</v>
+        <v>12463</v>
       </c>
       <c r="K198" s="5" t="n">
-        <v>589.7222222222222</v>
+        <v>593.4736842105264</v>
       </c>
     </row>
     <row r="199">
@@ -10269,7 +10269,7 @@
         </is>
       </c>
       <c r="G199" s="15" t="n">
-        <v>254</v>
+        <v>69</v>
       </c>
       <c r="H199" s="14" t="inlineStr">
         <is>
@@ -10282,10 +10282,10 @@
         </is>
       </c>
       <c r="J199" s="15" t="n">
-        <v>277</v>
+        <v>75</v>
       </c>
       <c r="K199" s="16" t="n">
-        <v>11.54545454545454</v>
+        <v>3.136363636363636</v>
       </c>
     </row>
     <row r="200">
@@ -10416,11 +10416,11 @@
         </is>
       </c>
       <c r="G202" s="8" t="n">
-        <v>2237</v>
+        <v>1738</v>
       </c>
       <c r="H202" s="7" t="inlineStr">
         <is>
-          <t>23/27</t>
+          <t>24/27</t>
         </is>
       </c>
       <c r="I202" s="7" t="inlineStr">
@@ -10429,10 +10429,10 @@
         </is>
       </c>
       <c r="J202" s="8" t="n">
-        <v>2626</v>
+        <v>1955</v>
       </c>
       <c r="K202" s="9" t="n">
-        <v>97.26086956521739</v>
+        <v>72.41666666666667</v>
       </c>
     </row>
     <row r="203">
@@ -10465,11 +10465,11 @@
         </is>
       </c>
       <c r="G203" s="4" t="n">
-        <v>60629</v>
+        <v>62316</v>
       </c>
       <c r="H203" s="3" t="inlineStr">
         <is>
-          <t>27/32</t>
+          <t>28/34</t>
         </is>
       </c>
       <c r="I203" s="3" t="inlineStr">
@@ -10478,10 +10478,10 @@
         </is>
       </c>
       <c r="J203" s="4" t="n">
-        <v>71857</v>
+        <v>75669</v>
       </c>
       <c r="K203" s="5" t="n">
-        <v>2245.518518518519</v>
+        <v>2225.571428571428</v>
       </c>
     </row>
     <row r="204">
@@ -10514,11 +10514,11 @@
         </is>
       </c>
       <c r="G204" s="4" t="n">
-        <v>11969</v>
+        <v>12901</v>
       </c>
       <c r="H204" s="3" t="inlineStr">
         <is>
-          <t>20/21</t>
+          <t>21/21</t>
         </is>
       </c>
       <c r="I204" s="3" t="inlineStr">
@@ -10527,10 +10527,10 @@
         </is>
       </c>
       <c r="J204" s="4" t="n">
-        <v>12567</v>
+        <v>12901</v>
       </c>
       <c r="K204" s="5" t="n">
-        <v>598.45</v>
+        <v>614.3333333333334</v>
       </c>
     </row>
     <row r="205">
@@ -10563,11 +10563,11 @@
         </is>
       </c>
       <c r="G205" s="4" t="n">
-        <v>6905</v>
+        <v>6679</v>
       </c>
       <c r="H205" s="3" t="inlineStr">
         <is>
-          <t>19/25</t>
+          <t>20/25</t>
         </is>
       </c>
       <c r="I205" s="3" t="inlineStr">
@@ -10576,10 +10576,10 @@
         </is>
       </c>
       <c r="J205" s="4" t="n">
-        <v>9086</v>
+        <v>8349</v>
       </c>
       <c r="K205" s="5" t="n">
-        <v>363.421052631579</v>
+        <v>333.95</v>
       </c>
     </row>
     <row r="206">
@@ -10661,11 +10661,11 @@
         </is>
       </c>
       <c r="G207" s="8" t="n">
-        <v>402</v>
+        <v>646</v>
       </c>
       <c r="H207" s="7" t="inlineStr">
         <is>
-          <t>16/23</t>
+          <t>17/23</t>
         </is>
       </c>
       <c r="I207" s="7" t="inlineStr">
@@ -10674,10 +10674,10 @@
         </is>
       </c>
       <c r="J207" s="8" t="n">
-        <v>578</v>
+        <v>874</v>
       </c>
       <c r="K207" s="9" t="n">
-        <v>25.125</v>
+        <v>38</v>
       </c>
     </row>
     <row r="208">
@@ -10710,11 +10710,11 @@
         </is>
       </c>
       <c r="G208" s="8" t="n">
-        <v>1445</v>
+        <v>2190</v>
       </c>
       <c r="H208" s="7" t="inlineStr">
         <is>
-          <t>18/20</t>
+          <t>19/20</t>
         </is>
       </c>
       <c r="I208" s="7" t="inlineStr">
@@ -10723,10 +10723,10 @@
         </is>
       </c>
       <c r="J208" s="8" t="n">
-        <v>1606</v>
+        <v>2305</v>
       </c>
       <c r="K208" s="9" t="n">
-        <v>80.27777777777777</v>
+        <v>115.2631578947368</v>
       </c>
     </row>
     <row r="209">
@@ -10906,11 +10906,11 @@
         </is>
       </c>
       <c r="G212" s="8" t="n">
-        <v>2374</v>
+        <v>1617</v>
       </c>
       <c r="H212" s="7" t="inlineStr">
         <is>
-          <t>22/25</t>
+          <t>24/25</t>
         </is>
       </c>
       <c r="I212" s="7" t="inlineStr">
@@ -10919,10 +10919,10 @@
         </is>
       </c>
       <c r="J212" s="8" t="n">
-        <v>2698</v>
+        <v>1684</v>
       </c>
       <c r="K212" s="9" t="n">
-        <v>107.9090909090909</v>
+        <v>67.375</v>
       </c>
     </row>
     <row r="213">
@@ -11160,7 +11160,7 @@
       </c>
       <c r="I217" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J217" s="8" t="n">
@@ -11347,11 +11347,11 @@
         </is>
       </c>
       <c r="G221" s="4" t="n">
-        <v>9922</v>
+        <v>10063</v>
       </c>
       <c r="H221" s="3" t="inlineStr">
         <is>
-          <t>25/27</t>
+          <t>27/27</t>
         </is>
       </c>
       <c r="I221" s="3" t="inlineStr">
@@ -11360,10 +11360,10 @@
         </is>
       </c>
       <c r="J221" s="4" t="n">
-        <v>10716</v>
+        <v>10063</v>
       </c>
       <c r="K221" s="5" t="n">
-        <v>396.88</v>
+        <v>372.7037037037037</v>
       </c>
     </row>
     <row r="222">
@@ -11543,11 +11543,11 @@
         </is>
       </c>
       <c r="G225" s="15" t="n">
-        <v>272</v>
+        <v>126</v>
       </c>
       <c r="H225" s="14" t="inlineStr">
         <is>
-          <t>25/27</t>
+          <t>26/27</t>
         </is>
       </c>
       <c r="I225" s="14" t="inlineStr">
@@ -11556,10 +11556,10 @@
         </is>
       </c>
       <c r="J225" s="15" t="n">
-        <v>294</v>
+        <v>131</v>
       </c>
       <c r="K225" s="16" t="n">
-        <v>10.88</v>
+        <v>4.846153846153846</v>
       </c>
     </row>
     <row r="226">
@@ -11886,11 +11886,11 @@
         </is>
       </c>
       <c r="G232" s="4" t="n">
-        <v>9206</v>
+        <v>9375</v>
       </c>
       <c r="H232" s="3" t="inlineStr">
         <is>
-          <t>21/23</t>
+          <t>22/23</t>
         </is>
       </c>
       <c r="I232" s="3" t="inlineStr">
@@ -11899,10 +11899,10 @@
         </is>
       </c>
       <c r="J232" s="4" t="n">
-        <v>10083</v>
+        <v>9801</v>
       </c>
       <c r="K232" s="5" t="n">
-        <v>438.3809523809524</v>
+        <v>426.1363636363636</v>
       </c>
     </row>
     <row r="233">
@@ -11935,11 +11935,11 @@
         </is>
       </c>
       <c r="G233" s="4" t="n">
-        <v>22165</v>
+        <v>24052</v>
       </c>
       <c r="H233" s="3" t="inlineStr">
         <is>
-          <t>19/23</t>
+          <t>20/23</t>
         </is>
       </c>
       <c r="I233" s="3" t="inlineStr">
@@ -11948,10 +11948,10 @@
         </is>
       </c>
       <c r="J233" s="4" t="n">
-        <v>26831</v>
+        <v>27660</v>
       </c>
       <c r="K233" s="5" t="n">
-        <v>1166.578947368421</v>
+        <v>1202.6</v>
       </c>
     </row>
     <row r="234">
@@ -12004,52 +12004,52 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="13" t="inlineStr">
+      <c r="A235" s="6" t="inlineStr">
         <is>
           <t>YERCAUD</t>
         </is>
       </c>
-      <c r="B235" s="14" t="n">
+      <c r="B235" s="7" t="n">
         <v>83</v>
       </c>
-      <c r="C235" s="14" t="inlineStr">
+      <c r="C235" s="7" t="inlineStr">
+        <is>
+          <t>USHARANI. P</t>
+        </is>
+      </c>
+      <c r="D235" s="7" t="inlineStr">
+        <is>
+          <t>All India Anna Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E235" s="7" t="inlineStr">
         <is>
           <t>LAKSHMI JANARTHANAN. J</t>
         </is>
       </c>
-      <c r="D235" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E235" s="14" t="inlineStr">
-        <is>
-          <t>USHARANI. P</t>
-        </is>
-      </c>
-      <c r="F235" s="14" t="inlineStr">
-        <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G235" s="15" t="n">
-        <v>312</v>
-      </c>
-      <c r="H235" s="14" t="inlineStr">
-        <is>
-          <t>22/24</t>
-        </is>
-      </c>
-      <c r="I235" s="14" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J235" s="15" t="n">
-        <v>340</v>
-      </c>
-      <c r="K235" s="16" t="n">
-        <v>14.18181818181818</v>
+      <c r="F235" s="7" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G235" s="8" t="n">
+        <v>564</v>
+      </c>
+      <c r="H235" s="7" t="inlineStr">
+        <is>
+          <t>23/24</t>
+        </is>
+      </c>
+      <c r="I235" s="7" t="inlineStr">
+        <is>
+          <t>Result in Progress</t>
+        </is>
+      </c>
+      <c r="J235" s="8" t="n">
+        <v>589</v>
+      </c>
+      <c r="K235" s="9" t="n">
+        <v>24.52173913043478</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Election snapshot: 97.8% counted — 144 declared, TVK 106, DMK 59, AIADMK 47
49 results declared; TIRUKKOYILUR flipped to AIADMK; POLUR (DMDK 67 votes, 8 rounds left).

https://claude.ai/code/session_01MizbUy44JG5sXyvaf3Wekb
</commit_message>
<xml_diff>
--- a/tn_election_results_may2026.xlsx
+++ b/tn_election_results_may2026.xlsx
@@ -616,11 +616,11 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>24195</v>
+        <v>26334</v>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>24/31</t>
+          <t>27/31</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -629,10 +629,10 @@
         </is>
       </c>
       <c r="J2" s="4" t="n">
-        <v>31252</v>
+        <v>30235</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>1008.125</v>
+        <v>975.3333333333334</v>
       </c>
     </row>
     <row r="3">
@@ -816,7 +816,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>27/27</t>
+          <t>27/28</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -825,7 +825,7 @@
         </is>
       </c>
       <c r="J6" s="4" t="n">
-        <v>57844</v>
+        <v>59986</v>
       </c>
       <c r="K6" s="5" t="n">
         <v>2142.37037037037</v>
@@ -861,11 +861,11 @@
         </is>
       </c>
       <c r="G7" s="4" t="n">
-        <v>8610</v>
+        <v>7875</v>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>20/22</t>
+          <t>21/22</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -874,10 +874,10 @@
         </is>
       </c>
       <c r="J7" s="4" t="n">
-        <v>9471</v>
+        <v>8250</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>430.5</v>
+        <v>375</v>
       </c>
     </row>
     <row r="8">
@@ -968,7 +968,7 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J9" s="4" t="n">
@@ -1302,23 +1302,23 @@
         </is>
       </c>
       <c r="G16" s="4" t="n">
-        <v>37822</v>
+        <v>42720</v>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>21/23</t>
+          <t>23/23</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J16" s="4" t="n">
-        <v>41424</v>
+        <v>42720</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>1801.047619047619</v>
+        <v>1857.391304347826</v>
       </c>
     </row>
     <row r="17">
@@ -1400,23 +1400,23 @@
         </is>
       </c>
       <c r="G18" s="11" t="n">
-        <v>3885</v>
+        <v>4943</v>
       </c>
       <c r="H18" s="10" t="inlineStr">
         <is>
-          <t>18/20</t>
+          <t>20/20</t>
         </is>
       </c>
       <c r="I18" s="10" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J18" s="11" t="n">
-        <v>4317</v>
+        <v>4943</v>
       </c>
       <c r="K18" s="12" t="n">
-        <v>215.8333333333333</v>
+        <v>247.15</v>
       </c>
     </row>
     <row r="19">
@@ -1449,23 +1449,23 @@
         </is>
       </c>
       <c r="G19" s="4" t="n">
-        <v>22240</v>
+        <v>22368</v>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>25/26</t>
+          <t>26/26</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J19" s="4" t="n">
-        <v>23130</v>
+        <v>22368</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>889.6</v>
+        <v>860.3076923076923</v>
       </c>
     </row>
     <row r="20">
@@ -1547,11 +1547,11 @@
         </is>
       </c>
       <c r="G21" s="4" t="n">
-        <v>70239</v>
+        <v>76311</v>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>23/26</t>
+          <t>27/27</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -1560,10 +1560,10 @@
         </is>
       </c>
       <c r="J21" s="4" t="n">
-        <v>79401</v>
+        <v>76311</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>3053.869565217391</v>
+        <v>2826.333333333333</v>
       </c>
     </row>
     <row r="22">
@@ -1645,11 +1645,11 @@
         </is>
       </c>
       <c r="G23" s="11" t="n">
-        <v>4182</v>
+        <v>4536</v>
       </c>
       <c r="H23" s="10" t="inlineStr">
         <is>
-          <t>22/24</t>
+          <t>23/24</t>
         </is>
       </c>
       <c r="I23" s="10" t="inlineStr">
@@ -1658,10 +1658,10 @@
         </is>
       </c>
       <c r="J23" s="11" t="n">
-        <v>4562</v>
+        <v>4733</v>
       </c>
       <c r="K23" s="12" t="n">
-        <v>190.0909090909091</v>
+        <v>197.2173913043478</v>
       </c>
     </row>
     <row r="24">
@@ -1763,52 +1763,52 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="10" t="inlineStr">
+      <c r="A26" s="6" t="inlineStr">
         <is>
           <t>BHUVANAGIRI</t>
         </is>
       </c>
-      <c r="B26" s="10" t="n">
+      <c r="B26" s="7" t="n">
         <v>157</v>
       </c>
-      <c r="C26" s="10" t="inlineStr">
+      <c r="C26" s="7" t="inlineStr">
         <is>
           <t>ARUNMOZHITHEVAN . A</t>
         </is>
       </c>
-      <c r="D26" s="10" t="inlineStr">
+      <c r="D26" s="7" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E26" s="10" t="inlineStr">
+      <c r="E26" s="7" t="inlineStr">
         <is>
           <t>SARAVANAN. DURAI . K</t>
         </is>
       </c>
-      <c r="F26" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G26" s="11" t="n">
-        <v>3966</v>
-      </c>
-      <c r="H26" s="10" t="inlineStr">
-        <is>
-          <t>21/22</t>
-        </is>
-      </c>
-      <c r="I26" s="10" t="inlineStr">
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="n">
+        <v>2487</v>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>26/26</t>
+        </is>
+      </c>
+      <c r="I26" s="7" t="inlineStr">
         <is>
           <t>Result in Progress</t>
         </is>
       </c>
-      <c r="J26" s="11" t="n">
-        <v>4155</v>
-      </c>
-      <c r="K26" s="12" t="n">
-        <v>188.8571428571429</v>
+      <c r="J26" s="8" t="n">
+        <v>2487</v>
+      </c>
+      <c r="K26" s="9" t="n">
+        <v>95.65384615384616</v>
       </c>
     </row>
     <row r="27">
@@ -1890,11 +1890,11 @@
         </is>
       </c>
       <c r="G28" s="4" t="n">
-        <v>25958</v>
+        <v>32441</v>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>23/36</t>
+          <t>28/36</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
@@ -1903,10 +1903,10 @@
         </is>
       </c>
       <c r="J28" s="4" t="n">
-        <v>40630</v>
+        <v>41710</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>1128.608695652174</v>
+        <v>1158.607142857143</v>
       </c>
     </row>
     <row r="29">
@@ -1939,7 +1939,7 @@
         </is>
       </c>
       <c r="G29" s="4" t="n">
-        <v>14252</v>
+        <v>14562</v>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
@@ -1952,10 +1952,10 @@
         </is>
       </c>
       <c r="J29" s="4" t="n">
-        <v>15491</v>
+        <v>15828</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>619.6521739130435</v>
+        <v>633.1304347826087</v>
       </c>
     </row>
     <row r="30">
@@ -2135,11 +2135,11 @@
         </is>
       </c>
       <c r="G33" s="4" t="n">
-        <v>6339</v>
+        <v>5773</v>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>20/22</t>
+          <t>22/24</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -2148,10 +2148,10 @@
         </is>
       </c>
       <c r="J33" s="4" t="n">
-        <v>6973</v>
+        <v>6298</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>316.95</v>
+        <v>262.4090909090909</v>
       </c>
     </row>
     <row r="34">
@@ -2184,11 +2184,11 @@
         </is>
       </c>
       <c r="G34" s="4" t="n">
-        <v>20055</v>
+        <v>21861</v>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>23/25</t>
+          <t>24/25</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
@@ -2197,10 +2197,10 @@
         </is>
       </c>
       <c r="J34" s="4" t="n">
-        <v>21799</v>
+        <v>22772</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>871.9565217391304</v>
+        <v>910.875</v>
       </c>
     </row>
     <row r="35">
@@ -2282,11 +2282,11 @@
         </is>
       </c>
       <c r="G36" s="11" t="n">
-        <v>2943</v>
+        <v>2748</v>
       </c>
       <c r="H36" s="10" t="inlineStr">
         <is>
-          <t>21/23</t>
+          <t>22/28</t>
         </is>
       </c>
       <c r="I36" s="10" t="inlineStr">
@@ -2295,10 +2295,10 @@
         </is>
       </c>
       <c r="J36" s="11" t="n">
-        <v>3223</v>
+        <v>3497</v>
       </c>
       <c r="K36" s="12" t="n">
-        <v>140.1428571428571</v>
+        <v>124.9090909090909</v>
       </c>
     </row>
     <row r="37">
@@ -2410,30 +2410,30 @@
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
+          <t>JEGANATHMISHRA PLA</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
           <t>ERAMAKRISHNAN N</t>
         </is>
       </c>
-      <c r="D39" s="7" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E39" s="7" t="inlineStr">
-        <is>
-          <t>JEGANATHMISHRA PLA</t>
-        </is>
-      </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>Tamilaga Vettri Kazhagam</t>
+          <t>Dravida Munnetra Kazhagam</t>
         </is>
       </c>
       <c r="G39" s="8" t="n">
-        <v>548</v>
+        <v>751</v>
       </c>
       <c r="H39" s="7" t="inlineStr">
         <is>
-          <t>22/25</t>
+          <t>25/25</t>
         </is>
       </c>
       <c r="I39" s="7" t="inlineStr">
@@ -2442,10 +2442,10 @@
         </is>
       </c>
       <c r="J39" s="8" t="n">
-        <v>623</v>
+        <v>751</v>
       </c>
       <c r="K39" s="9" t="n">
-        <v>24.90909090909091</v>
+        <v>30.04</v>
       </c>
     </row>
     <row r="40">
@@ -2585,7 +2585,7 @@
       </c>
       <c r="I42" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J42" s="8" t="n">
@@ -2625,23 +2625,23 @@
         </is>
       </c>
       <c r="G43" s="4" t="n">
-        <v>45324</v>
+        <v>49668</v>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>16/18</t>
+          <t>18/18</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J43" s="4" t="n">
-        <v>50990</v>
+        <v>49668</v>
       </c>
       <c r="K43" s="5" t="n">
-        <v>2832.75</v>
+        <v>2759.333333333333</v>
       </c>
     </row>
     <row r="44">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="I49" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J49" s="4" t="n">
@@ -2939,52 +2939,52 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="10" t="inlineStr">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>GINGEE</t>
         </is>
       </c>
-      <c r="B50" s="10" t="n">
+      <c r="B50" s="3" t="n">
         <v>70</v>
       </c>
-      <c r="C50" s="10" t="inlineStr">
+      <c r="C50" s="3" t="inlineStr">
         <is>
           <t>GANESHKUMAR A</t>
         </is>
       </c>
-      <c r="D50" s="10" t="inlineStr">
+      <c r="D50" s="3" t="inlineStr">
         <is>
           <t>Pattali Makkal Katchi</t>
         </is>
       </c>
-      <c r="E50" s="10" t="inlineStr">
-        <is>
-          <t>CHANDRASEKARAN B</t>
-        </is>
-      </c>
-      <c r="F50" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G50" s="11" t="n">
-        <v>12024</v>
-      </c>
-      <c r="H50" s="10" t="inlineStr">
-        <is>
-          <t>17/23</t>
-        </is>
-      </c>
-      <c r="I50" s="10" t="inlineStr">
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>GINGEE MASTHAN K S</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G50" s="4" t="n">
+        <v>12082</v>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>19/23</t>
+        </is>
+      </c>
+      <c r="I50" s="3" t="inlineStr">
         <is>
           <t>Result in Progress</t>
         </is>
       </c>
-      <c r="J50" s="11" t="n">
-        <v>16268</v>
-      </c>
-      <c r="K50" s="12" t="n">
-        <v>707.2941176470588</v>
+      <c r="J50" s="4" t="n">
+        <v>14626</v>
+      </c>
+      <c r="K50" s="5" t="n">
+        <v>635.8947368421053</v>
       </c>
     </row>
     <row r="51">
@@ -3124,7 +3124,7 @@
       </c>
       <c r="I53" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J53" s="4" t="n">
@@ -3320,7 +3320,7 @@
       </c>
       <c r="I57" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J57" s="4" t="n">
@@ -3458,23 +3458,23 @@
         </is>
       </c>
       <c r="G60" s="4" t="n">
-        <v>6063</v>
+        <v>6253</v>
       </c>
       <c r="H60" s="3" t="inlineStr">
         <is>
-          <t>25/26</t>
+          <t>27/27</t>
         </is>
       </c>
       <c r="I60" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J60" s="4" t="n">
-        <v>6306</v>
+        <v>6253</v>
       </c>
       <c r="K60" s="5" t="n">
-        <v>242.52</v>
+        <v>231.5925925925926</v>
       </c>
     </row>
     <row r="61">
@@ -3507,11 +3507,11 @@
         </is>
       </c>
       <c r="G61" s="4" t="n">
-        <v>21798</v>
+        <v>25763</v>
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>19/22</t>
+          <t>22/24</t>
         </is>
       </c>
       <c r="I61" s="3" t="inlineStr">
@@ -3520,10 +3520,10 @@
         </is>
       </c>
       <c r="J61" s="4" t="n">
-        <v>25240</v>
+        <v>28105</v>
       </c>
       <c r="K61" s="5" t="n">
-        <v>1147.263157894737</v>
+        <v>1171.045454545455</v>
       </c>
     </row>
     <row r="62">
@@ -3605,11 +3605,11 @@
         </is>
       </c>
       <c r="G63" s="4" t="n">
-        <v>13422</v>
+        <v>15488</v>
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
-          <t>24/26</t>
+          <t>26/26</t>
         </is>
       </c>
       <c r="I63" s="3" t="inlineStr">
@@ -3618,10 +3618,10 @@
         </is>
       </c>
       <c r="J63" s="4" t="n">
-        <v>14540</v>
+        <v>15488</v>
       </c>
       <c r="K63" s="5" t="n">
-        <v>559.25</v>
+        <v>595.6923076923077</v>
       </c>
     </row>
     <row r="64">
@@ -3654,11 +3654,11 @@
         </is>
       </c>
       <c r="G64" s="4" t="n">
-        <v>7938</v>
+        <v>8133</v>
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
-          <t>23/24</t>
+          <t>24/24</t>
         </is>
       </c>
       <c r="I64" s="3" t="inlineStr">
@@ -3667,10 +3667,10 @@
         </is>
       </c>
       <c r="J64" s="4" t="n">
-        <v>8283</v>
+        <v>8133</v>
       </c>
       <c r="K64" s="5" t="n">
-        <v>345.1304347826087</v>
+        <v>338.875</v>
       </c>
     </row>
     <row r="65">
@@ -3752,11 +3752,11 @@
         </is>
       </c>
       <c r="G66" s="4" t="n">
-        <v>41498</v>
+        <v>46010</v>
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>24/30</t>
+          <t>29/30</t>
         </is>
       </c>
       <c r="I66" s="3" t="inlineStr">
@@ -3765,10 +3765,10 @@
         </is>
       </c>
       <c r="J66" s="4" t="n">
-        <v>51872</v>
+        <v>47597</v>
       </c>
       <c r="K66" s="5" t="n">
-        <v>1729.083333333333</v>
+        <v>1586.551724137931</v>
       </c>
     </row>
     <row r="67">
@@ -3850,11 +3850,11 @@
         </is>
       </c>
       <c r="G68" s="4" t="n">
-        <v>6142</v>
+        <v>5670</v>
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>18/20</t>
+          <t>20/20</t>
         </is>
       </c>
       <c r="I68" s="3" t="inlineStr">
@@ -3863,10 +3863,10 @@
         </is>
       </c>
       <c r="J68" s="4" t="n">
-        <v>6824</v>
+        <v>5670</v>
       </c>
       <c r="K68" s="5" t="n">
-        <v>341.2222222222222</v>
+        <v>283.5</v>
       </c>
     </row>
     <row r="69">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="I69" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J69" s="4" t="n">
@@ -3968,52 +3968,52 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="10" t="inlineStr">
+      <c r="A71" s="6" t="inlineStr">
         <is>
           <t>KILLIYOOR</t>
         </is>
       </c>
-      <c r="B71" s="10" t="n">
+      <c r="B71" s="7" t="n">
         <v>234</v>
       </c>
-      <c r="C71" s="10" t="inlineStr">
+      <c r="C71" s="7" t="inlineStr">
         <is>
           <t>RAJESH KUMAR. S</t>
         </is>
       </c>
-      <c r="D71" s="10" t="inlineStr">
+      <c r="D71" s="7" t="inlineStr">
         <is>
           <t>Indian National Congress</t>
         </is>
       </c>
-      <c r="E71" s="10" t="inlineStr">
+      <c r="E71" s="7" t="inlineStr">
         <is>
           <t>SABIN. S</t>
         </is>
       </c>
-      <c r="F71" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G71" s="11" t="n">
-        <v>3285</v>
-      </c>
-      <c r="H71" s="10" t="inlineStr">
-        <is>
-          <t>20/22</t>
-        </is>
-      </c>
-      <c r="I71" s="10" t="inlineStr">
+      <c r="F71" s="7" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G71" s="8" t="n">
+        <v>1428</v>
+      </c>
+      <c r="H71" s="7" t="inlineStr">
+        <is>
+          <t>22/23</t>
+        </is>
+      </c>
+      <c r="I71" s="7" t="inlineStr">
         <is>
           <t>Result in Progress</t>
         </is>
       </c>
-      <c r="J71" s="11" t="n">
-        <v>3614</v>
-      </c>
-      <c r="K71" s="12" t="n">
-        <v>164.25</v>
+      <c r="J71" s="8" t="n">
+        <v>1493</v>
+      </c>
+      <c r="K71" s="9" t="n">
+        <v>64.90909090909091</v>
       </c>
     </row>
     <row r="72">
@@ -4055,7 +4055,7 @@
       </c>
       <c r="I72" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J72" s="4" t="n">
@@ -4153,7 +4153,7 @@
       </c>
       <c r="I74" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J74" s="8" t="n">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="I75" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J75" s="4" t="n">
@@ -4291,11 +4291,11 @@
         </is>
       </c>
       <c r="G77" s="8" t="n">
-        <v>962</v>
+        <v>843</v>
       </c>
       <c r="H77" s="7" t="inlineStr">
         <is>
-          <t>23/25</t>
+          <t>25/25</t>
         </is>
       </c>
       <c r="I77" s="7" t="inlineStr">
@@ -4304,10 +4304,10 @@
         </is>
       </c>
       <c r="J77" s="8" t="n">
-        <v>1046</v>
+        <v>843</v>
       </c>
       <c r="K77" s="9" t="n">
-        <v>41.82608695652174</v>
+        <v>33.72</v>
       </c>
     </row>
     <row r="78">
@@ -4389,11 +4389,11 @@
         </is>
       </c>
       <c r="G79" s="11" t="n">
-        <v>3523</v>
+        <v>3503</v>
       </c>
       <c r="H79" s="10" t="inlineStr">
         <is>
-          <t>20/21</t>
+          <t>21/21</t>
         </is>
       </c>
       <c r="I79" s="10" t="inlineStr">
@@ -4402,10 +4402,10 @@
         </is>
       </c>
       <c r="J79" s="11" t="n">
-        <v>3699</v>
+        <v>3503</v>
       </c>
       <c r="K79" s="12" t="n">
-        <v>176.15</v>
+        <v>166.8095238095238</v>
       </c>
     </row>
     <row r="80">
@@ -4487,11 +4487,11 @@
         </is>
       </c>
       <c r="G81" s="4" t="n">
-        <v>7682</v>
+        <v>7696</v>
       </c>
       <c r="H81" s="3" t="inlineStr">
         <is>
-          <t>23/24</t>
+          <t>24/24</t>
         </is>
       </c>
       <c r="I81" s="3" t="inlineStr">
@@ -4500,59 +4500,59 @@
         </is>
       </c>
       <c r="J81" s="4" t="n">
-        <v>8016</v>
+        <v>7696</v>
       </c>
       <c r="K81" s="5" t="n">
-        <v>334</v>
+        <v>320.6666666666667</v>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="13" t="inlineStr">
+      <c r="A82" s="6" t="inlineStr">
         <is>
           <t>KUMBAKONAM</t>
         </is>
       </c>
-      <c r="B82" s="14" t="n">
+      <c r="B82" s="7" t="n">
         <v>171</v>
       </c>
-      <c r="C82" s="14" t="inlineStr">
+      <c r="C82" s="7" t="inlineStr">
         <is>
           <t>VINOTH</t>
         </is>
       </c>
-      <c r="D82" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E82" s="14" t="inlineStr">
+      <c r="D82" s="7" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E82" s="7" t="inlineStr">
         <is>
           <t>ANBALAGAN G</t>
         </is>
       </c>
-      <c r="F82" s="14" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G82" s="15" t="n">
-        <v>432</v>
-      </c>
-      <c r="H82" s="14" t="inlineStr">
-        <is>
-          <t>20/22</t>
-        </is>
-      </c>
-      <c r="I82" s="14" t="inlineStr">
+      <c r="F82" s="7" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G82" s="8" t="n">
+        <v>535</v>
+      </c>
+      <c r="H82" s="7" t="inlineStr">
+        <is>
+          <t>21/22</t>
+        </is>
+      </c>
+      <c r="I82" s="7" t="inlineStr">
         <is>
           <t>Result in Progress</t>
         </is>
       </c>
-      <c r="J82" s="15" t="n">
-        <v>475</v>
-      </c>
-      <c r="K82" s="16" t="n">
-        <v>21.6</v>
+      <c r="J82" s="8" t="n">
+        <v>560</v>
+      </c>
+      <c r="K82" s="9" t="n">
+        <v>25.47619047619047</v>
       </c>
     </row>
     <row r="83">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="I84" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J84" s="4" t="n">
@@ -4732,23 +4732,23 @@
         </is>
       </c>
       <c r="G86" s="4" t="n">
-        <v>14572</v>
+        <v>15968</v>
       </c>
       <c r="H86" s="3" t="inlineStr">
         <is>
-          <t>20/21</t>
+          <t>22/22</t>
         </is>
       </c>
       <c r="I86" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J86" s="4" t="n">
-        <v>15301</v>
+        <v>15968</v>
       </c>
       <c r="K86" s="5" t="n">
-        <v>728.6</v>
+        <v>725.8181818181819</v>
       </c>
     </row>
     <row r="87">
@@ -5026,11 +5026,11 @@
         </is>
       </c>
       <c r="G92" s="4" t="n">
-        <v>11713</v>
+        <v>11793</v>
       </c>
       <c r="H92" s="3" t="inlineStr">
         <is>
-          <t>24/24</t>
+          <t>25/27</t>
         </is>
       </c>
       <c r="I92" s="3" t="inlineStr">
@@ -5039,10 +5039,10 @@
         </is>
       </c>
       <c r="J92" s="4" t="n">
-        <v>11713</v>
+        <v>12736</v>
       </c>
       <c r="K92" s="5" t="n">
-        <v>488.0416666666667</v>
+        <v>471.72</v>
       </c>
     </row>
     <row r="93">
@@ -5124,11 +5124,11 @@
         </is>
       </c>
       <c r="G94" s="4" t="n">
-        <v>59470</v>
+        <v>61255</v>
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
-          <t>23/25</t>
+          <t>26/27</t>
         </is>
       </c>
       <c r="I94" s="3" t="inlineStr">
@@ -5137,10 +5137,10 @@
         </is>
       </c>
       <c r="J94" s="4" t="n">
-        <v>64641</v>
+        <v>63611</v>
       </c>
       <c r="K94" s="5" t="n">
-        <v>2585.652173913043</v>
+        <v>2355.961538461539</v>
       </c>
     </row>
     <row r="95">
@@ -5242,52 +5242,52 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="10" t="inlineStr">
+      <c r="A97" s="6" t="inlineStr">
         <is>
           <t>MANAMADURAI</t>
         </is>
       </c>
-      <c r="B97" s="10" t="n">
+      <c r="B97" s="7" t="n">
         <v>187</v>
       </c>
-      <c r="C97" s="10" t="inlineStr">
+      <c r="C97" s="7" t="inlineStr">
         <is>
           <t>ELANGOVAN.D</t>
         </is>
       </c>
-      <c r="D97" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E97" s="10" t="inlineStr">
+      <c r="D97" s="7" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E97" s="7" t="inlineStr">
         <is>
           <t>TAMILARASI.A</t>
         </is>
       </c>
-      <c r="F97" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G97" s="11" t="n">
-        <v>2772</v>
-      </c>
-      <c r="H97" s="10" t="inlineStr">
-        <is>
-          <t>21/27</t>
-        </is>
-      </c>
-      <c r="I97" s="10" t="inlineStr">
+      <c r="F97" s="7" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G97" s="8" t="n">
+        <v>895</v>
+      </c>
+      <c r="H97" s="7" t="inlineStr">
+        <is>
+          <t>24/27</t>
+        </is>
+      </c>
+      <c r="I97" s="7" t="inlineStr">
         <is>
           <t>Result in Progress</t>
         </is>
       </c>
-      <c r="J97" s="11" t="n">
-        <v>3564</v>
-      </c>
-      <c r="K97" s="12" t="n">
-        <v>132</v>
+      <c r="J97" s="8" t="n">
+        <v>1007</v>
+      </c>
+      <c r="K97" s="9" t="n">
+        <v>37.29166666666666</v>
       </c>
     </row>
     <row r="98">
@@ -5516,11 +5516,11 @@
         </is>
       </c>
       <c r="G102" s="4" t="n">
-        <v>6281</v>
+        <v>7600</v>
       </c>
       <c r="H102" s="3" t="inlineStr">
         <is>
-          <t>24/26</t>
+          <t>26/27</t>
         </is>
       </c>
       <c r="I102" s="3" t="inlineStr">
@@ -5529,10 +5529,10 @@
         </is>
       </c>
       <c r="J102" s="4" t="n">
-        <v>6804</v>
+        <v>7892</v>
       </c>
       <c r="K102" s="5" t="n">
-        <v>261.7083333333333</v>
+        <v>292.3076923076923</v>
       </c>
     </row>
     <row r="103">
@@ -5565,11 +5565,11 @@
         </is>
       </c>
       <c r="G103" s="4" t="n">
-        <v>16100</v>
+        <v>18099</v>
       </c>
       <c r="H103" s="3" t="inlineStr">
         <is>
-          <t>22/24</t>
+          <t>24/30</t>
         </is>
       </c>
       <c r="I103" s="3" t="inlineStr">
@@ -5578,10 +5578,10 @@
         </is>
       </c>
       <c r="J103" s="4" t="n">
-        <v>17564</v>
+        <v>22624</v>
       </c>
       <c r="K103" s="5" t="n">
-        <v>731.8181818181819</v>
+        <v>754.125</v>
       </c>
     </row>
     <row r="104">
@@ -5663,23 +5663,23 @@
         </is>
       </c>
       <c r="G105" s="4" t="n">
-        <v>16527</v>
+        <v>16598</v>
       </c>
       <c r="H105" s="3" t="inlineStr">
         <is>
-          <t>30/31</t>
+          <t>31/31</t>
         </is>
       </c>
       <c r="I105" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J105" s="4" t="n">
-        <v>17078</v>
+        <v>16598</v>
       </c>
       <c r="K105" s="5" t="n">
-        <v>550.9</v>
+        <v>535.4193548387096</v>
       </c>
     </row>
     <row r="106">
@@ -5879,52 +5879,52 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="10" t="inlineStr">
+      <c r="A110" s="2" t="inlineStr">
         <is>
           <t>NAMAKKAL</t>
         </is>
       </c>
-      <c r="B110" s="10" t="n">
+      <c r="B110" s="3" t="n">
         <v>94</v>
       </c>
-      <c r="C110" s="10" t="inlineStr">
+      <c r="C110" s="3" t="inlineStr">
         <is>
           <t>DILIP C S</t>
         </is>
       </c>
-      <c r="D110" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E110" s="10" t="inlineStr">
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E110" s="3" t="inlineStr">
         <is>
           <t>SRIDEVI MOHAN P S</t>
         </is>
       </c>
-      <c r="F110" s="10" t="inlineStr">
+      <c r="F110" s="3" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G110" s="11" t="n">
-        <v>8865</v>
-      </c>
-      <c r="H110" s="10" t="inlineStr">
-        <is>
-          <t>16/23</t>
-        </is>
-      </c>
-      <c r="I110" s="10" t="inlineStr">
+      <c r="G110" s="4" t="n">
+        <v>11888</v>
+      </c>
+      <c r="H110" s="3" t="inlineStr">
+        <is>
+          <t>19/23</t>
+        </is>
+      </c>
+      <c r="I110" s="3" t="inlineStr">
         <is>
           <t>Result in Progress</t>
         </is>
       </c>
-      <c r="J110" s="11" t="n">
-        <v>12743</v>
-      </c>
-      <c r="K110" s="12" t="n">
-        <v>554.0625</v>
+      <c r="J110" s="4" t="n">
+        <v>14391</v>
+      </c>
+      <c r="K110" s="5" t="n">
+        <v>625.6842105263158</v>
       </c>
     </row>
     <row r="111">
@@ -6064,7 +6064,7 @@
       </c>
       <c r="I113" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J113" s="4" t="n">
@@ -6113,7 +6113,7 @@
       </c>
       <c r="I114" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J114" s="4" t="n">
@@ -6124,52 +6124,52 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="10" t="inlineStr">
+      <c r="A115" s="6" t="inlineStr">
         <is>
           <t>NILAKKOTTAI</t>
         </is>
       </c>
-      <c r="B115" s="10" t="n">
+      <c r="B115" s="7" t="n">
         <v>130</v>
       </c>
-      <c r="C115" s="10" t="inlineStr">
+      <c r="C115" s="7" t="inlineStr">
         <is>
           <t>AYYANAR.R</t>
         </is>
       </c>
-      <c r="D115" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E115" s="10" t="inlineStr">
+      <c r="D115" s="7" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E115" s="7" t="inlineStr">
         <is>
           <t>NAGAJOTHI.S</t>
         </is>
       </c>
-      <c r="F115" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G115" s="11" t="n">
-        <v>3038</v>
-      </c>
-      <c r="H115" s="10" t="inlineStr">
-        <is>
-          <t>22/25</t>
-        </is>
-      </c>
-      <c r="I115" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J115" s="11" t="n">
-        <v>3452</v>
-      </c>
-      <c r="K115" s="12" t="n">
-        <v>138.0909090909091</v>
+      <c r="F115" s="7" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G115" s="8" t="n">
+        <v>2925</v>
+      </c>
+      <c r="H115" s="7" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="I115" s="7" t="inlineStr">
+        <is>
+          <t>Result Declared</t>
+        </is>
+      </c>
+      <c r="J115" s="8" t="n">
+        <v>2925</v>
+      </c>
+      <c r="K115" s="9" t="n">
+        <v>117</v>
       </c>
     </row>
     <row r="116">
@@ -6260,7 +6260,7 @@
       </c>
       <c r="I117" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J117" s="4" t="n">
@@ -6309,7 +6309,7 @@
       </c>
       <c r="I118" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J118" s="4" t="n">
@@ -6349,23 +6349,23 @@
         </is>
       </c>
       <c r="G119" s="4" t="n">
-        <v>27807</v>
+        <v>29083</v>
       </c>
       <c r="H119" s="3" t="inlineStr">
         <is>
-          <t>22/24</t>
+          <t>24/24</t>
         </is>
       </c>
       <c r="I119" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J119" s="4" t="n">
-        <v>30335</v>
+        <v>29083</v>
       </c>
       <c r="K119" s="5" t="n">
-        <v>1263.954545454545</v>
+        <v>1211.791666666667</v>
       </c>
     </row>
     <row r="120">
@@ -6456,7 +6456,7 @@
       </c>
       <c r="I121" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J121" s="4" t="n">
@@ -6496,11 +6496,11 @@
         </is>
       </c>
       <c r="G122" s="8" t="n">
-        <v>753</v>
+        <v>693</v>
       </c>
       <c r="H122" s="7" t="inlineStr">
         <is>
-          <t>24/25</t>
+          <t>27/27</t>
         </is>
       </c>
       <c r="I122" s="7" t="inlineStr">
@@ -6509,10 +6509,10 @@
         </is>
       </c>
       <c r="J122" s="8" t="n">
-        <v>784</v>
+        <v>693</v>
       </c>
       <c r="K122" s="9" t="n">
-        <v>31.375</v>
+        <v>25.66666666666667</v>
       </c>
     </row>
     <row r="123">
@@ -6643,11 +6643,11 @@
         </is>
       </c>
       <c r="G125" s="4" t="n">
-        <v>46706</v>
+        <v>52009</v>
       </c>
       <c r="H125" s="3" t="inlineStr">
         <is>
-          <t>28/34</t>
+          <t>32/35</t>
         </is>
       </c>
       <c r="I125" s="3" t="inlineStr">
@@ -6656,10 +6656,10 @@
         </is>
       </c>
       <c r="J125" s="4" t="n">
-        <v>56714</v>
+        <v>56885</v>
       </c>
       <c r="K125" s="5" t="n">
-        <v>1668.071428571429</v>
+        <v>1625.28125</v>
       </c>
     </row>
     <row r="126">
@@ -6741,23 +6741,23 @@
         </is>
       </c>
       <c r="G127" s="8" t="n">
-        <v>1648</v>
+        <v>1065</v>
       </c>
       <c r="H127" s="7" t="inlineStr">
         <is>
-          <t>20/23</t>
+          <t>23/23</t>
         </is>
       </c>
       <c r="I127" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J127" s="8" t="n">
-        <v>1895</v>
+        <v>1065</v>
       </c>
       <c r="K127" s="9" t="n">
-        <v>82.40000000000001</v>
+        <v>46.30434782608695</v>
       </c>
     </row>
     <row r="128">
@@ -6859,52 +6859,52 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" s="6" t="inlineStr">
+      <c r="A130" s="13" t="inlineStr">
         <is>
           <t>PARAMATHI-VELUR</t>
         </is>
       </c>
-      <c r="B130" s="7" t="n">
+      <c r="B130" s="14" t="n">
         <v>95</v>
       </c>
-      <c r="C130" s="7" t="inlineStr">
+      <c r="C130" s="14" t="inlineStr">
         <is>
           <t>SEKAR S</t>
         </is>
       </c>
-      <c r="D130" s="7" t="inlineStr">
+      <c r="D130" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E130" s="7" t="inlineStr">
+      <c r="E130" s="14" t="inlineStr">
         <is>
           <t>MOORTHIY K S</t>
         </is>
       </c>
-      <c r="F130" s="7" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G130" s="8" t="n">
-        <v>665</v>
-      </c>
-      <c r="H130" s="7" t="inlineStr">
-        <is>
-          <t>18/20</t>
-        </is>
-      </c>
-      <c r="I130" s="7" t="inlineStr">
+      <c r="F130" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G130" s="15" t="n">
+        <v>402</v>
+      </c>
+      <c r="H130" s="14" t="inlineStr">
+        <is>
+          <t>19/20</t>
+        </is>
+      </c>
+      <c r="I130" s="14" t="inlineStr">
         <is>
           <t>Result in Progress</t>
         </is>
       </c>
-      <c r="J130" s="8" t="n">
-        <v>739</v>
-      </c>
-      <c r="K130" s="9" t="n">
-        <v>36.94444444444444</v>
+      <c r="J130" s="15" t="n">
+        <v>423</v>
+      </c>
+      <c r="K130" s="16" t="n">
+        <v>21.15789473684211</v>
       </c>
     </row>
     <row r="131">
@@ -6946,7 +6946,7 @@
       </c>
       <c r="I131" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J131" s="4" t="n">
@@ -6995,7 +6995,7 @@
       </c>
       <c r="I132" s="10" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J132" s="11" t="n">
@@ -7044,7 +7044,7 @@
       </c>
       <c r="I133" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J133" s="4" t="n">
@@ -7133,11 +7133,11 @@
         </is>
       </c>
       <c r="G135" s="8" t="n">
-        <v>415</v>
+        <v>760</v>
       </c>
       <c r="H135" s="7" t="inlineStr">
         <is>
-          <t>15/21</t>
+          <t>18/21</t>
         </is>
       </c>
       <c r="I135" s="7" t="inlineStr">
@@ -7146,10 +7146,10 @@
         </is>
       </c>
       <c r="J135" s="8" t="n">
-        <v>581</v>
+        <v>887</v>
       </c>
       <c r="K135" s="9" t="n">
-        <v>27.66666666666667</v>
+        <v>42.22222222222222</v>
       </c>
     </row>
     <row r="136">
@@ -7182,11 +7182,11 @@
         </is>
       </c>
       <c r="G136" s="4" t="n">
-        <v>16590</v>
+        <v>19321</v>
       </c>
       <c r="H136" s="3" t="inlineStr">
         <is>
-          <t>24/26</t>
+          <t>26/26</t>
         </is>
       </c>
       <c r="I136" s="3" t="inlineStr">
@@ -7195,10 +7195,10 @@
         </is>
       </c>
       <c r="J136" s="4" t="n">
-        <v>17972</v>
+        <v>19321</v>
       </c>
       <c r="K136" s="5" t="n">
-        <v>691.25</v>
+        <v>743.1153846153846</v>
       </c>
     </row>
     <row r="137">
@@ -7300,52 +7300,52 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="6" t="inlineStr">
+      <c r="A139" s="13" t="inlineStr">
         <is>
           <t>POLUR</t>
         </is>
       </c>
-      <c r="B139" s="7" t="n">
+      <c r="B139" s="14" t="n">
         <v>66</v>
       </c>
-      <c r="C139" s="7" t="inlineStr">
+      <c r="C139" s="14" t="inlineStr">
+        <is>
+          <t>SARAVANAN. P</t>
+        </is>
+      </c>
+      <c r="D139" s="14" t="inlineStr">
+        <is>
+          <t>Desiya Murpokku Dravida Kazhagam</t>
+        </is>
+      </c>
+      <c r="E139" s="14" t="inlineStr">
         <is>
           <t>ABISHEK. R</t>
         </is>
       </c>
-      <c r="D139" s="7" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E139" s="7" t="inlineStr">
-        <is>
-          <t>SARAVANAN. P</t>
-        </is>
-      </c>
-      <c r="F139" s="7" t="inlineStr">
-        <is>
-          <t>Desiya Murpokku Dravida Kazhagam</t>
-        </is>
-      </c>
-      <c r="G139" s="8" t="n">
-        <v>316</v>
-      </c>
-      <c r="H139" s="7" t="inlineStr">
-        <is>
-          <t>12/22</t>
-        </is>
-      </c>
-      <c r="I139" s="7" t="inlineStr">
+      <c r="F139" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G139" s="15" t="n">
+        <v>67</v>
+      </c>
+      <c r="H139" s="14" t="inlineStr">
+        <is>
+          <t>14/22</t>
+        </is>
+      </c>
+      <c r="I139" s="14" t="inlineStr">
         <is>
           <t>Result in Progress</t>
         </is>
       </c>
-      <c r="J139" s="8" t="n">
-        <v>579</v>
-      </c>
-      <c r="K139" s="9" t="n">
-        <v>26.33333333333333</v>
+      <c r="J139" s="15" t="n">
+        <v>105</v>
+      </c>
+      <c r="K139" s="16" t="n">
+        <v>4.785714285714286</v>
       </c>
     </row>
     <row r="140">
@@ -7378,11 +7378,11 @@
         </is>
       </c>
       <c r="G140" s="4" t="n">
-        <v>55627</v>
+        <v>55768</v>
       </c>
       <c r="H140" s="3" t="inlineStr">
         <is>
-          <t>25/26</t>
+          <t>26/26</t>
         </is>
       </c>
       <c r="I140" s="3" t="inlineStr">
@@ -7391,10 +7391,10 @@
         </is>
       </c>
       <c r="J140" s="4" t="n">
-        <v>57852</v>
+        <v>55768</v>
       </c>
       <c r="K140" s="5" t="n">
-        <v>2225.08</v>
+        <v>2144.923076923077</v>
       </c>
     </row>
     <row r="141">
@@ -7427,11 +7427,11 @@
         </is>
       </c>
       <c r="G141" s="4" t="n">
-        <v>5928</v>
+        <v>8013</v>
       </c>
       <c r="H141" s="3" t="inlineStr">
         <is>
-          <t>20/25</t>
+          <t>23/25</t>
         </is>
       </c>
       <c r="I141" s="3" t="inlineStr">
@@ -7440,10 +7440,10 @@
         </is>
       </c>
       <c r="J141" s="4" t="n">
-        <v>7410</v>
+        <v>8710</v>
       </c>
       <c r="K141" s="5" t="n">
-        <v>296.4</v>
+        <v>348.3913043478261</v>
       </c>
     </row>
     <row r="142">
@@ -7525,23 +7525,23 @@
         </is>
       </c>
       <c r="G143" s="8" t="n">
-        <v>2031</v>
+        <v>1867</v>
       </c>
       <c r="H143" s="7" t="inlineStr">
         <is>
-          <t>20/22</t>
+          <t>22/22</t>
         </is>
       </c>
       <c r="I143" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J143" s="8" t="n">
-        <v>2234</v>
+        <v>1867</v>
       </c>
       <c r="K143" s="9" t="n">
-        <v>101.55</v>
+        <v>84.86363636363636</v>
       </c>
     </row>
     <row r="144">
@@ -7790,52 +7790,52 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="10" t="inlineStr">
+      <c r="A149" s="2" t="inlineStr">
         <is>
           <t>RISHIVANDIYAM</t>
         </is>
       </c>
-      <c r="B149" s="10" t="n">
+      <c r="B149" s="3" t="n">
         <v>78</v>
       </c>
-      <c r="C149" s="10" t="inlineStr">
+      <c r="C149" s="3" t="inlineStr">
         <is>
           <t>KARTHIKEYAN K</t>
         </is>
       </c>
-      <c r="D149" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E149" s="10" t="inlineStr">
+      <c r="D149" s="3" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E149" s="3" t="inlineStr">
         <is>
           <t>ASHOK KUMAR G</t>
         </is>
       </c>
-      <c r="F149" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G149" s="11" t="n">
-        <v>4997</v>
-      </c>
-      <c r="H149" s="10" t="inlineStr">
-        <is>
-          <t>20/25</t>
-        </is>
-      </c>
-      <c r="I149" s="10" t="inlineStr">
+      <c r="F149" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G149" s="4" t="n">
+        <v>6297</v>
+      </c>
+      <c r="H149" s="3" t="inlineStr">
+        <is>
+          <t>23/25</t>
+        </is>
+      </c>
+      <c r="I149" s="3" t="inlineStr">
         <is>
           <t>Result in Progress</t>
         </is>
       </c>
-      <c r="J149" s="11" t="n">
-        <v>6246</v>
-      </c>
-      <c r="K149" s="12" t="n">
-        <v>249.85</v>
+      <c r="J149" s="4" t="n">
+        <v>6845</v>
+      </c>
+      <c r="K149" s="5" t="n">
+        <v>273.7826086956522</v>
       </c>
     </row>
     <row r="150">
@@ -7926,7 +7926,7 @@
       </c>
       <c r="I151" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J151" s="4" t="n">
@@ -8073,7 +8073,7 @@
       </c>
       <c r="I154" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J154" s="4" t="n">
@@ -8113,72 +8113,72 @@
         </is>
       </c>
       <c r="G155" s="4" t="n">
-        <v>5456</v>
+        <v>6489</v>
       </c>
       <c r="H155" s="3" t="inlineStr">
         <is>
-          <t>21/23</t>
+          <t>24/24</t>
         </is>
       </c>
       <c r="I155" s="3" t="inlineStr">
         <is>
+          <t>Result Declared</t>
+        </is>
+      </c>
+      <c r="J155" s="4" t="n">
+        <v>6489</v>
+      </c>
+      <c r="K155" s="5" t="n">
+        <v>270.375</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="10" t="inlineStr">
+        <is>
+          <t>SANKARAPURAM</t>
+        </is>
+      </c>
+      <c r="B156" s="10" t="n">
+        <v>79</v>
+      </c>
+      <c r="C156" s="10" t="inlineStr">
+        <is>
+          <t>RAKESH R</t>
+        </is>
+      </c>
+      <c r="D156" s="10" t="inlineStr">
+        <is>
+          <t>All India Anna Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E156" s="10" t="inlineStr">
+        <is>
+          <t>UDHAYASURIYAN T</t>
+        </is>
+      </c>
+      <c r="F156" s="10" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G156" s="11" t="n">
+        <v>3440</v>
+      </c>
+      <c r="H156" s="10" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="I156" s="10" t="inlineStr">
+        <is>
           <t>Result in Progress</t>
         </is>
       </c>
-      <c r="J155" s="4" t="n">
-        <v>5976</v>
-      </c>
-      <c r="K155" s="5" t="n">
-        <v>259.8095238095238</v>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" s="6" t="inlineStr">
-        <is>
-          <t>SANKARAPURAM</t>
-        </is>
-      </c>
-      <c r="B156" s="7" t="n">
-        <v>79</v>
-      </c>
-      <c r="C156" s="7" t="inlineStr">
-        <is>
-          <t>UDHAYASURIYAN T</t>
-        </is>
-      </c>
-      <c r="D156" s="7" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E156" s="7" t="inlineStr">
-        <is>
-          <t>RAKESH R</t>
-        </is>
-      </c>
-      <c r="F156" s="7" t="inlineStr">
-        <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G156" s="8" t="n">
-        <v>475</v>
-      </c>
-      <c r="H156" s="7" t="inlineStr">
-        <is>
-          <t>20/25</t>
-        </is>
-      </c>
-      <c r="I156" s="7" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J156" s="8" t="n">
-        <v>594</v>
-      </c>
-      <c r="K156" s="9" t="n">
-        <v>23.75</v>
+      <c r="J156" s="11" t="n">
+        <v>3440</v>
+      </c>
+      <c r="K156" s="12" t="n">
+        <v>137.6</v>
       </c>
     </row>
     <row r="157">
@@ -8260,11 +8260,11 @@
         </is>
       </c>
       <c r="G158" s="4" t="n">
-        <v>5443</v>
+        <v>6050</v>
       </c>
       <c r="H158" s="3" t="inlineStr">
         <is>
-          <t>19/21</t>
+          <t>20/21</t>
         </is>
       </c>
       <c r="I158" s="3" t="inlineStr">
@@ -8273,10 +8273,10 @@
         </is>
       </c>
       <c r="J158" s="4" t="n">
-        <v>6016</v>
+        <v>6352</v>
       </c>
       <c r="K158" s="5" t="n">
-        <v>286.4736842105263</v>
+        <v>302.5</v>
       </c>
     </row>
     <row r="159">
@@ -8378,52 +8378,52 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="10" t="inlineStr">
+      <c r="A161" s="6" t="inlineStr">
         <is>
           <t>SHOLINGUR</t>
         </is>
       </c>
-      <c r="B161" s="10" t="n">
+      <c r="B161" s="7" t="n">
         <v>39</v>
       </c>
-      <c r="C161" s="10" t="inlineStr">
+      <c r="C161" s="7" t="inlineStr">
         <is>
           <t>K.SARAVANAN</t>
         </is>
       </c>
-      <c r="D161" s="10" t="inlineStr">
+      <c r="D161" s="7" t="inlineStr">
         <is>
           <t>Pattali Makkal Katchi</t>
         </is>
       </c>
-      <c r="E161" s="10" t="inlineStr">
+      <c r="E161" s="7" t="inlineStr">
         <is>
           <t>G.KAPIL</t>
         </is>
       </c>
-      <c r="F161" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G161" s="11" t="n">
-        <v>2475</v>
-      </c>
-      <c r="H161" s="10" t="inlineStr">
-        <is>
-          <t>18/25</t>
-        </is>
-      </c>
-      <c r="I161" s="10" t="inlineStr">
+      <c r="F161" s="7" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G161" s="8" t="n">
+        <v>1948</v>
+      </c>
+      <c r="H161" s="7" t="inlineStr">
+        <is>
+          <t>19/25</t>
+        </is>
+      </c>
+      <c r="I161" s="7" t="inlineStr">
         <is>
           <t>Result in Progress</t>
         </is>
       </c>
-      <c r="J161" s="11" t="n">
-        <v>3438</v>
-      </c>
-      <c r="K161" s="12" t="n">
-        <v>137.5</v>
+      <c r="J161" s="8" t="n">
+        <v>2563</v>
+      </c>
+      <c r="K161" s="9" t="n">
+        <v>102.5263157894737</v>
       </c>
     </row>
     <row r="162">
@@ -8456,11 +8456,11 @@
         </is>
       </c>
       <c r="G162" s="4" t="n">
-        <v>77452</v>
+        <v>95496</v>
       </c>
       <c r="H162" s="3" t="inlineStr">
         <is>
-          <t>25/30</t>
+          <t>30/31</t>
         </is>
       </c>
       <c r="I162" s="3" t="inlineStr">
@@ -8469,10 +8469,10 @@
         </is>
       </c>
       <c r="J162" s="4" t="n">
-        <v>92942</v>
+        <v>98679</v>
       </c>
       <c r="K162" s="5" t="n">
-        <v>3098.08</v>
+        <v>3183.2</v>
       </c>
     </row>
     <row r="163">
@@ -8505,11 +8505,11 @@
         </is>
       </c>
       <c r="G163" s="4" t="n">
-        <v>18965</v>
+        <v>19098</v>
       </c>
       <c r="H163" s="3" t="inlineStr">
         <is>
-          <t>24/27</t>
+          <t>26/27</t>
         </is>
       </c>
       <c r="I163" s="3" t="inlineStr">
@@ -8518,10 +8518,10 @@
         </is>
       </c>
       <c r="J163" s="4" t="n">
-        <v>21336</v>
+        <v>19833</v>
       </c>
       <c r="K163" s="5" t="n">
-        <v>790.2083333333334</v>
+        <v>734.5384615384615</v>
       </c>
     </row>
     <row r="164">
@@ -8661,7 +8661,7 @@
       </c>
       <c r="I166" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J166" s="4" t="n">
@@ -8701,11 +8701,11 @@
         </is>
       </c>
       <c r="G167" s="4" t="n">
-        <v>45556</v>
+        <v>50921</v>
       </c>
       <c r="H167" s="3" t="inlineStr">
         <is>
-          <t>27/32</t>
+          <t>30/32</t>
         </is>
       </c>
       <c r="I167" s="3" t="inlineStr">
@@ -8714,10 +8714,10 @@
         </is>
       </c>
       <c r="J167" s="4" t="n">
-        <v>53992</v>
+        <v>54316</v>
       </c>
       <c r="K167" s="5" t="n">
-        <v>1687.259259259259</v>
+        <v>1697.366666666667</v>
       </c>
     </row>
     <row r="168">
@@ -8750,11 +8750,11 @@
         </is>
       </c>
       <c r="G168" s="4" t="n">
-        <v>33941</v>
+        <v>33590</v>
       </c>
       <c r="H168" s="3" t="inlineStr">
         <is>
-          <t>24/28</t>
+          <t>28/28</t>
         </is>
       </c>
       <c r="I168" s="3" t="inlineStr">
@@ -8763,10 +8763,10 @@
         </is>
       </c>
       <c r="J168" s="4" t="n">
-        <v>39598</v>
+        <v>33590</v>
       </c>
       <c r="K168" s="5" t="n">
-        <v>1414.208333333333</v>
+        <v>1199.642857142857</v>
       </c>
     </row>
     <row r="169">
@@ -8848,11 +8848,11 @@
         </is>
       </c>
       <c r="G170" s="4" t="n">
-        <v>8097</v>
+        <v>8664</v>
       </c>
       <c r="H170" s="3" t="inlineStr">
         <is>
-          <t>21/23</t>
+          <t>22/23</t>
         </is>
       </c>
       <c r="I170" s="3" t="inlineStr">
@@ -8861,59 +8861,59 @@
         </is>
       </c>
       <c r="J170" s="4" t="n">
-        <v>8868</v>
+        <v>9058</v>
       </c>
       <c r="K170" s="5" t="n">
-        <v>385.5714285714286</v>
+        <v>393.8181818181818</v>
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="2" t="inlineStr">
+      <c r="A171" s="10" t="inlineStr">
         <is>
           <t>SULUR</t>
         </is>
       </c>
-      <c r="B171" s="3" t="n">
+      <c r="B171" s="10" t="n">
         <v>116</v>
       </c>
-      <c r="C171" s="3" t="inlineStr">
+      <c r="C171" s="10" t="inlineStr">
         <is>
           <t>NM.SUKUMAR</t>
         </is>
       </c>
-      <c r="D171" s="3" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E171" s="3" t="inlineStr">
+      <c r="D171" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E171" s="10" t="inlineStr">
         <is>
           <t>V.P.KANDASAMY</t>
         </is>
       </c>
-      <c r="F171" s="3" t="inlineStr">
+      <c r="F171" s="10" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G171" s="4" t="n">
-        <v>5248</v>
-      </c>
-      <c r="H171" s="3" t="inlineStr">
-        <is>
-          <t>30/35</t>
-        </is>
-      </c>
-      <c r="I171" s="3" t="inlineStr">
+      <c r="G171" s="11" t="n">
+        <v>4790</v>
+      </c>
+      <c r="H171" s="10" t="inlineStr">
+        <is>
+          <t>30/30</t>
+        </is>
+      </c>
+      <c r="I171" s="10" t="inlineStr">
         <is>
           <t>Result in Progress</t>
         </is>
       </c>
-      <c r="J171" s="4" t="n">
-        <v>6123</v>
-      </c>
-      <c r="K171" s="5" t="n">
-        <v>174.9333333333333</v>
+      <c r="J171" s="11" t="n">
+        <v>4790</v>
+      </c>
+      <c r="K171" s="12" t="n">
+        <v>159.6666666666667</v>
       </c>
     </row>
     <row r="172">
@@ -8955,7 +8955,7 @@
       </c>
       <c r="I172" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J172" s="4" t="n">
@@ -8995,11 +8995,11 @@
         </is>
       </c>
       <c r="G173" s="4" t="n">
-        <v>9776</v>
+        <v>10299</v>
       </c>
       <c r="H173" s="3" t="inlineStr">
         <is>
-          <t>25/26</t>
+          <t>26/26</t>
         </is>
       </c>
       <c r="I173" s="3" t="inlineStr">
@@ -9008,10 +9008,10 @@
         </is>
       </c>
       <c r="J173" s="4" t="n">
-        <v>10167</v>
+        <v>10299</v>
       </c>
       <c r="K173" s="5" t="n">
-        <v>391.04</v>
+        <v>396.1153846153846</v>
       </c>
     </row>
     <row r="174">
@@ -9044,11 +9044,11 @@
         </is>
       </c>
       <c r="G174" s="11" t="n">
-        <v>2643</v>
+        <v>3174</v>
       </c>
       <c r="H174" s="10" t="inlineStr">
         <is>
-          <t>21/24</t>
+          <t>22/24</t>
         </is>
       </c>
       <c r="I174" s="10" t="inlineStr">
@@ -9057,10 +9057,10 @@
         </is>
       </c>
       <c r="J174" s="11" t="n">
-        <v>3021</v>
+        <v>3463</v>
       </c>
       <c r="K174" s="12" t="n">
-        <v>125.8571428571429</v>
+        <v>144.2727272727273</v>
       </c>
     </row>
     <row r="175">
@@ -9191,23 +9191,23 @@
         </is>
       </c>
       <c r="G177" s="4" t="n">
-        <v>22494</v>
+        <v>23807</v>
       </c>
       <c r="H177" s="3" t="inlineStr">
         <is>
-          <t>24/26</t>
+          <t>26/26</t>
         </is>
       </c>
       <c r="I177" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J177" s="4" t="n">
-        <v>24368</v>
+        <v>23807</v>
       </c>
       <c r="K177" s="5" t="n">
-        <v>937.25</v>
+        <v>915.6538461538462</v>
       </c>
     </row>
     <row r="178">
@@ -9240,11 +9240,11 @@
         </is>
       </c>
       <c r="G178" s="8" t="n">
-        <v>786</v>
+        <v>1492</v>
       </c>
       <c r="H178" s="7" t="inlineStr">
         <is>
-          <t>20/22</t>
+          <t>22/22</t>
         </is>
       </c>
       <c r="I178" s="7" t="inlineStr">
@@ -9253,10 +9253,10 @@
         </is>
       </c>
       <c r="J178" s="8" t="n">
-        <v>865</v>
+        <v>1492</v>
       </c>
       <c r="K178" s="9" t="n">
-        <v>39.3</v>
+        <v>67.81818181818181</v>
       </c>
     </row>
     <row r="179">
@@ -9289,11 +9289,11 @@
         </is>
       </c>
       <c r="G179" s="4" t="n">
-        <v>40016</v>
+        <v>41553</v>
       </c>
       <c r="H179" s="3" t="inlineStr">
         <is>
-          <t>24/26</t>
+          <t>27/27</t>
         </is>
       </c>
       <c r="I179" s="3" t="inlineStr">
@@ -9302,10 +9302,10 @@
         </is>
       </c>
       <c r="J179" s="4" t="n">
-        <v>43351</v>
+        <v>41553</v>
       </c>
       <c r="K179" s="5" t="n">
-        <v>1667.333333333333</v>
+        <v>1539</v>
       </c>
     </row>
     <row r="180">
@@ -9338,11 +9338,11 @@
         </is>
       </c>
       <c r="G180" s="4" t="n">
-        <v>36383</v>
+        <v>39107</v>
       </c>
       <c r="H180" s="3" t="inlineStr">
         <is>
-          <t>24/29</t>
+          <t>28/33</t>
         </is>
       </c>
       <c r="I180" s="3" t="inlineStr">
@@ -9351,10 +9351,10 @@
         </is>
       </c>
       <c r="J180" s="4" t="n">
-        <v>43963</v>
+        <v>46090</v>
       </c>
       <c r="K180" s="5" t="n">
-        <v>1515.958333333333</v>
+        <v>1396.678571428571</v>
       </c>
     </row>
     <row r="181">
@@ -9436,11 +9436,11 @@
         </is>
       </c>
       <c r="G182" s="4" t="n">
-        <v>7361</v>
+        <v>8178</v>
       </c>
       <c r="H182" s="3" t="inlineStr">
         <is>
-          <t>20/25</t>
+          <t>22/25</t>
         </is>
       </c>
       <c r="I182" s="3" t="inlineStr">
@@ -9449,10 +9449,10 @@
         </is>
       </c>
       <c r="J182" s="4" t="n">
-        <v>9201</v>
+        <v>9293</v>
       </c>
       <c r="K182" s="5" t="n">
-        <v>368.05</v>
+        <v>371.7272727272727</v>
       </c>
     </row>
     <row r="183">
@@ -9583,23 +9583,23 @@
         </is>
       </c>
       <c r="G185" s="4" t="n">
-        <v>8720</v>
+        <v>8705</v>
       </c>
       <c r="H185" s="3" t="inlineStr">
         <is>
-          <t>22/24</t>
+          <t>24/24</t>
         </is>
       </c>
       <c r="I185" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J185" s="4" t="n">
-        <v>9513</v>
+        <v>8705</v>
       </c>
       <c r="K185" s="5" t="n">
-        <v>396.3636363636364</v>
+        <v>362.7083333333333</v>
       </c>
     </row>
     <row r="186">
@@ -9681,7 +9681,7 @@
         </is>
       </c>
       <c r="G187" s="4" t="n">
-        <v>53337</v>
+        <v>53564</v>
       </c>
       <c r="H187" s="3" t="inlineStr">
         <is>
@@ -9690,14 +9690,14 @@
       </c>
       <c r="I187" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J187" s="4" t="n">
-        <v>53337</v>
+        <v>53564</v>
       </c>
       <c r="K187" s="5" t="n">
-        <v>2051.423076923077</v>
+        <v>2060.153846153846</v>
       </c>
     </row>
     <row r="188">
@@ -9779,11 +9779,11 @@
         </is>
       </c>
       <c r="G189" s="4" t="n">
-        <v>14785</v>
+        <v>14654</v>
       </c>
       <c r="H189" s="3" t="inlineStr">
         <is>
-          <t>25/27</t>
+          <t>27/28</t>
         </is>
       </c>
       <c r="I189" s="3" t="inlineStr">
@@ -9792,10 +9792,10 @@
         </is>
       </c>
       <c r="J189" s="4" t="n">
-        <v>15968</v>
+        <v>15197</v>
       </c>
       <c r="K189" s="5" t="n">
-        <v>591.4</v>
+        <v>542.7407407407408</v>
       </c>
     </row>
     <row r="190">
@@ -9946,52 +9946,52 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" s="13" t="inlineStr">
+      <c r="A193" s="6" t="inlineStr">
         <is>
           <t>TINDIVANAM</t>
         </is>
       </c>
-      <c r="B193" s="14" t="n">
+      <c r="B193" s="7" t="n">
         <v>72</v>
       </c>
-      <c r="C193" s="14" t="inlineStr">
+      <c r="C193" s="7" t="inlineStr">
         <is>
           <t>VANNI ARASU</t>
         </is>
       </c>
-      <c r="D193" s="14" t="inlineStr">
+      <c r="D193" s="7" t="inlineStr">
         <is>
           <t>Viduthalai Chiruthaigal Katchi</t>
         </is>
       </c>
-      <c r="E193" s="14" t="inlineStr">
+      <c r="E193" s="7" t="inlineStr">
         <is>
           <t>ARJUNAN. P</t>
         </is>
       </c>
-      <c r="F193" s="14" t="inlineStr">
+      <c r="F193" s="7" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G193" s="15" t="n">
-        <v>349</v>
-      </c>
-      <c r="H193" s="14" t="inlineStr">
-        <is>
-          <t>21/23</t>
-        </is>
-      </c>
-      <c r="I193" s="14" t="inlineStr">
+      <c r="G193" s="8" t="n">
+        <v>702</v>
+      </c>
+      <c r="H193" s="7" t="inlineStr">
+        <is>
+          <t>22/23</t>
+        </is>
+      </c>
+      <c r="I193" s="7" t="inlineStr">
         <is>
           <t>Result in Progress</t>
         </is>
       </c>
-      <c r="J193" s="15" t="n">
-        <v>382</v>
-      </c>
-      <c r="K193" s="16" t="n">
-        <v>16.61904761904762</v>
+      <c r="J193" s="8" t="n">
+        <v>734</v>
+      </c>
+      <c r="K193" s="9" t="n">
+        <v>31.90909090909091</v>
       </c>
     </row>
     <row r="194">
@@ -10082,7 +10082,7 @@
       </c>
       <c r="I195" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J195" s="4" t="n">
@@ -10122,11 +10122,11 @@
         </is>
       </c>
       <c r="G196" s="4" t="n">
-        <v>22869</v>
+        <v>25272</v>
       </c>
       <c r="H196" s="3" t="inlineStr">
         <is>
-          <t>18/22</t>
+          <t>20/22</t>
         </is>
       </c>
       <c r="I196" s="3" t="inlineStr">
@@ -10135,10 +10135,10 @@
         </is>
       </c>
       <c r="J196" s="4" t="n">
-        <v>27951</v>
+        <v>27799</v>
       </c>
       <c r="K196" s="5" t="n">
-        <v>1270.5</v>
+        <v>1263.6</v>
       </c>
     </row>
     <row r="197">
@@ -10220,11 +10220,11 @@
         </is>
       </c>
       <c r="G198" s="4" t="n">
-        <v>11276</v>
+        <v>13485</v>
       </c>
       <c r="H198" s="3" t="inlineStr">
         <is>
-          <t>19/21</t>
+          <t>23/23</t>
         </is>
       </c>
       <c r="I198" s="3" t="inlineStr">
@@ -10233,10 +10233,10 @@
         </is>
       </c>
       <c r="J198" s="4" t="n">
-        <v>12463</v>
+        <v>13485</v>
       </c>
       <c r="K198" s="5" t="n">
-        <v>593.4736842105264</v>
+        <v>586.304347826087</v>
       </c>
     </row>
     <row r="199">
@@ -10250,30 +10250,30 @@
       </c>
       <c r="C199" s="14" t="inlineStr">
         <is>
+          <t>PALANISAMY S</t>
+        </is>
+      </c>
+      <c r="D199" s="14" t="inlineStr">
+        <is>
+          <t>All India Anna Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E199" s="14" t="inlineStr">
+        <is>
           <t>VIJAY R BARANIBALAAJI</t>
         </is>
       </c>
-      <c r="D199" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E199" s="14" t="inlineStr">
-        <is>
-          <t>PALANISAMY S</t>
-        </is>
-      </c>
       <c r="F199" s="14" t="inlineStr">
         <is>
-          <t>All India Anna Dravida Munnetra Kazhagam</t>
+          <t>Tamilaga Vettri Kazhagam</t>
         </is>
       </c>
       <c r="G199" s="15" t="n">
-        <v>69</v>
+        <v>161</v>
       </c>
       <c r="H199" s="14" t="inlineStr">
         <is>
-          <t>22/24</t>
+          <t>23/24</t>
         </is>
       </c>
       <c r="I199" s="14" t="inlineStr">
@@ -10282,10 +10282,10 @@
         </is>
       </c>
       <c r="J199" s="15" t="n">
-        <v>75</v>
+        <v>168</v>
       </c>
       <c r="K199" s="16" t="n">
-        <v>3.136363636363636</v>
+        <v>7</v>
       </c>
     </row>
     <row r="200">
@@ -10367,11 +10367,11 @@
         </is>
       </c>
       <c r="G201" s="4" t="n">
-        <v>42858</v>
+        <v>47382</v>
       </c>
       <c r="H201" s="3" t="inlineStr">
         <is>
-          <t>19/22</t>
+          <t>21/22</t>
         </is>
       </c>
       <c r="I201" s="3" t="inlineStr">
@@ -10380,10 +10380,10 @@
         </is>
       </c>
       <c r="J201" s="4" t="n">
-        <v>49625</v>
+        <v>49638</v>
       </c>
       <c r="K201" s="5" t="n">
-        <v>2255.684210526316</v>
+        <v>2256.285714285714</v>
       </c>
     </row>
     <row r="202">
@@ -10416,11 +10416,11 @@
         </is>
       </c>
       <c r="G202" s="8" t="n">
-        <v>1738</v>
+        <v>1127</v>
       </c>
       <c r="H202" s="7" t="inlineStr">
         <is>
-          <t>24/27</t>
+          <t>25/27</t>
         </is>
       </c>
       <c r="I202" s="7" t="inlineStr">
@@ -10429,10 +10429,10 @@
         </is>
       </c>
       <c r="J202" s="8" t="n">
-        <v>1955</v>
+        <v>1217</v>
       </c>
       <c r="K202" s="9" t="n">
-        <v>72.41666666666667</v>
+        <v>45.08</v>
       </c>
     </row>
     <row r="203">
@@ -10465,11 +10465,11 @@
         </is>
       </c>
       <c r="G203" s="4" t="n">
-        <v>62316</v>
+        <v>67902</v>
       </c>
       <c r="H203" s="3" t="inlineStr">
         <is>
-          <t>28/34</t>
+          <t>31/34</t>
         </is>
       </c>
       <c r="I203" s="3" t="inlineStr">
@@ -10478,10 +10478,10 @@
         </is>
       </c>
       <c r="J203" s="4" t="n">
-        <v>75669</v>
+        <v>74473</v>
       </c>
       <c r="K203" s="5" t="n">
-        <v>2225.571428571428</v>
+        <v>2190.387096774194</v>
       </c>
     </row>
     <row r="204">
@@ -10523,7 +10523,7 @@
       </c>
       <c r="I204" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J204" s="4" t="n">
@@ -10563,11 +10563,11 @@
         </is>
       </c>
       <c r="G205" s="4" t="n">
-        <v>6679</v>
+        <v>6857</v>
       </c>
       <c r="H205" s="3" t="inlineStr">
         <is>
-          <t>20/25</t>
+          <t>23/25</t>
         </is>
       </c>
       <c r="I205" s="3" t="inlineStr">
@@ -10576,10 +10576,10 @@
         </is>
       </c>
       <c r="J205" s="4" t="n">
-        <v>8349</v>
+        <v>7453</v>
       </c>
       <c r="K205" s="5" t="n">
-        <v>333.95</v>
+        <v>298.1304347826087</v>
       </c>
     </row>
     <row r="206">
@@ -10621,7 +10621,7 @@
       </c>
       <c r="I206" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J206" s="8" t="n">
@@ -10632,52 +10632,52 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="6" t="inlineStr">
+      <c r="A207" s="10" t="inlineStr">
         <is>
           <t>TIRUVANNAMALAI</t>
         </is>
       </c>
-      <c r="B207" s="7" t="n">
+      <c r="B207" s="10" t="n">
         <v>63</v>
       </c>
-      <c r="C207" s="7" t="inlineStr">
+      <c r="C207" s="10" t="inlineStr">
         <is>
           <t>VELU. E.V</t>
         </is>
       </c>
-      <c r="D207" s="7" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E207" s="7" t="inlineStr">
+      <c r="D207" s="10" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E207" s="10" t="inlineStr">
         <is>
           <t>ARUL ARUMUGAM</t>
         </is>
       </c>
-      <c r="F207" s="7" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G207" s="8" t="n">
-        <v>646</v>
-      </c>
-      <c r="H207" s="7" t="inlineStr">
-        <is>
-          <t>17/23</t>
-        </is>
-      </c>
-      <c r="I207" s="7" t="inlineStr">
+      <c r="F207" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G207" s="11" t="n">
+        <v>2595</v>
+      </c>
+      <c r="H207" s="10" t="inlineStr">
+        <is>
+          <t>19/23</t>
+        </is>
+      </c>
+      <c r="I207" s="10" t="inlineStr">
         <is>
           <t>Result in Progress</t>
         </is>
       </c>
-      <c r="J207" s="8" t="n">
-        <v>874</v>
-      </c>
-      <c r="K207" s="9" t="n">
-        <v>38</v>
+      <c r="J207" s="11" t="n">
+        <v>3141</v>
+      </c>
+      <c r="K207" s="12" t="n">
+        <v>136.578947368421</v>
       </c>
     </row>
     <row r="208">
@@ -10710,11 +10710,11 @@
         </is>
       </c>
       <c r="G208" s="8" t="n">
-        <v>2190</v>
+        <v>2541</v>
       </c>
       <c r="H208" s="7" t="inlineStr">
         <is>
-          <t>19/20</t>
+          <t>20/20</t>
         </is>
       </c>
       <c r="I208" s="7" t="inlineStr">
@@ -10723,10 +10723,10 @@
         </is>
       </c>
       <c r="J208" s="8" t="n">
-        <v>2305</v>
+        <v>2541</v>
       </c>
       <c r="K208" s="9" t="n">
-        <v>115.2631578947368</v>
+        <v>127.05</v>
       </c>
     </row>
     <row r="209">
@@ -10828,52 +10828,52 @@
       </c>
     </row>
     <row r="211">
-      <c r="A211" s="13" t="inlineStr">
+      <c r="A211" s="6" t="inlineStr">
         <is>
           <t>ULUNDURPETTAI</t>
         </is>
       </c>
-      <c r="B211" s="14" t="n">
+      <c r="B211" s="7" t="n">
         <v>77</v>
       </c>
-      <c r="C211" s="14" t="inlineStr">
+      <c r="C211" s="7" t="inlineStr">
         <is>
           <t>VASANTHAVEL G R</t>
         </is>
       </c>
-      <c r="D211" s="14" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E211" s="14" t="inlineStr">
+      <c r="D211" s="7" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E211" s="7" t="inlineStr">
         <is>
           <t>KUMARAGURU R</t>
         </is>
       </c>
-      <c r="F211" s="14" t="inlineStr">
+      <c r="F211" s="7" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G211" s="15" t="n">
-        <v>72</v>
-      </c>
-      <c r="H211" s="14" t="inlineStr">
-        <is>
-          <t>25/27</t>
-        </is>
-      </c>
-      <c r="I211" s="14" t="inlineStr">
+      <c r="G211" s="8" t="n">
+        <v>567</v>
+      </c>
+      <c r="H211" s="7" t="inlineStr">
+        <is>
+          <t>26/27</t>
+        </is>
+      </c>
+      <c r="I211" s="7" t="inlineStr">
         <is>
           <t>Result in Progress</t>
         </is>
       </c>
-      <c r="J211" s="15" t="n">
-        <v>78</v>
-      </c>
-      <c r="K211" s="16" t="n">
-        <v>2.88</v>
+      <c r="J211" s="8" t="n">
+        <v>589</v>
+      </c>
+      <c r="K211" s="9" t="n">
+        <v>21.80769230769231</v>
       </c>
     </row>
     <row r="212">
@@ -10906,23 +10906,23 @@
         </is>
       </c>
       <c r="G212" s="8" t="n">
-        <v>1617</v>
+        <v>1805</v>
       </c>
       <c r="H212" s="7" t="inlineStr">
         <is>
-          <t>24/25</t>
+          <t>25/25</t>
         </is>
       </c>
       <c r="I212" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J212" s="8" t="n">
-        <v>1684</v>
+        <v>1805</v>
       </c>
       <c r="K212" s="9" t="n">
-        <v>67.375</v>
+        <v>72.2</v>
       </c>
     </row>
     <row r="213">
@@ -10964,7 +10964,7 @@
       </c>
       <c r="I213" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J213" s="4" t="n">
@@ -11102,23 +11102,23 @@
         </is>
       </c>
       <c r="G216" s="11" t="n">
-        <v>3722</v>
+        <v>3333</v>
       </c>
       <c r="H216" s="10" t="inlineStr">
         <is>
-          <t>20/21</t>
+          <t>21/21</t>
         </is>
       </c>
       <c r="I216" s="10" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J216" s="11" t="n">
-        <v>3908</v>
+        <v>3333</v>
       </c>
       <c r="K216" s="12" t="n">
-        <v>186.1</v>
+        <v>158.7142857142857</v>
       </c>
     </row>
     <row r="217">
@@ -11249,11 +11249,11 @@
         </is>
       </c>
       <c r="G219" s="4" t="n">
-        <v>6585</v>
+        <v>6635</v>
       </c>
       <c r="H219" s="3" t="inlineStr">
         <is>
-          <t>21/23</t>
+          <t>22/23</t>
         </is>
       </c>
       <c r="I219" s="3" t="inlineStr">
@@ -11262,10 +11262,10 @@
         </is>
       </c>
       <c r="J219" s="4" t="n">
-        <v>7212</v>
+        <v>6937</v>
       </c>
       <c r="K219" s="5" t="n">
-        <v>313.5714285714286</v>
+        <v>301.5909090909091</v>
       </c>
     </row>
     <row r="220">
@@ -11356,7 +11356,7 @@
       </c>
       <c r="I221" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J221" s="4" t="n">
@@ -11405,7 +11405,7 @@
       </c>
       <c r="I222" s="10" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J222" s="11" t="n">
@@ -11503,7 +11503,7 @@
       </c>
       <c r="I224" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J224" s="4" t="n">
@@ -11543,11 +11543,11 @@
         </is>
       </c>
       <c r="G225" s="15" t="n">
-        <v>126</v>
+        <v>138</v>
       </c>
       <c r="H225" s="14" t="inlineStr">
         <is>
-          <t>26/27</t>
+          <t>27/27</t>
         </is>
       </c>
       <c r="I225" s="14" t="inlineStr">
@@ -11556,59 +11556,59 @@
         </is>
       </c>
       <c r="J225" s="15" t="n">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="K225" s="16" t="n">
-        <v>4.846153846153846</v>
+        <v>5.111111111111111</v>
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="10" t="inlineStr">
+      <c r="A226" s="6" t="inlineStr">
         <is>
           <t>VIKRAVANDI</t>
         </is>
       </c>
-      <c r="B226" s="10" t="n">
+      <c r="B226" s="7" t="n">
         <v>75</v>
       </c>
-      <c r="C226" s="10" t="inlineStr">
+      <c r="C226" s="7" t="inlineStr">
         <is>
           <t>SIVAKUMAR C</t>
         </is>
       </c>
-      <c r="D226" s="10" t="inlineStr">
+      <c r="D226" s="7" t="inlineStr">
         <is>
           <t>Pattali Makkal Katchi</t>
         </is>
       </c>
-      <c r="E226" s="10" t="inlineStr">
+      <c r="E226" s="7" t="inlineStr">
         <is>
           <t>VIJAI VADIVEL A</t>
         </is>
       </c>
-      <c r="F226" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G226" s="11" t="n">
-        <v>3046</v>
-      </c>
-      <c r="H226" s="10" t="inlineStr">
-        <is>
-          <t>18/23</t>
-        </is>
-      </c>
-      <c r="I226" s="10" t="inlineStr">
+      <c r="F226" s="7" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G226" s="8" t="n">
+        <v>668</v>
+      </c>
+      <c r="H226" s="7" t="inlineStr">
+        <is>
+          <t>21/23</t>
+        </is>
+      </c>
+      <c r="I226" s="7" t="inlineStr">
         <is>
           <t>Result in Progress</t>
         </is>
       </c>
-      <c r="J226" s="11" t="n">
-        <v>3892</v>
-      </c>
-      <c r="K226" s="12" t="n">
-        <v>169.2222222222222</v>
+      <c r="J226" s="8" t="n">
+        <v>732</v>
+      </c>
+      <c r="K226" s="9" t="n">
+        <v>31.80952380952381</v>
       </c>
     </row>
     <row r="227">
@@ -11699,7 +11699,7 @@
       </c>
       <c r="I228" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J228" s="4" t="n">
@@ -11837,11 +11837,11 @@
         </is>
       </c>
       <c r="G231" s="4" t="n">
-        <v>44006</v>
+        <v>56186</v>
       </c>
       <c r="H231" s="3" t="inlineStr">
         <is>
-          <t>14/20</t>
+          <t>18/20</t>
         </is>
       </c>
       <c r="I231" s="3" t="inlineStr">
@@ -11850,10 +11850,10 @@
         </is>
       </c>
       <c r="J231" s="4" t="n">
-        <v>62866</v>
+        <v>62429</v>
       </c>
       <c r="K231" s="5" t="n">
-        <v>3143.285714285714</v>
+        <v>3121.444444444444</v>
       </c>
     </row>
     <row r="232">
@@ -11886,11 +11886,11 @@
         </is>
       </c>
       <c r="G232" s="4" t="n">
-        <v>9375</v>
+        <v>9391</v>
       </c>
       <c r="H232" s="3" t="inlineStr">
         <is>
-          <t>22/23</t>
+          <t>23/23</t>
         </is>
       </c>
       <c r="I232" s="3" t="inlineStr">
@@ -11899,10 +11899,10 @@
         </is>
       </c>
       <c r="J232" s="4" t="n">
-        <v>9801</v>
+        <v>9391</v>
       </c>
       <c r="K232" s="5" t="n">
-        <v>426.1363636363636</v>
+        <v>408.3043478260869</v>
       </c>
     </row>
     <row r="233">
@@ -11935,23 +11935,23 @@
         </is>
       </c>
       <c r="G233" s="4" t="n">
-        <v>24052</v>
+        <v>27086</v>
       </c>
       <c r="H233" s="3" t="inlineStr">
         <is>
-          <t>20/23</t>
+          <t>24/24</t>
         </is>
       </c>
       <c r="I233" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J233" s="4" t="n">
-        <v>27660</v>
+        <v>27086</v>
       </c>
       <c r="K233" s="5" t="n">
-        <v>1202.6</v>
+        <v>1128.583333333333</v>
       </c>
     </row>
     <row r="234">
@@ -11993,7 +11993,7 @@
       </c>
       <c r="I234" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J234" s="8" t="n">
@@ -12033,11 +12033,11 @@
         </is>
       </c>
       <c r="G235" s="8" t="n">
-        <v>564</v>
+        <v>2189</v>
       </c>
       <c r="H235" s="7" t="inlineStr">
         <is>
-          <t>23/24</t>
+          <t>25/25</t>
         </is>
       </c>
       <c r="I235" s="7" t="inlineStr">
@@ -12046,10 +12046,10 @@
         </is>
       </c>
       <c r="J235" s="8" t="n">
-        <v>589</v>
+        <v>2189</v>
       </c>
       <c r="K235" s="9" t="n">
-        <v>24.52173913043478</v>
+        <v>87.56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Election snapshot: 98.7% counted — 166 declared, POLUR down to 15 votes
POLUR (DMDK) leads by just 15 votes with 7 rounds left; KULITHALAI flipped to DMK.

https://claude.ai/code/session_01MizbUy44JG5sXyvaf3Wekb
</commit_message>
<xml_diff>
--- a/tn_election_results_may2026.xlsx
+++ b/tn_election_results_may2026.xlsx
@@ -616,11 +616,11 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>26334</v>
+        <v>27928</v>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>27/31</t>
+          <t>29/31</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -629,10 +629,10 @@
         </is>
       </c>
       <c r="J2" s="4" t="n">
-        <v>30235</v>
+        <v>29854</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>975.3333333333334</v>
+        <v>963.0344827586207</v>
       </c>
     </row>
     <row r="3">
@@ -812,11 +812,11 @@
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>57844</v>
+        <v>58781</v>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>27/28</t>
+          <t>28/28</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -825,10 +825,10 @@
         </is>
       </c>
       <c r="J6" s="4" t="n">
-        <v>59986</v>
+        <v>58781</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>2142.37037037037</v>
+        <v>2099.321428571428</v>
       </c>
     </row>
     <row r="7">
@@ -861,11 +861,11 @@
         </is>
       </c>
       <c r="G7" s="4" t="n">
-        <v>7875</v>
+        <v>7327</v>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>21/22</t>
+          <t>22/22</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -874,10 +874,10 @@
         </is>
       </c>
       <c r="J7" s="4" t="n">
-        <v>8250</v>
+        <v>7327</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>375</v>
+        <v>333.0454545454546</v>
       </c>
     </row>
     <row r="8">
@@ -1556,7 +1556,7 @@
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J21" s="4" t="n">
@@ -1645,11 +1645,11 @@
         </is>
       </c>
       <c r="G23" s="11" t="n">
-        <v>4536</v>
+        <v>4241</v>
       </c>
       <c r="H23" s="10" t="inlineStr">
         <is>
-          <t>23/24</t>
+          <t>24/24</t>
         </is>
       </c>
       <c r="I23" s="10" t="inlineStr">
@@ -1658,10 +1658,10 @@
         </is>
       </c>
       <c r="J23" s="11" t="n">
-        <v>4733</v>
+        <v>4241</v>
       </c>
       <c r="K23" s="12" t="n">
-        <v>197.2173913043478</v>
+        <v>176.7083333333333</v>
       </c>
     </row>
     <row r="24">
@@ -1890,11 +1890,11 @@
         </is>
       </c>
       <c r="G28" s="4" t="n">
-        <v>32441</v>
+        <v>34344</v>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>28/36</t>
+          <t>32/36</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
@@ -1903,10 +1903,10 @@
         </is>
       </c>
       <c r="J28" s="4" t="n">
-        <v>41710</v>
+        <v>38637</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>1158.607142857143</v>
+        <v>1073.25</v>
       </c>
     </row>
     <row r="29">
@@ -2135,11 +2135,11 @@
         </is>
       </c>
       <c r="G33" s="4" t="n">
-        <v>5773</v>
+        <v>5794</v>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>22/24</t>
+          <t>23/24</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -2148,10 +2148,10 @@
         </is>
       </c>
       <c r="J33" s="4" t="n">
-        <v>6298</v>
+        <v>6046</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>262.4090909090909</v>
+        <v>251.9130434782609</v>
       </c>
     </row>
     <row r="34">
@@ -2184,23 +2184,23 @@
         </is>
       </c>
       <c r="G34" s="4" t="n">
-        <v>21861</v>
+        <v>21992</v>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>24/25</t>
+          <t>25/25</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J34" s="4" t="n">
-        <v>22772</v>
+        <v>21992</v>
       </c>
       <c r="K34" s="5" t="n">
-        <v>910.875</v>
+        <v>879.6799999999999</v>
       </c>
     </row>
     <row r="35">
@@ -2242,7 +2242,7 @@
       </c>
       <c r="I35" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J35" s="8" t="n">
@@ -2282,11 +2282,11 @@
         </is>
       </c>
       <c r="G36" s="11" t="n">
-        <v>2748</v>
+        <v>2698</v>
       </c>
       <c r="H36" s="10" t="inlineStr">
         <is>
-          <t>22/28</t>
+          <t>24/28</t>
         </is>
       </c>
       <c r="I36" s="10" t="inlineStr">
@@ -2295,10 +2295,10 @@
         </is>
       </c>
       <c r="J36" s="11" t="n">
-        <v>3497</v>
+        <v>3148</v>
       </c>
       <c r="K36" s="12" t="n">
-        <v>124.9090909090909</v>
+        <v>112.4166666666667</v>
       </c>
     </row>
     <row r="37">
@@ -2389,7 +2389,7 @@
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J38" s="4" t="n">
@@ -2968,11 +2968,11 @@
         </is>
       </c>
       <c r="G50" s="4" t="n">
-        <v>12082</v>
+        <v>13274</v>
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>19/23</t>
+          <t>21/23</t>
         </is>
       </c>
       <c r="I50" s="3" t="inlineStr">
@@ -2981,10 +2981,10 @@
         </is>
       </c>
       <c r="J50" s="4" t="n">
-        <v>14626</v>
+        <v>14538</v>
       </c>
       <c r="K50" s="5" t="n">
-        <v>635.8947368421053</v>
+        <v>632.0952380952381</v>
       </c>
     </row>
     <row r="51">
@@ -3507,23 +3507,23 @@
         </is>
       </c>
       <c r="G61" s="4" t="n">
-        <v>25763</v>
+        <v>26740</v>
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>22/24</t>
+          <t>24/24</t>
         </is>
       </c>
       <c r="I61" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J61" s="4" t="n">
-        <v>28105</v>
+        <v>26740</v>
       </c>
       <c r="K61" s="5" t="n">
-        <v>1171.045454545455</v>
+        <v>1114.166666666667</v>
       </c>
     </row>
     <row r="62">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="I63" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J63" s="4" t="n">
@@ -3752,11 +3752,11 @@
         </is>
       </c>
       <c r="G66" s="4" t="n">
-        <v>46010</v>
+        <v>46074</v>
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>29/30</t>
+          <t>30/30</t>
         </is>
       </c>
       <c r="I66" s="3" t="inlineStr">
@@ -3765,10 +3765,10 @@
         </is>
       </c>
       <c r="J66" s="4" t="n">
-        <v>47597</v>
+        <v>46074</v>
       </c>
       <c r="K66" s="5" t="n">
-        <v>1586.551724137931</v>
+        <v>1535.8</v>
       </c>
     </row>
     <row r="67">
@@ -3997,23 +3997,23 @@
         </is>
       </c>
       <c r="G71" s="8" t="n">
-        <v>1428</v>
+        <v>1311</v>
       </c>
       <c r="H71" s="7" t="inlineStr">
         <is>
-          <t>22/23</t>
+          <t>23/23</t>
         </is>
       </c>
       <c r="I71" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J71" s="8" t="n">
-        <v>1493</v>
+        <v>1311</v>
       </c>
       <c r="K71" s="9" t="n">
-        <v>64.90909090909091</v>
+        <v>57</v>
       </c>
     </row>
     <row r="72">
@@ -4300,7 +4300,7 @@
       </c>
       <c r="I77" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J77" s="8" t="n">
@@ -4409,52 +4409,52 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="6" t="inlineStr">
+      <c r="A80" s="13" t="inlineStr">
         <is>
           <t>KULITHALAI</t>
         </is>
       </c>
-      <c r="B80" s="7" t="n">
+      <c r="B80" s="14" t="n">
         <v>137</v>
       </c>
-      <c r="C80" s="7" t="inlineStr">
+      <c r="C80" s="14" t="inlineStr">
+        <is>
+          <t>SURIYANUR. A. CHANDRAN</t>
+        </is>
+      </c>
+      <c r="D80" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E80" s="14" t="inlineStr">
         <is>
           <t>G.BALASUBRAMANI</t>
         </is>
       </c>
-      <c r="D80" s="7" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E80" s="7" t="inlineStr">
-        <is>
-          <t>SURIYANUR. A. CHANDRAN</t>
-        </is>
-      </c>
-      <c r="F80" s="7" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G80" s="8" t="n">
-        <v>560</v>
-      </c>
-      <c r="H80" s="7" t="inlineStr">
-        <is>
-          <t>19/21</t>
-        </is>
-      </c>
-      <c r="I80" s="7" t="inlineStr">
+      <c r="F80" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G80" s="15" t="n">
+        <v>233</v>
+      </c>
+      <c r="H80" s="14" t="inlineStr">
+        <is>
+          <t>20/21</t>
+        </is>
+      </c>
+      <c r="I80" s="14" t="inlineStr">
         <is>
           <t>Result in Progress</t>
         </is>
       </c>
-      <c r="J80" s="8" t="n">
-        <v>619</v>
-      </c>
-      <c r="K80" s="9" t="n">
-        <v>29.47368421052632</v>
+      <c r="J80" s="15" t="n">
+        <v>245</v>
+      </c>
+      <c r="K80" s="16" t="n">
+        <v>11.65</v>
       </c>
     </row>
     <row r="81">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="I81" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J81" s="4" t="n">
@@ -4536,11 +4536,11 @@
         </is>
       </c>
       <c r="G82" s="8" t="n">
-        <v>535</v>
+        <v>922</v>
       </c>
       <c r="H82" s="7" t="inlineStr">
         <is>
-          <t>21/22</t>
+          <t>22/22</t>
         </is>
       </c>
       <c r="I82" s="7" t="inlineStr">
@@ -4549,10 +4549,10 @@
         </is>
       </c>
       <c r="J82" s="8" t="n">
-        <v>560</v>
+        <v>922</v>
       </c>
       <c r="K82" s="9" t="n">
-        <v>25.47619047619047</v>
+        <v>41.90909090909091</v>
       </c>
     </row>
     <row r="83">
@@ -4594,7 +4594,7 @@
       </c>
       <c r="I83" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J83" s="4" t="n">
@@ -5026,23 +5026,23 @@
         </is>
       </c>
       <c r="G92" s="4" t="n">
-        <v>11793</v>
+        <v>11931</v>
       </c>
       <c r="H92" s="3" t="inlineStr">
         <is>
-          <t>25/27</t>
+          <t>27/27</t>
         </is>
       </c>
       <c r="I92" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J92" s="4" t="n">
-        <v>12736</v>
+        <v>11931</v>
       </c>
       <c r="K92" s="5" t="n">
-        <v>471.72</v>
+        <v>441.8888888888889</v>
       </c>
     </row>
     <row r="93">
@@ -5271,11 +5271,11 @@
         </is>
       </c>
       <c r="G97" s="8" t="n">
-        <v>895</v>
+        <v>911</v>
       </c>
       <c r="H97" s="7" t="inlineStr">
         <is>
-          <t>24/27</t>
+          <t>25/27</t>
         </is>
       </c>
       <c r="I97" s="7" t="inlineStr">
@@ -5284,10 +5284,10 @@
         </is>
       </c>
       <c r="J97" s="8" t="n">
-        <v>1007</v>
+        <v>984</v>
       </c>
       <c r="K97" s="9" t="n">
-        <v>37.29166666666666</v>
+        <v>36.44</v>
       </c>
     </row>
     <row r="98">
@@ -5329,7 +5329,7 @@
       </c>
       <c r="I98" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J98" s="8" t="n">
@@ -5565,11 +5565,11 @@
         </is>
       </c>
       <c r="G103" s="4" t="n">
-        <v>18099</v>
+        <v>18726</v>
       </c>
       <c r="H103" s="3" t="inlineStr">
         <is>
-          <t>24/30</t>
+          <t>28/30</t>
         </is>
       </c>
       <c r="I103" s="3" t="inlineStr">
@@ -5578,10 +5578,10 @@
         </is>
       </c>
       <c r="J103" s="4" t="n">
-        <v>22624</v>
+        <v>20064</v>
       </c>
       <c r="K103" s="5" t="n">
-        <v>754.125</v>
+        <v>668.7857142857143</v>
       </c>
     </row>
     <row r="104">
@@ -5908,11 +5908,11 @@
         </is>
       </c>
       <c r="G110" s="4" t="n">
-        <v>11888</v>
+        <v>11024</v>
       </c>
       <c r="H110" s="3" t="inlineStr">
         <is>
-          <t>19/23</t>
+          <t>21/23</t>
         </is>
       </c>
       <c r="I110" s="3" t="inlineStr">
@@ -5921,10 +5921,10 @@
         </is>
       </c>
       <c r="J110" s="4" t="n">
-        <v>14391</v>
+        <v>12074</v>
       </c>
       <c r="K110" s="5" t="n">
-        <v>625.6842105263158</v>
+        <v>524.952380952381</v>
       </c>
     </row>
     <row r="111">
@@ -6643,11 +6643,11 @@
         </is>
       </c>
       <c r="G125" s="4" t="n">
-        <v>52009</v>
+        <v>54693</v>
       </c>
       <c r="H125" s="3" t="inlineStr">
         <is>
-          <t>32/35</t>
+          <t>35/35</t>
         </is>
       </c>
       <c r="I125" s="3" t="inlineStr">
@@ -6656,10 +6656,10 @@
         </is>
       </c>
       <c r="J125" s="4" t="n">
-        <v>56885</v>
+        <v>54693</v>
       </c>
       <c r="K125" s="5" t="n">
-        <v>1625.28125</v>
+        <v>1562.657142857143</v>
       </c>
     </row>
     <row r="126">
@@ -6888,11 +6888,11 @@
         </is>
       </c>
       <c r="G130" s="15" t="n">
-        <v>402</v>
+        <v>319</v>
       </c>
       <c r="H130" s="14" t="inlineStr">
         <is>
-          <t>19/20</t>
+          <t>20/21</t>
         </is>
       </c>
       <c r="I130" s="14" t="inlineStr">
@@ -6901,10 +6901,10 @@
         </is>
       </c>
       <c r="J130" s="15" t="n">
-        <v>423</v>
+        <v>335</v>
       </c>
       <c r="K130" s="16" t="n">
-        <v>21.15789473684211</v>
+        <v>15.95</v>
       </c>
     </row>
     <row r="131">
@@ -7084,11 +7084,11 @@
         </is>
       </c>
       <c r="G134" s="4" t="n">
-        <v>49765</v>
+        <v>53542</v>
       </c>
       <c r="H134" s="3" t="inlineStr">
         <is>
-          <t>20/22</t>
+          <t>22/23</t>
         </is>
       </c>
       <c r="I134" s="3" t="inlineStr">
@@ -7097,59 +7097,59 @@
         </is>
       </c>
       <c r="J134" s="4" t="n">
-        <v>54742</v>
+        <v>55976</v>
       </c>
       <c r="K134" s="5" t="n">
-        <v>2488.25</v>
+        <v>2433.727272727273</v>
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="6" t="inlineStr">
+      <c r="A135" s="10" t="inlineStr">
         <is>
           <t>PERAVURANI</t>
         </is>
       </c>
-      <c r="B135" s="7" t="n">
+      <c r="B135" s="10" t="n">
         <v>177</v>
       </c>
-      <c r="C135" s="7" t="inlineStr">
+      <c r="C135" s="10" t="inlineStr">
         <is>
           <t>ASHOKKUMAR. N</t>
         </is>
       </c>
-      <c r="D135" s="7" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E135" s="7" t="inlineStr">
+      <c r="D135" s="10" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E135" s="10" t="inlineStr">
         <is>
           <t>GOVI.ELANGO</t>
         </is>
       </c>
-      <c r="F135" s="7" t="inlineStr">
+      <c r="F135" s="10" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="G135" s="8" t="n">
-        <v>760</v>
-      </c>
-      <c r="H135" s="7" t="inlineStr">
-        <is>
-          <t>18/21</t>
-        </is>
-      </c>
-      <c r="I135" s="7" t="inlineStr">
+      <c r="G135" s="11" t="n">
+        <v>3170</v>
+      </c>
+      <c r="H135" s="10" t="inlineStr">
+        <is>
+          <t>19/21</t>
+        </is>
+      </c>
+      <c r="I135" s="10" t="inlineStr">
         <is>
           <t>Result in Progress</t>
         </is>
       </c>
-      <c r="J135" s="8" t="n">
-        <v>887</v>
-      </c>
-      <c r="K135" s="9" t="n">
-        <v>42.22222222222222</v>
+      <c r="J135" s="11" t="n">
+        <v>3504</v>
+      </c>
+      <c r="K135" s="12" t="n">
+        <v>166.8421052631579</v>
       </c>
     </row>
     <row r="136">
@@ -7191,7 +7191,7 @@
       </c>
       <c r="I136" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J136" s="4" t="n">
@@ -7240,7 +7240,7 @@
       </c>
       <c r="I137" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J137" s="4" t="n">
@@ -7329,11 +7329,11 @@
         </is>
       </c>
       <c r="G139" s="15" t="n">
-        <v>67</v>
+        <v>15</v>
       </c>
       <c r="H139" s="14" t="inlineStr">
         <is>
-          <t>14/22</t>
+          <t>15/22</t>
         </is>
       </c>
       <c r="I139" s="14" t="inlineStr">
@@ -7342,10 +7342,10 @@
         </is>
       </c>
       <c r="J139" s="15" t="n">
-        <v>105</v>
+        <v>22</v>
       </c>
       <c r="K139" s="16" t="n">
-        <v>4.785714285714286</v>
+        <v>1</v>
       </c>
     </row>
     <row r="140">
@@ -7427,11 +7427,11 @@
         </is>
       </c>
       <c r="G141" s="4" t="n">
-        <v>8013</v>
+        <v>8260</v>
       </c>
       <c r="H141" s="3" t="inlineStr">
         <is>
-          <t>23/25</t>
+          <t>25/25</t>
         </is>
       </c>
       <c r="I141" s="3" t="inlineStr">
@@ -7440,10 +7440,10 @@
         </is>
       </c>
       <c r="J141" s="4" t="n">
-        <v>8710</v>
+        <v>8260</v>
       </c>
       <c r="K141" s="5" t="n">
-        <v>348.3913043478261</v>
+        <v>330.4</v>
       </c>
     </row>
     <row r="142">
@@ -7790,52 +7790,52 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="2" t="inlineStr">
+      <c r="A149" s="10" t="inlineStr">
         <is>
           <t>RISHIVANDIYAM</t>
         </is>
       </c>
-      <c r="B149" s="3" t="n">
+      <c r="B149" s="10" t="n">
         <v>78</v>
       </c>
-      <c r="C149" s="3" t="inlineStr">
+      <c r="C149" s="10" t="inlineStr">
         <is>
           <t>KARTHIKEYAN K</t>
         </is>
       </c>
-      <c r="D149" s="3" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E149" s="3" t="inlineStr">
+      <c r="D149" s="10" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E149" s="10" t="inlineStr">
         <is>
           <t>ASHOK KUMAR G</t>
         </is>
       </c>
-      <c r="F149" s="3" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G149" s="4" t="n">
-        <v>6297</v>
-      </c>
-      <c r="H149" s="3" t="inlineStr">
-        <is>
-          <t>23/25</t>
-        </is>
-      </c>
-      <c r="I149" s="3" t="inlineStr">
+      <c r="F149" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G149" s="11" t="n">
+        <v>4862</v>
+      </c>
+      <c r="H149" s="10" t="inlineStr">
+        <is>
+          <t>25/25</t>
+        </is>
+      </c>
+      <c r="I149" s="10" t="inlineStr">
         <is>
           <t>Result in Progress</t>
         </is>
       </c>
-      <c r="J149" s="4" t="n">
-        <v>6845</v>
-      </c>
-      <c r="K149" s="5" t="n">
-        <v>273.7826086956522</v>
+      <c r="J149" s="11" t="n">
+        <v>4862</v>
+      </c>
+      <c r="K149" s="12" t="n">
+        <v>194.48</v>
       </c>
     </row>
     <row r="150">
@@ -8171,7 +8171,7 @@
       </c>
       <c r="I156" s="10" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J156" s="11" t="n">
@@ -8260,11 +8260,11 @@
         </is>
       </c>
       <c r="G158" s="4" t="n">
-        <v>6050</v>
+        <v>5989</v>
       </c>
       <c r="H158" s="3" t="inlineStr">
         <is>
-          <t>20/21</t>
+          <t>21/21</t>
         </is>
       </c>
       <c r="I158" s="3" t="inlineStr">
@@ -8273,10 +8273,10 @@
         </is>
       </c>
       <c r="J158" s="4" t="n">
-        <v>6352</v>
+        <v>5989</v>
       </c>
       <c r="K158" s="5" t="n">
-        <v>302.5</v>
+        <v>285.1904761904762</v>
       </c>
     </row>
     <row r="159">
@@ -8388,30 +8388,30 @@
       </c>
       <c r="C161" s="7" t="inlineStr">
         <is>
+          <t>G.KAPIL</t>
+        </is>
+      </c>
+      <c r="D161" s="7" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E161" s="7" t="inlineStr">
+        <is>
           <t>K.SARAVANAN</t>
         </is>
       </c>
-      <c r="D161" s="7" t="inlineStr">
+      <c r="F161" s="7" t="inlineStr">
         <is>
           <t>Pattali Makkal Katchi</t>
         </is>
       </c>
-      <c r="E161" s="7" t="inlineStr">
-        <is>
-          <t>G.KAPIL</t>
-        </is>
-      </c>
-      <c r="F161" s="7" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
       <c r="G161" s="8" t="n">
-        <v>1948</v>
+        <v>603</v>
       </c>
       <c r="H161" s="7" t="inlineStr">
         <is>
-          <t>19/25</t>
+          <t>21/25</t>
         </is>
       </c>
       <c r="I161" s="7" t="inlineStr">
@@ -8420,10 +8420,10 @@
         </is>
       </c>
       <c r="J161" s="8" t="n">
-        <v>2563</v>
+        <v>718</v>
       </c>
       <c r="K161" s="9" t="n">
-        <v>102.5263157894737</v>
+        <v>28.71428571428572</v>
       </c>
     </row>
     <row r="162">
@@ -8456,7 +8456,7 @@
         </is>
       </c>
       <c r="G162" s="4" t="n">
-        <v>95496</v>
+        <v>95820</v>
       </c>
       <c r="H162" s="3" t="inlineStr">
         <is>
@@ -8469,10 +8469,10 @@
         </is>
       </c>
       <c r="J162" s="4" t="n">
-        <v>98679</v>
+        <v>99014</v>
       </c>
       <c r="K162" s="5" t="n">
-        <v>3183.2</v>
+        <v>3194</v>
       </c>
     </row>
     <row r="163">
@@ -8505,11 +8505,11 @@
         </is>
       </c>
       <c r="G163" s="4" t="n">
-        <v>19098</v>
+        <v>19139</v>
       </c>
       <c r="H163" s="3" t="inlineStr">
         <is>
-          <t>26/27</t>
+          <t>27/27</t>
         </is>
       </c>
       <c r="I163" s="3" t="inlineStr">
@@ -8518,10 +8518,10 @@
         </is>
       </c>
       <c r="J163" s="4" t="n">
-        <v>19833</v>
+        <v>19139</v>
       </c>
       <c r="K163" s="5" t="n">
-        <v>734.5384615384615</v>
+        <v>708.8518518518518</v>
       </c>
     </row>
     <row r="164">
@@ -8603,11 +8603,11 @@
         </is>
       </c>
       <c r="G165" s="4" t="n">
-        <v>15210</v>
+        <v>15120</v>
       </c>
       <c r="H165" s="3" t="inlineStr">
         <is>
-          <t>28/29</t>
+          <t>29/31</t>
         </is>
       </c>
       <c r="I165" s="3" t="inlineStr">
@@ -8616,10 +8616,10 @@
         </is>
       </c>
       <c r="J165" s="4" t="n">
-        <v>15753</v>
+        <v>16163</v>
       </c>
       <c r="K165" s="5" t="n">
-        <v>543.2142857142857</v>
+        <v>521.3793103448276</v>
       </c>
     </row>
     <row r="166">
@@ -8701,11 +8701,11 @@
         </is>
       </c>
       <c r="G167" s="4" t="n">
-        <v>50921</v>
+        <v>54246</v>
       </c>
       <c r="H167" s="3" t="inlineStr">
         <is>
-          <t>30/32</t>
+          <t>33/33</t>
         </is>
       </c>
       <c r="I167" s="3" t="inlineStr">
@@ -8714,10 +8714,10 @@
         </is>
       </c>
       <c r="J167" s="4" t="n">
-        <v>54316</v>
+        <v>54246</v>
       </c>
       <c r="K167" s="5" t="n">
-        <v>1697.366666666667</v>
+        <v>1643.818181818182</v>
       </c>
     </row>
     <row r="168">
@@ -8852,7 +8852,7 @@
       </c>
       <c r="H170" s="3" t="inlineStr">
         <is>
-          <t>22/23</t>
+          <t>22/24</t>
         </is>
       </c>
       <c r="I170" s="3" t="inlineStr">
@@ -8861,7 +8861,7 @@
         </is>
       </c>
       <c r="J170" s="4" t="n">
-        <v>9058</v>
+        <v>9452</v>
       </c>
       <c r="K170" s="5" t="n">
         <v>393.8181818181818</v>
@@ -8906,7 +8906,7 @@
       </c>
       <c r="I171" s="10" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J171" s="11" t="n">
@@ -9004,7 +9004,7 @@
       </c>
       <c r="I173" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J173" s="4" t="n">
@@ -9044,11 +9044,11 @@
         </is>
       </c>
       <c r="G174" s="11" t="n">
-        <v>3174</v>
+        <v>4601</v>
       </c>
       <c r="H174" s="10" t="inlineStr">
         <is>
-          <t>22/24</t>
+          <t>23/24</t>
         </is>
       </c>
       <c r="I174" s="10" t="inlineStr">
@@ -9057,10 +9057,10 @@
         </is>
       </c>
       <c r="J174" s="11" t="n">
-        <v>3463</v>
+        <v>4801</v>
       </c>
       <c r="K174" s="12" t="n">
-        <v>144.2727272727273</v>
+        <v>200.0434782608696</v>
       </c>
     </row>
     <row r="175">
@@ -9338,23 +9338,23 @@
         </is>
       </c>
       <c r="G180" s="4" t="n">
-        <v>39107</v>
+        <v>39351</v>
       </c>
       <c r="H180" s="3" t="inlineStr">
         <is>
-          <t>28/33</t>
+          <t>33/33</t>
         </is>
       </c>
       <c r="I180" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J180" s="4" t="n">
-        <v>46090</v>
+        <v>39351</v>
       </c>
       <c r="K180" s="5" t="n">
-        <v>1396.678571428571</v>
+        <v>1192.454545454545</v>
       </c>
     </row>
     <row r="181">
@@ -9436,11 +9436,11 @@
         </is>
       </c>
       <c r="G182" s="4" t="n">
-        <v>8178</v>
+        <v>8570</v>
       </c>
       <c r="H182" s="3" t="inlineStr">
         <is>
-          <t>22/25</t>
+          <t>23/25</t>
         </is>
       </c>
       <c r="I182" s="3" t="inlineStr">
@@ -9449,10 +9449,10 @@
         </is>
       </c>
       <c r="J182" s="4" t="n">
-        <v>9293</v>
+        <v>9315</v>
       </c>
       <c r="K182" s="5" t="n">
-        <v>371.7272727272727</v>
+        <v>372.6086956521739</v>
       </c>
     </row>
     <row r="183">
@@ -9779,11 +9779,11 @@
         </is>
       </c>
       <c r="G189" s="4" t="n">
-        <v>14654</v>
+        <v>14725</v>
       </c>
       <c r="H189" s="3" t="inlineStr">
         <is>
-          <t>27/28</t>
+          <t>28/28</t>
         </is>
       </c>
       <c r="I189" s="3" t="inlineStr">
@@ -9792,10 +9792,10 @@
         </is>
       </c>
       <c r="J189" s="4" t="n">
-        <v>15197</v>
+        <v>14725</v>
       </c>
       <c r="K189" s="5" t="n">
-        <v>542.7407407407408</v>
+        <v>525.8928571428571</v>
       </c>
     </row>
     <row r="190">
@@ -9975,11 +9975,11 @@
         </is>
       </c>
       <c r="G193" s="8" t="n">
-        <v>702</v>
+        <v>734</v>
       </c>
       <c r="H193" s="7" t="inlineStr">
         <is>
-          <t>22/23</t>
+          <t>23/23</t>
         </is>
       </c>
       <c r="I193" s="7" t="inlineStr">
@@ -9991,7 +9991,7 @@
         <v>734</v>
       </c>
       <c r="K193" s="9" t="n">
-        <v>31.90909090909091</v>
+        <v>31.91304347826087</v>
       </c>
     </row>
     <row r="194">
@@ -10122,11 +10122,11 @@
         </is>
       </c>
       <c r="G196" s="4" t="n">
-        <v>25272</v>
+        <v>26685</v>
       </c>
       <c r="H196" s="3" t="inlineStr">
         <is>
-          <t>20/22</t>
+          <t>22/28</t>
         </is>
       </c>
       <c r="I196" s="3" t="inlineStr">
@@ -10135,10 +10135,10 @@
         </is>
       </c>
       <c r="J196" s="4" t="n">
-        <v>27799</v>
+        <v>33963</v>
       </c>
       <c r="K196" s="5" t="n">
-        <v>1263.6</v>
+        <v>1212.954545454545</v>
       </c>
     </row>
     <row r="197">
@@ -10269,11 +10269,11 @@
         </is>
       </c>
       <c r="G199" s="15" t="n">
-        <v>161</v>
+        <v>285</v>
       </c>
       <c r="H199" s="14" t="inlineStr">
         <is>
-          <t>23/24</t>
+          <t>24/24</t>
         </is>
       </c>
       <c r="I199" s="14" t="inlineStr">
@@ -10282,10 +10282,10 @@
         </is>
       </c>
       <c r="J199" s="15" t="n">
-        <v>168</v>
+        <v>285</v>
       </c>
       <c r="K199" s="16" t="n">
-        <v>7</v>
+        <v>11.875</v>
       </c>
     </row>
     <row r="200">
@@ -10367,11 +10367,11 @@
         </is>
       </c>
       <c r="G201" s="4" t="n">
-        <v>47382</v>
+        <v>47959</v>
       </c>
       <c r="H201" s="3" t="inlineStr">
         <is>
-          <t>21/22</t>
+          <t>22/23</t>
         </is>
       </c>
       <c r="I201" s="3" t="inlineStr">
@@ -10380,10 +10380,10 @@
         </is>
       </c>
       <c r="J201" s="4" t="n">
-        <v>49638</v>
+        <v>50139</v>
       </c>
       <c r="K201" s="5" t="n">
-        <v>2256.285714285714</v>
+        <v>2179.954545454545</v>
       </c>
     </row>
     <row r="202">
@@ -10465,11 +10465,11 @@
         </is>
       </c>
       <c r="G203" s="4" t="n">
-        <v>67902</v>
+        <v>69860</v>
       </c>
       <c r="H203" s="3" t="inlineStr">
         <is>
-          <t>31/34</t>
+          <t>33/34</t>
         </is>
       </c>
       <c r="I203" s="3" t="inlineStr">
@@ -10478,10 +10478,10 @@
         </is>
       </c>
       <c r="J203" s="4" t="n">
-        <v>74473</v>
+        <v>71977</v>
       </c>
       <c r="K203" s="5" t="n">
-        <v>2190.387096774194</v>
+        <v>2116.969696969697</v>
       </c>
     </row>
     <row r="204">
@@ -10563,11 +10563,11 @@
         </is>
       </c>
       <c r="G205" s="4" t="n">
-        <v>6857</v>
+        <v>5793</v>
       </c>
       <c r="H205" s="3" t="inlineStr">
         <is>
-          <t>23/25</t>
+          <t>27/27</t>
         </is>
       </c>
       <c r="I205" s="3" t="inlineStr">
@@ -10576,10 +10576,10 @@
         </is>
       </c>
       <c r="J205" s="4" t="n">
-        <v>7453</v>
+        <v>5793</v>
       </c>
       <c r="K205" s="5" t="n">
-        <v>298.1304347826087</v>
+        <v>214.5555555555555</v>
       </c>
     </row>
     <row r="206">
@@ -10714,7 +10714,7 @@
       </c>
       <c r="H208" s="7" t="inlineStr">
         <is>
-          <t>20/20</t>
+          <t>20/21</t>
         </is>
       </c>
       <c r="I208" s="7" t="inlineStr">
@@ -10723,7 +10723,7 @@
         </is>
       </c>
       <c r="J208" s="8" t="n">
-        <v>2541</v>
+        <v>2668</v>
       </c>
       <c r="K208" s="9" t="n">
         <v>127.05</v>
@@ -10857,11 +10857,11 @@
         </is>
       </c>
       <c r="G211" s="8" t="n">
-        <v>567</v>
+        <v>2267</v>
       </c>
       <c r="H211" s="7" t="inlineStr">
         <is>
-          <t>26/27</t>
+          <t>27/29</t>
         </is>
       </c>
       <c r="I211" s="7" t="inlineStr">
@@ -10870,10 +10870,10 @@
         </is>
       </c>
       <c r="J211" s="8" t="n">
-        <v>589</v>
+        <v>2435</v>
       </c>
       <c r="K211" s="9" t="n">
-        <v>21.80769230769231</v>
+        <v>83.96296296296296</v>
       </c>
     </row>
     <row r="212">
@@ -11249,11 +11249,11 @@
         </is>
       </c>
       <c r="G219" s="4" t="n">
-        <v>6635</v>
+        <v>6583</v>
       </c>
       <c r="H219" s="3" t="inlineStr">
         <is>
-          <t>22/23</t>
+          <t>23/23</t>
         </is>
       </c>
       <c r="I219" s="3" t="inlineStr">
@@ -11262,10 +11262,10 @@
         </is>
       </c>
       <c r="J219" s="4" t="n">
-        <v>6937</v>
+        <v>6583</v>
       </c>
       <c r="K219" s="5" t="n">
-        <v>301.5909090909091</v>
+        <v>286.2173913043478</v>
       </c>
     </row>
     <row r="220">
@@ -11552,7 +11552,7 @@
       </c>
       <c r="I225" s="14" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J225" s="15" t="n">
@@ -11592,11 +11592,11 @@
         </is>
       </c>
       <c r="G226" s="8" t="n">
-        <v>668</v>
+        <v>875</v>
       </c>
       <c r="H226" s="7" t="inlineStr">
         <is>
-          <t>21/23</t>
+          <t>22/23</t>
         </is>
       </c>
       <c r="I226" s="7" t="inlineStr">
@@ -11605,10 +11605,10 @@
         </is>
       </c>
       <c r="J226" s="8" t="n">
-        <v>732</v>
+        <v>915</v>
       </c>
       <c r="K226" s="9" t="n">
-        <v>31.80952380952381</v>
+        <v>39.77272727272727</v>
       </c>
     </row>
     <row r="227">
@@ -11797,7 +11797,7 @@
       </c>
       <c r="I230" s="10" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J230" s="11" t="n">
@@ -11837,11 +11837,11 @@
         </is>
       </c>
       <c r="G231" s="4" t="n">
-        <v>56186</v>
+        <v>61539</v>
       </c>
       <c r="H231" s="3" t="inlineStr">
         <is>
-          <t>18/20</t>
+          <t>20/22</t>
         </is>
       </c>
       <c r="I231" s="3" t="inlineStr">
@@ -11850,10 +11850,10 @@
         </is>
       </c>
       <c r="J231" s="4" t="n">
-        <v>62429</v>
+        <v>67693</v>
       </c>
       <c r="K231" s="5" t="n">
-        <v>3121.444444444444</v>
+        <v>3076.95</v>
       </c>
     </row>
     <row r="232">
@@ -11895,7 +11895,7 @@
       </c>
       <c r="I232" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J232" s="4" t="n">
@@ -12042,7 +12042,7 @@
       </c>
       <c r="I235" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J235" s="8" t="n">

</xml_diff>

<commit_message>
Election snapshot: 99.1% counted — 174 declared, TVK 107, DMDK loses POLUR
POLUR flipped TVK (344 lead, 6 rounds left); VEPPANAHALLI & TIRUKKOYILUR done counting.

https://claude.ai/code/session_01MizbUy44JG5sXyvaf3Wekb
</commit_message>
<xml_diff>
--- a/tn_election_results_may2026.xlsx
+++ b/tn_election_results_may2026.xlsx
@@ -1262,7 +1262,7 @@
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J15" s="4" t="n">
@@ -1654,7 +1654,7 @@
       </c>
       <c r="I23" s="10" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J23" s="11" t="n">
@@ -2135,11 +2135,11 @@
         </is>
       </c>
       <c r="G33" s="4" t="n">
-        <v>5794</v>
+        <v>5747</v>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>23/24</t>
+          <t>24/24</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -2148,10 +2148,10 @@
         </is>
       </c>
       <c r="J33" s="4" t="n">
-        <v>6046</v>
+        <v>5747</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>251.9130434782609</v>
+        <v>239.4583333333333</v>
       </c>
     </row>
     <row r="34">
@@ -2253,52 +2253,52 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="10" t="inlineStr">
+      <c r="A36" s="6" t="inlineStr">
         <is>
           <t>COLACHAL</t>
         </is>
       </c>
-      <c r="B36" s="10" t="n">
+      <c r="B36" s="7" t="n">
         <v>231</v>
       </c>
-      <c r="C36" s="10" t="inlineStr">
+      <c r="C36" s="7" t="inlineStr">
         <is>
           <t>THARAHAI CUTHBERT</t>
         </is>
       </c>
-      <c r="D36" s="10" t="inlineStr">
+      <c r="D36" s="7" t="inlineStr">
         <is>
           <t>Indian National Congress</t>
         </is>
       </c>
-      <c r="E36" s="10" t="inlineStr">
+      <c r="E36" s="7" t="inlineStr">
         <is>
           <t>PREM ALEX LAWRENCE</t>
         </is>
       </c>
-      <c r="F36" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G36" s="11" t="n">
-        <v>2698</v>
-      </c>
-      <c r="H36" s="10" t="inlineStr">
-        <is>
-          <t>24/28</t>
-        </is>
-      </c>
-      <c r="I36" s="10" t="inlineStr">
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G36" s="8" t="n">
+        <v>2833</v>
+      </c>
+      <c r="H36" s="7" t="inlineStr">
+        <is>
+          <t>28/28</t>
+        </is>
+      </c>
+      <c r="I36" s="7" t="inlineStr">
         <is>
           <t>Result in Progress</t>
         </is>
       </c>
-      <c r="J36" s="11" t="n">
-        <v>3148</v>
-      </c>
-      <c r="K36" s="12" t="n">
-        <v>112.4166666666667</v>
+      <c r="J36" s="8" t="n">
+        <v>2833</v>
+      </c>
+      <c r="K36" s="9" t="n">
+        <v>101.1785714285714</v>
       </c>
     </row>
     <row r="37">
@@ -2968,7 +2968,7 @@
         </is>
       </c>
       <c r="G50" s="4" t="n">
-        <v>13274</v>
+        <v>13390</v>
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
@@ -2981,10 +2981,10 @@
         </is>
       </c>
       <c r="J50" s="4" t="n">
-        <v>14538</v>
+        <v>14665</v>
       </c>
       <c r="K50" s="5" t="n">
-        <v>632.0952380952381</v>
+        <v>637.6190476190476</v>
       </c>
     </row>
     <row r="51">
@@ -3854,7 +3854,7 @@
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>20/20</t>
+          <t>20/21</t>
         </is>
       </c>
       <c r="I68" s="3" t="inlineStr">
@@ -3863,7 +3863,7 @@
         </is>
       </c>
       <c r="J68" s="4" t="n">
-        <v>5670</v>
+        <v>5954</v>
       </c>
       <c r="K68" s="5" t="n">
         <v>283.5</v>
@@ -4409,52 +4409,52 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="13" t="inlineStr">
+      <c r="A80" s="6" t="inlineStr">
         <is>
           <t>KULITHALAI</t>
         </is>
       </c>
-      <c r="B80" s="14" t="n">
+      <c r="B80" s="7" t="n">
         <v>137</v>
       </c>
-      <c r="C80" s="14" t="inlineStr">
+      <c r="C80" s="7" t="inlineStr">
         <is>
           <t>SURIYANUR. A. CHANDRAN</t>
         </is>
       </c>
-      <c r="D80" s="14" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E80" s="14" t="inlineStr">
+      <c r="D80" s="7" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E80" s="7" t="inlineStr">
         <is>
           <t>G.BALASUBRAMANI</t>
         </is>
       </c>
-      <c r="F80" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G80" s="15" t="n">
-        <v>233</v>
-      </c>
-      <c r="H80" s="14" t="inlineStr">
-        <is>
-          <t>20/21</t>
-        </is>
-      </c>
-      <c r="I80" s="14" t="inlineStr">
+      <c r="F80" s="7" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G80" s="8" t="n">
+        <v>579</v>
+      </c>
+      <c r="H80" s="7" t="inlineStr">
+        <is>
+          <t>21/21</t>
+        </is>
+      </c>
+      <c r="I80" s="7" t="inlineStr">
         <is>
           <t>Result in Progress</t>
         </is>
       </c>
-      <c r="J80" s="15" t="n">
-        <v>245</v>
-      </c>
-      <c r="K80" s="16" t="n">
-        <v>11.65</v>
+      <c r="J80" s="8" t="n">
+        <v>579</v>
+      </c>
+      <c r="K80" s="9" t="n">
+        <v>27.57142857142857</v>
       </c>
     </row>
     <row r="81">
@@ -5124,11 +5124,11 @@
         </is>
       </c>
       <c r="G94" s="4" t="n">
-        <v>61255</v>
+        <v>61509</v>
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
-          <t>26/27</t>
+          <t>27/27</t>
         </is>
       </c>
       <c r="I94" s="3" t="inlineStr">
@@ -5137,10 +5137,10 @@
         </is>
       </c>
       <c r="J94" s="4" t="n">
-        <v>63611</v>
+        <v>61509</v>
       </c>
       <c r="K94" s="5" t="n">
-        <v>2355.961538461539</v>
+        <v>2278.111111111111</v>
       </c>
     </row>
     <row r="95">
@@ -5271,11 +5271,11 @@
         </is>
       </c>
       <c r="G97" s="8" t="n">
-        <v>911</v>
+        <v>1050</v>
       </c>
       <c r="H97" s="7" t="inlineStr">
         <is>
-          <t>25/27</t>
+          <t>26/27</t>
         </is>
       </c>
       <c r="I97" s="7" t="inlineStr">
@@ -5284,10 +5284,10 @@
         </is>
       </c>
       <c r="J97" s="8" t="n">
-        <v>984</v>
+        <v>1090</v>
       </c>
       <c r="K97" s="9" t="n">
-        <v>36.44</v>
+        <v>40.38461538461539</v>
       </c>
     </row>
     <row r="98">
@@ -5516,11 +5516,11 @@
         </is>
       </c>
       <c r="G102" s="4" t="n">
-        <v>7600</v>
+        <v>7768</v>
       </c>
       <c r="H102" s="3" t="inlineStr">
         <is>
-          <t>26/27</t>
+          <t>27/27</t>
         </is>
       </c>
       <c r="I102" s="3" t="inlineStr">
@@ -5529,10 +5529,10 @@
         </is>
       </c>
       <c r="J102" s="4" t="n">
-        <v>7892</v>
+        <v>7768</v>
       </c>
       <c r="K102" s="5" t="n">
-        <v>292.3076923076923</v>
+        <v>287.7037037037037</v>
       </c>
     </row>
     <row r="103">
@@ -5565,11 +5565,11 @@
         </is>
       </c>
       <c r="G103" s="4" t="n">
-        <v>18726</v>
+        <v>19011</v>
       </c>
       <c r="H103" s="3" t="inlineStr">
         <is>
-          <t>28/30</t>
+          <t>29/30</t>
         </is>
       </c>
       <c r="I103" s="3" t="inlineStr">
@@ -5578,10 +5578,10 @@
         </is>
       </c>
       <c r="J103" s="4" t="n">
-        <v>20064</v>
+        <v>19667</v>
       </c>
       <c r="K103" s="5" t="n">
-        <v>668.7857142857143</v>
+        <v>655.551724137931</v>
       </c>
     </row>
     <row r="104">
@@ -5908,7 +5908,7 @@
         </is>
       </c>
       <c r="G110" s="4" t="n">
-        <v>11024</v>
+        <v>10466</v>
       </c>
       <c r="H110" s="3" t="inlineStr">
         <is>
@@ -5921,10 +5921,10 @@
         </is>
       </c>
       <c r="J110" s="4" t="n">
-        <v>12074</v>
+        <v>11463</v>
       </c>
       <c r="K110" s="5" t="n">
-        <v>524.952380952381</v>
+        <v>498.3809523809524</v>
       </c>
     </row>
     <row r="111">
@@ -6652,7 +6652,7 @@
       </c>
       <c r="I125" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J125" s="4" t="n">
@@ -7084,23 +7084,23 @@
         </is>
       </c>
       <c r="G134" s="4" t="n">
-        <v>53542</v>
+        <v>53715</v>
       </c>
       <c r="H134" s="3" t="inlineStr">
         <is>
-          <t>22/23</t>
+          <t>23/23</t>
         </is>
       </c>
       <c r="I134" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J134" s="4" t="n">
-        <v>55976</v>
+        <v>53715</v>
       </c>
       <c r="K134" s="5" t="n">
-        <v>2433.727272727273</v>
+        <v>2335.434782608696</v>
       </c>
     </row>
     <row r="135">
@@ -7310,30 +7310,30 @@
       </c>
       <c r="C139" s="14" t="inlineStr">
         <is>
+          <t>ABISHEK. R</t>
+        </is>
+      </c>
+      <c r="D139" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E139" s="14" t="inlineStr">
+        <is>
           <t>SARAVANAN. P</t>
         </is>
       </c>
-      <c r="D139" s="14" t="inlineStr">
+      <c r="F139" s="14" t="inlineStr">
         <is>
           <t>Desiya Murpokku Dravida Kazhagam</t>
         </is>
       </c>
-      <c r="E139" s="14" t="inlineStr">
-        <is>
-          <t>ABISHEK. R</t>
-        </is>
-      </c>
-      <c r="F139" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
       <c r="G139" s="15" t="n">
-        <v>15</v>
+        <v>344</v>
       </c>
       <c r="H139" s="14" t="inlineStr">
         <is>
-          <t>15/22</t>
+          <t>16/22</t>
         </is>
       </c>
       <c r="I139" s="14" t="inlineStr">
@@ -7342,10 +7342,10 @@
         </is>
       </c>
       <c r="J139" s="15" t="n">
-        <v>22</v>
+        <v>473</v>
       </c>
       <c r="K139" s="16" t="n">
-        <v>1</v>
+        <v>21.5</v>
       </c>
     </row>
     <row r="140">
@@ -8378,52 +8378,52 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="6" t="inlineStr">
+      <c r="A161" s="10" t="inlineStr">
         <is>
           <t>SHOLINGUR</t>
         </is>
       </c>
-      <c r="B161" s="7" t="n">
+      <c r="B161" s="10" t="n">
         <v>39</v>
       </c>
-      <c r="C161" s="7" t="inlineStr">
+      <c r="C161" s="10" t="inlineStr">
         <is>
           <t>G.KAPIL</t>
         </is>
       </c>
-      <c r="D161" s="7" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E161" s="7" t="inlineStr">
+      <c r="D161" s="10" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E161" s="10" t="inlineStr">
         <is>
           <t>K.SARAVANAN</t>
         </is>
       </c>
-      <c r="F161" s="7" t="inlineStr">
+      <c r="F161" s="10" t="inlineStr">
         <is>
           <t>Pattali Makkal Katchi</t>
         </is>
       </c>
-      <c r="G161" s="8" t="n">
-        <v>603</v>
-      </c>
-      <c r="H161" s="7" t="inlineStr">
-        <is>
-          <t>21/25</t>
-        </is>
-      </c>
-      <c r="I161" s="7" t="inlineStr">
+      <c r="G161" s="11" t="n">
+        <v>2954</v>
+      </c>
+      <c r="H161" s="10" t="inlineStr">
+        <is>
+          <t>22/25</t>
+        </is>
+      </c>
+      <c r="I161" s="10" t="inlineStr">
         <is>
           <t>Result in Progress</t>
         </is>
       </c>
-      <c r="J161" s="8" t="n">
-        <v>718</v>
-      </c>
-      <c r="K161" s="9" t="n">
-        <v>28.71428571428572</v>
+      <c r="J161" s="11" t="n">
+        <v>3357</v>
+      </c>
+      <c r="K161" s="12" t="n">
+        <v>134.2727272727273</v>
       </c>
     </row>
     <row r="162">
@@ -8603,11 +8603,11 @@
         </is>
       </c>
       <c r="G165" s="4" t="n">
-        <v>15120</v>
+        <v>15017</v>
       </c>
       <c r="H165" s="3" t="inlineStr">
         <is>
-          <t>29/31</t>
+          <t>30/31</t>
         </is>
       </c>
       <c r="I165" s="3" t="inlineStr">
@@ -8616,10 +8616,10 @@
         </is>
       </c>
       <c r="J165" s="4" t="n">
-        <v>16163</v>
+        <v>15518</v>
       </c>
       <c r="K165" s="5" t="n">
-        <v>521.3793103448276</v>
+        <v>500.5666666666667</v>
       </c>
     </row>
     <row r="166">
@@ -8710,7 +8710,7 @@
       </c>
       <c r="I167" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J167" s="4" t="n">
@@ -9436,11 +9436,11 @@
         </is>
       </c>
       <c r="G182" s="4" t="n">
-        <v>8570</v>
+        <v>8555</v>
       </c>
       <c r="H182" s="3" t="inlineStr">
         <is>
-          <t>23/25</t>
+          <t>25/25</t>
         </is>
       </c>
       <c r="I182" s="3" t="inlineStr">
@@ -9449,10 +9449,10 @@
         </is>
       </c>
       <c r="J182" s="4" t="n">
-        <v>9315</v>
+        <v>8555</v>
       </c>
       <c r="K182" s="5" t="n">
-        <v>372.6086956521739</v>
+        <v>342.2</v>
       </c>
     </row>
     <row r="183">
@@ -10572,7 +10572,7 @@
       </c>
       <c r="I205" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J205" s="4" t="n">
@@ -10661,11 +10661,11 @@
         </is>
       </c>
       <c r="G207" s="11" t="n">
-        <v>2595</v>
+        <v>3343</v>
       </c>
       <c r="H207" s="10" t="inlineStr">
         <is>
-          <t>19/23</t>
+          <t>20/23</t>
         </is>
       </c>
       <c r="I207" s="10" t="inlineStr">
@@ -10674,10 +10674,10 @@
         </is>
       </c>
       <c r="J207" s="11" t="n">
-        <v>3141</v>
+        <v>3844</v>
       </c>
       <c r="K207" s="12" t="n">
-        <v>136.578947368421</v>
+        <v>167.15</v>
       </c>
     </row>
     <row r="208">
@@ -10710,11 +10710,11 @@
         </is>
       </c>
       <c r="G208" s="8" t="n">
-        <v>2541</v>
+        <v>2629</v>
       </c>
       <c r="H208" s="7" t="inlineStr">
         <is>
-          <t>20/21</t>
+          <t>21/21</t>
         </is>
       </c>
       <c r="I208" s="7" t="inlineStr">
@@ -10723,10 +10723,10 @@
         </is>
       </c>
       <c r="J208" s="8" t="n">
-        <v>2668</v>
+        <v>2629</v>
       </c>
       <c r="K208" s="9" t="n">
-        <v>127.05</v>
+        <v>125.1904761904762</v>
       </c>
     </row>
     <row r="209">
@@ -10857,11 +10857,11 @@
         </is>
       </c>
       <c r="G211" s="8" t="n">
-        <v>2267</v>
+        <v>2351</v>
       </c>
       <c r="H211" s="7" t="inlineStr">
         <is>
-          <t>27/29</t>
+          <t>28/29</t>
         </is>
       </c>
       <c r="I211" s="7" t="inlineStr">
@@ -10873,7 +10873,7 @@
         <v>2435</v>
       </c>
       <c r="K211" s="9" t="n">
-        <v>83.96296296296296</v>
+        <v>83.96428571428571</v>
       </c>
     </row>
     <row r="212">
@@ -11209,7 +11209,7 @@
       </c>
       <c r="I218" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J218" s="4" t="n">
@@ -11258,7 +11258,7 @@
       </c>
       <c r="I219" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J219" s="4" t="n">
@@ -11837,11 +11837,11 @@
         </is>
       </c>
       <c r="G231" s="4" t="n">
-        <v>61539</v>
+        <v>62073</v>
       </c>
       <c r="H231" s="3" t="inlineStr">
         <is>
-          <t>20/22</t>
+          <t>22/22</t>
         </is>
       </c>
       <c r="I231" s="3" t="inlineStr">
@@ -11850,10 +11850,10 @@
         </is>
       </c>
       <c r="J231" s="4" t="n">
-        <v>67693</v>
+        <v>62073</v>
       </c>
       <c r="K231" s="5" t="n">
-        <v>3076.95</v>
+        <v>2821.5</v>
       </c>
     </row>
     <row r="232">

</xml_diff>

<commit_message>
Election snapshot: 99.4% counted — 184 declared, all knife-edges done counting
VEPPANAHALLI (DMK 138), TIRUKKOYILUR (AIADMK 285), PARAMATHI-VELUR (AIADMK 319) await declaration.

https://claude.ai/code/session_01MizbUy44JG5sXyvaf3Wekb
</commit_message>
<xml_diff>
--- a/tn_election_results_may2026.xlsx
+++ b/tn_election_results_may2026.xlsx
@@ -616,11 +616,11 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>27928</v>
+        <v>28863</v>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>29/31</t>
+          <t>30/31</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -629,10 +629,10 @@
         </is>
       </c>
       <c r="J2" s="4" t="n">
-        <v>29854</v>
+        <v>29825</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>963.0344827586207</v>
+        <v>962.1</v>
       </c>
     </row>
     <row r="3">
@@ -821,7 +821,7 @@
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J6" s="4" t="n">
@@ -1890,11 +1890,11 @@
         </is>
       </c>
       <c r="G28" s="4" t="n">
-        <v>34344</v>
+        <v>34867</v>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>32/36</t>
+          <t>34/36</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
@@ -1903,10 +1903,10 @@
         </is>
       </c>
       <c r="J28" s="4" t="n">
-        <v>38637</v>
+        <v>36918</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>1073.25</v>
+        <v>1025.5</v>
       </c>
     </row>
     <row r="29">
@@ -1939,11 +1939,11 @@
         </is>
       </c>
       <c r="G29" s="4" t="n">
-        <v>14562</v>
+        <v>14346</v>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>23/25</t>
+          <t>24/25</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
@@ -1952,10 +1952,10 @@
         </is>
       </c>
       <c r="J29" s="4" t="n">
-        <v>15828</v>
+        <v>14944</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>633.1304347826087</v>
+        <v>597.75</v>
       </c>
     </row>
     <row r="30">
@@ -2968,11 +2968,11 @@
         </is>
       </c>
       <c r="G50" s="4" t="n">
-        <v>13390</v>
+        <v>12389</v>
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>21/23</t>
+          <t>22/23</t>
         </is>
       </c>
       <c r="I50" s="3" t="inlineStr">
@@ -2981,10 +2981,10 @@
         </is>
       </c>
       <c r="J50" s="4" t="n">
-        <v>14665</v>
+        <v>12952</v>
       </c>
       <c r="K50" s="5" t="n">
-        <v>637.6190476190476</v>
+        <v>563.1363636363636</v>
       </c>
     </row>
     <row r="51">
@@ -3663,7 +3663,7 @@
       </c>
       <c r="I64" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J64" s="4" t="n">
@@ -3703,11 +3703,11 @@
         </is>
       </c>
       <c r="G65" s="8" t="n">
-        <v>1770</v>
+        <v>935</v>
       </c>
       <c r="H65" s="7" t="inlineStr">
         <is>
-          <t>25/34</t>
+          <t>26/34</t>
         </is>
       </c>
       <c r="I65" s="7" t="inlineStr">
@@ -3716,10 +3716,10 @@
         </is>
       </c>
       <c r="J65" s="8" t="n">
-        <v>2407</v>
+        <v>1223</v>
       </c>
       <c r="K65" s="9" t="n">
-        <v>70.8</v>
+        <v>35.96153846153846</v>
       </c>
     </row>
     <row r="66">
@@ -3850,11 +3850,11 @@
         </is>
       </c>
       <c r="G68" s="4" t="n">
-        <v>5670</v>
+        <v>5870</v>
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>20/21</t>
+          <t>21/21</t>
         </is>
       </c>
       <c r="I68" s="3" t="inlineStr">
@@ -3863,10 +3863,10 @@
         </is>
       </c>
       <c r="J68" s="4" t="n">
-        <v>5954</v>
+        <v>5870</v>
       </c>
       <c r="K68" s="5" t="n">
-        <v>283.5</v>
+        <v>279.5238095238095</v>
       </c>
     </row>
     <row r="69">
@@ -5271,11 +5271,11 @@
         </is>
       </c>
       <c r="G97" s="8" t="n">
-        <v>1050</v>
+        <v>1208</v>
       </c>
       <c r="H97" s="7" t="inlineStr">
         <is>
-          <t>26/27</t>
+          <t>27/27</t>
         </is>
       </c>
       <c r="I97" s="7" t="inlineStr">
@@ -5284,10 +5284,10 @@
         </is>
       </c>
       <c r="J97" s="8" t="n">
-        <v>1090</v>
+        <v>1208</v>
       </c>
       <c r="K97" s="9" t="n">
-        <v>40.38461538461539</v>
+        <v>44.74074074074074</v>
       </c>
     </row>
     <row r="98">
@@ -5525,7 +5525,7 @@
       </c>
       <c r="I102" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J102" s="4" t="n">
@@ -5565,11 +5565,11 @@
         </is>
       </c>
       <c r="G103" s="4" t="n">
-        <v>19011</v>
+        <v>19105</v>
       </c>
       <c r="H103" s="3" t="inlineStr">
         <is>
-          <t>29/30</t>
+          <t>30/30</t>
         </is>
       </c>
       <c r="I103" s="3" t="inlineStr">
@@ -5578,10 +5578,10 @@
         </is>
       </c>
       <c r="J103" s="4" t="n">
-        <v>19667</v>
+        <v>19105</v>
       </c>
       <c r="K103" s="5" t="n">
-        <v>655.551724137931</v>
+        <v>636.8333333333334</v>
       </c>
     </row>
     <row r="104">
@@ -5908,11 +5908,11 @@
         </is>
       </c>
       <c r="G110" s="4" t="n">
-        <v>10466</v>
+        <v>10883</v>
       </c>
       <c r="H110" s="3" t="inlineStr">
         <is>
-          <t>21/23</t>
+          <t>22/23</t>
         </is>
       </c>
       <c r="I110" s="3" t="inlineStr">
@@ -5921,10 +5921,10 @@
         </is>
       </c>
       <c r="J110" s="4" t="n">
-        <v>11463</v>
+        <v>11378</v>
       </c>
       <c r="K110" s="5" t="n">
-        <v>498.3809523809524</v>
+        <v>494.6818181818182</v>
       </c>
     </row>
     <row r="111">
@@ -6892,7 +6892,7 @@
       </c>
       <c r="H130" s="14" t="inlineStr">
         <is>
-          <t>20/21</t>
+          <t>20/20</t>
         </is>
       </c>
       <c r="I130" s="14" t="inlineStr">
@@ -6901,7 +6901,7 @@
         </is>
       </c>
       <c r="J130" s="15" t="n">
-        <v>335</v>
+        <v>319</v>
       </c>
       <c r="K130" s="16" t="n">
         <v>15.95</v>
@@ -7300,52 +7300,52 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="13" t="inlineStr">
+      <c r="A139" s="6" t="inlineStr">
         <is>
           <t>POLUR</t>
         </is>
       </c>
-      <c r="B139" s="14" t="n">
+      <c r="B139" s="7" t="n">
         <v>66</v>
       </c>
-      <c r="C139" s="14" t="inlineStr">
+      <c r="C139" s="7" t="inlineStr">
         <is>
           <t>ABISHEK. R</t>
         </is>
       </c>
-      <c r="D139" s="14" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E139" s="14" t="inlineStr">
+      <c r="D139" s="7" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E139" s="7" t="inlineStr">
         <is>
           <t>SARAVANAN. P</t>
         </is>
       </c>
-      <c r="F139" s="14" t="inlineStr">
+      <c r="F139" s="7" t="inlineStr">
         <is>
           <t>Desiya Murpokku Dravida Kazhagam</t>
         </is>
       </c>
-      <c r="G139" s="15" t="n">
-        <v>344</v>
-      </c>
-      <c r="H139" s="14" t="inlineStr">
-        <is>
-          <t>16/22</t>
-        </is>
-      </c>
-      <c r="I139" s="14" t="inlineStr">
+      <c r="G139" s="8" t="n">
+        <v>944</v>
+      </c>
+      <c r="H139" s="7" t="inlineStr">
+        <is>
+          <t>17/22</t>
+        </is>
+      </c>
+      <c r="I139" s="7" t="inlineStr">
         <is>
           <t>Result in Progress</t>
         </is>
       </c>
-      <c r="J139" s="15" t="n">
-        <v>473</v>
-      </c>
-      <c r="K139" s="16" t="n">
-        <v>21.5</v>
+      <c r="J139" s="8" t="n">
+        <v>1222</v>
+      </c>
+      <c r="K139" s="9" t="n">
+        <v>55.52941176470588</v>
       </c>
     </row>
     <row r="140">
@@ -7387,7 +7387,7 @@
       </c>
       <c r="I140" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J140" s="4" t="n">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="I163" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J163" s="4" t="n">
@@ -8603,11 +8603,11 @@
         </is>
       </c>
       <c r="G165" s="4" t="n">
-        <v>15017</v>
+        <v>15081</v>
       </c>
       <c r="H165" s="3" t="inlineStr">
         <is>
-          <t>30/31</t>
+          <t>31/31</t>
         </is>
       </c>
       <c r="I165" s="3" t="inlineStr">
@@ -8616,10 +8616,10 @@
         </is>
       </c>
       <c r="J165" s="4" t="n">
-        <v>15518</v>
+        <v>15081</v>
       </c>
       <c r="K165" s="5" t="n">
-        <v>500.5666666666667</v>
+        <v>486.483870967742</v>
       </c>
     </row>
     <row r="166">
@@ -8759,7 +8759,7 @@
       </c>
       <c r="I168" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J168" s="4" t="n">
@@ -8848,23 +8848,23 @@
         </is>
       </c>
       <c r="G170" s="4" t="n">
-        <v>8664</v>
+        <v>8581</v>
       </c>
       <c r="H170" s="3" t="inlineStr">
         <is>
-          <t>22/24</t>
+          <t>24/24</t>
         </is>
       </c>
       <c r="I170" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J170" s="4" t="n">
-        <v>9452</v>
+        <v>8581</v>
       </c>
       <c r="K170" s="5" t="n">
-        <v>393.8181818181818</v>
+        <v>357.5416666666667</v>
       </c>
     </row>
     <row r="171">
@@ -9015,52 +9015,52 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="10" t="inlineStr">
+      <c r="A174" s="2" t="inlineStr">
         <is>
           <t>THALLI</t>
         </is>
       </c>
-      <c r="B174" s="10" t="n">
+      <c r="B174" s="3" t="n">
         <v>56</v>
       </c>
-      <c r="C174" s="10" t="inlineStr">
+      <c r="C174" s="3" t="inlineStr">
         <is>
           <t>RAMACHANDRAN. T</t>
         </is>
       </c>
-      <c r="D174" s="10" t="inlineStr">
+      <c r="D174" s="3" t="inlineStr">
         <is>
           <t>Communist Party of India</t>
         </is>
       </c>
-      <c r="E174" s="10" t="inlineStr">
+      <c r="E174" s="3" t="inlineStr">
         <is>
           <t>DR.NAGESH KUMAR. C</t>
         </is>
       </c>
-      <c r="F174" s="10" t="inlineStr">
+      <c r="F174" s="3" t="inlineStr">
         <is>
           <t>Bharatiya Janata Party</t>
         </is>
       </c>
-      <c r="G174" s="11" t="n">
-        <v>4601</v>
-      </c>
-      <c r="H174" s="10" t="inlineStr">
-        <is>
-          <t>23/24</t>
-        </is>
-      </c>
-      <c r="I174" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J174" s="11" t="n">
-        <v>4801</v>
-      </c>
-      <c r="K174" s="12" t="n">
-        <v>200.0434782608696</v>
+      <c r="G174" s="4" t="n">
+        <v>5240</v>
+      </c>
+      <c r="H174" s="3" t="inlineStr">
+        <is>
+          <t>24/24</t>
+        </is>
+      </c>
+      <c r="I174" s="3" t="inlineStr">
+        <is>
+          <t>Result Declared</t>
+        </is>
+      </c>
+      <c r="J174" s="4" t="n">
+        <v>5240</v>
+      </c>
+      <c r="K174" s="5" t="n">
+        <v>218.3333333333333</v>
       </c>
     </row>
     <row r="175">
@@ -9984,7 +9984,7 @@
       </c>
       <c r="I193" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J193" s="8" t="n">
@@ -10122,11 +10122,11 @@
         </is>
       </c>
       <c r="G196" s="4" t="n">
-        <v>26685</v>
+        <v>27140</v>
       </c>
       <c r="H196" s="3" t="inlineStr">
         <is>
-          <t>22/28</t>
+          <t>25/28</t>
         </is>
       </c>
       <c r="I196" s="3" t="inlineStr">
@@ -10135,10 +10135,10 @@
         </is>
       </c>
       <c r="J196" s="4" t="n">
-        <v>33963</v>
+        <v>30397</v>
       </c>
       <c r="K196" s="5" t="n">
-        <v>1212.954545454545</v>
+        <v>1085.6</v>
       </c>
     </row>
     <row r="197">
@@ -10367,11 +10367,11 @@
         </is>
       </c>
       <c r="G201" s="4" t="n">
-        <v>47959</v>
+        <v>48263</v>
       </c>
       <c r="H201" s="3" t="inlineStr">
         <is>
-          <t>22/23</t>
+          <t>23/23</t>
         </is>
       </c>
       <c r="I201" s="3" t="inlineStr">
@@ -10380,10 +10380,10 @@
         </is>
       </c>
       <c r="J201" s="4" t="n">
-        <v>50139</v>
+        <v>48263</v>
       </c>
       <c r="K201" s="5" t="n">
-        <v>2179.954545454545</v>
+        <v>2098.391304347826</v>
       </c>
     </row>
     <row r="202">
@@ -10465,11 +10465,11 @@
         </is>
       </c>
       <c r="G203" s="4" t="n">
-        <v>69860</v>
+        <v>69992</v>
       </c>
       <c r="H203" s="3" t="inlineStr">
         <is>
-          <t>33/34</t>
+          <t>34/34</t>
         </is>
       </c>
       <c r="I203" s="3" t="inlineStr">
@@ -10478,10 +10478,10 @@
         </is>
       </c>
       <c r="J203" s="4" t="n">
-        <v>71977</v>
+        <v>69992</v>
       </c>
       <c r="K203" s="5" t="n">
-        <v>2116.969696969697</v>
+        <v>2058.588235294118</v>
       </c>
     </row>
     <row r="204">
@@ -11846,7 +11846,7 @@
       </c>
       <c r="I231" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J231" s="4" t="n">

</xml_diff>

<commit_message>
Election snapshot: 99.7% counted — 209 declared, TIRUPPATTUR genuine DMK flip (212 votes)
KANNIYAKUMARI done counting (AIADMK 214); TIRUPPATTUR last live contest (DMK 212, 3 rounds left).

https://claude.ai/code/session_01MizbUy44JG5sXyvaf3Wekb
</commit_message>
<xml_diff>
--- a/tn_election_results_may2026.xlsx
+++ b/tn_election_results_may2026.xlsx
@@ -616,23 +616,23 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>28863</v>
+        <v>29609</v>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>30/31</t>
+          <t>31/31</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J2" s="4" t="n">
-        <v>29825</v>
+        <v>29609</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>962.1</v>
+        <v>955.1290322580645</v>
       </c>
     </row>
     <row r="3">
@@ -861,11 +861,11 @@
         </is>
       </c>
       <c r="G7" s="4" t="n">
-        <v>7327</v>
+        <v>7272</v>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>22/22</t>
+          <t>23/24</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -874,10 +874,10 @@
         </is>
       </c>
       <c r="J7" s="4" t="n">
-        <v>7327</v>
+        <v>7588</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>333.0454545454546</v>
+        <v>316.1739130434783</v>
       </c>
     </row>
     <row r="8">
@@ -1164,7 +1164,7 @@
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J13" s="4" t="n">
@@ -1801,7 +1801,7 @@
       </c>
       <c r="I26" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J26" s="8" t="n">
@@ -1890,11 +1890,11 @@
         </is>
       </c>
       <c r="G28" s="4" t="n">
-        <v>34867</v>
+        <v>35714</v>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>34/36</t>
+          <t>36/40</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
@@ -1903,10 +1903,10 @@
         </is>
       </c>
       <c r="J28" s="4" t="n">
-        <v>36918</v>
+        <v>39682</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>1025.5</v>
+        <v>992.0555555555555</v>
       </c>
     </row>
     <row r="29">
@@ -1939,11 +1939,11 @@
         </is>
       </c>
       <c r="G29" s="4" t="n">
-        <v>14346</v>
+        <v>13278</v>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>24/25</t>
+          <t>25/25</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
@@ -1952,10 +1952,10 @@
         </is>
       </c>
       <c r="J29" s="4" t="n">
-        <v>14944</v>
+        <v>13278</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>597.75</v>
+        <v>531.12</v>
       </c>
     </row>
     <row r="30">
@@ -2144,7 +2144,7 @@
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J33" s="4" t="n">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="I39" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J39" s="8" t="n">
@@ -2968,11 +2968,11 @@
         </is>
       </c>
       <c r="G50" s="4" t="n">
-        <v>12389</v>
+        <v>12645</v>
       </c>
       <c r="H50" s="3" t="inlineStr">
         <is>
-          <t>22/23</t>
+          <t>24/24</t>
         </is>
       </c>
       <c r="I50" s="3" t="inlineStr">
@@ -2981,10 +2981,10 @@
         </is>
       </c>
       <c r="J50" s="4" t="n">
-        <v>12952</v>
+        <v>12645</v>
       </c>
       <c r="K50" s="5" t="n">
-        <v>563.1363636363636</v>
+        <v>526.875</v>
       </c>
     </row>
     <row r="51">
@@ -3674,52 +3674,52 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="6" t="inlineStr">
+      <c r="A65" s="13" t="inlineStr">
         <is>
           <t>KANNIYAKUMARI</t>
         </is>
       </c>
-      <c r="B65" s="7" t="n">
+      <c r="B65" s="14" t="n">
         <v>229</v>
       </c>
-      <c r="C65" s="7" t="inlineStr">
+      <c r="C65" s="14" t="inlineStr">
         <is>
           <t>THALAVAI SUNDARAM. N</t>
         </is>
       </c>
-      <c r="D65" s="7" t="inlineStr">
+      <c r="D65" s="14" t="inlineStr">
         <is>
           <t>All India Anna Dravida Munnetra Kazhagam</t>
         </is>
       </c>
-      <c r="E65" s="7" t="inlineStr">
+      <c r="E65" s="14" t="inlineStr">
         <is>
           <t>MAHESH.R</t>
         </is>
       </c>
-      <c r="F65" s="7" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="G65" s="8" t="n">
-        <v>935</v>
-      </c>
-      <c r="H65" s="7" t="inlineStr">
-        <is>
-          <t>26/34</t>
-        </is>
-      </c>
-      <c r="I65" s="7" t="inlineStr">
+      <c r="F65" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="G65" s="15" t="n">
+        <v>214</v>
+      </c>
+      <c r="H65" s="14" t="inlineStr">
+        <is>
+          <t>34/34</t>
+        </is>
+      </c>
+      <c r="I65" s="14" t="inlineStr">
         <is>
           <t>Result in Progress</t>
         </is>
       </c>
-      <c r="J65" s="8" t="n">
-        <v>1223</v>
-      </c>
-      <c r="K65" s="9" t="n">
-        <v>35.96153846153846</v>
+      <c r="J65" s="15" t="n">
+        <v>214</v>
+      </c>
+      <c r="K65" s="16" t="n">
+        <v>6.294117647058823</v>
       </c>
     </row>
     <row r="66">
@@ -3801,11 +3801,11 @@
         </is>
       </c>
       <c r="G67" s="8" t="n">
-        <v>1340</v>
+        <v>1888</v>
       </c>
       <c r="H67" s="7" t="inlineStr">
         <is>
-          <t>19/21</t>
+          <t>20/21</t>
         </is>
       </c>
       <c r="I67" s="7" t="inlineStr">
@@ -3814,10 +3814,10 @@
         </is>
       </c>
       <c r="J67" s="8" t="n">
-        <v>1481</v>
+        <v>1982</v>
       </c>
       <c r="K67" s="9" t="n">
-        <v>70.52631578947368</v>
+        <v>94.40000000000001</v>
       </c>
     </row>
     <row r="68">
@@ -3859,7 +3859,7 @@
       </c>
       <c r="I68" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J68" s="4" t="n">
@@ -4536,23 +4536,23 @@
         </is>
       </c>
       <c r="G82" s="8" t="n">
-        <v>922</v>
+        <v>679</v>
       </c>
       <c r="H82" s="7" t="inlineStr">
         <is>
-          <t>22/22</t>
+          <t>23/23</t>
         </is>
       </c>
       <c r="I82" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J82" s="8" t="n">
-        <v>922</v>
+        <v>679</v>
       </c>
       <c r="K82" s="9" t="n">
-        <v>41.90909090909091</v>
+        <v>29.52173913043478</v>
       </c>
     </row>
     <row r="83">
@@ -4692,7 +4692,7 @@
       </c>
       <c r="I85" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J85" s="8" t="n">
@@ -5133,7 +5133,7 @@
       </c>
       <c r="I94" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J94" s="4" t="n">
@@ -5427,7 +5427,7 @@
       </c>
       <c r="I100" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J100" s="4" t="n">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="I103" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J103" s="4" t="n">
@@ -5868,7 +5868,7 @@
       </c>
       <c r="I109" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J109" s="4" t="n">
@@ -5908,23 +5908,23 @@
         </is>
       </c>
       <c r="G110" s="4" t="n">
-        <v>10883</v>
+        <v>11008</v>
       </c>
       <c r="H110" s="3" t="inlineStr">
         <is>
-          <t>22/23</t>
+          <t>23/23</t>
         </is>
       </c>
       <c r="I110" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J110" s="4" t="n">
-        <v>11378</v>
+        <v>11008</v>
       </c>
       <c r="K110" s="5" t="n">
-        <v>494.6818181818182</v>
+        <v>478.6086956521739</v>
       </c>
     </row>
     <row r="111">
@@ -6505,7 +6505,7 @@
       </c>
       <c r="I122" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J122" s="8" t="n">
@@ -6888,7 +6888,7 @@
         </is>
       </c>
       <c r="G130" s="15" t="n">
-        <v>319</v>
+        <v>308</v>
       </c>
       <c r="H130" s="14" t="inlineStr">
         <is>
@@ -6897,14 +6897,14 @@
       </c>
       <c r="I130" s="14" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J130" s="15" t="n">
-        <v>319</v>
+        <v>308</v>
       </c>
       <c r="K130" s="16" t="n">
-        <v>15.95</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="131">
@@ -7133,11 +7133,11 @@
         </is>
       </c>
       <c r="G135" s="11" t="n">
-        <v>3170</v>
+        <v>3162</v>
       </c>
       <c r="H135" s="10" t="inlineStr">
         <is>
-          <t>19/21</t>
+          <t>21/21</t>
         </is>
       </c>
       <c r="I135" s="10" t="inlineStr">
@@ -7146,10 +7146,10 @@
         </is>
       </c>
       <c r="J135" s="11" t="n">
-        <v>3504</v>
+        <v>3162</v>
       </c>
       <c r="K135" s="12" t="n">
-        <v>166.8421052631579</v>
+        <v>150.5714285714286</v>
       </c>
     </row>
     <row r="136">
@@ -7329,11 +7329,11 @@
         </is>
       </c>
       <c r="G139" s="8" t="n">
-        <v>944</v>
+        <v>855</v>
       </c>
       <c r="H139" s="7" t="inlineStr">
         <is>
-          <t>17/22</t>
+          <t>19/22</t>
         </is>
       </c>
       <c r="I139" s="7" t="inlineStr">
@@ -7342,10 +7342,10 @@
         </is>
       </c>
       <c r="J139" s="8" t="n">
-        <v>1222</v>
+        <v>990</v>
       </c>
       <c r="K139" s="9" t="n">
-        <v>55.52941176470588</v>
+        <v>45</v>
       </c>
     </row>
     <row r="140">
@@ -7436,7 +7436,7 @@
       </c>
       <c r="I141" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J141" s="4" t="n">
@@ -7828,7 +7828,7 @@
       </c>
       <c r="I149" s="10" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J149" s="11" t="n">
@@ -8269,7 +8269,7 @@
       </c>
       <c r="I158" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J158" s="4" t="n">
@@ -8407,11 +8407,11 @@
         </is>
       </c>
       <c r="G161" s="11" t="n">
-        <v>2954</v>
+        <v>3163</v>
       </c>
       <c r="H161" s="10" t="inlineStr">
         <is>
-          <t>22/25</t>
+          <t>23/25</t>
         </is>
       </c>
       <c r="I161" s="10" t="inlineStr">
@@ -8420,10 +8420,10 @@
         </is>
       </c>
       <c r="J161" s="11" t="n">
-        <v>3357</v>
+        <v>3438</v>
       </c>
       <c r="K161" s="12" t="n">
-        <v>134.2727272727273</v>
+        <v>137.5217391304348</v>
       </c>
     </row>
     <row r="162">
@@ -8456,11 +8456,11 @@
         </is>
       </c>
       <c r="G162" s="4" t="n">
-        <v>95820</v>
+        <v>96370</v>
       </c>
       <c r="H162" s="3" t="inlineStr">
         <is>
-          <t>30/31</t>
+          <t>33/33</t>
         </is>
       </c>
       <c r="I162" s="3" t="inlineStr">
@@ -8469,10 +8469,10 @@
         </is>
       </c>
       <c r="J162" s="4" t="n">
-        <v>99014</v>
+        <v>96370</v>
       </c>
       <c r="K162" s="5" t="n">
-        <v>3194</v>
+        <v>2920.30303030303</v>
       </c>
     </row>
     <row r="163">
@@ -9249,7 +9249,7 @@
       </c>
       <c r="I178" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J178" s="8" t="n">
@@ -9298,7 +9298,7 @@
       </c>
       <c r="I179" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J179" s="4" t="n">
@@ -9445,7 +9445,7 @@
       </c>
       <c r="I182" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J182" s="4" t="n">
@@ -9788,7 +9788,7 @@
       </c>
       <c r="I189" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J189" s="4" t="n">
@@ -10122,23 +10122,23 @@
         </is>
       </c>
       <c r="G196" s="4" t="n">
-        <v>27140</v>
+        <v>27416</v>
       </c>
       <c r="H196" s="3" t="inlineStr">
         <is>
-          <t>25/28</t>
+          <t>28/28</t>
         </is>
       </c>
       <c r="I196" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J196" s="4" t="n">
-        <v>30397</v>
+        <v>27416</v>
       </c>
       <c r="K196" s="5" t="n">
-        <v>1085.6</v>
+        <v>979.1428571428571</v>
       </c>
     </row>
     <row r="197">
@@ -10229,7 +10229,7 @@
       </c>
       <c r="I198" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J198" s="4" t="n">
@@ -10387,52 +10387,52 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" s="6" t="inlineStr">
+      <c r="A202" s="13" t="inlineStr">
         <is>
           <t>TIRUPPATTUR</t>
         </is>
       </c>
-      <c r="B202" s="7" t="n">
+      <c r="B202" s="14" t="n">
         <v>185</v>
       </c>
-      <c r="C202" s="7" t="inlineStr">
+      <c r="C202" s="14" t="inlineStr">
         <is>
           <t>PERIAKARUPPAN. KR</t>
         </is>
       </c>
-      <c r="D202" s="7" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E202" s="7" t="inlineStr">
+      <c r="D202" s="14" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E202" s="14" t="inlineStr">
         <is>
           <t>SEENIVASA SETHUPATHY. R</t>
         </is>
       </c>
-      <c r="F202" s="7" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G202" s="8" t="n">
-        <v>1127</v>
-      </c>
-      <c r="H202" s="7" t="inlineStr">
-        <is>
-          <t>25/27</t>
-        </is>
-      </c>
-      <c r="I202" s="7" t="inlineStr">
+      <c r="F202" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G202" s="15" t="n">
+        <v>212</v>
+      </c>
+      <c r="H202" s="14" t="inlineStr">
+        <is>
+          <t>27/30</t>
+        </is>
+      </c>
+      <c r="I202" s="14" t="inlineStr">
         <is>
           <t>Result in Progress</t>
         </is>
       </c>
-      <c r="J202" s="8" t="n">
-        <v>1217</v>
-      </c>
-      <c r="K202" s="9" t="n">
-        <v>45.08</v>
+      <c r="J202" s="15" t="n">
+        <v>236</v>
+      </c>
+      <c r="K202" s="16" t="n">
+        <v>7.851851851851852</v>
       </c>
     </row>
     <row r="203">
@@ -10661,11 +10661,11 @@
         </is>
       </c>
       <c r="G207" s="11" t="n">
-        <v>3343</v>
+        <v>3541</v>
       </c>
       <c r="H207" s="10" t="inlineStr">
         <is>
-          <t>20/23</t>
+          <t>21/23</t>
         </is>
       </c>
       <c r="I207" s="10" t="inlineStr">
@@ -10674,10 +10674,10 @@
         </is>
       </c>
       <c r="J207" s="11" t="n">
-        <v>3844</v>
+        <v>3878</v>
       </c>
       <c r="K207" s="12" t="n">
-        <v>167.15</v>
+        <v>168.6190476190476</v>
       </c>
     </row>
     <row r="208">
@@ -10719,7 +10719,7 @@
       </c>
       <c r="I208" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J208" s="8" t="n">
@@ -10857,11 +10857,11 @@
         </is>
       </c>
       <c r="G211" s="8" t="n">
-        <v>2351</v>
+        <v>2277</v>
       </c>
       <c r="H211" s="7" t="inlineStr">
         <is>
-          <t>28/29</t>
+          <t>29/29</t>
         </is>
       </c>
       <c r="I211" s="7" t="inlineStr">
@@ -10870,10 +10870,10 @@
         </is>
       </c>
       <c r="J211" s="8" t="n">
-        <v>2435</v>
+        <v>2277</v>
       </c>
       <c r="K211" s="9" t="n">
-        <v>83.96428571428571</v>
+        <v>78.51724137931035</v>
       </c>
     </row>
     <row r="212">

</xml_diff>

<commit_message>
Election snapshot: 100% counted — 222 declared, POLUR TVK 227, TIRUPPATTUR DMK 30
Counting complete; TIRUPPATTUR (DMK 30 votes) last undecided seat awaiting declaration.

https://claude.ai/code/session_01MizbUy44JG5sXyvaf3Wekb
</commit_message>
<xml_diff>
--- a/tn_election_results_may2026.xlsx
+++ b/tn_election_results_may2026.xlsx
@@ -861,23 +861,23 @@
         </is>
       </c>
       <c r="G7" s="4" t="n">
-        <v>7272</v>
+        <v>7131</v>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>23/24</t>
+          <t>24/24</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J7" s="4" t="n">
-        <v>7588</v>
+        <v>7131</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>316.1739130434783</v>
+        <v>297.125</v>
       </c>
     </row>
     <row r="8">
@@ -1850,7 +1850,7 @@
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J27" s="4" t="n">
@@ -1890,11 +1890,11 @@
         </is>
       </c>
       <c r="G28" s="4" t="n">
-        <v>35714</v>
+        <v>35641</v>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>36/40</t>
+          <t>40/40</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
@@ -1903,10 +1903,10 @@
         </is>
       </c>
       <c r="J28" s="4" t="n">
-        <v>39682</v>
+        <v>35641</v>
       </c>
       <c r="K28" s="5" t="n">
-        <v>992.0555555555555</v>
+        <v>891.025</v>
       </c>
     </row>
     <row r="29">
@@ -1948,7 +1948,7 @@
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J29" s="4" t="n">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="I36" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J36" s="8" t="n">
@@ -2879,7 +2879,7 @@
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J48" s="4" t="n">
@@ -3761,7 +3761,7 @@
       </c>
       <c r="I66" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J66" s="4" t="n">
@@ -3801,11 +3801,11 @@
         </is>
       </c>
       <c r="G67" s="8" t="n">
-        <v>1888</v>
+        <v>1821</v>
       </c>
       <c r="H67" s="7" t="inlineStr">
         <is>
-          <t>20/21</t>
+          <t>21/21</t>
         </is>
       </c>
       <c r="I67" s="7" t="inlineStr">
@@ -3814,10 +3814,10 @@
         </is>
       </c>
       <c r="J67" s="8" t="n">
-        <v>1982</v>
+        <v>1821</v>
       </c>
       <c r="K67" s="9" t="n">
-        <v>94.40000000000001</v>
+        <v>86.71428571428571</v>
       </c>
     </row>
     <row r="68">
@@ -4398,7 +4398,7 @@
       </c>
       <c r="I79" s="10" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J79" s="11" t="n">
@@ -4447,7 +4447,7 @@
       </c>
       <c r="I80" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J80" s="8" t="n">
@@ -7300,52 +7300,52 @@
       </c>
     </row>
     <row r="139">
-      <c r="A139" s="6" t="inlineStr">
+      <c r="A139" s="13" t="inlineStr">
         <is>
           <t>POLUR</t>
         </is>
       </c>
-      <c r="B139" s="7" t="n">
+      <c r="B139" s="14" t="n">
         <v>66</v>
       </c>
-      <c r="C139" s="7" t="inlineStr">
+      <c r="C139" s="14" t="inlineStr">
         <is>
           <t>ABISHEK. R</t>
         </is>
       </c>
-      <c r="D139" s="7" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E139" s="7" t="inlineStr">
+      <c r="D139" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E139" s="14" t="inlineStr">
         <is>
           <t>SARAVANAN. P</t>
         </is>
       </c>
-      <c r="F139" s="7" t="inlineStr">
+      <c r="F139" s="14" t="inlineStr">
         <is>
           <t>Desiya Murpokku Dravida Kazhagam</t>
         </is>
       </c>
-      <c r="G139" s="8" t="n">
-        <v>855</v>
-      </c>
-      <c r="H139" s="7" t="inlineStr">
-        <is>
-          <t>19/22</t>
-        </is>
-      </c>
-      <c r="I139" s="7" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J139" s="8" t="n">
-        <v>990</v>
-      </c>
-      <c r="K139" s="9" t="n">
-        <v>45</v>
+      <c r="G139" s="15" t="n">
+        <v>227</v>
+      </c>
+      <c r="H139" s="14" t="inlineStr">
+        <is>
+          <t>22/22</t>
+        </is>
+      </c>
+      <c r="I139" s="14" t="inlineStr">
+        <is>
+          <t>Result Declared</t>
+        </is>
+      </c>
+      <c r="J139" s="15" t="n">
+        <v>227</v>
+      </c>
+      <c r="K139" s="16" t="n">
+        <v>10.31818181818182</v>
       </c>
     </row>
     <row r="140">
@@ -8612,7 +8612,7 @@
       </c>
       <c r="I165" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J165" s="4" t="n">
@@ -10278,7 +10278,7 @@
       </c>
       <c r="I199" s="14" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J199" s="15" t="n">
@@ -10376,7 +10376,7 @@
       </c>
       <c r="I201" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J201" s="4" t="n">
@@ -10416,11 +10416,11 @@
         </is>
       </c>
       <c r="G202" s="15" t="n">
-        <v>212</v>
+        <v>30</v>
       </c>
       <c r="H202" s="14" t="inlineStr">
         <is>
-          <t>27/30</t>
+          <t>29/30</t>
         </is>
       </c>
       <c r="I202" s="14" t="inlineStr">
@@ -10429,10 +10429,10 @@
         </is>
       </c>
       <c r="J202" s="15" t="n">
-        <v>236</v>
+        <v>31</v>
       </c>
       <c r="K202" s="16" t="n">
-        <v>7.851851851851852</v>
+        <v>1.03448275862069</v>
       </c>
     </row>
     <row r="203">
@@ -10474,7 +10474,7 @@
       </c>
       <c r="I203" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J203" s="4" t="n">
@@ -10632,52 +10632,52 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="10" t="inlineStr">
+      <c r="A207" s="6" t="inlineStr">
         <is>
           <t>TIRUVANNAMALAI</t>
         </is>
       </c>
-      <c r="B207" s="10" t="n">
+      <c r="B207" s="7" t="n">
         <v>63</v>
       </c>
-      <c r="C207" s="10" t="inlineStr">
+      <c r="C207" s="7" t="inlineStr">
         <is>
           <t>VELU. E.V</t>
         </is>
       </c>
-      <c r="D207" s="10" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E207" s="10" t="inlineStr">
+      <c r="D207" s="7" t="inlineStr">
+        <is>
+          <t>Dravida Munnetra Kazhagam</t>
+        </is>
+      </c>
+      <c r="E207" s="7" t="inlineStr">
         <is>
           <t>ARUL ARUMUGAM</t>
         </is>
       </c>
-      <c r="F207" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="G207" s="11" t="n">
-        <v>3541</v>
-      </c>
-      <c r="H207" s="10" t="inlineStr">
-        <is>
-          <t>21/23</t>
-        </is>
-      </c>
-      <c r="I207" s="10" t="inlineStr">
+      <c r="F207" s="7" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="G207" s="8" t="n">
+        <v>2455</v>
+      </c>
+      <c r="H207" s="7" t="inlineStr">
+        <is>
+          <t>23/23</t>
+        </is>
+      </c>
+      <c r="I207" s="7" t="inlineStr">
         <is>
           <t>Result in Progress</t>
         </is>
       </c>
-      <c r="J207" s="11" t="n">
-        <v>3878</v>
-      </c>
-      <c r="K207" s="12" t="n">
-        <v>168.6190476190476</v>
+      <c r="J207" s="8" t="n">
+        <v>2455</v>
+      </c>
+      <c r="K207" s="9" t="n">
+        <v>106.7391304347826</v>
       </c>
     </row>
     <row r="208">
@@ -11592,11 +11592,11 @@
         </is>
       </c>
       <c r="G226" s="8" t="n">
-        <v>875</v>
+        <v>910</v>
       </c>
       <c r="H226" s="7" t="inlineStr">
         <is>
-          <t>22/23</t>
+          <t>23/23</t>
         </is>
       </c>
       <c r="I226" s="7" t="inlineStr">
@@ -11605,10 +11605,10 @@
         </is>
       </c>
       <c r="J226" s="8" t="n">
-        <v>915</v>
+        <v>910</v>
       </c>
       <c r="K226" s="9" t="n">
-        <v>39.77272727272727</v>
+        <v>39.56521739130435</v>
       </c>
     </row>
     <row r="227">

</xml_diff>

<commit_message>
Election snapshot: 100% counted — 229 declared, TIRUPPATTUR DMK wins by 30 votes
Final tally: TVK 106, DMK 61, AIADMK 47. 5 seats pending formal ECI declaration.

https://claude.ai/code/session_01MizbUy44JG5sXyvaf3Wekb
</commit_message>
<xml_diff>
--- a/tn_election_results_may2026.xlsx
+++ b/tn_election_results_may2026.xlsx
@@ -1899,7 +1899,7 @@
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J28" s="4" t="n">
@@ -2977,7 +2977,7 @@
       </c>
       <c r="I50" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J50" s="4" t="n">
@@ -3810,7 +3810,7 @@
       </c>
       <c r="I67" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J67" s="8" t="n">
@@ -5280,7 +5280,7 @@
       </c>
       <c r="I97" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J97" s="8" t="n">
@@ -7142,7 +7142,7 @@
       </c>
       <c r="I135" s="10" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J135" s="11" t="n">
@@ -8407,7 +8407,7 @@
         </is>
       </c>
       <c r="G161" s="11" t="n">
-        <v>3163</v>
+        <v>3198</v>
       </c>
       <c r="H161" s="10" t="inlineStr">
         <is>
@@ -8420,10 +8420,10 @@
         </is>
       </c>
       <c r="J161" s="11" t="n">
-        <v>3438</v>
+        <v>3476</v>
       </c>
       <c r="K161" s="12" t="n">
-        <v>137.5217391304348</v>
+        <v>139.0434782608696</v>
       </c>
     </row>
     <row r="162">
@@ -8456,7 +8456,7 @@
         </is>
       </c>
       <c r="G162" s="4" t="n">
-        <v>96370</v>
+        <v>96780</v>
       </c>
       <c r="H162" s="3" t="inlineStr">
         <is>
@@ -8469,10 +8469,10 @@
         </is>
       </c>
       <c r="J162" s="4" t="n">
-        <v>96370</v>
+        <v>96780</v>
       </c>
       <c r="K162" s="5" t="n">
-        <v>2920.30303030303</v>
+        <v>2932.727272727273</v>
       </c>
     </row>
     <row r="163">
@@ -10866,7 +10866,7 @@
       </c>
       <c r="I211" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J211" s="8" t="n">
@@ -11601,7 +11601,7 @@
       </c>
       <c r="I226" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J226" s="8" t="n">

</xml_diff>

<commit_message>
Election final: all 234 seats declared — TVK 108, DMK 59, AIADMK 47
TIRUPPATTUR result disputed (ECI showing duplicate entries: DMK 30 vs TVK 1).

https://claude.ai/code/session_01MizbUy44JG5sXyvaf3Wekb
</commit_message>
<xml_diff>
--- a/tn_election_results_may2026.xlsx
+++ b/tn_election_results_may2026.xlsx
@@ -3712,7 +3712,7 @@
       </c>
       <c r="I65" s="14" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J65" s="15" t="n">
@@ -8378,52 +8378,52 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="10" t="inlineStr">
+      <c r="A161" s="2" t="inlineStr">
         <is>
           <t>SHOLINGUR</t>
         </is>
       </c>
-      <c r="B161" s="10" t="n">
+      <c r="B161" s="3" t="n">
         <v>39</v>
       </c>
-      <c r="C161" s="10" t="inlineStr">
+      <c r="C161" s="3" t="inlineStr">
         <is>
           <t>G.KAPIL</t>
         </is>
       </c>
-      <c r="D161" s="10" t="inlineStr">
-        <is>
-          <t>Tamilaga Vettri Kazhagam</t>
-        </is>
-      </c>
-      <c r="E161" s="10" t="inlineStr">
+      <c r="D161" s="3" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E161" s="3" t="inlineStr">
         <is>
           <t>K.SARAVANAN</t>
         </is>
       </c>
-      <c r="F161" s="10" t="inlineStr">
+      <c r="F161" s="3" t="inlineStr">
         <is>
           <t>Pattali Makkal Katchi</t>
         </is>
       </c>
-      <c r="G161" s="11" t="n">
-        <v>3198</v>
-      </c>
-      <c r="H161" s="10" t="inlineStr">
-        <is>
-          <t>23/25</t>
-        </is>
-      </c>
-      <c r="I161" s="10" t="inlineStr">
-        <is>
-          <t>Result in Progress</t>
-        </is>
-      </c>
-      <c r="J161" s="11" t="n">
-        <v>3476</v>
-      </c>
-      <c r="K161" s="12" t="n">
-        <v>139.0434782608696</v>
+      <c r="G161" s="4" t="n">
+        <v>5686</v>
+      </c>
+      <c r="H161" s="3" t="inlineStr">
+        <is>
+          <t>26/26</t>
+        </is>
+      </c>
+      <c r="I161" s="3" t="inlineStr">
+        <is>
+          <t>Result Declared</t>
+        </is>
+      </c>
+      <c r="J161" s="4" t="n">
+        <v>5686</v>
+      </c>
+      <c r="K161" s="5" t="n">
+        <v>218.6923076923077</v>
       </c>
     </row>
     <row r="162">
@@ -8465,7 +8465,7 @@
       </c>
       <c r="I162" s="3" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J162" s="4" t="n">
@@ -10397,42 +10397,42 @@
       </c>
       <c r="C202" s="14" t="inlineStr">
         <is>
+          <t>SEENIVASA SETHUPATHY. R</t>
+        </is>
+      </c>
+      <c r="D202" s="14" t="inlineStr">
+        <is>
+          <t>Tamilaga Vettri Kazhagam</t>
+        </is>
+      </c>
+      <c r="E202" s="14" t="inlineStr">
+        <is>
           <t>PERIAKARUPPAN. KR</t>
         </is>
       </c>
-      <c r="D202" s="14" t="inlineStr">
-        <is>
-          <t>Dravida Munnetra Kazhagam</t>
-        </is>
-      </c>
-      <c r="E202" s="14" t="inlineStr">
-        <is>
-          <t>SEENIVASA SETHUPATHY. R</t>
-        </is>
-      </c>
       <c r="F202" s="14" t="inlineStr">
         <is>
-          <t>Tamilaga Vettri Kazhagam</t>
+          <t>Dravida Munnetra Kazhagam</t>
         </is>
       </c>
       <c r="G202" s="15" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="H202" s="14" t="inlineStr">
         <is>
-          <t>29/30</t>
+          <t>30/30</t>
         </is>
       </c>
       <c r="I202" s="14" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J202" s="15" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="K202" s="16" t="n">
-        <v>1.03448275862069</v>
+        <v>0.03333333333333333</v>
       </c>
     </row>
     <row r="203">
@@ -10670,7 +10670,7 @@
       </c>
       <c r="I207" s="7" t="inlineStr">
         <is>
-          <t>Result in Progress</t>
+          <t>Result Declared</t>
         </is>
       </c>
       <c r="J207" s="8" t="n">

</xml_diff>